<commit_message>
Complete draft of input_template.md
</commit_message>
<xml_diff>
--- a/docs/inputs/input_template.xlsx
+++ b/docs/inputs/input_template.xlsx
@@ -5,12 +5,12 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/njones/python_projects/xslope/inputs/seep/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/njones/python_projects/xslope/docs/inputs/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{61E2C959-74FE-774E-8809-918B9D7782BC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5BBBB099-0EF8-FB45-B361-D0BEF56F2FFA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="31200" yWindow="2160" windowWidth="28700" windowHeight="22660" xr2:uid="{BA54C293-CE08-6E4C-9212-B3317DAA148E}"/>
+    <workbookView xWindow="11860" yWindow="2300" windowWidth="28700" windowHeight="22660" xr2:uid="{BA54C293-CE08-6E4C-9212-B3317DAA148E}"/>
   </bookViews>
   <sheets>
     <sheet name="main" sheetId="1" r:id="rId1"/>
@@ -56,7 +56,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="248" uniqueCount="161">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="250" uniqueCount="163">
   <si>
     <t>X</t>
   </si>
@@ -643,6 +643,12 @@
   </si>
   <si>
     <t>Bedrock</t>
+  </si>
+  <si>
+    <t>plot</t>
+  </si>
+  <si>
+    <t>Plot of geometric inputs from other sheets</t>
   </si>
 </sst>
 </file>
@@ -6366,78 +6372,82 @@
     </row>
     <row r="8" spans="1:5" x14ac:dyDescent="0.2">
       <c r="B8" s="1" t="s">
-        <v>17</v>
+        <v>161</v>
       </c>
       <c r="C8" t="s">
-        <v>18</v>
-      </c>
-      <c r="D8"/>
+        <v>162</v>
+      </c>
     </row>
     <row r="9" spans="1:5" x14ac:dyDescent="0.2">
       <c r="B9" s="1" t="s">
-        <v>19</v>
+        <v>17</v>
       </c>
       <c r="C9" t="s">
-        <v>20</v>
+        <v>18</v>
       </c>
       <c r="D9"/>
     </row>
     <row r="10" spans="1:5" x14ac:dyDescent="0.2">
       <c r="B10" s="1" t="s">
-        <v>21</v>
+        <v>19</v>
       </c>
       <c r="C10" t="s">
-        <v>22</v>
+        <v>20</v>
       </c>
       <c r="D10"/>
     </row>
     <row r="11" spans="1:5" x14ac:dyDescent="0.2">
       <c r="B11" s="1" t="s">
-        <v>23</v>
+        <v>21</v>
       </c>
       <c r="C11" t="s">
-        <v>24</v>
+        <v>22</v>
       </c>
       <c r="D11"/>
     </row>
     <row r="12" spans="1:5" x14ac:dyDescent="0.2">
       <c r="B12" s="1" t="s">
-        <v>38</v>
+        <v>23</v>
       </c>
       <c r="C12" t="s">
-        <v>39</v>
+        <v>24</v>
       </c>
       <c r="D12"/>
     </row>
     <row r="13" spans="1:5" x14ac:dyDescent="0.2">
       <c r="B13" s="1" t="s">
-        <v>34</v>
+        <v>38</v>
       </c>
       <c r="C13" t="s">
-        <v>35</v>
+        <v>39</v>
       </c>
       <c r="D13"/>
     </row>
     <row r="14" spans="1:5" x14ac:dyDescent="0.2">
       <c r="B14" s="1" t="s">
-        <v>36</v>
+        <v>34</v>
       </c>
       <c r="C14" t="s">
-        <v>37</v>
+        <v>35</v>
       </c>
       <c r="D14"/>
     </row>
     <row r="15" spans="1:5" x14ac:dyDescent="0.2">
       <c r="B15" s="1" t="s">
+        <v>36</v>
+      </c>
+      <c r="C15" t="s">
+        <v>37</v>
+      </c>
+      <c r="D15"/>
+    </row>
+    <row r="16" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="B16" s="1" t="s">
         <v>111</v>
       </c>
-      <c r="C15" s="9" t="s">
+      <c r="C16" s="9" t="s">
         <v>110</v>
       </c>
-      <c r="D15" s="9"/>
-    </row>
-    <row r="16" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="B16" s="1"/>
       <c r="D16" s="9"/>
     </row>
     <row r="17" spans="2:4" x14ac:dyDescent="0.2">
@@ -7792,21 +7802,21 @@
     </row>
   </sheetData>
   <mergeCells count="15">
+    <mergeCell ref="A4:B4"/>
+    <mergeCell ref="D4:E4"/>
+    <mergeCell ref="G4:H4"/>
+    <mergeCell ref="J4:K4"/>
+    <mergeCell ref="M4:N4"/>
+    <mergeCell ref="A22:B22"/>
+    <mergeCell ref="D22:E22"/>
+    <mergeCell ref="G22:H22"/>
+    <mergeCell ref="J22:K22"/>
+    <mergeCell ref="M22:N22"/>
     <mergeCell ref="A40:B40"/>
     <mergeCell ref="D40:E40"/>
     <mergeCell ref="G40:H40"/>
     <mergeCell ref="J40:K40"/>
     <mergeCell ref="M40:N40"/>
-    <mergeCell ref="A22:B22"/>
-    <mergeCell ref="D22:E22"/>
-    <mergeCell ref="G22:H22"/>
-    <mergeCell ref="J22:K22"/>
-    <mergeCell ref="M22:N22"/>
-    <mergeCell ref="A4:B4"/>
-    <mergeCell ref="D4:E4"/>
-    <mergeCell ref="G4:H4"/>
-    <mergeCell ref="J4:K4"/>
-    <mergeCell ref="M4:N4"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>

<commit_message>
added cosmetic changes to input_template.xlsx
</commit_message>
<xml_diff>
--- a/docs/inputs/input_template.xlsx
+++ b/docs/inputs/input_template.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="11003"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="11214"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/njones/python_projects/xslope/docs/inputs/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5BBBB099-0EF8-FB45-B361-D0BEF56F2FFA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DCB041F0-5032-BD48-9DF2-1DFA485A090D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="11860" yWindow="2300" windowWidth="28700" windowHeight="22660" xr2:uid="{BA54C293-CE08-6E4C-9212-B3317DAA148E}"/>
+    <workbookView xWindow="36080" yWindow="2580" windowWidth="28700" windowHeight="22660" xr2:uid="{BA54C293-CE08-6E4C-9212-B3317DAA148E}"/>
   </bookViews>
   <sheets>
     <sheet name="main" sheetId="1" r:id="rId1"/>
@@ -56,7 +56,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="250" uniqueCount="163">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="262" uniqueCount="163">
   <si>
     <t>X</t>
   </si>
@@ -7802,21 +7802,21 @@
     </row>
   </sheetData>
   <mergeCells count="15">
+    <mergeCell ref="A40:B40"/>
+    <mergeCell ref="D40:E40"/>
+    <mergeCell ref="G40:H40"/>
+    <mergeCell ref="J40:K40"/>
+    <mergeCell ref="M40:N40"/>
+    <mergeCell ref="A22:B22"/>
+    <mergeCell ref="D22:E22"/>
+    <mergeCell ref="G22:H22"/>
+    <mergeCell ref="J22:K22"/>
+    <mergeCell ref="M22:N22"/>
     <mergeCell ref="A4:B4"/>
     <mergeCell ref="D4:E4"/>
     <mergeCell ref="G4:H4"/>
     <mergeCell ref="J4:K4"/>
     <mergeCell ref="M4:N4"/>
-    <mergeCell ref="A22:B22"/>
-    <mergeCell ref="D22:E22"/>
-    <mergeCell ref="G22:H22"/>
-    <mergeCell ref="J22:K22"/>
-    <mergeCell ref="M22:N22"/>
-    <mergeCell ref="A40:B40"/>
-    <mergeCell ref="D40:E40"/>
-    <mergeCell ref="G40:H40"/>
-    <mergeCell ref="J40:K40"/>
-    <mergeCell ref="M40:N40"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
@@ -7829,9 +7829,9 @@
   <cols>
     <col min="1" max="1" width="7" style="1" customWidth="1"/>
     <col min="2" max="2" width="17.33203125" style="1" customWidth="1"/>
-    <col min="3" max="9" width="8.5" style="1" hidden="1" customWidth="1"/>
-    <col min="10" max="13" width="8.5" hidden="1" customWidth="1"/>
-    <col min="14" max="17" width="0" hidden="1" customWidth="1"/>
+    <col min="3" max="9" width="8.5" style="1" customWidth="1"/>
+    <col min="10" max="13" width="8.5" customWidth="1"/>
+    <col min="14" max="17" width="10.83203125" customWidth="1"/>
     <col min="23" max="23" width="10.83203125" style="1"/>
   </cols>
   <sheetData>
@@ -7954,10 +7954,18 @@
       <c r="B4" s="3" t="s">
         <v>149</v>
       </c>
-      <c r="C4" s="3"/>
-      <c r="D4" s="3"/>
-      <c r="E4" s="3"/>
-      <c r="F4" s="3"/>
+      <c r="C4" s="3">
+        <v>140</v>
+      </c>
+      <c r="D4" s="3" t="s">
+        <v>68</v>
+      </c>
+      <c r="E4" s="3">
+        <v>0</v>
+      </c>
+      <c r="F4" s="3">
+        <v>38</v>
+      </c>
       <c r="G4" s="3"/>
       <c r="H4" s="3"/>
       <c r="I4" s="3"/>
@@ -7975,7 +7983,9 @@
       <c r="S4" s="3">
         <v>100000</v>
       </c>
-      <c r="T4" s="3"/>
+      <c r="T4" s="3">
+        <v>0</v>
+      </c>
       <c r="U4" s="3"/>
       <c r="V4" s="3"/>
       <c r="W4" s="3"/>
@@ -7988,10 +7998,18 @@
       <c r="B5" s="3" t="s">
         <v>150</v>
       </c>
-      <c r="C5" s="3"/>
-      <c r="D5" s="3"/>
-      <c r="E5" s="3"/>
-      <c r="F5" s="3"/>
+      <c r="C5" s="3">
+        <v>135</v>
+      </c>
+      <c r="D5" s="3" t="s">
+        <v>68</v>
+      </c>
+      <c r="E5" s="3">
+        <v>0</v>
+      </c>
+      <c r="F5" s="3">
+        <v>35</v>
+      </c>
       <c r="G5" s="3"/>
       <c r="H5" s="3"/>
       <c r="I5" s="3"/>
@@ -8022,10 +8040,18 @@
       <c r="B6" s="3" t="s">
         <v>151</v>
       </c>
-      <c r="C6" s="3"/>
-      <c r="D6" s="3"/>
-      <c r="E6" s="3"/>
-      <c r="F6" s="3"/>
+      <c r="C6" s="3">
+        <v>140</v>
+      </c>
+      <c r="D6" s="3" t="s">
+        <v>68</v>
+      </c>
+      <c r="E6" s="3">
+        <v>0</v>
+      </c>
+      <c r="F6" s="3">
+        <v>38</v>
+      </c>
       <c r="G6" s="3"/>
       <c r="H6" s="3"/>
       <c r="I6" s="3"/>
@@ -8056,10 +8082,18 @@
       <c r="B7" s="3" t="s">
         <v>152</v>
       </c>
-      <c r="C7" s="3"/>
-      <c r="D7" s="3"/>
-      <c r="E7" s="3"/>
-      <c r="F7" s="3"/>
+      <c r="C7" s="3">
+        <v>135</v>
+      </c>
+      <c r="D7" s="3" t="s">
+        <v>68</v>
+      </c>
+      <c r="E7" s="3">
+        <v>0</v>
+      </c>
+      <c r="F7" s="3">
+        <v>35</v>
+      </c>
       <c r="G7" s="3"/>
       <c r="H7" s="3"/>
       <c r="I7" s="3"/>
@@ -8090,10 +8124,18 @@
       <c r="B8" s="3" t="s">
         <v>153</v>
       </c>
-      <c r="C8" s="3"/>
-      <c r="D8" s="3"/>
-      <c r="E8" s="3"/>
-      <c r="F8" s="3"/>
+      <c r="C8" s="3">
+        <v>128</v>
+      </c>
+      <c r="D8" s="3" t="s">
+        <v>68</v>
+      </c>
+      <c r="E8" s="3">
+        <v>400</v>
+      </c>
+      <c r="F8" s="3">
+        <v>24</v>
+      </c>
       <c r="G8" s="3"/>
       <c r="H8" s="3"/>
       <c r="I8" s="3"/>
@@ -8124,10 +8166,18 @@
       <c r="B9" s="3" t="s">
         <v>154</v>
       </c>
-      <c r="C9" s="3"/>
-      <c r="D9" s="3"/>
-      <c r="E9" s="3"/>
-      <c r="F9" s="3"/>
+      <c r="C9" s="3">
+        <v>135</v>
+      </c>
+      <c r="D9" s="3" t="s">
+        <v>68</v>
+      </c>
+      <c r="E9" s="3">
+        <v>0</v>
+      </c>
+      <c r="F9" s="3">
+        <v>35</v>
+      </c>
       <c r="G9" s="3"/>
       <c r="H9" s="3"/>
       <c r="I9" s="3"/>
@@ -8158,10 +8208,18 @@
       <c r="B10" s="3" t="s">
         <v>155</v>
       </c>
-      <c r="C10" s="3"/>
-      <c r="D10" s="3"/>
-      <c r="E10" s="3"/>
-      <c r="F10" s="3"/>
+      <c r="C10" s="3">
+        <v>138</v>
+      </c>
+      <c r="D10" s="3" t="s">
+        <v>68</v>
+      </c>
+      <c r="E10" s="3">
+        <v>0</v>
+      </c>
+      <c r="F10" s="3">
+        <v>35</v>
+      </c>
       <c r="G10" s="3"/>
       <c r="H10" s="3"/>
       <c r="I10" s="3"/>
@@ -8192,10 +8250,18 @@
       <c r="B11" s="3" t="s">
         <v>156</v>
       </c>
-      <c r="C11" s="3"/>
-      <c r="D11" s="3"/>
-      <c r="E11" s="3"/>
-      <c r="F11" s="3"/>
+      <c r="C11" s="3">
+        <v>134</v>
+      </c>
+      <c r="D11" s="3" t="s">
+        <v>68</v>
+      </c>
+      <c r="E11" s="3">
+        <v>0</v>
+      </c>
+      <c r="F11" s="3">
+        <v>36</v>
+      </c>
       <c r="G11" s="3"/>
       <c r="H11" s="3"/>
       <c r="I11" s="3"/>
@@ -8226,12 +8292,20 @@
       <c r="B12" s="3" t="s">
         <v>157</v>
       </c>
-      <c r="C12" s="3"/>
-      <c r="D12" s="3"/>
+      <c r="C12" s="3">
+        <v>132</v>
+      </c>
+      <c r="D12" s="3" t="s">
+        <v>71</v>
+      </c>
       <c r="E12" s="3"/>
       <c r="F12" s="3"/>
-      <c r="G12" s="3"/>
-      <c r="H12" s="3"/>
+      <c r="G12" s="3">
+        <v>100</v>
+      </c>
+      <c r="H12" s="3">
+        <v>80</v>
+      </c>
       <c r="I12" s="3"/>
       <c r="J12" s="3"/>
       <c r="K12" s="3"/>
@@ -8260,12 +8334,20 @@
       <c r="B13" s="3" t="s">
         <v>158</v>
       </c>
-      <c r="C13" s="3"/>
-      <c r="D13" s="3"/>
+      <c r="C13" s="3">
+        <v>132</v>
+      </c>
+      <c r="D13" s="3" t="s">
+        <v>71</v>
+      </c>
       <c r="E13" s="3"/>
       <c r="F13" s="3"/>
-      <c r="G13" s="3"/>
-      <c r="H13" s="3"/>
+      <c r="G13" s="3">
+        <v>100</v>
+      </c>
+      <c r="H13" s="3">
+        <v>80</v>
+      </c>
       <c r="I13" s="3"/>
       <c r="J13" s="3"/>
       <c r="K13" s="3"/>
@@ -8294,10 +8376,18 @@
       <c r="B14" s="3" t="s">
         <v>159</v>
       </c>
-      <c r="C14" s="3"/>
-      <c r="D14" s="3"/>
-      <c r="E14" s="3"/>
-      <c r="F14" s="3"/>
+      <c r="C14" s="3">
+        <v>140</v>
+      </c>
+      <c r="D14" s="3" t="s">
+        <v>68</v>
+      </c>
+      <c r="E14" s="3">
+        <v>2000</v>
+      </c>
+      <c r="F14" s="3">
+        <v>40</v>
+      </c>
       <c r="G14" s="3"/>
       <c r="H14" s="3"/>
       <c r="I14" s="3"/>
@@ -8328,10 +8418,18 @@
       <c r="B15" s="3" t="s">
         <v>160</v>
       </c>
-      <c r="C15" s="3"/>
-      <c r="D15" s="3"/>
-      <c r="E15" s="3"/>
-      <c r="F15" s="3"/>
+      <c r="C15" s="3">
+        <v>140</v>
+      </c>
+      <c r="D15" s="3" t="s">
+        <v>68</v>
+      </c>
+      <c r="E15" s="3">
+        <v>2000</v>
+      </c>
+      <c r="F15" s="3">
+        <v>40</v>
+      </c>
       <c r="G15" s="3"/>
       <c r="H15" s="3"/>
       <c r="I15" s="3"/>
@@ -8591,12 +8689,12 @@
     <mergeCell ref="L22:Q22"/>
     <mergeCell ref="L2:Q2"/>
   </mergeCells>
-  <conditionalFormatting sqref="E4:F19 M4:N19 R19:V19">
+  <conditionalFormatting sqref="M4:N19 R19:V19 E4:F19">
     <cfRule type="expression" dxfId="3" priority="2">
       <formula>$D4="cp"</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="G4:H18 O4:O18 G19:J19 O19:Q19">
+  <conditionalFormatting sqref="O4:O18 G19:J19 O19:Q19 G4:H18">
     <cfRule type="expression" dxfId="2" priority="9">
       <formula>$D4="mc"</formula>
     </cfRule>

</xml_diff>

<commit_message>
Changed input template to NOT include the names of the mesh and seepage solution files when one of the materials has the "seep" option. Rather, it is assumed that if the input file is myfile.xlsx, the mesh file is myfile_mesh.json, and the seepage solution files are myfile_seep.csv and myfile_seep2.csv.
</commit_message>
<xml_diff>
--- a/docs/inputs/input_template.xlsx
+++ b/docs/inputs/input_template.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="11214"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10102"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/Jones/python_projects/xslope/docs/inputs/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/njones/python_projects/xslope/docs/inputs/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7882C987-C547-0D42-B78A-AD1046972FB1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{82220011-1717-904E-A1A8-1B94F8793234}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-20" yWindow="1060" windowWidth="34200" windowHeight="20240" xr2:uid="{BA54C293-CE08-6E4C-9212-B3317DAA148E}"/>
+    <workbookView xWindow="24520" yWindow="2880" windowWidth="34200" windowHeight="20240" activeTab="3" xr2:uid="{BA54C293-CE08-6E4C-9212-B3317DAA148E}"/>
   </bookViews>
   <sheets>
     <sheet name="main" sheetId="1" r:id="rId1"/>
@@ -58,7 +58,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="292" uniqueCount="162">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="286" uniqueCount="156">
   <si>
     <t>X</t>
   </si>
@@ -468,24 +468,6 @@
   </si>
   <si>
     <t>XSLOPE Input Template</t>
-  </si>
-  <si>
-    <t>Seepage files</t>
-  </si>
-  <si>
-    <t>mesh:</t>
-  </si>
-  <si>
-    <t>solution 2:</t>
-  </si>
-  <si>
-    <t>solution 1:</t>
-  </si>
-  <si>
-    <t>seep_mesh.json</t>
-  </si>
-  <si>
-    <t>seep_solution.csv</t>
   </si>
   <si>
     <t>Stress</t>
@@ -931,7 +913,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="55">
+  <cellXfs count="52">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -1025,6 +1007,25 @@
     <xf numFmtId="0" fontId="0" fillId="4" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" quotePrefix="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="2" fillId="12" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="13" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="13" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="14" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="14" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
     <xf numFmtId="0" fontId="4" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
@@ -1033,9 +1034,6 @@
     </xf>
     <xf numFmtId="0" fontId="10" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment horizontal="left"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="7" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -1049,48 +1047,18 @@
     <xf numFmtId="0" fontId="1" fillId="6" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" quotePrefix="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="2" fillId="12" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="2" fillId="13" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="13" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="14" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="14" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
     <xf numFmtId="0" fontId="1" fillId="10" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="15" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="8">
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor theme="0" tint="-0.499984740745262"/>
-        </patternFill>
-      </fill>
-    </dxf>
+  <dxfs count="6">
     <dxf>
       <fill>
         <patternFill>
@@ -1102,13 +1070,6 @@
       <fill>
         <patternFill>
           <bgColor theme="2" tint="-0.499984740745262"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor theme="0" tint="-0.499984740745262"/>
         </patternFill>
       </fill>
     </dxf>
@@ -3010,6 +2971,11 @@
               </a:ln>
               <a:effectLst/>
             </c:spPr>
+            <c:extLst>
+              <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+                <c16:uniqueId val="{00000001-3920-BF44-925A-9D95B0B535DF}"/>
+              </c:ext>
+            </c:extLst>
           </c:dPt>
           <c:dPt>
             <c:idx val="1"/>
@@ -3044,6 +3010,11 @@
               </a:ln>
               <a:effectLst/>
             </c:spPr>
+            <c:extLst>
+              <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+                <c16:uniqueId val="{00000003-3920-BF44-925A-9D95B0B535DF}"/>
+              </c:ext>
+            </c:extLst>
           </c:dPt>
           <c:dPt>
             <c:idx val="2"/>
@@ -3078,6 +3049,11 @@
               </a:ln>
               <a:effectLst/>
             </c:spPr>
+            <c:extLst>
+              <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+                <c16:uniqueId val="{00000005-3920-BF44-925A-9D95B0B535DF}"/>
+              </c:ext>
+            </c:extLst>
           </c:dPt>
           <c:dPt>
             <c:idx val="3"/>
@@ -3112,6 +3088,11 @@
               </a:ln>
               <a:effectLst/>
             </c:spPr>
+            <c:extLst>
+              <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+                <c16:uniqueId val="{00000007-3920-BF44-925A-9D95B0B535DF}"/>
+              </c:ext>
+            </c:extLst>
           </c:dPt>
           <c:dPt>
             <c:idx val="4"/>
@@ -3146,6 +3127,11 @@
               </a:ln>
               <a:effectLst/>
             </c:spPr>
+            <c:extLst>
+              <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+                <c16:uniqueId val="{00000009-3920-BF44-925A-9D95B0B535DF}"/>
+              </c:ext>
+            </c:extLst>
           </c:dPt>
           <c:dPt>
             <c:idx val="5"/>
@@ -3180,6 +3166,11 @@
               </a:ln>
               <a:effectLst/>
             </c:spPr>
+            <c:extLst>
+              <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+                <c16:uniqueId val="{0000000B-3920-BF44-925A-9D95B0B535DF}"/>
+              </c:ext>
+            </c:extLst>
           </c:dPt>
           <c:dPt>
             <c:idx val="6"/>
@@ -3214,6 +3205,11 @@
               </a:ln>
               <a:effectLst/>
             </c:spPr>
+            <c:extLst>
+              <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+                <c16:uniqueId val="{0000000D-3920-BF44-925A-9D95B0B535DF}"/>
+              </c:ext>
+            </c:extLst>
           </c:dPt>
           <c:dPt>
             <c:idx val="7"/>
@@ -3248,6 +3244,11 @@
               </a:ln>
               <a:effectLst/>
             </c:spPr>
+            <c:extLst>
+              <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+                <c16:uniqueId val="{0000000F-3920-BF44-925A-9D95B0B535DF}"/>
+              </c:ext>
+            </c:extLst>
           </c:dPt>
           <c:dPt>
             <c:idx val="8"/>
@@ -3282,6 +3283,11 @@
               </a:ln>
               <a:effectLst/>
             </c:spPr>
+            <c:extLst>
+              <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+                <c16:uniqueId val="{00000011-3920-BF44-925A-9D95B0B535DF}"/>
+              </c:ext>
+            </c:extLst>
           </c:dPt>
           <c:dPt>
             <c:idx val="9"/>
@@ -3316,6 +3322,11 @@
               </a:ln>
               <a:effectLst/>
             </c:spPr>
+            <c:extLst>
+              <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+                <c16:uniqueId val="{00000013-3920-BF44-925A-9D95B0B535DF}"/>
+              </c:ext>
+            </c:extLst>
           </c:dPt>
           <c:dPt>
             <c:idx val="10"/>
@@ -3350,6 +3361,11 @@
               </a:ln>
               <a:effectLst/>
             </c:spPr>
+            <c:extLst>
+              <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+                <c16:uniqueId val="{00000015-3920-BF44-925A-9D95B0B535DF}"/>
+              </c:ext>
+            </c:extLst>
           </c:dPt>
           <c:dPt>
             <c:idx val="11"/>
@@ -3384,6 +3400,11 @@
               </a:ln>
               <a:effectLst/>
             </c:spPr>
+            <c:extLst>
+              <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+                <c16:uniqueId val="{00000017-3920-BF44-925A-9D95B0B535DF}"/>
+              </c:ext>
+            </c:extLst>
           </c:dPt>
           <c:dPt>
             <c:idx val="12"/>
@@ -3418,6 +3439,11 @@
               </a:ln>
               <a:effectLst/>
             </c:spPr>
+            <c:extLst>
+              <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+                <c16:uniqueId val="{00000019-3920-BF44-925A-9D95B0B535DF}"/>
+              </c:ext>
+            </c:extLst>
           </c:dPt>
           <c:dPt>
             <c:idx val="13"/>
@@ -3452,6 +3478,11 @@
               </a:ln>
               <a:effectLst/>
             </c:spPr>
+            <c:extLst>
+              <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+                <c16:uniqueId val="{0000001B-3920-BF44-925A-9D95B0B535DF}"/>
+              </c:ext>
+            </c:extLst>
           </c:dPt>
           <c:dPt>
             <c:idx val="14"/>
@@ -3486,6 +3517,11 @@
               </a:ln>
               <a:effectLst/>
             </c:spPr>
+            <c:extLst>
+              <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+                <c16:uniqueId val="{0000001D-3920-BF44-925A-9D95B0B535DF}"/>
+              </c:ext>
+            </c:extLst>
           </c:dPt>
           <c:dPt>
             <c:idx val="15"/>
@@ -3520,6 +3556,11 @@
               </a:ln>
               <a:effectLst/>
             </c:spPr>
+            <c:extLst>
+              <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+                <c16:uniqueId val="{0000001F-3920-BF44-925A-9D95B0B535DF}"/>
+              </c:ext>
+            </c:extLst>
           </c:dPt>
           <c:dPt>
             <c:idx val="16"/>
@@ -3554,6 +3595,11 @@
               </a:ln>
               <a:effectLst/>
             </c:spPr>
+            <c:extLst>
+              <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+                <c16:uniqueId val="{00000021-3920-BF44-925A-9D95B0B535DF}"/>
+              </c:ext>
+            </c:extLst>
           </c:dPt>
           <c:dPt>
             <c:idx val="17"/>
@@ -3588,6 +3634,11 @@
               </a:ln>
               <a:effectLst/>
             </c:spPr>
+            <c:extLst>
+              <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+                <c16:uniqueId val="{00000023-3920-BF44-925A-9D95B0B535DF}"/>
+              </c:ext>
+            </c:extLst>
           </c:dPt>
           <c:dPt>
             <c:idx val="18"/>
@@ -3622,6 +3673,11 @@
               </a:ln>
               <a:effectLst/>
             </c:spPr>
+            <c:extLst>
+              <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+                <c16:uniqueId val="{00000025-3920-BF44-925A-9D95B0B535DF}"/>
+              </c:ext>
+            </c:extLst>
           </c:dPt>
           <c:xVal>
             <c:numRef>
@@ -5335,6 +5391,11 @@
               </c:spPr>
             </c:marker>
             <c:bubble3D val="0"/>
+            <c:extLst>
+              <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+                <c16:uniqueId val="{00000026-3920-BF44-925A-9D95B0B535DF}"/>
+              </c:ext>
+            </c:extLst>
           </c:dPt>
           <c:dPt>
             <c:idx val="1"/>
@@ -5360,6 +5421,11 @@
               </c:spPr>
             </c:marker>
             <c:bubble3D val="0"/>
+            <c:extLst>
+              <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+                <c16:uniqueId val="{00000027-3920-BF44-925A-9D95B0B535DF}"/>
+              </c:ext>
+            </c:extLst>
           </c:dPt>
           <c:dPt>
             <c:idx val="2"/>
@@ -5385,6 +5451,11 @@
               </c:spPr>
             </c:marker>
             <c:bubble3D val="0"/>
+            <c:extLst>
+              <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+                <c16:uniqueId val="{00000028-3920-BF44-925A-9D95B0B535DF}"/>
+              </c:ext>
+            </c:extLst>
           </c:dPt>
           <c:dPt>
             <c:idx val="3"/>
@@ -5410,6 +5481,11 @@
               </c:spPr>
             </c:marker>
             <c:bubble3D val="0"/>
+            <c:extLst>
+              <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+                <c16:uniqueId val="{00000029-3920-BF44-925A-9D95B0B535DF}"/>
+              </c:ext>
+            </c:extLst>
           </c:dPt>
           <c:dPt>
             <c:idx val="4"/>
@@ -5435,6 +5511,11 @@
               </c:spPr>
             </c:marker>
             <c:bubble3D val="0"/>
+            <c:extLst>
+              <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+                <c16:uniqueId val="{0000002A-3920-BF44-925A-9D95B0B535DF}"/>
+              </c:ext>
+            </c:extLst>
           </c:dPt>
           <c:dPt>
             <c:idx val="5"/>
@@ -5460,6 +5541,11 @@
               </c:spPr>
             </c:marker>
             <c:bubble3D val="0"/>
+            <c:extLst>
+              <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+                <c16:uniqueId val="{0000002B-3920-BF44-925A-9D95B0B535DF}"/>
+              </c:ext>
+            </c:extLst>
           </c:dPt>
           <c:dPt>
             <c:idx val="6"/>
@@ -5485,6 +5571,11 @@
               </c:spPr>
             </c:marker>
             <c:bubble3D val="0"/>
+            <c:extLst>
+              <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+                <c16:uniqueId val="{0000002C-3920-BF44-925A-9D95B0B535DF}"/>
+              </c:ext>
+            </c:extLst>
           </c:dPt>
           <c:dPt>
             <c:idx val="7"/>
@@ -5510,6 +5601,11 @@
               </c:spPr>
             </c:marker>
             <c:bubble3D val="0"/>
+            <c:extLst>
+              <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+                <c16:uniqueId val="{0000002D-3920-BF44-925A-9D95B0B535DF}"/>
+              </c:ext>
+            </c:extLst>
           </c:dPt>
           <c:dPt>
             <c:idx val="8"/>
@@ -5535,6 +5631,11 @@
               </c:spPr>
             </c:marker>
             <c:bubble3D val="0"/>
+            <c:extLst>
+              <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+                <c16:uniqueId val="{0000002E-3920-BF44-925A-9D95B0B535DF}"/>
+              </c:ext>
+            </c:extLst>
           </c:dPt>
           <c:dPt>
             <c:idx val="9"/>
@@ -5560,6 +5661,11 @@
               </c:spPr>
             </c:marker>
             <c:bubble3D val="0"/>
+            <c:extLst>
+              <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+                <c16:uniqueId val="{0000002F-3920-BF44-925A-9D95B0B535DF}"/>
+              </c:ext>
+            </c:extLst>
           </c:dPt>
           <c:dPt>
             <c:idx val="10"/>
@@ -5585,6 +5691,11 @@
               </c:spPr>
             </c:marker>
             <c:bubble3D val="0"/>
+            <c:extLst>
+              <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+                <c16:uniqueId val="{00000030-3920-BF44-925A-9D95B0B535DF}"/>
+              </c:ext>
+            </c:extLst>
           </c:dPt>
           <c:dPt>
             <c:idx val="11"/>
@@ -5610,6 +5721,11 @@
               </c:spPr>
             </c:marker>
             <c:bubble3D val="0"/>
+            <c:extLst>
+              <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+                <c16:uniqueId val="{00000031-3920-BF44-925A-9D95B0B535DF}"/>
+              </c:ext>
+            </c:extLst>
           </c:dPt>
           <c:dPt>
             <c:idx val="12"/>
@@ -5635,6 +5751,11 @@
               </c:spPr>
             </c:marker>
             <c:bubble3D val="0"/>
+            <c:extLst>
+              <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+                <c16:uniqueId val="{00000032-3920-BF44-925A-9D95B0B535DF}"/>
+              </c:ext>
+            </c:extLst>
           </c:dPt>
           <c:dPt>
             <c:idx val="13"/>
@@ -5660,6 +5781,11 @@
               </c:spPr>
             </c:marker>
             <c:bubble3D val="0"/>
+            <c:extLst>
+              <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+                <c16:uniqueId val="{00000033-3920-BF44-925A-9D95B0B535DF}"/>
+              </c:ext>
+            </c:extLst>
           </c:dPt>
           <c:dPt>
             <c:idx val="14"/>
@@ -5685,6 +5811,11 @@
               </c:spPr>
             </c:marker>
             <c:bubble3D val="0"/>
+            <c:extLst>
+              <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+                <c16:uniqueId val="{00000034-3920-BF44-925A-9D95B0B535DF}"/>
+              </c:ext>
+            </c:extLst>
           </c:dPt>
           <c:dPt>
             <c:idx val="15"/>
@@ -5710,6 +5841,11 @@
               </c:spPr>
             </c:marker>
             <c:bubble3D val="0"/>
+            <c:extLst>
+              <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+                <c16:uniqueId val="{00000035-3920-BF44-925A-9D95B0B535DF}"/>
+              </c:ext>
+            </c:extLst>
           </c:dPt>
           <c:dPt>
             <c:idx val="16"/>
@@ -5735,6 +5871,11 @@
               </c:spPr>
             </c:marker>
             <c:bubble3D val="0"/>
+            <c:extLst>
+              <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+                <c16:uniqueId val="{00000036-3920-BF44-925A-9D95B0B535DF}"/>
+              </c:ext>
+            </c:extLst>
           </c:dPt>
           <c:dPt>
             <c:idx val="17"/>
@@ -5760,6 +5901,11 @@
               </c:spPr>
             </c:marker>
             <c:bubble3D val="0"/>
+            <c:extLst>
+              <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+                <c16:uniqueId val="{00000037-3920-BF44-925A-9D95B0B535DF}"/>
+              </c:ext>
+            </c:extLst>
           </c:dPt>
           <c:xVal>
             <c:numRef>
@@ -7950,20 +8096,20 @@
       <c r="C5" s="14" t="s">
         <v>79</v>
       </c>
-      <c r="D5" s="43">
+      <c r="D5" s="35">
         <v>8</v>
       </c>
     </row>
     <row r="7" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="B7" s="35" t="s">
+      <c r="B7" s="42" t="s">
         <v>47</v>
       </c>
-      <c r="C7" s="35"/>
-      <c r="D7" s="35"/>
+      <c r="C7" s="42"/>
+      <c r="D7" s="42"/>
       <c r="F7" s="15" t="s">
         <v>15</v>
       </c>
-      <c r="G7" s="44" t="s">
+      <c r="G7" s="36" t="s">
         <v>16</v>
       </c>
     </row>
@@ -7975,10 +8121,10 @@
         <v>62.4</v>
       </c>
       <c r="F8" s="1" t="s">
-        <v>127</v>
+        <v>121</v>
       </c>
       <c r="G8" t="s">
-        <v>128</v>
+        <v>122</v>
       </c>
     </row>
     <row r="9" spans="1:7" x14ac:dyDescent="0.2">
@@ -8050,10 +8196,10 @@
     </row>
     <row r="15" spans="1:7" x14ac:dyDescent="0.2">
       <c r="F15" s="1" t="s">
-        <v>129</v>
+        <v>123</v>
       </c>
       <c r="G15" t="s">
-        <v>131</v>
+        <v>125</v>
       </c>
     </row>
     <row r="16" spans="1:7" x14ac:dyDescent="0.2">
@@ -8070,15 +8216,15 @@
         <v>98</v>
       </c>
       <c r="G17" s="9" t="s">
-        <v>133</v>
+        <v>127</v>
       </c>
     </row>
     <row r="18" spans="2:7" x14ac:dyDescent="0.2">
       <c r="F18" s="1" t="s">
-        <v>130</v>
+        <v>124</v>
       </c>
       <c r="G18" s="9" t="s">
-        <v>132</v>
+        <v>126</v>
       </c>
     </row>
     <row r="23" spans="2:7" x14ac:dyDescent="0.2">
@@ -8109,34 +8255,34 @@
         <v>25</v>
       </c>
       <c r="B2" s="12" t="s">
-        <v>111</v>
+        <v>105</v>
       </c>
       <c r="C2" s="12" t="s">
-        <v>112</v>
+        <v>106</v>
       </c>
       <c r="D2" s="12" t="s">
+        <v>107</v>
+      </c>
+      <c r="E2" s="12" t="s">
+        <v>108</v>
+      </c>
+      <c r="F2" s="32" t="s">
+        <v>110</v>
+      </c>
+      <c r="G2" s="33" t="s">
+        <v>115</v>
+      </c>
+      <c r="H2" s="32" t="s">
         <v>113</v>
       </c>
-      <c r="E2" s="12" t="s">
+      <c r="I2" s="32" t="s">
         <v>114</v>
       </c>
-      <c r="F2" s="32" t="s">
-        <v>116</v>
-      </c>
-      <c r="G2" s="33" t="s">
-        <v>121</v>
-      </c>
-      <c r="H2" s="32" t="s">
-        <v>119</v>
-      </c>
-      <c r="I2" s="32" t="s">
-        <v>120</v>
-      </c>
       <c r="J2" s="33" t="s">
+        <v>103</v>
+      </c>
+      <c r="K2" s="33" t="s">
         <v>109</v>
-      </c>
-      <c r="K2" s="33" t="s">
-        <v>115</v>
       </c>
     </row>
     <row r="3" spans="1:11" x14ac:dyDescent="0.2">
@@ -8395,7 +8541,7 @@
       <c r="K19" s="3"/>
       <c r="M19" s="31"/>
       <c r="N19" s="9" t="s">
-        <v>118</v>
+        <v>112</v>
       </c>
     </row>
     <row r="20" spans="1:14" x14ac:dyDescent="0.2">
@@ -8414,7 +8560,7 @@
       <c r="K20" s="3"/>
       <c r="M20" s="34"/>
       <c r="N20" s="9" t="s">
-        <v>117</v>
+        <v>111</v>
       </c>
     </row>
     <row r="21" spans="1:14" x14ac:dyDescent="0.2">
@@ -8475,56 +8621,56 @@
   </cols>
   <sheetData>
     <row r="2" spans="2:18" x14ac:dyDescent="0.2">
-      <c r="B2" s="53" t="s">
-        <v>149</v>
-      </c>
-      <c r="C2" s="53"/>
-      <c r="E2" s="39" t="s">
-        <v>144</v>
-      </c>
-      <c r="F2" s="39"/>
-      <c r="H2" s="39" t="s">
-        <v>145</v>
-      </c>
-      <c r="I2" s="39"/>
-      <c r="K2" s="39" t="s">
-        <v>146</v>
-      </c>
-      <c r="L2" s="39"/>
-      <c r="N2" s="39" t="s">
-        <v>147</v>
-      </c>
-      <c r="O2" s="39"/>
-      <c r="Q2" s="39" t="s">
-        <v>148</v>
-      </c>
-      <c r="R2" s="39"/>
+      <c r="B2" s="49" t="s">
+        <v>143</v>
+      </c>
+      <c r="C2" s="49"/>
+      <c r="E2" s="45" t="s">
+        <v>138</v>
+      </c>
+      <c r="F2" s="45"/>
+      <c r="H2" s="45" t="s">
+        <v>139</v>
+      </c>
+      <c r="I2" s="45"/>
+      <c r="K2" s="45" t="s">
+        <v>140</v>
+      </c>
+      <c r="L2" s="45"/>
+      <c r="N2" s="45" t="s">
+        <v>141</v>
+      </c>
+      <c r="O2" s="45"/>
+      <c r="Q2" s="45" t="s">
+        <v>142</v>
+      </c>
+      <c r="R2" s="45"/>
     </row>
     <row r="3" spans="2:18" x14ac:dyDescent="0.2">
-      <c r="B3" s="53"/>
-      <c r="C3" s="53"/>
-      <c r="E3" s="49" t="s">
+      <c r="B3" s="49"/>
+      <c r="C3" s="49"/>
+      <c r="E3" s="38" t="s">
         <v>97</v>
       </c>
-      <c r="F3" s="50">
+      <c r="F3" s="39">
         <v>80</v>
       </c>
-      <c r="H3" s="49" t="s">
+      <c r="H3" s="38" t="s">
         <v>97</v>
       </c>
-      <c r="I3" s="50"/>
-      <c r="K3" s="49" t="s">
+      <c r="I3" s="39"/>
+      <c r="K3" s="38" t="s">
         <v>97</v>
       </c>
-      <c r="L3" s="50"/>
-      <c r="N3" s="49" t="s">
+      <c r="L3" s="39"/>
+      <c r="N3" s="38" t="s">
         <v>97</v>
       </c>
-      <c r="O3" s="50"/>
-      <c r="Q3" s="49" t="s">
+      <c r="O3" s="39"/>
+      <c r="Q3" s="38" t="s">
         <v>97</v>
       </c>
-      <c r="R3" s="50"/>
+      <c r="R3" s="39"/>
     </row>
     <row r="4" spans="2:18" x14ac:dyDescent="0.2">
       <c r="B4" s="28" t="s">
@@ -8891,56 +9037,56 @@
   </cols>
   <sheetData>
     <row r="2" spans="2:18" x14ac:dyDescent="0.2">
-      <c r="B2" s="54" t="s">
-        <v>151</v>
-      </c>
-      <c r="C2" s="54"/>
-      <c r="E2" s="40" t="s">
-        <v>150</v>
-      </c>
-      <c r="F2" s="40"/>
-      <c r="H2" s="40" t="s">
-        <v>152</v>
-      </c>
-      <c r="I2" s="40"/>
-      <c r="K2" s="40" t="s">
-        <v>153</v>
-      </c>
-      <c r="L2" s="40"/>
-      <c r="N2" s="40" t="s">
-        <v>154</v>
-      </c>
-      <c r="O2" s="40"/>
-      <c r="Q2" s="40" t="s">
-        <v>155</v>
-      </c>
-      <c r="R2" s="40"/>
+      <c r="B2" s="50" t="s">
+        <v>145</v>
+      </c>
+      <c r="C2" s="50"/>
+      <c r="E2" s="46" t="s">
+        <v>144</v>
+      </c>
+      <c r="F2" s="46"/>
+      <c r="H2" s="46" t="s">
+        <v>146</v>
+      </c>
+      <c r="I2" s="46"/>
+      <c r="K2" s="46" t="s">
+        <v>147</v>
+      </c>
+      <c r="L2" s="46"/>
+      <c r="N2" s="46" t="s">
+        <v>148</v>
+      </c>
+      <c r="O2" s="46"/>
+      <c r="Q2" s="46" t="s">
+        <v>149</v>
+      </c>
+      <c r="R2" s="46"/>
     </row>
     <row r="3" spans="2:18" x14ac:dyDescent="0.2">
-      <c r="B3" s="54"/>
-      <c r="C3" s="54"/>
-      <c r="E3" s="51" t="s">
+      <c r="B3" s="50"/>
+      <c r="C3" s="50"/>
+      <c r="E3" s="40" t="s">
         <v>97</v>
       </c>
-      <c r="F3" s="52">
+      <c r="F3" s="41">
         <v>80</v>
       </c>
-      <c r="H3" s="51" t="s">
+      <c r="H3" s="40" t="s">
         <v>97</v>
       </c>
-      <c r="I3" s="52"/>
-      <c r="K3" s="51" t="s">
+      <c r="I3" s="41"/>
+      <c r="K3" s="40" t="s">
         <v>97</v>
       </c>
-      <c r="L3" s="52"/>
-      <c r="N3" s="51" t="s">
+      <c r="L3" s="41"/>
+      <c r="N3" s="40" t="s">
         <v>97</v>
       </c>
-      <c r="O3" s="52"/>
-      <c r="Q3" s="51" t="s">
+      <c r="O3" s="41"/>
+      <c r="Q3" s="40" t="s">
         <v>97</v>
       </c>
-      <c r="R3" s="52"/>
+      <c r="R3" s="41"/>
     </row>
     <row r="4" spans="2:18" x14ac:dyDescent="0.2">
       <c r="B4" s="28" t="s">
@@ -9282,12 +9428,12 @@
     </row>
   </sheetData>
   <mergeCells count="6">
+    <mergeCell ref="Q2:R2"/>
     <mergeCell ref="B2:C3"/>
     <mergeCell ref="E2:F2"/>
     <mergeCell ref="H2:I2"/>
     <mergeCell ref="K2:L2"/>
     <mergeCell ref="N2:O2"/>
-    <mergeCell ref="Q2:R2"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
@@ -9341,172 +9487,172 @@
       </c>
     </row>
     <row r="4" spans="1:44" x14ac:dyDescent="0.2">
-      <c r="A4" s="36" t="s">
+      <c r="A4" s="43" t="s">
         <v>2</v>
       </c>
-      <c r="B4" s="36"/>
-      <c r="D4" s="36" t="s">
+      <c r="B4" s="43"/>
+      <c r="D4" s="43" t="s">
         <v>5</v>
       </c>
-      <c r="E4" s="36"/>
-      <c r="G4" s="36" t="s">
+      <c r="E4" s="43"/>
+      <c r="G4" s="43" t="s">
         <v>6</v>
       </c>
-      <c r="H4" s="36"/>
-      <c r="J4" s="36" t="s">
+      <c r="H4" s="43"/>
+      <c r="J4" s="43" t="s">
         <v>7</v>
       </c>
-      <c r="K4" s="36"/>
-      <c r="M4" s="36" t="s">
+      <c r="K4" s="43"/>
+      <c r="M4" s="43" t="s">
         <v>8</v>
       </c>
-      <c r="N4" s="36"/>
-      <c r="P4" s="36" t="s">
+      <c r="N4" s="43"/>
+      <c r="P4" s="43" t="s">
         <v>9</v>
       </c>
-      <c r="Q4" s="36"/>
+      <c r="Q4" s="43"/>
       <c r="R4" s="1"/>
-      <c r="S4" s="36" t="s">
+      <c r="S4" s="43" t="s">
         <v>10</v>
       </c>
-      <c r="T4" s="36"/>
+      <c r="T4" s="43"/>
       <c r="U4" s="1"/>
-      <c r="V4" s="36" t="s">
+      <c r="V4" s="43" t="s">
         <v>11</v>
       </c>
-      <c r="W4" s="36"/>
+      <c r="W4" s="43"/>
       <c r="X4" s="1"/>
-      <c r="Y4" s="36" t="s">
+      <c r="Y4" s="43" t="s">
         <v>12</v>
       </c>
-      <c r="Z4" s="36"/>
+      <c r="Z4" s="43"/>
       <c r="AA4" s="1"/>
-      <c r="AB4" s="36" t="s">
+      <c r="AB4" s="43" t="s">
         <v>13</v>
       </c>
-      <c r="AC4" s="36"/>
-      <c r="AE4" s="36" t="s">
-        <v>122</v>
-      </c>
-      <c r="AF4" s="36"/>
+      <c r="AC4" s="43"/>
+      <c r="AE4" s="43" t="s">
+        <v>116</v>
+      </c>
+      <c r="AF4" s="43"/>
       <c r="AG4" s="1"/>
-      <c r="AH4" s="36" t="s">
-        <v>123</v>
-      </c>
-      <c r="AI4" s="36"/>
+      <c r="AH4" s="43" t="s">
+        <v>117</v>
+      </c>
+      <c r="AI4" s="43"/>
       <c r="AJ4" s="1"/>
-      <c r="AK4" s="36" t="s">
-        <v>124</v>
-      </c>
-      <c r="AL4" s="36"/>
+      <c r="AK4" s="43" t="s">
+        <v>118</v>
+      </c>
+      <c r="AL4" s="43"/>
       <c r="AM4" s="1"/>
-      <c r="AN4" s="36" t="s">
-        <v>125</v>
-      </c>
-      <c r="AO4" s="36"/>
+      <c r="AN4" s="43" t="s">
+        <v>119</v>
+      </c>
+      <c r="AO4" s="43"/>
       <c r="AP4" s="1"/>
-      <c r="AQ4" s="36" t="s">
-        <v>126</v>
-      </c>
-      <c r="AR4" s="36"/>
+      <c r="AQ4" s="43" t="s">
+        <v>120</v>
+      </c>
+      <c r="AR4" s="43"/>
     </row>
     <row r="5" spans="1:44" x14ac:dyDescent="0.2">
-      <c r="A5" s="45" t="s">
-        <v>134</v>
-      </c>
-      <c r="B5" s="45">
+      <c r="A5" s="37" t="s">
+        <v>128</v>
+      </c>
+      <c r="B5" s="37">
         <v>1</v>
       </c>
-      <c r="D5" s="45" t="s">
-        <v>134</v>
-      </c>
-      <c r="E5" s="45">
+      <c r="D5" s="37" t="s">
+        <v>128</v>
+      </c>
+      <c r="E5" s="37">
         <v>2</v>
       </c>
-      <c r="G5" s="45" t="s">
-        <v>134</v>
-      </c>
-      <c r="H5" s="45">
+      <c r="G5" s="37" t="s">
+        <v>128</v>
+      </c>
+      <c r="H5" s="37">
         <v>3</v>
       </c>
-      <c r="J5" s="45" t="s">
-        <v>134</v>
-      </c>
-      <c r="K5" s="45">
+      <c r="J5" s="37" t="s">
+        <v>128</v>
+      </c>
+      <c r="K5" s="37">
         <v>4</v>
       </c>
-      <c r="M5" s="45" t="s">
-        <v>134</v>
-      </c>
-      <c r="N5" s="45">
+      <c r="M5" s="37" t="s">
+        <v>128</v>
+      </c>
+      <c r="N5" s="37">
         <v>5</v>
       </c>
-      <c r="P5" s="45" t="s">
-        <v>134</v>
-      </c>
-      <c r="Q5" s="45">
+      <c r="P5" s="37" t="s">
+        <v>128</v>
+      </c>
+      <c r="Q5" s="37">
         <v>6</v>
       </c>
       <c r="R5" s="1"/>
-      <c r="S5" s="45" t="s">
-        <v>134</v>
-      </c>
-      <c r="T5" s="45">
+      <c r="S5" s="37" t="s">
+        <v>128</v>
+      </c>
+      <c r="T5" s="37">
         <v>7</v>
       </c>
       <c r="U5" s="1"/>
-      <c r="V5" s="45" t="s">
-        <v>134</v>
-      </c>
-      <c r="W5" s="45">
+      <c r="V5" s="37" t="s">
+        <v>128</v>
+      </c>
+      <c r="W5" s="37">
         <v>8</v>
       </c>
       <c r="X5" s="1"/>
-      <c r="Y5" s="45" t="s">
-        <v>134</v>
-      </c>
-      <c r="Z5" s="45">
+      <c r="Y5" s="37" t="s">
+        <v>128</v>
+      </c>
+      <c r="Z5" s="37">
         <v>9</v>
       </c>
       <c r="AA5" s="1"/>
-      <c r="AB5" s="45" t="s">
-        <v>134</v>
-      </c>
-      <c r="AC5" s="45">
+      <c r="AB5" s="37" t="s">
+        <v>128</v>
+      </c>
+      <c r="AC5" s="37">
         <v>10</v>
       </c>
-      <c r="AE5" s="45" t="s">
-        <v>134</v>
-      </c>
-      <c r="AF5" s="45">
+      <c r="AE5" s="37" t="s">
+        <v>128</v>
+      </c>
+      <c r="AF5" s="37">
         <v>11</v>
       </c>
       <c r="AG5" s="1"/>
-      <c r="AH5" s="45" t="s">
-        <v>134</v>
-      </c>
-      <c r="AI5" s="45">
+      <c r="AH5" s="37" t="s">
+        <v>128</v>
+      </c>
+      <c r="AI5" s="37">
         <v>12</v>
       </c>
       <c r="AJ5" s="1"/>
-      <c r="AK5" s="45" t="s">
-        <v>134</v>
-      </c>
-      <c r="AL5" s="45">
+      <c r="AK5" s="37" t="s">
+        <v>128</v>
+      </c>
+      <c r="AL5" s="37">
         <v>13</v>
       </c>
       <c r="AM5" s="1"/>
-      <c r="AN5" s="45" t="s">
-        <v>134</v>
-      </c>
-      <c r="AO5" s="45">
+      <c r="AN5" s="37" t="s">
+        <v>128</v>
+      </c>
+      <c r="AO5" s="37">
         <v>14</v>
       </c>
       <c r="AP5" s="1"/>
-      <c r="AQ5" s="45" t="s">
-        <v>134</v>
-      </c>
-      <c r="AR5" s="45">
+      <c r="AQ5" s="37" t="s">
+        <v>128</v>
+      </c>
+      <c r="AR5" s="37">
         <v>15</v>
       </c>
     </row>
@@ -10444,21 +10590,21 @@
     </row>
   </sheetData>
   <mergeCells count="15">
+    <mergeCell ref="A4:B4"/>
+    <mergeCell ref="D4:E4"/>
+    <mergeCell ref="G4:H4"/>
+    <mergeCell ref="J4:K4"/>
+    <mergeCell ref="M4:N4"/>
+    <mergeCell ref="P4:Q4"/>
+    <mergeCell ref="S4:T4"/>
+    <mergeCell ref="V4:W4"/>
+    <mergeCell ref="Y4:Z4"/>
+    <mergeCell ref="AB4:AC4"/>
     <mergeCell ref="AE4:AF4"/>
     <mergeCell ref="AH4:AI4"/>
     <mergeCell ref="AK4:AL4"/>
     <mergeCell ref="AN4:AO4"/>
     <mergeCell ref="AQ4:AR4"/>
-    <mergeCell ref="P4:Q4"/>
-    <mergeCell ref="S4:T4"/>
-    <mergeCell ref="V4:W4"/>
-    <mergeCell ref="Y4:Z4"/>
-    <mergeCell ref="AB4:AC4"/>
-    <mergeCell ref="A4:B4"/>
-    <mergeCell ref="D4:E4"/>
-    <mergeCell ref="G4:H4"/>
-    <mergeCell ref="J4:K4"/>
-    <mergeCell ref="M4:N4"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
@@ -10487,9 +10633,7 @@
       <c r="J2" s="6" t="s">
         <v>87</v>
       </c>
-      <c r="O2" s="6" t="s">
-        <v>102</v>
-      </c>
+      <c r="O2" s="6"/>
     </row>
     <row r="3" spans="1:24" x14ac:dyDescent="0.2">
       <c r="C3" s="1" t="s">
@@ -10506,18 +10650,12 @@
       <c r="K3" t="s">
         <v>59</v>
       </c>
-      <c r="O3" s="14" t="s">
-        <v>103</v>
-      </c>
-      <c r="P3" s="38" t="s">
-        <v>106</v>
-      </c>
-      <c r="Q3" s="38"/>
-      <c r="R3" s="38"/>
-      <c r="S3" s="38"/>
-      <c r="T3" s="38"/>
-      <c r="U3" s="46"/>
-      <c r="V3" s="46"/>
+      <c r="O3" s="14"/>
+      <c r="P3" s="51"/>
+      <c r="Q3" s="51"/>
+      <c r="R3" s="51"/>
+      <c r="S3" s="51"/>
+      <c r="T3" s="51"/>
     </row>
     <row r="4" spans="1:24" x14ac:dyDescent="0.2">
       <c r="C4" s="1" t="s">
@@ -10534,18 +10672,12 @@
       <c r="K4" t="s">
         <v>60</v>
       </c>
-      <c r="O4" s="14" t="s">
-        <v>105</v>
-      </c>
-      <c r="P4" s="38" t="s">
-        <v>107</v>
-      </c>
-      <c r="Q4" s="38"/>
-      <c r="R4" s="38"/>
-      <c r="S4" s="38"/>
-      <c r="T4" s="38"/>
-      <c r="U4" s="46"/>
-      <c r="V4" s="46"/>
+      <c r="O4" s="14"/>
+      <c r="P4" s="51"/>
+      <c r="Q4" s="51"/>
+      <c r="R4" s="51"/>
+      <c r="S4" s="51"/>
+      <c r="T4" s="51"/>
     </row>
     <row r="5" spans="1:24" x14ac:dyDescent="0.2">
       <c r="J5" s="1" t="s">
@@ -10554,16 +10686,12 @@
       <c r="K5" s="9" t="s">
         <v>89</v>
       </c>
-      <c r="O5" s="14" t="s">
-        <v>104</v>
-      </c>
-      <c r="P5" s="38"/>
-      <c r="Q5" s="38"/>
-      <c r="R5" s="38"/>
-      <c r="S5" s="38"/>
-      <c r="T5" s="38"/>
-      <c r="U5" s="46"/>
-      <c r="V5" s="46"/>
+      <c r="O5" s="14"/>
+      <c r="P5" s="51"/>
+      <c r="Q5" s="51"/>
+      <c r="R5" s="51"/>
+      <c r="S5" s="51"/>
+      <c r="T5" s="51"/>
     </row>
     <row r="6" spans="1:24" x14ac:dyDescent="0.2">
       <c r="J6" s="1"/>
@@ -10572,36 +10700,36 @@
       <c r="Q6" s="1"/>
     </row>
     <row r="7" spans="1:24" x14ac:dyDescent="0.2">
-      <c r="C7" s="37" t="s">
+      <c r="C7" s="44" t="s">
         <v>57</v>
       </c>
-      <c r="D7" s="37"/>
-      <c r="E7" s="37"/>
-      <c r="F7" s="37"/>
-      <c r="G7" s="37"/>
-      <c r="H7" s="37"/>
-      <c r="I7" s="37"/>
-      <c r="J7" s="37"/>
+      <c r="D7" s="44"/>
+      <c r="E7" s="44"/>
+      <c r="F7" s="44"/>
+      <c r="G7" s="44"/>
+      <c r="H7" s="44"/>
+      <c r="I7" s="44"/>
+      <c r="J7" s="44"/>
       <c r="K7" s="1"/>
-      <c r="L7" s="37" t="s">
+      <c r="L7" s="44" t="s">
         <v>58</v>
       </c>
-      <c r="M7" s="37"/>
-      <c r="N7" s="37"/>
-      <c r="O7" s="37"/>
-      <c r="P7" s="37"/>
-      <c r="Q7" s="37"/>
-      <c r="R7" s="37" t="s">
+      <c r="M7" s="44"/>
+      <c r="N7" s="44"/>
+      <c r="O7" s="44"/>
+      <c r="P7" s="44"/>
+      <c r="Q7" s="44"/>
+      <c r="R7" s="44" t="s">
         <v>95</v>
       </c>
-      <c r="S7" s="37"/>
-      <c r="T7" s="37"/>
-      <c r="U7" s="37"/>
-      <c r="V7" s="37"/>
-      <c r="W7" s="37" t="s">
-        <v>108</v>
-      </c>
-      <c r="X7" s="37"/>
+      <c r="S7" s="44"/>
+      <c r="T7" s="44"/>
+      <c r="U7" s="44"/>
+      <c r="V7" s="44"/>
+      <c r="W7" s="44" t="s">
+        <v>102</v>
+      </c>
+      <c r="X7" s="44"/>
     </row>
     <row r="8" spans="1:24" x14ac:dyDescent="0.2">
       <c r="A8" s="20" t="s">
@@ -10671,10 +10799,10 @@
         <v>100</v>
       </c>
       <c r="W8" s="29" t="s">
-        <v>109</v>
+        <v>103</v>
       </c>
       <c r="X8" s="30" t="s">
-        <v>110</v>
+        <v>104</v>
       </c>
     </row>
     <row r="9" spans="1:24" x14ac:dyDescent="0.2">
@@ -10682,7 +10810,7 @@
         <v>1</v>
       </c>
       <c r="B9" s="3" t="s">
-        <v>135</v>
+        <v>129</v>
       </c>
       <c r="C9" s="3">
         <v>130</v>
@@ -10736,7 +10864,7 @@
         <v>2</v>
       </c>
       <c r="B10" s="3" t="s">
-        <v>136</v>
+        <v>130</v>
       </c>
       <c r="C10" s="3">
         <v>120</v>
@@ -10790,7 +10918,7 @@
         <v>3</v>
       </c>
       <c r="B11" s="3" t="s">
-        <v>137</v>
+        <v>131</v>
       </c>
       <c r="C11" s="3">
         <v>132</v>
@@ -11175,588 +11303,315 @@
       <c r="W23" s="3"/>
       <c r="X23" s="3"/>
     </row>
-    <row r="24" spans="1:24" s="48" customFormat="1" x14ac:dyDescent="0.2">
-      <c r="A24" s="47"/>
-      <c r="B24" s="47"/>
-      <c r="C24" s="47"/>
-      <c r="D24" s="47"/>
-      <c r="E24" s="47"/>
-      <c r="F24" s="47"/>
-      <c r="G24" s="47"/>
-      <c r="H24" s="47"/>
-      <c r="I24" s="47"/>
-      <c r="J24" s="47"/>
-      <c r="K24" s="47"/>
-      <c r="L24" s="47"/>
-      <c r="M24" s="47"/>
-      <c r="N24" s="47"/>
-      <c r="O24" s="47"/>
-      <c r="P24" s="47"/>
-      <c r="Q24" s="47"/>
-      <c r="R24" s="47"/>
-      <c r="S24" s="47"/>
-      <c r="T24" s="47"/>
-      <c r="U24" s="47"/>
-      <c r="V24" s="47"/>
-      <c r="W24" s="47"/>
-    </row>
-    <row r="25" spans="1:24" s="48" customFormat="1" x14ac:dyDescent="0.2">
-      <c r="A25" s="47"/>
-      <c r="B25" s="47"/>
-      <c r="C25" s="47"/>
-      <c r="D25" s="47"/>
-      <c r="E25" s="47"/>
-      <c r="F25" s="47"/>
-      <c r="G25" s="47"/>
-      <c r="H25" s="47"/>
-      <c r="I25" s="47"/>
-      <c r="J25" s="47"/>
-      <c r="K25" s="47"/>
-      <c r="L25" s="47"/>
-      <c r="M25" s="47"/>
-      <c r="N25" s="47"/>
-      <c r="O25" s="47"/>
-      <c r="P25" s="47"/>
-      <c r="Q25" s="47"/>
-      <c r="W25" s="47"/>
-    </row>
-    <row r="26" spans="1:24" s="48" customFormat="1" x14ac:dyDescent="0.2">
-      <c r="A26" s="47"/>
-      <c r="B26" s="47"/>
-      <c r="C26" s="47"/>
-      <c r="D26" s="47"/>
-      <c r="E26" s="47"/>
-      <c r="F26" s="47"/>
-      <c r="G26" s="47"/>
-      <c r="H26" s="47"/>
-      <c r="I26" s="47"/>
-      <c r="J26" s="47"/>
-      <c r="K26" s="47"/>
-      <c r="L26" s="47"/>
-      <c r="M26" s="47"/>
-      <c r="N26" s="47"/>
-      <c r="O26" s="47"/>
-      <c r="P26" s="47"/>
-      <c r="Q26" s="47"/>
-      <c r="W26" s="47"/>
-    </row>
-    <row r="27" spans="1:24" s="48" customFormat="1" x14ac:dyDescent="0.2">
-      <c r="A27" s="47"/>
-      <c r="B27" s="47"/>
-      <c r="C27" s="47"/>
-      <c r="D27" s="47"/>
-      <c r="E27" s="47"/>
-      <c r="F27" s="47"/>
-      <c r="G27" s="47"/>
-      <c r="H27" s="47"/>
-      <c r="I27" s="47"/>
-      <c r="J27" s="47"/>
-      <c r="K27" s="47"/>
-      <c r="L27" s="47"/>
-      <c r="M27" s="47"/>
-      <c r="N27" s="47"/>
-      <c r="O27" s="47"/>
-      <c r="P27" s="47"/>
-      <c r="Q27" s="47"/>
-      <c r="W27" s="47"/>
-    </row>
-    <row r="28" spans="1:24" s="48" customFormat="1" x14ac:dyDescent="0.2">
-      <c r="A28" s="47"/>
-      <c r="B28" s="47"/>
-      <c r="C28" s="47"/>
-      <c r="D28" s="47"/>
-      <c r="E28" s="47"/>
-      <c r="F28" s="47"/>
-      <c r="G28" s="47"/>
-      <c r="H28" s="47"/>
-      <c r="I28" s="47"/>
-      <c r="J28" s="47"/>
-      <c r="K28" s="47"/>
-      <c r="L28" s="47"/>
-      <c r="M28" s="47"/>
-      <c r="N28" s="47"/>
-      <c r="O28" s="47"/>
-      <c r="P28" s="47"/>
-      <c r="Q28" s="47"/>
-      <c r="W28" s="47"/>
-    </row>
-    <row r="29" spans="1:24" s="48" customFormat="1" x14ac:dyDescent="0.2">
-      <c r="A29" s="47"/>
-      <c r="B29" s="47"/>
-      <c r="C29" s="47"/>
-      <c r="D29" s="47"/>
-      <c r="E29" s="47"/>
-      <c r="F29" s="47"/>
-      <c r="G29" s="47"/>
-      <c r="H29" s="47"/>
-      <c r="I29" s="47"/>
-      <c r="J29" s="47"/>
-      <c r="K29" s="47"/>
-      <c r="L29" s="47"/>
-      <c r="M29" s="47"/>
-      <c r="N29" s="47"/>
-      <c r="O29" s="47"/>
-      <c r="P29" s="47"/>
-      <c r="Q29" s="47"/>
-      <c r="W29" s="47"/>
-    </row>
-    <row r="30" spans="1:24" s="48" customFormat="1" x14ac:dyDescent="0.2">
-      <c r="A30" s="47"/>
-      <c r="B30" s="47"/>
-      <c r="C30" s="47"/>
-      <c r="D30" s="47"/>
-      <c r="E30" s="47"/>
-      <c r="F30" s="47"/>
-      <c r="G30" s="47"/>
-      <c r="H30" s="47"/>
-      <c r="I30" s="47"/>
-      <c r="J30" s="47"/>
-      <c r="K30" s="47"/>
-      <c r="L30" s="47"/>
-      <c r="M30" s="47"/>
-      <c r="N30" s="47"/>
-      <c r="O30" s="47"/>
-      <c r="P30" s="47"/>
-      <c r="Q30" s="47"/>
-      <c r="W30" s="47"/>
-    </row>
-    <row r="31" spans="1:24" s="48" customFormat="1" x14ac:dyDescent="0.2">
-      <c r="A31" s="47"/>
-      <c r="B31" s="47"/>
-      <c r="C31" s="47"/>
-      <c r="D31" s="47"/>
-      <c r="E31" s="47"/>
-      <c r="F31" s="47"/>
-      <c r="G31" s="47"/>
-      <c r="H31" s="47"/>
-      <c r="I31" s="47"/>
-      <c r="J31" s="47"/>
-      <c r="K31" s="47"/>
-      <c r="L31" s="47"/>
-      <c r="M31" s="47"/>
-      <c r="N31" s="47"/>
-      <c r="O31" s="47"/>
-      <c r="P31" s="47"/>
-      <c r="Q31" s="47"/>
-      <c r="W31" s="47"/>
-    </row>
-    <row r="32" spans="1:24" s="48" customFormat="1" x14ac:dyDescent="0.2">
-      <c r="A32" s="47"/>
-      <c r="B32" s="47"/>
-      <c r="C32" s="47"/>
-      <c r="D32" s="47"/>
-      <c r="E32" s="47"/>
-      <c r="F32" s="47"/>
-      <c r="G32" s="47"/>
-      <c r="H32" s="47"/>
-      <c r="I32" s="47"/>
-      <c r="J32" s="47"/>
-      <c r="K32" s="47"/>
-      <c r="L32" s="47"/>
-      <c r="M32" s="47"/>
-      <c r="N32" s="47"/>
-      <c r="O32" s="47"/>
-      <c r="P32" s="47"/>
-      <c r="Q32" s="47"/>
-      <c r="W32" s="47"/>
-    </row>
-    <row r="33" spans="1:23" s="48" customFormat="1" x14ac:dyDescent="0.2">
-      <c r="A33" s="47"/>
-      <c r="B33" s="47"/>
-      <c r="C33" s="47"/>
-      <c r="D33" s="47"/>
-      <c r="E33" s="47"/>
-      <c r="F33" s="47"/>
-      <c r="G33" s="47"/>
-      <c r="H33" s="47"/>
-      <c r="I33" s="47"/>
-      <c r="J33" s="47"/>
-      <c r="K33" s="47"/>
-      <c r="L33" s="47"/>
-      <c r="M33" s="47"/>
-      <c r="N33" s="47"/>
-      <c r="O33" s="47"/>
-      <c r="P33" s="47"/>
-      <c r="Q33" s="47"/>
-      <c r="W33" s="47"/>
-    </row>
-    <row r="34" spans="1:23" s="48" customFormat="1" x14ac:dyDescent="0.2">
-      <c r="A34" s="47"/>
-      <c r="B34" s="47"/>
-      <c r="C34" s="47"/>
-      <c r="D34" s="47"/>
-      <c r="E34" s="47"/>
-      <c r="F34" s="47"/>
-      <c r="G34" s="47"/>
-      <c r="H34" s="47"/>
-      <c r="I34" s="47"/>
-      <c r="J34" s="47"/>
-      <c r="K34" s="47"/>
-      <c r="L34" s="47"/>
-      <c r="M34" s="47"/>
-      <c r="N34" s="47"/>
-      <c r="O34" s="47"/>
-      <c r="P34" s="47"/>
-      <c r="Q34" s="47"/>
-      <c r="W34" s="47"/>
-    </row>
-    <row r="35" spans="1:23" s="48" customFormat="1" x14ac:dyDescent="0.2">
-      <c r="A35" s="47"/>
-      <c r="B35" s="47"/>
-      <c r="C35" s="47"/>
-      <c r="D35" s="47"/>
-      <c r="E35" s="47"/>
-      <c r="F35" s="47"/>
-      <c r="G35" s="47"/>
-      <c r="H35" s="47"/>
-      <c r="I35" s="47"/>
-      <c r="J35" s="47"/>
-      <c r="K35" s="47"/>
-      <c r="L35" s="47"/>
-      <c r="M35" s="47"/>
-      <c r="N35" s="47"/>
-      <c r="O35" s="47"/>
-      <c r="P35" s="47"/>
-      <c r="Q35" s="47"/>
-      <c r="W35" s="47"/>
-    </row>
-    <row r="36" spans="1:23" s="48" customFormat="1" x14ac:dyDescent="0.2">
-      <c r="A36" s="47"/>
-      <c r="B36" s="47"/>
-      <c r="C36" s="47"/>
-      <c r="D36" s="47"/>
-      <c r="E36" s="47"/>
-      <c r="F36" s="47"/>
-      <c r="G36" s="47"/>
-      <c r="H36" s="47"/>
-      <c r="I36" s="47"/>
-      <c r="J36" s="47"/>
-      <c r="K36" s="47"/>
-      <c r="L36" s="47"/>
-      <c r="M36" s="47"/>
-      <c r="N36" s="47"/>
-      <c r="O36" s="47"/>
-      <c r="P36" s="47"/>
-      <c r="Q36" s="47"/>
-      <c r="W36" s="47"/>
-    </row>
-    <row r="37" spans="1:23" s="48" customFormat="1" x14ac:dyDescent="0.2">
-      <c r="A37" s="47"/>
-      <c r="B37" s="47"/>
-      <c r="C37" s="47"/>
-      <c r="D37" s="47"/>
-      <c r="E37" s="47"/>
-      <c r="F37" s="47"/>
-      <c r="G37" s="47"/>
-      <c r="H37" s="47"/>
-      <c r="I37" s="47"/>
-      <c r="J37" s="47"/>
-      <c r="K37" s="47"/>
-      <c r="L37" s="47"/>
-      <c r="M37" s="47"/>
-      <c r="N37" s="47"/>
-      <c r="O37" s="47"/>
-      <c r="P37" s="47"/>
-      <c r="Q37" s="47"/>
-      <c r="W37" s="47"/>
-    </row>
-    <row r="38" spans="1:23" s="48" customFormat="1" x14ac:dyDescent="0.2">
-      <c r="A38" s="47"/>
-      <c r="B38" s="47"/>
-      <c r="C38" s="47"/>
-      <c r="D38" s="47"/>
-      <c r="E38" s="47"/>
-      <c r="F38" s="47"/>
-      <c r="G38" s="47"/>
-      <c r="H38" s="47"/>
-      <c r="I38" s="47"/>
-      <c r="J38" s="47"/>
-      <c r="K38" s="47"/>
-      <c r="L38" s="47"/>
-      <c r="M38" s="47"/>
-      <c r="N38" s="47"/>
-      <c r="O38" s="47"/>
-      <c r="P38" s="47"/>
-      <c r="Q38" s="47"/>
-      <c r="W38" s="47"/>
-    </row>
-    <row r="39" spans="1:23" s="48" customFormat="1" x14ac:dyDescent="0.2">
-      <c r="A39" s="47"/>
-      <c r="B39" s="47"/>
-      <c r="C39" s="47"/>
-      <c r="D39" s="47"/>
-      <c r="E39" s="47"/>
-      <c r="F39" s="47"/>
-      <c r="G39" s="47"/>
-      <c r="H39" s="47"/>
-      <c r="I39" s="47"/>
-      <c r="J39" s="47"/>
-      <c r="K39" s="47"/>
-      <c r="L39" s="47"/>
-      <c r="M39" s="47"/>
-      <c r="N39" s="47"/>
-      <c r="O39" s="47"/>
-      <c r="P39" s="47"/>
-      <c r="Q39" s="47"/>
-      <c r="W39" s="47"/>
-    </row>
-    <row r="40" spans="1:23" s="48" customFormat="1" x14ac:dyDescent="0.2">
-      <c r="A40" s="47"/>
-      <c r="B40" s="47"/>
-      <c r="C40" s="47"/>
-      <c r="D40" s="47"/>
-      <c r="E40" s="47"/>
-      <c r="F40" s="47"/>
-      <c r="G40" s="47"/>
-      <c r="H40" s="47"/>
-      <c r="I40" s="47"/>
-      <c r="J40" s="47"/>
-      <c r="K40" s="47"/>
-      <c r="L40" s="47"/>
-      <c r="M40" s="47"/>
-      <c r="N40" s="47"/>
-      <c r="O40" s="47"/>
-      <c r="P40" s="47"/>
-      <c r="Q40" s="47"/>
-      <c r="W40" s="47"/>
-    </row>
-    <row r="41" spans="1:23" s="48" customFormat="1" x14ac:dyDescent="0.2">
-      <c r="A41" s="47"/>
-      <c r="B41" s="47"/>
-      <c r="C41" s="47"/>
-      <c r="D41" s="47"/>
-      <c r="E41" s="47"/>
-      <c r="F41" s="47"/>
-      <c r="G41" s="47"/>
-      <c r="H41" s="47"/>
-      <c r="I41" s="47"/>
-      <c r="J41" s="47"/>
-      <c r="K41" s="47"/>
-      <c r="L41" s="47"/>
-      <c r="M41" s="47"/>
-      <c r="N41" s="47"/>
-      <c r="O41" s="47"/>
-      <c r="P41" s="47"/>
-      <c r="Q41" s="47"/>
-      <c r="W41" s="47"/>
-    </row>
-    <row r="42" spans="1:23" s="48" customFormat="1" x14ac:dyDescent="0.2">
-      <c r="A42" s="47"/>
-      <c r="B42" s="47"/>
-      <c r="C42" s="47"/>
-      <c r="D42" s="47"/>
-      <c r="E42" s="47"/>
-      <c r="F42" s="47"/>
-      <c r="G42" s="47"/>
-      <c r="H42" s="47"/>
-      <c r="I42" s="47"/>
-      <c r="J42" s="47"/>
-      <c r="K42" s="47"/>
-      <c r="L42" s="47"/>
-      <c r="M42" s="47"/>
-      <c r="N42" s="47"/>
-      <c r="O42" s="47"/>
-      <c r="P42" s="47"/>
-      <c r="Q42" s="47"/>
-      <c r="W42" s="47"/>
-    </row>
-    <row r="43" spans="1:23" s="48" customFormat="1" x14ac:dyDescent="0.2">
-      <c r="A43" s="47"/>
-      <c r="B43" s="47"/>
-      <c r="C43" s="47"/>
-      <c r="D43" s="47"/>
-      <c r="E43" s="47"/>
-      <c r="F43" s="47"/>
-      <c r="G43" s="47"/>
-      <c r="H43" s="47"/>
-      <c r="I43" s="47"/>
-      <c r="J43" s="47"/>
-      <c r="K43" s="47"/>
-      <c r="L43" s="47"/>
-      <c r="M43" s="47"/>
-      <c r="N43" s="47"/>
-      <c r="O43" s="47"/>
-      <c r="P43" s="47"/>
-      <c r="Q43" s="47"/>
-      <c r="W43" s="47"/>
-    </row>
-    <row r="44" spans="1:23" s="48" customFormat="1" x14ac:dyDescent="0.2">
-      <c r="A44" s="47"/>
-      <c r="B44" s="47"/>
-      <c r="C44" s="47"/>
-      <c r="D44" s="47"/>
-      <c r="E44" s="47"/>
-      <c r="F44" s="47"/>
-      <c r="G44" s="47"/>
-      <c r="H44" s="47"/>
-      <c r="I44" s="47"/>
-      <c r="J44" s="47"/>
-      <c r="K44" s="47"/>
-      <c r="L44" s="47"/>
-      <c r="M44" s="47"/>
-      <c r="N44" s="47"/>
-      <c r="O44" s="47"/>
-      <c r="P44" s="47"/>
-      <c r="Q44" s="47"/>
-      <c r="W44" s="47"/>
-    </row>
-    <row r="45" spans="1:23" s="48" customFormat="1" x14ac:dyDescent="0.2">
-      <c r="A45" s="47"/>
-      <c r="B45" s="47"/>
-      <c r="C45" s="47"/>
-      <c r="D45" s="47"/>
-      <c r="E45" s="47"/>
-      <c r="F45" s="47"/>
-      <c r="G45" s="47"/>
-      <c r="H45" s="47"/>
-      <c r="I45" s="47"/>
-      <c r="J45" s="47"/>
-      <c r="K45" s="47"/>
-      <c r="L45" s="47"/>
-      <c r="M45" s="47"/>
-      <c r="N45" s="47"/>
-      <c r="O45" s="47"/>
-      <c r="P45" s="47"/>
-      <c r="Q45" s="47"/>
-      <c r="W45" s="47"/>
-    </row>
-    <row r="46" spans="1:23" s="48" customFormat="1" x14ac:dyDescent="0.2">
-      <c r="A46" s="47"/>
-      <c r="B46" s="47"/>
-      <c r="C46" s="47"/>
-      <c r="D46" s="47"/>
-      <c r="E46" s="47"/>
-      <c r="F46" s="47"/>
-      <c r="G46" s="47"/>
-      <c r="H46" s="47"/>
-      <c r="I46" s="47"/>
-      <c r="J46" s="47"/>
-      <c r="K46" s="47"/>
-      <c r="L46" s="47"/>
-      <c r="M46" s="47"/>
-      <c r="N46" s="47"/>
-      <c r="O46" s="47"/>
-      <c r="P46" s="47"/>
-      <c r="Q46" s="47"/>
-      <c r="W46" s="47"/>
-    </row>
-    <row r="47" spans="1:23" s="48" customFormat="1" x14ac:dyDescent="0.2">
-      <c r="A47" s="47"/>
-      <c r="B47" s="47"/>
-      <c r="C47" s="47"/>
-      <c r="D47" s="47"/>
-      <c r="E47" s="47"/>
-      <c r="F47" s="47"/>
-      <c r="G47" s="47"/>
-      <c r="H47" s="47"/>
-      <c r="I47" s="47"/>
-      <c r="J47" s="47"/>
-      <c r="K47" s="47"/>
-      <c r="L47" s="47"/>
-      <c r="M47" s="47"/>
-      <c r="N47" s="47"/>
-      <c r="O47" s="47"/>
-      <c r="P47" s="47"/>
-      <c r="Q47" s="47"/>
-      <c r="W47" s="47"/>
-    </row>
-    <row r="48" spans="1:23" s="48" customFormat="1" x14ac:dyDescent="0.2">
-      <c r="A48" s="47"/>
-      <c r="B48" s="47"/>
-      <c r="C48" s="47"/>
-      <c r="D48" s="47"/>
-      <c r="E48" s="47"/>
-      <c r="F48" s="47"/>
-      <c r="G48" s="47"/>
-      <c r="H48" s="47"/>
-      <c r="I48" s="47"/>
-      <c r="J48" s="47"/>
-      <c r="K48" s="47"/>
-      <c r="L48" s="47"/>
-      <c r="M48" s="47"/>
-      <c r="N48" s="47"/>
-      <c r="O48" s="47"/>
-      <c r="P48" s="47"/>
-      <c r="Q48" s="47"/>
-      <c r="W48" s="47"/>
-    </row>
-    <row r="49" spans="1:23" s="48" customFormat="1" x14ac:dyDescent="0.2">
-      <c r="A49" s="47"/>
-      <c r="B49" s="47"/>
-      <c r="C49" s="47"/>
-      <c r="D49" s="47"/>
-      <c r="E49" s="47"/>
-      <c r="F49" s="47"/>
-      <c r="G49" s="47"/>
-      <c r="H49" s="47"/>
-      <c r="I49" s="47"/>
-      <c r="J49" s="47"/>
-      <c r="K49" s="47"/>
-      <c r="L49" s="47"/>
-      <c r="M49" s="47"/>
-      <c r="N49" s="47"/>
-      <c r="O49" s="47"/>
-      <c r="P49" s="47"/>
-      <c r="Q49" s="47"/>
-      <c r="W49" s="47"/>
-    </row>
-    <row r="50" spans="1:23" s="48" customFormat="1" x14ac:dyDescent="0.2">
-      <c r="A50" s="47"/>
-      <c r="B50" s="47"/>
-      <c r="C50" s="47"/>
-      <c r="D50" s="47"/>
-      <c r="E50" s="47"/>
-      <c r="F50" s="47"/>
-      <c r="G50" s="47"/>
-      <c r="H50" s="47"/>
-      <c r="I50" s="47"/>
-      <c r="J50" s="47"/>
-      <c r="K50" s="47"/>
-      <c r="L50" s="47"/>
-      <c r="M50" s="47"/>
-      <c r="N50" s="47"/>
-      <c r="O50" s="47"/>
-      <c r="P50" s="47"/>
-      <c r="Q50" s="47"/>
-      <c r="W50" s="47"/>
+    <row r="24" spans="1:24" x14ac:dyDescent="0.2">
+      <c r="J24" s="1"/>
+      <c r="K24" s="1"/>
+      <c r="L24" s="1"/>
+      <c r="M24" s="1"/>
+      <c r="N24" s="1"/>
+      <c r="O24" s="1"/>
+      <c r="P24" s="1"/>
+      <c r="Q24" s="1"/>
+      <c r="R24" s="1"/>
+      <c r="S24" s="1"/>
+      <c r="T24" s="1"/>
+      <c r="U24" s="1"/>
+      <c r="V24" s="1"/>
+    </row>
+    <row r="25" spans="1:24" x14ac:dyDescent="0.2">
+      <c r="J25" s="1"/>
+      <c r="K25" s="1"/>
+      <c r="L25" s="1"/>
+      <c r="M25" s="1"/>
+      <c r="N25" s="1"/>
+      <c r="O25" s="1"/>
+      <c r="P25" s="1"/>
+      <c r="Q25" s="1"/>
+    </row>
+    <row r="26" spans="1:24" x14ac:dyDescent="0.2">
+      <c r="J26" s="1"/>
+      <c r="K26" s="1"/>
+      <c r="L26" s="1"/>
+      <c r="M26" s="1"/>
+      <c r="N26" s="1"/>
+      <c r="O26" s="1"/>
+      <c r="P26" s="1"/>
+      <c r="Q26" s="1"/>
+    </row>
+    <row r="27" spans="1:24" x14ac:dyDescent="0.2">
+      <c r="J27" s="1"/>
+      <c r="K27" s="1"/>
+      <c r="L27" s="1"/>
+      <c r="M27" s="1"/>
+      <c r="N27" s="1"/>
+      <c r="O27" s="1"/>
+      <c r="P27" s="1"/>
+      <c r="Q27" s="1"/>
+    </row>
+    <row r="28" spans="1:24" x14ac:dyDescent="0.2">
+      <c r="J28" s="1"/>
+      <c r="K28" s="1"/>
+      <c r="L28" s="1"/>
+      <c r="M28" s="1"/>
+      <c r="N28" s="1"/>
+      <c r="O28" s="1"/>
+      <c r="P28" s="1"/>
+      <c r="Q28" s="1"/>
+    </row>
+    <row r="29" spans="1:24" x14ac:dyDescent="0.2">
+      <c r="J29" s="1"/>
+      <c r="K29" s="1"/>
+      <c r="L29" s="1"/>
+      <c r="M29" s="1"/>
+      <c r="N29" s="1"/>
+      <c r="O29" s="1"/>
+      <c r="P29" s="1"/>
+      <c r="Q29" s="1"/>
+    </row>
+    <row r="30" spans="1:24" x14ac:dyDescent="0.2">
+      <c r="J30" s="1"/>
+      <c r="K30" s="1"/>
+      <c r="L30" s="1"/>
+      <c r="M30" s="1"/>
+      <c r="N30" s="1"/>
+      <c r="O30" s="1"/>
+      <c r="P30" s="1"/>
+      <c r="Q30" s="1"/>
+    </row>
+    <row r="31" spans="1:24" x14ac:dyDescent="0.2">
+      <c r="J31" s="1"/>
+      <c r="K31" s="1"/>
+      <c r="L31" s="1"/>
+      <c r="M31" s="1"/>
+      <c r="N31" s="1"/>
+      <c r="O31" s="1"/>
+      <c r="P31" s="1"/>
+      <c r="Q31" s="1"/>
+    </row>
+    <row r="32" spans="1:24" x14ac:dyDescent="0.2">
+      <c r="J32" s="1"/>
+      <c r="K32" s="1"/>
+      <c r="L32" s="1"/>
+      <c r="M32" s="1"/>
+      <c r="N32" s="1"/>
+      <c r="O32" s="1"/>
+      <c r="P32" s="1"/>
+      <c r="Q32" s="1"/>
+    </row>
+    <row r="33" spans="10:17" x14ac:dyDescent="0.2">
+      <c r="J33" s="1"/>
+      <c r="K33" s="1"/>
+      <c r="L33" s="1"/>
+      <c r="M33" s="1"/>
+      <c r="N33" s="1"/>
+      <c r="O33" s="1"/>
+      <c r="P33" s="1"/>
+      <c r="Q33" s="1"/>
+    </row>
+    <row r="34" spans="10:17" x14ac:dyDescent="0.2">
+      <c r="J34" s="1"/>
+      <c r="K34" s="1"/>
+      <c r="L34" s="1"/>
+      <c r="M34" s="1"/>
+      <c r="N34" s="1"/>
+      <c r="O34" s="1"/>
+      <c r="P34" s="1"/>
+      <c r="Q34" s="1"/>
+    </row>
+    <row r="35" spans="10:17" x14ac:dyDescent="0.2">
+      <c r="J35" s="1"/>
+      <c r="K35" s="1"/>
+      <c r="L35" s="1"/>
+      <c r="M35" s="1"/>
+      <c r="N35" s="1"/>
+      <c r="O35" s="1"/>
+      <c r="P35" s="1"/>
+      <c r="Q35" s="1"/>
+    </row>
+    <row r="36" spans="10:17" x14ac:dyDescent="0.2">
+      <c r="J36" s="1"/>
+      <c r="K36" s="1"/>
+      <c r="L36" s="1"/>
+      <c r="M36" s="1"/>
+      <c r="N36" s="1"/>
+      <c r="O36" s="1"/>
+      <c r="P36" s="1"/>
+      <c r="Q36" s="1"/>
+    </row>
+    <row r="37" spans="10:17" x14ac:dyDescent="0.2">
+      <c r="J37" s="1"/>
+      <c r="K37" s="1"/>
+      <c r="L37" s="1"/>
+      <c r="M37" s="1"/>
+      <c r="N37" s="1"/>
+      <c r="O37" s="1"/>
+      <c r="P37" s="1"/>
+      <c r="Q37" s="1"/>
+    </row>
+    <row r="38" spans="10:17" x14ac:dyDescent="0.2">
+      <c r="J38" s="1"/>
+      <c r="K38" s="1"/>
+      <c r="L38" s="1"/>
+      <c r="M38" s="1"/>
+      <c r="N38" s="1"/>
+      <c r="O38" s="1"/>
+      <c r="P38" s="1"/>
+      <c r="Q38" s="1"/>
+    </row>
+    <row r="39" spans="10:17" x14ac:dyDescent="0.2">
+      <c r="J39" s="1"/>
+      <c r="K39" s="1"/>
+      <c r="L39" s="1"/>
+      <c r="M39" s="1"/>
+      <c r="N39" s="1"/>
+      <c r="O39" s="1"/>
+      <c r="P39" s="1"/>
+      <c r="Q39" s="1"/>
+    </row>
+    <row r="40" spans="10:17" x14ac:dyDescent="0.2">
+      <c r="J40" s="1"/>
+      <c r="K40" s="1"/>
+      <c r="L40" s="1"/>
+      <c r="M40" s="1"/>
+      <c r="N40" s="1"/>
+      <c r="O40" s="1"/>
+      <c r="P40" s="1"/>
+      <c r="Q40" s="1"/>
+    </row>
+    <row r="41" spans="10:17" x14ac:dyDescent="0.2">
+      <c r="J41" s="1"/>
+      <c r="K41" s="1"/>
+      <c r="L41" s="1"/>
+      <c r="M41" s="1"/>
+      <c r="N41" s="1"/>
+      <c r="O41" s="1"/>
+      <c r="P41" s="1"/>
+      <c r="Q41" s="1"/>
+    </row>
+    <row r="42" spans="10:17" x14ac:dyDescent="0.2">
+      <c r="J42" s="1"/>
+      <c r="K42" s="1"/>
+      <c r="L42" s="1"/>
+      <c r="M42" s="1"/>
+      <c r="N42" s="1"/>
+      <c r="O42" s="1"/>
+      <c r="P42" s="1"/>
+      <c r="Q42" s="1"/>
+    </row>
+    <row r="43" spans="10:17" x14ac:dyDescent="0.2">
+      <c r="J43" s="1"/>
+      <c r="K43" s="1"/>
+      <c r="L43" s="1"/>
+      <c r="M43" s="1"/>
+      <c r="N43" s="1"/>
+      <c r="O43" s="1"/>
+      <c r="P43" s="1"/>
+      <c r="Q43" s="1"/>
+    </row>
+    <row r="44" spans="10:17" x14ac:dyDescent="0.2">
+      <c r="J44" s="1"/>
+      <c r="K44" s="1"/>
+      <c r="L44" s="1"/>
+      <c r="M44" s="1"/>
+      <c r="N44" s="1"/>
+      <c r="O44" s="1"/>
+      <c r="P44" s="1"/>
+      <c r="Q44" s="1"/>
+    </row>
+    <row r="45" spans="10:17" x14ac:dyDescent="0.2">
+      <c r="J45" s="1"/>
+      <c r="K45" s="1"/>
+      <c r="L45" s="1"/>
+      <c r="M45" s="1"/>
+      <c r="N45" s="1"/>
+      <c r="O45" s="1"/>
+      <c r="P45" s="1"/>
+      <c r="Q45" s="1"/>
+    </row>
+    <row r="46" spans="10:17" x14ac:dyDescent="0.2">
+      <c r="J46" s="1"/>
+      <c r="K46" s="1"/>
+      <c r="L46" s="1"/>
+      <c r="M46" s="1"/>
+      <c r="N46" s="1"/>
+      <c r="O46" s="1"/>
+      <c r="P46" s="1"/>
+      <c r="Q46" s="1"/>
+    </row>
+    <row r="47" spans="10:17" x14ac:dyDescent="0.2">
+      <c r="J47" s="1"/>
+      <c r="K47" s="1"/>
+      <c r="L47" s="1"/>
+      <c r="M47" s="1"/>
+      <c r="N47" s="1"/>
+      <c r="O47" s="1"/>
+      <c r="P47" s="1"/>
+      <c r="Q47" s="1"/>
+    </row>
+    <row r="48" spans="10:17" x14ac:dyDescent="0.2">
+      <c r="J48" s="1"/>
+      <c r="K48" s="1"/>
+      <c r="L48" s="1"/>
+      <c r="M48" s="1"/>
+      <c r="N48" s="1"/>
+      <c r="O48" s="1"/>
+      <c r="P48" s="1"/>
+      <c r="Q48" s="1"/>
+    </row>
+    <row r="49" spans="10:17" x14ac:dyDescent="0.2">
+      <c r="J49" s="1"/>
+      <c r="K49" s="1"/>
+      <c r="L49" s="1"/>
+      <c r="M49" s="1"/>
+      <c r="N49" s="1"/>
+      <c r="O49" s="1"/>
+      <c r="P49" s="1"/>
+      <c r="Q49" s="1"/>
+    </row>
+    <row r="50" spans="10:17" x14ac:dyDescent="0.2">
+      <c r="J50" s="1"/>
+      <c r="K50" s="1"/>
+      <c r="L50" s="1"/>
+      <c r="M50" s="1"/>
+      <c r="N50" s="1"/>
+      <c r="O50" s="1"/>
+      <c r="P50" s="1"/>
+      <c r="Q50" s="1"/>
     </row>
   </sheetData>
-  <mergeCells count="7">
-    <mergeCell ref="P3:T3"/>
-    <mergeCell ref="P4:T4"/>
-    <mergeCell ref="P5:T5"/>
+  <mergeCells count="4">
+    <mergeCell ref="C7:J7"/>
+    <mergeCell ref="L7:Q7"/>
     <mergeCell ref="W7:X7"/>
     <mergeCell ref="R7:V7"/>
-    <mergeCell ref="C7:J7"/>
-    <mergeCell ref="L7:Q7"/>
   </mergeCells>
+  <conditionalFormatting sqref="E9:F50">
+    <cfRule type="expression" dxfId="5" priority="3">
+      <formula>$D9="cp"</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="G9:H50">
+    <cfRule type="expression" dxfId="4" priority="2">
+      <formula>$D9="mc"</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="I9:J50">
+    <cfRule type="expression" dxfId="3" priority="4">
+      <formula>$D9="cp"</formula>
+    </cfRule>
+  </conditionalFormatting>
   <conditionalFormatting sqref="M9:N50">
-    <cfRule type="expression" dxfId="7" priority="6">
+    <cfRule type="expression" dxfId="2" priority="6">
       <formula>$D9="cp"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="O9:O50">
-    <cfRule type="expression" dxfId="6" priority="13">
+    <cfRule type="expression" dxfId="1" priority="13">
       <formula>$D9="mc"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="P9:Q50">
-    <cfRule type="expression" dxfId="4" priority="8">
-      <formula>$D9="cp"</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="E9:F50">
-    <cfRule type="expression" dxfId="3" priority="3">
-      <formula>$D9="cp"</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="G9:H50">
-    <cfRule type="expression" dxfId="2" priority="2">
-      <formula>$D9="mc"</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="I9:J50">
-    <cfRule type="expression" dxfId="1" priority="4">
+    <cfRule type="expression" dxfId="0" priority="8">
       <formula>$D9="cp"</formula>
     </cfRule>
   </conditionalFormatting>
@@ -11782,14 +11637,14 @@
   </cols>
   <sheetData>
     <row r="2" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A2" s="39" t="s">
+      <c r="A2" s="45" t="s">
         <v>86</v>
       </c>
-      <c r="B2" s="39"/>
-      <c r="D2" s="40" t="s">
+      <c r="B2" s="45"/>
+      <c r="D2" s="46" t="s">
         <v>84</v>
       </c>
-      <c r="E2" s="40"/>
+      <c r="E2" s="46"/>
       <c r="G2" s="24" t="s">
         <v>85</v>
       </c>
@@ -12364,36 +12219,36 @@
   </cols>
   <sheetData>
     <row r="2" spans="2:24" x14ac:dyDescent="0.2">
-      <c r="B2" s="41" t="s">
-        <v>138</v>
-      </c>
-      <c r="C2" s="41"/>
-      <c r="D2" s="41"/>
-      <c r="F2" s="41" t="s">
-        <v>139</v>
-      </c>
-      <c r="G2" s="41"/>
-      <c r="H2" s="41"/>
-      <c r="J2" s="41" t="s">
-        <v>140</v>
-      </c>
-      <c r="K2" s="41"/>
-      <c r="L2" s="41"/>
-      <c r="N2" s="41" t="s">
-        <v>141</v>
-      </c>
-      <c r="O2" s="41"/>
-      <c r="P2" s="41"/>
-      <c r="R2" s="41" t="s">
-        <v>142</v>
-      </c>
-      <c r="S2" s="41"/>
-      <c r="T2" s="41"/>
-      <c r="V2" s="41" t="s">
-        <v>143</v>
-      </c>
-      <c r="W2" s="41"/>
-      <c r="X2" s="41"/>
+      <c r="B2" s="47" t="s">
+        <v>132</v>
+      </c>
+      <c r="C2" s="47"/>
+      <c r="D2" s="47"/>
+      <c r="F2" s="47" t="s">
+        <v>133</v>
+      </c>
+      <c r="G2" s="47"/>
+      <c r="H2" s="47"/>
+      <c r="J2" s="47" t="s">
+        <v>134</v>
+      </c>
+      <c r="K2" s="47"/>
+      <c r="L2" s="47"/>
+      <c r="N2" s="47" t="s">
+        <v>135</v>
+      </c>
+      <c r="O2" s="47"/>
+      <c r="P2" s="47"/>
+      <c r="R2" s="47" t="s">
+        <v>136</v>
+      </c>
+      <c r="S2" s="47"/>
+      <c r="T2" s="47"/>
+      <c r="V2" s="47" t="s">
+        <v>137</v>
+      </c>
+      <c r="W2" s="47"/>
+      <c r="X2" s="47"/>
     </row>
     <row r="3" spans="2:24" x14ac:dyDescent="0.2">
       <c r="B3" s="2" t="s">
@@ -12906,36 +12761,36 @@
   </cols>
   <sheetData>
     <row r="2" spans="2:24" x14ac:dyDescent="0.2">
-      <c r="B2" s="42" t="s">
-        <v>156</v>
-      </c>
-      <c r="C2" s="42"/>
-      <c r="D2" s="42"/>
-      <c r="F2" s="42" t="s">
-        <v>157</v>
-      </c>
-      <c r="G2" s="42"/>
-      <c r="H2" s="42"/>
-      <c r="J2" s="42" t="s">
-        <v>158</v>
-      </c>
-      <c r="K2" s="42"/>
-      <c r="L2" s="42"/>
-      <c r="N2" s="42" t="s">
-        <v>159</v>
-      </c>
-      <c r="O2" s="42"/>
-      <c r="P2" s="42"/>
-      <c r="R2" s="42" t="s">
-        <v>160</v>
-      </c>
-      <c r="S2" s="42"/>
-      <c r="T2" s="42"/>
-      <c r="V2" s="42" t="s">
-        <v>161</v>
-      </c>
-      <c r="W2" s="42"/>
-      <c r="X2" s="42"/>
+      <c r="B2" s="48" t="s">
+        <v>150</v>
+      </c>
+      <c r="C2" s="48"/>
+      <c r="D2" s="48"/>
+      <c r="F2" s="48" t="s">
+        <v>151</v>
+      </c>
+      <c r="G2" s="48"/>
+      <c r="H2" s="48"/>
+      <c r="J2" s="48" t="s">
+        <v>152</v>
+      </c>
+      <c r="K2" s="48"/>
+      <c r="L2" s="48"/>
+      <c r="N2" s="48" t="s">
+        <v>153</v>
+      </c>
+      <c r="O2" s="48"/>
+      <c r="P2" s="48"/>
+      <c r="R2" s="48" t="s">
+        <v>154</v>
+      </c>
+      <c r="S2" s="48"/>
+      <c r="T2" s="48"/>
+      <c r="V2" s="48" t="s">
+        <v>155</v>
+      </c>
+      <c r="W2" s="48"/>
+      <c r="X2" s="48"/>
     </row>
     <row r="3" spans="2:24" x14ac:dyDescent="0.2">
       <c r="B3" s="2" t="s">

</xml_diff>

<commit_message>
fixed an error in the input template
</commit_message>
<xml_diff>
--- a/docs/inputs/input_template.xlsx
+++ b/docs/inputs/input_template.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10102"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10118"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/njones/python_projects/xslope/docs/inputs/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{36D0CDE2-AEA0-474C-BEE8-CC42CBD1BD33}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{997720BA-1A6A-DF4F-940B-790C034221B6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="5900" yWindow="4020" windowWidth="34200" windowHeight="20240" xr2:uid="{BA54C293-CE08-6E4C-9212-B3317DAA148E}"/>
+    <workbookView xWindow="20540" yWindow="3900" windowWidth="34200" windowHeight="20240" xr2:uid="{BA54C293-CE08-6E4C-9212-B3317DAA148E}"/>
   </bookViews>
   <sheets>
     <sheet name="main" sheetId="1" r:id="rId1"/>
@@ -1047,13 +1047,13 @@
     <xf numFmtId="0" fontId="10" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
     <xf numFmtId="0" fontId="2" fillId="15" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="15" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="7" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
@@ -1078,7 +1078,35 @@
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="6">
+  <dxfs count="10">
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="1" tint="0.499984740745262"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="1" tint="0.499984740745262"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="1" tint="0.499984740745262"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="1" tint="0.499984740745262"/>
+        </patternFill>
+      </fill>
+    </dxf>
     <dxf>
       <fill>
         <patternFill>
@@ -10071,32 +10099,32 @@
     <mergeCell ref="R7:V7"/>
   </mergeCells>
   <conditionalFormatting sqref="E9:F50">
-    <cfRule type="expression" dxfId="5" priority="3">
+    <cfRule type="expression" dxfId="9" priority="3">
       <formula>$D9="cp"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="G9:H50">
-    <cfRule type="expression" dxfId="4" priority="2">
+    <cfRule type="expression" dxfId="8" priority="2">
       <formula>$D9="mc"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="I9:J50">
-    <cfRule type="expression" dxfId="3" priority="4">
+    <cfRule type="expression" dxfId="7" priority="4">
       <formula>$D9="cp"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="M9:N50">
-    <cfRule type="expression" dxfId="2" priority="6">
+    <cfRule type="expression" dxfId="6" priority="6">
       <formula>$D9="cp"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="O9:O50">
-    <cfRule type="expression" dxfId="1" priority="13">
+    <cfRule type="expression" dxfId="5" priority="13">
       <formula>$D9="mc"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="P9:Q50">
-    <cfRule type="expression" dxfId="0" priority="8">
+    <cfRule type="expression" dxfId="4" priority="8">
       <formula>$D9="cp"</formula>
     </cfRule>
   </conditionalFormatting>
@@ -10150,74 +10178,74 @@
       </c>
     </row>
     <row r="4" spans="1:44" x14ac:dyDescent="0.2">
-      <c r="A4" s="45" t="s">
+      <c r="A4" s="47" t="s">
         <v>2</v>
       </c>
-      <c r="B4" s="45"/>
-      <c r="D4" s="45" t="s">
+      <c r="B4" s="47"/>
+      <c r="D4" s="47" t="s">
         <v>5</v>
       </c>
-      <c r="E4" s="45"/>
-      <c r="G4" s="45" t="s">
+      <c r="E4" s="47"/>
+      <c r="G4" s="47" t="s">
         <v>6</v>
       </c>
-      <c r="H4" s="45"/>
-      <c r="J4" s="45" t="s">
+      <c r="H4" s="47"/>
+      <c r="J4" s="47" t="s">
         <v>7</v>
       </c>
-      <c r="K4" s="45"/>
-      <c r="M4" s="45" t="s">
+      <c r="K4" s="47"/>
+      <c r="M4" s="47" t="s">
         <v>8</v>
       </c>
-      <c r="N4" s="45"/>
-      <c r="P4" s="45" t="s">
+      <c r="N4" s="47"/>
+      <c r="P4" s="47" t="s">
         <v>9</v>
       </c>
-      <c r="Q4" s="45"/>
+      <c r="Q4" s="47"/>
       <c r="R4" s="1"/>
-      <c r="S4" s="45" t="s">
+      <c r="S4" s="47" t="s">
         <v>10</v>
       </c>
-      <c r="T4" s="45"/>
+      <c r="T4" s="47"/>
       <c r="U4" s="1"/>
-      <c r="V4" s="45" t="s">
+      <c r="V4" s="47" t="s">
         <v>11</v>
       </c>
-      <c r="W4" s="45"/>
+      <c r="W4" s="47"/>
       <c r="X4" s="1"/>
-      <c r="Y4" s="45" t="s">
+      <c r="Y4" s="47" t="s">
         <v>12</v>
       </c>
-      <c r="Z4" s="45"/>
+      <c r="Z4" s="47"/>
       <c r="AA4" s="1"/>
-      <c r="AB4" s="45" t="s">
+      <c r="AB4" s="47" t="s">
         <v>13</v>
       </c>
-      <c r="AC4" s="45"/>
-      <c r="AE4" s="45" t="s">
+      <c r="AC4" s="47"/>
+      <c r="AE4" s="47" t="s">
         <v>116</v>
       </c>
-      <c r="AF4" s="45"/>
+      <c r="AF4" s="47"/>
       <c r="AG4" s="1"/>
-      <c r="AH4" s="45" t="s">
+      <c r="AH4" s="47" t="s">
         <v>117</v>
       </c>
-      <c r="AI4" s="45"/>
+      <c r="AI4" s="47"/>
       <c r="AJ4" s="1"/>
-      <c r="AK4" s="45" t="s">
+      <c r="AK4" s="47" t="s">
         <v>118</v>
       </c>
-      <c r="AL4" s="45"/>
+      <c r="AL4" s="47"/>
       <c r="AM4" s="1"/>
-      <c r="AN4" s="45" t="s">
+      <c r="AN4" s="47" t="s">
         <v>119</v>
       </c>
-      <c r="AO4" s="45"/>
+      <c r="AO4" s="47"/>
       <c r="AP4" s="1"/>
-      <c r="AQ4" s="45" t="s">
+      <c r="AQ4" s="47" t="s">
         <v>120</v>
       </c>
-      <c r="AR4" s="45"/>
+      <c r="AR4" s="47"/>
     </row>
     <row r="5" spans="1:44" x14ac:dyDescent="0.2">
       <c r="A5" s="41" t="s">
@@ -10320,89 +10348,89 @@
       </c>
     </row>
     <row r="6" spans="1:44" x14ac:dyDescent="0.2">
-      <c r="A6" s="46" t="str">
+      <c r="A6" s="45" t="str">
         <f>_xlfn.XLOOKUP(B5,mat!$A:$A, mat!$B:$B,"") &amp; ""</f>
         <v/>
       </c>
-      <c r="B6" s="47"/>
-      <c r="D6" s="46" t="str">
+      <c r="B6" s="46"/>
+      <c r="D6" s="45" t="str">
         <f>_xlfn.XLOOKUP(E5,mat!$A:$A, mat!$B:$B,"") &amp; ""</f>
         <v/>
       </c>
-      <c r="E6" s="47"/>
-      <c r="G6" s="46" t="str">
+      <c r="E6" s="46"/>
+      <c r="G6" s="45" t="str">
         <f>_xlfn.XLOOKUP(H5,mat!$A:$A, mat!$B:$B,"") &amp; ""</f>
         <v/>
       </c>
-      <c r="H6" s="47"/>
-      <c r="J6" s="46" t="str">
+      <c r="H6" s="46"/>
+      <c r="J6" s="45" t="str">
         <f>_xlfn.XLOOKUP(K5,mat!$A:$A, mat!$B:$B,"") &amp; ""</f>
         <v/>
       </c>
-      <c r="K6" s="47"/>
-      <c r="M6" s="46" t="str">
+      <c r="K6" s="46"/>
+      <c r="M6" s="45" t="str">
         <f>_xlfn.XLOOKUP(N5,mat!$A:$A, mat!$B:$B,"") &amp; ""</f>
         <v/>
       </c>
-      <c r="N6" s="47"/>
-      <c r="P6" s="46" t="str">
+      <c r="N6" s="46"/>
+      <c r="P6" s="45" t="str">
         <f>_xlfn.XLOOKUP(Q5,mat!$A:$A, mat!$B:$B,"") &amp; ""</f>
         <v/>
       </c>
-      <c r="Q6" s="47"/>
+      <c r="Q6" s="46"/>
       <c r="R6" s="1"/>
-      <c r="S6" s="46" t="str">
+      <c r="S6" s="45" t="str">
         <f>_xlfn.XLOOKUP(T5,mat!$A:$A, mat!$B:$B,"") &amp; ""</f>
         <v/>
       </c>
-      <c r="T6" s="47"/>
+      <c r="T6" s="46"/>
       <c r="U6" s="1"/>
-      <c r="V6" s="46" t="str">
+      <c r="V6" s="45" t="str">
         <f>_xlfn.XLOOKUP(W5,mat!$A:$A, mat!$B:$B,"") &amp; ""</f>
         <v/>
       </c>
-      <c r="W6" s="47"/>
+      <c r="W6" s="46"/>
       <c r="X6" s="1"/>
-      <c r="Y6" s="46" t="str">
+      <c r="Y6" s="45" t="str">
         <f>_xlfn.XLOOKUP(Z5,mat!$A:$A, mat!$B:$B,"") &amp; ""</f>
         <v/>
       </c>
-      <c r="Z6" s="47"/>
+      <c r="Z6" s="46"/>
       <c r="AA6" s="1"/>
-      <c r="AB6" s="46" t="str">
+      <c r="AB6" s="45" t="str">
         <f>_xlfn.XLOOKUP(AC5,mat!$A:$A, mat!$B:$B,"") &amp; ""</f>
         <v/>
       </c>
-      <c r="AC6" s="47"/>
-      <c r="AE6" s="46" t="str">
+      <c r="AC6" s="46"/>
+      <c r="AE6" s="45" t="str">
         <f>_xlfn.XLOOKUP(AF5,mat!$A:$A, mat!$B:$B,"") &amp; ""</f>
         <v/>
       </c>
-      <c r="AF6" s="47"/>
+      <c r="AF6" s="46"/>
       <c r="AG6" s="1"/>
-      <c r="AH6" s="46" t="str">
+      <c r="AH6" s="45" t="str">
         <f>_xlfn.XLOOKUP(AI5,mat!$A:$A, mat!$B:$B,"") &amp; ""</f>
         <v/>
       </c>
-      <c r="AI6" s="47"/>
+      <c r="AI6" s="46"/>
       <c r="AJ6" s="1"/>
-      <c r="AK6" s="46" t="str">
+      <c r="AK6" s="45" t="str">
         <f>_xlfn.XLOOKUP(AL5,mat!$A:$A, mat!$B:$B,"") &amp; ""</f>
         <v/>
       </c>
-      <c r="AL6" s="47"/>
+      <c r="AL6" s="46"/>
       <c r="AM6" s="1"/>
-      <c r="AN6" s="46" t="str">
+      <c r="AN6" s="45" t="str">
         <f>_xlfn.XLOOKUP(AO5,mat!$A:$A, mat!$B:$B,"") &amp; ""</f>
         <v/>
       </c>
-      <c r="AO6" s="47"/>
+      <c r="AO6" s="46"/>
       <c r="AP6" s="1"/>
-      <c r="AQ6" s="46" t="str">
+      <c r="AQ6" s="45" t="str">
         <f>_xlfn.XLOOKUP(AR5,mat!$A:$A, mat!$B:$B,"") &amp; ""</f>
         <v/>
       </c>
-      <c r="AR6" s="47"/>
+      <c r="AR6" s="46"/>
     </row>
     <row r="7" spans="1:44" x14ac:dyDescent="0.2">
       <c r="A7" s="2" t="s">
@@ -11306,36 +11334,36 @@
     </row>
   </sheetData>
   <mergeCells count="30">
+    <mergeCell ref="A4:B4"/>
+    <mergeCell ref="D4:E4"/>
+    <mergeCell ref="G4:H4"/>
+    <mergeCell ref="J4:K4"/>
+    <mergeCell ref="M4:N4"/>
+    <mergeCell ref="P4:Q4"/>
+    <mergeCell ref="S4:T4"/>
+    <mergeCell ref="V4:W4"/>
+    <mergeCell ref="Y4:Z4"/>
+    <mergeCell ref="AB4:AC4"/>
+    <mergeCell ref="AE4:AF4"/>
+    <mergeCell ref="AH4:AI4"/>
+    <mergeCell ref="AK4:AL4"/>
+    <mergeCell ref="AN4:AO4"/>
+    <mergeCell ref="AQ4:AR4"/>
+    <mergeCell ref="A6:B6"/>
+    <mergeCell ref="D6:E6"/>
+    <mergeCell ref="G6:H6"/>
+    <mergeCell ref="J6:K6"/>
+    <mergeCell ref="M6:N6"/>
+    <mergeCell ref="P6:Q6"/>
+    <mergeCell ref="S6:T6"/>
+    <mergeCell ref="V6:W6"/>
+    <mergeCell ref="Y6:Z6"/>
+    <mergeCell ref="AB6:AC6"/>
     <mergeCell ref="AE6:AF6"/>
     <mergeCell ref="AH6:AI6"/>
     <mergeCell ref="AK6:AL6"/>
     <mergeCell ref="AN6:AO6"/>
     <mergeCell ref="AQ6:AR6"/>
-    <mergeCell ref="P6:Q6"/>
-    <mergeCell ref="S6:T6"/>
-    <mergeCell ref="V6:W6"/>
-    <mergeCell ref="Y6:Z6"/>
-    <mergeCell ref="AB6:AC6"/>
-    <mergeCell ref="A6:B6"/>
-    <mergeCell ref="D6:E6"/>
-    <mergeCell ref="G6:H6"/>
-    <mergeCell ref="J6:K6"/>
-    <mergeCell ref="M6:N6"/>
-    <mergeCell ref="AE4:AF4"/>
-    <mergeCell ref="AH4:AI4"/>
-    <mergeCell ref="AK4:AL4"/>
-    <mergeCell ref="AN4:AO4"/>
-    <mergeCell ref="AQ4:AR4"/>
-    <mergeCell ref="P4:Q4"/>
-    <mergeCell ref="S4:T4"/>
-    <mergeCell ref="V4:W4"/>
-    <mergeCell ref="Y4:Z4"/>
-    <mergeCell ref="AB4:AC4"/>
-    <mergeCell ref="A4:B4"/>
-    <mergeCell ref="D4:E4"/>
-    <mergeCell ref="G4:H4"/>
-    <mergeCell ref="J4:K4"/>
-    <mergeCell ref="M4:N4"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
@@ -11693,12 +11721,24 @@
       <c r="N16" s="1"/>
     </row>
   </sheetData>
-  <dataValidations count="2">
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="D5:D12" xr:uid="{06E9E004-FC39-FE49-926A-912F810F5089}">
+  <conditionalFormatting sqref="E3:E42">
+    <cfRule type="expression" dxfId="3" priority="3">
+      <formula>OR($D3="Intercept", $D3="Radius")</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="F3:G42">
+    <cfRule type="expression" dxfId="1" priority="2">
+      <formula>OR($D3="Depth",$D3="Radius")</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="H3:H42">
+    <cfRule type="expression" dxfId="0" priority="1">
+      <formula>OR($D3="Depth",$D3="Intercept")</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <dataValidations count="1">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="D3:D52" xr:uid="{06E9E004-FC39-FE49-926A-912F810F5089}">
       <formula1>$J$3:$J$5</formula1>
-    </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="D3:D4" xr:uid="{AEFC92A9-AB07-FF4B-9461-938B9BDCD07D}">
-      <formula1>$J$5:$J$7</formula1>
     </dataValidation>
   </dataValidations>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>

<commit_message>
Add polygon-sheet seepage examples; fix xlsx writer for Excel display
Add poly_test/ build scripts and polygon-based input files for the sea
trench, levee, Johnson reservoir, and earth dam seepage problems,
derived from the existing profile-based inputs via build_polygons().

Fix write_cells_to_xlsx in the xslope skill (docs/usage/claude/xslope.md)
so generated files display correctly in Excel:
- set fullCalcOnLoad so row-6 XLOOKUP material names recompute on open
- drop the now-stale calcChain.xml (+ its refs) so Excel rebuilds it
  instead of "recovering" and blanking the edited sheet
- reset each populated sheet's saved view to A1 (the template ships the
  polygon sheet scrolled to AA1, which made it look empty on open)

Co-Authored-By: Claude Opus 4.8 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/inputs/input_template.xlsx
+++ b/docs/inputs/input_template.xlsx
@@ -1,7 +1,7 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10315"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10322"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
@@ -10,7 +10,7 @@
   </mc:AlternateContent>
   <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BB3293A3-B1F8-4840-BCCF-D44260C5241D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="25040" yWindow="2500" windowWidth="42700" windowHeight="22800" activeTab="11" xr2:uid="{BA54C293-CE08-6E4C-9212-B3317DAA148E}"/>
+    <workbookView xWindow="25040" yWindow="2500" windowWidth="42700" windowHeight="22800" xr2:uid="{BA54C293-CE08-6E4C-9212-B3317DAA148E}"/>
   </bookViews>
   <sheets>
     <sheet name="main" sheetId="1" r:id="rId1"/>
@@ -1209,13 +1209,13 @@
     <xf numFmtId="0" fontId="10" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
     <xf numFmtId="0" fontId="2" fillId="15" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="15" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="16" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -13208,74 +13208,74 @@
       </c>
     </row>
     <row r="4" spans="1:44" x14ac:dyDescent="0.2">
-      <c r="A4" s="50" t="s">
+      <c r="A4" s="52" t="s">
         <v>2</v>
       </c>
-      <c r="B4" s="50"/>
-      <c r="D4" s="50" t="s">
+      <c r="B4" s="52"/>
+      <c r="D4" s="52" t="s">
         <v>5</v>
       </c>
-      <c r="E4" s="50"/>
-      <c r="G4" s="50" t="s">
+      <c r="E4" s="52"/>
+      <c r="G4" s="52" t="s">
         <v>6</v>
       </c>
-      <c r="H4" s="50"/>
-      <c r="J4" s="50" t="s">
+      <c r="H4" s="52"/>
+      <c r="J4" s="52" t="s">
         <v>7</v>
       </c>
-      <c r="K4" s="50"/>
-      <c r="M4" s="50" t="s">
+      <c r="K4" s="52"/>
+      <c r="M4" s="52" t="s">
         <v>8</v>
       </c>
-      <c r="N4" s="50"/>
-      <c r="P4" s="50" t="s">
+      <c r="N4" s="52"/>
+      <c r="P4" s="52" t="s">
         <v>9</v>
       </c>
-      <c r="Q4" s="50"/>
+      <c r="Q4" s="52"/>
       <c r="R4" s="1"/>
-      <c r="S4" s="50" t="s">
+      <c r="S4" s="52" t="s">
         <v>10</v>
       </c>
-      <c r="T4" s="50"/>
+      <c r="T4" s="52"/>
       <c r="U4" s="1"/>
-      <c r="V4" s="50" t="s">
+      <c r="V4" s="52" t="s">
         <v>11</v>
       </c>
-      <c r="W4" s="50"/>
+      <c r="W4" s="52"/>
       <c r="X4" s="1"/>
-      <c r="Y4" s="50" t="s">
+      <c r="Y4" s="52" t="s">
         <v>12</v>
       </c>
-      <c r="Z4" s="50"/>
+      <c r="Z4" s="52"/>
       <c r="AA4" s="1"/>
-      <c r="AB4" s="50" t="s">
+      <c r="AB4" s="52" t="s">
         <v>13</v>
       </c>
-      <c r="AC4" s="50"/>
-      <c r="AE4" s="50" t="s">
+      <c r="AC4" s="52"/>
+      <c r="AE4" s="52" t="s">
         <v>114</v>
       </c>
-      <c r="AF4" s="50"/>
+      <c r="AF4" s="52"/>
       <c r="AG4" s="1"/>
-      <c r="AH4" s="50" t="s">
+      <c r="AH4" s="52" t="s">
         <v>115</v>
       </c>
-      <c r="AI4" s="50"/>
+      <c r="AI4" s="52"/>
       <c r="AJ4" s="1"/>
-      <c r="AK4" s="50" t="s">
+      <c r="AK4" s="52" t="s">
         <v>116</v>
       </c>
-      <c r="AL4" s="50"/>
+      <c r="AL4" s="52"/>
       <c r="AM4" s="1"/>
-      <c r="AN4" s="50" t="s">
+      <c r="AN4" s="52" t="s">
         <v>117</v>
       </c>
-      <c r="AO4" s="50"/>
+      <c r="AO4" s="52"/>
       <c r="AP4" s="1"/>
-      <c r="AQ4" s="50" t="s">
+      <c r="AQ4" s="52" t="s">
         <v>118</v>
       </c>
-      <c r="AR4" s="50"/>
+      <c r="AR4" s="52"/>
     </row>
     <row r="5" spans="1:44" x14ac:dyDescent="0.2">
       <c r="A5" s="41" t="s">
@@ -13378,89 +13378,89 @@
       </c>
     </row>
     <row r="6" spans="1:44" x14ac:dyDescent="0.2">
-      <c r="A6" s="51" t="str">
+      <c r="A6" s="50" t="str">
         <f>_xlfn.XLOOKUP(B5,mat!$A:$A, mat!$B:$B,"") &amp; ""</f>
         <v/>
       </c>
-      <c r="B6" s="52"/>
-      <c r="D6" s="51" t="str">
+      <c r="B6" s="51"/>
+      <c r="D6" s="50" t="str">
         <f>_xlfn.XLOOKUP(E5,mat!$A:$A, mat!$B:$B,"") &amp; ""</f>
         <v/>
       </c>
-      <c r="E6" s="52"/>
-      <c r="G6" s="51" t="str">
+      <c r="E6" s="51"/>
+      <c r="G6" s="50" t="str">
         <f>_xlfn.XLOOKUP(H5,mat!$A:$A, mat!$B:$B,"") &amp; ""</f>
         <v/>
       </c>
-      <c r="H6" s="52"/>
-      <c r="J6" s="51" t="str">
+      <c r="H6" s="51"/>
+      <c r="J6" s="50" t="str">
         <f>_xlfn.XLOOKUP(K5,mat!$A:$A, mat!$B:$B,"") &amp; ""</f>
         <v/>
       </c>
-      <c r="K6" s="52"/>
-      <c r="M6" s="51" t="str">
+      <c r="K6" s="51"/>
+      <c r="M6" s="50" t="str">
         <f>_xlfn.XLOOKUP(N5,mat!$A:$A, mat!$B:$B,"") &amp; ""</f>
         <v/>
       </c>
-      <c r="N6" s="52"/>
-      <c r="P6" s="51" t="str">
+      <c r="N6" s="51"/>
+      <c r="P6" s="50" t="str">
         <f>_xlfn.XLOOKUP(Q5,mat!$A:$A, mat!$B:$B,"") &amp; ""</f>
         <v/>
       </c>
-      <c r="Q6" s="52"/>
+      <c r="Q6" s="51"/>
       <c r="R6" s="1"/>
-      <c r="S6" s="51" t="str">
+      <c r="S6" s="50" t="str">
         <f>_xlfn.XLOOKUP(T5,mat!$A:$A, mat!$B:$B,"") &amp; ""</f>
         <v/>
       </c>
-      <c r="T6" s="52"/>
+      <c r="T6" s="51"/>
       <c r="U6" s="1"/>
-      <c r="V6" s="51" t="str">
+      <c r="V6" s="50" t="str">
         <f>_xlfn.XLOOKUP(W5,mat!$A:$A, mat!$B:$B,"") &amp; ""</f>
         <v/>
       </c>
-      <c r="W6" s="52"/>
+      <c r="W6" s="51"/>
       <c r="X6" s="1"/>
-      <c r="Y6" s="51" t="str">
+      <c r="Y6" s="50" t="str">
         <f>_xlfn.XLOOKUP(Z5,mat!$A:$A, mat!$B:$B,"") &amp; ""</f>
         <v/>
       </c>
-      <c r="Z6" s="52"/>
+      <c r="Z6" s="51"/>
       <c r="AA6" s="1"/>
-      <c r="AB6" s="51" t="str">
+      <c r="AB6" s="50" t="str">
         <f>_xlfn.XLOOKUP(AC5,mat!$A:$A, mat!$B:$B,"") &amp; ""</f>
         <v/>
       </c>
-      <c r="AC6" s="52"/>
-      <c r="AE6" s="51" t="str">
+      <c r="AC6" s="51"/>
+      <c r="AE6" s="50" t="str">
         <f>_xlfn.XLOOKUP(AF5,mat!$A:$A, mat!$B:$B,"") &amp; ""</f>
         <v/>
       </c>
-      <c r="AF6" s="52"/>
+      <c r="AF6" s="51"/>
       <c r="AG6" s="1"/>
-      <c r="AH6" s="51" t="str">
+      <c r="AH6" s="50" t="str">
         <f>_xlfn.XLOOKUP(AI5,mat!$A:$A, mat!$B:$B,"") &amp; ""</f>
         <v/>
       </c>
-      <c r="AI6" s="52"/>
+      <c r="AI6" s="51"/>
       <c r="AJ6" s="1"/>
-      <c r="AK6" s="51" t="str">
+      <c r="AK6" s="50" t="str">
         <f>_xlfn.XLOOKUP(AL5,mat!$A:$A, mat!$B:$B,"") &amp; ""</f>
         <v/>
       </c>
-      <c r="AL6" s="52"/>
+      <c r="AL6" s="51"/>
       <c r="AM6" s="1"/>
-      <c r="AN6" s="51" t="str">
+      <c r="AN6" s="50" t="str">
         <f>_xlfn.XLOOKUP(AO5,mat!$A:$A, mat!$B:$B,"") &amp; ""</f>
         <v/>
       </c>
-      <c r="AO6" s="52"/>
+      <c r="AO6" s="51"/>
       <c r="AP6" s="1"/>
-      <c r="AQ6" s="51" t="str">
+      <c r="AQ6" s="50" t="str">
         <f>_xlfn.XLOOKUP(AR5,mat!$A:$A, mat!$B:$B,"") &amp; ""</f>
         <v/>
       </c>
-      <c r="AR6" s="52"/>
+      <c r="AR6" s="51"/>
     </row>
     <row r="7" spans="1:44" x14ac:dyDescent="0.2">
       <c r="A7" s="2" t="s">
@@ -14364,36 +14364,36 @@
     </row>
   </sheetData>
   <mergeCells count="30">
+    <mergeCell ref="A4:B4"/>
+    <mergeCell ref="D4:E4"/>
+    <mergeCell ref="G4:H4"/>
+    <mergeCell ref="J4:K4"/>
+    <mergeCell ref="M4:N4"/>
+    <mergeCell ref="P4:Q4"/>
+    <mergeCell ref="S4:T4"/>
+    <mergeCell ref="V4:W4"/>
+    <mergeCell ref="Y4:Z4"/>
+    <mergeCell ref="AB4:AC4"/>
+    <mergeCell ref="AE4:AF4"/>
+    <mergeCell ref="AH4:AI4"/>
+    <mergeCell ref="AK4:AL4"/>
+    <mergeCell ref="AN4:AO4"/>
+    <mergeCell ref="AQ4:AR4"/>
+    <mergeCell ref="A6:B6"/>
+    <mergeCell ref="D6:E6"/>
+    <mergeCell ref="G6:H6"/>
+    <mergeCell ref="J6:K6"/>
+    <mergeCell ref="M6:N6"/>
+    <mergeCell ref="P6:Q6"/>
+    <mergeCell ref="S6:T6"/>
+    <mergeCell ref="V6:W6"/>
+    <mergeCell ref="Y6:Z6"/>
+    <mergeCell ref="AB6:AC6"/>
     <mergeCell ref="AE6:AF6"/>
     <mergeCell ref="AH6:AI6"/>
     <mergeCell ref="AK6:AL6"/>
     <mergeCell ref="AN6:AO6"/>
     <mergeCell ref="AQ6:AR6"/>
-    <mergeCell ref="P6:Q6"/>
-    <mergeCell ref="S6:T6"/>
-    <mergeCell ref="V6:W6"/>
-    <mergeCell ref="Y6:Z6"/>
-    <mergeCell ref="AB6:AC6"/>
-    <mergeCell ref="A6:B6"/>
-    <mergeCell ref="D6:E6"/>
-    <mergeCell ref="G6:H6"/>
-    <mergeCell ref="J6:K6"/>
-    <mergeCell ref="M6:N6"/>
-    <mergeCell ref="AE4:AF4"/>
-    <mergeCell ref="AH4:AI4"/>
-    <mergeCell ref="AK4:AL4"/>
-    <mergeCell ref="AN4:AO4"/>
-    <mergeCell ref="AQ4:AR4"/>
-    <mergeCell ref="P4:Q4"/>
-    <mergeCell ref="S4:T4"/>
-    <mergeCell ref="V4:W4"/>
-    <mergeCell ref="Y4:Z4"/>
-    <mergeCell ref="AB4:AC4"/>
-    <mergeCell ref="A4:B4"/>
-    <mergeCell ref="D4:E4"/>
-    <mergeCell ref="G4:H4"/>
-    <mergeCell ref="J4:K4"/>
-    <mergeCell ref="M4:N4"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
@@ -14431,74 +14431,74 @@
       </c>
     </row>
     <row r="4" spans="1:44" x14ac:dyDescent="0.2">
-      <c r="A4" s="50" t="s">
+      <c r="A4" s="52" t="s">
         <v>153</v>
       </c>
-      <c r="B4" s="50"/>
-      <c r="D4" s="50" t="s">
+      <c r="B4" s="52"/>
+      <c r="D4" s="52" t="s">
         <v>154</v>
       </c>
-      <c r="E4" s="50"/>
-      <c r="G4" s="50" t="s">
+      <c r="E4" s="52"/>
+      <c r="G4" s="52" t="s">
         <v>155</v>
       </c>
-      <c r="H4" s="50"/>
-      <c r="J4" s="50" t="s">
+      <c r="H4" s="52"/>
+      <c r="J4" s="52" t="s">
         <v>156</v>
       </c>
-      <c r="K4" s="50"/>
-      <c r="M4" s="50" t="s">
+      <c r="K4" s="52"/>
+      <c r="M4" s="52" t="s">
         <v>157</v>
       </c>
-      <c r="N4" s="50"/>
-      <c r="P4" s="50" t="s">
+      <c r="N4" s="52"/>
+      <c r="P4" s="52" t="s">
         <v>158</v>
       </c>
-      <c r="Q4" s="50"/>
+      <c r="Q4" s="52"/>
       <c r="R4" s="1"/>
-      <c r="S4" s="50" t="s">
+      <c r="S4" s="52" t="s">
         <v>159</v>
       </c>
-      <c r="T4" s="50"/>
+      <c r="T4" s="52"/>
       <c r="U4" s="1"/>
-      <c r="V4" s="50" t="s">
+      <c r="V4" s="52" t="s">
         <v>160</v>
       </c>
-      <c r="W4" s="50"/>
+      <c r="W4" s="52"/>
       <c r="X4" s="1"/>
-      <c r="Y4" s="50" t="s">
+      <c r="Y4" s="52" t="s">
         <v>161</v>
       </c>
-      <c r="Z4" s="50"/>
+      <c r="Z4" s="52"/>
       <c r="AA4" s="1"/>
-      <c r="AB4" s="50" t="s">
+      <c r="AB4" s="52" t="s">
         <v>162</v>
       </c>
-      <c r="AC4" s="50"/>
-      <c r="AE4" s="50" t="s">
+      <c r="AC4" s="52"/>
+      <c r="AE4" s="52" t="s">
         <v>163</v>
       </c>
-      <c r="AF4" s="50"/>
+      <c r="AF4" s="52"/>
       <c r="AG4" s="1"/>
-      <c r="AH4" s="50" t="s">
+      <c r="AH4" s="52" t="s">
         <v>164</v>
       </c>
-      <c r="AI4" s="50"/>
+      <c r="AI4" s="52"/>
       <c r="AJ4" s="1"/>
-      <c r="AK4" s="50" t="s">
+      <c r="AK4" s="52" t="s">
         <v>165</v>
       </c>
-      <c r="AL4" s="50"/>
+      <c r="AL4" s="52"/>
       <c r="AM4" s="1"/>
-      <c r="AN4" s="50" t="s">
+      <c r="AN4" s="52" t="s">
         <v>166</v>
       </c>
-      <c r="AO4" s="50"/>
+      <c r="AO4" s="52"/>
       <c r="AP4" s="1"/>
-      <c r="AQ4" s="50" t="s">
+      <c r="AQ4" s="52" t="s">
         <v>167</v>
       </c>
-      <c r="AR4" s="50"/>
+      <c r="AR4" s="52"/>
     </row>
     <row r="5" spans="1:44" x14ac:dyDescent="0.2">
       <c r="A5" s="43" t="s">
@@ -15587,14 +15587,12 @@
     </row>
   </sheetData>
   <mergeCells count="30">
-    <mergeCell ref="AN6:AO6"/>
-    <mergeCell ref="AQ6:AR6"/>
-    <mergeCell ref="V6:W6"/>
-    <mergeCell ref="Y6:Z6"/>
-    <mergeCell ref="AB6:AC6"/>
-    <mergeCell ref="AE6:AF6"/>
-    <mergeCell ref="AH6:AI6"/>
-    <mergeCell ref="AK6:AL6"/>
+    <mergeCell ref="P4:Q4"/>
+    <mergeCell ref="A4:B4"/>
+    <mergeCell ref="D4:E4"/>
+    <mergeCell ref="G4:H4"/>
+    <mergeCell ref="J4:K4"/>
+    <mergeCell ref="M4:N4"/>
     <mergeCell ref="AK4:AL4"/>
     <mergeCell ref="AN4:AO4"/>
     <mergeCell ref="AQ4:AR4"/>
@@ -15611,12 +15609,14 @@
     <mergeCell ref="AB4:AC4"/>
     <mergeCell ref="AE4:AF4"/>
     <mergeCell ref="AH4:AI4"/>
-    <mergeCell ref="P4:Q4"/>
-    <mergeCell ref="A4:B4"/>
-    <mergeCell ref="D4:E4"/>
-    <mergeCell ref="G4:H4"/>
-    <mergeCell ref="J4:K4"/>
-    <mergeCell ref="M4:N4"/>
+    <mergeCell ref="AN6:AO6"/>
+    <mergeCell ref="AQ6:AR6"/>
+    <mergeCell ref="V6:W6"/>
+    <mergeCell ref="Y6:Z6"/>
+    <mergeCell ref="AB6:AC6"/>
+    <mergeCell ref="AE6:AF6"/>
+    <mergeCell ref="AH6:AI6"/>
+    <mergeCell ref="AK6:AL6"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>

<commit_message>
template: main-sheet Sheet list now names every sheet (piles, lloads, polygon)
Norm's edit to the master (docs/inputs/input_template.xlsx), closing the gap
the sheet-renderer audit flagged. Cosmetic — no version bump, his call. The
packaged copy (xslope/resources/) is synced byte-for-byte, and sheet_main.png
is regenerated through the new renderer, which is the whole point of it:
template edited, one command, docs current. Roundtrip gate 17/17.

Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_0147GB4LGVZuqGHCRMVzZTsR
</commit_message>
<xml_diff>
--- a/docs/inputs/input_template.xlsx
+++ b/docs/inputs/input_template.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10628"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10713"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/njones/python_projects/xslope/docs/inputs/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4DDD943A-8E76-F046-B66C-342D6E3A3C91}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6E95D610-588A-C249-B900-E3D88174AD4C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="12240" yWindow="4480" windowWidth="53960" windowHeight="22800" xr2:uid="{BA54C293-CE08-6E4C-9212-B3317DAA148E}"/>
+    <workbookView xWindow="0" yWindow="600" windowWidth="38400" windowHeight="19900" xr2:uid="{BA54C293-CE08-6E4C-9212-B3317DAA148E}"/>
   </bookViews>
   <sheets>
     <sheet name="main" sheetId="1" r:id="rId1"/>
@@ -62,7 +62,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="437" uniqueCount="229">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="443" uniqueCount="235">
   <si>
     <t>X</t>
   </si>
@@ -914,6 +914,24 @@
   </si>
   <si>
     <t>Neumann flux - normal Darcy velocity (len/time), + = inflow</t>
+  </si>
+  <si>
+    <t>polygon</t>
+  </si>
+  <si>
+    <t>Polygons describing the slope geometry</t>
+  </si>
+  <si>
+    <t>piles</t>
+  </si>
+  <si>
+    <t>Piles</t>
+  </si>
+  <si>
+    <t>lloads</t>
+  </si>
+  <si>
+    <t>Line loads</t>
   </si>
 </sst>
 </file>
@@ -1385,13 +1403,13 @@
     <xf numFmtId="0" fontId="10" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
     <xf numFmtId="0" fontId="2" fillId="15" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="15" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="16" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -10456,71 +10474,92 @@
         <v>0</v>
       </c>
       <c r="F11" s="1" t="s">
-        <v>21</v>
+        <v>229</v>
       </c>
       <c r="G11" t="s">
-        <v>22</v>
+        <v>230</v>
       </c>
     </row>
     <row r="12" spans="1:7" x14ac:dyDescent="0.2">
       <c r="F12" s="1" t="s">
-        <v>23</v>
+        <v>21</v>
       </c>
       <c r="G12" t="s">
-        <v>24</v>
+        <v>22</v>
       </c>
     </row>
     <row r="13" spans="1:7" x14ac:dyDescent="0.2">
       <c r="F13" s="1" t="s">
-        <v>38</v>
+        <v>23</v>
       </c>
       <c r="G13" t="s">
-        <v>39</v>
+        <v>24</v>
       </c>
     </row>
     <row r="14" spans="1:7" x14ac:dyDescent="0.2">
       <c r="F14" s="1" t="s">
-        <v>34</v>
+        <v>38</v>
       </c>
       <c r="G14" t="s">
-        <v>35</v>
+        <v>39</v>
       </c>
     </row>
     <row r="15" spans="1:7" x14ac:dyDescent="0.2">
       <c r="F15" s="1" t="s">
-        <v>117</v>
+        <v>34</v>
       </c>
       <c r="G15" t="s">
-        <v>119</v>
+        <v>35</v>
       </c>
     </row>
     <row r="16" spans="1:7" x14ac:dyDescent="0.2">
       <c r="F16" s="1" t="s">
-        <v>36</v>
+        <v>117</v>
       </c>
       <c r="G16" t="s">
-        <v>37</v>
+        <v>119</v>
       </c>
     </row>
     <row r="17" spans="2:7" x14ac:dyDescent="0.2">
       <c r="B17" s="1"/>
       <c r="F17" s="1" t="s">
-        <v>94</v>
-      </c>
-      <c r="G17" s="9" t="s">
-        <v>121</v>
+        <v>36</v>
+      </c>
+      <c r="G17" t="s">
+        <v>37</v>
       </c>
     </row>
     <row r="18" spans="2:7" x14ac:dyDescent="0.2">
       <c r="F18" s="1" t="s">
+        <v>231</v>
+      </c>
+      <c r="G18" t="s">
+        <v>232</v>
+      </c>
+    </row>
+    <row r="19" spans="2:7" x14ac:dyDescent="0.2">
+      <c r="F19" s="1" t="s">
+        <v>233</v>
+      </c>
+      <c r="G19" t="s">
+        <v>234</v>
+      </c>
+    </row>
+    <row r="20" spans="2:7" x14ac:dyDescent="0.2">
+      <c r="F20" s="1" t="s">
+        <v>94</v>
+      </c>
+      <c r="G20" s="9" t="s">
+        <v>121</v>
+      </c>
+    </row>
+    <row r="21" spans="2:7" x14ac:dyDescent="0.2">
+      <c r="F21" s="1" t="s">
         <v>118</v>
       </c>
-      <c r="G18" s="9" t="s">
+      <c r="G21" s="9" t="s">
         <v>120</v>
       </c>
-    </row>
-    <row r="20" spans="2:7" x14ac:dyDescent="0.2">
-      <c r="F20" s="1"/>
     </row>
     <row r="23" spans="2:7" x14ac:dyDescent="0.2">
       <c r="B23" s="1"/>
@@ -14698,74 +14737,74 @@
       </c>
     </row>
     <row r="4" spans="1:44" x14ac:dyDescent="0.2">
-      <c r="A4" s="53" t="s">
+      <c r="A4" s="51" t="s">
         <v>2</v>
       </c>
-      <c r="B4" s="53"/>
-      <c r="D4" s="53" t="s">
+      <c r="B4" s="51"/>
+      <c r="D4" s="51" t="s">
         <v>5</v>
       </c>
-      <c r="E4" s="53"/>
-      <c r="G4" s="53" t="s">
+      <c r="E4" s="51"/>
+      <c r="G4" s="51" t="s">
         <v>6</v>
       </c>
-      <c r="H4" s="53"/>
-      <c r="J4" s="53" t="s">
+      <c r="H4" s="51"/>
+      <c r="J4" s="51" t="s">
         <v>7</v>
       </c>
-      <c r="K4" s="53"/>
-      <c r="M4" s="53" t="s">
+      <c r="K4" s="51"/>
+      <c r="M4" s="51" t="s">
         <v>8</v>
       </c>
-      <c r="N4" s="53"/>
-      <c r="P4" s="53" t="s">
+      <c r="N4" s="51"/>
+      <c r="P4" s="51" t="s">
         <v>9</v>
       </c>
-      <c r="Q4" s="53"/>
+      <c r="Q4" s="51"/>
       <c r="R4" s="1"/>
-      <c r="S4" s="53" t="s">
+      <c r="S4" s="51" t="s">
         <v>10</v>
       </c>
-      <c r="T4" s="53"/>
+      <c r="T4" s="51"/>
       <c r="U4" s="1"/>
-      <c r="V4" s="53" t="s">
+      <c r="V4" s="51" t="s">
         <v>11</v>
       </c>
-      <c r="W4" s="53"/>
+      <c r="W4" s="51"/>
       <c r="X4" s="1"/>
-      <c r="Y4" s="53" t="s">
+      <c r="Y4" s="51" t="s">
         <v>12</v>
       </c>
-      <c r="Z4" s="53"/>
+      <c r="Z4" s="51"/>
       <c r="AA4" s="1"/>
-      <c r="AB4" s="53" t="s">
+      <c r="AB4" s="51" t="s">
         <v>13</v>
       </c>
-      <c r="AC4" s="53"/>
-      <c r="AE4" s="53" t="s">
+      <c r="AC4" s="51"/>
+      <c r="AE4" s="51" t="s">
         <v>110</v>
       </c>
-      <c r="AF4" s="53"/>
+      <c r="AF4" s="51"/>
       <c r="AG4" s="1"/>
-      <c r="AH4" s="53" t="s">
+      <c r="AH4" s="51" t="s">
         <v>111</v>
       </c>
-      <c r="AI4" s="53"/>
+      <c r="AI4" s="51"/>
       <c r="AJ4" s="1"/>
-      <c r="AK4" s="53" t="s">
+      <c r="AK4" s="51" t="s">
         <v>112</v>
       </c>
-      <c r="AL4" s="53"/>
+      <c r="AL4" s="51"/>
       <c r="AM4" s="1"/>
-      <c r="AN4" s="53" t="s">
+      <c r="AN4" s="51" t="s">
         <v>113</v>
       </c>
-      <c r="AO4" s="53"/>
+      <c r="AO4" s="51"/>
       <c r="AP4" s="1"/>
-      <c r="AQ4" s="53" t="s">
+      <c r="AQ4" s="51" t="s">
         <v>114</v>
       </c>
-      <c r="AR4" s="53"/>
+      <c r="AR4" s="51"/>
     </row>
     <row r="5" spans="1:44" x14ac:dyDescent="0.2">
       <c r="A5" s="40" t="s">
@@ -14868,89 +14907,89 @@
       </c>
     </row>
     <row r="6" spans="1:44" x14ac:dyDescent="0.2">
-      <c r="A6" s="51" t="str">
+      <c r="A6" s="52" t="str">
         <f>_xlfn.XLOOKUP(B5,mat!$A:$A, mat!$B:$B,"") &amp; ""</f>
         <v/>
       </c>
-      <c r="B6" s="52"/>
-      <c r="D6" s="51" t="str">
+      <c r="B6" s="53"/>
+      <c r="D6" s="52" t="str">
         <f>_xlfn.XLOOKUP(E5,mat!$A:$A, mat!$B:$B,"") &amp; ""</f>
         <v/>
       </c>
-      <c r="E6" s="52"/>
-      <c r="G6" s="51" t="str">
+      <c r="E6" s="53"/>
+      <c r="G6" s="52" t="str">
         <f>_xlfn.XLOOKUP(H5,mat!$A:$A, mat!$B:$B,"") &amp; ""</f>
         <v/>
       </c>
-      <c r="H6" s="52"/>
-      <c r="J6" s="51" t="str">
+      <c r="H6" s="53"/>
+      <c r="J6" s="52" t="str">
         <f>_xlfn.XLOOKUP(K5,mat!$A:$A, mat!$B:$B,"") &amp; ""</f>
         <v/>
       </c>
-      <c r="K6" s="52"/>
-      <c r="M6" s="51" t="str">
+      <c r="K6" s="53"/>
+      <c r="M6" s="52" t="str">
         <f>_xlfn.XLOOKUP(N5,mat!$A:$A, mat!$B:$B,"") &amp; ""</f>
         <v/>
       </c>
-      <c r="N6" s="52"/>
-      <c r="P6" s="51" t="str">
+      <c r="N6" s="53"/>
+      <c r="P6" s="52" t="str">
         <f>_xlfn.XLOOKUP(Q5,mat!$A:$A, mat!$B:$B,"") &amp; ""</f>
         <v/>
       </c>
-      <c r="Q6" s="52"/>
+      <c r="Q6" s="53"/>
       <c r="R6" s="1"/>
-      <c r="S6" s="51" t="str">
+      <c r="S6" s="52" t="str">
         <f>_xlfn.XLOOKUP(T5,mat!$A:$A, mat!$B:$B,"") &amp; ""</f>
         <v/>
       </c>
-      <c r="T6" s="52"/>
+      <c r="T6" s="53"/>
       <c r="U6" s="1"/>
-      <c r="V6" s="51" t="str">
+      <c r="V6" s="52" t="str">
         <f>_xlfn.XLOOKUP(W5,mat!$A:$A, mat!$B:$B,"") &amp; ""</f>
         <v/>
       </c>
-      <c r="W6" s="52"/>
+      <c r="W6" s="53"/>
       <c r="X6" s="1"/>
-      <c r="Y6" s="51" t="str">
+      <c r="Y6" s="52" t="str">
         <f>_xlfn.XLOOKUP(Z5,mat!$A:$A, mat!$B:$B,"") &amp; ""</f>
         <v/>
       </c>
-      <c r="Z6" s="52"/>
+      <c r="Z6" s="53"/>
       <c r="AA6" s="1"/>
-      <c r="AB6" s="51" t="str">
+      <c r="AB6" s="52" t="str">
         <f>_xlfn.XLOOKUP(AC5,mat!$A:$A, mat!$B:$B,"") &amp; ""</f>
         <v/>
       </c>
-      <c r="AC6" s="52"/>
-      <c r="AE6" s="51" t="str">
+      <c r="AC6" s="53"/>
+      <c r="AE6" s="52" t="str">
         <f>_xlfn.XLOOKUP(AF5,mat!$A:$A, mat!$B:$B,"") &amp; ""</f>
         <v/>
       </c>
-      <c r="AF6" s="52"/>
+      <c r="AF6" s="53"/>
       <c r="AG6" s="1"/>
-      <c r="AH6" s="51" t="str">
+      <c r="AH6" s="52" t="str">
         <f>_xlfn.XLOOKUP(AI5,mat!$A:$A, mat!$B:$B,"") &amp; ""</f>
         <v/>
       </c>
-      <c r="AI6" s="52"/>
+      <c r="AI6" s="53"/>
       <c r="AJ6" s="1"/>
-      <c r="AK6" s="51" t="str">
+      <c r="AK6" s="52" t="str">
         <f>_xlfn.XLOOKUP(AL5,mat!$A:$A, mat!$B:$B,"") &amp; ""</f>
         <v/>
       </c>
-      <c r="AL6" s="52"/>
+      <c r="AL6" s="53"/>
       <c r="AM6" s="1"/>
-      <c r="AN6" s="51" t="str">
+      <c r="AN6" s="52" t="str">
         <f>_xlfn.XLOOKUP(AO5,mat!$A:$A, mat!$B:$B,"") &amp; ""</f>
         <v/>
       </c>
-      <c r="AO6" s="52"/>
+      <c r="AO6" s="53"/>
       <c r="AP6" s="1"/>
-      <c r="AQ6" s="51" t="str">
+      <c r="AQ6" s="52" t="str">
         <f>_xlfn.XLOOKUP(AR5,mat!$A:$A, mat!$B:$B,"") &amp; ""</f>
         <v/>
       </c>
-      <c r="AR6" s="52"/>
+      <c r="AR6" s="53"/>
     </row>
     <row r="7" spans="1:44" x14ac:dyDescent="0.2">
       <c r="A7" s="2" t="s">
@@ -15854,36 +15893,36 @@
     </row>
   </sheetData>
   <mergeCells count="30">
+    <mergeCell ref="AE6:AF6"/>
+    <mergeCell ref="AH6:AI6"/>
+    <mergeCell ref="AK6:AL6"/>
+    <mergeCell ref="AN6:AO6"/>
+    <mergeCell ref="AQ6:AR6"/>
+    <mergeCell ref="P6:Q6"/>
+    <mergeCell ref="S6:T6"/>
+    <mergeCell ref="V6:W6"/>
+    <mergeCell ref="Y6:Z6"/>
+    <mergeCell ref="AB6:AC6"/>
+    <mergeCell ref="A6:B6"/>
+    <mergeCell ref="D6:E6"/>
+    <mergeCell ref="G6:H6"/>
+    <mergeCell ref="J6:K6"/>
+    <mergeCell ref="M6:N6"/>
+    <mergeCell ref="AE4:AF4"/>
+    <mergeCell ref="AH4:AI4"/>
+    <mergeCell ref="AK4:AL4"/>
+    <mergeCell ref="AN4:AO4"/>
+    <mergeCell ref="AQ4:AR4"/>
+    <mergeCell ref="P4:Q4"/>
+    <mergeCell ref="S4:T4"/>
+    <mergeCell ref="V4:W4"/>
+    <mergeCell ref="Y4:Z4"/>
+    <mergeCell ref="AB4:AC4"/>
     <mergeCell ref="A4:B4"/>
     <mergeCell ref="D4:E4"/>
     <mergeCell ref="G4:H4"/>
     <mergeCell ref="J4:K4"/>
     <mergeCell ref="M4:N4"/>
-    <mergeCell ref="P4:Q4"/>
-    <mergeCell ref="S4:T4"/>
-    <mergeCell ref="V4:W4"/>
-    <mergeCell ref="Y4:Z4"/>
-    <mergeCell ref="AB4:AC4"/>
-    <mergeCell ref="AE4:AF4"/>
-    <mergeCell ref="AH4:AI4"/>
-    <mergeCell ref="AK4:AL4"/>
-    <mergeCell ref="AN4:AO4"/>
-    <mergeCell ref="AQ4:AR4"/>
-    <mergeCell ref="A6:B6"/>
-    <mergeCell ref="D6:E6"/>
-    <mergeCell ref="G6:H6"/>
-    <mergeCell ref="J6:K6"/>
-    <mergeCell ref="M6:N6"/>
-    <mergeCell ref="P6:Q6"/>
-    <mergeCell ref="S6:T6"/>
-    <mergeCell ref="V6:W6"/>
-    <mergeCell ref="Y6:Z6"/>
-    <mergeCell ref="AB6:AC6"/>
-    <mergeCell ref="AE6:AF6"/>
-    <mergeCell ref="AH6:AI6"/>
-    <mergeCell ref="AK6:AL6"/>
-    <mergeCell ref="AN6:AO6"/>
-    <mergeCell ref="AQ6:AR6"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
@@ -15921,74 +15960,74 @@
       </c>
     </row>
     <row r="4" spans="1:44" x14ac:dyDescent="0.2">
-      <c r="A4" s="53" t="s">
+      <c r="A4" s="51" t="s">
         <v>139</v>
       </c>
-      <c r="B4" s="53"/>
-      <c r="D4" s="53" t="s">
+      <c r="B4" s="51"/>
+      <c r="D4" s="51" t="s">
         <v>140</v>
       </c>
-      <c r="E4" s="53"/>
-      <c r="G4" s="53" t="s">
+      <c r="E4" s="51"/>
+      <c r="G4" s="51" t="s">
         <v>141</v>
       </c>
-      <c r="H4" s="53"/>
-      <c r="J4" s="53" t="s">
+      <c r="H4" s="51"/>
+      <c r="J4" s="51" t="s">
         <v>142</v>
       </c>
-      <c r="K4" s="53"/>
-      <c r="M4" s="53" t="s">
+      <c r="K4" s="51"/>
+      <c r="M4" s="51" t="s">
         <v>143</v>
       </c>
-      <c r="N4" s="53"/>
-      <c r="P4" s="53" t="s">
+      <c r="N4" s="51"/>
+      <c r="P4" s="51" t="s">
         <v>144</v>
       </c>
-      <c r="Q4" s="53"/>
+      <c r="Q4" s="51"/>
       <c r="R4" s="1"/>
-      <c r="S4" s="53" t="s">
+      <c r="S4" s="51" t="s">
         <v>145</v>
       </c>
-      <c r="T4" s="53"/>
+      <c r="T4" s="51"/>
       <c r="U4" s="1"/>
-      <c r="V4" s="53" t="s">
+      <c r="V4" s="51" t="s">
         <v>146</v>
       </c>
-      <c r="W4" s="53"/>
+      <c r="W4" s="51"/>
       <c r="X4" s="1"/>
-      <c r="Y4" s="53" t="s">
+      <c r="Y4" s="51" t="s">
         <v>147</v>
       </c>
-      <c r="Z4" s="53"/>
+      <c r="Z4" s="51"/>
       <c r="AA4" s="1"/>
-      <c r="AB4" s="53" t="s">
+      <c r="AB4" s="51" t="s">
         <v>148</v>
       </c>
-      <c r="AC4" s="53"/>
-      <c r="AE4" s="53" t="s">
+      <c r="AC4" s="51"/>
+      <c r="AE4" s="51" t="s">
         <v>149</v>
       </c>
-      <c r="AF4" s="53"/>
+      <c r="AF4" s="51"/>
       <c r="AG4" s="1"/>
-      <c r="AH4" s="53" t="s">
+      <c r="AH4" s="51" t="s">
         <v>150</v>
       </c>
-      <c r="AI4" s="53"/>
+      <c r="AI4" s="51"/>
       <c r="AJ4" s="1"/>
-      <c r="AK4" s="53" t="s">
+      <c r="AK4" s="51" t="s">
         <v>151</v>
       </c>
-      <c r="AL4" s="53"/>
+      <c r="AL4" s="51"/>
       <c r="AM4" s="1"/>
-      <c r="AN4" s="53" t="s">
+      <c r="AN4" s="51" t="s">
         <v>152</v>
       </c>
-      <c r="AO4" s="53"/>
+      <c r="AO4" s="51"/>
       <c r="AP4" s="1"/>
-      <c r="AQ4" s="53" t="s">
+      <c r="AQ4" s="51" t="s">
         <v>153</v>
       </c>
-      <c r="AR4" s="53"/>
+      <c r="AR4" s="51"/>
     </row>
     <row r="5" spans="1:44" x14ac:dyDescent="0.2">
       <c r="A5" s="42" t="s">
@@ -17077,12 +17116,14 @@
     </row>
   </sheetData>
   <mergeCells count="30">
-    <mergeCell ref="P4:Q4"/>
-    <mergeCell ref="A4:B4"/>
-    <mergeCell ref="D4:E4"/>
-    <mergeCell ref="G4:H4"/>
-    <mergeCell ref="J4:K4"/>
-    <mergeCell ref="M4:N4"/>
+    <mergeCell ref="AN6:AO6"/>
+    <mergeCell ref="AQ6:AR6"/>
+    <mergeCell ref="V6:W6"/>
+    <mergeCell ref="Y6:Z6"/>
+    <mergeCell ref="AB6:AC6"/>
+    <mergeCell ref="AE6:AF6"/>
+    <mergeCell ref="AH6:AI6"/>
+    <mergeCell ref="AK6:AL6"/>
     <mergeCell ref="AK4:AL4"/>
     <mergeCell ref="AN4:AO4"/>
     <mergeCell ref="AQ4:AR4"/>
@@ -17099,14 +17140,12 @@
     <mergeCell ref="AB4:AC4"/>
     <mergeCell ref="AE4:AF4"/>
     <mergeCell ref="AH4:AI4"/>
-    <mergeCell ref="AN6:AO6"/>
-    <mergeCell ref="AQ6:AR6"/>
-    <mergeCell ref="V6:W6"/>
-    <mergeCell ref="Y6:Z6"/>
-    <mergeCell ref="AB6:AC6"/>
-    <mergeCell ref="AE6:AF6"/>
-    <mergeCell ref="AH6:AI6"/>
-    <mergeCell ref="AK6:AL6"/>
+    <mergeCell ref="P4:Q4"/>
+    <mergeCell ref="A4:B4"/>
+    <mergeCell ref="D4:E4"/>
+    <mergeCell ref="G4:H4"/>
+    <mergeCell ref="J4:K4"/>
+    <mergeCell ref="M4:N4"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>

<commit_message>
template v16: Norm's mat-sheet reorg — t_cut/E/nu adjacent to strengths, elastic option, color legend (pre CF-fix snapshot)
Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_0147GB4LGVZuqGHCRMVzZTsR
</commit_message>
<xml_diff>
--- a/docs/inputs/input_template.xlsx
+++ b/docs/inputs/input_template.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/njones/python_projects/xslope/docs/inputs/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6E95D610-588A-C249-B900-E3D88174AD4C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{448736C4-E2C8-EB41-827A-888C500BCAB7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="600" windowWidth="38400" windowHeight="19900" xr2:uid="{BA54C293-CE08-6E4C-9212-B3317DAA148E}"/>
   </bookViews>
@@ -62,7 +62,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="443" uniqueCount="235">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="449" uniqueCount="238">
   <si>
     <t>X</t>
   </si>
@@ -305,9 +305,6 @@
     <t>s(f)</t>
   </si>
   <si>
-    <t>Base Values</t>
-  </si>
-  <si>
     <t>Standard Deviations</t>
   </si>
   <si>
@@ -460,9 +457,6 @@
   </si>
   <si>
     <t>XSLOPE Input Template</t>
-  </si>
-  <si>
-    <t>Stress</t>
   </si>
   <si>
     <t>E</t>
@@ -932,6 +926,21 @@
   </si>
   <si>
     <t>Line loads</t>
+  </si>
+  <si>
+    <t>elastic</t>
+  </si>
+  <si>
+    <t>Elastic / infinite strength (cannot fail). FEM: no yield; LEM: impenetrable</t>
+  </si>
+  <si>
+    <t>t_cut</t>
+  </si>
+  <si>
+    <t>Shear Strength/Stiffness</t>
+  </si>
+  <si>
+    <t>Color legend</t>
   </si>
 </sst>
 </file>
@@ -1081,7 +1090,7 @@
       <name val="Aptos Narrow"/>
     </font>
   </fonts>
-  <fills count="17">
+  <fills count="18">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -1144,12 +1153,6 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="FFFF0000"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
         <fgColor theme="7" tint="0.79998168889431442"/>
         <bgColor indexed="64"/>
       </patternFill>
@@ -1175,6 +1178,18 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor theme="3" tint="0.89999084444715716"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="2" tint="-0.499984740745262"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="9" tint="-0.499984740745262"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -1265,7 +1280,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="62">
+  <cellXfs count="63">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -1322,26 +1337,14 @@
     <xf numFmtId="0" fontId="5" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
     <xf numFmtId="0" fontId="13" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="5" fillId="8" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="14" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="9" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="11" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="6" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
@@ -1360,28 +1363,28 @@
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="2" fillId="11" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="11" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
     <xf numFmtId="0" fontId="2" fillId="12" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="15" fillId="12" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="13" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="14" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="15" fillId="13" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="16" fillId="14" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="15" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="16" fillId="15" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="16" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="16" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -1394,13 +1397,16 @@
     <xf numFmtId="0" fontId="20" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="20" fillId="11" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
     <xf numFmtId="0" fontId="4" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="10" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="14" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="14" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
@@ -1410,12 +1416,6 @@
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="15" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="16" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="16" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="7" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
@@ -1433,8 +1433,26 @@
     <xf numFmtId="0" fontId="1" fillId="10" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="14" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="13" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="6" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="6" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="16" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="16" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="17" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="6" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -10394,7 +10412,7 @@
   <sheetData>
     <row r="1" spans="1:7" ht="32" x14ac:dyDescent="0.4">
       <c r="A1" s="7" t="s">
-        <v>97</v>
+        <v>96</v>
       </c>
     </row>
     <row r="3" spans="1:7" ht="19" x14ac:dyDescent="0.25">
@@ -10404,22 +10422,22 @@
     </row>
     <row r="5" spans="1:7" x14ac:dyDescent="0.2">
       <c r="C5" s="14" t="s">
-        <v>79</v>
-      </c>
-      <c r="D5" s="34">
-        <v>15</v>
+        <v>78</v>
+      </c>
+      <c r="D5" s="30">
+        <v>16</v>
       </c>
     </row>
     <row r="7" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="B7" s="49" t="s">
+      <c r="B7" s="44" t="s">
         <v>47</v>
       </c>
-      <c r="C7" s="49"/>
-      <c r="D7" s="49"/>
+      <c r="C7" s="44"/>
+      <c r="D7" s="44"/>
       <c r="F7" s="15" t="s">
         <v>15</v>
       </c>
-      <c r="G7" s="35" t="s">
+      <c r="G7" s="31" t="s">
         <v>16</v>
       </c>
     </row>
@@ -10431,10 +10449,10 @@
         <v>62.4</v>
       </c>
       <c r="F8" s="1" t="s">
-        <v>115</v>
+        <v>113</v>
       </c>
       <c r="G8" t="s">
-        <v>116</v>
+        <v>114</v>
       </c>
     </row>
     <row r="9" spans="1:7" x14ac:dyDescent="0.2">
@@ -10468,16 +10486,16 @@
     <row r="11" spans="1:7" x14ac:dyDescent="0.2">
       <c r="B11" s="1"/>
       <c r="C11" s="14" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="D11" s="1">
         <v>0</v>
       </c>
       <c r="F11" s="1" t="s">
-        <v>229</v>
+        <v>227</v>
       </c>
       <c r="G11" t="s">
-        <v>230</v>
+        <v>228</v>
       </c>
     </row>
     <row r="12" spans="1:7" x14ac:dyDescent="0.2">
@@ -10514,10 +10532,10 @@
     </row>
     <row r="16" spans="1:7" x14ac:dyDescent="0.2">
       <c r="F16" s="1" t="s">
+        <v>115</v>
+      </c>
+      <c r="G16" t="s">
         <v>117</v>
-      </c>
-      <c r="G16" t="s">
-        <v>119</v>
       </c>
     </row>
     <row r="17" spans="2:7" x14ac:dyDescent="0.2">
@@ -10531,34 +10549,34 @@
     </row>
     <row r="18" spans="2:7" x14ac:dyDescent="0.2">
       <c r="F18" s="1" t="s">
-        <v>231</v>
+        <v>229</v>
       </c>
       <c r="G18" t="s">
-        <v>232</v>
+        <v>230</v>
       </c>
     </row>
     <row r="19" spans="2:7" x14ac:dyDescent="0.2">
       <c r="F19" s="1" t="s">
-        <v>233</v>
+        <v>231</v>
       </c>
       <c r="G19" t="s">
-        <v>234</v>
+        <v>232</v>
       </c>
     </row>
     <row r="20" spans="2:7" x14ac:dyDescent="0.2">
       <c r="F20" s="1" t="s">
-        <v>94</v>
+        <v>93</v>
       </c>
       <c r="G20" s="9" t="s">
-        <v>121</v>
+        <v>119</v>
       </c>
     </row>
     <row r="21" spans="2:7" x14ac:dyDescent="0.2">
       <c r="F21" s="1" t="s">
+        <v>116</v>
+      </c>
+      <c r="G21" s="9" t="s">
         <v>118</v>
-      </c>
-      <c r="G21" s="9" t="s">
-        <v>120</v>
       </c>
     </row>
     <row r="23" spans="2:7" x14ac:dyDescent="0.2">
@@ -10595,36 +10613,36 @@
   </cols>
   <sheetData>
     <row r="2" spans="2:24" x14ac:dyDescent="0.2">
-      <c r="B2" s="59" t="s">
+      <c r="B2" s="54" t="s">
+        <v>129</v>
+      </c>
+      <c r="C2" s="54"/>
+      <c r="D2" s="54"/>
+      <c r="F2" s="54" t="s">
+        <v>130</v>
+      </c>
+      <c r="G2" s="54"/>
+      <c r="H2" s="54"/>
+      <c r="J2" s="54" t="s">
         <v>131</v>
       </c>
-      <c r="C2" s="59"/>
-      <c r="D2" s="59"/>
-      <c r="F2" s="59" t="s">
+      <c r="K2" s="54"/>
+      <c r="L2" s="54"/>
+      <c r="N2" s="54" t="s">
         <v>132</v>
       </c>
-      <c r="G2" s="59"/>
-      <c r="H2" s="59"/>
-      <c r="J2" s="59" t="s">
+      <c r="O2" s="54"/>
+      <c r="P2" s="54"/>
+      <c r="R2" s="54" t="s">
         <v>133</v>
       </c>
-      <c r="K2" s="59"/>
-      <c r="L2" s="59"/>
-      <c r="N2" s="59" t="s">
+      <c r="S2" s="54"/>
+      <c r="T2" s="54"/>
+      <c r="V2" s="54" t="s">
         <v>134</v>
       </c>
-      <c r="O2" s="59"/>
-      <c r="P2" s="59"/>
-      <c r="R2" s="59" t="s">
-        <v>135</v>
-      </c>
-      <c r="S2" s="59"/>
-      <c r="T2" s="59"/>
-      <c r="V2" s="59" t="s">
-        <v>136</v>
-      </c>
-      <c r="W2" s="59"/>
-      <c r="X2" s="59"/>
+      <c r="W2" s="54"/>
+      <c r="X2" s="54"/>
     </row>
     <row r="3" spans="2:24" x14ac:dyDescent="0.2">
       <c r="B3" s="2" t="s">
@@ -11093,64 +11111,64 @@
         <v>25</v>
       </c>
       <c r="B2" s="12" t="s">
-        <v>161</v>
+        <v>159</v>
       </c>
       <c r="C2" s="12" t="s">
+        <v>99</v>
+      </c>
+      <c r="D2" s="12" t="s">
+        <v>100</v>
+      </c>
+      <c r="E2" s="12" t="s">
         <v>101</v>
       </c>
-      <c r="D2" s="12" t="s">
+      <c r="F2" s="12" t="s">
         <v>102</v>
       </c>
-      <c r="E2" s="12" t="s">
+      <c r="G2" s="40" t="s">
+        <v>192</v>
+      </c>
+      <c r="H2" s="40" t="s">
+        <v>193</v>
+      </c>
+      <c r="I2" s="40" t="s">
+        <v>177</v>
+      </c>
+      <c r="J2" s="27" t="s">
+        <v>104</v>
+      </c>
+      <c r="K2" s="27" t="s">
+        <v>105</v>
+      </c>
+      <c r="L2" s="27" t="s">
+        <v>106</v>
+      </c>
+      <c r="M2" s="27" t="s">
+        <v>178</v>
+      </c>
+      <c r="N2" s="27" t="s">
+        <v>179</v>
+      </c>
+      <c r="O2" s="27" t="s">
+        <v>194</v>
+      </c>
+      <c r="P2" s="28" t="s">
+        <v>107</v>
+      </c>
+      <c r="Q2" s="28" t="s">
+        <v>97</v>
+      </c>
+      <c r="R2" s="28" t="s">
         <v>103</v>
       </c>
-      <c r="F2" s="12" t="s">
-        <v>104</v>
-      </c>
-      <c r="G2" s="44" t="s">
-        <v>194</v>
-      </c>
-      <c r="H2" s="44" t="s">
-        <v>195</v>
-      </c>
-      <c r="I2" s="44" t="s">
-        <v>179</v>
-      </c>
-      <c r="J2" s="31" t="s">
-        <v>106</v>
-      </c>
-      <c r="K2" s="31" t="s">
-        <v>107</v>
-      </c>
-      <c r="L2" s="31" t="s">
-        <v>108</v>
-      </c>
-      <c r="M2" s="31" t="s">
+      <c r="Z2" t="s">
         <v>180</v>
       </c>
-      <c r="N2" s="31" t="s">
+      <c r="AA2" t="s">
         <v>181</v>
       </c>
-      <c r="O2" s="31" t="s">
-        <v>196</v>
-      </c>
-      <c r="P2" s="32" t="s">
-        <v>109</v>
-      </c>
-      <c r="Q2" s="32" t="s">
-        <v>99</v>
-      </c>
-      <c r="R2" s="32" t="s">
-        <v>105</v>
-      </c>
-      <c r="Z2" t="s">
+      <c r="AB2" t="s">
         <v>182</v>
-      </c>
-      <c r="AA2" t="s">
-        <v>183</v>
-      </c>
-      <c r="AB2" t="s">
-        <v>184</v>
       </c>
     </row>
     <row r="3" spans="1:28" x14ac:dyDescent="0.2">
@@ -11181,13 +11199,13 @@
       <c r="Q3" s="3"/>
       <c r="R3" s="3"/>
       <c r="Z3" t="s">
+        <v>183</v>
+      </c>
+      <c r="AA3" t="s">
+        <v>184</v>
+      </c>
+      <c r="AB3" t="s">
         <v>185</v>
-      </c>
-      <c r="AA3" t="s">
-        <v>186</v>
-      </c>
-      <c r="AB3" t="s">
-        <v>187</v>
       </c>
     </row>
     <row r="4" spans="1:28" x14ac:dyDescent="0.2">
@@ -11218,7 +11236,7 @@
       <c r="Q4" s="3"/>
       <c r="R4" s="3"/>
       <c r="Z4" t="s">
-        <v>188</v>
+        <v>186</v>
       </c>
     </row>
     <row r="5" spans="1:28" x14ac:dyDescent="0.2">
@@ -11249,7 +11267,7 @@
       <c r="Q5" s="3"/>
       <c r="R5" s="3"/>
       <c r="Z5" t="s">
-        <v>189</v>
+        <v>187</v>
       </c>
     </row>
     <row r="6" spans="1:28" x14ac:dyDescent="0.2">
@@ -11336,13 +11354,13 @@
       <c r="Q8" s="3"/>
       <c r="R8" s="3"/>
       <c r="Z8" t="s">
+        <v>180</v>
+      </c>
+      <c r="AA8" t="s">
+        <v>181</v>
+      </c>
+      <c r="AB8" t="s">
         <v>182</v>
-      </c>
-      <c r="AA8" t="s">
-        <v>183</v>
-      </c>
-      <c r="AB8" t="s">
-        <v>184</v>
       </c>
     </row>
     <row r="9" spans="1:28" x14ac:dyDescent="0.2">
@@ -11373,13 +11391,13 @@
       <c r="Q9" s="3"/>
       <c r="R9" s="3"/>
       <c r="Z9" t="s">
+        <v>183</v>
+      </c>
+      <c r="AA9" t="s">
+        <v>184</v>
+      </c>
+      <c r="AB9" t="s">
         <v>185</v>
-      </c>
-      <c r="AA9" t="s">
-        <v>186</v>
-      </c>
-      <c r="AB9" t="s">
-        <v>187</v>
       </c>
     </row>
     <row r="10" spans="1:28" x14ac:dyDescent="0.2">
@@ -11410,13 +11428,13 @@
       <c r="Q10" s="3"/>
       <c r="R10" s="3"/>
       <c r="Z10" t="s">
-        <v>188</v>
+        <v>186</v>
       </c>
       <c r="AA10" t="s">
-        <v>186</v>
+        <v>184</v>
       </c>
       <c r="AB10" t="s">
-        <v>184</v>
+        <v>182</v>
       </c>
     </row>
     <row r="11" spans="1:28" x14ac:dyDescent="0.2">
@@ -11447,13 +11465,13 @@
       <c r="Q11" s="3"/>
       <c r="R11" s="3"/>
       <c r="Z11" t="s">
-        <v>189</v>
+        <v>187</v>
       </c>
       <c r="AA11" t="s">
-        <v>186</v>
+        <v>184</v>
       </c>
       <c r="AB11" t="s">
-        <v>184</v>
+        <v>182</v>
       </c>
     </row>
     <row r="12" spans="1:28" x14ac:dyDescent="0.2">
@@ -11765,25 +11783,25 @@
       <c r="R22" s="3"/>
     </row>
     <row r="23" spans="1:21" x14ac:dyDescent="0.2">
-      <c r="T23" s="46"/>
+      <c r="T23" s="42"/>
       <c r="U23" t="s">
-        <v>163</v>
+        <v>161</v>
       </c>
     </row>
     <row r="24" spans="1:21" x14ac:dyDescent="0.2">
       <c r="K24" s="9"/>
       <c r="L24" s="9"/>
-      <c r="T24" s="30"/>
+      <c r="T24" s="26"/>
       <c r="U24" s="9" t="s">
-        <v>164</v>
+        <v>162</v>
       </c>
     </row>
     <row r="25" spans="1:21" x14ac:dyDescent="0.2">
       <c r="K25" s="9"/>
       <c r="L25" s="9"/>
-      <c r="T25" s="33"/>
+      <c r="T25" s="29"/>
       <c r="U25" s="9" t="s">
-        <v>165</v>
+        <v>163</v>
       </c>
     </row>
   </sheetData>
@@ -11821,58 +11839,58 @@
         <v>25</v>
       </c>
       <c r="B2" s="12" t="s">
-        <v>161</v>
+        <v>159</v>
       </c>
       <c r="C2" s="12" t="s">
+        <v>99</v>
+      </c>
+      <c r="D2" s="12" t="s">
+        <v>100</v>
+      </c>
+      <c r="E2" s="12" t="s">
         <v>101</v>
       </c>
-      <c r="D2" s="12" t="s">
+      <c r="F2" s="12" t="s">
         <v>102</v>
       </c>
-      <c r="E2" s="12" t="s">
+      <c r="G2" s="40" t="s">
+        <v>152</v>
+      </c>
+      <c r="H2" s="40" t="s">
+        <v>160</v>
+      </c>
+      <c r="I2" s="40" t="s">
+        <v>177</v>
+      </c>
+      <c r="J2" s="27" t="s">
+        <v>153</v>
+      </c>
+      <c r="K2" s="27" t="s">
+        <v>154</v>
+      </c>
+      <c r="L2" s="41" t="s">
+        <v>157</v>
+      </c>
+      <c r="M2" s="41" t="s">
+        <v>158</v>
+      </c>
+      <c r="N2" s="28" t="s">
+        <v>97</v>
+      </c>
+      <c r="O2" s="28" t="s">
+        <v>155</v>
+      </c>
+      <c r="P2" s="28" t="s">
         <v>103</v>
       </c>
-      <c r="F2" s="12" t="s">
-        <v>104</v>
-      </c>
-      <c r="G2" s="44" t="s">
-        <v>154</v>
-      </c>
-      <c r="H2" s="44" t="s">
-        <v>162</v>
-      </c>
-      <c r="I2" s="44" t="s">
-        <v>179</v>
-      </c>
-      <c r="J2" s="31" t="s">
-        <v>155</v>
-      </c>
-      <c r="K2" s="31" t="s">
-        <v>156</v>
-      </c>
-      <c r="L2" s="45" t="s">
-        <v>159</v>
-      </c>
-      <c r="M2" s="45" t="s">
-        <v>160</v>
-      </c>
-      <c r="N2" s="32" t="s">
-        <v>99</v>
-      </c>
-      <c r="O2" s="32" t="s">
-        <v>157</v>
-      </c>
-      <c r="P2" s="32" t="s">
-        <v>105</v>
-      </c>
-      <c r="Q2" s="32" t="s">
-        <v>166</v>
+      <c r="Q2" s="28" t="s">
+        <v>164</v>
       </c>
       <c r="Z2" t="s">
         <v>40</v>
       </c>
       <c r="AA2" t="s">
-        <v>184</v>
+        <v>182</v>
       </c>
     </row>
     <row r="3" spans="1:27" x14ac:dyDescent="0.2">
@@ -11896,10 +11914,10 @@
       <c r="P3" s="3"/>
       <c r="Q3" s="3"/>
       <c r="Z3" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="AA3" t="s">
-        <v>187</v>
+        <v>185</v>
       </c>
     </row>
     <row r="4" spans="1:27" x14ac:dyDescent="0.2">
@@ -12100,21 +12118,21 @@
       <c r="K15" s="9"/>
     </row>
     <row r="16" spans="1:27" x14ac:dyDescent="0.2">
-      <c r="S16" s="46"/>
+      <c r="S16" s="42"/>
       <c r="T16" t="s">
+        <v>161</v>
+      </c>
+    </row>
+    <row r="17" spans="19:20" x14ac:dyDescent="0.2">
+      <c r="S17" s="26"/>
+      <c r="T17" s="9" t="s">
+        <v>162</v>
+      </c>
+    </row>
+    <row r="18" spans="19:20" x14ac:dyDescent="0.2">
+      <c r="S18" s="29"/>
+      <c r="T18" s="9" t="s">
         <v>163</v>
-      </c>
-    </row>
-    <row r="17" spans="19:20" x14ac:dyDescent="0.2">
-      <c r="S17" s="30"/>
-      <c r="T17" s="9" t="s">
-        <v>164</v>
-      </c>
-    </row>
-    <row r="18" spans="19:20" x14ac:dyDescent="0.2">
-      <c r="S18" s="33"/>
-      <c r="T18" s="9" t="s">
-        <v>165</v>
       </c>
     </row>
   </sheetData>
@@ -12146,7 +12164,7 @@
         <v>25</v>
       </c>
       <c r="B2" s="12" t="s">
-        <v>161</v>
+        <v>159</v>
       </c>
       <c r="C2" s="12" t="s">
         <v>3</v>
@@ -12155,10 +12173,10 @@
         <v>4</v>
       </c>
       <c r="E2" s="12" t="s">
-        <v>190</v>
+        <v>188</v>
       </c>
       <c r="F2" s="12" t="s">
-        <v>197</v>
+        <v>195</v>
       </c>
     </row>
     <row r="3" spans="1:6" x14ac:dyDescent="0.2">
@@ -12380,100 +12398,100 @@
   </cols>
   <sheetData>
     <row r="2" spans="2:21" x14ac:dyDescent="0.2">
-      <c r="B2" s="60" t="s">
-        <v>129</v>
-      </c>
-      <c r="C2" s="60"/>
-      <c r="E2" s="56" t="s">
+      <c r="B2" s="55" t="s">
+        <v>127</v>
+      </c>
+      <c r="C2" s="55"/>
+      <c r="E2" s="51" t="s">
+        <v>215</v>
+      </c>
+      <c r="F2" s="51"/>
+      <c r="H2" s="51" t="s">
         <v>217</v>
       </c>
-      <c r="F2" s="56"/>
-      <c r="H2" s="56" t="s">
+      <c r="I2" s="51"/>
+      <c r="K2" s="51" t="s">
+        <v>218</v>
+      </c>
+      <c r="L2" s="51"/>
+      <c r="N2" s="51" t="s">
         <v>219</v>
       </c>
-      <c r="I2" s="56"/>
-      <c r="K2" s="56" t="s">
+      <c r="O2" s="51"/>
+      <c r="Q2" s="51" t="s">
         <v>220</v>
       </c>
-      <c r="L2" s="56"/>
-      <c r="N2" s="56" t="s">
-        <v>221</v>
-      </c>
-      <c r="O2" s="56"/>
-      <c r="Q2" s="56" t="s">
-        <v>222</v>
-      </c>
-      <c r="R2" s="56"/>
+      <c r="R2" s="51"/>
     </row>
     <row r="3" spans="2:21" x14ac:dyDescent="0.2">
-      <c r="B3" s="60"/>
-      <c r="C3" s="60"/>
-      <c r="E3" s="36" t="s">
-        <v>215</v>
-      </c>
-      <c r="F3" s="37"/>
-      <c r="H3" s="36" t="s">
-        <v>215</v>
-      </c>
-      <c r="I3" s="37"/>
-      <c r="K3" s="36" t="s">
-        <v>215</v>
-      </c>
-      <c r="L3" s="37"/>
-      <c r="N3" s="36" t="s">
-        <v>215</v>
-      </c>
-      <c r="O3" s="37"/>
-      <c r="Q3" s="36" t="s">
-        <v>215</v>
-      </c>
-      <c r="R3" s="37"/>
+      <c r="B3" s="55"/>
+      <c r="C3" s="55"/>
+      <c r="E3" s="32" t="s">
+        <v>213</v>
+      </c>
+      <c r="F3" s="33"/>
+      <c r="H3" s="32" t="s">
+        <v>213</v>
+      </c>
+      <c r="I3" s="33"/>
+      <c r="K3" s="32" t="s">
+        <v>213</v>
+      </c>
+      <c r="L3" s="33"/>
+      <c r="N3" s="32" t="s">
+        <v>213</v>
+      </c>
+      <c r="O3" s="33"/>
+      <c r="Q3" s="32" t="s">
+        <v>213</v>
+      </c>
+      <c r="R3" s="33"/>
       <c r="T3" s="6" t="s">
-        <v>214</v>
+        <v>212</v>
       </c>
     </row>
     <row r="4" spans="2:21" x14ac:dyDescent="0.2">
-      <c r="B4" s="28" t="s">
+      <c r="B4" s="25" t="s">
         <v>3</v>
       </c>
-      <c r="C4" s="28" t="s">
+      <c r="C4" s="25" t="s">
         <v>4</v>
       </c>
-      <c r="E4" s="28" t="s">
+      <c r="E4" s="25" t="s">
         <v>3</v>
       </c>
-      <c r="F4" s="28" t="s">
+      <c r="F4" s="25" t="s">
         <v>4</v>
       </c>
-      <c r="H4" s="28" t="s">
+      <c r="H4" s="25" t="s">
         <v>3</v>
       </c>
-      <c r="I4" s="28" t="s">
+      <c r="I4" s="25" t="s">
         <v>4</v>
       </c>
-      <c r="K4" s="28" t="s">
+      <c r="K4" s="25" t="s">
         <v>3</v>
       </c>
-      <c r="L4" s="28" t="s">
+      <c r="L4" s="25" t="s">
         <v>4</v>
       </c>
-      <c r="N4" s="28" t="s">
+      <c r="N4" s="25" t="s">
         <v>3</v>
       </c>
-      <c r="O4" s="28" t="s">
+      <c r="O4" s="25" t="s">
         <v>4</v>
       </c>
-      <c r="Q4" s="28" t="s">
+      <c r="Q4" s="25" t="s">
         <v>3</v>
       </c>
-      <c r="R4" s="28" t="s">
+      <c r="R4" s="25" t="s">
         <v>4</v>
       </c>
       <c r="T4" s="1" t="s">
-        <v>215</v>
+        <v>213</v>
       </c>
       <c r="U4" t="s">
-        <v>218</v>
+        <v>216</v>
       </c>
     </row>
     <row r="5" spans="2:21" x14ac:dyDescent="0.2">
@@ -12490,10 +12508,10 @@
       <c r="Q5" s="3"/>
       <c r="R5" s="3"/>
       <c r="T5" s="1" t="s">
-        <v>216</v>
+        <v>214</v>
       </c>
       <c r="U5" t="s">
-        <v>228</v>
+        <v>226</v>
       </c>
     </row>
     <row r="6" spans="2:21" x14ac:dyDescent="0.2">
@@ -12796,100 +12814,100 @@
   </cols>
   <sheetData>
     <row r="2" spans="2:21" x14ac:dyDescent="0.2">
-      <c r="B2" s="61" t="s">
-        <v>130</v>
-      </c>
-      <c r="C2" s="61"/>
-      <c r="E2" s="57" t="s">
+      <c r="B2" s="56" t="s">
+        <v>128</v>
+      </c>
+      <c r="C2" s="56"/>
+      <c r="E2" s="52" t="s">
+        <v>221</v>
+      </c>
+      <c r="F2" s="52"/>
+      <c r="H2" s="52" t="s">
+        <v>222</v>
+      </c>
+      <c r="I2" s="52"/>
+      <c r="K2" s="52" t="s">
         <v>223</v>
       </c>
-      <c r="F2" s="57"/>
-      <c r="H2" s="57" t="s">
+      <c r="L2" s="52"/>
+      <c r="N2" s="52" t="s">
         <v>224</v>
       </c>
-      <c r="I2" s="57"/>
-      <c r="K2" s="57" t="s">
+      <c r="O2" s="52"/>
+      <c r="Q2" s="52" t="s">
         <v>225</v>
       </c>
-      <c r="L2" s="57"/>
-      <c r="N2" s="57" t="s">
-        <v>226</v>
-      </c>
-      <c r="O2" s="57"/>
-      <c r="Q2" s="57" t="s">
-        <v>227</v>
-      </c>
-      <c r="R2" s="57"/>
+      <c r="R2" s="52"/>
     </row>
     <row r="3" spans="2:21" x14ac:dyDescent="0.2">
-      <c r="B3" s="61"/>
-      <c r="C3" s="61"/>
-      <c r="E3" s="38" t="s">
-        <v>215</v>
-      </c>
-      <c r="F3" s="39"/>
-      <c r="H3" s="38" t="s">
-        <v>215</v>
-      </c>
-      <c r="I3" s="39"/>
-      <c r="K3" s="38" t="s">
-        <v>215</v>
-      </c>
-      <c r="L3" s="39"/>
-      <c r="N3" s="38" t="s">
-        <v>215</v>
-      </c>
-      <c r="O3" s="39"/>
-      <c r="Q3" s="38" t="s">
-        <v>215</v>
-      </c>
-      <c r="R3" s="39"/>
+      <c r="B3" s="56"/>
+      <c r="C3" s="56"/>
+      <c r="E3" s="34" t="s">
+        <v>213</v>
+      </c>
+      <c r="F3" s="35"/>
+      <c r="H3" s="34" t="s">
+        <v>213</v>
+      </c>
+      <c r="I3" s="35"/>
+      <c r="K3" s="34" t="s">
+        <v>213</v>
+      </c>
+      <c r="L3" s="35"/>
+      <c r="N3" s="34" t="s">
+        <v>213</v>
+      </c>
+      <c r="O3" s="35"/>
+      <c r="Q3" s="34" t="s">
+        <v>213</v>
+      </c>
+      <c r="R3" s="35"/>
       <c r="T3" s="6" t="s">
-        <v>214</v>
+        <v>212</v>
       </c>
     </row>
     <row r="4" spans="2:21" x14ac:dyDescent="0.2">
-      <c r="B4" s="28" t="s">
+      <c r="B4" s="25" t="s">
         <v>3</v>
       </c>
-      <c r="C4" s="28" t="s">
+      <c r="C4" s="25" t="s">
         <v>4</v>
       </c>
-      <c r="E4" s="28" t="s">
+      <c r="E4" s="25" t="s">
         <v>3</v>
       </c>
-      <c r="F4" s="28" t="s">
+      <c r="F4" s="25" t="s">
         <v>4</v>
       </c>
-      <c r="H4" s="28" t="s">
+      <c r="H4" s="25" t="s">
         <v>3</v>
       </c>
-      <c r="I4" s="28" t="s">
+      <c r="I4" s="25" t="s">
         <v>4</v>
       </c>
-      <c r="K4" s="28" t="s">
+      <c r="K4" s="25" t="s">
         <v>3</v>
       </c>
-      <c r="L4" s="28" t="s">
+      <c r="L4" s="25" t="s">
         <v>4</v>
       </c>
-      <c r="N4" s="28" t="s">
+      <c r="N4" s="25" t="s">
         <v>3</v>
       </c>
-      <c r="O4" s="28" t="s">
+      <c r="O4" s="25" t="s">
         <v>4</v>
       </c>
-      <c r="Q4" s="28" t="s">
+      <c r="Q4" s="25" t="s">
         <v>3</v>
       </c>
-      <c r="R4" s="28" t="s">
+      <c r="R4" s="25" t="s">
         <v>4</v>
       </c>
       <c r="T4" s="1" t="s">
-        <v>215</v>
+        <v>213</v>
       </c>
       <c r="U4" t="s">
-        <v>218</v>
+        <v>216</v>
       </c>
     </row>
     <row r="5" spans="2:21" x14ac:dyDescent="0.2">
@@ -12906,10 +12924,10 @@
       <c r="Q5" s="3"/>
       <c r="R5" s="3"/>
       <c r="T5" s="1" t="s">
-        <v>216</v>
+        <v>214</v>
       </c>
       <c r="U5" t="s">
-        <v>228</v>
+        <v>226</v>
       </c>
     </row>
     <row r="6" spans="2:21" x14ac:dyDescent="0.2">
@@ -13208,318 +13226,301 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{60A900FC-A692-B445-95C9-59E70352B291}">
-  <dimension ref="A2:AK51"/>
+  <dimension ref="A2:AL52"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="7" style="1" customWidth="1"/>
     <col min="2" max="2" width="17.33203125" style="1" customWidth="1"/>
     <col min="3" max="10" width="8.5" style="1" customWidth="1"/>
-    <col min="11" max="35" width="8.5" customWidth="1"/>
-    <col min="36" max="36" width="8.5" style="1" customWidth="1"/>
-    <col min="37" max="37" width="8.5" customWidth="1"/>
+    <col min="11" max="38" width="8.5" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="2" spans="1:37" x14ac:dyDescent="0.2">
+    <row r="2" spans="1:38" x14ac:dyDescent="0.2">
       <c r="C2" s="6" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="E2"/>
       <c r="F2"/>
       <c r="G2"/>
-      <c r="K2" s="6" t="s">
-        <v>172</v>
-      </c>
-      <c r="Y2" s="6"/>
-      <c r="AE2" s="6" t="s">
-        <v>171</v>
-      </c>
-    </row>
-    <row r="3" spans="1:37" x14ac:dyDescent="0.2">
+      <c r="L2" s="6" t="s">
+        <v>237</v>
+      </c>
+      <c r="O2" s="6" t="s">
+        <v>170</v>
+      </c>
+      <c r="AB2" s="6"/>
+      <c r="AH2" s="6" t="s">
+        <v>169</v>
+      </c>
+    </row>
+    <row r="3" spans="1:38" x14ac:dyDescent="0.2">
       <c r="C3" s="1" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="D3" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="F3"/>
       <c r="G3"/>
-      <c r="K3" s="1" t="s">
-        <v>87</v>
-      </c>
-      <c r="L3" t="s">
-        <v>59</v>
-      </c>
-      <c r="Y3" s="14"/>
-      <c r="AE3" s="1" t="s">
+      <c r="O3" s="1" t="s">
+        <v>86</v>
+      </c>
+      <c r="P3" t="s">
+        <v>58</v>
+      </c>
+      <c r="AB3" s="14"/>
+      <c r="AH3" s="1" t="s">
+        <v>166</v>
+      </c>
+      <c r="AI3" t="s">
         <v>168</v>
       </c>
-      <c r="AF3" t="s">
-        <v>170</v>
-      </c>
-    </row>
-    <row r="4" spans="1:37" x14ac:dyDescent="0.2">
+    </row>
+    <row r="4" spans="1:38" x14ac:dyDescent="0.2">
       <c r="C4" s="1" t="s">
+        <v>69</v>
+      </c>
+      <c r="D4" t="s">
         <v>70</v>
-      </c>
-      <c r="D4" t="s">
-        <v>71</v>
       </c>
       <c r="F4"/>
       <c r="G4"/>
-      <c r="K4" s="1" t="s">
+      <c r="L4" s="42"/>
+      <c r="M4" t="s">
+        <v>161</v>
+      </c>
+      <c r="O4" s="1" t="s">
         <v>21</v>
       </c>
-      <c r="L4" t="s">
-        <v>60</v>
-      </c>
-      <c r="Y4" s="14"/>
-      <c r="AE4" s="1" t="s">
-        <v>169</v>
-      </c>
-      <c r="AF4" t="s">
+      <c r="P4" t="s">
+        <v>59</v>
+      </c>
+      <c r="AB4" s="14"/>
+      <c r="AH4" s="1" t="s">
+        <v>167</v>
+      </c>
+      <c r="AI4" t="s">
+        <v>204</v>
+      </c>
+    </row>
+    <row r="5" spans="1:38" x14ac:dyDescent="0.2">
+      <c r="C5" s="1" t="s">
+        <v>171</v>
+      </c>
+      <c r="D5" t="s">
+        <v>191</v>
+      </c>
+      <c r="L5" s="26"/>
+      <c r="M5" s="9" t="s">
+        <v>162</v>
+      </c>
+      <c r="O5" s="1" t="s">
+        <v>87</v>
+      </c>
+      <c r="P5" s="9" t="s">
+        <v>85</v>
+      </c>
+      <c r="AB5" s="14"/>
+      <c r="AH5" s="1" t="s">
+        <v>202</v>
+      </c>
+      <c r="AI5" s="9" t="s">
+        <v>203</v>
+      </c>
+    </row>
+    <row r="6" spans="1:38" x14ac:dyDescent="0.2">
+      <c r="C6" s="1" t="s">
+        <v>201</v>
+      </c>
+      <c r="D6" s="9" t="s">
+        <v>207</v>
+      </c>
+      <c r="L6" s="29"/>
+      <c r="M6" s="9" t="s">
+        <v>163</v>
+      </c>
+      <c r="O6" s="1" t="s">
+        <v>172</v>
+      </c>
+      <c r="P6" t="s">
+        <v>190</v>
+      </c>
+      <c r="AC6" s="1"/>
+      <c r="AD6" s="1"/>
+    </row>
+    <row r="7" spans="1:38" x14ac:dyDescent="0.2">
+      <c r="C7" s="1" t="s">
+        <v>233</v>
+      </c>
+      <c r="D7" s="9" t="s">
+        <v>234</v>
+      </c>
+      <c r="AC7" s="1"/>
+      <c r="AD7" s="1"/>
+    </row>
+    <row r="9" spans="1:38" x14ac:dyDescent="0.2">
+      <c r="C9" s="45" t="s">
+        <v>236</v>
+      </c>
+      <c r="D9" s="45"/>
+      <c r="E9" s="45"/>
+      <c r="F9" s="45"/>
+      <c r="G9" s="45"/>
+      <c r="H9" s="45"/>
+      <c r="I9" s="45"/>
+      <c r="J9" s="45"/>
+      <c r="K9" s="45"/>
+      <c r="L9" s="45"/>
+      <c r="M9" s="45"/>
+      <c r="N9" s="45"/>
+      <c r="O9" s="45"/>
+      <c r="P9" s="45"/>
+      <c r="Q9" s="45"/>
+      <c r="R9" s="45"/>
+      <c r="S9" s="45"/>
+      <c r="T9" s="45"/>
+      <c r="U9" s="45"/>
+      <c r="V9" s="45"/>
+      <c r="W9" s="45"/>
+      <c r="X9" s="45"/>
+      <c r="Y9" s="45" t="s">
+        <v>57</v>
+      </c>
+      <c r="Z9" s="45"/>
+      <c r="AA9" s="45"/>
+      <c r="AB9" s="45"/>
+      <c r="AC9" s="45"/>
+      <c r="AD9" s="45"/>
+      <c r="AE9" s="45" t="s">
+        <v>91</v>
+      </c>
+      <c r="AF9" s="45"/>
+      <c r="AG9" s="45"/>
+      <c r="AH9" s="45"/>
+      <c r="AI9" s="45"/>
+      <c r="AJ9" s="45"/>
+      <c r="AK9" s="45"/>
+      <c r="AL9" s="45"/>
+    </row>
+    <row r="10" spans="1:38" ht="18" x14ac:dyDescent="0.25">
+      <c r="A10" s="20" t="s">
+        <v>19</v>
+      </c>
+      <c r="B10" s="20" t="s">
+        <v>77</v>
+      </c>
+      <c r="C10" s="58" t="s">
+        <v>52</v>
+      </c>
+      <c r="D10" s="62" t="s">
+        <v>189</v>
+      </c>
+      <c r="E10" s="57" t="s">
+        <v>65</v>
+      </c>
+      <c r="F10" s="57" t="s">
+        <v>53</v>
+      </c>
+      <c r="G10" s="58" t="s">
+        <v>51</v>
+      </c>
+      <c r="H10" s="57" t="s">
+        <v>72</v>
+      </c>
+      <c r="I10" s="57" t="s">
+        <v>71</v>
+      </c>
+      <c r="J10" s="61" t="s">
+        <v>79</v>
+      </c>
+      <c r="K10" s="61" t="s">
+        <v>135</v>
+      </c>
+      <c r="L10" s="57" t="s">
+        <v>235</v>
+      </c>
+      <c r="M10" s="21" t="s">
+        <v>97</v>
+      </c>
+      <c r="N10" s="43" t="s">
+        <v>211</v>
+      </c>
+      <c r="O10" s="57" t="s">
+        <v>84</v>
+      </c>
+      <c r="P10" s="57" t="s">
+        <v>172</v>
+      </c>
+      <c r="Q10" s="57" t="s">
+        <v>173</v>
+      </c>
+      <c r="R10" s="57" t="s">
+        <v>174</v>
+      </c>
+      <c r="S10" s="57" t="s">
+        <v>175</v>
+      </c>
+      <c r="T10" s="57" t="s">
+        <v>176</v>
+      </c>
+      <c r="U10" s="57" t="s">
         <v>206</v>
       </c>
-    </row>
-    <row r="5" spans="1:37" x14ac:dyDescent="0.2">
-      <c r="C5" s="1" t="s">
-        <v>173</v>
-      </c>
-      <c r="D5" t="s">
-        <v>193</v>
-      </c>
-      <c r="K5" s="1" t="s">
+      <c r="V10" s="57" t="s">
+        <v>208</v>
+      </c>
+      <c r="W10" s="57" t="s">
+        <v>209</v>
+      </c>
+      <c r="X10" s="57" t="s">
+        <v>210</v>
+      </c>
+      <c r="Y10" s="59" t="s">
+        <v>54</v>
+      </c>
+      <c r="Z10" s="59" t="s">
+        <v>55</v>
+      </c>
+      <c r="AA10" s="60" t="s">
+        <v>56</v>
+      </c>
+      <c r="AB10" s="59" t="s">
+        <v>73</v>
+      </c>
+      <c r="AC10" s="59" t="s">
+        <v>80</v>
+      </c>
+      <c r="AD10" s="60" t="s">
+        <v>136</v>
+      </c>
+      <c r="AE10" s="23" t="s">
         <v>88</v>
       </c>
-      <c r="L5" s="9" t="s">
-        <v>86</v>
-      </c>
-      <c r="Y5" s="14"/>
-      <c r="AE5" s="1" t="s">
-        <v>204</v>
-      </c>
-      <c r="AF5" s="9" t="s">
+      <c r="AF10" s="23" t="s">
+        <v>89</v>
+      </c>
+      <c r="AG10" s="23" t="s">
+        <v>90</v>
+      </c>
+      <c r="AH10" s="23" t="s">
+        <v>165</v>
+      </c>
+      <c r="AI10" s="23" t="s">
+        <v>94</v>
+      </c>
+      <c r="AJ10" s="23" t="s">
+        <v>95</v>
+      </c>
+      <c r="AK10" s="23" t="s">
         <v>205</v>
       </c>
-    </row>
-    <row r="6" spans="1:37" x14ac:dyDescent="0.2">
-      <c r="C6" s="1" t="s">
-        <v>203</v>
-      </c>
-      <c r="D6" s="9" t="s">
-        <v>209</v>
-      </c>
-      <c r="K6" s="1" t="s">
-        <v>174</v>
-      </c>
-      <c r="L6" t="s">
-        <v>192</v>
-      </c>
-      <c r="T6" s="1"/>
-      <c r="Z6" s="1"/>
-      <c r="AA6" s="1"/>
-    </row>
-    <row r="8" spans="1:37" x14ac:dyDescent="0.2">
-      <c r="C8" s="50" t="s">
-        <v>57</v>
-      </c>
-      <c r="D8" s="50"/>
-      <c r="E8" s="50"/>
-      <c r="F8" s="50"/>
-      <c r="G8" s="50"/>
-      <c r="H8" s="50"/>
-      <c r="I8" s="50"/>
-      <c r="J8" s="50"/>
-      <c r="K8" s="50"/>
-      <c r="L8" s="50"/>
-      <c r="M8" s="50"/>
-      <c r="N8" s="50"/>
-      <c r="O8" s="50"/>
-      <c r="P8" s="50"/>
-      <c r="Q8" s="50"/>
-      <c r="R8" s="50"/>
-      <c r="S8" s="50"/>
-      <c r="T8" s="50"/>
-      <c r="U8" s="50"/>
-      <c r="V8" s="50" t="s">
-        <v>58</v>
-      </c>
-      <c r="W8" s="50"/>
-      <c r="X8" s="50"/>
-      <c r="Y8" s="50"/>
-      <c r="Z8" s="50"/>
-      <c r="AA8" s="50"/>
-      <c r="AB8" s="50" t="s">
-        <v>92</v>
-      </c>
-      <c r="AC8" s="50"/>
-      <c r="AD8" s="50"/>
-      <c r="AE8" s="50"/>
-      <c r="AF8" s="50"/>
-      <c r="AG8" s="50"/>
-      <c r="AH8" s="50"/>
-      <c r="AI8" s="50"/>
-      <c r="AJ8" s="50" t="s">
+      <c r="AL10" s="23" t="s">
         <v>98</v>
       </c>
-      <c r="AK8" s="50"/>
-    </row>
-    <row r="9" spans="1:37" ht="18" x14ac:dyDescent="0.25">
-      <c r="A9" s="20" t="s">
-        <v>19</v>
-      </c>
-      <c r="B9" s="20" t="s">
-        <v>78</v>
-      </c>
-      <c r="C9" s="26" t="s">
-        <v>52</v>
-      </c>
-      <c r="D9" s="47" t="s">
-        <v>191</v>
-      </c>
-      <c r="E9" s="21" t="s">
-        <v>66</v>
-      </c>
-      <c r="F9" s="21" t="s">
-        <v>53</v>
-      </c>
-      <c r="G9" s="26" t="s">
-        <v>51</v>
-      </c>
-      <c r="H9" s="21" t="s">
-        <v>73</v>
-      </c>
-      <c r="I9" s="21" t="s">
-        <v>72</v>
-      </c>
-      <c r="J9" s="21" t="s">
-        <v>80</v>
-      </c>
-      <c r="K9" s="21" t="s">
-        <v>137</v>
-      </c>
-      <c r="L9" s="21" t="s">
-        <v>175</v>
-      </c>
-      <c r="M9" s="21" t="s">
-        <v>176</v>
-      </c>
-      <c r="N9" s="21" t="s">
-        <v>177</v>
-      </c>
-      <c r="O9" s="21" t="s">
-        <v>178</v>
-      </c>
-      <c r="P9" s="21" t="s">
-        <v>208</v>
-      </c>
-      <c r="Q9" s="21" t="s">
-        <v>210</v>
-      </c>
-      <c r="R9" s="21" t="s">
-        <v>211</v>
-      </c>
-      <c r="S9" s="21" t="s">
-        <v>212</v>
-      </c>
-      <c r="T9" s="21" t="s">
-        <v>85</v>
-      </c>
-      <c r="U9" s="21" t="s">
-        <v>174</v>
-      </c>
-      <c r="V9" s="22" t="s">
-        <v>54</v>
-      </c>
-      <c r="W9" s="22" t="s">
-        <v>55</v>
-      </c>
-      <c r="X9" s="23" t="s">
-        <v>56</v>
-      </c>
-      <c r="Y9" s="22" t="s">
-        <v>74</v>
-      </c>
-      <c r="Z9" s="22" t="s">
-        <v>81</v>
-      </c>
-      <c r="AA9" s="23" t="s">
-        <v>138</v>
-      </c>
-      <c r="AB9" s="25" t="s">
-        <v>89</v>
-      </c>
-      <c r="AC9" s="25" t="s">
-        <v>90</v>
-      </c>
-      <c r="AD9" s="25" t="s">
-        <v>91</v>
-      </c>
-      <c r="AE9" s="25" t="s">
-        <v>167</v>
-      </c>
-      <c r="AF9" s="25" t="s">
-        <v>95</v>
-      </c>
-      <c r="AG9" s="25" t="s">
-        <v>96</v>
-      </c>
-      <c r="AH9" s="25" t="s">
-        <v>207</v>
-      </c>
-      <c r="AI9" s="25" t="s">
-        <v>100</v>
-      </c>
-      <c r="AJ9" s="29" t="s">
-        <v>99</v>
-      </c>
-      <c r="AK9" s="48" t="s">
-        <v>213</v>
-      </c>
-    </row>
-    <row r="10" spans="1:37" x14ac:dyDescent="0.2">
-      <c r="A10" s="3">
+    </row>
+    <row r="11" spans="1:38" x14ac:dyDescent="0.2">
+      <c r="A11" s="3">
         <v>1</v>
-      </c>
-      <c r="B10" s="3"/>
-      <c r="C10" s="3"/>
-      <c r="D10" s="3"/>
-      <c r="E10" s="3"/>
-      <c r="F10" s="3"/>
-      <c r="G10" s="3"/>
-      <c r="H10" s="3"/>
-      <c r="I10" s="3"/>
-      <c r="J10" s="3"/>
-      <c r="K10" s="3"/>
-      <c r="L10" s="3"/>
-      <c r="M10" s="3"/>
-      <c r="N10" s="3"/>
-      <c r="O10" s="3"/>
-      <c r="P10" s="3"/>
-      <c r="Q10" s="3"/>
-      <c r="R10" s="3"/>
-      <c r="S10" s="3"/>
-      <c r="T10" s="3"/>
-      <c r="U10" s="3"/>
-      <c r="V10" s="3"/>
-      <c r="W10" s="3"/>
-      <c r="X10" s="3"/>
-      <c r="Y10" s="3"/>
-      <c r="Z10" s="3"/>
-      <c r="AA10" s="3"/>
-      <c r="AB10" s="3"/>
-      <c r="AC10" s="3"/>
-      <c r="AD10" s="3"/>
-      <c r="AE10" s="3"/>
-      <c r="AF10" s="3"/>
-      <c r="AG10" s="3"/>
-      <c r="AH10" s="3"/>
-      <c r="AI10" s="3"/>
-      <c r="AJ10" s="3"/>
-      <c r="AK10" s="3"/>
-    </row>
-    <row r="11" spans="1:37" x14ac:dyDescent="0.2">
-      <c r="A11" s="3">
-        <v>2</v>
       </c>
       <c r="B11" s="3"/>
       <c r="C11" s="3"/>
@@ -13553,14 +13554,15 @@
       <c r="AE11" s="3"/>
       <c r="AF11" s="3"/>
       <c r="AG11" s="3"/>
-      <c r="AH11" s="18"/>
-      <c r="AI11" s="19"/>
+      <c r="AH11" s="3"/>
+      <c r="AI11" s="3"/>
       <c r="AJ11" s="3"/>
       <c r="AK11" s="3"/>
-    </row>
-    <row r="12" spans="1:37" x14ac:dyDescent="0.2">
+      <c r="AL11" s="3"/>
+    </row>
+    <row r="12" spans="1:38" x14ac:dyDescent="0.2">
       <c r="A12" s="3">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="B12" s="3"/>
       <c r="C12" s="3"/>
@@ -13594,14 +13596,15 @@
       <c r="AE12" s="3"/>
       <c r="AF12" s="3"/>
       <c r="AG12" s="3"/>
-      <c r="AH12" s="18"/>
-      <c r="AI12" s="19"/>
+      <c r="AH12" s="3"/>
+      <c r="AI12" s="3"/>
       <c r="AJ12" s="3"/>
-      <c r="AK12" s="3"/>
-    </row>
-    <row r="13" spans="1:37" x14ac:dyDescent="0.2">
+      <c r="AK12" s="18"/>
+      <c r="AL12" s="19"/>
+    </row>
+    <row r="13" spans="1:38" x14ac:dyDescent="0.2">
       <c r="A13" s="3">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="B13" s="3"/>
       <c r="C13" s="3"/>
@@ -13638,11 +13641,12 @@
       <c r="AH13" s="3"/>
       <c r="AI13" s="3"/>
       <c r="AJ13" s="3"/>
-      <c r="AK13" s="3"/>
-    </row>
-    <row r="14" spans="1:37" x14ac:dyDescent="0.2">
+      <c r="AK13" s="18"/>
+      <c r="AL13" s="19"/>
+    </row>
+    <row r="14" spans="1:38" x14ac:dyDescent="0.2">
       <c r="A14" s="3">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="B14" s="3"/>
       <c r="C14" s="3"/>
@@ -13680,10 +13684,11 @@
       <c r="AI14" s="3"/>
       <c r="AJ14" s="3"/>
       <c r="AK14" s="3"/>
-    </row>
-    <row r="15" spans="1:37" x14ac:dyDescent="0.2">
+      <c r="AL14" s="3"/>
+    </row>
+    <row r="15" spans="1:38" x14ac:dyDescent="0.2">
       <c r="A15" s="3">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="B15" s="3"/>
       <c r="C15" s="3"/>
@@ -13721,10 +13726,11 @@
       <c r="AI15" s="3"/>
       <c r="AJ15" s="3"/>
       <c r="AK15" s="3"/>
-    </row>
-    <row r="16" spans="1:37" x14ac:dyDescent="0.2">
+      <c r="AL15" s="3"/>
+    </row>
+    <row r="16" spans="1:38" x14ac:dyDescent="0.2">
       <c r="A16" s="3">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="B16" s="3"/>
       <c r="C16" s="3"/>
@@ -13762,10 +13768,11 @@
       <c r="AI16" s="3"/>
       <c r="AJ16" s="3"/>
       <c r="AK16" s="3"/>
-    </row>
-    <row r="17" spans="1:37" x14ac:dyDescent="0.2">
+      <c r="AL16" s="3"/>
+    </row>
+    <row r="17" spans="1:38" x14ac:dyDescent="0.2">
       <c r="A17" s="3">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="B17" s="3"/>
       <c r="C17" s="3"/>
@@ -13803,10 +13810,11 @@
       <c r="AI17" s="3"/>
       <c r="AJ17" s="3"/>
       <c r="AK17" s="3"/>
-    </row>
-    <row r="18" spans="1:37" x14ac:dyDescent="0.2">
+      <c r="AL17" s="3"/>
+    </row>
+    <row r="18" spans="1:38" x14ac:dyDescent="0.2">
       <c r="A18" s="3">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="B18" s="3"/>
       <c r="C18" s="3"/>
@@ -13844,10 +13852,11 @@
       <c r="AI18" s="3"/>
       <c r="AJ18" s="3"/>
       <c r="AK18" s="3"/>
-    </row>
-    <row r="19" spans="1:37" x14ac:dyDescent="0.2">
+      <c r="AL18" s="3"/>
+    </row>
+    <row r="19" spans="1:38" x14ac:dyDescent="0.2">
       <c r="A19" s="3">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="B19" s="3"/>
       <c r="C19" s="3"/>
@@ -13885,10 +13894,11 @@
       <c r="AI19" s="3"/>
       <c r="AJ19" s="3"/>
       <c r="AK19" s="3"/>
-    </row>
-    <row r="20" spans="1:37" x14ac:dyDescent="0.2">
+      <c r="AL19" s="3"/>
+    </row>
+    <row r="20" spans="1:38" x14ac:dyDescent="0.2">
       <c r="A20" s="3">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="B20" s="3"/>
       <c r="C20" s="3"/>
@@ -13926,10 +13936,11 @@
       <c r="AI20" s="3"/>
       <c r="AJ20" s="3"/>
       <c r="AK20" s="3"/>
-    </row>
-    <row r="21" spans="1:37" x14ac:dyDescent="0.2">
+      <c r="AL20" s="3"/>
+    </row>
+    <row r="21" spans="1:38" x14ac:dyDescent="0.2">
       <c r="A21" s="3">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="B21" s="3"/>
       <c r="C21" s="3"/>
@@ -13967,10 +13978,11 @@
       <c r="AI21" s="3"/>
       <c r="AJ21" s="3"/>
       <c r="AK21" s="3"/>
-    </row>
-    <row r="22" spans="1:37" x14ac:dyDescent="0.2">
+      <c r="AL21" s="3"/>
+    </row>
+    <row r="22" spans="1:38" x14ac:dyDescent="0.2">
       <c r="A22" s="3">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="B22" s="3"/>
       <c r="C22" s="3"/>
@@ -14008,10 +14020,11 @@
       <c r="AI22" s="3"/>
       <c r="AJ22" s="3"/>
       <c r="AK22" s="3"/>
-    </row>
-    <row r="23" spans="1:37" x14ac:dyDescent="0.2">
+      <c r="AL22" s="3"/>
+    </row>
+    <row r="23" spans="1:38" x14ac:dyDescent="0.2">
       <c r="A23" s="3">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="B23" s="3"/>
       <c r="C23" s="3"/>
@@ -14049,10 +14062,11 @@
       <c r="AI23" s="3"/>
       <c r="AJ23" s="3"/>
       <c r="AK23" s="3"/>
-    </row>
-    <row r="24" spans="1:37" x14ac:dyDescent="0.2">
+      <c r="AL23" s="3"/>
+    </row>
+    <row r="24" spans="1:38" x14ac:dyDescent="0.2">
       <c r="A24" s="3">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="B24" s="3"/>
       <c r="C24" s="3"/>
@@ -14090,35 +14104,51 @@
       <c r="AI24" s="3"/>
       <c r="AJ24" s="3"/>
       <c r="AK24" s="3"/>
-    </row>
-    <row r="25" spans="1:37" x14ac:dyDescent="0.2">
-      <c r="K25" s="1"/>
-      <c r="L25" s="1"/>
-      <c r="M25" s="1"/>
-      <c r="N25" s="1"/>
-      <c r="O25" s="1"/>
-      <c r="P25" s="1"/>
-      <c r="Q25" s="1"/>
-      <c r="R25" s="1"/>
-      <c r="S25" s="1"/>
-      <c r="T25" s="1"/>
-      <c r="U25" s="1"/>
-      <c r="V25" s="1"/>
-      <c r="W25" s="1"/>
-      <c r="X25" s="1"/>
-      <c r="Y25" s="1"/>
-      <c r="Z25" s="1"/>
-      <c r="AA25" s="1"/>
-      <c r="AB25" s="1"/>
-      <c r="AC25" s="1"/>
-      <c r="AD25" s="1"/>
-      <c r="AE25" s="1"/>
-      <c r="AF25" s="1"/>
-      <c r="AG25" s="1"/>
-      <c r="AH25" s="1"/>
-      <c r="AI25" s="1"/>
-    </row>
-    <row r="26" spans="1:37" x14ac:dyDescent="0.2">
+      <c r="AL24" s="3"/>
+    </row>
+    <row r="25" spans="1:38" x14ac:dyDescent="0.2">
+      <c r="A25" s="3">
+        <v>15</v>
+      </c>
+      <c r="B25" s="3"/>
+      <c r="C25" s="3"/>
+      <c r="D25" s="3"/>
+      <c r="E25" s="3"/>
+      <c r="F25" s="3"/>
+      <c r="G25" s="3"/>
+      <c r="H25" s="3"/>
+      <c r="I25" s="3"/>
+      <c r="J25" s="3"/>
+      <c r="K25" s="3"/>
+      <c r="L25" s="3"/>
+      <c r="M25" s="3"/>
+      <c r="N25" s="3"/>
+      <c r="O25" s="3"/>
+      <c r="P25" s="3"/>
+      <c r="Q25" s="3"/>
+      <c r="R25" s="3"/>
+      <c r="S25" s="3"/>
+      <c r="T25" s="3"/>
+      <c r="U25" s="3"/>
+      <c r="V25" s="3"/>
+      <c r="W25" s="3"/>
+      <c r="X25" s="3"/>
+      <c r="Y25" s="3"/>
+      <c r="Z25" s="3"/>
+      <c r="AA25" s="3"/>
+      <c r="AB25" s="3"/>
+      <c r="AC25" s="3"/>
+      <c r="AD25" s="3"/>
+      <c r="AE25" s="3"/>
+      <c r="AF25" s="3"/>
+      <c r="AG25" s="3"/>
+      <c r="AH25" s="3"/>
+      <c r="AI25" s="3"/>
+      <c r="AJ25" s="3"/>
+      <c r="AK25" s="3"/>
+      <c r="AL25" s="3"/>
+    </row>
+    <row r="26" spans="1:38" x14ac:dyDescent="0.2">
       <c r="K26" s="1"/>
       <c r="L26" s="1"/>
       <c r="M26" s="1"/>
@@ -14136,8 +14166,19 @@
       <c r="Y26" s="1"/>
       <c r="Z26" s="1"/>
       <c r="AA26" s="1"/>
-    </row>
-    <row r="27" spans="1:37" x14ac:dyDescent="0.2">
+      <c r="AB26" s="1"/>
+      <c r="AC26" s="1"/>
+      <c r="AD26" s="1"/>
+      <c r="AE26" s="1"/>
+      <c r="AF26" s="1"/>
+      <c r="AG26" s="1"/>
+      <c r="AH26" s="1"/>
+      <c r="AI26" s="1"/>
+      <c r="AJ26" s="1"/>
+      <c r="AK26" s="1"/>
+      <c r="AL26" s="1"/>
+    </row>
+    <row r="27" spans="1:38" x14ac:dyDescent="0.2">
       <c r="K27" s="1"/>
       <c r="L27" s="1"/>
       <c r="M27" s="1"/>
@@ -14155,8 +14196,11 @@
       <c r="Y27" s="1"/>
       <c r="Z27" s="1"/>
       <c r="AA27" s="1"/>
-    </row>
-    <row r="28" spans="1:37" x14ac:dyDescent="0.2">
+      <c r="AB27" s="1"/>
+      <c r="AC27" s="1"/>
+      <c r="AD27" s="1"/>
+    </row>
+    <row r="28" spans="1:38" x14ac:dyDescent="0.2">
       <c r="K28" s="1"/>
       <c r="L28" s="1"/>
       <c r="M28" s="1"/>
@@ -14174,8 +14218,11 @@
       <c r="Y28" s="1"/>
       <c r="Z28" s="1"/>
       <c r="AA28" s="1"/>
-    </row>
-    <row r="29" spans="1:37" x14ac:dyDescent="0.2">
+      <c r="AB28" s="1"/>
+      <c r="AC28" s="1"/>
+      <c r="AD28" s="1"/>
+    </row>
+    <row r="29" spans="1:38" x14ac:dyDescent="0.2">
       <c r="K29" s="1"/>
       <c r="L29" s="1"/>
       <c r="M29" s="1"/>
@@ -14193,8 +14240,11 @@
       <c r="Y29" s="1"/>
       <c r="Z29" s="1"/>
       <c r="AA29" s="1"/>
-    </row>
-    <row r="30" spans="1:37" x14ac:dyDescent="0.2">
+      <c r="AB29" s="1"/>
+      <c r="AC29" s="1"/>
+      <c r="AD29" s="1"/>
+    </row>
+    <row r="30" spans="1:38" x14ac:dyDescent="0.2">
       <c r="K30" s="1"/>
       <c r="L30" s="1"/>
       <c r="M30" s="1"/>
@@ -14212,8 +14262,11 @@
       <c r="Y30" s="1"/>
       <c r="Z30" s="1"/>
       <c r="AA30" s="1"/>
-    </row>
-    <row r="31" spans="1:37" x14ac:dyDescent="0.2">
+      <c r="AB30" s="1"/>
+      <c r="AC30" s="1"/>
+      <c r="AD30" s="1"/>
+    </row>
+    <row r="31" spans="1:38" x14ac:dyDescent="0.2">
       <c r="K31" s="1"/>
       <c r="L31" s="1"/>
       <c r="M31" s="1"/>
@@ -14231,8 +14284,11 @@
       <c r="Y31" s="1"/>
       <c r="Z31" s="1"/>
       <c r="AA31" s="1"/>
-    </row>
-    <row r="32" spans="1:37" x14ac:dyDescent="0.2">
+      <c r="AB31" s="1"/>
+      <c r="AC31" s="1"/>
+      <c r="AD31" s="1"/>
+    </row>
+    <row r="32" spans="1:38" x14ac:dyDescent="0.2">
       <c r="K32" s="1"/>
       <c r="L32" s="1"/>
       <c r="M32" s="1"/>
@@ -14250,8 +14306,11 @@
       <c r="Y32" s="1"/>
       <c r="Z32" s="1"/>
       <c r="AA32" s="1"/>
-    </row>
-    <row r="33" spans="11:27" x14ac:dyDescent="0.2">
+      <c r="AB32" s="1"/>
+      <c r="AC32" s="1"/>
+      <c r="AD32" s="1"/>
+    </row>
+    <row r="33" spans="11:30" x14ac:dyDescent="0.2">
       <c r="K33" s="1"/>
       <c r="L33" s="1"/>
       <c r="M33" s="1"/>
@@ -14269,8 +14328,11 @@
       <c r="Y33" s="1"/>
       <c r="Z33" s="1"/>
       <c r="AA33" s="1"/>
-    </row>
-    <row r="34" spans="11:27" x14ac:dyDescent="0.2">
+      <c r="AB33" s="1"/>
+      <c r="AC33" s="1"/>
+      <c r="AD33" s="1"/>
+    </row>
+    <row r="34" spans="11:30" x14ac:dyDescent="0.2">
       <c r="K34" s="1"/>
       <c r="L34" s="1"/>
       <c r="M34" s="1"/>
@@ -14288,8 +14350,11 @@
       <c r="Y34" s="1"/>
       <c r="Z34" s="1"/>
       <c r="AA34" s="1"/>
-    </row>
-    <row r="35" spans="11:27" x14ac:dyDescent="0.2">
+      <c r="AB34" s="1"/>
+      <c r="AC34" s="1"/>
+      <c r="AD34" s="1"/>
+    </row>
+    <row r="35" spans="11:30" x14ac:dyDescent="0.2">
       <c r="K35" s="1"/>
       <c r="L35" s="1"/>
       <c r="M35" s="1"/>
@@ -14307,8 +14372,11 @@
       <c r="Y35" s="1"/>
       <c r="Z35" s="1"/>
       <c r="AA35" s="1"/>
-    </row>
-    <row r="36" spans="11:27" x14ac:dyDescent="0.2">
+      <c r="AB35" s="1"/>
+      <c r="AC35" s="1"/>
+      <c r="AD35" s="1"/>
+    </row>
+    <row r="36" spans="11:30" x14ac:dyDescent="0.2">
       <c r="K36" s="1"/>
       <c r="L36" s="1"/>
       <c r="M36" s="1"/>
@@ -14326,8 +14394,11 @@
       <c r="Y36" s="1"/>
       <c r="Z36" s="1"/>
       <c r="AA36" s="1"/>
-    </row>
-    <row r="37" spans="11:27" x14ac:dyDescent="0.2">
+      <c r="AB36" s="1"/>
+      <c r="AC36" s="1"/>
+      <c r="AD36" s="1"/>
+    </row>
+    <row r="37" spans="11:30" x14ac:dyDescent="0.2">
       <c r="K37" s="1"/>
       <c r="L37" s="1"/>
       <c r="M37" s="1"/>
@@ -14345,8 +14416,11 @@
       <c r="Y37" s="1"/>
       <c r="Z37" s="1"/>
       <c r="AA37" s="1"/>
-    </row>
-    <row r="38" spans="11:27" x14ac:dyDescent="0.2">
+      <c r="AB37" s="1"/>
+      <c r="AC37" s="1"/>
+      <c r="AD37" s="1"/>
+    </row>
+    <row r="38" spans="11:30" x14ac:dyDescent="0.2">
       <c r="K38" s="1"/>
       <c r="L38" s="1"/>
       <c r="M38" s="1"/>
@@ -14364,8 +14438,11 @@
       <c r="Y38" s="1"/>
       <c r="Z38" s="1"/>
       <c r="AA38" s="1"/>
-    </row>
-    <row r="39" spans="11:27" x14ac:dyDescent="0.2">
+      <c r="AB38" s="1"/>
+      <c r="AC38" s="1"/>
+      <c r="AD38" s="1"/>
+    </row>
+    <row r="39" spans="11:30" x14ac:dyDescent="0.2">
       <c r="K39" s="1"/>
       <c r="L39" s="1"/>
       <c r="M39" s="1"/>
@@ -14383,8 +14460,11 @@
       <c r="Y39" s="1"/>
       <c r="Z39" s="1"/>
       <c r="AA39" s="1"/>
-    </row>
-    <row r="40" spans="11:27" x14ac:dyDescent="0.2">
+      <c r="AB39" s="1"/>
+      <c r="AC39" s="1"/>
+      <c r="AD39" s="1"/>
+    </row>
+    <row r="40" spans="11:30" x14ac:dyDescent="0.2">
       <c r="K40" s="1"/>
       <c r="L40" s="1"/>
       <c r="M40" s="1"/>
@@ -14402,8 +14482,11 @@
       <c r="Y40" s="1"/>
       <c r="Z40" s="1"/>
       <c r="AA40" s="1"/>
-    </row>
-    <row r="41" spans="11:27" x14ac:dyDescent="0.2">
+      <c r="AB40" s="1"/>
+      <c r="AC40" s="1"/>
+      <c r="AD40" s="1"/>
+    </row>
+    <row r="41" spans="11:30" x14ac:dyDescent="0.2">
       <c r="K41" s="1"/>
       <c r="L41" s="1"/>
       <c r="M41" s="1"/>
@@ -14421,8 +14504,11 @@
       <c r="Y41" s="1"/>
       <c r="Z41" s="1"/>
       <c r="AA41" s="1"/>
-    </row>
-    <row r="42" spans="11:27" x14ac:dyDescent="0.2">
+      <c r="AB41" s="1"/>
+      <c r="AC41" s="1"/>
+      <c r="AD41" s="1"/>
+    </row>
+    <row r="42" spans="11:30" x14ac:dyDescent="0.2">
       <c r="K42" s="1"/>
       <c r="L42" s="1"/>
       <c r="M42" s="1"/>
@@ -14440,8 +14526,11 @@
       <c r="Y42" s="1"/>
       <c r="Z42" s="1"/>
       <c r="AA42" s="1"/>
-    </row>
-    <row r="43" spans="11:27" x14ac:dyDescent="0.2">
+      <c r="AB42" s="1"/>
+      <c r="AC42" s="1"/>
+      <c r="AD42" s="1"/>
+    </row>
+    <row r="43" spans="11:30" x14ac:dyDescent="0.2">
       <c r="K43" s="1"/>
       <c r="L43" s="1"/>
       <c r="M43" s="1"/>
@@ -14459,8 +14548,11 @@
       <c r="Y43" s="1"/>
       <c r="Z43" s="1"/>
       <c r="AA43" s="1"/>
-    </row>
-    <row r="44" spans="11:27" x14ac:dyDescent="0.2">
+      <c r="AB43" s="1"/>
+      <c r="AC43" s="1"/>
+      <c r="AD43" s="1"/>
+    </row>
+    <row r="44" spans="11:30" x14ac:dyDescent="0.2">
       <c r="K44" s="1"/>
       <c r="L44" s="1"/>
       <c r="M44" s="1"/>
@@ -14478,8 +14570,11 @@
       <c r="Y44" s="1"/>
       <c r="Z44" s="1"/>
       <c r="AA44" s="1"/>
-    </row>
-    <row r="45" spans="11:27" x14ac:dyDescent="0.2">
+      <c r="AB44" s="1"/>
+      <c r="AC44" s="1"/>
+      <c r="AD44" s="1"/>
+    </row>
+    <row r="45" spans="11:30" x14ac:dyDescent="0.2">
       <c r="K45" s="1"/>
       <c r="L45" s="1"/>
       <c r="M45" s="1"/>
@@ -14497,8 +14592,11 @@
       <c r="Y45" s="1"/>
       <c r="Z45" s="1"/>
       <c r="AA45" s="1"/>
-    </row>
-    <row r="46" spans="11:27" x14ac:dyDescent="0.2">
+      <c r="AB45" s="1"/>
+      <c r="AC45" s="1"/>
+      <c r="AD45" s="1"/>
+    </row>
+    <row r="46" spans="11:30" x14ac:dyDescent="0.2">
       <c r="K46" s="1"/>
       <c r="L46" s="1"/>
       <c r="M46" s="1"/>
@@ -14516,8 +14614,11 @@
       <c r="Y46" s="1"/>
       <c r="Z46" s="1"/>
       <c r="AA46" s="1"/>
-    </row>
-    <row r="47" spans="11:27" x14ac:dyDescent="0.2">
+      <c r="AB46" s="1"/>
+      <c r="AC46" s="1"/>
+      <c r="AD46" s="1"/>
+    </row>
+    <row r="47" spans="11:30" x14ac:dyDescent="0.2">
       <c r="K47" s="1"/>
       <c r="L47" s="1"/>
       <c r="M47" s="1"/>
@@ -14535,8 +14636,11 @@
       <c r="Y47" s="1"/>
       <c r="Z47" s="1"/>
       <c r="AA47" s="1"/>
-    </row>
-    <row r="48" spans="11:27" x14ac:dyDescent="0.2">
+      <c r="AB47" s="1"/>
+      <c r="AC47" s="1"/>
+      <c r="AD47" s="1"/>
+    </row>
+    <row r="48" spans="11:30" x14ac:dyDescent="0.2">
       <c r="K48" s="1"/>
       <c r="L48" s="1"/>
       <c r="M48" s="1"/>
@@ -14554,8 +14658,11 @@
       <c r="Y48" s="1"/>
       <c r="Z48" s="1"/>
       <c r="AA48" s="1"/>
-    </row>
-    <row r="49" spans="11:27" x14ac:dyDescent="0.2">
+      <c r="AB48" s="1"/>
+      <c r="AC48" s="1"/>
+      <c r="AD48" s="1"/>
+    </row>
+    <row r="49" spans="11:30" x14ac:dyDescent="0.2">
       <c r="K49" s="1"/>
       <c r="L49" s="1"/>
       <c r="M49" s="1"/>
@@ -14573,8 +14680,11 @@
       <c r="Y49" s="1"/>
       <c r="Z49" s="1"/>
       <c r="AA49" s="1"/>
-    </row>
-    <row r="50" spans="11:27" x14ac:dyDescent="0.2">
+      <c r="AB49" s="1"/>
+      <c r="AC49" s="1"/>
+      <c r="AD49" s="1"/>
+    </row>
+    <row r="50" spans="11:30" x14ac:dyDescent="0.2">
       <c r="K50" s="1"/>
       <c r="L50" s="1"/>
       <c r="M50" s="1"/>
@@ -14592,8 +14702,11 @@
       <c r="Y50" s="1"/>
       <c r="Z50" s="1"/>
       <c r="AA50" s="1"/>
-    </row>
-    <row r="51" spans="11:27" x14ac:dyDescent="0.2">
+      <c r="AB50" s="1"/>
+      <c r="AC50" s="1"/>
+      <c r="AD50" s="1"/>
+    </row>
+    <row r="51" spans="11:30" x14ac:dyDescent="0.2">
       <c r="K51" s="1"/>
       <c r="L51" s="1"/>
       <c r="M51" s="1"/>
@@ -14611,88 +14724,107 @@
       <c r="Y51" s="1"/>
       <c r="Z51" s="1"/>
       <c r="AA51" s="1"/>
+      <c r="AB51" s="1"/>
+      <c r="AC51" s="1"/>
+      <c r="AD51" s="1"/>
+    </row>
+    <row r="52" spans="11:30" x14ac:dyDescent="0.2">
+      <c r="K52" s="1"/>
+      <c r="L52" s="1"/>
+      <c r="M52" s="1"/>
+      <c r="N52" s="1"/>
+      <c r="O52" s="1"/>
+      <c r="P52" s="1"/>
+      <c r="Q52" s="1"/>
+      <c r="R52" s="1"/>
+      <c r="S52" s="1"/>
+      <c r="T52" s="1"/>
+      <c r="U52" s="1"/>
+      <c r="V52" s="1"/>
+      <c r="W52" s="1"/>
+      <c r="X52" s="1"/>
+      <c r="Y52" s="1"/>
+      <c r="Z52" s="1"/>
+      <c r="AA52" s="1"/>
+      <c r="AB52" s="1"/>
+      <c r="AC52" s="1"/>
+      <c r="AD52" s="1"/>
     </row>
   </sheetData>
-  <mergeCells count="4">
-    <mergeCell ref="V8:AA8"/>
-    <mergeCell ref="AJ8:AK8"/>
-    <mergeCell ref="AB8:AI8"/>
-    <mergeCell ref="C8:U8"/>
+  <mergeCells count="3">
+    <mergeCell ref="Y9:AD9"/>
+    <mergeCell ref="AE9:AL9"/>
+    <mergeCell ref="C9:X9"/>
   </mergeCells>
-  <conditionalFormatting sqref="F10:K51 W10:AA51">
+  <conditionalFormatting sqref="F51:P52 Z11:AD52 F11:L25 F26:N50 P26:P50">
     <cfRule type="expression" dxfId="15" priority="2">
-      <formula>$E10="hb"</formula>
+      <formula>$E11="hb"</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="G10:G51">
+  <conditionalFormatting sqref="G11:G52">
     <cfRule type="expression" dxfId="14" priority="7">
-      <formula>$E10="cp"</formula>
+      <formula>$E11="cp"</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="H10:I51">
+  <conditionalFormatting sqref="H11:I52">
     <cfRule type="expression" dxfId="13" priority="6">
-      <formula>$E10="mc"</formula>
+      <formula>$E11="mc"</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="J10:K51">
+  <conditionalFormatting sqref="J51:P52 J11:L25 J26:N50 P26:P50">
     <cfRule type="expression" dxfId="12" priority="8">
-      <formula>$E10="cp"</formula>
+      <formula>$E11="cp"</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="L10:O51">
+  <conditionalFormatting sqref="Q11:T52">
     <cfRule type="expression" dxfId="11" priority="21">
-      <formula>AND($E10&lt;&gt;"",$E10&lt;&gt;"pow")</formula>
+      <formula>AND($E11&lt;&gt;"",$E11&lt;&gt;"pow")</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="P10:S51">
+  <conditionalFormatting sqref="U11:X52">
     <cfRule type="expression" dxfId="10" priority="1">
-      <formula>AND($E10&lt;&gt;"",$E10&lt;&gt;"hb")</formula>
+      <formula>AND($E11&lt;&gt;"",$E11&lt;&gt;"hb")</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="U10:U51">
-    <cfRule type="expression" dxfId="9" priority="22">
-      <formula>AND($T10&lt;&gt;"",$T10&lt;&gt;"ru")</formula>
+  <conditionalFormatting sqref="Z11:AD52 F51:P52 F11:L25 F26:N50 P26:P50">
+    <cfRule type="expression" dxfId="8" priority="18">
+      <formula>$E11="pow"</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="W10:AA51 F10:K51">
-    <cfRule type="expression" dxfId="8" priority="18">
-      <formula>$E10="pow"</formula>
+  <conditionalFormatting sqref="AA11:AA52">
+    <cfRule type="expression" dxfId="7" priority="10">
+      <formula>$E11="cp"</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="X10:X51">
-    <cfRule type="expression" dxfId="7" priority="10">
-      <formula>$E10="cp"</formula>
+  <conditionalFormatting sqref="AB11:AB52">
+    <cfRule type="expression" dxfId="6" priority="17">
+      <formula>$E11="mc"</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="Y10:Y51">
-    <cfRule type="expression" dxfId="6" priority="17">
-      <formula>$E10="mc"</formula>
+  <conditionalFormatting sqref="AC11:AD52">
+    <cfRule type="expression" dxfId="5" priority="12">
+      <formula>$E11="cp"</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="Z10:AA51">
-    <cfRule type="expression" dxfId="5" priority="12">
-      <formula>$E10="cp"</formula>
+  <conditionalFormatting sqref="AI11:AJ102">
+    <cfRule type="expression" dxfId="4" priority="4">
+      <formula>OR($AH11="vg",$AH11="gard")</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="AF10:AG101">
-    <cfRule type="expression" dxfId="4" priority="4">
-      <formula>OR($AE10="vg",$AE10="gard")</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="AH10:AI101">
+  <conditionalFormatting sqref="AK11:AL102">
     <cfRule type="expression" dxfId="3" priority="3">
-      <formula>$AE10="lf"</formula>
+      <formula>$AH11="lf"</formula>
     </cfRule>
   </conditionalFormatting>
   <dataValidations count="3">
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="E10:E51" xr:uid="{374AFD2C-B540-DD4B-A245-8B781F76E64C}">
-      <formula1>$C$3:$C$6</formula1>
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="E11:E52" xr:uid="{374AFD2C-B540-DD4B-A245-8B781F76E64C}">
+      <formula1>$C$3:$C$7</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="T10:T51" xr:uid="{D770415C-1ECE-F44B-9D8C-08EF1CF31C8E}">
-      <formula1>$K$3:$K$6</formula1>
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="AH11:AH102" xr:uid="{E00A94A9-D864-5843-8FBD-E84775B1C100}">
+      <formula1>$AH$3:$AH$5</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="AE10:AE101" xr:uid="{E00A94A9-D864-5843-8FBD-E84775B1C100}">
-      <formula1>$AE$3:$AE$5</formula1>
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="O11:O50" xr:uid="{D770415C-1ECE-F44B-9D8C-08EF1CF31C8E}">
+      <formula1>$O$3:$O$6</formula1>
     </dataValidation>
   </dataValidations>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -14732,264 +14864,264 @@
       <c r="B2" s="3">
         <v>0</v>
       </c>
-      <c r="D2" s="27" t="s">
-        <v>93</v>
+      <c r="D2" s="24" t="s">
+        <v>92</v>
       </c>
     </row>
     <row r="4" spans="1:44" x14ac:dyDescent="0.2">
-      <c r="A4" s="51" t="s">
+      <c r="A4" s="48" t="s">
         <v>2</v>
       </c>
-      <c r="B4" s="51"/>
-      <c r="D4" s="51" t="s">
+      <c r="B4" s="48"/>
+      <c r="D4" s="48" t="s">
         <v>5</v>
       </c>
-      <c r="E4" s="51"/>
-      <c r="G4" s="51" t="s">
+      <c r="E4" s="48"/>
+      <c r="G4" s="48" t="s">
         <v>6</v>
       </c>
-      <c r="H4" s="51"/>
-      <c r="J4" s="51" t="s">
+      <c r="H4" s="48"/>
+      <c r="J4" s="48" t="s">
         <v>7</v>
       </c>
-      <c r="K4" s="51"/>
-      <c r="M4" s="51" t="s">
+      <c r="K4" s="48"/>
+      <c r="M4" s="48" t="s">
         <v>8</v>
       </c>
-      <c r="N4" s="51"/>
-      <c r="P4" s="51" t="s">
+      <c r="N4" s="48"/>
+      <c r="P4" s="48" t="s">
         <v>9</v>
       </c>
-      <c r="Q4" s="51"/>
+      <c r="Q4" s="48"/>
       <c r="R4" s="1"/>
-      <c r="S4" s="51" t="s">
+      <c r="S4" s="48" t="s">
         <v>10</v>
       </c>
-      <c r="T4" s="51"/>
+      <c r="T4" s="48"/>
       <c r="U4" s="1"/>
-      <c r="V4" s="51" t="s">
+      <c r="V4" s="48" t="s">
         <v>11</v>
       </c>
-      <c r="W4" s="51"/>
+      <c r="W4" s="48"/>
       <c r="X4" s="1"/>
-      <c r="Y4" s="51" t="s">
+      <c r="Y4" s="48" t="s">
         <v>12</v>
       </c>
-      <c r="Z4" s="51"/>
+      <c r="Z4" s="48"/>
       <c r="AA4" s="1"/>
-      <c r="AB4" s="51" t="s">
+      <c r="AB4" s="48" t="s">
         <v>13</v>
       </c>
-      <c r="AC4" s="51"/>
-      <c r="AE4" s="51" t="s">
+      <c r="AC4" s="48"/>
+      <c r="AE4" s="48" t="s">
+        <v>108</v>
+      </c>
+      <c r="AF4" s="48"/>
+      <c r="AG4" s="1"/>
+      <c r="AH4" s="48" t="s">
+        <v>109</v>
+      </c>
+      <c r="AI4" s="48"/>
+      <c r="AJ4" s="1"/>
+      <c r="AK4" s="48" t="s">
         <v>110</v>
       </c>
-      <c r="AF4" s="51"/>
-      <c r="AG4" s="1"/>
-      <c r="AH4" s="51" t="s">
+      <c r="AL4" s="48"/>
+      <c r="AM4" s="1"/>
+      <c r="AN4" s="48" t="s">
         <v>111</v>
       </c>
-      <c r="AI4" s="51"/>
-      <c r="AJ4" s="1"/>
-      <c r="AK4" s="51" t="s">
+      <c r="AO4" s="48"/>
+      <c r="AP4" s="1"/>
+      <c r="AQ4" s="48" t="s">
         <v>112</v>
       </c>
-      <c r="AL4" s="51"/>
-      <c r="AM4" s="1"/>
-      <c r="AN4" s="51" t="s">
-        <v>113</v>
-      </c>
-      <c r="AO4" s="51"/>
-      <c r="AP4" s="1"/>
-      <c r="AQ4" s="51" t="s">
-        <v>114</v>
-      </c>
-      <c r="AR4" s="51"/>
+      <c r="AR4" s="48"/>
     </row>
     <row r="5" spans="1:44" x14ac:dyDescent="0.2">
-      <c r="A5" s="40" t="s">
-        <v>122</v>
-      </c>
-      <c r="B5" s="41">
+      <c r="A5" s="36" t="s">
+        <v>120</v>
+      </c>
+      <c r="B5" s="37">
         <v>1</v>
       </c>
-      <c r="D5" s="40" t="s">
-        <v>122</v>
-      </c>
-      <c r="E5" s="41">
+      <c r="D5" s="36" t="s">
+        <v>120</v>
+      </c>
+      <c r="E5" s="37">
         <v>2</v>
       </c>
-      <c r="G5" s="40" t="s">
-        <v>122</v>
-      </c>
-      <c r="H5" s="41">
+      <c r="G5" s="36" t="s">
+        <v>120</v>
+      </c>
+      <c r="H5" s="37">
         <v>3</v>
       </c>
-      <c r="J5" s="40" t="s">
-        <v>122</v>
-      </c>
-      <c r="K5" s="41">
+      <c r="J5" s="36" t="s">
+        <v>120</v>
+      </c>
+      <c r="K5" s="37">
         <v>4</v>
       </c>
-      <c r="M5" s="40" t="s">
-        <v>122</v>
-      </c>
-      <c r="N5" s="41">
+      <c r="M5" s="36" t="s">
+        <v>120</v>
+      </c>
+      <c r="N5" s="37">
         <v>5</v>
       </c>
-      <c r="P5" s="40" t="s">
-        <v>122</v>
-      </c>
-      <c r="Q5" s="41">
+      <c r="P5" s="36" t="s">
+        <v>120</v>
+      </c>
+      <c r="Q5" s="37">
         <v>6</v>
       </c>
       <c r="R5" s="1"/>
-      <c r="S5" s="40" t="s">
-        <v>122</v>
-      </c>
-      <c r="T5" s="41">
+      <c r="S5" s="36" t="s">
+        <v>120</v>
+      </c>
+      <c r="T5" s="37">
         <v>7</v>
       </c>
       <c r="U5" s="1"/>
-      <c r="V5" s="40" t="s">
-        <v>122</v>
-      </c>
-      <c r="W5" s="41">
+      <c r="V5" s="36" t="s">
+        <v>120</v>
+      </c>
+      <c r="W5" s="37">
         <v>8</v>
       </c>
       <c r="X5" s="1"/>
-      <c r="Y5" s="40" t="s">
-        <v>122</v>
-      </c>
-      <c r="Z5" s="41">
+      <c r="Y5" s="36" t="s">
+        <v>120</v>
+      </c>
+      <c r="Z5" s="37">
         <v>9</v>
       </c>
       <c r="AA5" s="1"/>
-      <c r="AB5" s="40" t="s">
-        <v>122</v>
-      </c>
-      <c r="AC5" s="41">
+      <c r="AB5" s="36" t="s">
+        <v>120</v>
+      </c>
+      <c r="AC5" s="37">
         <v>10</v>
       </c>
-      <c r="AE5" s="40" t="s">
-        <v>122</v>
-      </c>
-      <c r="AF5" s="41">
+      <c r="AE5" s="36" t="s">
+        <v>120</v>
+      </c>
+      <c r="AF5" s="37">
         <v>11</v>
       </c>
       <c r="AG5" s="1"/>
-      <c r="AH5" s="40" t="s">
-        <v>122</v>
-      </c>
-      <c r="AI5" s="41">
+      <c r="AH5" s="36" t="s">
+        <v>120</v>
+      </c>
+      <c r="AI5" s="37">
         <v>12</v>
       </c>
       <c r="AJ5" s="1"/>
-      <c r="AK5" s="40" t="s">
-        <v>122</v>
-      </c>
-      <c r="AL5" s="41">
+      <c r="AK5" s="36" t="s">
+        <v>120</v>
+      </c>
+      <c r="AL5" s="37">
         <v>13</v>
       </c>
       <c r="AM5" s="1"/>
-      <c r="AN5" s="40" t="s">
-        <v>122</v>
-      </c>
-      <c r="AO5" s="41">
+      <c r="AN5" s="36" t="s">
+        <v>120</v>
+      </c>
+      <c r="AO5" s="37">
         <v>14</v>
       </c>
       <c r="AP5" s="1"/>
-      <c r="AQ5" s="40" t="s">
-        <v>122</v>
-      </c>
-      <c r="AR5" s="41">
+      <c r="AQ5" s="36" t="s">
+        <v>120</v>
+      </c>
+      <c r="AR5" s="37">
         <v>15</v>
       </c>
     </row>
     <row r="6" spans="1:44" x14ac:dyDescent="0.2">
-      <c r="A6" s="52" t="str">
+      <c r="A6" s="46" t="str">
         <f>_xlfn.XLOOKUP(B5,mat!$A:$A, mat!$B:$B,"") &amp; ""</f>
         <v/>
       </c>
-      <c r="B6" s="53"/>
-      <c r="D6" s="52" t="str">
+      <c r="B6" s="47"/>
+      <c r="D6" s="46" t="str">
         <f>_xlfn.XLOOKUP(E5,mat!$A:$A, mat!$B:$B,"") &amp; ""</f>
         <v/>
       </c>
-      <c r="E6" s="53"/>
-      <c r="G6" s="52" t="str">
+      <c r="E6" s="47"/>
+      <c r="G6" s="46" t="str">
         <f>_xlfn.XLOOKUP(H5,mat!$A:$A, mat!$B:$B,"") &amp; ""</f>
         <v/>
       </c>
-      <c r="H6" s="53"/>
-      <c r="J6" s="52" t="str">
+      <c r="H6" s="47"/>
+      <c r="J6" s="46" t="str">
         <f>_xlfn.XLOOKUP(K5,mat!$A:$A, mat!$B:$B,"") &amp; ""</f>
         <v/>
       </c>
-      <c r="K6" s="53"/>
-      <c r="M6" s="52" t="str">
+      <c r="K6" s="47"/>
+      <c r="M6" s="46" t="str">
         <f>_xlfn.XLOOKUP(N5,mat!$A:$A, mat!$B:$B,"") &amp; ""</f>
         <v/>
       </c>
-      <c r="N6" s="53"/>
-      <c r="P6" s="52" t="str">
+      <c r="N6" s="47"/>
+      <c r="P6" s="46" t="str">
         <f>_xlfn.XLOOKUP(Q5,mat!$A:$A, mat!$B:$B,"") &amp; ""</f>
         <v/>
       </c>
-      <c r="Q6" s="53"/>
+      <c r="Q6" s="47"/>
       <c r="R6" s="1"/>
-      <c r="S6" s="52" t="str">
+      <c r="S6" s="46" t="str">
         <f>_xlfn.XLOOKUP(T5,mat!$A:$A, mat!$B:$B,"") &amp; ""</f>
         <v/>
       </c>
-      <c r="T6" s="53"/>
+      <c r="T6" s="47"/>
       <c r="U6" s="1"/>
-      <c r="V6" s="52" t="str">
+      <c r="V6" s="46" t="str">
         <f>_xlfn.XLOOKUP(W5,mat!$A:$A, mat!$B:$B,"") &amp; ""</f>
         <v/>
       </c>
-      <c r="W6" s="53"/>
+      <c r="W6" s="47"/>
       <c r="X6" s="1"/>
-      <c r="Y6" s="52" t="str">
+      <c r="Y6" s="46" t="str">
         <f>_xlfn.XLOOKUP(Z5,mat!$A:$A, mat!$B:$B,"") &amp; ""</f>
         <v/>
       </c>
-      <c r="Z6" s="53"/>
+      <c r="Z6" s="47"/>
       <c r="AA6" s="1"/>
-      <c r="AB6" s="52" t="str">
+      <c r="AB6" s="46" t="str">
         <f>_xlfn.XLOOKUP(AC5,mat!$A:$A, mat!$B:$B,"") &amp; ""</f>
         <v/>
       </c>
-      <c r="AC6" s="53"/>
-      <c r="AE6" s="52" t="str">
+      <c r="AC6" s="47"/>
+      <c r="AE6" s="46" t="str">
         <f>_xlfn.XLOOKUP(AF5,mat!$A:$A, mat!$B:$B,"") &amp; ""</f>
         <v/>
       </c>
-      <c r="AF6" s="53"/>
+      <c r="AF6" s="47"/>
       <c r="AG6" s="1"/>
-      <c r="AH6" s="52" t="str">
+      <c r="AH6" s="46" t="str">
         <f>_xlfn.XLOOKUP(AI5,mat!$A:$A, mat!$B:$B,"") &amp; ""</f>
         <v/>
       </c>
-      <c r="AI6" s="53"/>
+      <c r="AI6" s="47"/>
       <c r="AJ6" s="1"/>
-      <c r="AK6" s="52" t="str">
+      <c r="AK6" s="46" t="str">
         <f>_xlfn.XLOOKUP(AL5,mat!$A:$A, mat!$B:$B,"") &amp; ""</f>
         <v/>
       </c>
-      <c r="AL6" s="53"/>
+      <c r="AL6" s="47"/>
       <c r="AM6" s="1"/>
-      <c r="AN6" s="52" t="str">
+      <c r="AN6" s="46" t="str">
         <f>_xlfn.XLOOKUP(AO5,mat!$A:$A, mat!$B:$B,"") &amp; ""</f>
         <v/>
       </c>
-      <c r="AO6" s="53"/>
+      <c r="AO6" s="47"/>
       <c r="AP6" s="1"/>
-      <c r="AQ6" s="52" t="str">
+      <c r="AQ6" s="46" t="str">
         <f>_xlfn.XLOOKUP(AR5,mat!$A:$A, mat!$B:$B,"") &amp; ""</f>
         <v/>
       </c>
-      <c r="AR6" s="53"/>
+      <c r="AR6" s="47"/>
     </row>
     <row r="7" spans="1:44" x14ac:dyDescent="0.2">
       <c r="A7" s="2" t="s">
@@ -15893,36 +16025,36 @@
     </row>
   </sheetData>
   <mergeCells count="30">
+    <mergeCell ref="A4:B4"/>
+    <mergeCell ref="D4:E4"/>
+    <mergeCell ref="G4:H4"/>
+    <mergeCell ref="J4:K4"/>
+    <mergeCell ref="M4:N4"/>
+    <mergeCell ref="P4:Q4"/>
+    <mergeCell ref="S4:T4"/>
+    <mergeCell ref="V4:W4"/>
+    <mergeCell ref="Y4:Z4"/>
+    <mergeCell ref="AB4:AC4"/>
+    <mergeCell ref="AE4:AF4"/>
+    <mergeCell ref="AH4:AI4"/>
+    <mergeCell ref="AK4:AL4"/>
+    <mergeCell ref="AN4:AO4"/>
+    <mergeCell ref="AQ4:AR4"/>
+    <mergeCell ref="A6:B6"/>
+    <mergeCell ref="D6:E6"/>
+    <mergeCell ref="G6:H6"/>
+    <mergeCell ref="J6:K6"/>
+    <mergeCell ref="M6:N6"/>
+    <mergeCell ref="P6:Q6"/>
+    <mergeCell ref="S6:T6"/>
+    <mergeCell ref="V6:W6"/>
+    <mergeCell ref="Y6:Z6"/>
+    <mergeCell ref="AB6:AC6"/>
     <mergeCell ref="AE6:AF6"/>
     <mergeCell ref="AH6:AI6"/>
     <mergeCell ref="AK6:AL6"/>
     <mergeCell ref="AN6:AO6"/>
     <mergeCell ref="AQ6:AR6"/>
-    <mergeCell ref="P6:Q6"/>
-    <mergeCell ref="S6:T6"/>
-    <mergeCell ref="V6:W6"/>
-    <mergeCell ref="Y6:Z6"/>
-    <mergeCell ref="AB6:AC6"/>
-    <mergeCell ref="A6:B6"/>
-    <mergeCell ref="D6:E6"/>
-    <mergeCell ref="G6:H6"/>
-    <mergeCell ref="J6:K6"/>
-    <mergeCell ref="M6:N6"/>
-    <mergeCell ref="AE4:AF4"/>
-    <mergeCell ref="AH4:AI4"/>
-    <mergeCell ref="AK4:AL4"/>
-    <mergeCell ref="AN4:AO4"/>
-    <mergeCell ref="AQ4:AR4"/>
-    <mergeCell ref="P4:Q4"/>
-    <mergeCell ref="S4:T4"/>
-    <mergeCell ref="V4:W4"/>
-    <mergeCell ref="Y4:Z4"/>
-    <mergeCell ref="AB4:AC4"/>
-    <mergeCell ref="A4:B4"/>
-    <mergeCell ref="D4:E4"/>
-    <mergeCell ref="G4:H4"/>
-    <mergeCell ref="J4:K4"/>
-    <mergeCell ref="M4:N4"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
@@ -15955,264 +16087,264 @@
   </cols>
   <sheetData>
     <row r="2" spans="1:44" x14ac:dyDescent="0.2">
-      <c r="A2" s="27" t="s">
-        <v>158</v>
+      <c r="A2" s="24" t="s">
+        <v>156</v>
       </c>
     </row>
     <row r="4" spans="1:44" x14ac:dyDescent="0.2">
-      <c r="A4" s="51" t="s">
+      <c r="A4" s="48" t="s">
+        <v>137</v>
+      </c>
+      <c r="B4" s="48"/>
+      <c r="D4" s="48" t="s">
+        <v>138</v>
+      </c>
+      <c r="E4" s="48"/>
+      <c r="G4" s="48" t="s">
         <v>139</v>
       </c>
-      <c r="B4" s="51"/>
-      <c r="D4" s="51" t="s">
+      <c r="H4" s="48"/>
+      <c r="J4" s="48" t="s">
         <v>140</v>
       </c>
-      <c r="E4" s="51"/>
-      <c r="G4" s="51" t="s">
+      <c r="K4" s="48"/>
+      <c r="M4" s="48" t="s">
         <v>141</v>
       </c>
-      <c r="H4" s="51"/>
-      <c r="J4" s="51" t="s">
+      <c r="N4" s="48"/>
+      <c r="P4" s="48" t="s">
         <v>142</v>
       </c>
-      <c r="K4" s="51"/>
-      <c r="M4" s="51" t="s">
+      <c r="Q4" s="48"/>
+      <c r="R4" s="1"/>
+      <c r="S4" s="48" t="s">
         <v>143</v>
       </c>
-      <c r="N4" s="51"/>
-      <c r="P4" s="51" t="s">
+      <c r="T4" s="48"/>
+      <c r="U4" s="1"/>
+      <c r="V4" s="48" t="s">
         <v>144</v>
       </c>
-      <c r="Q4" s="51"/>
-      <c r="R4" s="1"/>
-      <c r="S4" s="51" t="s">
+      <c r="W4" s="48"/>
+      <c r="X4" s="1"/>
+      <c r="Y4" s="48" t="s">
         <v>145</v>
       </c>
-      <c r="T4" s="51"/>
-      <c r="U4" s="1"/>
-      <c r="V4" s="51" t="s">
+      <c r="Z4" s="48"/>
+      <c r="AA4" s="1"/>
+      <c r="AB4" s="48" t="s">
         <v>146</v>
       </c>
-      <c r="W4" s="51"/>
-      <c r="X4" s="1"/>
-      <c r="Y4" s="51" t="s">
+      <c r="AC4" s="48"/>
+      <c r="AE4" s="48" t="s">
         <v>147</v>
       </c>
-      <c r="Z4" s="51"/>
-      <c r="AA4" s="1"/>
-      <c r="AB4" s="51" t="s">
+      <c r="AF4" s="48"/>
+      <c r="AG4" s="1"/>
+      <c r="AH4" s="48" t="s">
         <v>148</v>
       </c>
-      <c r="AC4" s="51"/>
-      <c r="AE4" s="51" t="s">
+      <c r="AI4" s="48"/>
+      <c r="AJ4" s="1"/>
+      <c r="AK4" s="48" t="s">
         <v>149</v>
       </c>
-      <c r="AF4" s="51"/>
-      <c r="AG4" s="1"/>
-      <c r="AH4" s="51" t="s">
+      <c r="AL4" s="48"/>
+      <c r="AM4" s="1"/>
+      <c r="AN4" s="48" t="s">
         <v>150</v>
       </c>
-      <c r="AI4" s="51"/>
-      <c r="AJ4" s="1"/>
-      <c r="AK4" s="51" t="s">
+      <c r="AO4" s="48"/>
+      <c r="AP4" s="1"/>
+      <c r="AQ4" s="48" t="s">
         <v>151</v>
       </c>
-      <c r="AL4" s="51"/>
-      <c r="AM4" s="1"/>
-      <c r="AN4" s="51" t="s">
-        <v>152</v>
-      </c>
-      <c r="AO4" s="51"/>
-      <c r="AP4" s="1"/>
-      <c r="AQ4" s="51" t="s">
-        <v>153</v>
-      </c>
-      <c r="AR4" s="51"/>
+      <c r="AR4" s="48"/>
     </row>
     <row r="5" spans="1:44" x14ac:dyDescent="0.2">
-      <c r="A5" s="42" t="s">
-        <v>122</v>
-      </c>
-      <c r="B5" s="43">
+      <c r="A5" s="38" t="s">
+        <v>120</v>
+      </c>
+      <c r="B5" s="39">
         <v>1</v>
       </c>
-      <c r="D5" s="42" t="s">
-        <v>122</v>
-      </c>
-      <c r="E5" s="43">
+      <c r="D5" s="38" t="s">
+        <v>120</v>
+      </c>
+      <c r="E5" s="39">
         <v>2</v>
       </c>
-      <c r="G5" s="42" t="s">
-        <v>122</v>
-      </c>
-      <c r="H5" s="43">
+      <c r="G5" s="38" t="s">
+        <v>120</v>
+      </c>
+      <c r="H5" s="39">
         <v>3</v>
       </c>
-      <c r="J5" s="42" t="s">
-        <v>122</v>
-      </c>
-      <c r="K5" s="43">
+      <c r="J5" s="38" t="s">
+        <v>120</v>
+      </c>
+      <c r="K5" s="39">
         <v>4</v>
       </c>
-      <c r="M5" s="42" t="s">
-        <v>122</v>
-      </c>
-      <c r="N5" s="43">
+      <c r="M5" s="38" t="s">
+        <v>120</v>
+      </c>
+      <c r="N5" s="39">
         <v>5</v>
       </c>
-      <c r="P5" s="42" t="s">
-        <v>122</v>
-      </c>
-      <c r="Q5" s="43">
+      <c r="P5" s="38" t="s">
+        <v>120</v>
+      </c>
+      <c r="Q5" s="39">
         <v>6</v>
       </c>
       <c r="R5" s="1"/>
-      <c r="S5" s="42" t="s">
-        <v>122</v>
-      </c>
-      <c r="T5" s="43">
+      <c r="S5" s="38" t="s">
+        <v>120</v>
+      </c>
+      <c r="T5" s="39">
         <v>7</v>
       </c>
       <c r="U5" s="1"/>
-      <c r="V5" s="42" t="s">
-        <v>122</v>
-      </c>
-      <c r="W5" s="43">
+      <c r="V5" s="38" t="s">
+        <v>120</v>
+      </c>
+      <c r="W5" s="39">
         <v>8</v>
       </c>
       <c r="X5" s="1"/>
-      <c r="Y5" s="42" t="s">
-        <v>122</v>
-      </c>
-      <c r="Z5" s="43">
+      <c r="Y5" s="38" t="s">
+        <v>120</v>
+      </c>
+      <c r="Z5" s="39">
         <v>9</v>
       </c>
       <c r="AA5" s="1"/>
-      <c r="AB5" s="42" t="s">
-        <v>122</v>
-      </c>
-      <c r="AC5" s="43">
+      <c r="AB5" s="38" t="s">
+        <v>120</v>
+      </c>
+      <c r="AC5" s="39">
         <v>10</v>
       </c>
-      <c r="AE5" s="42" t="s">
-        <v>122</v>
-      </c>
-      <c r="AF5" s="43">
+      <c r="AE5" s="38" t="s">
+        <v>120</v>
+      </c>
+      <c r="AF5" s="39">
         <v>11</v>
       </c>
       <c r="AG5" s="1"/>
-      <c r="AH5" s="42" t="s">
-        <v>122</v>
-      </c>
-      <c r="AI5" s="43">
+      <c r="AH5" s="38" t="s">
+        <v>120</v>
+      </c>
+      <c r="AI5" s="39">
         <v>12</v>
       </c>
       <c r="AJ5" s="1"/>
-      <c r="AK5" s="42" t="s">
-        <v>122</v>
-      </c>
-      <c r="AL5" s="43">
+      <c r="AK5" s="38" t="s">
+        <v>120</v>
+      </c>
+      <c r="AL5" s="39">
         <v>13</v>
       </c>
       <c r="AM5" s="1"/>
-      <c r="AN5" s="42" t="s">
-        <v>122</v>
-      </c>
-      <c r="AO5" s="43">
+      <c r="AN5" s="38" t="s">
+        <v>120</v>
+      </c>
+      <c r="AO5" s="39">
         <v>14</v>
       </c>
       <c r="AP5" s="1"/>
-      <c r="AQ5" s="42" t="s">
-        <v>122</v>
-      </c>
-      <c r="AR5" s="43">
+      <c r="AQ5" s="38" t="s">
+        <v>120</v>
+      </c>
+      <c r="AR5" s="39">
         <v>15</v>
       </c>
     </row>
     <row r="6" spans="1:44" x14ac:dyDescent="0.2">
-      <c r="A6" s="54" t="str">
+      <c r="A6" s="49" t="str">
         <f>_xlfn.XLOOKUP(B5,mat!$A:$A, mat!$B:$B,"") &amp; ""</f>
         <v/>
       </c>
-      <c r="B6" s="55"/>
-      <c r="D6" s="54" t="str">
+      <c r="B6" s="50"/>
+      <c r="D6" s="49" t="str">
         <f>_xlfn.XLOOKUP(E5,mat!$A:$A, mat!$B:$B,"") &amp; ""</f>
         <v/>
       </c>
-      <c r="E6" s="55"/>
-      <c r="G6" s="54" t="str">
+      <c r="E6" s="50"/>
+      <c r="G6" s="49" t="str">
         <f>_xlfn.XLOOKUP(H5,mat!$A:$A, mat!$B:$B,"") &amp; ""</f>
         <v/>
       </c>
-      <c r="H6" s="55"/>
-      <c r="J6" s="54" t="str">
+      <c r="H6" s="50"/>
+      <c r="J6" s="49" t="str">
         <f>_xlfn.XLOOKUP(K5,mat!$A:$A, mat!$B:$B,"") &amp; ""</f>
         <v/>
       </c>
-      <c r="K6" s="55"/>
-      <c r="M6" s="54" t="str">
+      <c r="K6" s="50"/>
+      <c r="M6" s="49" t="str">
         <f>_xlfn.XLOOKUP(N5,mat!$A:$A, mat!$B:$B,"") &amp; ""</f>
         <v/>
       </c>
-      <c r="N6" s="55"/>
-      <c r="P6" s="54" t="str">
+      <c r="N6" s="50"/>
+      <c r="P6" s="49" t="str">
         <f>_xlfn.XLOOKUP(Q5,mat!$A:$A, mat!$B:$B,"") &amp; ""</f>
         <v/>
       </c>
-      <c r="Q6" s="55"/>
+      <c r="Q6" s="50"/>
       <c r="R6" s="1"/>
-      <c r="S6" s="54" t="str">
+      <c r="S6" s="49" t="str">
         <f>_xlfn.XLOOKUP(T5,mat!$A:$A, mat!$B:$B,"") &amp; ""</f>
         <v/>
       </c>
-      <c r="T6" s="55"/>
+      <c r="T6" s="50"/>
       <c r="U6" s="1"/>
-      <c r="V6" s="54" t="str">
+      <c r="V6" s="49" t="str">
         <f>_xlfn.XLOOKUP(W5,mat!$A:$A, mat!$B:$B,"") &amp; ""</f>
         <v/>
       </c>
-      <c r="W6" s="55"/>
+      <c r="W6" s="50"/>
       <c r="X6" s="1"/>
-      <c r="Y6" s="54" t="str">
+      <c r="Y6" s="49" t="str">
         <f>_xlfn.XLOOKUP(Z5,mat!$A:$A, mat!$B:$B,"") &amp; ""</f>
         <v/>
       </c>
-      <c r="Z6" s="55"/>
+      <c r="Z6" s="50"/>
       <c r="AA6" s="1"/>
-      <c r="AB6" s="54" t="str">
+      <c r="AB6" s="49" t="str">
         <f>_xlfn.XLOOKUP(AC5,mat!$A:$A, mat!$B:$B,"") &amp; ""</f>
         <v/>
       </c>
-      <c r="AC6" s="55"/>
-      <c r="AE6" s="54" t="str">
+      <c r="AC6" s="50"/>
+      <c r="AE6" s="49" t="str">
         <f>_xlfn.XLOOKUP(AF5,mat!$A:$A, mat!$B:$B,"") &amp; ""</f>
         <v/>
       </c>
-      <c r="AF6" s="55"/>
+      <c r="AF6" s="50"/>
       <c r="AG6" s="1"/>
-      <c r="AH6" s="54" t="str">
+      <c r="AH6" s="49" t="str">
         <f>_xlfn.XLOOKUP(AI5,mat!$A:$A, mat!$B:$B,"") &amp; ""</f>
         <v/>
       </c>
-      <c r="AI6" s="55"/>
+      <c r="AI6" s="50"/>
       <c r="AJ6" s="1"/>
-      <c r="AK6" s="54" t="str">
+      <c r="AK6" s="49" t="str">
         <f>_xlfn.XLOOKUP(AL5,mat!$A:$A, mat!$B:$B,"") &amp; ""</f>
         <v/>
       </c>
-      <c r="AL6" s="55"/>
+      <c r="AL6" s="50"/>
       <c r="AM6" s="1"/>
-      <c r="AN6" s="54" t="str">
+      <c r="AN6" s="49" t="str">
         <f>_xlfn.XLOOKUP(AO5,mat!$A:$A, mat!$B:$B,"") &amp; ""</f>
         <v/>
       </c>
-      <c r="AO6" s="55"/>
+      <c r="AO6" s="50"/>
       <c r="AP6" s="1"/>
-      <c r="AQ6" s="54" t="str">
+      <c r="AQ6" s="49" t="str">
         <f>_xlfn.XLOOKUP(AR5,mat!$A:$A, mat!$B:$B,"") &amp; ""</f>
         <v/>
       </c>
-      <c r="AR6" s="55"/>
+      <c r="AR6" s="50"/>
     </row>
     <row r="7" spans="1:44" x14ac:dyDescent="0.2">
       <c r="A7" s="2" t="s">
@@ -17116,14 +17248,12 @@
     </row>
   </sheetData>
   <mergeCells count="30">
-    <mergeCell ref="AN6:AO6"/>
-    <mergeCell ref="AQ6:AR6"/>
-    <mergeCell ref="V6:W6"/>
-    <mergeCell ref="Y6:Z6"/>
-    <mergeCell ref="AB6:AC6"/>
-    <mergeCell ref="AE6:AF6"/>
-    <mergeCell ref="AH6:AI6"/>
-    <mergeCell ref="AK6:AL6"/>
+    <mergeCell ref="P4:Q4"/>
+    <mergeCell ref="A4:B4"/>
+    <mergeCell ref="D4:E4"/>
+    <mergeCell ref="G4:H4"/>
+    <mergeCell ref="J4:K4"/>
+    <mergeCell ref="M4:N4"/>
     <mergeCell ref="AK4:AL4"/>
     <mergeCell ref="AN4:AO4"/>
     <mergeCell ref="AQ4:AR4"/>
@@ -17140,12 +17270,14 @@
     <mergeCell ref="AB4:AC4"/>
     <mergeCell ref="AE4:AF4"/>
     <mergeCell ref="AH4:AI4"/>
-    <mergeCell ref="P4:Q4"/>
-    <mergeCell ref="A4:B4"/>
-    <mergeCell ref="D4:E4"/>
-    <mergeCell ref="G4:H4"/>
-    <mergeCell ref="J4:K4"/>
-    <mergeCell ref="M4:N4"/>
+    <mergeCell ref="AN6:AO6"/>
+    <mergeCell ref="AQ6:AR6"/>
+    <mergeCell ref="V6:W6"/>
+    <mergeCell ref="Y6:Z6"/>
+    <mergeCell ref="AB6:AC6"/>
+    <mergeCell ref="AE6:AF6"/>
+    <mergeCell ref="AH6:AI6"/>
+    <mergeCell ref="AK6:AL6"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
@@ -17161,28 +17293,28 @@
   </cols>
   <sheetData>
     <row r="2" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A2" s="56" t="s">
-        <v>84</v>
-      </c>
-      <c r="B2" s="56"/>
-      <c r="D2" s="57" t="s">
+      <c r="A2" s="51" t="s">
+        <v>83</v>
+      </c>
+      <c r="B2" s="51"/>
+      <c r="D2" s="52" t="s">
+        <v>81</v>
+      </c>
+      <c r="E2" s="52"/>
+      <c r="G2" s="22" t="s">
         <v>82</v>
       </c>
-      <c r="E2" s="57"/>
-      <c r="G2" s="24" t="s">
-        <v>83</v>
-      </c>
     </row>
     <row r="3" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A3" s="36" t="s">
-        <v>198</v>
-      </c>
-      <c r="B3" s="37"/>
-      <c r="D3" s="38" t="s">
-        <v>198</v>
-      </c>
-      <c r="E3" s="39"/>
-      <c r="G3" s="24"/>
+      <c r="A3" s="32" t="s">
+        <v>196</v>
+      </c>
+      <c r="B3" s="33"/>
+      <c r="D3" s="34" t="s">
+        <v>196</v>
+      </c>
+      <c r="E3" s="35"/>
+      <c r="G3" s="22"/>
     </row>
     <row r="4" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A4" s="2" t="s">
@@ -17198,7 +17330,7 @@
         <v>4</v>
       </c>
       <c r="G4" s="6" t="s">
-        <v>199</v>
+        <v>197</v>
       </c>
       <c r="H4" s="1"/>
     </row>
@@ -17211,7 +17343,7 @@
         <v>21</v>
       </c>
       <c r="H5" t="s">
-        <v>202</v>
+        <v>200</v>
       </c>
     </row>
     <row r="6" spans="1:8" x14ac:dyDescent="0.2">
@@ -17220,10 +17352,10 @@
       <c r="D6" s="3"/>
       <c r="E6" s="3"/>
       <c r="G6" s="1" t="s">
-        <v>200</v>
+        <v>198</v>
       </c>
       <c r="H6" t="s">
-        <v>201</v>
+        <v>199</v>
       </c>
     </row>
     <row r="7" spans="1:8" x14ac:dyDescent="0.2">
@@ -17363,10 +17495,10 @@
         <v>25</v>
       </c>
       <c r="B2" s="13" t="s">
+        <v>60</v>
+      </c>
+      <c r="C2" s="13" t="s">
         <v>61</v>
-      </c>
-      <c r="C2" s="13" t="s">
-        <v>62</v>
       </c>
       <c r="D2" s="13" t="s">
         <v>29</v>
@@ -17381,7 +17513,7 @@
         <v>28</v>
       </c>
       <c r="H2" s="13" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="J2" s="5" t="s">
         <v>30</v>
@@ -17438,10 +17570,10 @@
       <c r="G5" s="3"/>
       <c r="H5" s="3"/>
       <c r="J5" s="1" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="K5" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
     </row>
     <row r="6" spans="1:14" x14ac:dyDescent="0.2">
@@ -17613,10 +17745,10 @@
       <c r="B5" s="3"/>
       <c r="C5" s="3"/>
       <c r="E5" t="s">
+        <v>75</v>
+      </c>
+      <c r="F5" t="s">
         <v>76</v>
-      </c>
-      <c r="F5" t="s">
-        <v>77</v>
       </c>
     </row>
     <row r="6" spans="1:6" x14ac:dyDescent="0.2">
@@ -17739,36 +17871,36 @@
   </cols>
   <sheetData>
     <row r="2" spans="2:24" x14ac:dyDescent="0.2">
-      <c r="B2" s="58" t="s">
+      <c r="B2" s="53" t="s">
+        <v>121</v>
+      </c>
+      <c r="C2" s="53"/>
+      <c r="D2" s="53"/>
+      <c r="F2" s="53" t="s">
+        <v>122</v>
+      </c>
+      <c r="G2" s="53"/>
+      <c r="H2" s="53"/>
+      <c r="J2" s="53" t="s">
         <v>123</v>
       </c>
-      <c r="C2" s="58"/>
-      <c r="D2" s="58"/>
-      <c r="F2" s="58" t="s">
+      <c r="K2" s="53"/>
+      <c r="L2" s="53"/>
+      <c r="N2" s="53" t="s">
         <v>124</v>
       </c>
-      <c r="G2" s="58"/>
-      <c r="H2" s="58"/>
-      <c r="J2" s="58" t="s">
+      <c r="O2" s="53"/>
+      <c r="P2" s="53"/>
+      <c r="R2" s="53" t="s">
         <v>125</v>
       </c>
-      <c r="K2" s="58"/>
-      <c r="L2" s="58"/>
-      <c r="N2" s="58" t="s">
+      <c r="S2" s="53"/>
+      <c r="T2" s="53"/>
+      <c r="V2" s="53" t="s">
         <v>126</v>
       </c>
-      <c r="O2" s="58"/>
-      <c r="P2" s="58"/>
-      <c r="R2" s="58" t="s">
-        <v>127</v>
-      </c>
-      <c r="S2" s="58"/>
-      <c r="T2" s="58"/>
-      <c r="V2" s="58" t="s">
-        <v>128</v>
-      </c>
-      <c r="W2" s="58"/>
-      <c r="X2" s="58"/>
+      <c r="W2" s="53"/>
+      <c r="X2" s="53"/>
     </row>
     <row r="3" spans="2:24" x14ac:dyDescent="0.2">
       <c r="B3" s="2" t="s">

</xml_diff>

<commit_message>
template v16: complete the conditional formatting + fix header colors (surgical XML edit)
t_cut header red->blue (FEM only, LEM ignores it); d/psi headers aligned to the
legend's LEM-only tint (-0.25, the reinforce/piles convention); conditional
formatting rebuilt as 16 clean rules — the v15 dependency semantics remapped to
the v16 columns plus three new elastic rules (grays strengths+t_cut, u/ru, and
strength SDs; keeps g/gsat, E/nu, s(g)); u-column dropdown range extended to row
52. Only xl/styles.xml and the mat sheet XML differ from Norm's snapshot — all
other parts byte-identical (charts untouched).

Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_0147GB4LGVZuqGHCRMVzZTsR
</commit_message>
<xml_diff>
--- a/docs/inputs/input_template.xlsx
+++ b/docs/inputs/input_template.xlsx
@@ -1280,7 +1280,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="63">
+  <cellXfs count="65">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -1452,6 +1452,12 @@
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="20" fillId="6" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
   </cellXfs>
@@ -13430,13 +13436,13 @@
       <c r="I10" s="57" t="s">
         <v>71</v>
       </c>
-      <c r="J10" s="61" t="s">
+      <c r="J10" s="64" t="s">
         <v>79</v>
       </c>
-      <c r="K10" s="61" t="s">
+      <c r="K10" s="64" t="s">
         <v>135</v>
       </c>
-      <c r="L10" s="57" t="s">
+      <c r="L10" s="63" t="s">
         <v>235</v>
       </c>
       <c r="M10" s="21" t="s">
@@ -14756,64 +14762,82 @@
     <mergeCell ref="AE9:AL9"/>
     <mergeCell ref="C9:X9"/>
   </mergeCells>
-  <conditionalFormatting sqref="F51:P52 Z11:AD52 F11:L25 F26:N50 P26:P50">
-    <cfRule type="expression" dxfId="15" priority="2">
+  <conditionalFormatting sqref="F11:K52 Z11:AD52">
+    <cfRule type="expression" dxfId="5" priority="1">
       <formula>$E11="hb"</formula>
+    </cfRule>
+    <cfRule type="expression" dxfId="5" priority="2">
+      <formula>$E11="pow"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="G11:G52">
-    <cfRule type="expression" dxfId="14" priority="7">
+    <cfRule type="expression" dxfId="5" priority="3">
       <formula>$E11="cp"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="H11:I52">
-    <cfRule type="expression" dxfId="13" priority="6">
+    <cfRule type="expression" dxfId="5" priority="4">
       <formula>$E11="mc"</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="J51:P52 J11:L25 J26:N50 P26:P50">
-    <cfRule type="expression" dxfId="12" priority="8">
+  <conditionalFormatting sqref="J11:K52">
+    <cfRule type="expression" dxfId="5" priority="5">
       <formula>$E11="cp"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="Q11:T52">
-    <cfRule type="expression" dxfId="11" priority="21">
+    <cfRule type="expression" dxfId="5" priority="6">
       <formula>AND($E11&lt;&gt;"",$E11&lt;&gt;"pow")</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="U11:X52">
-    <cfRule type="expression" dxfId="10" priority="1">
+    <cfRule type="expression" dxfId="5" priority="7">
       <formula>AND($E11&lt;&gt;"",$E11&lt;&gt;"hb")</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="Z11:AD52 F51:P52 F11:L25 F26:N50 P26:P50">
-    <cfRule type="expression" dxfId="8" priority="18">
-      <formula>$E11="pow"</formula>
+  <conditionalFormatting sqref="P11:P52">
+    <cfRule type="expression" dxfId="5" priority="8">
+      <formula>AND($O11&lt;&gt;"",$O11&lt;&gt;"ru")</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="AA11:AA52">
-    <cfRule type="expression" dxfId="7" priority="10">
+    <cfRule type="expression" dxfId="5" priority="9">
       <formula>$E11="cp"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="AB11:AB52">
-    <cfRule type="expression" dxfId="6" priority="17">
+    <cfRule type="expression" dxfId="5" priority="10">
       <formula>$E11="mc"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="AC11:AD52">
-    <cfRule type="expression" dxfId="5" priority="12">
+    <cfRule type="expression" dxfId="5" priority="11">
       <formula>$E11="cp"</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="AI11:AJ102">
-    <cfRule type="expression" dxfId="4" priority="4">
+  <conditionalFormatting sqref="AI11:AJ52">
+    <cfRule type="expression" dxfId="5" priority="12">
       <formula>OR($AH11="vg",$AH11="gard")</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="AK11:AL102">
-    <cfRule type="expression" dxfId="3" priority="3">
+  <conditionalFormatting sqref="AK11:AL52">
+    <cfRule type="expression" dxfId="5" priority="13">
       <formula>$AH11="lf"</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="F11:L52">
+    <cfRule type="expression" dxfId="5" priority="14">
+      <formula>$E11="elastic"</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="O11:P52">
+    <cfRule type="expression" dxfId="5" priority="15">
+      <formula>$E11="elastic"</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="Z11:AD52">
+    <cfRule type="expression" dxfId="5" priority="16">
+      <formula>$E11="elastic"</formula>
     </cfRule>
   </conditionalFormatting>
   <dataValidations count="3">
@@ -14823,7 +14847,7 @@
     <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="AH11:AH102" xr:uid="{E00A94A9-D864-5843-8FBD-E84775B1C100}">
       <formula1>$AH$3:$AH$5</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="O11:O50" xr:uid="{D770415C-1ECE-F44B-9D8C-08EF1CF31C8E}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="O11:O52" xr:uid="{D770415C-1ECE-F44B-9D8C-08EF1CF31C8E}">
       <formula1>$O$3:$O$6</formula1>
     </dataValidation>
   </dataValidations>

</xml_diff>

<commit_message>
template v17: complete the conditional formatting (surgical XML edit)
Excel's auto-shift handled 15 of 16 rules and created the cp-gray over phi_b/s_cap
by range expansion; fixed the hb/pow rules' wrongly-expanded gray (F11:M52 ->
F11:K52 — phi_b/s_cap stay active for hb/pow per the dependency matrix) and added
the u-source rule (gray L:M when u is set but neither piezo nor seep). Only the
mat sheet XML differs from Norm's snapshot — all other parts byte-identical.

Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_0147GB4LGVZuqGHCRMVzZTsR
</commit_message>
<xml_diff>
--- a/docs/inputs/input_template.xlsx
+++ b/docs/inputs/input_template.xlsx
@@ -14869,7 +14869,12 @@
     <mergeCell ref="AG9:AN9"/>
     <mergeCell ref="C9:Z9"/>
   </mergeCells>
-  <conditionalFormatting sqref="F11:M52 AB11:AF52">
+  <conditionalFormatting sqref="L11:M52">
+    <cfRule type="expression" dxfId="5" priority="17">
+      <formula>AND($Q11&lt;&gt;"",$Q11&lt;&gt;"piezo",$Q11&lt;&gt;"seep")</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="F11:K52 AB11:AF52">
     <cfRule type="expression" dxfId="18" priority="1">
       <formula>$E11="hb"</formula>
     </cfRule>

</xml_diff>

<commit_message>
template v17: Norm's phi_b/s_cap columns (pre CF-fix snapshot)
Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_0147GB4LGVZuqGHCRMVzZTsR
</commit_message>
<xml_diff>
--- a/docs/inputs/input_template.xlsx
+++ b/docs/inputs/input_template.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/njones/python_projects/xslope/docs/inputs/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{448736C4-E2C8-EB41-827A-888C500BCAB7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E9AE3CBE-0B2A-ED44-BB50-AACC6A5490D5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="600" windowWidth="38400" windowHeight="19900" xr2:uid="{BA54C293-CE08-6E4C-9212-B3317DAA148E}"/>
+    <workbookView xWindow="0" yWindow="600" windowWidth="35040" windowHeight="19900" xr2:uid="{BA54C293-CE08-6E4C-9212-B3317DAA148E}"/>
   </bookViews>
   <sheets>
     <sheet name="main" sheetId="1" r:id="rId1"/>
@@ -62,7 +62,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="449" uniqueCount="238">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="451" uniqueCount="240">
   <si>
     <t>X</t>
   </si>
@@ -941,6 +941,12 @@
   </si>
   <si>
     <t>Color legend</t>
+  </si>
+  <si>
+    <t>phi_b</t>
+  </si>
+  <si>
+    <t>s_cap</t>
   </si>
 </sst>
 </file>
@@ -1090,7 +1096,7 @@
       <name val="Aptos Narrow"/>
     </font>
   </fonts>
-  <fills count="18">
+  <fills count="17">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -1187,12 +1193,6 @@
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="9" tint="-0.499984740745262"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
   </fills>
   <borders count="7">
     <border>
@@ -1280,7 +1280,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="65">
+  <cellXfs count="63">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -1397,19 +1397,37 @@
     <xf numFmtId="0" fontId="20" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="0" fontId="5" fillId="6" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="6" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="16" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="16" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="6" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
     <xf numFmtId="0" fontId="4" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="10" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
     <xf numFmtId="0" fontId="2" fillId="14" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="14" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="15" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -1436,35 +1454,11 @@
     <xf numFmtId="0" fontId="1" fillId="13" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="6" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="6" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="16" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="16" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="17" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="6" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="16">
+  <dxfs count="19">
     <dxf>
       <fill>
         <patternFill>
@@ -1483,34 +1477,6 @@
       <fill>
         <patternFill>
           <bgColor theme="1" tint="0.499984740745262"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor theme="2" tint="-0.499984740745262"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor theme="2" tint="-0.499984740745262"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor theme="0" tint="-0.499984740745262"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor theme="2" tint="-0.499984740745262"/>
         </patternFill>
       </fill>
     </dxf>
@@ -1559,7 +1525,56 @@
     <dxf>
       <fill>
         <patternFill>
-          <bgColor theme="2" tint="-0.499984740745262"/>
+          <bgColor theme="0" tint="-0.499984740745262"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="0" tint="-0.499984740745262"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="0" tint="-0.499984740745262"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="0" tint="-0.499984740745262"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="0" tint="-0.499984740745262"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="0" tint="-0.499984740745262"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="0" tint="-0.499984740745262"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="0" tint="-0.499984740745262"/>
         </patternFill>
       </fill>
     </dxf>
@@ -10431,15 +10446,15 @@
         <v>78</v>
       </c>
       <c r="D5" s="30">
-        <v>16</v>
+        <v>17</v>
       </c>
     </row>
     <row r="7" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="B7" s="44" t="s">
+      <c r="B7" s="50" t="s">
         <v>47</v>
       </c>
-      <c r="C7" s="44"/>
-      <c r="D7" s="44"/>
+      <c r="C7" s="50"/>
+      <c r="D7" s="50"/>
       <c r="F7" s="15" t="s">
         <v>15</v>
       </c>
@@ -10619,36 +10634,36 @@
   </cols>
   <sheetData>
     <row r="2" spans="2:24" x14ac:dyDescent="0.2">
-      <c r="B2" s="54" t="s">
+      <c r="B2" s="60" t="s">
         <v>129</v>
       </c>
-      <c r="C2" s="54"/>
-      <c r="D2" s="54"/>
-      <c r="F2" s="54" t="s">
+      <c r="C2" s="60"/>
+      <c r="D2" s="60"/>
+      <c r="F2" s="60" t="s">
         <v>130</v>
       </c>
-      <c r="G2" s="54"/>
-      <c r="H2" s="54"/>
-      <c r="J2" s="54" t="s">
+      <c r="G2" s="60"/>
+      <c r="H2" s="60"/>
+      <c r="J2" s="60" t="s">
         <v>131</v>
       </c>
-      <c r="K2" s="54"/>
-      <c r="L2" s="54"/>
-      <c r="N2" s="54" t="s">
+      <c r="K2" s="60"/>
+      <c r="L2" s="60"/>
+      <c r="N2" s="60" t="s">
         <v>132</v>
       </c>
-      <c r="O2" s="54"/>
-      <c r="P2" s="54"/>
-      <c r="R2" s="54" t="s">
+      <c r="O2" s="60"/>
+      <c r="P2" s="60"/>
+      <c r="R2" s="60" t="s">
         <v>133</v>
       </c>
-      <c r="S2" s="54"/>
-      <c r="T2" s="54"/>
-      <c r="V2" s="54" t="s">
+      <c r="S2" s="60"/>
+      <c r="T2" s="60"/>
+      <c r="V2" s="60" t="s">
         <v>134</v>
       </c>
-      <c r="W2" s="54"/>
-      <c r="X2" s="54"/>
+      <c r="W2" s="60"/>
+      <c r="X2" s="60"/>
     </row>
     <row r="3" spans="2:24" x14ac:dyDescent="0.2">
       <c r="B3" s="2" t="s">
@@ -12404,34 +12419,34 @@
   </cols>
   <sheetData>
     <row r="2" spans="2:21" x14ac:dyDescent="0.2">
-      <c r="B2" s="55" t="s">
+      <c r="B2" s="61" t="s">
         <v>127</v>
       </c>
-      <c r="C2" s="55"/>
-      <c r="E2" s="51" t="s">
+      <c r="C2" s="61"/>
+      <c r="E2" s="57" t="s">
         <v>215</v>
       </c>
-      <c r="F2" s="51"/>
-      <c r="H2" s="51" t="s">
+      <c r="F2" s="57"/>
+      <c r="H2" s="57" t="s">
         <v>217</v>
       </c>
-      <c r="I2" s="51"/>
-      <c r="K2" s="51" t="s">
+      <c r="I2" s="57"/>
+      <c r="K2" s="57" t="s">
         <v>218</v>
       </c>
-      <c r="L2" s="51"/>
-      <c r="N2" s="51" t="s">
+      <c r="L2" s="57"/>
+      <c r="N2" s="57" t="s">
         <v>219</v>
       </c>
-      <c r="O2" s="51"/>
-      <c r="Q2" s="51" t="s">
+      <c r="O2" s="57"/>
+      <c r="Q2" s="57" t="s">
         <v>220</v>
       </c>
-      <c r="R2" s="51"/>
+      <c r="R2" s="57"/>
     </row>
     <row r="3" spans="2:21" x14ac:dyDescent="0.2">
-      <c r="B3" s="55"/>
-      <c r="C3" s="55"/>
+      <c r="B3" s="61"/>
+      <c r="C3" s="61"/>
       <c r="E3" s="32" t="s">
         <v>213</v>
       </c>
@@ -12820,34 +12835,34 @@
   </cols>
   <sheetData>
     <row r="2" spans="2:21" x14ac:dyDescent="0.2">
-      <c r="B2" s="56" t="s">
+      <c r="B2" s="62" t="s">
         <v>128</v>
       </c>
-      <c r="C2" s="56"/>
-      <c r="E2" s="52" t="s">
+      <c r="C2" s="62"/>
+      <c r="E2" s="58" t="s">
         <v>221</v>
       </c>
-      <c r="F2" s="52"/>
-      <c r="H2" s="52" t="s">
+      <c r="F2" s="58"/>
+      <c r="H2" s="58" t="s">
         <v>222</v>
       </c>
-      <c r="I2" s="52"/>
-      <c r="K2" s="52" t="s">
+      <c r="I2" s="58"/>
+      <c r="K2" s="58" t="s">
         <v>223</v>
       </c>
-      <c r="L2" s="52"/>
-      <c r="N2" s="52" t="s">
+      <c r="L2" s="58"/>
+      <c r="N2" s="58" t="s">
         <v>224</v>
       </c>
-      <c r="O2" s="52"/>
-      <c r="Q2" s="52" t="s">
+      <c r="O2" s="58"/>
+      <c r="Q2" s="58" t="s">
         <v>225</v>
       </c>
-      <c r="R2" s="52"/>
+      <c r="R2" s="58"/>
     </row>
     <row r="3" spans="2:21" x14ac:dyDescent="0.2">
-      <c r="B3" s="56"/>
-      <c r="C3" s="56"/>
+      <c r="B3" s="62"/>
+      <c r="C3" s="62"/>
       <c r="E3" s="34" t="s">
         <v>213</v>
       </c>
@@ -13232,34 +13247,34 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{60A900FC-A692-B445-95C9-59E70352B291}">
-  <dimension ref="A2:AL52"/>
+  <dimension ref="A2:AN52"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="7" style="1" customWidth="1"/>
     <col min="2" max="2" width="17.33203125" style="1" customWidth="1"/>
     <col min="3" max="10" width="8.5" style="1" customWidth="1"/>
-    <col min="11" max="38" width="8.5" customWidth="1"/>
+    <col min="11" max="40" width="8.5" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="2" spans="1:38" x14ac:dyDescent="0.2">
+    <row r="2" spans="1:40" x14ac:dyDescent="0.2">
       <c r="C2" s="6" t="s">
         <v>67</v>
       </c>
       <c r="E2"/>
       <c r="F2"/>
       <c r="G2"/>
-      <c r="L2" s="6" t="s">
+      <c r="N2" s="6" t="s">
         <v>237</v>
       </c>
-      <c r="O2" s="6" t="s">
+      <c r="Q2" s="6" t="s">
         <v>170</v>
       </c>
-      <c r="AB2" s="6"/>
-      <c r="AH2" s="6" t="s">
+      <c r="AD2" s="6"/>
+      <c r="AJ2" s="6" t="s">
         <v>169</v>
       </c>
     </row>
-    <row r="3" spans="1:38" x14ac:dyDescent="0.2">
+    <row r="3" spans="1:40" x14ac:dyDescent="0.2">
       <c r="C3" s="1" t="s">
         <v>66</v>
       </c>
@@ -13268,21 +13283,21 @@
       </c>
       <c r="F3"/>
       <c r="G3"/>
-      <c r="O3" s="1" t="s">
+      <c r="Q3" s="1" t="s">
         <v>86</v>
       </c>
-      <c r="P3" t="s">
+      <c r="R3" t="s">
         <v>58</v>
       </c>
-      <c r="AB3" s="14"/>
-      <c r="AH3" s="1" t="s">
+      <c r="AD3" s="14"/>
+      <c r="AJ3" s="1" t="s">
         <v>166</v>
       </c>
-      <c r="AI3" t="s">
+      <c r="AK3" t="s">
         <v>168</v>
       </c>
     </row>
-    <row r="4" spans="1:38" x14ac:dyDescent="0.2">
+    <row r="4" spans="1:40" x14ac:dyDescent="0.2">
       <c r="C4" s="1" t="s">
         <v>69</v>
       </c>
@@ -13291,240 +13306,248 @@
       </c>
       <c r="F4"/>
       <c r="G4"/>
-      <c r="L4" s="42"/>
-      <c r="M4" t="s">
+      <c r="N4" s="42"/>
+      <c r="O4" t="s">
         <v>161</v>
       </c>
-      <c r="O4" s="1" t="s">
+      <c r="Q4" s="1" t="s">
         <v>21</v>
       </c>
-      <c r="P4" t="s">
+      <c r="R4" t="s">
         <v>59</v>
       </c>
-      <c r="AB4" s="14"/>
-      <c r="AH4" s="1" t="s">
+      <c r="AD4" s="14"/>
+      <c r="AJ4" s="1" t="s">
         <v>167</v>
       </c>
-      <c r="AI4" t="s">
+      <c r="AK4" t="s">
         <v>204</v>
       </c>
     </row>
-    <row r="5" spans="1:38" x14ac:dyDescent="0.2">
+    <row r="5" spans="1:40" x14ac:dyDescent="0.2">
       <c r="C5" s="1" t="s">
         <v>171</v>
       </c>
       <c r="D5" t="s">
         <v>191</v>
       </c>
-      <c r="L5" s="26"/>
-      <c r="M5" s="9" t="s">
+      <c r="N5" s="26"/>
+      <c r="O5" s="9" t="s">
         <v>162</v>
       </c>
-      <c r="O5" s="1" t="s">
+      <c r="Q5" s="1" t="s">
         <v>87</v>
       </c>
-      <c r="P5" s="9" t="s">
+      <c r="R5" s="9" t="s">
         <v>85</v>
       </c>
-      <c r="AB5" s="14"/>
-      <c r="AH5" s="1" t="s">
+      <c r="AD5" s="14"/>
+      <c r="AJ5" s="1" t="s">
         <v>202</v>
       </c>
-      <c r="AI5" s="9" t="s">
+      <c r="AK5" s="9" t="s">
         <v>203</v>
       </c>
     </row>
-    <row r="6" spans="1:38" x14ac:dyDescent="0.2">
+    <row r="6" spans="1:40" x14ac:dyDescent="0.2">
       <c r="C6" s="1" t="s">
         <v>201</v>
       </c>
       <c r="D6" s="9" t="s">
         <v>207</v>
       </c>
-      <c r="L6" s="29"/>
-      <c r="M6" s="9" t="s">
+      <c r="N6" s="29"/>
+      <c r="O6" s="9" t="s">
         <v>163</v>
       </c>
-      <c r="O6" s="1" t="s">
+      <c r="Q6" s="1" t="s">
         <v>172</v>
       </c>
-      <c r="P6" t="s">
+      <c r="R6" t="s">
         <v>190</v>
       </c>
-      <c r="AC6" s="1"/>
-      <c r="AD6" s="1"/>
-    </row>
-    <row r="7" spans="1:38" x14ac:dyDescent="0.2">
+      <c r="AE6" s="1"/>
+      <c r="AF6" s="1"/>
+    </row>
+    <row r="7" spans="1:40" x14ac:dyDescent="0.2">
       <c r="C7" s="1" t="s">
         <v>233</v>
       </c>
       <c r="D7" s="9" t="s">
         <v>234</v>
       </c>
-      <c r="AC7" s="1"/>
-      <c r="AD7" s="1"/>
-    </row>
-    <row r="9" spans="1:38" x14ac:dyDescent="0.2">
-      <c r="C9" s="45" t="s">
+      <c r="AE7" s="1"/>
+      <c r="AF7" s="1"/>
+    </row>
+    <row r="9" spans="1:40" x14ac:dyDescent="0.2">
+      <c r="C9" s="51" t="s">
         <v>236</v>
       </c>
-      <c r="D9" s="45"/>
-      <c r="E9" s="45"/>
-      <c r="F9" s="45"/>
-      <c r="G9" s="45"/>
-      <c r="H9" s="45"/>
-      <c r="I9" s="45"/>
-      <c r="J9" s="45"/>
-      <c r="K9" s="45"/>
-      <c r="L9" s="45"/>
-      <c r="M9" s="45"/>
-      <c r="N9" s="45"/>
-      <c r="O9" s="45"/>
-      <c r="P9" s="45"/>
-      <c r="Q9" s="45"/>
-      <c r="R9" s="45"/>
-      <c r="S9" s="45"/>
-      <c r="T9" s="45"/>
-      <c r="U9" s="45"/>
-      <c r="V9" s="45"/>
-      <c r="W9" s="45"/>
-      <c r="X9" s="45"/>
-      <c r="Y9" s="45" t="s">
+      <c r="D9" s="51"/>
+      <c r="E9" s="51"/>
+      <c r="F9" s="51"/>
+      <c r="G9" s="51"/>
+      <c r="H9" s="51"/>
+      <c r="I9" s="51"/>
+      <c r="J9" s="51"/>
+      <c r="K9" s="51"/>
+      <c r="L9" s="51"/>
+      <c r="M9" s="51"/>
+      <c r="N9" s="51"/>
+      <c r="O9" s="51"/>
+      <c r="P9" s="51"/>
+      <c r="Q9" s="51"/>
+      <c r="R9" s="51"/>
+      <c r="S9" s="51"/>
+      <c r="T9" s="51"/>
+      <c r="U9" s="51"/>
+      <c r="V9" s="51"/>
+      <c r="W9" s="51"/>
+      <c r="X9" s="51"/>
+      <c r="Y9" s="51"/>
+      <c r="Z9" s="51"/>
+      <c r="AA9" s="51" t="s">
         <v>57</v>
       </c>
-      <c r="Z9" s="45"/>
-      <c r="AA9" s="45"/>
-      <c r="AB9" s="45"/>
-      <c r="AC9" s="45"/>
-      <c r="AD9" s="45"/>
-      <c r="AE9" s="45" t="s">
+      <c r="AB9" s="51"/>
+      <c r="AC9" s="51"/>
+      <c r="AD9" s="51"/>
+      <c r="AE9" s="51"/>
+      <c r="AF9" s="51"/>
+      <c r="AG9" s="51" t="s">
         <v>91</v>
       </c>
-      <c r="AF9" s="45"/>
-      <c r="AG9" s="45"/>
-      <c r="AH9" s="45"/>
-      <c r="AI9" s="45"/>
-      <c r="AJ9" s="45"/>
-      <c r="AK9" s="45"/>
-      <c r="AL9" s="45"/>
-    </row>
-    <row r="10" spans="1:38" ht="18" x14ac:dyDescent="0.25">
+      <c r="AH9" s="51"/>
+      <c r="AI9" s="51"/>
+      <c r="AJ9" s="51"/>
+      <c r="AK9" s="51"/>
+      <c r="AL9" s="51"/>
+      <c r="AM9" s="51"/>
+      <c r="AN9" s="51"/>
+    </row>
+    <row r="10" spans="1:40" ht="18" x14ac:dyDescent="0.25">
       <c r="A10" s="20" t="s">
         <v>19</v>
       </c>
       <c r="B10" s="20" t="s">
         <v>77</v>
       </c>
-      <c r="C10" s="58" t="s">
+      <c r="C10" s="45" t="s">
         <v>52</v>
       </c>
-      <c r="D10" s="62" t="s">
+      <c r="D10" s="48" t="s">
         <v>189</v>
       </c>
-      <c r="E10" s="57" t="s">
+      <c r="E10" s="44" t="s">
         <v>65</v>
       </c>
-      <c r="F10" s="57" t="s">
+      <c r="F10" s="44" t="s">
         <v>53</v>
       </c>
-      <c r="G10" s="58" t="s">
+      <c r="G10" s="45" t="s">
         <v>51</v>
       </c>
-      <c r="H10" s="57" t="s">
+      <c r="H10" s="44" t="s">
         <v>72</v>
       </c>
-      <c r="I10" s="57" t="s">
+      <c r="I10" s="44" t="s">
         <v>71</v>
       </c>
-      <c r="J10" s="64" t="s">
+      <c r="J10" s="49" t="s">
         <v>79</v>
       </c>
-      <c r="K10" s="64" t="s">
+      <c r="K10" s="49" t="s">
         <v>135</v>
       </c>
-      <c r="L10" s="63" t="s">
+      <c r="L10" s="49" t="s">
+        <v>238</v>
+      </c>
+      <c r="M10" s="49" t="s">
+        <v>239</v>
+      </c>
+      <c r="N10" s="21" t="s">
         <v>235</v>
       </c>
-      <c r="M10" s="21" t="s">
+      <c r="O10" s="21" t="s">
         <v>97</v>
       </c>
-      <c r="N10" s="43" t="s">
+      <c r="P10" s="43" t="s">
         <v>211</v>
       </c>
-      <c r="O10" s="57" t="s">
+      <c r="Q10" s="44" t="s">
         <v>84</v>
       </c>
-      <c r="P10" s="57" t="s">
+      <c r="R10" s="44" t="s">
         <v>172</v>
       </c>
-      <c r="Q10" s="57" t="s">
+      <c r="S10" s="44" t="s">
         <v>173</v>
       </c>
-      <c r="R10" s="57" t="s">
+      <c r="T10" s="44" t="s">
         <v>174</v>
       </c>
-      <c r="S10" s="57" t="s">
+      <c r="U10" s="44" t="s">
         <v>175</v>
       </c>
-      <c r="T10" s="57" t="s">
+      <c r="V10" s="44" t="s">
         <v>176</v>
       </c>
-      <c r="U10" s="57" t="s">
+      <c r="W10" s="44" t="s">
         <v>206</v>
       </c>
-      <c r="V10" s="57" t="s">
+      <c r="X10" s="44" t="s">
         <v>208</v>
       </c>
-      <c r="W10" s="57" t="s">
+      <c r="Y10" s="44" t="s">
         <v>209</v>
       </c>
-      <c r="X10" s="57" t="s">
+      <c r="Z10" s="44" t="s">
         <v>210</v>
       </c>
-      <c r="Y10" s="59" t="s">
+      <c r="AA10" s="46" t="s">
         <v>54</v>
       </c>
-      <c r="Z10" s="59" t="s">
+      <c r="AB10" s="46" t="s">
         <v>55</v>
       </c>
-      <c r="AA10" s="60" t="s">
+      <c r="AC10" s="47" t="s">
         <v>56</v>
       </c>
-      <c r="AB10" s="59" t="s">
+      <c r="AD10" s="46" t="s">
         <v>73</v>
       </c>
-      <c r="AC10" s="59" t="s">
+      <c r="AE10" s="46" t="s">
         <v>80</v>
       </c>
-      <c r="AD10" s="60" t="s">
+      <c r="AF10" s="47" t="s">
         <v>136</v>
       </c>
-      <c r="AE10" s="23" t="s">
+      <c r="AG10" s="23" t="s">
         <v>88</v>
       </c>
-      <c r="AF10" s="23" t="s">
+      <c r="AH10" s="23" t="s">
         <v>89</v>
       </c>
-      <c r="AG10" s="23" t="s">
+      <c r="AI10" s="23" t="s">
         <v>90</v>
       </c>
-      <c r="AH10" s="23" t="s">
+      <c r="AJ10" s="23" t="s">
         <v>165</v>
       </c>
-      <c r="AI10" s="23" t="s">
+      <c r="AK10" s="23" t="s">
         <v>94</v>
       </c>
-      <c r="AJ10" s="23" t="s">
+      <c r="AL10" s="23" t="s">
         <v>95</v>
       </c>
-      <c r="AK10" s="23" t="s">
+      <c r="AM10" s="23" t="s">
         <v>205</v>
       </c>
-      <c r="AL10" s="23" t="s">
+      <c r="AN10" s="23" t="s">
         <v>98</v>
       </c>
     </row>
-    <row r="11" spans="1:38" x14ac:dyDescent="0.2">
+    <row r="11" spans="1:40" x14ac:dyDescent="0.2">
       <c r="A11" s="3">
         <v>1</v>
       </c>
@@ -13565,8 +13588,10 @@
       <c r="AJ11" s="3"/>
       <c r="AK11" s="3"/>
       <c r="AL11" s="3"/>
-    </row>
-    <row r="12" spans="1:38" x14ac:dyDescent="0.2">
+      <c r="AM11" s="3"/>
+      <c r="AN11" s="3"/>
+    </row>
+    <row r="12" spans="1:40" x14ac:dyDescent="0.2">
       <c r="A12" s="3">
         <v>2</v>
       </c>
@@ -13605,10 +13630,12 @@
       <c r="AH12" s="3"/>
       <c r="AI12" s="3"/>
       <c r="AJ12" s="3"/>
-      <c r="AK12" s="18"/>
-      <c r="AL12" s="19"/>
-    </row>
-    <row r="13" spans="1:38" x14ac:dyDescent="0.2">
+      <c r="AK12" s="3"/>
+      <c r="AL12" s="3"/>
+      <c r="AM12" s="18"/>
+      <c r="AN12" s="19"/>
+    </row>
+    <row r="13" spans="1:40" x14ac:dyDescent="0.2">
       <c r="A13" s="3">
         <v>3</v>
       </c>
@@ -13647,10 +13674,12 @@
       <c r="AH13" s="3"/>
       <c r="AI13" s="3"/>
       <c r="AJ13" s="3"/>
-      <c r="AK13" s="18"/>
-      <c r="AL13" s="19"/>
-    </row>
-    <row r="14" spans="1:38" x14ac:dyDescent="0.2">
+      <c r="AK13" s="3"/>
+      <c r="AL13" s="3"/>
+      <c r="AM13" s="18"/>
+      <c r="AN13" s="19"/>
+    </row>
+    <row r="14" spans="1:40" x14ac:dyDescent="0.2">
       <c r="A14" s="3">
         <v>4</v>
       </c>
@@ -13691,8 +13720,10 @@
       <c r="AJ14" s="3"/>
       <c r="AK14" s="3"/>
       <c r="AL14" s="3"/>
-    </row>
-    <row r="15" spans="1:38" x14ac:dyDescent="0.2">
+      <c r="AM14" s="3"/>
+      <c r="AN14" s="3"/>
+    </row>
+    <row r="15" spans="1:40" x14ac:dyDescent="0.2">
       <c r="A15" s="3">
         <v>5</v>
       </c>
@@ -13733,8 +13764,10 @@
       <c r="AJ15" s="3"/>
       <c r="AK15" s="3"/>
       <c r="AL15" s="3"/>
-    </row>
-    <row r="16" spans="1:38" x14ac:dyDescent="0.2">
+      <c r="AM15" s="3"/>
+      <c r="AN15" s="3"/>
+    </row>
+    <row r="16" spans="1:40" x14ac:dyDescent="0.2">
       <c r="A16" s="3">
         <v>6</v>
       </c>
@@ -13775,8 +13808,10 @@
       <c r="AJ16" s="3"/>
       <c r="AK16" s="3"/>
       <c r="AL16" s="3"/>
-    </row>
-    <row r="17" spans="1:38" x14ac:dyDescent="0.2">
+      <c r="AM16" s="3"/>
+      <c r="AN16" s="3"/>
+    </row>
+    <row r="17" spans="1:40" x14ac:dyDescent="0.2">
       <c r="A17" s="3">
         <v>7</v>
       </c>
@@ -13817,8 +13852,10 @@
       <c r="AJ17" s="3"/>
       <c r="AK17" s="3"/>
       <c r="AL17" s="3"/>
-    </row>
-    <row r="18" spans="1:38" x14ac:dyDescent="0.2">
+      <c r="AM17" s="3"/>
+      <c r="AN17" s="3"/>
+    </row>
+    <row r="18" spans="1:40" x14ac:dyDescent="0.2">
       <c r="A18" s="3">
         <v>8</v>
       </c>
@@ -13859,8 +13896,10 @@
       <c r="AJ18" s="3"/>
       <c r="AK18" s="3"/>
       <c r="AL18" s="3"/>
-    </row>
-    <row r="19" spans="1:38" x14ac:dyDescent="0.2">
+      <c r="AM18" s="3"/>
+      <c r="AN18" s="3"/>
+    </row>
+    <row r="19" spans="1:40" x14ac:dyDescent="0.2">
       <c r="A19" s="3">
         <v>9</v>
       </c>
@@ -13901,8 +13940,10 @@
       <c r="AJ19" s="3"/>
       <c r="AK19" s="3"/>
       <c r="AL19" s="3"/>
-    </row>
-    <row r="20" spans="1:38" x14ac:dyDescent="0.2">
+      <c r="AM19" s="3"/>
+      <c r="AN19" s="3"/>
+    </row>
+    <row r="20" spans="1:40" x14ac:dyDescent="0.2">
       <c r="A20" s="3">
         <v>10</v>
       </c>
@@ -13943,8 +13984,10 @@
       <c r="AJ20" s="3"/>
       <c r="AK20" s="3"/>
       <c r="AL20" s="3"/>
-    </row>
-    <row r="21" spans="1:38" x14ac:dyDescent="0.2">
+      <c r="AM20" s="3"/>
+      <c r="AN20" s="3"/>
+    </row>
+    <row r="21" spans="1:40" x14ac:dyDescent="0.2">
       <c r="A21" s="3">
         <v>11</v>
       </c>
@@ -13985,8 +14028,10 @@
       <c r="AJ21" s="3"/>
       <c r="AK21" s="3"/>
       <c r="AL21" s="3"/>
-    </row>
-    <row r="22" spans="1:38" x14ac:dyDescent="0.2">
+      <c r="AM21" s="3"/>
+      <c r="AN21" s="3"/>
+    </row>
+    <row r="22" spans="1:40" x14ac:dyDescent="0.2">
       <c r="A22" s="3">
         <v>12</v>
       </c>
@@ -14027,8 +14072,10 @@
       <c r="AJ22" s="3"/>
       <c r="AK22" s="3"/>
       <c r="AL22" s="3"/>
-    </row>
-    <row r="23" spans="1:38" x14ac:dyDescent="0.2">
+      <c r="AM22" s="3"/>
+      <c r="AN22" s="3"/>
+    </row>
+    <row r="23" spans="1:40" x14ac:dyDescent="0.2">
       <c r="A23" s="3">
         <v>13</v>
       </c>
@@ -14069,8 +14116,10 @@
       <c r="AJ23" s="3"/>
       <c r="AK23" s="3"/>
       <c r="AL23" s="3"/>
-    </row>
-    <row r="24" spans="1:38" x14ac:dyDescent="0.2">
+      <c r="AM23" s="3"/>
+      <c r="AN23" s="3"/>
+    </row>
+    <row r="24" spans="1:40" x14ac:dyDescent="0.2">
       <c r="A24" s="3">
         <v>14</v>
       </c>
@@ -14111,8 +14160,10 @@
       <c r="AJ24" s="3"/>
       <c r="AK24" s="3"/>
       <c r="AL24" s="3"/>
-    </row>
-    <row r="25" spans="1:38" x14ac:dyDescent="0.2">
+      <c r="AM24" s="3"/>
+      <c r="AN24" s="3"/>
+    </row>
+    <row r="25" spans="1:40" x14ac:dyDescent="0.2">
       <c r="A25" s="3">
         <v>15</v>
       </c>
@@ -14153,8 +14204,10 @@
       <c r="AJ25" s="3"/>
       <c r="AK25" s="3"/>
       <c r="AL25" s="3"/>
-    </row>
-    <row r="26" spans="1:38" x14ac:dyDescent="0.2">
+      <c r="AM25" s="3"/>
+      <c r="AN25" s="3"/>
+    </row>
+    <row r="26" spans="1:40" x14ac:dyDescent="0.2">
       <c r="K26" s="1"/>
       <c r="L26" s="1"/>
       <c r="M26" s="1"/>
@@ -14183,8 +14236,10 @@
       <c r="AJ26" s="1"/>
       <c r="AK26" s="1"/>
       <c r="AL26" s="1"/>
-    </row>
-    <row r="27" spans="1:38" x14ac:dyDescent="0.2">
+      <c r="AM26" s="1"/>
+      <c r="AN26" s="1"/>
+    </row>
+    <row r="27" spans="1:40" x14ac:dyDescent="0.2">
       <c r="K27" s="1"/>
       <c r="L27" s="1"/>
       <c r="M27" s="1"/>
@@ -14205,8 +14260,10 @@
       <c r="AB27" s="1"/>
       <c r="AC27" s="1"/>
       <c r="AD27" s="1"/>
-    </row>
-    <row r="28" spans="1:38" x14ac:dyDescent="0.2">
+      <c r="AE27" s="1"/>
+      <c r="AF27" s="1"/>
+    </row>
+    <row r="28" spans="1:40" x14ac:dyDescent="0.2">
       <c r="K28" s="1"/>
       <c r="L28" s="1"/>
       <c r="M28" s="1"/>
@@ -14227,8 +14284,10 @@
       <c r="AB28" s="1"/>
       <c r="AC28" s="1"/>
       <c r="AD28" s="1"/>
-    </row>
-    <row r="29" spans="1:38" x14ac:dyDescent="0.2">
+      <c r="AE28" s="1"/>
+      <c r="AF28" s="1"/>
+    </row>
+    <row r="29" spans="1:40" x14ac:dyDescent="0.2">
       <c r="K29" s="1"/>
       <c r="L29" s="1"/>
       <c r="M29" s="1"/>
@@ -14249,8 +14308,10 @@
       <c r="AB29" s="1"/>
       <c r="AC29" s="1"/>
       <c r="AD29" s="1"/>
-    </row>
-    <row r="30" spans="1:38" x14ac:dyDescent="0.2">
+      <c r="AE29" s="1"/>
+      <c r="AF29" s="1"/>
+    </row>
+    <row r="30" spans="1:40" x14ac:dyDescent="0.2">
       <c r="K30" s="1"/>
       <c r="L30" s="1"/>
       <c r="M30" s="1"/>
@@ -14271,8 +14332,10 @@
       <c r="AB30" s="1"/>
       <c r="AC30" s="1"/>
       <c r="AD30" s="1"/>
-    </row>
-    <row r="31" spans="1:38" x14ac:dyDescent="0.2">
+      <c r="AE30" s="1"/>
+      <c r="AF30" s="1"/>
+    </row>
+    <row r="31" spans="1:40" x14ac:dyDescent="0.2">
       <c r="K31" s="1"/>
       <c r="L31" s="1"/>
       <c r="M31" s="1"/>
@@ -14293,8 +14356,10 @@
       <c r="AB31" s="1"/>
       <c r="AC31" s="1"/>
       <c r="AD31" s="1"/>
-    </row>
-    <row r="32" spans="1:38" x14ac:dyDescent="0.2">
+      <c r="AE31" s="1"/>
+      <c r="AF31" s="1"/>
+    </row>
+    <row r="32" spans="1:40" x14ac:dyDescent="0.2">
       <c r="K32" s="1"/>
       <c r="L32" s="1"/>
       <c r="M32" s="1"/>
@@ -14315,8 +14380,10 @@
       <c r="AB32" s="1"/>
       <c r="AC32" s="1"/>
       <c r="AD32" s="1"/>
-    </row>
-    <row r="33" spans="11:30" x14ac:dyDescent="0.2">
+      <c r="AE32" s="1"/>
+      <c r="AF32" s="1"/>
+    </row>
+    <row r="33" spans="11:32" x14ac:dyDescent="0.2">
       <c r="K33" s="1"/>
       <c r="L33" s="1"/>
       <c r="M33" s="1"/>
@@ -14337,8 +14404,10 @@
       <c r="AB33" s="1"/>
       <c r="AC33" s="1"/>
       <c r="AD33" s="1"/>
-    </row>
-    <row r="34" spans="11:30" x14ac:dyDescent="0.2">
+      <c r="AE33" s="1"/>
+      <c r="AF33" s="1"/>
+    </row>
+    <row r="34" spans="11:32" x14ac:dyDescent="0.2">
       <c r="K34" s="1"/>
       <c r="L34" s="1"/>
       <c r="M34" s="1"/>
@@ -14359,8 +14428,10 @@
       <c r="AB34" s="1"/>
       <c r="AC34" s="1"/>
       <c r="AD34" s="1"/>
-    </row>
-    <row r="35" spans="11:30" x14ac:dyDescent="0.2">
+      <c r="AE34" s="1"/>
+      <c r="AF34" s="1"/>
+    </row>
+    <row r="35" spans="11:32" x14ac:dyDescent="0.2">
       <c r="K35" s="1"/>
       <c r="L35" s="1"/>
       <c r="M35" s="1"/>
@@ -14381,8 +14452,10 @@
       <c r="AB35" s="1"/>
       <c r="AC35" s="1"/>
       <c r="AD35" s="1"/>
-    </row>
-    <row r="36" spans="11:30" x14ac:dyDescent="0.2">
+      <c r="AE35" s="1"/>
+      <c r="AF35" s="1"/>
+    </row>
+    <row r="36" spans="11:32" x14ac:dyDescent="0.2">
       <c r="K36" s="1"/>
       <c r="L36" s="1"/>
       <c r="M36" s="1"/>
@@ -14403,8 +14476,10 @@
       <c r="AB36" s="1"/>
       <c r="AC36" s="1"/>
       <c r="AD36" s="1"/>
-    </row>
-    <row r="37" spans="11:30" x14ac:dyDescent="0.2">
+      <c r="AE36" s="1"/>
+      <c r="AF36" s="1"/>
+    </row>
+    <row r="37" spans="11:32" x14ac:dyDescent="0.2">
       <c r="K37" s="1"/>
       <c r="L37" s="1"/>
       <c r="M37" s="1"/>
@@ -14425,8 +14500,10 @@
       <c r="AB37" s="1"/>
       <c r="AC37" s="1"/>
       <c r="AD37" s="1"/>
-    </row>
-    <row r="38" spans="11:30" x14ac:dyDescent="0.2">
+      <c r="AE37" s="1"/>
+      <c r="AF37" s="1"/>
+    </row>
+    <row r="38" spans="11:32" x14ac:dyDescent="0.2">
       <c r="K38" s="1"/>
       <c r="L38" s="1"/>
       <c r="M38" s="1"/>
@@ -14447,8 +14524,10 @@
       <c r="AB38" s="1"/>
       <c r="AC38" s="1"/>
       <c r="AD38" s="1"/>
-    </row>
-    <row r="39" spans="11:30" x14ac:dyDescent="0.2">
+      <c r="AE38" s="1"/>
+      <c r="AF38" s="1"/>
+    </row>
+    <row r="39" spans="11:32" x14ac:dyDescent="0.2">
       <c r="K39" s="1"/>
       <c r="L39" s="1"/>
       <c r="M39" s="1"/>
@@ -14469,8 +14548,10 @@
       <c r="AB39" s="1"/>
       <c r="AC39" s="1"/>
       <c r="AD39" s="1"/>
-    </row>
-    <row r="40" spans="11:30" x14ac:dyDescent="0.2">
+      <c r="AE39" s="1"/>
+      <c r="AF39" s="1"/>
+    </row>
+    <row r="40" spans="11:32" x14ac:dyDescent="0.2">
       <c r="K40" s="1"/>
       <c r="L40" s="1"/>
       <c r="M40" s="1"/>
@@ -14491,8 +14572,10 @@
       <c r="AB40" s="1"/>
       <c r="AC40" s="1"/>
       <c r="AD40" s="1"/>
-    </row>
-    <row r="41" spans="11:30" x14ac:dyDescent="0.2">
+      <c r="AE40" s="1"/>
+      <c r="AF40" s="1"/>
+    </row>
+    <row r="41" spans="11:32" x14ac:dyDescent="0.2">
       <c r="K41" s="1"/>
       <c r="L41" s="1"/>
       <c r="M41" s="1"/>
@@ -14513,8 +14596,10 @@
       <c r="AB41" s="1"/>
       <c r="AC41" s="1"/>
       <c r="AD41" s="1"/>
-    </row>
-    <row r="42" spans="11:30" x14ac:dyDescent="0.2">
+      <c r="AE41" s="1"/>
+      <c r="AF41" s="1"/>
+    </row>
+    <row r="42" spans="11:32" x14ac:dyDescent="0.2">
       <c r="K42" s="1"/>
       <c r="L42" s="1"/>
       <c r="M42" s="1"/>
@@ -14535,8 +14620,10 @@
       <c r="AB42" s="1"/>
       <c r="AC42" s="1"/>
       <c r="AD42" s="1"/>
-    </row>
-    <row r="43" spans="11:30" x14ac:dyDescent="0.2">
+      <c r="AE42" s="1"/>
+      <c r="AF42" s="1"/>
+    </row>
+    <row r="43" spans="11:32" x14ac:dyDescent="0.2">
       <c r="K43" s="1"/>
       <c r="L43" s="1"/>
       <c r="M43" s="1"/>
@@ -14557,8 +14644,10 @@
       <c r="AB43" s="1"/>
       <c r="AC43" s="1"/>
       <c r="AD43" s="1"/>
-    </row>
-    <row r="44" spans="11:30" x14ac:dyDescent="0.2">
+      <c r="AE43" s="1"/>
+      <c r="AF43" s="1"/>
+    </row>
+    <row r="44" spans="11:32" x14ac:dyDescent="0.2">
       <c r="K44" s="1"/>
       <c r="L44" s="1"/>
       <c r="M44" s="1"/>
@@ -14579,8 +14668,10 @@
       <c r="AB44" s="1"/>
       <c r="AC44" s="1"/>
       <c r="AD44" s="1"/>
-    </row>
-    <row r="45" spans="11:30" x14ac:dyDescent="0.2">
+      <c r="AE44" s="1"/>
+      <c r="AF44" s="1"/>
+    </row>
+    <row r="45" spans="11:32" x14ac:dyDescent="0.2">
       <c r="K45" s="1"/>
       <c r="L45" s="1"/>
       <c r="M45" s="1"/>
@@ -14601,8 +14692,10 @@
       <c r="AB45" s="1"/>
       <c r="AC45" s="1"/>
       <c r="AD45" s="1"/>
-    </row>
-    <row r="46" spans="11:30" x14ac:dyDescent="0.2">
+      <c r="AE45" s="1"/>
+      <c r="AF45" s="1"/>
+    </row>
+    <row r="46" spans="11:32" x14ac:dyDescent="0.2">
       <c r="K46" s="1"/>
       <c r="L46" s="1"/>
       <c r="M46" s="1"/>
@@ -14623,8 +14716,10 @@
       <c r="AB46" s="1"/>
       <c r="AC46" s="1"/>
       <c r="AD46" s="1"/>
-    </row>
-    <row r="47" spans="11:30" x14ac:dyDescent="0.2">
+      <c r="AE46" s="1"/>
+      <c r="AF46" s="1"/>
+    </row>
+    <row r="47" spans="11:32" x14ac:dyDescent="0.2">
       <c r="K47" s="1"/>
       <c r="L47" s="1"/>
       <c r="M47" s="1"/>
@@ -14645,8 +14740,10 @@
       <c r="AB47" s="1"/>
       <c r="AC47" s="1"/>
       <c r="AD47" s="1"/>
-    </row>
-    <row r="48" spans="11:30" x14ac:dyDescent="0.2">
+      <c r="AE47" s="1"/>
+      <c r="AF47" s="1"/>
+    </row>
+    <row r="48" spans="11:32" x14ac:dyDescent="0.2">
       <c r="K48" s="1"/>
       <c r="L48" s="1"/>
       <c r="M48" s="1"/>
@@ -14667,8 +14764,10 @@
       <c r="AB48" s="1"/>
       <c r="AC48" s="1"/>
       <c r="AD48" s="1"/>
-    </row>
-    <row r="49" spans="11:30" x14ac:dyDescent="0.2">
+      <c r="AE48" s="1"/>
+      <c r="AF48" s="1"/>
+    </row>
+    <row r="49" spans="11:32" x14ac:dyDescent="0.2">
       <c r="K49" s="1"/>
       <c r="L49" s="1"/>
       <c r="M49" s="1"/>
@@ -14689,8 +14788,10 @@
       <c r="AB49" s="1"/>
       <c r="AC49" s="1"/>
       <c r="AD49" s="1"/>
-    </row>
-    <row r="50" spans="11:30" x14ac:dyDescent="0.2">
+      <c r="AE49" s="1"/>
+      <c r="AF49" s="1"/>
+    </row>
+    <row r="50" spans="11:32" x14ac:dyDescent="0.2">
       <c r="K50" s="1"/>
       <c r="L50" s="1"/>
       <c r="M50" s="1"/>
@@ -14711,8 +14812,10 @@
       <c r="AB50" s="1"/>
       <c r="AC50" s="1"/>
       <c r="AD50" s="1"/>
-    </row>
-    <row r="51" spans="11:30" x14ac:dyDescent="0.2">
+      <c r="AE50" s="1"/>
+      <c r="AF50" s="1"/>
+    </row>
+    <row r="51" spans="11:32" x14ac:dyDescent="0.2">
       <c r="K51" s="1"/>
       <c r="L51" s="1"/>
       <c r="M51" s="1"/>
@@ -14733,8 +14836,10 @@
       <c r="AB51" s="1"/>
       <c r="AC51" s="1"/>
       <c r="AD51" s="1"/>
-    </row>
-    <row r="52" spans="11:30" x14ac:dyDescent="0.2">
+      <c r="AE51" s="1"/>
+      <c r="AF51" s="1"/>
+    </row>
+    <row r="52" spans="11:32" x14ac:dyDescent="0.2">
       <c r="K52" s="1"/>
       <c r="L52" s="1"/>
       <c r="M52" s="1"/>
@@ -14755,100 +14860,102 @@
       <c r="AB52" s="1"/>
       <c r="AC52" s="1"/>
       <c r="AD52" s="1"/>
+      <c r="AE52" s="1"/>
+      <c r="AF52" s="1"/>
     </row>
   </sheetData>
   <mergeCells count="3">
-    <mergeCell ref="Y9:AD9"/>
-    <mergeCell ref="AE9:AL9"/>
-    <mergeCell ref="C9:X9"/>
+    <mergeCell ref="AA9:AF9"/>
+    <mergeCell ref="AG9:AN9"/>
+    <mergeCell ref="C9:Z9"/>
   </mergeCells>
-  <conditionalFormatting sqref="F11:K52 Z11:AD52">
-    <cfRule type="expression" dxfId="5" priority="1">
+  <conditionalFormatting sqref="F11:M52 AB11:AF52">
+    <cfRule type="expression" dxfId="18" priority="1">
       <formula>$E11="hb"</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="5" priority="2">
+    <cfRule type="expression" dxfId="17" priority="2">
       <formula>$E11="pow"</formula>
     </cfRule>
   </conditionalFormatting>
+  <conditionalFormatting sqref="F11:N52">
+    <cfRule type="expression" dxfId="16" priority="14">
+      <formula>$E11="elastic"</formula>
+    </cfRule>
+  </conditionalFormatting>
   <conditionalFormatting sqref="G11:G52">
-    <cfRule type="expression" dxfId="5" priority="3">
+    <cfRule type="expression" dxfId="15" priority="3">
       <formula>$E11="cp"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="H11:I52">
-    <cfRule type="expression" dxfId="5" priority="4">
+    <cfRule type="expression" dxfId="14" priority="4">
       <formula>$E11="mc"</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="J11:K52">
-    <cfRule type="expression" dxfId="5" priority="5">
+  <conditionalFormatting sqref="J11:M52">
+    <cfRule type="expression" dxfId="13" priority="5">
       <formula>$E11="cp"</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="Q11:T52">
-    <cfRule type="expression" dxfId="5" priority="6">
+  <conditionalFormatting sqref="Q11:R52">
+    <cfRule type="expression" dxfId="12" priority="15">
+      <formula>$E11="elastic"</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="R11:R52">
+    <cfRule type="expression" dxfId="11" priority="8">
+      <formula>AND($Q11&lt;&gt;"",$Q11&lt;&gt;"ru")</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="S11:V52">
+    <cfRule type="expression" dxfId="10" priority="6">
       <formula>AND($E11&lt;&gt;"",$E11&lt;&gt;"pow")</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="U11:X52">
-    <cfRule type="expression" dxfId="5" priority="7">
+  <conditionalFormatting sqref="W11:Z52">
+    <cfRule type="expression" dxfId="9" priority="7">
       <formula>AND($E11&lt;&gt;"",$E11&lt;&gt;"hb")</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="P11:P52">
-    <cfRule type="expression" dxfId="5" priority="8">
-      <formula>AND($O11&lt;&gt;"",$O11&lt;&gt;"ru")</formula>
+  <conditionalFormatting sqref="AB11:AF52">
+    <cfRule type="expression" dxfId="8" priority="16">
+      <formula>$E11="elastic"</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="AA11:AA52">
-    <cfRule type="expression" dxfId="5" priority="9">
+  <conditionalFormatting sqref="AC11:AC52">
+    <cfRule type="expression" dxfId="7" priority="9">
       <formula>$E11="cp"</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="AB11:AB52">
-    <cfRule type="expression" dxfId="5" priority="10">
+  <conditionalFormatting sqref="AD11:AD52">
+    <cfRule type="expression" dxfId="6" priority="10">
       <formula>$E11="mc"</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="AC11:AD52">
+  <conditionalFormatting sqref="AE11:AF52">
     <cfRule type="expression" dxfId="5" priority="11">
       <formula>$E11="cp"</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="AI11:AJ52">
-    <cfRule type="expression" dxfId="5" priority="12">
-      <formula>OR($AH11="vg",$AH11="gard")</formula>
+  <conditionalFormatting sqref="AK11:AL52">
+    <cfRule type="expression" dxfId="4" priority="12">
+      <formula>OR($AJ11="vg",$AJ11="gard")</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="AK11:AL52">
-    <cfRule type="expression" dxfId="5" priority="13">
-      <formula>$AH11="lf"</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="F11:L52">
-    <cfRule type="expression" dxfId="5" priority="14">
-      <formula>$E11="elastic"</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="O11:P52">
-    <cfRule type="expression" dxfId="5" priority="15">
-      <formula>$E11="elastic"</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="Z11:AD52">
-    <cfRule type="expression" dxfId="5" priority="16">
-      <formula>$E11="elastic"</formula>
+  <conditionalFormatting sqref="AM11:AN52">
+    <cfRule type="expression" dxfId="3" priority="13">
+      <formula>$AJ11="lf"</formula>
     </cfRule>
   </conditionalFormatting>
   <dataValidations count="3">
     <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="E11:E52" xr:uid="{374AFD2C-B540-DD4B-A245-8B781F76E64C}">
       <formula1>$C$3:$C$7</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="AH11:AH102" xr:uid="{E00A94A9-D864-5843-8FBD-E84775B1C100}">
-      <formula1>$AH$3:$AH$5</formula1>
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="AJ11:AJ102" xr:uid="{E00A94A9-D864-5843-8FBD-E84775B1C100}">
+      <formula1>$AJ$3:$AJ$5</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="O11:O52" xr:uid="{D770415C-1ECE-F44B-9D8C-08EF1CF31C8E}">
-      <formula1>$O$3:$O$6</formula1>
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="Q11:Q52" xr:uid="{D770415C-1ECE-F44B-9D8C-08EF1CF31C8E}">
+      <formula1>$Q$3:$Q$6</formula1>
     </dataValidation>
   </dataValidations>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -14893,74 +15000,74 @@
       </c>
     </row>
     <row r="4" spans="1:44" x14ac:dyDescent="0.2">
-      <c r="A4" s="48" t="s">
+      <c r="A4" s="52" t="s">
         <v>2</v>
       </c>
-      <c r="B4" s="48"/>
-      <c r="D4" s="48" t="s">
+      <c r="B4" s="52"/>
+      <c r="D4" s="52" t="s">
         <v>5</v>
       </c>
-      <c r="E4" s="48"/>
-      <c r="G4" s="48" t="s">
+      <c r="E4" s="52"/>
+      <c r="G4" s="52" t="s">
         <v>6</v>
       </c>
-      <c r="H4" s="48"/>
-      <c r="J4" s="48" t="s">
+      <c r="H4" s="52"/>
+      <c r="J4" s="52" t="s">
         <v>7</v>
       </c>
-      <c r="K4" s="48"/>
-      <c r="M4" s="48" t="s">
+      <c r="K4" s="52"/>
+      <c r="M4" s="52" t="s">
         <v>8</v>
       </c>
-      <c r="N4" s="48"/>
-      <c r="P4" s="48" t="s">
+      <c r="N4" s="52"/>
+      <c r="P4" s="52" t="s">
         <v>9</v>
       </c>
-      <c r="Q4" s="48"/>
+      <c r="Q4" s="52"/>
       <c r="R4" s="1"/>
-      <c r="S4" s="48" t="s">
+      <c r="S4" s="52" t="s">
         <v>10</v>
       </c>
-      <c r="T4" s="48"/>
+      <c r="T4" s="52"/>
       <c r="U4" s="1"/>
-      <c r="V4" s="48" t="s">
+      <c r="V4" s="52" t="s">
         <v>11</v>
       </c>
-      <c r="W4" s="48"/>
+      <c r="W4" s="52"/>
       <c r="X4" s="1"/>
-      <c r="Y4" s="48" t="s">
+      <c r="Y4" s="52" t="s">
         <v>12</v>
       </c>
-      <c r="Z4" s="48"/>
+      <c r="Z4" s="52"/>
       <c r="AA4" s="1"/>
-      <c r="AB4" s="48" t="s">
+      <c r="AB4" s="52" t="s">
         <v>13</v>
       </c>
-      <c r="AC4" s="48"/>
-      <c r="AE4" s="48" t="s">
+      <c r="AC4" s="52"/>
+      <c r="AE4" s="52" t="s">
         <v>108</v>
       </c>
-      <c r="AF4" s="48"/>
+      <c r="AF4" s="52"/>
       <c r="AG4" s="1"/>
-      <c r="AH4" s="48" t="s">
+      <c r="AH4" s="52" t="s">
         <v>109</v>
       </c>
-      <c r="AI4" s="48"/>
+      <c r="AI4" s="52"/>
       <c r="AJ4" s="1"/>
-      <c r="AK4" s="48" t="s">
+      <c r="AK4" s="52" t="s">
         <v>110</v>
       </c>
-      <c r="AL4" s="48"/>
+      <c r="AL4" s="52"/>
       <c r="AM4" s="1"/>
-      <c r="AN4" s="48" t="s">
+      <c r="AN4" s="52" t="s">
         <v>111</v>
       </c>
-      <c r="AO4" s="48"/>
+      <c r="AO4" s="52"/>
       <c r="AP4" s="1"/>
-      <c r="AQ4" s="48" t="s">
+      <c r="AQ4" s="52" t="s">
         <v>112</v>
       </c>
-      <c r="AR4" s="48"/>
+      <c r="AR4" s="52"/>
     </row>
     <row r="5" spans="1:44" x14ac:dyDescent="0.2">
       <c r="A5" s="36" t="s">
@@ -15063,89 +15170,89 @@
       </c>
     </row>
     <row r="6" spans="1:44" x14ac:dyDescent="0.2">
-      <c r="A6" s="46" t="str">
+      <c r="A6" s="53" t="str">
         <f>_xlfn.XLOOKUP(B5,mat!$A:$A, mat!$B:$B,"") &amp; ""</f>
         <v/>
       </c>
-      <c r="B6" s="47"/>
-      <c r="D6" s="46" t="str">
+      <c r="B6" s="54"/>
+      <c r="D6" s="53" t="str">
         <f>_xlfn.XLOOKUP(E5,mat!$A:$A, mat!$B:$B,"") &amp; ""</f>
         <v/>
       </c>
-      <c r="E6" s="47"/>
-      <c r="G6" s="46" t="str">
+      <c r="E6" s="54"/>
+      <c r="G6" s="53" t="str">
         <f>_xlfn.XLOOKUP(H5,mat!$A:$A, mat!$B:$B,"") &amp; ""</f>
         <v/>
       </c>
-      <c r="H6" s="47"/>
-      <c r="J6" s="46" t="str">
+      <c r="H6" s="54"/>
+      <c r="J6" s="53" t="str">
         <f>_xlfn.XLOOKUP(K5,mat!$A:$A, mat!$B:$B,"") &amp; ""</f>
         <v/>
       </c>
-      <c r="K6" s="47"/>
-      <c r="M6" s="46" t="str">
+      <c r="K6" s="54"/>
+      <c r="M6" s="53" t="str">
         <f>_xlfn.XLOOKUP(N5,mat!$A:$A, mat!$B:$B,"") &amp; ""</f>
         <v/>
       </c>
-      <c r="N6" s="47"/>
-      <c r="P6" s="46" t="str">
+      <c r="N6" s="54"/>
+      <c r="P6" s="53" t="str">
         <f>_xlfn.XLOOKUP(Q5,mat!$A:$A, mat!$B:$B,"") &amp; ""</f>
         <v/>
       </c>
-      <c r="Q6" s="47"/>
+      <c r="Q6" s="54"/>
       <c r="R6" s="1"/>
-      <c r="S6" s="46" t="str">
+      <c r="S6" s="53" t="str">
         <f>_xlfn.XLOOKUP(T5,mat!$A:$A, mat!$B:$B,"") &amp; ""</f>
         <v/>
       </c>
-      <c r="T6" s="47"/>
+      <c r="T6" s="54"/>
       <c r="U6" s="1"/>
-      <c r="V6" s="46" t="str">
+      <c r="V6" s="53" t="str">
         <f>_xlfn.XLOOKUP(W5,mat!$A:$A, mat!$B:$B,"") &amp; ""</f>
         <v/>
       </c>
-      <c r="W6" s="47"/>
+      <c r="W6" s="54"/>
       <c r="X6" s="1"/>
-      <c r="Y6" s="46" t="str">
+      <c r="Y6" s="53" t="str">
         <f>_xlfn.XLOOKUP(Z5,mat!$A:$A, mat!$B:$B,"") &amp; ""</f>
         <v/>
       </c>
-      <c r="Z6" s="47"/>
+      <c r="Z6" s="54"/>
       <c r="AA6" s="1"/>
-      <c r="AB6" s="46" t="str">
+      <c r="AB6" s="53" t="str">
         <f>_xlfn.XLOOKUP(AC5,mat!$A:$A, mat!$B:$B,"") &amp; ""</f>
         <v/>
       </c>
-      <c r="AC6" s="47"/>
-      <c r="AE6" s="46" t="str">
+      <c r="AC6" s="54"/>
+      <c r="AE6" s="53" t="str">
         <f>_xlfn.XLOOKUP(AF5,mat!$A:$A, mat!$B:$B,"") &amp; ""</f>
         <v/>
       </c>
-      <c r="AF6" s="47"/>
+      <c r="AF6" s="54"/>
       <c r="AG6" s="1"/>
-      <c r="AH6" s="46" t="str">
+      <c r="AH6" s="53" t="str">
         <f>_xlfn.XLOOKUP(AI5,mat!$A:$A, mat!$B:$B,"") &amp; ""</f>
         <v/>
       </c>
-      <c r="AI6" s="47"/>
+      <c r="AI6" s="54"/>
       <c r="AJ6" s="1"/>
-      <c r="AK6" s="46" t="str">
+      <c r="AK6" s="53" t="str">
         <f>_xlfn.XLOOKUP(AL5,mat!$A:$A, mat!$B:$B,"") &amp; ""</f>
         <v/>
       </c>
-      <c r="AL6" s="47"/>
+      <c r="AL6" s="54"/>
       <c r="AM6" s="1"/>
-      <c r="AN6" s="46" t="str">
+      <c r="AN6" s="53" t="str">
         <f>_xlfn.XLOOKUP(AO5,mat!$A:$A, mat!$B:$B,"") &amp; ""</f>
         <v/>
       </c>
-      <c r="AO6" s="47"/>
+      <c r="AO6" s="54"/>
       <c r="AP6" s="1"/>
-      <c r="AQ6" s="46" t="str">
+      <c r="AQ6" s="53" t="str">
         <f>_xlfn.XLOOKUP(AR5,mat!$A:$A, mat!$B:$B,"") &amp; ""</f>
         <v/>
       </c>
-      <c r="AR6" s="47"/>
+      <c r="AR6" s="54"/>
     </row>
     <row r="7" spans="1:44" x14ac:dyDescent="0.2">
       <c r="A7" s="2" t="s">
@@ -16049,36 +16156,36 @@
     </row>
   </sheetData>
   <mergeCells count="30">
+    <mergeCell ref="AE6:AF6"/>
+    <mergeCell ref="AH6:AI6"/>
+    <mergeCell ref="AK6:AL6"/>
+    <mergeCell ref="AN6:AO6"/>
+    <mergeCell ref="AQ6:AR6"/>
+    <mergeCell ref="P6:Q6"/>
+    <mergeCell ref="S6:T6"/>
+    <mergeCell ref="V6:W6"/>
+    <mergeCell ref="Y6:Z6"/>
+    <mergeCell ref="AB6:AC6"/>
+    <mergeCell ref="A6:B6"/>
+    <mergeCell ref="D6:E6"/>
+    <mergeCell ref="G6:H6"/>
+    <mergeCell ref="J6:K6"/>
+    <mergeCell ref="M6:N6"/>
+    <mergeCell ref="AE4:AF4"/>
+    <mergeCell ref="AH4:AI4"/>
+    <mergeCell ref="AK4:AL4"/>
+    <mergeCell ref="AN4:AO4"/>
+    <mergeCell ref="AQ4:AR4"/>
+    <mergeCell ref="P4:Q4"/>
+    <mergeCell ref="S4:T4"/>
+    <mergeCell ref="V4:W4"/>
+    <mergeCell ref="Y4:Z4"/>
+    <mergeCell ref="AB4:AC4"/>
     <mergeCell ref="A4:B4"/>
     <mergeCell ref="D4:E4"/>
     <mergeCell ref="G4:H4"/>
     <mergeCell ref="J4:K4"/>
     <mergeCell ref="M4:N4"/>
-    <mergeCell ref="P4:Q4"/>
-    <mergeCell ref="S4:T4"/>
-    <mergeCell ref="V4:W4"/>
-    <mergeCell ref="Y4:Z4"/>
-    <mergeCell ref="AB4:AC4"/>
-    <mergeCell ref="AE4:AF4"/>
-    <mergeCell ref="AH4:AI4"/>
-    <mergeCell ref="AK4:AL4"/>
-    <mergeCell ref="AN4:AO4"/>
-    <mergeCell ref="AQ4:AR4"/>
-    <mergeCell ref="A6:B6"/>
-    <mergeCell ref="D6:E6"/>
-    <mergeCell ref="G6:H6"/>
-    <mergeCell ref="J6:K6"/>
-    <mergeCell ref="M6:N6"/>
-    <mergeCell ref="P6:Q6"/>
-    <mergeCell ref="S6:T6"/>
-    <mergeCell ref="V6:W6"/>
-    <mergeCell ref="Y6:Z6"/>
-    <mergeCell ref="AB6:AC6"/>
-    <mergeCell ref="AE6:AF6"/>
-    <mergeCell ref="AH6:AI6"/>
-    <mergeCell ref="AK6:AL6"/>
-    <mergeCell ref="AN6:AO6"/>
-    <mergeCell ref="AQ6:AR6"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
@@ -16116,74 +16223,74 @@
       </c>
     </row>
     <row r="4" spans="1:44" x14ac:dyDescent="0.2">
-      <c r="A4" s="48" t="s">
+      <c r="A4" s="52" t="s">
         <v>137</v>
       </c>
-      <c r="B4" s="48"/>
-      <c r="D4" s="48" t="s">
+      <c r="B4" s="52"/>
+      <c r="D4" s="52" t="s">
         <v>138</v>
       </c>
-      <c r="E4" s="48"/>
-      <c r="G4" s="48" t="s">
+      <c r="E4" s="52"/>
+      <c r="G4" s="52" t="s">
         <v>139</v>
       </c>
-      <c r="H4" s="48"/>
-      <c r="J4" s="48" t="s">
+      <c r="H4" s="52"/>
+      <c r="J4" s="52" t="s">
         <v>140</v>
       </c>
-      <c r="K4" s="48"/>
-      <c r="M4" s="48" t="s">
+      <c r="K4" s="52"/>
+      <c r="M4" s="52" t="s">
         <v>141</v>
       </c>
-      <c r="N4" s="48"/>
-      <c r="P4" s="48" t="s">
+      <c r="N4" s="52"/>
+      <c r="P4" s="52" t="s">
         <v>142</v>
       </c>
-      <c r="Q4" s="48"/>
+      <c r="Q4" s="52"/>
       <c r="R4" s="1"/>
-      <c r="S4" s="48" t="s">
+      <c r="S4" s="52" t="s">
         <v>143</v>
       </c>
-      <c r="T4" s="48"/>
+      <c r="T4" s="52"/>
       <c r="U4" s="1"/>
-      <c r="V4" s="48" t="s">
+      <c r="V4" s="52" t="s">
         <v>144</v>
       </c>
-      <c r="W4" s="48"/>
+      <c r="W4" s="52"/>
       <c r="X4" s="1"/>
-      <c r="Y4" s="48" t="s">
+      <c r="Y4" s="52" t="s">
         <v>145</v>
       </c>
-      <c r="Z4" s="48"/>
+      <c r="Z4" s="52"/>
       <c r="AA4" s="1"/>
-      <c r="AB4" s="48" t="s">
+      <c r="AB4" s="52" t="s">
         <v>146</v>
       </c>
-      <c r="AC4" s="48"/>
-      <c r="AE4" s="48" t="s">
+      <c r="AC4" s="52"/>
+      <c r="AE4" s="52" t="s">
         <v>147</v>
       </c>
-      <c r="AF4" s="48"/>
+      <c r="AF4" s="52"/>
       <c r="AG4" s="1"/>
-      <c r="AH4" s="48" t="s">
+      <c r="AH4" s="52" t="s">
         <v>148</v>
       </c>
-      <c r="AI4" s="48"/>
+      <c r="AI4" s="52"/>
       <c r="AJ4" s="1"/>
-      <c r="AK4" s="48" t="s">
+      <c r="AK4" s="52" t="s">
         <v>149</v>
       </c>
-      <c r="AL4" s="48"/>
+      <c r="AL4" s="52"/>
       <c r="AM4" s="1"/>
-      <c r="AN4" s="48" t="s">
+      <c r="AN4" s="52" t="s">
         <v>150</v>
       </c>
-      <c r="AO4" s="48"/>
+      <c r="AO4" s="52"/>
       <c r="AP4" s="1"/>
-      <c r="AQ4" s="48" t="s">
+      <c r="AQ4" s="52" t="s">
         <v>151</v>
       </c>
-      <c r="AR4" s="48"/>
+      <c r="AR4" s="52"/>
     </row>
     <row r="5" spans="1:44" x14ac:dyDescent="0.2">
       <c r="A5" s="38" t="s">
@@ -16286,89 +16393,89 @@
       </c>
     </row>
     <row r="6" spans="1:44" x14ac:dyDescent="0.2">
-      <c r="A6" s="49" t="str">
+      <c r="A6" s="55" t="str">
         <f>_xlfn.XLOOKUP(B5,mat!$A:$A, mat!$B:$B,"") &amp; ""</f>
         <v/>
       </c>
-      <c r="B6" s="50"/>
-      <c r="D6" s="49" t="str">
+      <c r="B6" s="56"/>
+      <c r="D6" s="55" t="str">
         <f>_xlfn.XLOOKUP(E5,mat!$A:$A, mat!$B:$B,"") &amp; ""</f>
         <v/>
       </c>
-      <c r="E6" s="50"/>
-      <c r="G6" s="49" t="str">
+      <c r="E6" s="56"/>
+      <c r="G6" s="55" t="str">
         <f>_xlfn.XLOOKUP(H5,mat!$A:$A, mat!$B:$B,"") &amp; ""</f>
         <v/>
       </c>
-      <c r="H6" s="50"/>
-      <c r="J6" s="49" t="str">
+      <c r="H6" s="56"/>
+      <c r="J6" s="55" t="str">
         <f>_xlfn.XLOOKUP(K5,mat!$A:$A, mat!$B:$B,"") &amp; ""</f>
         <v/>
       </c>
-      <c r="K6" s="50"/>
-      <c r="M6" s="49" t="str">
+      <c r="K6" s="56"/>
+      <c r="M6" s="55" t="str">
         <f>_xlfn.XLOOKUP(N5,mat!$A:$A, mat!$B:$B,"") &amp; ""</f>
         <v/>
       </c>
-      <c r="N6" s="50"/>
-      <c r="P6" s="49" t="str">
+      <c r="N6" s="56"/>
+      <c r="P6" s="55" t="str">
         <f>_xlfn.XLOOKUP(Q5,mat!$A:$A, mat!$B:$B,"") &amp; ""</f>
         <v/>
       </c>
-      <c r="Q6" s="50"/>
+      <c r="Q6" s="56"/>
       <c r="R6" s="1"/>
-      <c r="S6" s="49" t="str">
+      <c r="S6" s="55" t="str">
         <f>_xlfn.XLOOKUP(T5,mat!$A:$A, mat!$B:$B,"") &amp; ""</f>
         <v/>
       </c>
-      <c r="T6" s="50"/>
+      <c r="T6" s="56"/>
       <c r="U6" s="1"/>
-      <c r="V6" s="49" t="str">
+      <c r="V6" s="55" t="str">
         <f>_xlfn.XLOOKUP(W5,mat!$A:$A, mat!$B:$B,"") &amp; ""</f>
         <v/>
       </c>
-      <c r="W6" s="50"/>
+      <c r="W6" s="56"/>
       <c r="X6" s="1"/>
-      <c r="Y6" s="49" t="str">
+      <c r="Y6" s="55" t="str">
         <f>_xlfn.XLOOKUP(Z5,mat!$A:$A, mat!$B:$B,"") &amp; ""</f>
         <v/>
       </c>
-      <c r="Z6" s="50"/>
+      <c r="Z6" s="56"/>
       <c r="AA6" s="1"/>
-      <c r="AB6" s="49" t="str">
+      <c r="AB6" s="55" t="str">
         <f>_xlfn.XLOOKUP(AC5,mat!$A:$A, mat!$B:$B,"") &amp; ""</f>
         <v/>
       </c>
-      <c r="AC6" s="50"/>
-      <c r="AE6" s="49" t="str">
+      <c r="AC6" s="56"/>
+      <c r="AE6" s="55" t="str">
         <f>_xlfn.XLOOKUP(AF5,mat!$A:$A, mat!$B:$B,"") &amp; ""</f>
         <v/>
       </c>
-      <c r="AF6" s="50"/>
+      <c r="AF6" s="56"/>
       <c r="AG6" s="1"/>
-      <c r="AH6" s="49" t="str">
+      <c r="AH6" s="55" t="str">
         <f>_xlfn.XLOOKUP(AI5,mat!$A:$A, mat!$B:$B,"") &amp; ""</f>
         <v/>
       </c>
-      <c r="AI6" s="50"/>
+      <c r="AI6" s="56"/>
       <c r="AJ6" s="1"/>
-      <c r="AK6" s="49" t="str">
+      <c r="AK6" s="55" t="str">
         <f>_xlfn.XLOOKUP(AL5,mat!$A:$A, mat!$B:$B,"") &amp; ""</f>
         <v/>
       </c>
-      <c r="AL6" s="50"/>
+      <c r="AL6" s="56"/>
       <c r="AM6" s="1"/>
-      <c r="AN6" s="49" t="str">
+      <c r="AN6" s="55" t="str">
         <f>_xlfn.XLOOKUP(AO5,mat!$A:$A, mat!$B:$B,"") &amp; ""</f>
         <v/>
       </c>
-      <c r="AO6" s="50"/>
+      <c r="AO6" s="56"/>
       <c r="AP6" s="1"/>
-      <c r="AQ6" s="49" t="str">
+      <c r="AQ6" s="55" t="str">
         <f>_xlfn.XLOOKUP(AR5,mat!$A:$A, mat!$B:$B,"") &amp; ""</f>
         <v/>
       </c>
-      <c r="AR6" s="50"/>
+      <c r="AR6" s="56"/>
     </row>
     <row r="7" spans="1:44" x14ac:dyDescent="0.2">
       <c r="A7" s="2" t="s">
@@ -17272,12 +17379,14 @@
     </row>
   </sheetData>
   <mergeCells count="30">
-    <mergeCell ref="P4:Q4"/>
-    <mergeCell ref="A4:B4"/>
-    <mergeCell ref="D4:E4"/>
-    <mergeCell ref="G4:H4"/>
-    <mergeCell ref="J4:K4"/>
-    <mergeCell ref="M4:N4"/>
+    <mergeCell ref="AN6:AO6"/>
+    <mergeCell ref="AQ6:AR6"/>
+    <mergeCell ref="V6:W6"/>
+    <mergeCell ref="Y6:Z6"/>
+    <mergeCell ref="AB6:AC6"/>
+    <mergeCell ref="AE6:AF6"/>
+    <mergeCell ref="AH6:AI6"/>
+    <mergeCell ref="AK6:AL6"/>
     <mergeCell ref="AK4:AL4"/>
     <mergeCell ref="AN4:AO4"/>
     <mergeCell ref="AQ4:AR4"/>
@@ -17294,14 +17403,12 @@
     <mergeCell ref="AB4:AC4"/>
     <mergeCell ref="AE4:AF4"/>
     <mergeCell ref="AH4:AI4"/>
-    <mergeCell ref="AN6:AO6"/>
-    <mergeCell ref="AQ6:AR6"/>
-    <mergeCell ref="V6:W6"/>
-    <mergeCell ref="Y6:Z6"/>
-    <mergeCell ref="AB6:AC6"/>
-    <mergeCell ref="AE6:AF6"/>
-    <mergeCell ref="AH6:AI6"/>
-    <mergeCell ref="AK6:AL6"/>
+    <mergeCell ref="P4:Q4"/>
+    <mergeCell ref="A4:B4"/>
+    <mergeCell ref="D4:E4"/>
+    <mergeCell ref="G4:H4"/>
+    <mergeCell ref="J4:K4"/>
+    <mergeCell ref="M4:N4"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
@@ -17317,14 +17424,14 @@
   </cols>
   <sheetData>
     <row r="2" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A2" s="51" t="s">
+      <c r="A2" s="57" t="s">
         <v>83</v>
       </c>
-      <c r="B2" s="51"/>
-      <c r="D2" s="52" t="s">
+      <c r="B2" s="57"/>
+      <c r="D2" s="58" t="s">
         <v>81</v>
       </c>
-      <c r="E2" s="52"/>
+      <c r="E2" s="58"/>
       <c r="G2" s="22" t="s">
         <v>82</v>
       </c>
@@ -17895,36 +18002,36 @@
   </cols>
   <sheetData>
     <row r="2" spans="2:24" x14ac:dyDescent="0.2">
-      <c r="B2" s="53" t="s">
+      <c r="B2" s="59" t="s">
         <v>121</v>
       </c>
-      <c r="C2" s="53"/>
-      <c r="D2" s="53"/>
-      <c r="F2" s="53" t="s">
+      <c r="C2" s="59"/>
+      <c r="D2" s="59"/>
+      <c r="F2" s="59" t="s">
         <v>122</v>
       </c>
-      <c r="G2" s="53"/>
-      <c r="H2" s="53"/>
-      <c r="J2" s="53" t="s">
+      <c r="G2" s="59"/>
+      <c r="H2" s="59"/>
+      <c r="J2" s="59" t="s">
         <v>123</v>
       </c>
-      <c r="K2" s="53"/>
-      <c r="L2" s="53"/>
-      <c r="N2" s="53" t="s">
+      <c r="K2" s="59"/>
+      <c r="L2" s="59"/>
+      <c r="N2" s="59" t="s">
         <v>124</v>
       </c>
-      <c r="O2" s="53"/>
-      <c r="P2" s="53"/>
-      <c r="R2" s="53" t="s">
+      <c r="O2" s="59"/>
+      <c r="P2" s="59"/>
+      <c r="R2" s="59" t="s">
         <v>125</v>
       </c>
-      <c r="S2" s="53"/>
-      <c r="T2" s="53"/>
-      <c r="V2" s="53" t="s">
+      <c r="S2" s="59"/>
+      <c r="T2" s="59"/>
+      <c r="V2" s="59" t="s">
         <v>126</v>
       </c>
-      <c r="W2" s="53"/>
-      <c r="X2" s="53"/>
+      <c r="W2" s="59"/>
+      <c r="X2" s="59"/>
     </row>
     <row r="3" spans="2:24" x14ac:dyDescent="0.2">
       <c r="B3" s="2" t="s">

</xml_diff>

<commit_message>
new version 18 template
</commit_message>
<xml_diff>
--- a/docs/inputs/input_template.xlsx
+++ b/docs/inputs/input_template.xlsx
@@ -1,40 +1,42 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10713"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10719"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/njones/python_projects/xslope/docs/inputs/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/Jones/python_projects/xslope/docs/inputs/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{920EFD39-E0D9-5841-8A8C-9199354BBCB5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{69AB93CB-4984-D04D-83D8-31B63690B3CE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="600" windowWidth="35040" windowHeight="19900" xr2:uid="{BA54C293-CE08-6E4C-9212-B3317DAA148E}"/>
+    <workbookView xWindow="0" yWindow="680" windowWidth="34200" windowHeight="19900" activeTab="16" xr2:uid="{BA54C293-CE08-6E4C-9212-B3317DAA148E}"/>
   </bookViews>
   <sheets>
     <sheet name="main" sheetId="1" r:id="rId1"/>
-    <sheet name="plot" sheetId="9" r:id="rId2"/>
-    <sheet name="mat" sheetId="3" r:id="rId3"/>
-    <sheet name="profile" sheetId="2" r:id="rId4"/>
-    <sheet name="polygon" sheetId="15" r:id="rId5"/>
-    <sheet name="piezo" sheetId="4" r:id="rId6"/>
-    <sheet name="circles" sheetId="5" r:id="rId7"/>
-    <sheet name="non-circ" sheetId="7" r:id="rId8"/>
-    <sheet name="dloads" sheetId="8" r:id="rId9"/>
-    <sheet name="dloads (2)" sheetId="13" r:id="rId10"/>
-    <sheet name="reinforce" sheetId="12" r:id="rId11"/>
-    <sheet name="piles" sheetId="16" r:id="rId12"/>
-    <sheet name="lloads" sheetId="17" r:id="rId13"/>
-    <sheet name="seep bc" sheetId="11" r:id="rId14"/>
-    <sheet name="seep bc (2)" sheetId="14" r:id="rId15"/>
+    <sheet name="Sheet1" sheetId="18" r:id="rId2"/>
+    <sheet name="plot" sheetId="9" r:id="rId3"/>
+    <sheet name="mat" sheetId="3" r:id="rId4"/>
+    <sheet name="profile" sheetId="2" r:id="rId5"/>
+    <sheet name="polygon" sheetId="15" r:id="rId6"/>
+    <sheet name="piezo" sheetId="4" r:id="rId7"/>
+    <sheet name="circles" sheetId="5" r:id="rId8"/>
+    <sheet name="non-circ" sheetId="7" r:id="rId9"/>
+    <sheet name="dloads" sheetId="8" r:id="rId10"/>
+    <sheet name="dloads (2)" sheetId="13" r:id="rId11"/>
+    <sheet name="reinforce" sheetId="12" r:id="rId12"/>
+    <sheet name="piles" sheetId="16" r:id="rId13"/>
+    <sheet name="lloads" sheetId="17" r:id="rId14"/>
+    <sheet name="seep bc" sheetId="11" r:id="rId15"/>
+    <sheet name="seep bc (2)" sheetId="14" r:id="rId16"/>
+    <sheet name="tseep" sheetId="19" r:id="rId17"/>
   </sheets>
   <definedNames>
-    <definedName name="crack_depth">main!$D$9</definedName>
-    <definedName name="crack_depth_water">main!$D$10</definedName>
-    <definedName name="gamma_w">main!$D$8</definedName>
-    <definedName name="k">main!$D$11</definedName>
-    <definedName name="max_depth" localSheetId="4">polygon!#REF!</definedName>
+    <definedName name="crack_depth">main!$D$11</definedName>
+    <definedName name="crack_depth_water">main!$D$12</definedName>
+    <definedName name="gamma_w">main!$D$10</definedName>
+    <definedName name="k">main!$D$13</definedName>
+    <definedName name="max_depth" localSheetId="5">polygon!#REF!</definedName>
     <definedName name="max_depth">profile!$B$2</definedName>
     <definedName name="mesh">mat!#REF!</definedName>
     <definedName name="solution1">mat!#REF!</definedName>
@@ -62,7 +64,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="451" uniqueCount="240">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="475" uniqueCount="262">
   <si>
     <t>X</t>
   </si>
@@ -947,6 +949,72 @@
   </si>
   <si>
     <t>s_cap</t>
+  </si>
+  <si>
+    <t>Unit Options:</t>
+  </si>
+  <si>
+    <t>SI</t>
+  </si>
+  <si>
+    <t>Imperial</t>
+  </si>
+  <si>
+    <t>Units:</t>
+  </si>
+  <si>
+    <t>Time Units:</t>
+  </si>
+  <si>
+    <t>sec</t>
+  </si>
+  <si>
+    <t>min</t>
+  </si>
+  <si>
+    <t>hr</t>
+  </si>
+  <si>
+    <t>day</t>
+  </si>
+  <si>
+    <t>Time:</t>
+  </si>
+  <si>
+    <t>t1</t>
+  </si>
+  <si>
+    <t>t2</t>
+  </si>
+  <si>
+    <t>t3</t>
+  </si>
+  <si>
+    <t>t4</t>
+  </si>
+  <si>
+    <t>t5</t>
+  </si>
+  <si>
+    <t>time</t>
+  </si>
+  <si>
+    <t>save_interval:</t>
+  </si>
+  <si>
+    <t>duration:</t>
+  </si>
+  <si>
+    <t>stage_1:</t>
+  </si>
+  <si>
+    <t>stage_2:</t>
+  </si>
+  <si>
+    <t>tseep</t>
+  </si>
+  <si>
+    <t>Transient seepage boundary conditions and run options</t>
   </si>
 </sst>
 </file>
@@ -1096,7 +1164,7 @@
       <name val="Aptos Narrow"/>
     </font>
   </fonts>
-  <fills count="17">
+  <fills count="18">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -1193,6 +1261,12 @@
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="3" tint="9.9978637043366805E-2"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
   </fills>
   <borders count="7">
     <border>
@@ -1280,7 +1354,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="63">
+  <cellXfs count="65">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -1454,11 +1528,17 @@
     <xf numFmtId="0" fontId="1" fillId="13" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="17" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="22">
+  <dxfs count="21">
     <dxf>
       <fill>
         <patternFill>
@@ -1477,13 +1557,6 @@
       <fill>
         <patternFill>
           <bgColor theme="1" tint="0.499984740745262"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor theme="0" tint="-0.499984740745262"/>
         </patternFill>
       </fill>
     </dxf>
@@ -10442,7 +10515,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{71FAED0A-C8CC-8343-BA2E-B8E4255891E7}">
-  <dimension ref="A1:G24"/>
+  <dimension ref="A1:G57"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="5.6640625" customWidth="1"/>
@@ -10467,7 +10540,7 @@
         <v>78</v>
       </c>
       <c r="D5" s="30">
-        <v>17</v>
+        <v>18</v>
       </c>
     </row>
     <row r="7" spans="1:7" x14ac:dyDescent="0.2">
@@ -10485,10 +10558,10 @@
     </row>
     <row r="8" spans="1:7" x14ac:dyDescent="0.2">
       <c r="C8" s="14" t="s">
-        <v>50</v>
-      </c>
-      <c r="D8" s="1">
-        <v>62.4</v>
+        <v>243</v>
+      </c>
+      <c r="D8" s="1" t="s">
+        <v>242</v>
       </c>
       <c r="F8" s="1" t="s">
         <v>113</v>
@@ -10499,10 +10572,10 @@
     </row>
     <row r="9" spans="1:7" x14ac:dyDescent="0.2">
       <c r="C9" s="14" t="s">
-        <v>49</v>
-      </c>
-      <c r="D9" s="1">
-        <v>0</v>
+        <v>249</v>
+      </c>
+      <c r="D9" s="1" t="s">
+        <v>248</v>
       </c>
       <c r="F9" s="1" t="s">
         <v>19</v>
@@ -10513,10 +10586,10 @@
     </row>
     <row r="10" spans="1:7" x14ac:dyDescent="0.2">
       <c r="C10" s="14" t="s">
-        <v>48</v>
+        <v>50</v>
       </c>
       <c r="D10" s="1">
-        <v>0</v>
+        <v>62.4</v>
       </c>
       <c r="F10" s="1" t="s">
         <v>17</v>
@@ -10528,7 +10601,7 @@
     <row r="11" spans="1:7" x14ac:dyDescent="0.2">
       <c r="B11" s="1"/>
       <c r="C11" s="14" t="s">
-        <v>74</v>
+        <v>49</v>
       </c>
       <c r="D11" s="1">
         <v>0</v>
@@ -10541,6 +10614,12 @@
       </c>
     </row>
     <row r="12" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="C12" s="14" t="s">
+        <v>48</v>
+      </c>
+      <c r="D12" s="1">
+        <v>0</v>
+      </c>
       <c r="F12" s="1" t="s">
         <v>21</v>
       </c>
@@ -10549,6 +10628,12 @@
       </c>
     </row>
     <row r="13" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="C13" s="14" t="s">
+        <v>74</v>
+      </c>
+      <c r="D13" s="1">
+        <v>0</v>
+      </c>
       <c r="F13" s="1" t="s">
         <v>23</v>
       </c>
@@ -10621,21 +10706,577 @@
         <v>118</v>
       </c>
     </row>
+    <row r="22" spans="2:7" x14ac:dyDescent="0.2">
+      <c r="F22" s="1" t="s">
+        <v>260</v>
+      </c>
+      <c r="G22" t="s">
+        <v>261</v>
+      </c>
+    </row>
     <row r="23" spans="2:7" x14ac:dyDescent="0.2">
       <c r="B23" s="1"/>
     </row>
     <row r="24" spans="2:7" x14ac:dyDescent="0.2">
       <c r="B24" s="1"/>
+    </row>
+    <row r="49" spans="4:4" x14ac:dyDescent="0.2">
+      <c r="D49" s="1" t="s">
+        <v>240</v>
+      </c>
+    </row>
+    <row r="50" spans="4:4" x14ac:dyDescent="0.2">
+      <c r="D50" s="1" t="s">
+        <v>241</v>
+      </c>
+    </row>
+    <row r="51" spans="4:4" x14ac:dyDescent="0.2">
+      <c r="D51" s="1" t="s">
+        <v>242</v>
+      </c>
+    </row>
+    <row r="53" spans="4:4" x14ac:dyDescent="0.2">
+      <c r="D53" s="1" t="s">
+        <v>244</v>
+      </c>
+    </row>
+    <row r="54" spans="4:4" x14ac:dyDescent="0.2">
+      <c r="D54" s="1" t="s">
+        <v>245</v>
+      </c>
+    </row>
+    <row r="55" spans="4:4" x14ac:dyDescent="0.2">
+      <c r="D55" s="1" t="s">
+        <v>246</v>
+      </c>
+    </row>
+    <row r="56" spans="4:4" x14ac:dyDescent="0.2">
+      <c r="D56" s="1" t="s">
+        <v>247</v>
+      </c>
+    </row>
+    <row r="57" spans="4:4" x14ac:dyDescent="0.2">
+      <c r="D57" s="1" t="s">
+        <v>248</v>
+      </c>
     </row>
   </sheetData>
   <mergeCells count="1">
     <mergeCell ref="B7:D7"/>
+  </mergeCells>
+  <dataValidations count="2">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="D8" xr:uid="{BAE3FC11-E776-8E44-B1AE-D9B052583E4F}">
+      <formula1>$D$50:$D$51</formula1>
+    </dataValidation>
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="D9" xr:uid="{73E87265-AF9F-0944-800E-CFF30E3B4CA4}">
+      <formula1>$D$54:$D$57</formula1>
+    </dataValidation>
+  </dataValidations>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{8D19B78E-FBCC-4E41-BB37-C8D0D27B23E8}">
+  <dimension ref="B2:X22"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
+  <cols>
+    <col min="1" max="1" width="3" customWidth="1"/>
+    <col min="2" max="4" width="7.6640625" customWidth="1"/>
+    <col min="5" max="5" width="3" customWidth="1"/>
+    <col min="6" max="8" width="7.6640625" customWidth="1"/>
+    <col min="9" max="9" width="3" customWidth="1"/>
+    <col min="10" max="12" width="7.6640625" customWidth="1"/>
+    <col min="13" max="13" width="3" customWidth="1"/>
+    <col min="14" max="16" width="7.6640625" customWidth="1"/>
+    <col min="17" max="17" width="3" customWidth="1"/>
+    <col min="18" max="20" width="7.6640625" customWidth="1"/>
+    <col min="21" max="21" width="3" customWidth="1"/>
+    <col min="22" max="24" width="7.6640625" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="2" spans="2:24" x14ac:dyDescent="0.2">
+      <c r="B2" s="59" t="s">
+        <v>121</v>
+      </c>
+      <c r="C2" s="59"/>
+      <c r="D2" s="59"/>
+      <c r="F2" s="59" t="s">
+        <v>122</v>
+      </c>
+      <c r="G2" s="59"/>
+      <c r="H2" s="59"/>
+      <c r="J2" s="59" t="s">
+        <v>123</v>
+      </c>
+      <c r="K2" s="59"/>
+      <c r="L2" s="59"/>
+      <c r="N2" s="59" t="s">
+        <v>124</v>
+      </c>
+      <c r="O2" s="59"/>
+      <c r="P2" s="59"/>
+      <c r="R2" s="59" t="s">
+        <v>125</v>
+      </c>
+      <c r="S2" s="59"/>
+      <c r="T2" s="59"/>
+      <c r="V2" s="59" t="s">
+        <v>126</v>
+      </c>
+      <c r="W2" s="59"/>
+      <c r="X2" s="59"/>
+    </row>
+    <row r="3" spans="2:24" x14ac:dyDescent="0.2">
+      <c r="B3" s="2" t="s">
+        <v>0</v>
+      </c>
+      <c r="C3" s="2" t="s">
+        <v>1</v>
+      </c>
+      <c r="D3" s="2" t="s">
+        <v>45</v>
+      </c>
+      <c r="F3" s="2" t="s">
+        <v>0</v>
+      </c>
+      <c r="G3" s="2" t="s">
+        <v>1</v>
+      </c>
+      <c r="H3" s="2" t="s">
+        <v>45</v>
+      </c>
+      <c r="J3" s="2" t="s">
+        <v>0</v>
+      </c>
+      <c r="K3" s="2" t="s">
+        <v>1</v>
+      </c>
+      <c r="L3" s="2" t="s">
+        <v>45</v>
+      </c>
+      <c r="N3" s="2" t="s">
+        <v>0</v>
+      </c>
+      <c r="O3" s="2" t="s">
+        <v>1</v>
+      </c>
+      <c r="P3" s="2" t="s">
+        <v>45</v>
+      </c>
+      <c r="R3" s="2" t="s">
+        <v>0</v>
+      </c>
+      <c r="S3" s="2" t="s">
+        <v>1</v>
+      </c>
+      <c r="T3" s="2" t="s">
+        <v>45</v>
+      </c>
+      <c r="V3" s="2" t="s">
+        <v>0</v>
+      </c>
+      <c r="W3" s="2" t="s">
+        <v>1</v>
+      </c>
+      <c r="X3" s="2" t="s">
+        <v>45</v>
+      </c>
+    </row>
+    <row r="4" spans="2:24" x14ac:dyDescent="0.2">
+      <c r="B4" s="3"/>
+      <c r="C4" s="3"/>
+      <c r="D4" s="3"/>
+      <c r="F4" s="3"/>
+      <c r="G4" s="3"/>
+      <c r="H4" s="3"/>
+      <c r="J4" s="3"/>
+      <c r="K4" s="3"/>
+      <c r="L4" s="3"/>
+      <c r="N4" s="3"/>
+      <c r="O4" s="3"/>
+      <c r="P4" s="3"/>
+      <c r="R4" s="3"/>
+      <c r="S4" s="3"/>
+      <c r="T4" s="3"/>
+      <c r="V4" s="3"/>
+      <c r="W4" s="3"/>
+      <c r="X4" s="3"/>
+    </row>
+    <row r="5" spans="2:24" x14ac:dyDescent="0.2">
+      <c r="B5" s="3"/>
+      <c r="C5" s="3"/>
+      <c r="D5" s="3"/>
+      <c r="F5" s="3"/>
+      <c r="G5" s="3"/>
+      <c r="H5" s="3"/>
+      <c r="J5" s="3"/>
+      <c r="K5" s="3"/>
+      <c r="L5" s="3"/>
+      <c r="N5" s="3"/>
+      <c r="O5" s="3"/>
+      <c r="P5" s="3"/>
+      <c r="R5" s="3"/>
+      <c r="S5" s="3"/>
+      <c r="T5" s="3"/>
+      <c r="V5" s="3"/>
+      <c r="W5" s="3"/>
+      <c r="X5" s="3"/>
+    </row>
+    <row r="6" spans="2:24" x14ac:dyDescent="0.2">
+      <c r="B6" s="3"/>
+      <c r="C6" s="3"/>
+      <c r="D6" s="3"/>
+      <c r="F6" s="3"/>
+      <c r="G6" s="3"/>
+      <c r="H6" s="3"/>
+      <c r="J6" s="3"/>
+      <c r="K6" s="3"/>
+      <c r="L6" s="3"/>
+      <c r="N6" s="3"/>
+      <c r="O6" s="3"/>
+      <c r="P6" s="3"/>
+      <c r="R6" s="3"/>
+      <c r="S6" s="3"/>
+      <c r="T6" s="3"/>
+      <c r="V6" s="3"/>
+      <c r="W6" s="3"/>
+      <c r="X6" s="3"/>
+    </row>
+    <row r="7" spans="2:24" x14ac:dyDescent="0.2">
+      <c r="B7" s="3"/>
+      <c r="C7" s="3"/>
+      <c r="D7" s="3"/>
+      <c r="F7" s="3"/>
+      <c r="G7" s="3"/>
+      <c r="H7" s="3"/>
+      <c r="J7" s="3"/>
+      <c r="K7" s="3"/>
+      <c r="L7" s="3"/>
+      <c r="N7" s="3"/>
+      <c r="O7" s="3"/>
+      <c r="P7" s="3"/>
+      <c r="R7" s="3"/>
+      <c r="S7" s="3"/>
+      <c r="T7" s="3"/>
+      <c r="V7" s="3"/>
+      <c r="W7" s="3"/>
+      <c r="X7" s="3"/>
+    </row>
+    <row r="8" spans="2:24" x14ac:dyDescent="0.2">
+      <c r="B8" s="3"/>
+      <c r="C8" s="3"/>
+      <c r="D8" s="3"/>
+      <c r="F8" s="3"/>
+      <c r="G8" s="3"/>
+      <c r="H8" s="3"/>
+      <c r="J8" s="3"/>
+      <c r="K8" s="3"/>
+      <c r="L8" s="3"/>
+      <c r="N8" s="3"/>
+      <c r="O8" s="3"/>
+      <c r="P8" s="3"/>
+      <c r="R8" s="3"/>
+      <c r="S8" s="3"/>
+      <c r="T8" s="3"/>
+      <c r="V8" s="3"/>
+      <c r="W8" s="3"/>
+      <c r="X8" s="3"/>
+    </row>
+    <row r="9" spans="2:24" x14ac:dyDescent="0.2">
+      <c r="B9" s="3"/>
+      <c r="C9" s="3"/>
+      <c r="D9" s="3"/>
+      <c r="F9" s="3"/>
+      <c r="G9" s="3"/>
+      <c r="H9" s="3"/>
+      <c r="J9" s="3"/>
+      <c r="K9" s="3"/>
+      <c r="L9" s="3"/>
+      <c r="N9" s="3"/>
+      <c r="O9" s="3"/>
+      <c r="P9" s="3"/>
+      <c r="R9" s="3"/>
+      <c r="S9" s="3"/>
+      <c r="T9" s="3"/>
+      <c r="V9" s="3"/>
+      <c r="W9" s="3"/>
+      <c r="X9" s="3"/>
+    </row>
+    <row r="10" spans="2:24" x14ac:dyDescent="0.2">
+      <c r="B10" s="3"/>
+      <c r="C10" s="3"/>
+      <c r="D10" s="3"/>
+      <c r="F10" s="3"/>
+      <c r="G10" s="3"/>
+      <c r="H10" s="3"/>
+      <c r="J10" s="3"/>
+      <c r="K10" s="3"/>
+      <c r="L10" s="3"/>
+      <c r="N10" s="3"/>
+      <c r="O10" s="3"/>
+      <c r="P10" s="3"/>
+      <c r="R10" s="3"/>
+      <c r="S10" s="3"/>
+      <c r="T10" s="3"/>
+      <c r="V10" s="3"/>
+      <c r="W10" s="3"/>
+      <c r="X10" s="3"/>
+    </row>
+    <row r="11" spans="2:24" x14ac:dyDescent="0.2">
+      <c r="B11" s="3"/>
+      <c r="C11" s="3"/>
+      <c r="D11" s="3"/>
+      <c r="F11" s="3"/>
+      <c r="G11" s="3"/>
+      <c r="H11" s="3"/>
+      <c r="J11" s="3"/>
+      <c r="K11" s="3"/>
+      <c r="L11" s="3"/>
+      <c r="N11" s="3"/>
+      <c r="O11" s="3"/>
+      <c r="P11" s="3"/>
+      <c r="R11" s="3"/>
+      <c r="S11" s="3"/>
+      <c r="T11" s="3"/>
+      <c r="V11" s="3"/>
+      <c r="W11" s="3"/>
+      <c r="X11" s="3"/>
+    </row>
+    <row r="12" spans="2:24" x14ac:dyDescent="0.2">
+      <c r="B12" s="3"/>
+      <c r="C12" s="3"/>
+      <c r="D12" s="3"/>
+      <c r="F12" s="3"/>
+      <c r="G12" s="3"/>
+      <c r="H12" s="3"/>
+      <c r="J12" s="3"/>
+      <c r="K12" s="3"/>
+      <c r="L12" s="3"/>
+      <c r="N12" s="3"/>
+      <c r="O12" s="3"/>
+      <c r="P12" s="3"/>
+      <c r="R12" s="3"/>
+      <c r="S12" s="3"/>
+      <c r="T12" s="3"/>
+      <c r="V12" s="3"/>
+      <c r="W12" s="3"/>
+      <c r="X12" s="3"/>
+    </row>
+    <row r="13" spans="2:24" x14ac:dyDescent="0.2">
+      <c r="B13" s="3"/>
+      <c r="C13" s="3"/>
+      <c r="D13" s="3"/>
+      <c r="F13" s="3"/>
+      <c r="G13" s="3"/>
+      <c r="H13" s="3"/>
+      <c r="J13" s="3"/>
+      <c r="K13" s="3"/>
+      <c r="L13" s="3"/>
+      <c r="N13" s="3"/>
+      <c r="O13" s="3"/>
+      <c r="P13" s="3"/>
+      <c r="R13" s="3"/>
+      <c r="S13" s="3"/>
+      <c r="T13" s="3"/>
+      <c r="V13" s="3"/>
+      <c r="W13" s="3"/>
+      <c r="X13" s="3"/>
+    </row>
+    <row r="14" spans="2:24" x14ac:dyDescent="0.2">
+      <c r="B14" s="3"/>
+      <c r="C14" s="3"/>
+      <c r="D14" s="3"/>
+      <c r="F14" s="3"/>
+      <c r="G14" s="3"/>
+      <c r="H14" s="3"/>
+      <c r="J14" s="3"/>
+      <c r="K14" s="3"/>
+      <c r="L14" s="3"/>
+      <c r="N14" s="3"/>
+      <c r="O14" s="3"/>
+      <c r="P14" s="3"/>
+      <c r="R14" s="3"/>
+      <c r="S14" s="3"/>
+      <c r="T14" s="3"/>
+      <c r="V14" s="3"/>
+      <c r="W14" s="3"/>
+      <c r="X14" s="3"/>
+    </row>
+    <row r="15" spans="2:24" x14ac:dyDescent="0.2">
+      <c r="B15" s="3"/>
+      <c r="C15" s="3"/>
+      <c r="D15" s="3"/>
+      <c r="F15" s="3"/>
+      <c r="G15" s="3"/>
+      <c r="H15" s="3"/>
+      <c r="J15" s="3"/>
+      <c r="K15" s="3"/>
+      <c r="L15" s="3"/>
+      <c r="N15" s="3"/>
+      <c r="O15" s="3"/>
+      <c r="P15" s="3"/>
+      <c r="R15" s="3"/>
+      <c r="S15" s="3"/>
+      <c r="T15" s="3"/>
+      <c r="V15" s="3"/>
+      <c r="W15" s="3"/>
+      <c r="X15" s="3"/>
+    </row>
+    <row r="16" spans="2:24" x14ac:dyDescent="0.2">
+      <c r="B16" s="3"/>
+      <c r="C16" s="3"/>
+      <c r="D16" s="3"/>
+      <c r="F16" s="3"/>
+      <c r="G16" s="3"/>
+      <c r="H16" s="3"/>
+      <c r="J16" s="3"/>
+      <c r="K16" s="3"/>
+      <c r="L16" s="3"/>
+      <c r="N16" s="3"/>
+      <c r="O16" s="3"/>
+      <c r="P16" s="3"/>
+      <c r="R16" s="3"/>
+      <c r="S16" s="3"/>
+      <c r="T16" s="3"/>
+      <c r="V16" s="3"/>
+      <c r="W16" s="3"/>
+      <c r="X16" s="3"/>
+    </row>
+    <row r="17" spans="2:24" x14ac:dyDescent="0.2">
+      <c r="B17" s="3"/>
+      <c r="C17" s="3"/>
+      <c r="D17" s="3"/>
+      <c r="F17" s="3"/>
+      <c r="G17" s="3"/>
+      <c r="H17" s="3"/>
+      <c r="J17" s="3"/>
+      <c r="K17" s="3"/>
+      <c r="L17" s="3"/>
+      <c r="N17" s="3"/>
+      <c r="O17" s="3"/>
+      <c r="P17" s="3"/>
+      <c r="R17" s="3"/>
+      <c r="S17" s="3"/>
+      <c r="T17" s="3"/>
+      <c r="V17" s="3"/>
+      <c r="W17" s="3"/>
+      <c r="X17" s="3"/>
+    </row>
+    <row r="18" spans="2:24" x14ac:dyDescent="0.2">
+      <c r="B18" s="3"/>
+      <c r="C18" s="3"/>
+      <c r="D18" s="3"/>
+      <c r="F18" s="3"/>
+      <c r="G18" s="3"/>
+      <c r="H18" s="3"/>
+      <c r="J18" s="3"/>
+      <c r="K18" s="3"/>
+      <c r="L18" s="3"/>
+      <c r="N18" s="3"/>
+      <c r="O18" s="3"/>
+      <c r="P18" s="3"/>
+      <c r="R18" s="3"/>
+      <c r="S18" s="3"/>
+      <c r="T18" s="3"/>
+      <c r="V18" s="3"/>
+      <c r="W18" s="3"/>
+      <c r="X18" s="3"/>
+    </row>
+    <row r="19" spans="2:24" x14ac:dyDescent="0.2">
+      <c r="B19" s="3"/>
+      <c r="C19" s="3"/>
+      <c r="D19" s="3"/>
+      <c r="F19" s="3"/>
+      <c r="G19" s="3"/>
+      <c r="H19" s="3"/>
+      <c r="J19" s="3"/>
+      <c r="K19" s="3"/>
+      <c r="L19" s="3"/>
+      <c r="N19" s="3"/>
+      <c r="O19" s="3"/>
+      <c r="P19" s="3"/>
+      <c r="R19" s="3"/>
+      <c r="S19" s="3"/>
+      <c r="T19" s="3"/>
+      <c r="V19" s="3"/>
+      <c r="W19" s="3"/>
+      <c r="X19" s="3"/>
+    </row>
+    <row r="20" spans="2:24" x14ac:dyDescent="0.2">
+      <c r="B20" s="3"/>
+      <c r="C20" s="3"/>
+      <c r="D20" s="3"/>
+      <c r="F20" s="3"/>
+      <c r="G20" s="3"/>
+      <c r="H20" s="3"/>
+      <c r="J20" s="3"/>
+      <c r="K20" s="3"/>
+      <c r="L20" s="3"/>
+      <c r="N20" s="3"/>
+      <c r="O20" s="3"/>
+      <c r="P20" s="3"/>
+      <c r="R20" s="3"/>
+      <c r="S20" s="3"/>
+      <c r="T20" s="3"/>
+      <c r="V20" s="3"/>
+      <c r="W20" s="3"/>
+      <c r="X20" s="3"/>
+    </row>
+    <row r="21" spans="2:24" x14ac:dyDescent="0.2">
+      <c r="B21" s="3"/>
+      <c r="C21" s="3"/>
+      <c r="D21" s="3"/>
+      <c r="F21" s="3"/>
+      <c r="G21" s="3"/>
+      <c r="H21" s="3"/>
+      <c r="J21" s="3"/>
+      <c r="K21" s="3"/>
+      <c r="L21" s="3"/>
+      <c r="N21" s="3"/>
+      <c r="O21" s="3"/>
+      <c r="P21" s="3"/>
+      <c r="R21" s="3"/>
+      <c r="S21" s="3"/>
+      <c r="T21" s="3"/>
+      <c r="V21" s="3"/>
+      <c r="W21" s="3"/>
+      <c r="X21" s="3"/>
+    </row>
+    <row r="22" spans="2:24" x14ac:dyDescent="0.2">
+      <c r="B22" s="3"/>
+      <c r="C22" s="3"/>
+      <c r="D22" s="3"/>
+      <c r="F22" s="3"/>
+      <c r="G22" s="3"/>
+      <c r="H22" s="3"/>
+      <c r="J22" s="3"/>
+      <c r="K22" s="3"/>
+      <c r="L22" s="3"/>
+      <c r="N22" s="3"/>
+      <c r="O22" s="3"/>
+      <c r="P22" s="3"/>
+      <c r="R22" s="3"/>
+      <c r="S22" s="3"/>
+      <c r="T22" s="3"/>
+      <c r="V22" s="3"/>
+      <c r="W22" s="3"/>
+      <c r="X22" s="3"/>
+    </row>
+  </sheetData>
+  <mergeCells count="6">
+    <mergeCell ref="R2:T2"/>
+    <mergeCell ref="V2:X2"/>
+    <mergeCell ref="B2:D2"/>
+    <mergeCell ref="F2:H2"/>
+    <mergeCell ref="J2:L2"/>
+    <mergeCell ref="N2:P2"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{028A122E-8CB6-264D-BE4D-4184948E7CD8}">
   <dimension ref="B2:X22"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
@@ -11135,7 +11776,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C37CF166-6531-CC44-B460-D72E6A0F66E6}">
   <dimension ref="A2:AB25"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
@@ -11863,7 +12504,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet13.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F3B6221D-E989-B546-ACAF-CEB4607C51A1}">
   <dimension ref="A2:AA18"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
@@ -12191,7 +12832,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet13.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet14.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{1FA07123-52EA-314A-81EF-989A42CB4DFE}">
   <dimension ref="A2:F22"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
@@ -12426,7 +13067,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet14.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet15.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{8D036245-91C1-5842-93DD-735018175DE8}">
   <dimension ref="B2:U24"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
@@ -12842,7 +13483,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet15.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet16.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{E4C3C734-6227-7445-884D-1F1A5F3909C7}">
   <dimension ref="B2:U24"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
@@ -13256,7 +13897,295 @@
 </worksheet>
 </file>
 
+<file path=xl/worksheets/sheet17.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B20D353C-FC33-C347-9989-88B2E3FC7B94}">
+  <dimension ref="G2:O30"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
+  <cols>
+    <col min="6" max="6" width="3.5" customWidth="1"/>
+    <col min="7" max="12" width="10.83203125" style="1"/>
+    <col min="13" max="13" width="10" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="2" spans="7:15" x14ac:dyDescent="0.2">
+      <c r="G2" s="64" t="s">
+        <v>255</v>
+      </c>
+      <c r="H2" s="64" t="s">
+        <v>250</v>
+      </c>
+      <c r="I2" s="64" t="s">
+        <v>251</v>
+      </c>
+      <c r="J2" s="64" t="s">
+        <v>252</v>
+      </c>
+      <c r="K2" s="64" t="s">
+        <v>253</v>
+      </c>
+      <c r="L2" s="64" t="s">
+        <v>254</v>
+      </c>
+    </row>
+    <row r="3" spans="7:15" x14ac:dyDescent="0.2">
+      <c r="G3" s="3"/>
+      <c r="H3" s="3"/>
+      <c r="I3" s="3"/>
+      <c r="J3" s="3"/>
+      <c r="K3" s="3"/>
+      <c r="L3" s="3"/>
+      <c r="N3" s="14" t="s">
+        <v>257</v>
+      </c>
+      <c r="O3" s="63"/>
+    </row>
+    <row r="4" spans="7:15" x14ac:dyDescent="0.2">
+      <c r="G4" s="3"/>
+      <c r="H4" s="3"/>
+      <c r="I4" s="3"/>
+      <c r="J4" s="3"/>
+      <c r="K4" s="3"/>
+      <c r="L4" s="3"/>
+      <c r="N4" s="14"/>
+      <c r="O4" s="63"/>
+    </row>
+    <row r="5" spans="7:15" x14ac:dyDescent="0.2">
+      <c r="G5" s="3"/>
+      <c r="H5" s="3"/>
+      <c r="I5" s="3"/>
+      <c r="J5" s="3"/>
+      <c r="K5" s="3"/>
+      <c r="L5" s="3"/>
+      <c r="N5" s="14" t="s">
+        <v>256</v>
+      </c>
+      <c r="O5" s="63"/>
+    </row>
+    <row r="6" spans="7:15" x14ac:dyDescent="0.2">
+      <c r="G6" s="3"/>
+      <c r="H6" s="3"/>
+      <c r="I6" s="3"/>
+      <c r="J6" s="3"/>
+      <c r="K6" s="3"/>
+      <c r="L6" s="3"/>
+      <c r="N6" s="14"/>
+      <c r="O6" s="63"/>
+    </row>
+    <row r="7" spans="7:15" x14ac:dyDescent="0.2">
+      <c r="G7" s="3"/>
+      <c r="H7" s="3"/>
+      <c r="I7" s="3"/>
+      <c r="J7" s="3"/>
+      <c r="K7" s="3"/>
+      <c r="L7" s="3"/>
+      <c r="N7" s="14" t="s">
+        <v>258</v>
+      </c>
+      <c r="O7" s="63"/>
+    </row>
+    <row r="8" spans="7:15" x14ac:dyDescent="0.2">
+      <c r="G8" s="3"/>
+      <c r="H8" s="3"/>
+      <c r="I8" s="3"/>
+      <c r="J8" s="3"/>
+      <c r="K8" s="3"/>
+      <c r="L8" s="3"/>
+      <c r="N8" s="14" t="s">
+        <v>259</v>
+      </c>
+      <c r="O8" s="63"/>
+    </row>
+    <row r="9" spans="7:15" x14ac:dyDescent="0.2">
+      <c r="G9" s="3"/>
+      <c r="H9" s="3"/>
+      <c r="I9" s="3"/>
+      <c r="J9" s="3"/>
+      <c r="K9" s="3"/>
+      <c r="L9" s="3"/>
+    </row>
+    <row r="10" spans="7:15" x14ac:dyDescent="0.2">
+      <c r="G10" s="3"/>
+      <c r="H10" s="3"/>
+      <c r="I10" s="3"/>
+      <c r="J10" s="3"/>
+      <c r="K10" s="3"/>
+      <c r="L10" s="3"/>
+    </row>
+    <row r="11" spans="7:15" x14ac:dyDescent="0.2">
+      <c r="G11" s="3"/>
+      <c r="H11" s="3"/>
+      <c r="I11" s="3"/>
+      <c r="J11" s="3"/>
+      <c r="K11" s="3"/>
+      <c r="L11" s="3"/>
+    </row>
+    <row r="12" spans="7:15" x14ac:dyDescent="0.2">
+      <c r="G12" s="3"/>
+      <c r="H12" s="3"/>
+      <c r="I12" s="3"/>
+      <c r="J12" s="3"/>
+      <c r="K12" s="3"/>
+      <c r="L12" s="3"/>
+    </row>
+    <row r="13" spans="7:15" x14ac:dyDescent="0.2">
+      <c r="G13" s="3"/>
+      <c r="H13" s="3"/>
+      <c r="I13" s="3"/>
+      <c r="J13" s="3"/>
+      <c r="K13" s="3"/>
+      <c r="L13" s="3"/>
+    </row>
+    <row r="14" spans="7:15" x14ac:dyDescent="0.2">
+      <c r="G14" s="3"/>
+      <c r="H14" s="3"/>
+      <c r="I14" s="3"/>
+      <c r="J14" s="3"/>
+      <c r="K14" s="3"/>
+      <c r="L14" s="3"/>
+    </row>
+    <row r="15" spans="7:15" x14ac:dyDescent="0.2">
+      <c r="G15" s="3"/>
+      <c r="H15" s="3"/>
+      <c r="I15" s="3"/>
+      <c r="J15" s="3"/>
+      <c r="K15" s="3"/>
+      <c r="L15" s="3"/>
+    </row>
+    <row r="16" spans="7:15" x14ac:dyDescent="0.2">
+      <c r="G16" s="3"/>
+      <c r="H16" s="3"/>
+      <c r="I16" s="3"/>
+      <c r="J16" s="3"/>
+      <c r="K16" s="3"/>
+      <c r="L16" s="3"/>
+    </row>
+    <row r="17" spans="7:12" x14ac:dyDescent="0.2">
+      <c r="G17" s="3"/>
+      <c r="H17" s="3"/>
+      <c r="I17" s="3"/>
+      <c r="J17" s="3"/>
+      <c r="K17" s="3"/>
+      <c r="L17" s="3"/>
+    </row>
+    <row r="18" spans="7:12" x14ac:dyDescent="0.2">
+      <c r="G18" s="3"/>
+      <c r="H18" s="3"/>
+      <c r="I18" s="3"/>
+      <c r="J18" s="3"/>
+      <c r="K18" s="3"/>
+      <c r="L18" s="3"/>
+    </row>
+    <row r="19" spans="7:12" x14ac:dyDescent="0.2">
+      <c r="G19" s="3"/>
+      <c r="H19" s="3"/>
+      <c r="I19" s="3"/>
+      <c r="J19" s="3"/>
+      <c r="K19" s="3"/>
+      <c r="L19" s="3"/>
+    </row>
+    <row r="20" spans="7:12" x14ac:dyDescent="0.2">
+      <c r="G20" s="3"/>
+      <c r="H20" s="3"/>
+      <c r="I20" s="3"/>
+      <c r="J20" s="3"/>
+      <c r="K20" s="3"/>
+      <c r="L20" s="3"/>
+    </row>
+    <row r="21" spans="7:12" x14ac:dyDescent="0.2">
+      <c r="G21" s="3"/>
+      <c r="H21" s="3"/>
+      <c r="I21" s="3"/>
+      <c r="J21" s="3"/>
+      <c r="K21" s="3"/>
+      <c r="L21" s="3"/>
+    </row>
+    <row r="22" spans="7:12" x14ac:dyDescent="0.2">
+      <c r="G22" s="3"/>
+      <c r="H22" s="3"/>
+      <c r="I22" s="3"/>
+      <c r="J22" s="3"/>
+      <c r="K22" s="3"/>
+      <c r="L22" s="3"/>
+    </row>
+    <row r="23" spans="7:12" x14ac:dyDescent="0.2">
+      <c r="G23" s="3"/>
+      <c r="H23" s="3"/>
+      <c r="I23" s="3"/>
+      <c r="J23" s="3"/>
+      <c r="K23" s="3"/>
+      <c r="L23" s="3"/>
+    </row>
+    <row r="24" spans="7:12" x14ac:dyDescent="0.2">
+      <c r="G24" s="3"/>
+      <c r="H24" s="3"/>
+      <c r="I24" s="3"/>
+      <c r="J24" s="3"/>
+      <c r="K24" s="3"/>
+      <c r="L24" s="3"/>
+    </row>
+    <row r="25" spans="7:12" x14ac:dyDescent="0.2">
+      <c r="G25" s="3"/>
+      <c r="H25" s="3"/>
+      <c r="I25" s="3"/>
+      <c r="J25" s="3"/>
+      <c r="K25" s="3"/>
+      <c r="L25" s="3"/>
+    </row>
+    <row r="26" spans="7:12" x14ac:dyDescent="0.2">
+      <c r="G26" s="3"/>
+      <c r="H26" s="3"/>
+      <c r="I26" s="3"/>
+      <c r="J26" s="3"/>
+      <c r="K26" s="3"/>
+      <c r="L26" s="3"/>
+    </row>
+    <row r="27" spans="7:12" x14ac:dyDescent="0.2">
+      <c r="G27" s="3"/>
+      <c r="H27" s="3"/>
+      <c r="I27" s="3"/>
+      <c r="J27" s="3"/>
+      <c r="K27" s="3"/>
+      <c r="L27" s="3"/>
+    </row>
+    <row r="28" spans="7:12" x14ac:dyDescent="0.2">
+      <c r="G28" s="3"/>
+      <c r="H28" s="3"/>
+      <c r="I28" s="3"/>
+      <c r="J28" s="3"/>
+      <c r="K28" s="3"/>
+      <c r="L28" s="3"/>
+    </row>
+    <row r="29" spans="7:12" x14ac:dyDescent="0.2">
+      <c r="G29" s="3"/>
+      <c r="H29" s="3"/>
+      <c r="I29" s="3"/>
+      <c r="J29" s="3"/>
+      <c r="K29" s="3"/>
+      <c r="L29" s="3"/>
+    </row>
+    <row r="30" spans="7:12" x14ac:dyDescent="0.2">
+      <c r="G30" s="3"/>
+      <c r="H30" s="3"/>
+      <c r="I30" s="3"/>
+      <c r="J30" s="3"/>
+      <c r="K30" s="3"/>
+      <c r="L30" s="3"/>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F4216D5A-7B51-8B45-AAAC-BBE34074B3B1}">
+  <dimension ref="A1"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
+  <sheetData/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{FDB4949D-EAAF-AE4C-9BAF-D5BF753E34CD}">
   <dimension ref="A1"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
@@ -13266,7 +14195,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{60A900FC-A692-B445-95C9-59E70352B291}">
   <dimension ref="A2:AN52"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
@@ -14891,96 +15820,89 @@
     <mergeCell ref="C9:Z9"/>
   </mergeCells>
   <conditionalFormatting sqref="F11:K52 AB11:AF52">
-    <cfRule type="expression" dxfId="21" priority="4">
+    <cfRule type="expression" dxfId="20" priority="4">
       <formula>$E11="hb"</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="20" priority="5">
+    <cfRule type="expression" dxfId="19" priority="5">
       <formula>$E11="pow"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="F11:L52">
-    <cfRule type="expression" dxfId="19" priority="17">
+    <cfRule type="expression" dxfId="18" priority="17">
       <formula>$E11="elastic"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="G11:G52">
-    <cfRule type="expression" dxfId="18" priority="6">
+    <cfRule type="expression" dxfId="17" priority="6">
       <formula>$E11="cp"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="H11:I52">
-    <cfRule type="expression" dxfId="17" priority="7">
+    <cfRule type="expression" dxfId="16" priority="7">
       <formula>$E11="mc"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="J11:K52">
-    <cfRule type="expression" dxfId="16" priority="8">
+    <cfRule type="expression" dxfId="15" priority="8">
       <formula>$E11="cp"</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="O11:P52">
-    <cfRule type="expression" dxfId="15" priority="18">
+  <conditionalFormatting sqref="O11:R52">
+    <cfRule type="expression" dxfId="14" priority="2">
       <formula>$E11="elastic"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="P11:P52">
-    <cfRule type="expression" dxfId="14" priority="11">
+    <cfRule type="expression" dxfId="13" priority="11">
       <formula>AND($O11&lt;&gt;"",$O11&lt;&gt;"ru")</formula>
     </cfRule>
   </conditionalFormatting>
+  <conditionalFormatting sqref="Q11:R52">
+    <cfRule type="expression" dxfId="12" priority="1">
+      <formula>$E11="cp"</formula>
+    </cfRule>
+    <cfRule type="expression" dxfId="11" priority="3">
+      <formula>AND($O11&lt;&gt;"",$O11&lt;&gt;"piezo",$O11&lt;&gt;"seep")</formula>
+    </cfRule>
+  </conditionalFormatting>
   <conditionalFormatting sqref="S11:V52">
-    <cfRule type="expression" dxfId="13" priority="9">
+    <cfRule type="expression" dxfId="10" priority="9">
       <formula>AND($E11&lt;&gt;"",$E11&lt;&gt;"pow")</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="W11:Z52">
-    <cfRule type="expression" dxfId="12" priority="10">
+    <cfRule type="expression" dxfId="9" priority="10">
       <formula>AND($E11&lt;&gt;"",$E11&lt;&gt;"hb")</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="AB11:AF52">
-    <cfRule type="expression" dxfId="11" priority="19">
+    <cfRule type="expression" dxfId="8" priority="19">
       <formula>$E11="elastic"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="AC11:AC52">
-    <cfRule type="expression" dxfId="10" priority="12">
+    <cfRule type="expression" dxfId="7" priority="12">
       <formula>$E11="cp"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="AD11:AD52">
-    <cfRule type="expression" dxfId="9" priority="13">
+    <cfRule type="expression" dxfId="6" priority="13">
       <formula>$E11="mc"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="AE11:AF52">
-    <cfRule type="expression" dxfId="8" priority="14">
+    <cfRule type="expression" dxfId="5" priority="14">
       <formula>$E11="cp"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="AK11:AL52">
-    <cfRule type="expression" dxfId="7" priority="15">
+    <cfRule type="expression" dxfId="4" priority="15">
       <formula>OR($AJ11="vg",$AJ11="gard")</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="AM11:AN52">
-    <cfRule type="expression" dxfId="6" priority="16">
+    <cfRule type="expression" dxfId="3" priority="16">
       <formula>$AJ11="lf"</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="Q11:R52">
-    <cfRule type="expression" dxfId="5" priority="2">
-      <formula>$E11="elastic"</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="Q11:R52">
-    <cfRule type="expression" dxfId="4" priority="1">
-      <formula>$E11="cp"</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="Q11:R52">
-    <cfRule type="expression" dxfId="3" priority="3">
-      <formula>AND($O11&lt;&gt;"",$O11&lt;&gt;"piezo",$O11&lt;&gt;"seep")</formula>
     </cfRule>
   </conditionalFormatting>
   <dataValidations count="3">
@@ -14998,7 +15920,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{6D14E9FA-AFF6-A74D-8120-64FF6A371536}">
   <dimension ref="A2:AR27"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
@@ -16227,7 +17149,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{88992C43-9D03-6445-8931-028E950C2356}">
   <dimension ref="A2:AR27"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
@@ -17450,7 +18372,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A7E1F343-68A5-3340-AF23-43D8E7E1F914}">
   <dimension ref="A2:H24"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
@@ -17647,7 +18569,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{9E0556E9-786A-E84F-BF20-677A5EE9D63D}">
   <dimension ref="A2:N16"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
@@ -17858,7 +18780,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{6620242D-B699-0640-AD9C-590D8F82AC0F}">
   <dimension ref="A2:F23"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
@@ -18016,504 +18938,4 @@
   </dataValidations>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
-</file>
-
-<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{8D19B78E-FBCC-4E41-BB37-C8D0D27B23E8}">
-  <dimension ref="B2:X22"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
-  <cols>
-    <col min="1" max="1" width="3" customWidth="1"/>
-    <col min="2" max="4" width="7.6640625" customWidth="1"/>
-    <col min="5" max="5" width="3" customWidth="1"/>
-    <col min="6" max="8" width="7.6640625" customWidth="1"/>
-    <col min="9" max="9" width="3" customWidth="1"/>
-    <col min="10" max="12" width="7.6640625" customWidth="1"/>
-    <col min="13" max="13" width="3" customWidth="1"/>
-    <col min="14" max="16" width="7.6640625" customWidth="1"/>
-    <col min="17" max="17" width="3" customWidth="1"/>
-    <col min="18" max="20" width="7.6640625" customWidth="1"/>
-    <col min="21" max="21" width="3" customWidth="1"/>
-    <col min="22" max="24" width="7.6640625" customWidth="1"/>
-  </cols>
-  <sheetData>
-    <row r="2" spans="2:24" x14ac:dyDescent="0.2">
-      <c r="B2" s="59" t="s">
-        <v>121</v>
-      </c>
-      <c r="C2" s="59"/>
-      <c r="D2" s="59"/>
-      <c r="F2" s="59" t="s">
-        <v>122</v>
-      </c>
-      <c r="G2" s="59"/>
-      <c r="H2" s="59"/>
-      <c r="J2" s="59" t="s">
-        <v>123</v>
-      </c>
-      <c r="K2" s="59"/>
-      <c r="L2" s="59"/>
-      <c r="N2" s="59" t="s">
-        <v>124</v>
-      </c>
-      <c r="O2" s="59"/>
-      <c r="P2" s="59"/>
-      <c r="R2" s="59" t="s">
-        <v>125</v>
-      </c>
-      <c r="S2" s="59"/>
-      <c r="T2" s="59"/>
-      <c r="V2" s="59" t="s">
-        <v>126</v>
-      </c>
-      <c r="W2" s="59"/>
-      <c r="X2" s="59"/>
-    </row>
-    <row r="3" spans="2:24" x14ac:dyDescent="0.2">
-      <c r="B3" s="2" t="s">
-        <v>0</v>
-      </c>
-      <c r="C3" s="2" t="s">
-        <v>1</v>
-      </c>
-      <c r="D3" s="2" t="s">
-        <v>45</v>
-      </c>
-      <c r="F3" s="2" t="s">
-        <v>0</v>
-      </c>
-      <c r="G3" s="2" t="s">
-        <v>1</v>
-      </c>
-      <c r="H3" s="2" t="s">
-        <v>45</v>
-      </c>
-      <c r="J3" s="2" t="s">
-        <v>0</v>
-      </c>
-      <c r="K3" s="2" t="s">
-        <v>1</v>
-      </c>
-      <c r="L3" s="2" t="s">
-        <v>45</v>
-      </c>
-      <c r="N3" s="2" t="s">
-        <v>0</v>
-      </c>
-      <c r="O3" s="2" t="s">
-        <v>1</v>
-      </c>
-      <c r="P3" s="2" t="s">
-        <v>45</v>
-      </c>
-      <c r="R3" s="2" t="s">
-        <v>0</v>
-      </c>
-      <c r="S3" s="2" t="s">
-        <v>1</v>
-      </c>
-      <c r="T3" s="2" t="s">
-        <v>45</v>
-      </c>
-      <c r="V3" s="2" t="s">
-        <v>0</v>
-      </c>
-      <c r="W3" s="2" t="s">
-        <v>1</v>
-      </c>
-      <c r="X3" s="2" t="s">
-        <v>45</v>
-      </c>
-    </row>
-    <row r="4" spans="2:24" x14ac:dyDescent="0.2">
-      <c r="B4" s="3"/>
-      <c r="C4" s="3"/>
-      <c r="D4" s="3"/>
-      <c r="F4" s="3"/>
-      <c r="G4" s="3"/>
-      <c r="H4" s="3"/>
-      <c r="J4" s="3"/>
-      <c r="K4" s="3"/>
-      <c r="L4" s="3"/>
-      <c r="N4" s="3"/>
-      <c r="O4" s="3"/>
-      <c r="P4" s="3"/>
-      <c r="R4" s="3"/>
-      <c r="S4" s="3"/>
-      <c r="T4" s="3"/>
-      <c r="V4" s="3"/>
-      <c r="W4" s="3"/>
-      <c r="X4" s="3"/>
-    </row>
-    <row r="5" spans="2:24" x14ac:dyDescent="0.2">
-      <c r="B5" s="3"/>
-      <c r="C5" s="3"/>
-      <c r="D5" s="3"/>
-      <c r="F5" s="3"/>
-      <c r="G5" s="3"/>
-      <c r="H5" s="3"/>
-      <c r="J5" s="3"/>
-      <c r="K5" s="3"/>
-      <c r="L5" s="3"/>
-      <c r="N5" s="3"/>
-      <c r="O5" s="3"/>
-      <c r="P5" s="3"/>
-      <c r="R5" s="3"/>
-      <c r="S5" s="3"/>
-      <c r="T5" s="3"/>
-      <c r="V5" s="3"/>
-      <c r="W5" s="3"/>
-      <c r="X5" s="3"/>
-    </row>
-    <row r="6" spans="2:24" x14ac:dyDescent="0.2">
-      <c r="B6" s="3"/>
-      <c r="C6" s="3"/>
-      <c r="D6" s="3"/>
-      <c r="F6" s="3"/>
-      <c r="G6" s="3"/>
-      <c r="H6" s="3"/>
-      <c r="J6" s="3"/>
-      <c r="K6" s="3"/>
-      <c r="L6" s="3"/>
-      <c r="N6" s="3"/>
-      <c r="O6" s="3"/>
-      <c r="P6" s="3"/>
-      <c r="R6" s="3"/>
-      <c r="S6" s="3"/>
-      <c r="T6" s="3"/>
-      <c r="V6" s="3"/>
-      <c r="W6" s="3"/>
-      <c r="X6" s="3"/>
-    </row>
-    <row r="7" spans="2:24" x14ac:dyDescent="0.2">
-      <c r="B7" s="3"/>
-      <c r="C7" s="3"/>
-      <c r="D7" s="3"/>
-      <c r="F7" s="3"/>
-      <c r="G7" s="3"/>
-      <c r="H7" s="3"/>
-      <c r="J7" s="3"/>
-      <c r="K7" s="3"/>
-      <c r="L7" s="3"/>
-      <c r="N7" s="3"/>
-      <c r="O7" s="3"/>
-      <c r="P7" s="3"/>
-      <c r="R7" s="3"/>
-      <c r="S7" s="3"/>
-      <c r="T7" s="3"/>
-      <c r="V7" s="3"/>
-      <c r="W7" s="3"/>
-      <c r="X7" s="3"/>
-    </row>
-    <row r="8" spans="2:24" x14ac:dyDescent="0.2">
-      <c r="B8" s="3"/>
-      <c r="C8" s="3"/>
-      <c r="D8" s="3"/>
-      <c r="F8" s="3"/>
-      <c r="G8" s="3"/>
-      <c r="H8" s="3"/>
-      <c r="J8" s="3"/>
-      <c r="K8" s="3"/>
-      <c r="L8" s="3"/>
-      <c r="N8" s="3"/>
-      <c r="O8" s="3"/>
-      <c r="P8" s="3"/>
-      <c r="R8" s="3"/>
-      <c r="S8" s="3"/>
-      <c r="T8" s="3"/>
-      <c r="V8" s="3"/>
-      <c r="W8" s="3"/>
-      <c r="X8" s="3"/>
-    </row>
-    <row r="9" spans="2:24" x14ac:dyDescent="0.2">
-      <c r="B9" s="3"/>
-      <c r="C9" s="3"/>
-      <c r="D9" s="3"/>
-      <c r="F9" s="3"/>
-      <c r="G9" s="3"/>
-      <c r="H9" s="3"/>
-      <c r="J9" s="3"/>
-      <c r="K9" s="3"/>
-      <c r="L9" s="3"/>
-      <c r="N9" s="3"/>
-      <c r="O9" s="3"/>
-      <c r="P9" s="3"/>
-      <c r="R9" s="3"/>
-      <c r="S9" s="3"/>
-      <c r="T9" s="3"/>
-      <c r="V9" s="3"/>
-      <c r="W9" s="3"/>
-      <c r="X9" s="3"/>
-    </row>
-    <row r="10" spans="2:24" x14ac:dyDescent="0.2">
-      <c r="B10" s="3"/>
-      <c r="C10" s="3"/>
-      <c r="D10" s="3"/>
-      <c r="F10" s="3"/>
-      <c r="G10" s="3"/>
-      <c r="H10" s="3"/>
-      <c r="J10" s="3"/>
-      <c r="K10" s="3"/>
-      <c r="L10" s="3"/>
-      <c r="N10" s="3"/>
-      <c r="O10" s="3"/>
-      <c r="P10" s="3"/>
-      <c r="R10" s="3"/>
-      <c r="S10" s="3"/>
-      <c r="T10" s="3"/>
-      <c r="V10" s="3"/>
-      <c r="W10" s="3"/>
-      <c r="X10" s="3"/>
-    </row>
-    <row r="11" spans="2:24" x14ac:dyDescent="0.2">
-      <c r="B11" s="3"/>
-      <c r="C11" s="3"/>
-      <c r="D11" s="3"/>
-      <c r="F11" s="3"/>
-      <c r="G11" s="3"/>
-      <c r="H11" s="3"/>
-      <c r="J11" s="3"/>
-      <c r="K11" s="3"/>
-      <c r="L11" s="3"/>
-      <c r="N11" s="3"/>
-      <c r="O11" s="3"/>
-      <c r="P11" s="3"/>
-      <c r="R11" s="3"/>
-      <c r="S11" s="3"/>
-      <c r="T11" s="3"/>
-      <c r="V11" s="3"/>
-      <c r="W11" s="3"/>
-      <c r="X11" s="3"/>
-    </row>
-    <row r="12" spans="2:24" x14ac:dyDescent="0.2">
-      <c r="B12" s="3"/>
-      <c r="C12" s="3"/>
-      <c r="D12" s="3"/>
-      <c r="F12" s="3"/>
-      <c r="G12" s="3"/>
-      <c r="H12" s="3"/>
-      <c r="J12" s="3"/>
-      <c r="K12" s="3"/>
-      <c r="L12" s="3"/>
-      <c r="N12" s="3"/>
-      <c r="O12" s="3"/>
-      <c r="P12" s="3"/>
-      <c r="R12" s="3"/>
-      <c r="S12" s="3"/>
-      <c r="T12" s="3"/>
-      <c r="V12" s="3"/>
-      <c r="W12" s="3"/>
-      <c r="X12" s="3"/>
-    </row>
-    <row r="13" spans="2:24" x14ac:dyDescent="0.2">
-      <c r="B13" s="3"/>
-      <c r="C13" s="3"/>
-      <c r="D13" s="3"/>
-      <c r="F13" s="3"/>
-      <c r="G13" s="3"/>
-      <c r="H13" s="3"/>
-      <c r="J13" s="3"/>
-      <c r="K13" s="3"/>
-      <c r="L13" s="3"/>
-      <c r="N13" s="3"/>
-      <c r="O13" s="3"/>
-      <c r="P13" s="3"/>
-      <c r="R13" s="3"/>
-      <c r="S13" s="3"/>
-      <c r="T13" s="3"/>
-      <c r="V13" s="3"/>
-      <c r="W13" s="3"/>
-      <c r="X13" s="3"/>
-    </row>
-    <row r="14" spans="2:24" x14ac:dyDescent="0.2">
-      <c r="B14" s="3"/>
-      <c r="C14" s="3"/>
-      <c r="D14" s="3"/>
-      <c r="F14" s="3"/>
-      <c r="G14" s="3"/>
-      <c r="H14" s="3"/>
-      <c r="J14" s="3"/>
-      <c r="K14" s="3"/>
-      <c r="L14" s="3"/>
-      <c r="N14" s="3"/>
-      <c r="O14" s="3"/>
-      <c r="P14" s="3"/>
-      <c r="R14" s="3"/>
-      <c r="S14" s="3"/>
-      <c r="T14" s="3"/>
-      <c r="V14" s="3"/>
-      <c r="W14" s="3"/>
-      <c r="X14" s="3"/>
-    </row>
-    <row r="15" spans="2:24" x14ac:dyDescent="0.2">
-      <c r="B15" s="3"/>
-      <c r="C15" s="3"/>
-      <c r="D15" s="3"/>
-      <c r="F15" s="3"/>
-      <c r="G15" s="3"/>
-      <c r="H15" s="3"/>
-      <c r="J15" s="3"/>
-      <c r="K15" s="3"/>
-      <c r="L15" s="3"/>
-      <c r="N15" s="3"/>
-      <c r="O15" s="3"/>
-      <c r="P15" s="3"/>
-      <c r="R15" s="3"/>
-      <c r="S15" s="3"/>
-      <c r="T15" s="3"/>
-      <c r="V15" s="3"/>
-      <c r="W15" s="3"/>
-      <c r="X15" s="3"/>
-    </row>
-    <row r="16" spans="2:24" x14ac:dyDescent="0.2">
-      <c r="B16" s="3"/>
-      <c r="C16" s="3"/>
-      <c r="D16" s="3"/>
-      <c r="F16" s="3"/>
-      <c r="G16" s="3"/>
-      <c r="H16" s="3"/>
-      <c r="J16" s="3"/>
-      <c r="K16" s="3"/>
-      <c r="L16" s="3"/>
-      <c r="N16" s="3"/>
-      <c r="O16" s="3"/>
-      <c r="P16" s="3"/>
-      <c r="R16" s="3"/>
-      <c r="S16" s="3"/>
-      <c r="T16" s="3"/>
-      <c r="V16" s="3"/>
-      <c r="W16" s="3"/>
-      <c r="X16" s="3"/>
-    </row>
-    <row r="17" spans="2:24" x14ac:dyDescent="0.2">
-      <c r="B17" s="3"/>
-      <c r="C17" s="3"/>
-      <c r="D17" s="3"/>
-      <c r="F17" s="3"/>
-      <c r="G17" s="3"/>
-      <c r="H17" s="3"/>
-      <c r="J17" s="3"/>
-      <c r="K17" s="3"/>
-      <c r="L17" s="3"/>
-      <c r="N17" s="3"/>
-      <c r="O17" s="3"/>
-      <c r="P17" s="3"/>
-      <c r="R17" s="3"/>
-      <c r="S17" s="3"/>
-      <c r="T17" s="3"/>
-      <c r="V17" s="3"/>
-      <c r="W17" s="3"/>
-      <c r="X17" s="3"/>
-    </row>
-    <row r="18" spans="2:24" x14ac:dyDescent="0.2">
-      <c r="B18" s="3"/>
-      <c r="C18" s="3"/>
-      <c r="D18" s="3"/>
-      <c r="F18" s="3"/>
-      <c r="G18" s="3"/>
-      <c r="H18" s="3"/>
-      <c r="J18" s="3"/>
-      <c r="K18" s="3"/>
-      <c r="L18" s="3"/>
-      <c r="N18" s="3"/>
-      <c r="O18" s="3"/>
-      <c r="P18" s="3"/>
-      <c r="R18" s="3"/>
-      <c r="S18" s="3"/>
-      <c r="T18" s="3"/>
-      <c r="V18" s="3"/>
-      <c r="W18" s="3"/>
-      <c r="X18" s="3"/>
-    </row>
-    <row r="19" spans="2:24" x14ac:dyDescent="0.2">
-      <c r="B19" s="3"/>
-      <c r="C19" s="3"/>
-      <c r="D19" s="3"/>
-      <c r="F19" s="3"/>
-      <c r="G19" s="3"/>
-      <c r="H19" s="3"/>
-      <c r="J19" s="3"/>
-      <c r="K19" s="3"/>
-      <c r="L19" s="3"/>
-      <c r="N19" s="3"/>
-      <c r="O19" s="3"/>
-      <c r="P19" s="3"/>
-      <c r="R19" s="3"/>
-      <c r="S19" s="3"/>
-      <c r="T19" s="3"/>
-      <c r="V19" s="3"/>
-      <c r="W19" s="3"/>
-      <c r="X19" s="3"/>
-    </row>
-    <row r="20" spans="2:24" x14ac:dyDescent="0.2">
-      <c r="B20" s="3"/>
-      <c r="C20" s="3"/>
-      <c r="D20" s="3"/>
-      <c r="F20" s="3"/>
-      <c r="G20" s="3"/>
-      <c r="H20" s="3"/>
-      <c r="J20" s="3"/>
-      <c r="K20" s="3"/>
-      <c r="L20" s="3"/>
-      <c r="N20" s="3"/>
-      <c r="O20" s="3"/>
-      <c r="P20" s="3"/>
-      <c r="R20" s="3"/>
-      <c r="S20" s="3"/>
-      <c r="T20" s="3"/>
-      <c r="V20" s="3"/>
-      <c r="W20" s="3"/>
-      <c r="X20" s="3"/>
-    </row>
-    <row r="21" spans="2:24" x14ac:dyDescent="0.2">
-      <c r="B21" s="3"/>
-      <c r="C21" s="3"/>
-      <c r="D21" s="3"/>
-      <c r="F21" s="3"/>
-      <c r="G21" s="3"/>
-      <c r="H21" s="3"/>
-      <c r="J21" s="3"/>
-      <c r="K21" s="3"/>
-      <c r="L21" s="3"/>
-      <c r="N21" s="3"/>
-      <c r="O21" s="3"/>
-      <c r="P21" s="3"/>
-      <c r="R21" s="3"/>
-      <c r="S21" s="3"/>
-      <c r="T21" s="3"/>
-      <c r="V21" s="3"/>
-      <c r="W21" s="3"/>
-      <c r="X21" s="3"/>
-    </row>
-    <row r="22" spans="2:24" x14ac:dyDescent="0.2">
-      <c r="B22" s="3"/>
-      <c r="C22" s="3"/>
-      <c r="D22" s="3"/>
-      <c r="F22" s="3"/>
-      <c r="G22" s="3"/>
-      <c r="H22" s="3"/>
-      <c r="J22" s="3"/>
-      <c r="K22" s="3"/>
-      <c r="L22" s="3"/>
-      <c r="N22" s="3"/>
-      <c r="O22" s="3"/>
-      <c r="P22" s="3"/>
-      <c r="R22" s="3"/>
-      <c r="S22" s="3"/>
-      <c r="T22" s="3"/>
-      <c r="V22" s="3"/>
-      <c r="W22" s="3"/>
-      <c r="X22" s="3"/>
-    </row>
-  </sheetData>
-  <mergeCells count="6">
-    <mergeCell ref="R2:T2"/>
-    <mergeCell ref="V2:X2"/>
-    <mergeCell ref="B2:D2"/>
-    <mergeCell ref="F2:H2"/>
-    <mergeCell ref="J2:L2"/>
-    <mergeCell ref="N2:P2"/>
-  </mergeCells>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-</worksheet>
 </file>
</xml_diff>

<commit_message>
template v18: Ss/Sy mat columns added; stray sheet removed (Norm)
Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_0147GB4LGVZuqGHCRMVzZTsR
</commit_message>
<xml_diff>
--- a/docs/inputs/input_template.xlsx
+++ b/docs/inputs/input_template.xlsx
@@ -1,42 +1,41 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10719"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10713"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/Jones/python_projects/xslope/docs/inputs/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/njones/python_projects/xslope/docs/inputs/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{69AB93CB-4984-D04D-83D8-31B63690B3CE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{525EDD25-6AD6-D045-8DB4-9766BDA4A811}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="680" windowWidth="34200" windowHeight="19900" activeTab="16" xr2:uid="{BA54C293-CE08-6E4C-9212-B3317DAA148E}"/>
+    <workbookView xWindow="0" yWindow="620" windowWidth="34200" windowHeight="19900" xr2:uid="{BA54C293-CE08-6E4C-9212-B3317DAA148E}"/>
   </bookViews>
   <sheets>
     <sheet name="main" sheetId="1" r:id="rId1"/>
-    <sheet name="Sheet1" sheetId="18" r:id="rId2"/>
-    <sheet name="plot" sheetId="9" r:id="rId3"/>
-    <sheet name="mat" sheetId="3" r:id="rId4"/>
-    <sheet name="profile" sheetId="2" r:id="rId5"/>
-    <sheet name="polygon" sheetId="15" r:id="rId6"/>
-    <sheet name="piezo" sheetId="4" r:id="rId7"/>
-    <sheet name="circles" sheetId="5" r:id="rId8"/>
-    <sheet name="non-circ" sheetId="7" r:id="rId9"/>
-    <sheet name="dloads" sheetId="8" r:id="rId10"/>
-    <sheet name="dloads (2)" sheetId="13" r:id="rId11"/>
-    <sheet name="reinforce" sheetId="12" r:id="rId12"/>
-    <sheet name="piles" sheetId="16" r:id="rId13"/>
-    <sheet name="lloads" sheetId="17" r:id="rId14"/>
-    <sheet name="seep bc" sheetId="11" r:id="rId15"/>
-    <sheet name="seep bc (2)" sheetId="14" r:id="rId16"/>
-    <sheet name="tseep" sheetId="19" r:id="rId17"/>
+    <sheet name="plot" sheetId="9" r:id="rId2"/>
+    <sheet name="mat" sheetId="3" r:id="rId3"/>
+    <sheet name="profile" sheetId="2" r:id="rId4"/>
+    <sheet name="polygon" sheetId="15" r:id="rId5"/>
+    <sheet name="piezo" sheetId="4" r:id="rId6"/>
+    <sheet name="circles" sheetId="5" r:id="rId7"/>
+    <sheet name="non-circ" sheetId="7" r:id="rId8"/>
+    <sheet name="dloads" sheetId="8" r:id="rId9"/>
+    <sheet name="dloads (2)" sheetId="13" r:id="rId10"/>
+    <sheet name="reinforce" sheetId="12" r:id="rId11"/>
+    <sheet name="piles" sheetId="16" r:id="rId12"/>
+    <sheet name="lloads" sheetId="17" r:id="rId13"/>
+    <sheet name="seep bc" sheetId="11" r:id="rId14"/>
+    <sheet name="seep bc (2)" sheetId="14" r:id="rId15"/>
+    <sheet name="tseep" sheetId="19" r:id="rId16"/>
   </sheets>
   <definedNames>
     <definedName name="crack_depth">main!$D$11</definedName>
     <definedName name="crack_depth_water">main!$D$12</definedName>
     <definedName name="gamma_w">main!$D$10</definedName>
     <definedName name="k">main!$D$13</definedName>
-    <definedName name="max_depth" localSheetId="5">polygon!#REF!</definedName>
+    <definedName name="max_depth" localSheetId="4">polygon!#REF!</definedName>
     <definedName name="max_depth">profile!$B$2</definedName>
     <definedName name="mesh">mat!#REF!</definedName>
     <definedName name="solution1">mat!#REF!</definedName>
@@ -64,7 +63,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="475" uniqueCount="262">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="477" uniqueCount="264">
   <si>
     <t>X</t>
   </si>
@@ -1015,6 +1014,12 @@
   </si>
   <si>
     <t>Transient seepage boundary conditions and run options</t>
+  </si>
+  <si>
+    <t>Ss</t>
+  </si>
+  <si>
+    <t>Sy</t>
   </si>
 </sst>
 </file>
@@ -1354,7 +1359,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="65">
+  <cellXfs count="64">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -1489,19 +1494,22 @@
     <xf numFmtId="0" fontId="5" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="0" fontId="4" fillId="17" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
     <xf numFmtId="0" fontId="4" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="10" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
     <xf numFmtId="0" fontId="2" fillId="14" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="14" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="15" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -1528,17 +1536,25 @@
     <xf numFmtId="0" fontId="1" fillId="13" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="17" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="21">
+  <dxfs count="23">
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="0" tint="-0.499984740745262"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="0" tint="-0.499984740745262"/>
+        </patternFill>
+      </fill>
+    </dxf>
     <dxf>
       <fill>
         <patternFill>
@@ -9034,6 +9050,499 @@
 </c:chartSpace>
 </file>
 
+<file path=xl/charts/chart2.xml><?xml version="1.0" encoding="utf-8"?>
+<c:chartSpace xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c16r2="http://schemas.microsoft.com/office/drawing/2015/06/chart">
+  <c:date1904 val="0"/>
+  <c:lang val="en-US"/>
+  <c:roundedCorners val="0"/>
+  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+    <mc:Choice xmlns:c14="http://schemas.microsoft.com/office/drawing/2007/8/2/chart" Requires="c14">
+      <c14:style val="102"/>
+    </mc:Choice>
+    <mc:Fallback>
+      <c:style val="2"/>
+    </mc:Fallback>
+  </mc:AlternateContent>
+  <c:chart>
+    <c:autoTitleDeleted val="1"/>
+    <c:plotArea>
+      <c:layout/>
+      <c:scatterChart>
+        <c:scatterStyle val="smoothMarker"/>
+        <c:varyColors val="0"/>
+        <c:ser>
+          <c:idx val="0"/>
+          <c:order val="0"/>
+          <c:tx>
+            <c:strRef>
+              <c:f>tseep!$H$2</c:f>
+              <c:strCache>
+                <c:ptCount val="1"/>
+                <c:pt idx="0">
+                  <c:v>t1</c:v>
+                </c:pt>
+              </c:strCache>
+            </c:strRef>
+          </c:tx>
+          <c:spPr>
+            <a:ln w="19050" cap="rnd">
+              <a:solidFill>
+                <a:schemeClr val="accent1"/>
+              </a:solidFill>
+              <a:round/>
+            </a:ln>
+            <a:effectLst/>
+          </c:spPr>
+          <c:marker>
+            <c:symbol val="none"/>
+          </c:marker>
+          <c:xVal>
+            <c:numRef>
+              <c:f>tseep!$G$3:$G$30</c:f>
+              <c:numCache>
+                <c:formatCode>General</c:formatCode>
+                <c:ptCount val="28"/>
+              </c:numCache>
+            </c:numRef>
+          </c:xVal>
+          <c:yVal>
+            <c:numRef>
+              <c:f>tseep!$H$3:$H$30</c:f>
+              <c:numCache>
+                <c:formatCode>General</c:formatCode>
+                <c:ptCount val="28"/>
+              </c:numCache>
+            </c:numRef>
+          </c:yVal>
+          <c:smooth val="1"/>
+          <c:extLst>
+            <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+              <c16:uniqueId val="{00000000-538B-9247-859A-D6EC9732CE9B}"/>
+            </c:ext>
+          </c:extLst>
+        </c:ser>
+        <c:ser>
+          <c:idx val="1"/>
+          <c:order val="1"/>
+          <c:tx>
+            <c:strRef>
+              <c:f>tseep!$I$2</c:f>
+              <c:strCache>
+                <c:ptCount val="1"/>
+                <c:pt idx="0">
+                  <c:v>t2</c:v>
+                </c:pt>
+              </c:strCache>
+            </c:strRef>
+          </c:tx>
+          <c:spPr>
+            <a:ln w="19050" cap="rnd">
+              <a:solidFill>
+                <a:schemeClr val="accent2"/>
+              </a:solidFill>
+              <a:round/>
+            </a:ln>
+            <a:effectLst/>
+          </c:spPr>
+          <c:marker>
+            <c:symbol val="none"/>
+          </c:marker>
+          <c:xVal>
+            <c:numRef>
+              <c:f>tseep!$G$3:$G$30</c:f>
+              <c:numCache>
+                <c:formatCode>General</c:formatCode>
+                <c:ptCount val="28"/>
+              </c:numCache>
+            </c:numRef>
+          </c:xVal>
+          <c:yVal>
+            <c:numRef>
+              <c:f>tseep!$I$3:$I$30</c:f>
+              <c:numCache>
+                <c:formatCode>General</c:formatCode>
+                <c:ptCount val="28"/>
+              </c:numCache>
+            </c:numRef>
+          </c:yVal>
+          <c:smooth val="1"/>
+          <c:extLst>
+            <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+              <c16:uniqueId val="{00000001-538B-9247-859A-D6EC9732CE9B}"/>
+            </c:ext>
+          </c:extLst>
+        </c:ser>
+        <c:ser>
+          <c:idx val="2"/>
+          <c:order val="2"/>
+          <c:tx>
+            <c:strRef>
+              <c:f>tseep!$J$2</c:f>
+              <c:strCache>
+                <c:ptCount val="1"/>
+                <c:pt idx="0">
+                  <c:v>t3</c:v>
+                </c:pt>
+              </c:strCache>
+            </c:strRef>
+          </c:tx>
+          <c:spPr>
+            <a:ln w="19050" cap="rnd">
+              <a:solidFill>
+                <a:schemeClr val="accent3"/>
+              </a:solidFill>
+              <a:round/>
+            </a:ln>
+            <a:effectLst/>
+          </c:spPr>
+          <c:marker>
+            <c:symbol val="none"/>
+          </c:marker>
+          <c:xVal>
+            <c:numRef>
+              <c:f>tseep!$G$3:$G$30</c:f>
+              <c:numCache>
+                <c:formatCode>General</c:formatCode>
+                <c:ptCount val="28"/>
+              </c:numCache>
+            </c:numRef>
+          </c:xVal>
+          <c:yVal>
+            <c:numRef>
+              <c:f>tseep!$J$3:$J$30</c:f>
+              <c:numCache>
+                <c:formatCode>General</c:formatCode>
+                <c:ptCount val="28"/>
+              </c:numCache>
+            </c:numRef>
+          </c:yVal>
+          <c:smooth val="1"/>
+          <c:extLst>
+            <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+              <c16:uniqueId val="{00000002-538B-9247-859A-D6EC9732CE9B}"/>
+            </c:ext>
+          </c:extLst>
+        </c:ser>
+        <c:ser>
+          <c:idx val="3"/>
+          <c:order val="3"/>
+          <c:tx>
+            <c:strRef>
+              <c:f>tseep!$K$2</c:f>
+              <c:strCache>
+                <c:ptCount val="1"/>
+                <c:pt idx="0">
+                  <c:v>t4</c:v>
+                </c:pt>
+              </c:strCache>
+            </c:strRef>
+          </c:tx>
+          <c:spPr>
+            <a:ln w="19050" cap="rnd">
+              <a:solidFill>
+                <a:schemeClr val="accent4"/>
+              </a:solidFill>
+              <a:round/>
+            </a:ln>
+            <a:effectLst/>
+          </c:spPr>
+          <c:marker>
+            <c:symbol val="none"/>
+          </c:marker>
+          <c:xVal>
+            <c:numRef>
+              <c:f>tseep!$G$3:$G$30</c:f>
+              <c:numCache>
+                <c:formatCode>General</c:formatCode>
+                <c:ptCount val="28"/>
+              </c:numCache>
+            </c:numRef>
+          </c:xVal>
+          <c:yVal>
+            <c:numRef>
+              <c:f>tseep!$K$3:$K$30</c:f>
+              <c:numCache>
+                <c:formatCode>General</c:formatCode>
+                <c:ptCount val="28"/>
+              </c:numCache>
+            </c:numRef>
+          </c:yVal>
+          <c:smooth val="1"/>
+          <c:extLst>
+            <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+              <c16:uniqueId val="{00000003-538B-9247-859A-D6EC9732CE9B}"/>
+            </c:ext>
+          </c:extLst>
+        </c:ser>
+        <c:ser>
+          <c:idx val="4"/>
+          <c:order val="4"/>
+          <c:tx>
+            <c:strRef>
+              <c:f>tseep!$L$2</c:f>
+              <c:strCache>
+                <c:ptCount val="1"/>
+                <c:pt idx="0">
+                  <c:v>t5</c:v>
+                </c:pt>
+              </c:strCache>
+            </c:strRef>
+          </c:tx>
+          <c:spPr>
+            <a:ln w="19050" cap="rnd">
+              <a:solidFill>
+                <a:schemeClr val="accent5"/>
+              </a:solidFill>
+              <a:round/>
+            </a:ln>
+            <a:effectLst/>
+          </c:spPr>
+          <c:marker>
+            <c:symbol val="none"/>
+          </c:marker>
+          <c:xVal>
+            <c:numRef>
+              <c:f>tseep!$G$3:$G$30</c:f>
+              <c:numCache>
+                <c:formatCode>General</c:formatCode>
+                <c:ptCount val="28"/>
+              </c:numCache>
+            </c:numRef>
+          </c:xVal>
+          <c:yVal>
+            <c:numRef>
+              <c:f>tseep!$L$3:$L$30</c:f>
+              <c:numCache>
+                <c:formatCode>General</c:formatCode>
+                <c:ptCount val="28"/>
+              </c:numCache>
+            </c:numRef>
+          </c:yVal>
+          <c:smooth val="1"/>
+          <c:extLst>
+            <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+              <c16:uniqueId val="{00000004-538B-9247-859A-D6EC9732CE9B}"/>
+            </c:ext>
+          </c:extLst>
+        </c:ser>
+        <c:dLbls>
+          <c:showLegendKey val="0"/>
+          <c:showVal val="0"/>
+          <c:showCatName val="0"/>
+          <c:showSerName val="0"/>
+          <c:showPercent val="0"/>
+          <c:showBubbleSize val="0"/>
+        </c:dLbls>
+        <c:axId val="782614975"/>
+        <c:axId val="782616767"/>
+      </c:scatterChart>
+      <c:valAx>
+        <c:axId val="782614975"/>
+        <c:scaling>
+          <c:orientation val="minMax"/>
+        </c:scaling>
+        <c:delete val="0"/>
+        <c:axPos val="b"/>
+        <c:majorGridlines>
+          <c:spPr>
+            <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+              <a:solidFill>
+                <a:schemeClr val="tx1">
+                  <a:lumMod val="15000"/>
+                  <a:lumOff val="85000"/>
+                </a:schemeClr>
+              </a:solidFill>
+              <a:round/>
+            </a:ln>
+            <a:effectLst/>
+          </c:spPr>
+        </c:majorGridlines>
+        <c:numFmt formatCode="General" sourceLinked="1"/>
+        <c:majorTickMark val="none"/>
+        <c:minorTickMark val="none"/>
+        <c:tickLblPos val="nextTo"/>
+        <c:spPr>
+          <a:noFill/>
+          <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+            <a:solidFill>
+              <a:schemeClr val="tx1">
+                <a:lumMod val="25000"/>
+                <a:lumOff val="75000"/>
+              </a:schemeClr>
+            </a:solidFill>
+            <a:round/>
+          </a:ln>
+          <a:effectLst/>
+        </c:spPr>
+        <c:txPr>
+          <a:bodyPr rot="-60000000" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+          <a:lstStyle/>
+          <a:p>
+            <a:pPr>
+              <a:defRPr sz="900" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                <a:solidFill>
+                  <a:schemeClr val="tx1">
+                    <a:lumMod val="65000"/>
+                    <a:lumOff val="35000"/>
+                  </a:schemeClr>
+                </a:solidFill>
+                <a:latin typeface="+mn-lt"/>
+                <a:ea typeface="+mn-ea"/>
+                <a:cs typeface="+mn-cs"/>
+              </a:defRPr>
+            </a:pPr>
+            <a:endParaRPr lang="en-US"/>
+          </a:p>
+        </c:txPr>
+        <c:crossAx val="782616767"/>
+        <c:crosses val="autoZero"/>
+        <c:crossBetween val="midCat"/>
+      </c:valAx>
+      <c:valAx>
+        <c:axId val="782616767"/>
+        <c:scaling>
+          <c:orientation val="minMax"/>
+        </c:scaling>
+        <c:delete val="0"/>
+        <c:axPos val="l"/>
+        <c:majorGridlines>
+          <c:spPr>
+            <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+              <a:solidFill>
+                <a:schemeClr val="tx1">
+                  <a:lumMod val="15000"/>
+                  <a:lumOff val="85000"/>
+                </a:schemeClr>
+              </a:solidFill>
+              <a:round/>
+            </a:ln>
+            <a:effectLst/>
+          </c:spPr>
+        </c:majorGridlines>
+        <c:numFmt formatCode="General" sourceLinked="1"/>
+        <c:majorTickMark val="none"/>
+        <c:minorTickMark val="none"/>
+        <c:tickLblPos val="nextTo"/>
+        <c:spPr>
+          <a:noFill/>
+          <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+            <a:solidFill>
+              <a:schemeClr val="tx1">
+                <a:lumMod val="25000"/>
+                <a:lumOff val="75000"/>
+              </a:schemeClr>
+            </a:solidFill>
+            <a:round/>
+          </a:ln>
+          <a:effectLst/>
+        </c:spPr>
+        <c:txPr>
+          <a:bodyPr rot="-60000000" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+          <a:lstStyle/>
+          <a:p>
+            <a:pPr>
+              <a:defRPr sz="900" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                <a:solidFill>
+                  <a:schemeClr val="tx1">
+                    <a:lumMod val="65000"/>
+                    <a:lumOff val="35000"/>
+                  </a:schemeClr>
+                </a:solidFill>
+                <a:latin typeface="+mn-lt"/>
+                <a:ea typeface="+mn-ea"/>
+                <a:cs typeface="+mn-cs"/>
+              </a:defRPr>
+            </a:pPr>
+            <a:endParaRPr lang="en-US"/>
+          </a:p>
+        </c:txPr>
+        <c:crossAx val="782614975"/>
+        <c:crosses val="autoZero"/>
+        <c:crossBetween val="midCat"/>
+      </c:valAx>
+      <c:spPr>
+        <a:noFill/>
+        <a:ln>
+          <a:noFill/>
+        </a:ln>
+        <a:effectLst/>
+      </c:spPr>
+    </c:plotArea>
+    <c:legend>
+      <c:legendPos val="b"/>
+      <c:overlay val="0"/>
+      <c:spPr>
+        <a:noFill/>
+        <a:ln>
+          <a:noFill/>
+        </a:ln>
+        <a:effectLst/>
+      </c:spPr>
+      <c:txPr>
+        <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+        <a:lstStyle/>
+        <a:p>
+          <a:pPr>
+            <a:defRPr sz="900" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+              <a:solidFill>
+                <a:schemeClr val="tx1">
+                  <a:lumMod val="65000"/>
+                  <a:lumOff val="35000"/>
+                </a:schemeClr>
+              </a:solidFill>
+              <a:latin typeface="+mn-lt"/>
+              <a:ea typeface="+mn-ea"/>
+              <a:cs typeface="+mn-cs"/>
+            </a:defRPr>
+          </a:pPr>
+          <a:endParaRPr lang="en-US"/>
+        </a:p>
+      </c:txPr>
+    </c:legend>
+    <c:plotVisOnly val="1"/>
+    <c:dispBlanksAs val="gap"/>
+    <c:showDLblsOverMax val="0"/>
+    <c:extLst>
+      <c:ext xmlns:c16r3="http://schemas.microsoft.com/office/drawing/2017/03/chart" uri="{56B9EC1D-385E-4148-901F-78D8002777C0}">
+        <c16r3:dataDisplayOptions16>
+          <c16r3:dispNaAsBlank val="1"/>
+        </c16r3:dataDisplayOptions16>
+      </c:ext>
+    </c:extLst>
+  </c:chart>
+  <c:spPr>
+    <a:solidFill>
+      <a:schemeClr val="bg1"/>
+    </a:solidFill>
+    <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+      <a:solidFill>
+        <a:schemeClr val="tx1">
+          <a:lumMod val="15000"/>
+          <a:lumOff val="85000"/>
+        </a:schemeClr>
+      </a:solidFill>
+      <a:round/>
+    </a:ln>
+    <a:effectLst/>
+  </c:spPr>
+  <c:txPr>
+    <a:bodyPr/>
+    <a:lstStyle/>
+    <a:p>
+      <a:pPr>
+        <a:defRPr/>
+      </a:pPr>
+      <a:endParaRPr lang="en-US"/>
+    </a:p>
+  </c:txPr>
+  <c:printSettings>
+    <c:headerFooter/>
+    <c:pageMargins b="0.75" l="0.7" r="0.7" t="0.75" header="0.3" footer="0.3"/>
+    <c:pageSetup/>
+  </c:printSettings>
+</c:chartSpace>
+</file>
+
 <file path=xl/charts/colors1.xml><?xml version="1.0" encoding="utf-8"?>
 <cs:colorStyle xmlns:cs="http://schemas.microsoft.com/office/drawing/2012/chartStyle" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" meth="cycle" id="10">
   <a:schemeClr val="accent1"/>
@@ -9074,7 +9583,563 @@
 </cs:colorStyle>
 </file>
 
+<file path=xl/charts/colors2.xml><?xml version="1.0" encoding="utf-8"?>
+<cs:colorStyle xmlns:cs="http://schemas.microsoft.com/office/drawing/2012/chartStyle" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" meth="cycle" id="10">
+  <a:schemeClr val="accent1"/>
+  <a:schemeClr val="accent2"/>
+  <a:schemeClr val="accent3"/>
+  <a:schemeClr val="accent4"/>
+  <a:schemeClr val="accent5"/>
+  <a:schemeClr val="accent6"/>
+  <cs:variation/>
+  <cs:variation>
+    <a:lumMod val="60000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="80000"/>
+    <a:lumOff val="20000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="80000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="60000"/>
+    <a:lumOff val="40000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="50000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="70000"/>
+    <a:lumOff val="30000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="70000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="50000"/>
+    <a:lumOff val="50000"/>
+  </cs:variation>
+</cs:colorStyle>
+</file>
+
 <file path=xl/charts/style1.xml><?xml version="1.0" encoding="utf-8"?>
+<cs:chartStyle xmlns:cs="http://schemas.microsoft.com/office/drawing/2012/chartStyle" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" id="240">
+  <cs:axisTitle>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="1000" kern="1200"/>
+  </cs:axisTitle>
+  <cs:categoryAxis>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="25000"/>
+            <a:lumOff val="75000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:categoryAxis>
+  <cs:chartArea mods="allowNoFillOverride allowNoLineOverride">
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="bg1"/>
+      </a:solidFill>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="1000" kern="1200"/>
+  </cs:chartArea>
+  <cs:dataLabel>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="75000"/>
+        <a:lumOff val="25000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:dataLabel>
+  <cs:dataLabelCallout>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="dk1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="lt1"/>
+      </a:solidFill>
+      <a:ln>
+        <a:solidFill>
+          <a:schemeClr val="dk1">
+            <a:lumMod val="25000"/>
+            <a:lumOff val="75000"/>
+          </a:schemeClr>
+        </a:solidFill>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="900" kern="1200"/>
+    <cs:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="clip" horzOverflow="clip" vert="horz" wrap="square" lIns="36576" tIns="18288" rIns="36576" bIns="18288" anchor="ctr" anchorCtr="1">
+      <a:spAutoFit/>
+    </cs:bodyPr>
+  </cs:dataLabelCallout>
+  <cs:dataPoint>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="1">
+      <cs:styleClr val="auto"/>
+    </cs:fillRef>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+  </cs:dataPoint>
+  <cs:dataPoint3D>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="1">
+      <cs:styleClr val="auto"/>
+    </cs:fillRef>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+  </cs:dataPoint3D>
+  <cs:dataPointLine>
+    <cs:lnRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:lnRef>
+    <cs:fillRef idx="1"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="19050" cap="rnd">
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:dataPointLine>
+  <cs:dataPointMarker>
+    <cs:lnRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:lnRef>
+    <cs:fillRef idx="1">
+      <cs:styleClr val="auto"/>
+    </cs:fillRef>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525">
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+      </a:ln>
+    </cs:spPr>
+  </cs:dataPointMarker>
+  <cs:dataPointMarkerLayout symbol="circle" size="5"/>
+  <cs:dataPointWireframe>
+    <cs:lnRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:lnRef>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="dk1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="rnd">
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:dataPointWireframe>
+  <cs:dataTable>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:noFill/>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:dataTable>
+  <cs:downBar>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="dk1">
+          <a:lumMod val="75000"/>
+          <a:lumOff val="25000"/>
+        </a:schemeClr>
+      </a:solidFill>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="65000"/>
+            <a:lumOff val="35000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:downBar>
+  <cs:dropLine>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="35000"/>
+            <a:lumOff val="65000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:dropLine>
+  <cs:errorBar>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="65000"/>
+            <a:lumOff val="35000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:errorBar>
+  <cs:floor>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:noFill/>
+      <a:ln>
+        <a:noFill/>
+      </a:ln>
+    </cs:spPr>
+  </cs:floor>
+  <cs:gridlineMajor>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:gridlineMajor>
+  <cs:gridlineMinor>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="5000"/>
+            <a:lumOff val="95000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:gridlineMinor>
+  <cs:hiLoLine>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="50000"/>
+            <a:lumOff val="50000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:hiLoLine>
+  <cs:leaderLine>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="35000"/>
+            <a:lumOff val="65000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:leaderLine>
+  <cs:legend>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:legend>
+  <cs:plotArea mods="allowNoFillOverride allowNoLineOverride">
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+  </cs:plotArea>
+  <cs:plotArea3D mods="allowNoFillOverride allowNoLineOverride">
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+  </cs:plotArea3D>
+  <cs:seriesAxis>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:seriesAxis>
+  <cs:seriesLine>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="35000"/>
+            <a:lumOff val="65000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:seriesLine>
+  <cs:title>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="1400" b="0" kern="1200" spc="0" baseline="0"/>
+  </cs:title>
+  <cs:trendline>
+    <cs:lnRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:lnRef>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="19050" cap="rnd">
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+        <a:prstDash val="sysDot"/>
+      </a:ln>
+    </cs:spPr>
+  </cs:trendline>
+  <cs:trendlineLabel>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:trendlineLabel>
+  <cs:upBar>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="lt1"/>
+      </a:solidFill>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="65000"/>
+            <a:lumOff val="35000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:upBar>
+  <cs:valueAxis>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="25000"/>
+            <a:lumOff val="75000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:valueAxis>
+  <cs:wall>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:noFill/>
+      <a:ln>
+        <a:noFill/>
+      </a:ln>
+    </cs:spPr>
+  </cs:wall>
+</cs:chartStyle>
+</file>
+
+<file path=xl/charts/style2.xml><?xml version="1.0" encoding="utf-8"?>
 <cs:chartStyle xmlns:cs="http://schemas.microsoft.com/office/drawing/2012/chartStyle" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" id="240">
   <cs:axisTitle>
     <cs:lnRef idx="0"/>
@@ -10198,6 +11263,47 @@
 </xdr:wsDr>
 </file>
 
+<file path=xl/drawings/drawing4.xml><?xml version="1.0" encoding="utf-8"?>
+<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>15</xdr:col>
+      <xdr:colOff>444499</xdr:colOff>
+      <xdr:row>1</xdr:row>
+      <xdr:rowOff>88901</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>22</xdr:col>
+      <xdr:colOff>644071</xdr:colOff>
+      <xdr:row>22</xdr:row>
+      <xdr:rowOff>99787</xdr:rowOff>
+    </xdr:to>
+    <xdr:graphicFrame macro="">
+      <xdr:nvGraphicFramePr>
+        <xdr:cNvPr id="2" name="Chart 1">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{7655F65D-6FA7-DB16-246F-5BDA3120EC02}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvGraphicFramePr/>
+      </xdr:nvGraphicFramePr>
+      <xdr:xfrm>
+        <a:off x="0" y="0"/>
+        <a:ext cx="0" cy="0"/>
+      </xdr:xfrm>
+      <a:graphic>
+        <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
+          <c:chart xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
+        </a:graphicData>
+      </a:graphic>
+    </xdr:graphicFrame>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+</xdr:wsDr>
+</file>
+
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
 <a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
   <a:themeElements>
@@ -10544,11 +11650,11 @@
       </c>
     </row>
     <row r="7" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="B7" s="50" t="s">
+      <c r="B7" s="51" t="s">
         <v>47</v>
       </c>
-      <c r="C7" s="50"/>
-      <c r="D7" s="50"/>
+      <c r="C7" s="51"/>
+      <c r="D7" s="51"/>
       <c r="F7" s="15" t="s">
         <v>15</v>
       </c>
@@ -10777,7 +11883,7 @@
 </file>
 
 <file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{8D19B78E-FBCC-4E41-BB37-C8D0D27B23E8}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{028A122E-8CB6-264D-BE4D-4184948E7CD8}">
   <dimension ref="B2:X22"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
@@ -10796,36 +11902,36 @@
   </cols>
   <sheetData>
     <row r="2" spans="2:24" x14ac:dyDescent="0.2">
-      <c r="B2" s="59" t="s">
-        <v>121</v>
-      </c>
-      <c r="C2" s="59"/>
-      <c r="D2" s="59"/>
-      <c r="F2" s="59" t="s">
-        <v>122</v>
-      </c>
-      <c r="G2" s="59"/>
-      <c r="H2" s="59"/>
-      <c r="J2" s="59" t="s">
-        <v>123</v>
-      </c>
-      <c r="K2" s="59"/>
-      <c r="L2" s="59"/>
-      <c r="N2" s="59" t="s">
-        <v>124</v>
-      </c>
-      <c r="O2" s="59"/>
-      <c r="P2" s="59"/>
-      <c r="R2" s="59" t="s">
-        <v>125</v>
-      </c>
-      <c r="S2" s="59"/>
-      <c r="T2" s="59"/>
-      <c r="V2" s="59" t="s">
-        <v>126</v>
-      </c>
-      <c r="W2" s="59"/>
-      <c r="X2" s="59"/>
+      <c r="B2" s="61" t="s">
+        <v>129</v>
+      </c>
+      <c r="C2" s="61"/>
+      <c r="D2" s="61"/>
+      <c r="F2" s="61" t="s">
+        <v>130</v>
+      </c>
+      <c r="G2" s="61"/>
+      <c r="H2" s="61"/>
+      <c r="J2" s="61" t="s">
+        <v>131</v>
+      </c>
+      <c r="K2" s="61"/>
+      <c r="L2" s="61"/>
+      <c r="N2" s="61" t="s">
+        <v>132</v>
+      </c>
+      <c r="O2" s="61"/>
+      <c r="P2" s="61"/>
+      <c r="R2" s="61" t="s">
+        <v>133</v>
+      </c>
+      <c r="S2" s="61"/>
+      <c r="T2" s="61"/>
+      <c r="V2" s="61" t="s">
+        <v>134</v>
+      </c>
+      <c r="W2" s="61"/>
+      <c r="X2" s="61"/>
     </row>
     <row r="3" spans="2:24" x14ac:dyDescent="0.2">
       <c r="B3" s="2" t="s">
@@ -11277,506 +12383,6 @@
 </file>
 
 <file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{028A122E-8CB6-264D-BE4D-4184948E7CD8}">
-  <dimension ref="B2:X22"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
-  <cols>
-    <col min="1" max="1" width="3" customWidth="1"/>
-    <col min="2" max="4" width="7.6640625" customWidth="1"/>
-    <col min="5" max="5" width="3" customWidth="1"/>
-    <col min="6" max="8" width="7.6640625" customWidth="1"/>
-    <col min="9" max="9" width="3" customWidth="1"/>
-    <col min="10" max="12" width="7.6640625" customWidth="1"/>
-    <col min="13" max="13" width="3" customWidth="1"/>
-    <col min="14" max="16" width="7.6640625" customWidth="1"/>
-    <col min="17" max="17" width="3" customWidth="1"/>
-    <col min="18" max="20" width="7.6640625" customWidth="1"/>
-    <col min="21" max="21" width="3" customWidth="1"/>
-    <col min="22" max="24" width="7.6640625" customWidth="1"/>
-  </cols>
-  <sheetData>
-    <row r="2" spans="2:24" x14ac:dyDescent="0.2">
-      <c r="B2" s="60" t="s">
-        <v>129</v>
-      </c>
-      <c r="C2" s="60"/>
-      <c r="D2" s="60"/>
-      <c r="F2" s="60" t="s">
-        <v>130</v>
-      </c>
-      <c r="G2" s="60"/>
-      <c r="H2" s="60"/>
-      <c r="J2" s="60" t="s">
-        <v>131</v>
-      </c>
-      <c r="K2" s="60"/>
-      <c r="L2" s="60"/>
-      <c r="N2" s="60" t="s">
-        <v>132</v>
-      </c>
-      <c r="O2" s="60"/>
-      <c r="P2" s="60"/>
-      <c r="R2" s="60" t="s">
-        <v>133</v>
-      </c>
-      <c r="S2" s="60"/>
-      <c r="T2" s="60"/>
-      <c r="V2" s="60" t="s">
-        <v>134</v>
-      </c>
-      <c r="W2" s="60"/>
-      <c r="X2" s="60"/>
-    </row>
-    <row r="3" spans="2:24" x14ac:dyDescent="0.2">
-      <c r="B3" s="2" t="s">
-        <v>0</v>
-      </c>
-      <c r="C3" s="2" t="s">
-        <v>1</v>
-      </c>
-      <c r="D3" s="2" t="s">
-        <v>45</v>
-      </c>
-      <c r="F3" s="2" t="s">
-        <v>0</v>
-      </c>
-      <c r="G3" s="2" t="s">
-        <v>1</v>
-      </c>
-      <c r="H3" s="2" t="s">
-        <v>45</v>
-      </c>
-      <c r="J3" s="2" t="s">
-        <v>0</v>
-      </c>
-      <c r="K3" s="2" t="s">
-        <v>1</v>
-      </c>
-      <c r="L3" s="2" t="s">
-        <v>45</v>
-      </c>
-      <c r="N3" s="2" t="s">
-        <v>0</v>
-      </c>
-      <c r="O3" s="2" t="s">
-        <v>1</v>
-      </c>
-      <c r="P3" s="2" t="s">
-        <v>45</v>
-      </c>
-      <c r="R3" s="2" t="s">
-        <v>0</v>
-      </c>
-      <c r="S3" s="2" t="s">
-        <v>1</v>
-      </c>
-      <c r="T3" s="2" t="s">
-        <v>45</v>
-      </c>
-      <c r="V3" s="2" t="s">
-        <v>0</v>
-      </c>
-      <c r="W3" s="2" t="s">
-        <v>1</v>
-      </c>
-      <c r="X3" s="2" t="s">
-        <v>45</v>
-      </c>
-    </row>
-    <row r="4" spans="2:24" x14ac:dyDescent="0.2">
-      <c r="B4" s="3"/>
-      <c r="C4" s="3"/>
-      <c r="D4" s="3"/>
-      <c r="F4" s="3"/>
-      <c r="G4" s="3"/>
-      <c r="H4" s="3"/>
-      <c r="J4" s="3"/>
-      <c r="K4" s="3"/>
-      <c r="L4" s="3"/>
-      <c r="N4" s="3"/>
-      <c r="O4" s="3"/>
-      <c r="P4" s="3"/>
-      <c r="R4" s="3"/>
-      <c r="S4" s="3"/>
-      <c r="T4" s="3"/>
-      <c r="V4" s="3"/>
-      <c r="W4" s="3"/>
-      <c r="X4" s="3"/>
-    </row>
-    <row r="5" spans="2:24" x14ac:dyDescent="0.2">
-      <c r="B5" s="3"/>
-      <c r="C5" s="3"/>
-      <c r="D5" s="3"/>
-      <c r="F5" s="3"/>
-      <c r="G5" s="3"/>
-      <c r="H5" s="3"/>
-      <c r="J5" s="3"/>
-      <c r="K5" s="3"/>
-      <c r="L5" s="3"/>
-      <c r="N5" s="3"/>
-      <c r="O5" s="3"/>
-      <c r="P5" s="3"/>
-      <c r="R5" s="3"/>
-      <c r="S5" s="3"/>
-      <c r="T5" s="3"/>
-      <c r="V5" s="3"/>
-      <c r="W5" s="3"/>
-      <c r="X5" s="3"/>
-    </row>
-    <row r="6" spans="2:24" x14ac:dyDescent="0.2">
-      <c r="B6" s="3"/>
-      <c r="C6" s="3"/>
-      <c r="D6" s="3"/>
-      <c r="F6" s="3"/>
-      <c r="G6" s="3"/>
-      <c r="H6" s="3"/>
-      <c r="J6" s="3"/>
-      <c r="K6" s="3"/>
-      <c r="L6" s="3"/>
-      <c r="N6" s="3"/>
-      <c r="O6" s="3"/>
-      <c r="P6" s="3"/>
-      <c r="R6" s="3"/>
-      <c r="S6" s="3"/>
-      <c r="T6" s="3"/>
-      <c r="V6" s="3"/>
-      <c r="W6" s="3"/>
-      <c r="X6" s="3"/>
-    </row>
-    <row r="7" spans="2:24" x14ac:dyDescent="0.2">
-      <c r="B7" s="3"/>
-      <c r="C7" s="3"/>
-      <c r="D7" s="3"/>
-      <c r="F7" s="3"/>
-      <c r="G7" s="3"/>
-      <c r="H7" s="3"/>
-      <c r="J7" s="3"/>
-      <c r="K7" s="3"/>
-      <c r="L7" s="3"/>
-      <c r="N7" s="3"/>
-      <c r="O7" s="3"/>
-      <c r="P7" s="3"/>
-      <c r="R7" s="3"/>
-      <c r="S7" s="3"/>
-      <c r="T7" s="3"/>
-      <c r="V7" s="3"/>
-      <c r="W7" s="3"/>
-      <c r="X7" s="3"/>
-    </row>
-    <row r="8" spans="2:24" x14ac:dyDescent="0.2">
-      <c r="B8" s="3"/>
-      <c r="C8" s="3"/>
-      <c r="D8" s="3"/>
-      <c r="F8" s="3"/>
-      <c r="G8" s="3"/>
-      <c r="H8" s="3"/>
-      <c r="J8" s="3"/>
-      <c r="K8" s="3"/>
-      <c r="L8" s="3"/>
-      <c r="N8" s="3"/>
-      <c r="O8" s="3"/>
-      <c r="P8" s="3"/>
-      <c r="R8" s="3"/>
-      <c r="S8" s="3"/>
-      <c r="T8" s="3"/>
-      <c r="V8" s="3"/>
-      <c r="W8" s="3"/>
-      <c r="X8" s="3"/>
-    </row>
-    <row r="9" spans="2:24" x14ac:dyDescent="0.2">
-      <c r="B9" s="3"/>
-      <c r="C9" s="3"/>
-      <c r="D9" s="3"/>
-      <c r="F9" s="3"/>
-      <c r="G9" s="3"/>
-      <c r="H9" s="3"/>
-      <c r="J9" s="3"/>
-      <c r="K9" s="3"/>
-      <c r="L9" s="3"/>
-      <c r="N9" s="3"/>
-      <c r="O9" s="3"/>
-      <c r="P9" s="3"/>
-      <c r="R9" s="3"/>
-      <c r="S9" s="3"/>
-      <c r="T9" s="3"/>
-      <c r="V9" s="3"/>
-      <c r="W9" s="3"/>
-      <c r="X9" s="3"/>
-    </row>
-    <row r="10" spans="2:24" x14ac:dyDescent="0.2">
-      <c r="B10" s="3"/>
-      <c r="C10" s="3"/>
-      <c r="D10" s="3"/>
-      <c r="F10" s="3"/>
-      <c r="G10" s="3"/>
-      <c r="H10" s="3"/>
-      <c r="J10" s="3"/>
-      <c r="K10" s="3"/>
-      <c r="L10" s="3"/>
-      <c r="N10" s="3"/>
-      <c r="O10" s="3"/>
-      <c r="P10" s="3"/>
-      <c r="R10" s="3"/>
-      <c r="S10" s="3"/>
-      <c r="T10" s="3"/>
-      <c r="V10" s="3"/>
-      <c r="W10" s="3"/>
-      <c r="X10" s="3"/>
-    </row>
-    <row r="11" spans="2:24" x14ac:dyDescent="0.2">
-      <c r="B11" s="3"/>
-      <c r="C11" s="3"/>
-      <c r="D11" s="3"/>
-      <c r="F11" s="3"/>
-      <c r="G11" s="3"/>
-      <c r="H11" s="3"/>
-      <c r="J11" s="3"/>
-      <c r="K11" s="3"/>
-      <c r="L11" s="3"/>
-      <c r="N11" s="3"/>
-      <c r="O11" s="3"/>
-      <c r="P11" s="3"/>
-      <c r="R11" s="3"/>
-      <c r="S11" s="3"/>
-      <c r="T11" s="3"/>
-      <c r="V11" s="3"/>
-      <c r="W11" s="3"/>
-      <c r="X11" s="3"/>
-    </row>
-    <row r="12" spans="2:24" x14ac:dyDescent="0.2">
-      <c r="B12" s="3"/>
-      <c r="C12" s="3"/>
-      <c r="D12" s="3"/>
-      <c r="F12" s="3"/>
-      <c r="G12" s="3"/>
-      <c r="H12" s="3"/>
-      <c r="J12" s="3"/>
-      <c r="K12" s="3"/>
-      <c r="L12" s="3"/>
-      <c r="N12" s="3"/>
-      <c r="O12" s="3"/>
-      <c r="P12" s="3"/>
-      <c r="R12" s="3"/>
-      <c r="S12" s="3"/>
-      <c r="T12" s="3"/>
-      <c r="V12" s="3"/>
-      <c r="W12" s="3"/>
-      <c r="X12" s="3"/>
-    </row>
-    <row r="13" spans="2:24" x14ac:dyDescent="0.2">
-      <c r="B13" s="3"/>
-      <c r="C13" s="3"/>
-      <c r="D13" s="3"/>
-      <c r="F13" s="3"/>
-      <c r="G13" s="3"/>
-      <c r="H13" s="3"/>
-      <c r="J13" s="3"/>
-      <c r="K13" s="3"/>
-      <c r="L13" s="3"/>
-      <c r="N13" s="3"/>
-      <c r="O13" s="3"/>
-      <c r="P13" s="3"/>
-      <c r="R13" s="3"/>
-      <c r="S13" s="3"/>
-      <c r="T13" s="3"/>
-      <c r="V13" s="3"/>
-      <c r="W13" s="3"/>
-      <c r="X13" s="3"/>
-    </row>
-    <row r="14" spans="2:24" x14ac:dyDescent="0.2">
-      <c r="B14" s="3"/>
-      <c r="C14" s="3"/>
-      <c r="D14" s="3"/>
-      <c r="F14" s="3"/>
-      <c r="G14" s="3"/>
-      <c r="H14" s="3"/>
-      <c r="J14" s="3"/>
-      <c r="K14" s="3"/>
-      <c r="L14" s="3"/>
-      <c r="N14" s="3"/>
-      <c r="O14" s="3"/>
-      <c r="P14" s="3"/>
-      <c r="R14" s="3"/>
-      <c r="S14" s="3"/>
-      <c r="T14" s="3"/>
-      <c r="V14" s="3"/>
-      <c r="W14" s="3"/>
-      <c r="X14" s="3"/>
-    </row>
-    <row r="15" spans="2:24" x14ac:dyDescent="0.2">
-      <c r="B15" s="3"/>
-      <c r="C15" s="3"/>
-      <c r="D15" s="3"/>
-      <c r="F15" s="3"/>
-      <c r="G15" s="3"/>
-      <c r="H15" s="3"/>
-      <c r="J15" s="3"/>
-      <c r="K15" s="3"/>
-      <c r="L15" s="3"/>
-      <c r="N15" s="3"/>
-      <c r="O15" s="3"/>
-      <c r="P15" s="3"/>
-      <c r="R15" s="3"/>
-      <c r="S15" s="3"/>
-      <c r="T15" s="3"/>
-      <c r="V15" s="3"/>
-      <c r="W15" s="3"/>
-      <c r="X15" s="3"/>
-    </row>
-    <row r="16" spans="2:24" x14ac:dyDescent="0.2">
-      <c r="B16" s="3"/>
-      <c r="C16" s="3"/>
-      <c r="D16" s="3"/>
-      <c r="F16" s="3"/>
-      <c r="G16" s="3"/>
-      <c r="H16" s="3"/>
-      <c r="J16" s="3"/>
-      <c r="K16" s="3"/>
-      <c r="L16" s="3"/>
-      <c r="N16" s="3"/>
-      <c r="O16" s="3"/>
-      <c r="P16" s="3"/>
-      <c r="R16" s="3"/>
-      <c r="S16" s="3"/>
-      <c r="T16" s="3"/>
-      <c r="V16" s="3"/>
-      <c r="W16" s="3"/>
-      <c r="X16" s="3"/>
-    </row>
-    <row r="17" spans="2:24" x14ac:dyDescent="0.2">
-      <c r="B17" s="3"/>
-      <c r="C17" s="3"/>
-      <c r="D17" s="3"/>
-      <c r="F17" s="3"/>
-      <c r="G17" s="3"/>
-      <c r="H17" s="3"/>
-      <c r="J17" s="3"/>
-      <c r="K17" s="3"/>
-      <c r="L17" s="3"/>
-      <c r="N17" s="3"/>
-      <c r="O17" s="3"/>
-      <c r="P17" s="3"/>
-      <c r="R17" s="3"/>
-      <c r="S17" s="3"/>
-      <c r="T17" s="3"/>
-      <c r="V17" s="3"/>
-      <c r="W17" s="3"/>
-      <c r="X17" s="3"/>
-    </row>
-    <row r="18" spans="2:24" x14ac:dyDescent="0.2">
-      <c r="B18" s="3"/>
-      <c r="C18" s="3"/>
-      <c r="D18" s="3"/>
-      <c r="F18" s="3"/>
-      <c r="G18" s="3"/>
-      <c r="H18" s="3"/>
-      <c r="J18" s="3"/>
-      <c r="K18" s="3"/>
-      <c r="L18" s="3"/>
-      <c r="N18" s="3"/>
-      <c r="O18" s="3"/>
-      <c r="P18" s="3"/>
-      <c r="R18" s="3"/>
-      <c r="S18" s="3"/>
-      <c r="T18" s="3"/>
-      <c r="V18" s="3"/>
-      <c r="W18" s="3"/>
-      <c r="X18" s="3"/>
-    </row>
-    <row r="19" spans="2:24" x14ac:dyDescent="0.2">
-      <c r="B19" s="3"/>
-      <c r="C19" s="3"/>
-      <c r="D19" s="3"/>
-      <c r="F19" s="3"/>
-      <c r="G19" s="3"/>
-      <c r="H19" s="3"/>
-      <c r="J19" s="3"/>
-      <c r="K19" s="3"/>
-      <c r="L19" s="3"/>
-      <c r="N19" s="3"/>
-      <c r="O19" s="3"/>
-      <c r="P19" s="3"/>
-      <c r="R19" s="3"/>
-      <c r="S19" s="3"/>
-      <c r="T19" s="3"/>
-      <c r="V19" s="3"/>
-      <c r="W19" s="3"/>
-      <c r="X19" s="3"/>
-    </row>
-    <row r="20" spans="2:24" x14ac:dyDescent="0.2">
-      <c r="B20" s="3"/>
-      <c r="C20" s="3"/>
-      <c r="D20" s="3"/>
-      <c r="F20" s="3"/>
-      <c r="G20" s="3"/>
-      <c r="H20" s="3"/>
-      <c r="J20" s="3"/>
-      <c r="K20" s="3"/>
-      <c r="L20" s="3"/>
-      <c r="N20" s="3"/>
-      <c r="O20" s="3"/>
-      <c r="P20" s="3"/>
-      <c r="R20" s="3"/>
-      <c r="S20" s="3"/>
-      <c r="T20" s="3"/>
-      <c r="V20" s="3"/>
-      <c r="W20" s="3"/>
-      <c r="X20" s="3"/>
-    </row>
-    <row r="21" spans="2:24" x14ac:dyDescent="0.2">
-      <c r="B21" s="3"/>
-      <c r="C21" s="3"/>
-      <c r="D21" s="3"/>
-      <c r="F21" s="3"/>
-      <c r="G21" s="3"/>
-      <c r="H21" s="3"/>
-      <c r="J21" s="3"/>
-      <c r="K21" s="3"/>
-      <c r="L21" s="3"/>
-      <c r="N21" s="3"/>
-      <c r="O21" s="3"/>
-      <c r="P21" s="3"/>
-      <c r="R21" s="3"/>
-      <c r="S21" s="3"/>
-      <c r="T21" s="3"/>
-      <c r="V21" s="3"/>
-      <c r="W21" s="3"/>
-      <c r="X21" s="3"/>
-    </row>
-    <row r="22" spans="2:24" x14ac:dyDescent="0.2">
-      <c r="B22" s="3"/>
-      <c r="C22" s="3"/>
-      <c r="D22" s="3"/>
-      <c r="F22" s="3"/>
-      <c r="G22" s="3"/>
-      <c r="H22" s="3"/>
-      <c r="J22" s="3"/>
-      <c r="K22" s="3"/>
-      <c r="L22" s="3"/>
-      <c r="N22" s="3"/>
-      <c r="O22" s="3"/>
-      <c r="P22" s="3"/>
-      <c r="R22" s="3"/>
-      <c r="S22" s="3"/>
-      <c r="T22" s="3"/>
-      <c r="V22" s="3"/>
-      <c r="W22" s="3"/>
-      <c r="X22" s="3"/>
-    </row>
-  </sheetData>
-  <mergeCells count="6">
-    <mergeCell ref="R2:T2"/>
-    <mergeCell ref="V2:X2"/>
-    <mergeCell ref="B2:D2"/>
-    <mergeCell ref="F2:H2"/>
-    <mergeCell ref="J2:L2"/>
-    <mergeCell ref="N2:P2"/>
-  </mergeCells>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C37CF166-6531-CC44-B460-D72E6A0F66E6}">
   <dimension ref="A2:AB25"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
@@ -12504,7 +13110,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet13.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F3B6221D-E989-B546-ACAF-CEB4607C51A1}">
   <dimension ref="A2:AA18"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
@@ -12832,7 +13438,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet14.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet13.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{1FA07123-52EA-314A-81EF-989A42CB4DFE}">
   <dimension ref="A2:F22"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
@@ -13067,7 +13673,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet15.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet14.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{8D036245-91C1-5842-93DD-735018175DE8}">
   <dimension ref="B2:U24"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
@@ -13081,34 +13687,34 @@
   </cols>
   <sheetData>
     <row r="2" spans="2:21" x14ac:dyDescent="0.2">
-      <c r="B2" s="61" t="s">
+      <c r="B2" s="62" t="s">
         <v>127</v>
       </c>
-      <c r="C2" s="61"/>
-      <c r="E2" s="57" t="s">
+      <c r="C2" s="62"/>
+      <c r="E2" s="58" t="s">
         <v>215</v>
       </c>
-      <c r="F2" s="57"/>
-      <c r="H2" s="57" t="s">
+      <c r="F2" s="58"/>
+      <c r="H2" s="58" t="s">
         <v>217</v>
       </c>
-      <c r="I2" s="57"/>
-      <c r="K2" s="57" t="s">
+      <c r="I2" s="58"/>
+      <c r="K2" s="58" t="s">
         <v>218</v>
       </c>
-      <c r="L2" s="57"/>
-      <c r="N2" s="57" t="s">
+      <c r="L2" s="58"/>
+      <c r="N2" s="58" t="s">
         <v>219</v>
       </c>
-      <c r="O2" s="57"/>
-      <c r="Q2" s="57" t="s">
+      <c r="O2" s="58"/>
+      <c r="Q2" s="58" t="s">
         <v>220</v>
       </c>
-      <c r="R2" s="57"/>
+      <c r="R2" s="58"/>
     </row>
     <row r="3" spans="2:21" x14ac:dyDescent="0.2">
-      <c r="B3" s="61"/>
-      <c r="C3" s="61"/>
+      <c r="B3" s="62"/>
+      <c r="C3" s="62"/>
       <c r="E3" s="32" t="s">
         <v>213</v>
       </c>
@@ -13483,7 +14089,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet16.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet15.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{E4C3C734-6227-7445-884D-1F1A5F3909C7}">
   <dimension ref="B2:U24"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
@@ -13497,34 +14103,34 @@
   </cols>
   <sheetData>
     <row r="2" spans="2:21" x14ac:dyDescent="0.2">
-      <c r="B2" s="62" t="s">
+      <c r="B2" s="63" t="s">
         <v>128</v>
       </c>
-      <c r="C2" s="62"/>
-      <c r="E2" s="58" t="s">
+      <c r="C2" s="63"/>
+      <c r="E2" s="59" t="s">
         <v>221</v>
       </c>
-      <c r="F2" s="58"/>
-      <c r="H2" s="58" t="s">
+      <c r="F2" s="59"/>
+      <c r="H2" s="59" t="s">
         <v>222</v>
       </c>
-      <c r="I2" s="58"/>
-      <c r="K2" s="58" t="s">
+      <c r="I2" s="59"/>
+      <c r="K2" s="59" t="s">
         <v>223</v>
       </c>
-      <c r="L2" s="58"/>
-      <c r="N2" s="58" t="s">
+      <c r="L2" s="59"/>
+      <c r="N2" s="59" t="s">
         <v>224</v>
       </c>
-      <c r="O2" s="58"/>
-      <c r="Q2" s="58" t="s">
+      <c r="O2" s="59"/>
+      <c r="Q2" s="59" t="s">
         <v>225</v>
       </c>
-      <c r="R2" s="58"/>
+      <c r="R2" s="59"/>
     </row>
     <row r="3" spans="2:21" x14ac:dyDescent="0.2">
-      <c r="B3" s="62"/>
-      <c r="C3" s="62"/>
+      <c r="B3" s="63"/>
+      <c r="C3" s="63"/>
       <c r="E3" s="34" t="s">
         <v>213</v>
       </c>
@@ -13897,33 +14503,33 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet17.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet16.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B20D353C-FC33-C347-9989-88B2E3FC7B94}">
   <dimension ref="G2:O30"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="6" max="6" width="3.5" customWidth="1"/>
     <col min="7" max="12" width="10.83203125" style="1"/>
-    <col min="13" max="13" width="10" customWidth="1"/>
+    <col min="13" max="13" width="7.1640625" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="2" spans="7:15" x14ac:dyDescent="0.2">
-      <c r="G2" s="64" t="s">
+      <c r="G2" s="50" t="s">
         <v>255</v>
       </c>
-      <c r="H2" s="64" t="s">
+      <c r="H2" s="50" t="s">
         <v>250</v>
       </c>
-      <c r="I2" s="64" t="s">
+      <c r="I2" s="50" t="s">
         <v>251</v>
       </c>
-      <c r="J2" s="64" t="s">
+      <c r="J2" s="50" t="s">
         <v>252</v>
       </c>
-      <c r="K2" s="64" t="s">
+      <c r="K2" s="50" t="s">
         <v>253</v>
       </c>
-      <c r="L2" s="64" t="s">
+      <c r="L2" s="50" t="s">
         <v>254</v>
       </c>
     </row>
@@ -13937,7 +14543,7 @@
       <c r="N3" s="14" t="s">
         <v>257</v>
       </c>
-      <c r="O3" s="63"/>
+      <c r="O3" s="1"/>
     </row>
     <row r="4" spans="7:15" x14ac:dyDescent="0.2">
       <c r="G4" s="3"/>
@@ -13947,7 +14553,7 @@
       <c r="K4" s="3"/>
       <c r="L4" s="3"/>
       <c r="N4" s="14"/>
-      <c r="O4" s="63"/>
+      <c r="O4" s="1"/>
     </row>
     <row r="5" spans="7:15" x14ac:dyDescent="0.2">
       <c r="G5" s="3"/>
@@ -13959,7 +14565,7 @@
       <c r="N5" s="14" t="s">
         <v>256</v>
       </c>
-      <c r="O5" s="63"/>
+      <c r="O5" s="1"/>
     </row>
     <row r="6" spans="7:15" x14ac:dyDescent="0.2">
       <c r="G6" s="3"/>
@@ -13969,7 +14575,7 @@
       <c r="K6" s="3"/>
       <c r="L6" s="3"/>
       <c r="N6" s="14"/>
-      <c r="O6" s="63"/>
+      <c r="O6" s="1"/>
     </row>
     <row r="7" spans="7:15" x14ac:dyDescent="0.2">
       <c r="G7" s="3"/>
@@ -13981,7 +14587,7 @@
       <c r="N7" s="14" t="s">
         <v>258</v>
       </c>
-      <c r="O7" s="63"/>
+      <c r="O7" s="1"/>
     </row>
     <row r="8" spans="7:15" x14ac:dyDescent="0.2">
       <c r="G8" s="3"/>
@@ -13993,7 +14599,7 @@
       <c r="N8" s="14" t="s">
         <v>259</v>
       </c>
-      <c r="O8" s="63"/>
+      <c r="O8" s="1"/>
     </row>
     <row r="9" spans="7:15" x14ac:dyDescent="0.2">
       <c r="G9" s="3"/>
@@ -14173,19 +14779,11 @@
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <drawing r:id="rId1"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F4216D5A-7B51-8B45-AAAC-BBE34074B3B1}">
-  <dimension ref="A1"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
-  <sheetData/>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{FDB4949D-EAAF-AE4C-9BAF-D5BF753E34CD}">
   <dimension ref="A1"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
@@ -14195,18 +14793,18 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{60A900FC-A692-B445-95C9-59E70352B291}">
-  <dimension ref="A2:AN52"/>
+  <dimension ref="A2:AP52"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="7" style="1" customWidth="1"/>
     <col min="2" max="2" width="17.33203125" style="1" customWidth="1"/>
     <col min="3" max="10" width="8.5" style="1" customWidth="1"/>
-    <col min="11" max="40" width="8.5" customWidth="1"/>
+    <col min="11" max="42" width="8.5" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="2" spans="1:40" x14ac:dyDescent="0.2">
+    <row r="2" spans="1:42" x14ac:dyDescent="0.2">
       <c r="C2" s="6" t="s">
         <v>67</v>
       </c>
@@ -14224,7 +14822,7 @@
         <v>169</v>
       </c>
     </row>
-    <row r="3" spans="1:40" x14ac:dyDescent="0.2">
+    <row r="3" spans="1:42" x14ac:dyDescent="0.2">
       <c r="C3" s="1" t="s">
         <v>66</v>
       </c>
@@ -14247,7 +14845,7 @@
         <v>168</v>
       </c>
     </row>
-    <row r="4" spans="1:40" x14ac:dyDescent="0.2">
+    <row r="4" spans="1:42" x14ac:dyDescent="0.2">
       <c r="C4" s="1" t="s">
         <v>69</v>
       </c>
@@ -14274,7 +14872,7 @@
         <v>204</v>
       </c>
     </row>
-    <row r="5" spans="1:40" x14ac:dyDescent="0.2">
+    <row r="5" spans="1:42" x14ac:dyDescent="0.2">
       <c r="C5" s="1" t="s">
         <v>171</v>
       </c>
@@ -14299,7 +14897,7 @@
         <v>203</v>
       </c>
     </row>
-    <row r="6" spans="1:40" x14ac:dyDescent="0.2">
+    <row r="6" spans="1:42" x14ac:dyDescent="0.2">
       <c r="C6" s="1" t="s">
         <v>201</v>
       </c>
@@ -14319,7 +14917,7 @@
       <c r="AE6" s="1"/>
       <c r="AF6" s="1"/>
     </row>
-    <row r="7" spans="1:40" x14ac:dyDescent="0.2">
+    <row r="7" spans="1:42" x14ac:dyDescent="0.2">
       <c r="C7" s="1" t="s">
         <v>233</v>
       </c>
@@ -14329,53 +14927,55 @@
       <c r="AE7" s="1"/>
       <c r="AF7" s="1"/>
     </row>
-    <row r="9" spans="1:40" x14ac:dyDescent="0.2">
-      <c r="C9" s="51" t="s">
+    <row r="9" spans="1:42" x14ac:dyDescent="0.2">
+      <c r="C9" s="52" t="s">
         <v>236</v>
       </c>
-      <c r="D9" s="51"/>
-      <c r="E9" s="51"/>
-      <c r="F9" s="51"/>
-      <c r="G9" s="51"/>
-      <c r="H9" s="51"/>
-      <c r="I9" s="51"/>
-      <c r="J9" s="51"/>
-      <c r="K9" s="51"/>
-      <c r="L9" s="51"/>
-      <c r="M9" s="51"/>
-      <c r="N9" s="51"/>
-      <c r="O9" s="51"/>
-      <c r="P9" s="51"/>
-      <c r="Q9" s="51"/>
-      <c r="R9" s="51"/>
-      <c r="S9" s="51"/>
-      <c r="T9" s="51"/>
-      <c r="U9" s="51"/>
-      <c r="V9" s="51"/>
-      <c r="W9" s="51"/>
-      <c r="X9" s="51"/>
-      <c r="Y9" s="51"/>
-      <c r="Z9" s="51"/>
-      <c r="AA9" s="51" t="s">
+      <c r="D9" s="52"/>
+      <c r="E9" s="52"/>
+      <c r="F9" s="52"/>
+      <c r="G9" s="52"/>
+      <c r="H9" s="52"/>
+      <c r="I9" s="52"/>
+      <c r="J9" s="52"/>
+      <c r="K9" s="52"/>
+      <c r="L9" s="52"/>
+      <c r="M9" s="52"/>
+      <c r="N9" s="52"/>
+      <c r="O9" s="52"/>
+      <c r="P9" s="52"/>
+      <c r="Q9" s="52"/>
+      <c r="R9" s="52"/>
+      <c r="S9" s="52"/>
+      <c r="T9" s="52"/>
+      <c r="U9" s="52"/>
+      <c r="V9" s="52"/>
+      <c r="W9" s="52"/>
+      <c r="X9" s="52"/>
+      <c r="Y9" s="52"/>
+      <c r="Z9" s="52"/>
+      <c r="AA9" s="52" t="s">
         <v>57</v>
       </c>
-      <c r="AB9" s="51"/>
-      <c r="AC9" s="51"/>
-      <c r="AD9" s="51"/>
-      <c r="AE9" s="51"/>
-      <c r="AF9" s="51"/>
-      <c r="AG9" s="51" t="s">
+      <c r="AB9" s="52"/>
+      <c r="AC9" s="52"/>
+      <c r="AD9" s="52"/>
+      <c r="AE9" s="52"/>
+      <c r="AF9" s="52"/>
+      <c r="AG9" s="52" t="s">
         <v>91</v>
       </c>
-      <c r="AH9" s="51"/>
-      <c r="AI9" s="51"/>
-      <c r="AJ9" s="51"/>
-      <c r="AK9" s="51"/>
-      <c r="AL9" s="51"/>
-      <c r="AM9" s="51"/>
-      <c r="AN9" s="51"/>
-    </row>
-    <row r="10" spans="1:40" ht="18" x14ac:dyDescent="0.25">
+      <c r="AH9" s="52"/>
+      <c r="AI9" s="52"/>
+      <c r="AJ9" s="52"/>
+      <c r="AK9" s="52"/>
+      <c r="AL9" s="52"/>
+      <c r="AM9" s="52"/>
+      <c r="AN9" s="52"/>
+      <c r="AO9" s="52"/>
+      <c r="AP9" s="52"/>
+    </row>
+    <row r="10" spans="1:42" ht="18" x14ac:dyDescent="0.25">
       <c r="A10" s="20" t="s">
         <v>19</v>
       </c>
@@ -14496,8 +15096,14 @@
       <c r="AN10" s="23" t="s">
         <v>98</v>
       </c>
-    </row>
-    <row r="11" spans="1:40" x14ac:dyDescent="0.2">
+      <c r="AO10" s="23" t="s">
+        <v>262</v>
+      </c>
+      <c r="AP10" s="23" t="s">
+        <v>263</v>
+      </c>
+    </row>
+    <row r="11" spans="1:42" x14ac:dyDescent="0.2">
       <c r="A11" s="3">
         <v>1</v>
       </c>
@@ -14540,8 +15146,10 @@
       <c r="AL11" s="3"/>
       <c r="AM11" s="3"/>
       <c r="AN11" s="3"/>
-    </row>
-    <row r="12" spans="1:40" x14ac:dyDescent="0.2">
+      <c r="AO11" s="3"/>
+      <c r="AP11" s="3"/>
+    </row>
+    <row r="12" spans="1:42" x14ac:dyDescent="0.2">
       <c r="A12" s="3">
         <v>2</v>
       </c>
@@ -14584,8 +15192,10 @@
       <c r="AL12" s="3"/>
       <c r="AM12" s="18"/>
       <c r="AN12" s="19"/>
-    </row>
-    <row r="13" spans="1:40" x14ac:dyDescent="0.2">
+      <c r="AO12" s="19"/>
+      <c r="AP12" s="19"/>
+    </row>
+    <row r="13" spans="1:42" x14ac:dyDescent="0.2">
       <c r="A13" s="3">
         <v>3</v>
       </c>
@@ -14628,8 +15238,10 @@
       <c r="AL13" s="3"/>
       <c r="AM13" s="18"/>
       <c r="AN13" s="19"/>
-    </row>
-    <row r="14" spans="1:40" x14ac:dyDescent="0.2">
+      <c r="AO13" s="19"/>
+      <c r="AP13" s="19"/>
+    </row>
+    <row r="14" spans="1:42" x14ac:dyDescent="0.2">
       <c r="A14" s="3">
         <v>4</v>
       </c>
@@ -14672,8 +15284,10 @@
       <c r="AL14" s="3"/>
       <c r="AM14" s="3"/>
       <c r="AN14" s="3"/>
-    </row>
-    <row r="15" spans="1:40" x14ac:dyDescent="0.2">
+      <c r="AO14" s="3"/>
+      <c r="AP14" s="3"/>
+    </row>
+    <row r="15" spans="1:42" x14ac:dyDescent="0.2">
       <c r="A15" s="3">
         <v>5</v>
       </c>
@@ -14716,8 +15330,10 @@
       <c r="AL15" s="3"/>
       <c r="AM15" s="3"/>
       <c r="AN15" s="3"/>
-    </row>
-    <row r="16" spans="1:40" x14ac:dyDescent="0.2">
+      <c r="AO15" s="3"/>
+      <c r="AP15" s="3"/>
+    </row>
+    <row r="16" spans="1:42" x14ac:dyDescent="0.2">
       <c r="A16" s="3">
         <v>6</v>
       </c>
@@ -14760,8 +15376,10 @@
       <c r="AL16" s="3"/>
       <c r="AM16" s="3"/>
       <c r="AN16" s="3"/>
-    </row>
-    <row r="17" spans="1:40" x14ac:dyDescent="0.2">
+      <c r="AO16" s="3"/>
+      <c r="AP16" s="3"/>
+    </row>
+    <row r="17" spans="1:42" x14ac:dyDescent="0.2">
       <c r="A17" s="3">
         <v>7</v>
       </c>
@@ -14804,8 +15422,10 @@
       <c r="AL17" s="3"/>
       <c r="AM17" s="3"/>
       <c r="AN17" s="3"/>
-    </row>
-    <row r="18" spans="1:40" x14ac:dyDescent="0.2">
+      <c r="AO17" s="3"/>
+      <c r="AP17" s="3"/>
+    </row>
+    <row r="18" spans="1:42" x14ac:dyDescent="0.2">
       <c r="A18" s="3">
         <v>8</v>
       </c>
@@ -14848,8 +15468,10 @@
       <c r="AL18" s="3"/>
       <c r="AM18" s="3"/>
       <c r="AN18" s="3"/>
-    </row>
-    <row r="19" spans="1:40" x14ac:dyDescent="0.2">
+      <c r="AO18" s="3"/>
+      <c r="AP18" s="3"/>
+    </row>
+    <row r="19" spans="1:42" x14ac:dyDescent="0.2">
       <c r="A19" s="3">
         <v>9</v>
       </c>
@@ -14892,8 +15514,10 @@
       <c r="AL19" s="3"/>
       <c r="AM19" s="3"/>
       <c r="AN19" s="3"/>
-    </row>
-    <row r="20" spans="1:40" x14ac:dyDescent="0.2">
+      <c r="AO19" s="3"/>
+      <c r="AP19" s="3"/>
+    </row>
+    <row r="20" spans="1:42" x14ac:dyDescent="0.2">
       <c r="A20" s="3">
         <v>10</v>
       </c>
@@ -14936,8 +15560,10 @@
       <c r="AL20" s="3"/>
       <c r="AM20" s="3"/>
       <c r="AN20" s="3"/>
-    </row>
-    <row r="21" spans="1:40" x14ac:dyDescent="0.2">
+      <c r="AO20" s="3"/>
+      <c r="AP20" s="3"/>
+    </row>
+    <row r="21" spans="1:42" x14ac:dyDescent="0.2">
       <c r="A21" s="3">
         <v>11</v>
       </c>
@@ -14980,8 +15606,10 @@
       <c r="AL21" s="3"/>
       <c r="AM21" s="3"/>
       <c r="AN21" s="3"/>
-    </row>
-    <row r="22" spans="1:40" x14ac:dyDescent="0.2">
+      <c r="AO21" s="3"/>
+      <c r="AP21" s="3"/>
+    </row>
+    <row r="22" spans="1:42" x14ac:dyDescent="0.2">
       <c r="A22" s="3">
         <v>12</v>
       </c>
@@ -15024,8 +15652,10 @@
       <c r="AL22" s="3"/>
       <c r="AM22" s="3"/>
       <c r="AN22" s="3"/>
-    </row>
-    <row r="23" spans="1:40" x14ac:dyDescent="0.2">
+      <c r="AO22" s="3"/>
+      <c r="AP22" s="3"/>
+    </row>
+    <row r="23" spans="1:42" x14ac:dyDescent="0.2">
       <c r="A23" s="3">
         <v>13</v>
       </c>
@@ -15068,8 +15698,10 @@
       <c r="AL23" s="3"/>
       <c r="AM23" s="3"/>
       <c r="AN23" s="3"/>
-    </row>
-    <row r="24" spans="1:40" x14ac:dyDescent="0.2">
+      <c r="AO23" s="3"/>
+      <c r="AP23" s="3"/>
+    </row>
+    <row r="24" spans="1:42" x14ac:dyDescent="0.2">
       <c r="A24" s="3">
         <v>14</v>
       </c>
@@ -15112,8 +15744,10 @@
       <c r="AL24" s="3"/>
       <c r="AM24" s="3"/>
       <c r="AN24" s="3"/>
-    </row>
-    <row r="25" spans="1:40" x14ac:dyDescent="0.2">
+      <c r="AO24" s="3"/>
+      <c r="AP24" s="3"/>
+    </row>
+    <row r="25" spans="1:42" x14ac:dyDescent="0.2">
       <c r="A25" s="3">
         <v>15</v>
       </c>
@@ -15156,8 +15790,10 @@
       <c r="AL25" s="3"/>
       <c r="AM25" s="3"/>
       <c r="AN25" s="3"/>
-    </row>
-    <row r="26" spans="1:40" x14ac:dyDescent="0.2">
+      <c r="AO25" s="3"/>
+      <c r="AP25" s="3"/>
+    </row>
+    <row r="26" spans="1:42" x14ac:dyDescent="0.2">
       <c r="K26" s="1"/>
       <c r="L26" s="1"/>
       <c r="M26" s="1"/>
@@ -15188,8 +15824,10 @@
       <c r="AL26" s="1"/>
       <c r="AM26" s="1"/>
       <c r="AN26" s="1"/>
-    </row>
-    <row r="27" spans="1:40" x14ac:dyDescent="0.2">
+      <c r="AO26" s="1"/>
+      <c r="AP26" s="1"/>
+    </row>
+    <row r="27" spans="1:42" x14ac:dyDescent="0.2">
       <c r="K27" s="1"/>
       <c r="L27" s="1"/>
       <c r="M27" s="1"/>
@@ -15213,7 +15851,7 @@
       <c r="AE27" s="1"/>
       <c r="AF27" s="1"/>
     </row>
-    <row r="28" spans="1:40" x14ac:dyDescent="0.2">
+    <row r="28" spans="1:42" x14ac:dyDescent="0.2">
       <c r="K28" s="1"/>
       <c r="L28" s="1"/>
       <c r="M28" s="1"/>
@@ -15237,7 +15875,7 @@
       <c r="AE28" s="1"/>
       <c r="AF28" s="1"/>
     </row>
-    <row r="29" spans="1:40" x14ac:dyDescent="0.2">
+    <row r="29" spans="1:42" x14ac:dyDescent="0.2">
       <c r="K29" s="1"/>
       <c r="L29" s="1"/>
       <c r="M29" s="1"/>
@@ -15261,7 +15899,7 @@
       <c r="AE29" s="1"/>
       <c r="AF29" s="1"/>
     </row>
-    <row r="30" spans="1:40" x14ac:dyDescent="0.2">
+    <row r="30" spans="1:42" x14ac:dyDescent="0.2">
       <c r="K30" s="1"/>
       <c r="L30" s="1"/>
       <c r="M30" s="1"/>
@@ -15285,7 +15923,7 @@
       <c r="AE30" s="1"/>
       <c r="AF30" s="1"/>
     </row>
-    <row r="31" spans="1:40" x14ac:dyDescent="0.2">
+    <row r="31" spans="1:42" x14ac:dyDescent="0.2">
       <c r="K31" s="1"/>
       <c r="L31" s="1"/>
       <c r="M31" s="1"/>
@@ -15309,7 +15947,7 @@
       <c r="AE31" s="1"/>
       <c r="AF31" s="1"/>
     </row>
-    <row r="32" spans="1:40" x14ac:dyDescent="0.2">
+    <row r="32" spans="1:42" x14ac:dyDescent="0.2">
       <c r="K32" s="1"/>
       <c r="L32" s="1"/>
       <c r="M32" s="1"/>
@@ -15816,92 +16454,102 @@
   </sheetData>
   <mergeCells count="3">
     <mergeCell ref="AA9:AF9"/>
-    <mergeCell ref="AG9:AN9"/>
     <mergeCell ref="C9:Z9"/>
+    <mergeCell ref="AG9:AP9"/>
   </mergeCells>
   <conditionalFormatting sqref="F11:K52 AB11:AF52">
-    <cfRule type="expression" dxfId="20" priority="4">
+    <cfRule type="expression" dxfId="22" priority="6">
       <formula>$E11="hb"</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="19" priority="5">
+    <cfRule type="expression" dxfId="21" priority="7">
       <formula>$E11="pow"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="F11:L52">
-    <cfRule type="expression" dxfId="18" priority="17">
+    <cfRule type="expression" dxfId="20" priority="19">
       <formula>$E11="elastic"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="G11:G52">
-    <cfRule type="expression" dxfId="17" priority="6">
+    <cfRule type="expression" dxfId="19" priority="8">
       <formula>$E11="cp"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="H11:I52">
-    <cfRule type="expression" dxfId="16" priority="7">
+    <cfRule type="expression" dxfId="18" priority="9">
       <formula>$E11="mc"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="J11:K52">
-    <cfRule type="expression" dxfId="15" priority="8">
+    <cfRule type="expression" dxfId="17" priority="10">
       <formula>$E11="cp"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="O11:R52">
-    <cfRule type="expression" dxfId="14" priority="2">
+    <cfRule type="expression" dxfId="16" priority="4">
       <formula>$E11="elastic"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="P11:P52">
-    <cfRule type="expression" dxfId="13" priority="11">
+    <cfRule type="expression" dxfId="15" priority="13">
       <formula>AND($O11&lt;&gt;"",$O11&lt;&gt;"ru")</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="Q11:R52">
-    <cfRule type="expression" dxfId="12" priority="1">
+    <cfRule type="expression" dxfId="14" priority="3">
       <formula>$E11="cp"</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="11" priority="3">
+    <cfRule type="expression" dxfId="13" priority="5">
       <formula>AND($O11&lt;&gt;"",$O11&lt;&gt;"piezo",$O11&lt;&gt;"seep")</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="S11:V52">
-    <cfRule type="expression" dxfId="10" priority="9">
+    <cfRule type="expression" dxfId="12" priority="11">
       <formula>AND($E11&lt;&gt;"",$E11&lt;&gt;"pow")</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="W11:Z52">
-    <cfRule type="expression" dxfId="9" priority="10">
+    <cfRule type="expression" dxfId="11" priority="12">
       <formula>AND($E11&lt;&gt;"",$E11&lt;&gt;"hb")</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="AB11:AF52">
-    <cfRule type="expression" dxfId="8" priority="19">
+    <cfRule type="expression" dxfId="10" priority="21">
       <formula>$E11="elastic"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="AC11:AC52">
-    <cfRule type="expression" dxfId="7" priority="12">
+    <cfRule type="expression" dxfId="9" priority="14">
       <formula>$E11="cp"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="AD11:AD52">
-    <cfRule type="expression" dxfId="6" priority="13">
+    <cfRule type="expression" dxfId="8" priority="15">
       <formula>$E11="mc"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="AE11:AF52">
-    <cfRule type="expression" dxfId="5" priority="14">
+    <cfRule type="expression" dxfId="7" priority="16">
       <formula>$E11="cp"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="AK11:AL52">
-    <cfRule type="expression" dxfId="4" priority="15">
+    <cfRule type="expression" dxfId="6" priority="17">
       <formula>OR($AJ11="vg",$AJ11="gard")</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="AM11:AN52">
-    <cfRule type="expression" dxfId="3" priority="16">
+    <cfRule type="expression" dxfId="5" priority="18">
+      <formula>$AJ11="lf"</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="AO11:AO52">
+    <cfRule type="expression" dxfId="1" priority="2">
+      <formula>$AJ11="lf"</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="AP11:AP52">
+    <cfRule type="expression" dxfId="0" priority="1">
       <formula>$AJ11="lf"</formula>
     </cfRule>
   </conditionalFormatting>
@@ -15920,7 +16568,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{6D14E9FA-AFF6-A74D-8120-64FF6A371536}">
   <dimension ref="A2:AR27"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
@@ -15958,74 +16606,74 @@
       </c>
     </row>
     <row r="4" spans="1:44" x14ac:dyDescent="0.2">
-      <c r="A4" s="54" t="s">
+      <c r="A4" s="53" t="s">
         <v>2</v>
       </c>
-      <c r="B4" s="54"/>
-      <c r="D4" s="54" t="s">
+      <c r="B4" s="53"/>
+      <c r="D4" s="53" t="s">
         <v>5</v>
       </c>
-      <c r="E4" s="54"/>
-      <c r="G4" s="54" t="s">
+      <c r="E4" s="53"/>
+      <c r="G4" s="53" t="s">
         <v>6</v>
       </c>
-      <c r="H4" s="54"/>
-      <c r="J4" s="54" t="s">
+      <c r="H4" s="53"/>
+      <c r="J4" s="53" t="s">
         <v>7</v>
       </c>
-      <c r="K4" s="54"/>
-      <c r="M4" s="54" t="s">
+      <c r="K4" s="53"/>
+      <c r="M4" s="53" t="s">
         <v>8</v>
       </c>
-      <c r="N4" s="54"/>
-      <c r="P4" s="54" t="s">
+      <c r="N4" s="53"/>
+      <c r="P4" s="53" t="s">
         <v>9</v>
       </c>
-      <c r="Q4" s="54"/>
+      <c r="Q4" s="53"/>
       <c r="R4" s="1"/>
-      <c r="S4" s="54" t="s">
+      <c r="S4" s="53" t="s">
         <v>10</v>
       </c>
-      <c r="T4" s="54"/>
+      <c r="T4" s="53"/>
       <c r="U4" s="1"/>
-      <c r="V4" s="54" t="s">
+      <c r="V4" s="53" t="s">
         <v>11</v>
       </c>
-      <c r="W4" s="54"/>
+      <c r="W4" s="53"/>
       <c r="X4" s="1"/>
-      <c r="Y4" s="54" t="s">
+      <c r="Y4" s="53" t="s">
         <v>12</v>
       </c>
-      <c r="Z4" s="54"/>
+      <c r="Z4" s="53"/>
       <c r="AA4" s="1"/>
-      <c r="AB4" s="54" t="s">
+      <c r="AB4" s="53" t="s">
         <v>13</v>
       </c>
-      <c r="AC4" s="54"/>
-      <c r="AE4" s="54" t="s">
+      <c r="AC4" s="53"/>
+      <c r="AE4" s="53" t="s">
         <v>108</v>
       </c>
-      <c r="AF4" s="54"/>
+      <c r="AF4" s="53"/>
       <c r="AG4" s="1"/>
-      <c r="AH4" s="54" t="s">
+      <c r="AH4" s="53" t="s">
         <v>109</v>
       </c>
-      <c r="AI4" s="54"/>
+      <c r="AI4" s="53"/>
       <c r="AJ4" s="1"/>
-      <c r="AK4" s="54" t="s">
+      <c r="AK4" s="53" t="s">
         <v>110</v>
       </c>
-      <c r="AL4" s="54"/>
+      <c r="AL4" s="53"/>
       <c r="AM4" s="1"/>
-      <c r="AN4" s="54" t="s">
+      <c r="AN4" s="53" t="s">
         <v>111</v>
       </c>
-      <c r="AO4" s="54"/>
+      <c r="AO4" s="53"/>
       <c r="AP4" s="1"/>
-      <c r="AQ4" s="54" t="s">
+      <c r="AQ4" s="53" t="s">
         <v>112</v>
       </c>
-      <c r="AR4" s="54"/>
+      <c r="AR4" s="53"/>
     </row>
     <row r="5" spans="1:44" x14ac:dyDescent="0.2">
       <c r="A5" s="36" t="s">
@@ -16128,89 +16776,89 @@
       </c>
     </row>
     <row r="6" spans="1:44" x14ac:dyDescent="0.2">
-      <c r="A6" s="52" t="str">
+      <c r="A6" s="54" t="str">
         <f>_xlfn.XLOOKUP(B5,mat!$A:$A, mat!$B:$B,"") &amp; ""</f>
         <v/>
       </c>
-      <c r="B6" s="53"/>
-      <c r="D6" s="52" t="str">
+      <c r="B6" s="55"/>
+      <c r="D6" s="54" t="str">
         <f>_xlfn.XLOOKUP(E5,mat!$A:$A, mat!$B:$B,"") &amp; ""</f>
         <v/>
       </c>
-      <c r="E6" s="53"/>
-      <c r="G6" s="52" t="str">
+      <c r="E6" s="55"/>
+      <c r="G6" s="54" t="str">
         <f>_xlfn.XLOOKUP(H5,mat!$A:$A, mat!$B:$B,"") &amp; ""</f>
         <v/>
       </c>
-      <c r="H6" s="53"/>
-      <c r="J6" s="52" t="str">
+      <c r="H6" s="55"/>
+      <c r="J6" s="54" t="str">
         <f>_xlfn.XLOOKUP(K5,mat!$A:$A, mat!$B:$B,"") &amp; ""</f>
         <v/>
       </c>
-      <c r="K6" s="53"/>
-      <c r="M6" s="52" t="str">
+      <c r="K6" s="55"/>
+      <c r="M6" s="54" t="str">
         <f>_xlfn.XLOOKUP(N5,mat!$A:$A, mat!$B:$B,"") &amp; ""</f>
         <v/>
       </c>
-      <c r="N6" s="53"/>
-      <c r="P6" s="52" t="str">
+      <c r="N6" s="55"/>
+      <c r="P6" s="54" t="str">
         <f>_xlfn.XLOOKUP(Q5,mat!$A:$A, mat!$B:$B,"") &amp; ""</f>
         <v/>
       </c>
-      <c r="Q6" s="53"/>
+      <c r="Q6" s="55"/>
       <c r="R6" s="1"/>
-      <c r="S6" s="52" t="str">
+      <c r="S6" s="54" t="str">
         <f>_xlfn.XLOOKUP(T5,mat!$A:$A, mat!$B:$B,"") &amp; ""</f>
         <v/>
       </c>
-      <c r="T6" s="53"/>
+      <c r="T6" s="55"/>
       <c r="U6" s="1"/>
-      <c r="V6" s="52" t="str">
+      <c r="V6" s="54" t="str">
         <f>_xlfn.XLOOKUP(W5,mat!$A:$A, mat!$B:$B,"") &amp; ""</f>
         <v/>
       </c>
-      <c r="W6" s="53"/>
+      <c r="W6" s="55"/>
       <c r="X6" s="1"/>
-      <c r="Y6" s="52" t="str">
+      <c r="Y6" s="54" t="str">
         <f>_xlfn.XLOOKUP(Z5,mat!$A:$A, mat!$B:$B,"") &amp; ""</f>
         <v/>
       </c>
-      <c r="Z6" s="53"/>
+      <c r="Z6" s="55"/>
       <c r="AA6" s="1"/>
-      <c r="AB6" s="52" t="str">
+      <c r="AB6" s="54" t="str">
         <f>_xlfn.XLOOKUP(AC5,mat!$A:$A, mat!$B:$B,"") &amp; ""</f>
         <v/>
       </c>
-      <c r="AC6" s="53"/>
-      <c r="AE6" s="52" t="str">
+      <c r="AC6" s="55"/>
+      <c r="AE6" s="54" t="str">
         <f>_xlfn.XLOOKUP(AF5,mat!$A:$A, mat!$B:$B,"") &amp; ""</f>
         <v/>
       </c>
-      <c r="AF6" s="53"/>
+      <c r="AF6" s="55"/>
       <c r="AG6" s="1"/>
-      <c r="AH6" s="52" t="str">
+      <c r="AH6" s="54" t="str">
         <f>_xlfn.XLOOKUP(AI5,mat!$A:$A, mat!$B:$B,"") &amp; ""</f>
         <v/>
       </c>
-      <c r="AI6" s="53"/>
+      <c r="AI6" s="55"/>
       <c r="AJ6" s="1"/>
-      <c r="AK6" s="52" t="str">
+      <c r="AK6" s="54" t="str">
         <f>_xlfn.XLOOKUP(AL5,mat!$A:$A, mat!$B:$B,"") &amp; ""</f>
         <v/>
       </c>
-      <c r="AL6" s="53"/>
+      <c r="AL6" s="55"/>
       <c r="AM6" s="1"/>
-      <c r="AN6" s="52" t="str">
+      <c r="AN6" s="54" t="str">
         <f>_xlfn.XLOOKUP(AO5,mat!$A:$A, mat!$B:$B,"") &amp; ""</f>
         <v/>
       </c>
-      <c r="AO6" s="53"/>
+      <c r="AO6" s="55"/>
       <c r="AP6" s="1"/>
-      <c r="AQ6" s="52" t="str">
+      <c r="AQ6" s="54" t="str">
         <f>_xlfn.XLOOKUP(AR5,mat!$A:$A, mat!$B:$B,"") &amp; ""</f>
         <v/>
       </c>
-      <c r="AR6" s="53"/>
+      <c r="AR6" s="55"/>
     </row>
     <row r="7" spans="1:44" x14ac:dyDescent="0.2">
       <c r="A7" s="2" t="s">
@@ -17114,42 +17762,42 @@
     </row>
   </sheetData>
   <mergeCells count="30">
+    <mergeCell ref="AE6:AF6"/>
+    <mergeCell ref="AH6:AI6"/>
+    <mergeCell ref="AK6:AL6"/>
+    <mergeCell ref="AN6:AO6"/>
+    <mergeCell ref="AQ6:AR6"/>
+    <mergeCell ref="P6:Q6"/>
+    <mergeCell ref="S6:T6"/>
+    <mergeCell ref="V6:W6"/>
+    <mergeCell ref="Y6:Z6"/>
+    <mergeCell ref="AB6:AC6"/>
+    <mergeCell ref="A6:B6"/>
+    <mergeCell ref="D6:E6"/>
+    <mergeCell ref="G6:H6"/>
+    <mergeCell ref="J6:K6"/>
+    <mergeCell ref="M6:N6"/>
+    <mergeCell ref="AE4:AF4"/>
+    <mergeCell ref="AH4:AI4"/>
+    <mergeCell ref="AK4:AL4"/>
+    <mergeCell ref="AN4:AO4"/>
+    <mergeCell ref="AQ4:AR4"/>
+    <mergeCell ref="P4:Q4"/>
+    <mergeCell ref="S4:T4"/>
+    <mergeCell ref="V4:W4"/>
+    <mergeCell ref="Y4:Z4"/>
+    <mergeCell ref="AB4:AC4"/>
     <mergeCell ref="A4:B4"/>
     <mergeCell ref="D4:E4"/>
     <mergeCell ref="G4:H4"/>
     <mergeCell ref="J4:K4"/>
     <mergeCell ref="M4:N4"/>
-    <mergeCell ref="P4:Q4"/>
-    <mergeCell ref="S4:T4"/>
-    <mergeCell ref="V4:W4"/>
-    <mergeCell ref="Y4:Z4"/>
-    <mergeCell ref="AB4:AC4"/>
-    <mergeCell ref="AE4:AF4"/>
-    <mergeCell ref="AH4:AI4"/>
-    <mergeCell ref="AK4:AL4"/>
-    <mergeCell ref="AN4:AO4"/>
-    <mergeCell ref="AQ4:AR4"/>
-    <mergeCell ref="A6:B6"/>
-    <mergeCell ref="D6:E6"/>
-    <mergeCell ref="G6:H6"/>
-    <mergeCell ref="J6:K6"/>
-    <mergeCell ref="M6:N6"/>
-    <mergeCell ref="P6:Q6"/>
-    <mergeCell ref="S6:T6"/>
-    <mergeCell ref="V6:W6"/>
-    <mergeCell ref="Y6:Z6"/>
-    <mergeCell ref="AB6:AC6"/>
-    <mergeCell ref="AE6:AF6"/>
-    <mergeCell ref="AH6:AI6"/>
-    <mergeCell ref="AK6:AL6"/>
-    <mergeCell ref="AN6:AO6"/>
-    <mergeCell ref="AQ6:AR6"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{88992C43-9D03-6445-8931-028E950C2356}">
   <dimension ref="A2:AR27"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
@@ -17181,74 +17829,74 @@
       </c>
     </row>
     <row r="4" spans="1:44" x14ac:dyDescent="0.2">
-      <c r="A4" s="54" t="s">
+      <c r="A4" s="53" t="s">
         <v>137</v>
       </c>
-      <c r="B4" s="54"/>
-      <c r="D4" s="54" t="s">
+      <c r="B4" s="53"/>
+      <c r="D4" s="53" t="s">
         <v>138</v>
       </c>
-      <c r="E4" s="54"/>
-      <c r="G4" s="54" t="s">
+      <c r="E4" s="53"/>
+      <c r="G4" s="53" t="s">
         <v>139</v>
       </c>
-      <c r="H4" s="54"/>
-      <c r="J4" s="54" t="s">
+      <c r="H4" s="53"/>
+      <c r="J4" s="53" t="s">
         <v>140</v>
       </c>
-      <c r="K4" s="54"/>
-      <c r="M4" s="54" t="s">
+      <c r="K4" s="53"/>
+      <c r="M4" s="53" t="s">
         <v>141</v>
       </c>
-      <c r="N4" s="54"/>
-      <c r="P4" s="54" t="s">
+      <c r="N4" s="53"/>
+      <c r="P4" s="53" t="s">
         <v>142</v>
       </c>
-      <c r="Q4" s="54"/>
+      <c r="Q4" s="53"/>
       <c r="R4" s="1"/>
-      <c r="S4" s="54" t="s">
+      <c r="S4" s="53" t="s">
         <v>143</v>
       </c>
-      <c r="T4" s="54"/>
+      <c r="T4" s="53"/>
       <c r="U4" s="1"/>
-      <c r="V4" s="54" t="s">
+      <c r="V4" s="53" t="s">
         <v>144</v>
       </c>
-      <c r="W4" s="54"/>
+      <c r="W4" s="53"/>
       <c r="X4" s="1"/>
-      <c r="Y4" s="54" t="s">
+      <c r="Y4" s="53" t="s">
         <v>145</v>
       </c>
-      <c r="Z4" s="54"/>
+      <c r="Z4" s="53"/>
       <c r="AA4" s="1"/>
-      <c r="AB4" s="54" t="s">
+      <c r="AB4" s="53" t="s">
         <v>146</v>
       </c>
-      <c r="AC4" s="54"/>
-      <c r="AE4" s="54" t="s">
+      <c r="AC4" s="53"/>
+      <c r="AE4" s="53" t="s">
         <v>147</v>
       </c>
-      <c r="AF4" s="54"/>
+      <c r="AF4" s="53"/>
       <c r="AG4" s="1"/>
-      <c r="AH4" s="54" t="s">
+      <c r="AH4" s="53" t="s">
         <v>148</v>
       </c>
-      <c r="AI4" s="54"/>
+      <c r="AI4" s="53"/>
       <c r="AJ4" s="1"/>
-      <c r="AK4" s="54" t="s">
+      <c r="AK4" s="53" t="s">
         <v>149</v>
       </c>
-      <c r="AL4" s="54"/>
+      <c r="AL4" s="53"/>
       <c r="AM4" s="1"/>
-      <c r="AN4" s="54" t="s">
+      <c r="AN4" s="53" t="s">
         <v>150</v>
       </c>
-      <c r="AO4" s="54"/>
+      <c r="AO4" s="53"/>
       <c r="AP4" s="1"/>
-      <c r="AQ4" s="54" t="s">
+      <c r="AQ4" s="53" t="s">
         <v>151</v>
       </c>
-      <c r="AR4" s="54"/>
+      <c r="AR4" s="53"/>
     </row>
     <row r="5" spans="1:44" x14ac:dyDescent="0.2">
       <c r="A5" s="38" t="s">
@@ -17351,89 +17999,89 @@
       </c>
     </row>
     <row r="6" spans="1:44" x14ac:dyDescent="0.2">
-      <c r="A6" s="55" t="str">
+      <c r="A6" s="56" t="str">
         <f>_xlfn.XLOOKUP(B5,mat!$A:$A, mat!$B:$B,"") &amp; ""</f>
         <v/>
       </c>
-      <c r="B6" s="56"/>
-      <c r="D6" s="55" t="str">
+      <c r="B6" s="57"/>
+      <c r="D6" s="56" t="str">
         <f>_xlfn.XLOOKUP(E5,mat!$A:$A, mat!$B:$B,"") &amp; ""</f>
         <v/>
       </c>
-      <c r="E6" s="56"/>
-      <c r="G6" s="55" t="str">
+      <c r="E6" s="57"/>
+      <c r="G6" s="56" t="str">
         <f>_xlfn.XLOOKUP(H5,mat!$A:$A, mat!$B:$B,"") &amp; ""</f>
         <v/>
       </c>
-      <c r="H6" s="56"/>
-      <c r="J6" s="55" t="str">
+      <c r="H6" s="57"/>
+      <c r="J6" s="56" t="str">
         <f>_xlfn.XLOOKUP(K5,mat!$A:$A, mat!$B:$B,"") &amp; ""</f>
         <v/>
       </c>
-      <c r="K6" s="56"/>
-      <c r="M6" s="55" t="str">
+      <c r="K6" s="57"/>
+      <c r="M6" s="56" t="str">
         <f>_xlfn.XLOOKUP(N5,mat!$A:$A, mat!$B:$B,"") &amp; ""</f>
         <v/>
       </c>
-      <c r="N6" s="56"/>
-      <c r="P6" s="55" t="str">
+      <c r="N6" s="57"/>
+      <c r="P6" s="56" t="str">
         <f>_xlfn.XLOOKUP(Q5,mat!$A:$A, mat!$B:$B,"") &amp; ""</f>
         <v/>
       </c>
-      <c r="Q6" s="56"/>
+      <c r="Q6" s="57"/>
       <c r="R6" s="1"/>
-      <c r="S6" s="55" t="str">
+      <c r="S6" s="56" t="str">
         <f>_xlfn.XLOOKUP(T5,mat!$A:$A, mat!$B:$B,"") &amp; ""</f>
         <v/>
       </c>
-      <c r="T6" s="56"/>
+      <c r="T6" s="57"/>
       <c r="U6" s="1"/>
-      <c r="V6" s="55" t="str">
+      <c r="V6" s="56" t="str">
         <f>_xlfn.XLOOKUP(W5,mat!$A:$A, mat!$B:$B,"") &amp; ""</f>
         <v/>
       </c>
-      <c r="W6" s="56"/>
+      <c r="W6" s="57"/>
       <c r="X6" s="1"/>
-      <c r="Y6" s="55" t="str">
+      <c r="Y6" s="56" t="str">
         <f>_xlfn.XLOOKUP(Z5,mat!$A:$A, mat!$B:$B,"") &amp; ""</f>
         <v/>
       </c>
-      <c r="Z6" s="56"/>
+      <c r="Z6" s="57"/>
       <c r="AA6" s="1"/>
-      <c r="AB6" s="55" t="str">
+      <c r="AB6" s="56" t="str">
         <f>_xlfn.XLOOKUP(AC5,mat!$A:$A, mat!$B:$B,"") &amp; ""</f>
         <v/>
       </c>
-      <c r="AC6" s="56"/>
-      <c r="AE6" s="55" t="str">
+      <c r="AC6" s="57"/>
+      <c r="AE6" s="56" t="str">
         <f>_xlfn.XLOOKUP(AF5,mat!$A:$A, mat!$B:$B,"") &amp; ""</f>
         <v/>
       </c>
-      <c r="AF6" s="56"/>
+      <c r="AF6" s="57"/>
       <c r="AG6" s="1"/>
-      <c r="AH6" s="55" t="str">
+      <c r="AH6" s="56" t="str">
         <f>_xlfn.XLOOKUP(AI5,mat!$A:$A, mat!$B:$B,"") &amp; ""</f>
         <v/>
       </c>
-      <c r="AI6" s="56"/>
+      <c r="AI6" s="57"/>
       <c r="AJ6" s="1"/>
-      <c r="AK6" s="55" t="str">
+      <c r="AK6" s="56" t="str">
         <f>_xlfn.XLOOKUP(AL5,mat!$A:$A, mat!$B:$B,"") &amp; ""</f>
         <v/>
       </c>
-      <c r="AL6" s="56"/>
+      <c r="AL6" s="57"/>
       <c r="AM6" s="1"/>
-      <c r="AN6" s="55" t="str">
+      <c r="AN6" s="56" t="str">
         <f>_xlfn.XLOOKUP(AO5,mat!$A:$A, mat!$B:$B,"") &amp; ""</f>
         <v/>
       </c>
-      <c r="AO6" s="56"/>
+      <c r="AO6" s="57"/>
       <c r="AP6" s="1"/>
-      <c r="AQ6" s="55" t="str">
+      <c r="AQ6" s="56" t="str">
         <f>_xlfn.XLOOKUP(AR5,mat!$A:$A, mat!$B:$B,"") &amp; ""</f>
         <v/>
       </c>
-      <c r="AR6" s="56"/>
+      <c r="AR6" s="57"/>
     </row>
     <row r="7" spans="1:44" x14ac:dyDescent="0.2">
       <c r="A7" s="2" t="s">
@@ -18337,12 +18985,14 @@
     </row>
   </sheetData>
   <mergeCells count="30">
-    <mergeCell ref="P4:Q4"/>
-    <mergeCell ref="A4:B4"/>
-    <mergeCell ref="D4:E4"/>
-    <mergeCell ref="G4:H4"/>
-    <mergeCell ref="J4:K4"/>
-    <mergeCell ref="M4:N4"/>
+    <mergeCell ref="AN6:AO6"/>
+    <mergeCell ref="AQ6:AR6"/>
+    <mergeCell ref="V6:W6"/>
+    <mergeCell ref="Y6:Z6"/>
+    <mergeCell ref="AB6:AC6"/>
+    <mergeCell ref="AE6:AF6"/>
+    <mergeCell ref="AH6:AI6"/>
+    <mergeCell ref="AK6:AL6"/>
     <mergeCell ref="AK4:AL4"/>
     <mergeCell ref="AN4:AO4"/>
     <mergeCell ref="AQ4:AR4"/>
@@ -18359,20 +19009,18 @@
     <mergeCell ref="AB4:AC4"/>
     <mergeCell ref="AE4:AF4"/>
     <mergeCell ref="AH4:AI4"/>
-    <mergeCell ref="AN6:AO6"/>
-    <mergeCell ref="AQ6:AR6"/>
-    <mergeCell ref="V6:W6"/>
-    <mergeCell ref="Y6:Z6"/>
-    <mergeCell ref="AB6:AC6"/>
-    <mergeCell ref="AE6:AF6"/>
-    <mergeCell ref="AH6:AI6"/>
-    <mergeCell ref="AK6:AL6"/>
+    <mergeCell ref="P4:Q4"/>
+    <mergeCell ref="A4:B4"/>
+    <mergeCell ref="D4:E4"/>
+    <mergeCell ref="G4:H4"/>
+    <mergeCell ref="J4:K4"/>
+    <mergeCell ref="M4:N4"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A7E1F343-68A5-3340-AF23-43D8E7E1F914}">
   <dimension ref="A2:H24"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
@@ -18382,14 +19030,14 @@
   </cols>
   <sheetData>
     <row r="2" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A2" s="57" t="s">
+      <c r="A2" s="58" t="s">
         <v>83</v>
       </c>
-      <c r="B2" s="57"/>
-      <c r="D2" s="58" t="s">
+      <c r="B2" s="58"/>
+      <c r="D2" s="59" t="s">
         <v>81</v>
       </c>
-      <c r="E2" s="58"/>
+      <c r="E2" s="59"/>
       <c r="G2" s="22" t="s">
         <v>82</v>
       </c>
@@ -18569,7 +19217,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{9E0556E9-786A-E84F-BF20-677A5EE9D63D}">
   <dimension ref="A2:N16"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
@@ -18757,17 +19405,17 @@
     </row>
   </sheetData>
   <conditionalFormatting sqref="E3:E42">
-    <cfRule type="expression" dxfId="2" priority="3">
+    <cfRule type="expression" dxfId="4" priority="3">
       <formula>OR($D3="Intercept", $D3="Radius")</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="F3:G42">
-    <cfRule type="expression" dxfId="1" priority="2">
+    <cfRule type="expression" dxfId="3" priority="2">
       <formula>OR($D3="Depth",$D3="Radius")</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="H3:H42">
-    <cfRule type="expression" dxfId="0" priority="1">
+    <cfRule type="expression" dxfId="2" priority="1">
       <formula>OR($D3="Depth",$D3="Intercept")</formula>
     </cfRule>
   </conditionalFormatting>
@@ -18780,7 +19428,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{6620242D-B699-0640-AD9C-590D8F82AC0F}">
   <dimension ref="A2:F23"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
@@ -18938,4 +19586,504 @@
   </dataValidations>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{8D19B78E-FBCC-4E41-BB37-C8D0D27B23E8}">
+  <dimension ref="B2:X22"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
+  <cols>
+    <col min="1" max="1" width="3" customWidth="1"/>
+    <col min="2" max="4" width="7.6640625" customWidth="1"/>
+    <col min="5" max="5" width="3" customWidth="1"/>
+    <col min="6" max="8" width="7.6640625" customWidth="1"/>
+    <col min="9" max="9" width="3" customWidth="1"/>
+    <col min="10" max="12" width="7.6640625" customWidth="1"/>
+    <col min="13" max="13" width="3" customWidth="1"/>
+    <col min="14" max="16" width="7.6640625" customWidth="1"/>
+    <col min="17" max="17" width="3" customWidth="1"/>
+    <col min="18" max="20" width="7.6640625" customWidth="1"/>
+    <col min="21" max="21" width="3" customWidth="1"/>
+    <col min="22" max="24" width="7.6640625" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="2" spans="2:24" x14ac:dyDescent="0.2">
+      <c r="B2" s="60" t="s">
+        <v>121</v>
+      </c>
+      <c r="C2" s="60"/>
+      <c r="D2" s="60"/>
+      <c r="F2" s="60" t="s">
+        <v>122</v>
+      </c>
+      <c r="G2" s="60"/>
+      <c r="H2" s="60"/>
+      <c r="J2" s="60" t="s">
+        <v>123</v>
+      </c>
+      <c r="K2" s="60"/>
+      <c r="L2" s="60"/>
+      <c r="N2" s="60" t="s">
+        <v>124</v>
+      </c>
+      <c r="O2" s="60"/>
+      <c r="P2" s="60"/>
+      <c r="R2" s="60" t="s">
+        <v>125</v>
+      </c>
+      <c r="S2" s="60"/>
+      <c r="T2" s="60"/>
+      <c r="V2" s="60" t="s">
+        <v>126</v>
+      </c>
+      <c r="W2" s="60"/>
+      <c r="X2" s="60"/>
+    </row>
+    <row r="3" spans="2:24" x14ac:dyDescent="0.2">
+      <c r="B3" s="2" t="s">
+        <v>0</v>
+      </c>
+      <c r="C3" s="2" t="s">
+        <v>1</v>
+      </c>
+      <c r="D3" s="2" t="s">
+        <v>45</v>
+      </c>
+      <c r="F3" s="2" t="s">
+        <v>0</v>
+      </c>
+      <c r="G3" s="2" t="s">
+        <v>1</v>
+      </c>
+      <c r="H3" s="2" t="s">
+        <v>45</v>
+      </c>
+      <c r="J3" s="2" t="s">
+        <v>0</v>
+      </c>
+      <c r="K3" s="2" t="s">
+        <v>1</v>
+      </c>
+      <c r="L3" s="2" t="s">
+        <v>45</v>
+      </c>
+      <c r="N3" s="2" t="s">
+        <v>0</v>
+      </c>
+      <c r="O3" s="2" t="s">
+        <v>1</v>
+      </c>
+      <c r="P3" s="2" t="s">
+        <v>45</v>
+      </c>
+      <c r="R3" s="2" t="s">
+        <v>0</v>
+      </c>
+      <c r="S3" s="2" t="s">
+        <v>1</v>
+      </c>
+      <c r="T3" s="2" t="s">
+        <v>45</v>
+      </c>
+      <c r="V3" s="2" t="s">
+        <v>0</v>
+      </c>
+      <c r="W3" s="2" t="s">
+        <v>1</v>
+      </c>
+      <c r="X3" s="2" t="s">
+        <v>45</v>
+      </c>
+    </row>
+    <row r="4" spans="2:24" x14ac:dyDescent="0.2">
+      <c r="B4" s="3"/>
+      <c r="C4" s="3"/>
+      <c r="D4" s="3"/>
+      <c r="F4" s="3"/>
+      <c r="G4" s="3"/>
+      <c r="H4" s="3"/>
+      <c r="J4" s="3"/>
+      <c r="K4" s="3"/>
+      <c r="L4" s="3"/>
+      <c r="N4" s="3"/>
+      <c r="O4" s="3"/>
+      <c r="P4" s="3"/>
+      <c r="R4" s="3"/>
+      <c r="S4" s="3"/>
+      <c r="T4" s="3"/>
+      <c r="V4" s="3"/>
+      <c r="W4" s="3"/>
+      <c r="X4" s="3"/>
+    </row>
+    <row r="5" spans="2:24" x14ac:dyDescent="0.2">
+      <c r="B5" s="3"/>
+      <c r="C5" s="3"/>
+      <c r="D5" s="3"/>
+      <c r="F5" s="3"/>
+      <c r="G5" s="3"/>
+      <c r="H5" s="3"/>
+      <c r="J5" s="3"/>
+      <c r="K5" s="3"/>
+      <c r="L5" s="3"/>
+      <c r="N5" s="3"/>
+      <c r="O5" s="3"/>
+      <c r="P5" s="3"/>
+      <c r="R5" s="3"/>
+      <c r="S5" s="3"/>
+      <c r="T5" s="3"/>
+      <c r="V5" s="3"/>
+      <c r="W5" s="3"/>
+      <c r="X5" s="3"/>
+    </row>
+    <row r="6" spans="2:24" x14ac:dyDescent="0.2">
+      <c r="B6" s="3"/>
+      <c r="C6" s="3"/>
+      <c r="D6" s="3"/>
+      <c r="F6" s="3"/>
+      <c r="G6" s="3"/>
+      <c r="H6" s="3"/>
+      <c r="J6" s="3"/>
+      <c r="K6" s="3"/>
+      <c r="L6" s="3"/>
+      <c r="N6" s="3"/>
+      <c r="O6" s="3"/>
+      <c r="P6" s="3"/>
+      <c r="R6" s="3"/>
+      <c r="S6" s="3"/>
+      <c r="T6" s="3"/>
+      <c r="V6" s="3"/>
+      <c r="W6" s="3"/>
+      <c r="X6" s="3"/>
+    </row>
+    <row r="7" spans="2:24" x14ac:dyDescent="0.2">
+      <c r="B7" s="3"/>
+      <c r="C7" s="3"/>
+      <c r="D7" s="3"/>
+      <c r="F7" s="3"/>
+      <c r="G7" s="3"/>
+      <c r="H7" s="3"/>
+      <c r="J7" s="3"/>
+      <c r="K7" s="3"/>
+      <c r="L7" s="3"/>
+      <c r="N7" s="3"/>
+      <c r="O7" s="3"/>
+      <c r="P7" s="3"/>
+      <c r="R7" s="3"/>
+      <c r="S7" s="3"/>
+      <c r="T7" s="3"/>
+      <c r="V7" s="3"/>
+      <c r="W7" s="3"/>
+      <c r="X7" s="3"/>
+    </row>
+    <row r="8" spans="2:24" x14ac:dyDescent="0.2">
+      <c r="B8" s="3"/>
+      <c r="C8" s="3"/>
+      <c r="D8" s="3"/>
+      <c r="F8" s="3"/>
+      <c r="G8" s="3"/>
+      <c r="H8" s="3"/>
+      <c r="J8" s="3"/>
+      <c r="K8" s="3"/>
+      <c r="L8" s="3"/>
+      <c r="N8" s="3"/>
+      <c r="O8" s="3"/>
+      <c r="P8" s="3"/>
+      <c r="R8" s="3"/>
+      <c r="S8" s="3"/>
+      <c r="T8" s="3"/>
+      <c r="V8" s="3"/>
+      <c r="W8" s="3"/>
+      <c r="X8" s="3"/>
+    </row>
+    <row r="9" spans="2:24" x14ac:dyDescent="0.2">
+      <c r="B9" s="3"/>
+      <c r="C9" s="3"/>
+      <c r="D9" s="3"/>
+      <c r="F9" s="3"/>
+      <c r="G9" s="3"/>
+      <c r="H9" s="3"/>
+      <c r="J9" s="3"/>
+      <c r="K9" s="3"/>
+      <c r="L9" s="3"/>
+      <c r="N9" s="3"/>
+      <c r="O9" s="3"/>
+      <c r="P9" s="3"/>
+      <c r="R9" s="3"/>
+      <c r="S9" s="3"/>
+      <c r="T9" s="3"/>
+      <c r="V9" s="3"/>
+      <c r="W9" s="3"/>
+      <c r="X9" s="3"/>
+    </row>
+    <row r="10" spans="2:24" x14ac:dyDescent="0.2">
+      <c r="B10" s="3"/>
+      <c r="C10" s="3"/>
+      <c r="D10" s="3"/>
+      <c r="F10" s="3"/>
+      <c r="G10" s="3"/>
+      <c r="H10" s="3"/>
+      <c r="J10" s="3"/>
+      <c r="K10" s="3"/>
+      <c r="L10" s="3"/>
+      <c r="N10" s="3"/>
+      <c r="O10" s="3"/>
+      <c r="P10" s="3"/>
+      <c r="R10" s="3"/>
+      <c r="S10" s="3"/>
+      <c r="T10" s="3"/>
+      <c r="V10" s="3"/>
+      <c r="W10" s="3"/>
+      <c r="X10" s="3"/>
+    </row>
+    <row r="11" spans="2:24" x14ac:dyDescent="0.2">
+      <c r="B11" s="3"/>
+      <c r="C11" s="3"/>
+      <c r="D11" s="3"/>
+      <c r="F11" s="3"/>
+      <c r="G11" s="3"/>
+      <c r="H11" s="3"/>
+      <c r="J11" s="3"/>
+      <c r="K11" s="3"/>
+      <c r="L11" s="3"/>
+      <c r="N11" s="3"/>
+      <c r="O11" s="3"/>
+      <c r="P11" s="3"/>
+      <c r="R11" s="3"/>
+      <c r="S11" s="3"/>
+      <c r="T11" s="3"/>
+      <c r="V11" s="3"/>
+      <c r="W11" s="3"/>
+      <c r="X11" s="3"/>
+    </row>
+    <row r="12" spans="2:24" x14ac:dyDescent="0.2">
+      <c r="B12" s="3"/>
+      <c r="C12" s="3"/>
+      <c r="D12" s="3"/>
+      <c r="F12" s="3"/>
+      <c r="G12" s="3"/>
+      <c r="H12" s="3"/>
+      <c r="J12" s="3"/>
+      <c r="K12" s="3"/>
+      <c r="L12" s="3"/>
+      <c r="N12" s="3"/>
+      <c r="O12" s="3"/>
+      <c r="P12" s="3"/>
+      <c r="R12" s="3"/>
+      <c r="S12" s="3"/>
+      <c r="T12" s="3"/>
+      <c r="V12" s="3"/>
+      <c r="W12" s="3"/>
+      <c r="X12" s="3"/>
+    </row>
+    <row r="13" spans="2:24" x14ac:dyDescent="0.2">
+      <c r="B13" s="3"/>
+      <c r="C13" s="3"/>
+      <c r="D13" s="3"/>
+      <c r="F13" s="3"/>
+      <c r="G13" s="3"/>
+      <c r="H13" s="3"/>
+      <c r="J13" s="3"/>
+      <c r="K13" s="3"/>
+      <c r="L13" s="3"/>
+      <c r="N13" s="3"/>
+      <c r="O13" s="3"/>
+      <c r="P13" s="3"/>
+      <c r="R13" s="3"/>
+      <c r="S13" s="3"/>
+      <c r="T13" s="3"/>
+      <c r="V13" s="3"/>
+      <c r="W13" s="3"/>
+      <c r="X13" s="3"/>
+    </row>
+    <row r="14" spans="2:24" x14ac:dyDescent="0.2">
+      <c r="B14" s="3"/>
+      <c r="C14" s="3"/>
+      <c r="D14" s="3"/>
+      <c r="F14" s="3"/>
+      <c r="G14" s="3"/>
+      <c r="H14" s="3"/>
+      <c r="J14" s="3"/>
+      <c r="K14" s="3"/>
+      <c r="L14" s="3"/>
+      <c r="N14" s="3"/>
+      <c r="O14" s="3"/>
+      <c r="P14" s="3"/>
+      <c r="R14" s="3"/>
+      <c r="S14" s="3"/>
+      <c r="T14" s="3"/>
+      <c r="V14" s="3"/>
+      <c r="W14" s="3"/>
+      <c r="X14" s="3"/>
+    </row>
+    <row r="15" spans="2:24" x14ac:dyDescent="0.2">
+      <c r="B15" s="3"/>
+      <c r="C15" s="3"/>
+      <c r="D15" s="3"/>
+      <c r="F15" s="3"/>
+      <c r="G15" s="3"/>
+      <c r="H15" s="3"/>
+      <c r="J15" s="3"/>
+      <c r="K15" s="3"/>
+      <c r="L15" s="3"/>
+      <c r="N15" s="3"/>
+      <c r="O15" s="3"/>
+      <c r="P15" s="3"/>
+      <c r="R15" s="3"/>
+      <c r="S15" s="3"/>
+      <c r="T15" s="3"/>
+      <c r="V15" s="3"/>
+      <c r="W15" s="3"/>
+      <c r="X15" s="3"/>
+    </row>
+    <row r="16" spans="2:24" x14ac:dyDescent="0.2">
+      <c r="B16" s="3"/>
+      <c r="C16" s="3"/>
+      <c r="D16" s="3"/>
+      <c r="F16" s="3"/>
+      <c r="G16" s="3"/>
+      <c r="H16" s="3"/>
+      <c r="J16" s="3"/>
+      <c r="K16" s="3"/>
+      <c r="L16" s="3"/>
+      <c r="N16" s="3"/>
+      <c r="O16" s="3"/>
+      <c r="P16" s="3"/>
+      <c r="R16" s="3"/>
+      <c r="S16" s="3"/>
+      <c r="T16" s="3"/>
+      <c r="V16" s="3"/>
+      <c r="W16" s="3"/>
+      <c r="X16" s="3"/>
+    </row>
+    <row r="17" spans="2:24" x14ac:dyDescent="0.2">
+      <c r="B17" s="3"/>
+      <c r="C17" s="3"/>
+      <c r="D17" s="3"/>
+      <c r="F17" s="3"/>
+      <c r="G17" s="3"/>
+      <c r="H17" s="3"/>
+      <c r="J17" s="3"/>
+      <c r="K17" s="3"/>
+      <c r="L17" s="3"/>
+      <c r="N17" s="3"/>
+      <c r="O17" s="3"/>
+      <c r="P17" s="3"/>
+      <c r="R17" s="3"/>
+      <c r="S17" s="3"/>
+      <c r="T17" s="3"/>
+      <c r="V17" s="3"/>
+      <c r="W17" s="3"/>
+      <c r="X17" s="3"/>
+    </row>
+    <row r="18" spans="2:24" x14ac:dyDescent="0.2">
+      <c r="B18" s="3"/>
+      <c r="C18" s="3"/>
+      <c r="D18" s="3"/>
+      <c r="F18" s="3"/>
+      <c r="G18" s="3"/>
+      <c r="H18" s="3"/>
+      <c r="J18" s="3"/>
+      <c r="K18" s="3"/>
+      <c r="L18" s="3"/>
+      <c r="N18" s="3"/>
+      <c r="O18" s="3"/>
+      <c r="P18" s="3"/>
+      <c r="R18" s="3"/>
+      <c r="S18" s="3"/>
+      <c r="T18" s="3"/>
+      <c r="V18" s="3"/>
+      <c r="W18" s="3"/>
+      <c r="X18" s="3"/>
+    </row>
+    <row r="19" spans="2:24" x14ac:dyDescent="0.2">
+      <c r="B19" s="3"/>
+      <c r="C19" s="3"/>
+      <c r="D19" s="3"/>
+      <c r="F19" s="3"/>
+      <c r="G19" s="3"/>
+      <c r="H19" s="3"/>
+      <c r="J19" s="3"/>
+      <c r="K19" s="3"/>
+      <c r="L19" s="3"/>
+      <c r="N19" s="3"/>
+      <c r="O19" s="3"/>
+      <c r="P19" s="3"/>
+      <c r="R19" s="3"/>
+      <c r="S19" s="3"/>
+      <c r="T19" s="3"/>
+      <c r="V19" s="3"/>
+      <c r="W19" s="3"/>
+      <c r="X19" s="3"/>
+    </row>
+    <row r="20" spans="2:24" x14ac:dyDescent="0.2">
+      <c r="B20" s="3"/>
+      <c r="C20" s="3"/>
+      <c r="D20" s="3"/>
+      <c r="F20" s="3"/>
+      <c r="G20" s="3"/>
+      <c r="H20" s="3"/>
+      <c r="J20" s="3"/>
+      <c r="K20" s="3"/>
+      <c r="L20" s="3"/>
+      <c r="N20" s="3"/>
+      <c r="O20" s="3"/>
+      <c r="P20" s="3"/>
+      <c r="R20" s="3"/>
+      <c r="S20" s="3"/>
+      <c r="T20" s="3"/>
+      <c r="V20" s="3"/>
+      <c r="W20" s="3"/>
+      <c r="X20" s="3"/>
+    </row>
+    <row r="21" spans="2:24" x14ac:dyDescent="0.2">
+      <c r="B21" s="3"/>
+      <c r="C21" s="3"/>
+      <c r="D21" s="3"/>
+      <c r="F21" s="3"/>
+      <c r="G21" s="3"/>
+      <c r="H21" s="3"/>
+      <c r="J21" s="3"/>
+      <c r="K21" s="3"/>
+      <c r="L21" s="3"/>
+      <c r="N21" s="3"/>
+      <c r="O21" s="3"/>
+      <c r="P21" s="3"/>
+      <c r="R21" s="3"/>
+      <c r="S21" s="3"/>
+      <c r="T21" s="3"/>
+      <c r="V21" s="3"/>
+      <c r="W21" s="3"/>
+      <c r="X21" s="3"/>
+    </row>
+    <row r="22" spans="2:24" x14ac:dyDescent="0.2">
+      <c r="B22" s="3"/>
+      <c r="C22" s="3"/>
+      <c r="D22" s="3"/>
+      <c r="F22" s="3"/>
+      <c r="G22" s="3"/>
+      <c r="H22" s="3"/>
+      <c r="J22" s="3"/>
+      <c r="K22" s="3"/>
+      <c r="L22" s="3"/>
+      <c r="N22" s="3"/>
+      <c r="O22" s="3"/>
+      <c r="P22" s="3"/>
+      <c r="R22" s="3"/>
+      <c r="S22" s="3"/>
+      <c r="T22" s="3"/>
+      <c r="V22" s="3"/>
+      <c r="W22" s="3"/>
+      <c r="X22" s="3"/>
+    </row>
+  </sheetData>
+  <mergeCells count="6">
+    <mergeCell ref="R2:T2"/>
+    <mergeCell ref="V2:X2"/>
+    <mergeCell ref="B2:D2"/>
+    <mergeCell ref="F2:H2"/>
+    <mergeCell ref="J2:L2"/>
+    <mergeCell ref="N2:P2"/>
+  </mergeCells>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
template v18: save_times list on tseep (J10 header, vertical values; Norm)
Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_0147GB4LGVZuqGHCRMVzZTsR
</commit_message>
<xml_diff>
--- a/docs/inputs/input_template.xlsx
+++ b/docs/inputs/input_template.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/njones/python_projects/xslope/docs/inputs/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{525EDD25-6AD6-D045-8DB4-9766BDA4A811}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{31D06D1B-9F8B-4A48-B6E0-097F17D68253}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="620" windowWidth="34200" windowHeight="19900" xr2:uid="{BA54C293-CE08-6E4C-9212-B3317DAA148E}"/>
+    <workbookView xWindow="0" yWindow="620" windowWidth="34200" windowHeight="19900" activeTab="15" xr2:uid="{BA54C293-CE08-6E4C-9212-B3317DAA148E}"/>
   </bookViews>
   <sheets>
     <sheet name="main" sheetId="1" r:id="rId1"/>
@@ -63,7 +63,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="477" uniqueCount="264">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="478" uniqueCount="265">
   <si>
     <t>X</t>
   </si>
@@ -1020,6 +1020,9 @@
   </si>
   <si>
     <t>Sy</t>
+  </si>
+  <si>
+    <t>save_times</t>
   </si>
 </sst>
 </file>
@@ -1503,13 +1506,13 @@
     <xf numFmtId="0" fontId="10" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
     <xf numFmtId="0" fontId="2" fillId="14" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="14" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="15" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -1540,21 +1543,7 @@
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="23">
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor theme="0" tint="-0.499984740745262"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor theme="0" tint="-0.499984740745262"/>
-        </patternFill>
-      </fill>
-    </dxf>
+  <dxfs count="21">
     <dxf>
       <fill>
         <patternFill>
@@ -9075,7 +9064,7 @@
           <c:order val="0"/>
           <c:tx>
             <c:strRef>
-              <c:f>tseep!$H$2</c:f>
+              <c:f>tseep!$C$2</c:f>
               <c:strCache>
                 <c:ptCount val="1"/>
                 <c:pt idx="0">
@@ -9098,19 +9087,19 @@
           </c:marker>
           <c:xVal>
             <c:numRef>
-              <c:f>tseep!$G$3:$G$30</c:f>
+              <c:f>tseep!$B$3:$B$100</c:f>
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
-                <c:ptCount val="28"/>
+                <c:ptCount val="98"/>
               </c:numCache>
             </c:numRef>
           </c:xVal>
           <c:yVal>
             <c:numRef>
-              <c:f>tseep!$H$3:$H$30</c:f>
+              <c:f>tseep!$C$3:$C$100</c:f>
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
-                <c:ptCount val="28"/>
+                <c:ptCount val="98"/>
               </c:numCache>
             </c:numRef>
           </c:yVal>
@@ -9126,7 +9115,7 @@
           <c:order val="1"/>
           <c:tx>
             <c:strRef>
-              <c:f>tseep!$I$2</c:f>
+              <c:f>tseep!$D$2</c:f>
               <c:strCache>
                 <c:ptCount val="1"/>
                 <c:pt idx="0">
@@ -9149,19 +9138,19 @@
           </c:marker>
           <c:xVal>
             <c:numRef>
-              <c:f>tseep!$G$3:$G$30</c:f>
+              <c:f>tseep!$B$3:$B$100</c:f>
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
-                <c:ptCount val="28"/>
+                <c:ptCount val="98"/>
               </c:numCache>
             </c:numRef>
           </c:xVal>
           <c:yVal>
             <c:numRef>
-              <c:f>tseep!$I$3:$I$30</c:f>
+              <c:f>tseep!$D$3:$D$100</c:f>
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
-                <c:ptCount val="28"/>
+                <c:ptCount val="98"/>
               </c:numCache>
             </c:numRef>
           </c:yVal>
@@ -9177,7 +9166,7 @@
           <c:order val="2"/>
           <c:tx>
             <c:strRef>
-              <c:f>tseep!$J$2</c:f>
+              <c:f>tseep!$E$2</c:f>
               <c:strCache>
                 <c:ptCount val="1"/>
                 <c:pt idx="0">
@@ -9200,19 +9189,19 @@
           </c:marker>
           <c:xVal>
             <c:numRef>
-              <c:f>tseep!$G$3:$G$30</c:f>
+              <c:f>tseep!$B$3:$B$100</c:f>
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
-                <c:ptCount val="28"/>
+                <c:ptCount val="98"/>
               </c:numCache>
             </c:numRef>
           </c:xVal>
           <c:yVal>
             <c:numRef>
-              <c:f>tseep!$J$3:$J$30</c:f>
+              <c:f>tseep!$E$3:$E$100</c:f>
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
-                <c:ptCount val="28"/>
+                <c:ptCount val="98"/>
               </c:numCache>
             </c:numRef>
           </c:yVal>
@@ -9228,7 +9217,7 @@
           <c:order val="3"/>
           <c:tx>
             <c:strRef>
-              <c:f>tseep!$K$2</c:f>
+              <c:f>tseep!$F$2</c:f>
               <c:strCache>
                 <c:ptCount val="1"/>
                 <c:pt idx="0">
@@ -9251,19 +9240,19 @@
           </c:marker>
           <c:xVal>
             <c:numRef>
-              <c:f>tseep!$G$3:$G$30</c:f>
+              <c:f>tseep!$B$3:$B$100</c:f>
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
-                <c:ptCount val="28"/>
+                <c:ptCount val="98"/>
               </c:numCache>
             </c:numRef>
           </c:xVal>
           <c:yVal>
             <c:numRef>
-              <c:f>tseep!$K$3:$K$30</c:f>
+              <c:f>tseep!$F$3:$F$100</c:f>
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
-                <c:ptCount val="28"/>
+                <c:ptCount val="98"/>
               </c:numCache>
             </c:numRef>
           </c:yVal>
@@ -9279,7 +9268,7 @@
           <c:order val="4"/>
           <c:tx>
             <c:strRef>
-              <c:f>tseep!$L$2</c:f>
+              <c:f>tseep!$G$2</c:f>
               <c:strCache>
                 <c:ptCount val="1"/>
                 <c:pt idx="0">
@@ -9302,19 +9291,19 @@
           </c:marker>
           <c:xVal>
             <c:numRef>
-              <c:f>tseep!$G$3:$G$30</c:f>
+              <c:f>tseep!$B$3:$B$100</c:f>
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
-                <c:ptCount val="28"/>
+                <c:ptCount val="98"/>
               </c:numCache>
             </c:numRef>
           </c:xVal>
           <c:yVal>
             <c:numRef>
-              <c:f>tseep!$L$3:$L$30</c:f>
+              <c:f>tseep!$G$3:$G$100</c:f>
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
-                <c:ptCount val="28"/>
+                <c:ptCount val="98"/>
               </c:numCache>
             </c:numRef>
           </c:yVal>
@@ -11267,14 +11256,14 @@
 <xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
   <xdr:twoCellAnchor>
     <xdr:from>
-      <xdr:col>15</xdr:col>
-      <xdr:colOff>444499</xdr:colOff>
+      <xdr:col>11</xdr:col>
+      <xdr:colOff>99785</xdr:colOff>
       <xdr:row>1</xdr:row>
       <xdr:rowOff>88901</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>22</xdr:col>
-      <xdr:colOff>644071</xdr:colOff>
+      <xdr:col>18</xdr:col>
+      <xdr:colOff>299357</xdr:colOff>
       <xdr:row>22</xdr:row>
       <xdr:rowOff>99787</xdr:rowOff>
     </xdr:to>
@@ -14505,277 +14494,930 @@
 
 <file path=xl/worksheets/sheet16.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B20D353C-FC33-C347-9989-88B2E3FC7B94}">
-  <dimension ref="G2:O30"/>
+  <dimension ref="B2:J100"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="6" max="6" width="3.5" customWidth="1"/>
-    <col min="7" max="12" width="10.83203125" style="1"/>
-    <col min="13" max="13" width="7.1640625" customWidth="1"/>
+    <col min="1" max="1" width="3.5" customWidth="1"/>
+    <col min="2" max="7" width="10.83203125" style="1"/>
+    <col min="8" max="8" width="7.1640625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="2" spans="7:15" x14ac:dyDescent="0.2">
+    <row r="2" spans="2:10" x14ac:dyDescent="0.2">
+      <c r="B2" s="50" t="s">
+        <v>255</v>
+      </c>
+      <c r="C2" s="50" t="s">
+        <v>250</v>
+      </c>
+      <c r="D2" s="50" t="s">
+        <v>251</v>
+      </c>
+      <c r="E2" s="50" t="s">
+        <v>252</v>
+      </c>
+      <c r="F2" s="50" t="s">
+        <v>253</v>
+      </c>
       <c r="G2" s="50" t="s">
-        <v>255</v>
-      </c>
-      <c r="H2" s="50" t="s">
-        <v>250</v>
-      </c>
-      <c r="I2" s="50" t="s">
-        <v>251</v>
-      </c>
-      <c r="J2" s="50" t="s">
-        <v>252</v>
-      </c>
-      <c r="K2" s="50" t="s">
-        <v>253</v>
-      </c>
-      <c r="L2" s="50" t="s">
         <v>254</v>
       </c>
     </row>
-    <row r="3" spans="7:15" x14ac:dyDescent="0.2">
+    <row r="3" spans="2:10" x14ac:dyDescent="0.2">
+      <c r="B3" s="3"/>
+      <c r="C3" s="3"/>
+      <c r="D3" s="3"/>
+      <c r="E3" s="3"/>
+      <c r="F3" s="3"/>
       <c r="G3" s="3"/>
-      <c r="H3" s="3"/>
-      <c r="I3" s="3"/>
+      <c r="I3" s="14" t="s">
+        <v>257</v>
+      </c>
       <c r="J3" s="3"/>
-      <c r="K3" s="3"/>
-      <c r="L3" s="3"/>
-      <c r="N3" s="14" t="s">
-        <v>257</v>
-      </c>
-      <c r="O3" s="1"/>
-    </row>
-    <row r="4" spans="7:15" x14ac:dyDescent="0.2">
+    </row>
+    <row r="4" spans="2:10" x14ac:dyDescent="0.2">
+      <c r="B4" s="3"/>
+      <c r="C4" s="3"/>
+      <c r="D4" s="3"/>
+      <c r="E4" s="3"/>
+      <c r="F4" s="3"/>
       <c r="G4" s="3"/>
-      <c r="H4" s="3"/>
-      <c r="I4" s="3"/>
-      <c r="J4" s="3"/>
-      <c r="K4" s="3"/>
-      <c r="L4" s="3"/>
-      <c r="N4" s="14"/>
-      <c r="O4" s="1"/>
-    </row>
-    <row r="5" spans="7:15" x14ac:dyDescent="0.2">
+      <c r="I4" s="14"/>
+      <c r="J4" s="1"/>
+    </row>
+    <row r="5" spans="2:10" x14ac:dyDescent="0.2">
+      <c r="B5" s="3"/>
+      <c r="C5" s="3"/>
+      <c r="D5" s="3"/>
+      <c r="E5" s="3"/>
+      <c r="F5" s="3"/>
       <c r="G5" s="3"/>
-      <c r="H5" s="3"/>
-      <c r="I5" s="3"/>
+      <c r="I5" s="14" t="s">
+        <v>256</v>
+      </c>
       <c r="J5" s="3"/>
-      <c r="K5" s="3"/>
-      <c r="L5" s="3"/>
-      <c r="N5" s="14" t="s">
-        <v>256</v>
-      </c>
-      <c r="O5" s="1"/>
-    </row>
-    <row r="6" spans="7:15" x14ac:dyDescent="0.2">
+    </row>
+    <row r="6" spans="2:10" x14ac:dyDescent="0.2">
+      <c r="B6" s="3"/>
+      <c r="C6" s="3"/>
+      <c r="D6" s="3"/>
+      <c r="E6" s="3"/>
+      <c r="F6" s="3"/>
       <c r="G6" s="3"/>
-      <c r="H6" s="3"/>
-      <c r="I6" s="3"/>
-      <c r="J6" s="3"/>
-      <c r="K6" s="3"/>
-      <c r="L6" s="3"/>
-      <c r="N6" s="14"/>
-      <c r="O6" s="1"/>
-    </row>
-    <row r="7" spans="7:15" x14ac:dyDescent="0.2">
+      <c r="I6" s="14"/>
+      <c r="J6" s="1"/>
+    </row>
+    <row r="7" spans="2:10" x14ac:dyDescent="0.2">
+      <c r="B7" s="3"/>
+      <c r="C7" s="3"/>
+      <c r="D7" s="3"/>
+      <c r="E7" s="3"/>
+      <c r="F7" s="3"/>
       <c r="G7" s="3"/>
-      <c r="H7" s="3"/>
-      <c r="I7" s="3"/>
+      <c r="I7" s="14" t="s">
+        <v>258</v>
+      </c>
       <c r="J7" s="3"/>
-      <c r="K7" s="3"/>
-      <c r="L7" s="3"/>
-      <c r="N7" s="14" t="s">
-        <v>258</v>
-      </c>
-      <c r="O7" s="1"/>
-    </row>
-    <row r="8" spans="7:15" x14ac:dyDescent="0.2">
+    </row>
+    <row r="8" spans="2:10" x14ac:dyDescent="0.2">
+      <c r="B8" s="3"/>
+      <c r="C8" s="3"/>
+      <c r="D8" s="3"/>
+      <c r="E8" s="3"/>
+      <c r="F8" s="3"/>
       <c r="G8" s="3"/>
-      <c r="H8" s="3"/>
-      <c r="I8" s="3"/>
+      <c r="I8" s="14" t="s">
+        <v>259</v>
+      </c>
       <c r="J8" s="3"/>
-      <c r="K8" s="3"/>
-      <c r="L8" s="3"/>
-      <c r="N8" s="14" t="s">
-        <v>259</v>
-      </c>
-      <c r="O8" s="1"/>
-    </row>
-    <row r="9" spans="7:15" x14ac:dyDescent="0.2">
+    </row>
+    <row r="9" spans="2:10" x14ac:dyDescent="0.2">
+      <c r="B9" s="3"/>
+      <c r="C9" s="3"/>
+      <c r="D9" s="3"/>
+      <c r="E9" s="3"/>
+      <c r="F9" s="3"/>
       <c r="G9" s="3"/>
-      <c r="H9" s="3"/>
-      <c r="I9" s="3"/>
-      <c r="J9" s="3"/>
-      <c r="K9" s="3"/>
-      <c r="L9" s="3"/>
-    </row>
-    <row r="10" spans="7:15" x14ac:dyDescent="0.2">
+    </row>
+    <row r="10" spans="2:10" x14ac:dyDescent="0.2">
+      <c r="B10" s="3"/>
+      <c r="C10" s="3"/>
+      <c r="D10" s="3"/>
+      <c r="E10" s="3"/>
+      <c r="F10" s="3"/>
       <c r="G10" s="3"/>
-      <c r="H10" s="3"/>
-      <c r="I10" s="3"/>
-      <c r="J10" s="3"/>
-      <c r="K10" s="3"/>
-      <c r="L10" s="3"/>
-    </row>
-    <row r="11" spans="7:15" x14ac:dyDescent="0.2">
+      <c r="J10" t="s">
+        <v>264</v>
+      </c>
+    </row>
+    <row r="11" spans="2:10" x14ac:dyDescent="0.2">
+      <c r="B11" s="3"/>
+      <c r="C11" s="3"/>
+      <c r="D11" s="3"/>
+      <c r="E11" s="3"/>
+      <c r="F11" s="3"/>
       <c r="G11" s="3"/>
-      <c r="H11" s="3"/>
-      <c r="I11" s="3"/>
-      <c r="J11" s="3"/>
-      <c r="K11" s="3"/>
-      <c r="L11" s="3"/>
-    </row>
-    <row r="12" spans="7:15" x14ac:dyDescent="0.2">
+      <c r="J11" s="4"/>
+    </row>
+    <row r="12" spans="2:10" x14ac:dyDescent="0.2">
+      <c r="B12" s="3"/>
+      <c r="C12" s="3"/>
+      <c r="D12" s="3"/>
+      <c r="E12" s="3"/>
+      <c r="F12" s="3"/>
       <c r="G12" s="3"/>
-      <c r="H12" s="3"/>
-      <c r="I12" s="3"/>
-      <c r="J12" s="3"/>
-      <c r="K12" s="3"/>
-      <c r="L12" s="3"/>
-    </row>
-    <row r="13" spans="7:15" x14ac:dyDescent="0.2">
+      <c r="J12" s="4"/>
+    </row>
+    <row r="13" spans="2:10" x14ac:dyDescent="0.2">
+      <c r="B13" s="3"/>
+      <c r="C13" s="3"/>
+      <c r="D13" s="3"/>
+      <c r="E13" s="3"/>
+      <c r="F13" s="3"/>
       <c r="G13" s="3"/>
-      <c r="H13" s="3"/>
-      <c r="I13" s="3"/>
-      <c r="J13" s="3"/>
-      <c r="K13" s="3"/>
-      <c r="L13" s="3"/>
-    </row>
-    <row r="14" spans="7:15" x14ac:dyDescent="0.2">
+      <c r="J13" s="4"/>
+    </row>
+    <row r="14" spans="2:10" x14ac:dyDescent="0.2">
+      <c r="B14" s="3"/>
+      <c r="C14" s="3"/>
+      <c r="D14" s="3"/>
+      <c r="E14" s="3"/>
+      <c r="F14" s="3"/>
       <c r="G14" s="3"/>
-      <c r="H14" s="3"/>
-      <c r="I14" s="3"/>
-      <c r="J14" s="3"/>
-      <c r="K14" s="3"/>
-      <c r="L14" s="3"/>
-    </row>
-    <row r="15" spans="7:15" x14ac:dyDescent="0.2">
+      <c r="J14" s="4"/>
+    </row>
+    <row r="15" spans="2:10" x14ac:dyDescent="0.2">
+      <c r="B15" s="3"/>
+      <c r="C15" s="3"/>
+      <c r="D15" s="3"/>
+      <c r="E15" s="3"/>
+      <c r="F15" s="3"/>
       <c r="G15" s="3"/>
-      <c r="H15" s="3"/>
-      <c r="I15" s="3"/>
-      <c r="J15" s="3"/>
-      <c r="K15" s="3"/>
-      <c r="L15" s="3"/>
-    </row>
-    <row r="16" spans="7:15" x14ac:dyDescent="0.2">
+      <c r="J15" s="4"/>
+    </row>
+    <row r="16" spans="2:10" x14ac:dyDescent="0.2">
+      <c r="B16" s="3"/>
+      <c r="C16" s="3"/>
+      <c r="D16" s="3"/>
+      <c r="E16" s="3"/>
+      <c r="F16" s="3"/>
       <c r="G16" s="3"/>
-      <c r="H16" s="3"/>
-      <c r="I16" s="3"/>
-      <c r="J16" s="3"/>
-      <c r="K16" s="3"/>
-      <c r="L16" s="3"/>
-    </row>
-    <row r="17" spans="7:12" x14ac:dyDescent="0.2">
+      <c r="J16" s="4"/>
+    </row>
+    <row r="17" spans="2:10" x14ac:dyDescent="0.2">
+      <c r="B17" s="3"/>
+      <c r="C17" s="3"/>
+      <c r="D17" s="3"/>
+      <c r="E17" s="3"/>
+      <c r="F17" s="3"/>
       <c r="G17" s="3"/>
-      <c r="H17" s="3"/>
-      <c r="I17" s="3"/>
-      <c r="J17" s="3"/>
-      <c r="K17" s="3"/>
-      <c r="L17" s="3"/>
-    </row>
-    <row r="18" spans="7:12" x14ac:dyDescent="0.2">
+      <c r="J17" s="4"/>
+    </row>
+    <row r="18" spans="2:10" x14ac:dyDescent="0.2">
+      <c r="B18" s="3"/>
+      <c r="C18" s="3"/>
+      <c r="D18" s="3"/>
+      <c r="E18" s="3"/>
+      <c r="F18" s="3"/>
       <c r="G18" s="3"/>
-      <c r="H18" s="3"/>
-      <c r="I18" s="3"/>
-      <c r="J18" s="3"/>
-      <c r="K18" s="3"/>
-      <c r="L18" s="3"/>
-    </row>
-    <row r="19" spans="7:12" x14ac:dyDescent="0.2">
+      <c r="J18" s="4"/>
+    </row>
+    <row r="19" spans="2:10" x14ac:dyDescent="0.2">
+      <c r="B19" s="3"/>
+      <c r="C19" s="3"/>
+      <c r="D19" s="3"/>
+      <c r="E19" s="3"/>
+      <c r="F19" s="3"/>
       <c r="G19" s="3"/>
-      <c r="H19" s="3"/>
-      <c r="I19" s="3"/>
-      <c r="J19" s="3"/>
-      <c r="K19" s="3"/>
-      <c r="L19" s="3"/>
-    </row>
-    <row r="20" spans="7:12" x14ac:dyDescent="0.2">
+      <c r="J19" s="4"/>
+    </row>
+    <row r="20" spans="2:10" x14ac:dyDescent="0.2">
+      <c r="B20" s="3"/>
+      <c r="C20" s="3"/>
+      <c r="D20" s="3"/>
+      <c r="E20" s="3"/>
+      <c r="F20" s="3"/>
       <c r="G20" s="3"/>
-      <c r="H20" s="3"/>
-      <c r="I20" s="3"/>
-      <c r="J20" s="3"/>
-      <c r="K20" s="3"/>
-      <c r="L20" s="3"/>
-    </row>
-    <row r="21" spans="7:12" x14ac:dyDescent="0.2">
+      <c r="J20" s="4"/>
+    </row>
+    <row r="21" spans="2:10" x14ac:dyDescent="0.2">
+      <c r="B21" s="3"/>
+      <c r="C21" s="3"/>
+      <c r="D21" s="3"/>
+      <c r="E21" s="3"/>
+      <c r="F21" s="3"/>
       <c r="G21" s="3"/>
-      <c r="H21" s="3"/>
-      <c r="I21" s="3"/>
-      <c r="J21" s="3"/>
-      <c r="K21" s="3"/>
-      <c r="L21" s="3"/>
-    </row>
-    <row r="22" spans="7:12" x14ac:dyDescent="0.2">
+      <c r="J21" s="4"/>
+    </row>
+    <row r="22" spans="2:10" x14ac:dyDescent="0.2">
+      <c r="B22" s="3"/>
+      <c r="C22" s="3"/>
+      <c r="D22" s="3"/>
+      <c r="E22" s="3"/>
+      <c r="F22" s="3"/>
       <c r="G22" s="3"/>
-      <c r="H22" s="3"/>
-      <c r="I22" s="3"/>
-      <c r="J22" s="3"/>
-      <c r="K22" s="3"/>
-      <c r="L22" s="3"/>
-    </row>
-    <row r="23" spans="7:12" x14ac:dyDescent="0.2">
+      <c r="J22" s="4"/>
+    </row>
+    <row r="23" spans="2:10" x14ac:dyDescent="0.2">
+      <c r="B23" s="3"/>
+      <c r="C23" s="3"/>
+      <c r="D23" s="3"/>
+      <c r="E23" s="3"/>
+      <c r="F23" s="3"/>
       <c r="G23" s="3"/>
-      <c r="H23" s="3"/>
-      <c r="I23" s="3"/>
-      <c r="J23" s="3"/>
-      <c r="K23" s="3"/>
-      <c r="L23" s="3"/>
-    </row>
-    <row r="24" spans="7:12" x14ac:dyDescent="0.2">
+      <c r="J23" s="4"/>
+    </row>
+    <row r="24" spans="2:10" x14ac:dyDescent="0.2">
+      <c r="B24" s="3"/>
+      <c r="C24" s="3"/>
+      <c r="D24" s="3"/>
+      <c r="E24" s="3"/>
+      <c r="F24" s="3"/>
       <c r="G24" s="3"/>
-      <c r="H24" s="3"/>
-      <c r="I24" s="3"/>
-      <c r="J24" s="3"/>
-      <c r="K24" s="3"/>
-      <c r="L24" s="3"/>
-    </row>
-    <row r="25" spans="7:12" x14ac:dyDescent="0.2">
+      <c r="J24" s="4"/>
+    </row>
+    <row r="25" spans="2:10" x14ac:dyDescent="0.2">
+      <c r="B25" s="3"/>
+      <c r="C25" s="3"/>
+      <c r="D25" s="3"/>
+      <c r="E25" s="3"/>
+      <c r="F25" s="3"/>
       <c r="G25" s="3"/>
-      <c r="H25" s="3"/>
-      <c r="I25" s="3"/>
-      <c r="J25" s="3"/>
-      <c r="K25" s="3"/>
-      <c r="L25" s="3"/>
-    </row>
-    <row r="26" spans="7:12" x14ac:dyDescent="0.2">
+      <c r="J25" s="4"/>
+    </row>
+    <row r="26" spans="2:10" x14ac:dyDescent="0.2">
+      <c r="B26" s="3"/>
+      <c r="C26" s="3"/>
+      <c r="D26" s="3"/>
+      <c r="E26" s="3"/>
+      <c r="F26" s="3"/>
       <c r="G26" s="3"/>
-      <c r="H26" s="3"/>
-      <c r="I26" s="3"/>
-      <c r="J26" s="3"/>
-      <c r="K26" s="3"/>
-      <c r="L26" s="3"/>
-    </row>
-    <row r="27" spans="7:12" x14ac:dyDescent="0.2">
+      <c r="J26" s="4"/>
+    </row>
+    <row r="27" spans="2:10" x14ac:dyDescent="0.2">
+      <c r="B27" s="3"/>
+      <c r="C27" s="3"/>
+      <c r="D27" s="3"/>
+      <c r="E27" s="3"/>
+      <c r="F27" s="3"/>
       <c r="G27" s="3"/>
-      <c r="H27" s="3"/>
-      <c r="I27" s="3"/>
-      <c r="J27" s="3"/>
-      <c r="K27" s="3"/>
-      <c r="L27" s="3"/>
-    </row>
-    <row r="28" spans="7:12" x14ac:dyDescent="0.2">
+      <c r="J27" s="4"/>
+    </row>
+    <row r="28" spans="2:10" x14ac:dyDescent="0.2">
+      <c r="B28" s="3"/>
+      <c r="C28" s="3"/>
+      <c r="D28" s="3"/>
+      <c r="E28" s="3"/>
+      <c r="F28" s="3"/>
       <c r="G28" s="3"/>
-      <c r="H28" s="3"/>
-      <c r="I28" s="3"/>
-      <c r="J28" s="3"/>
-      <c r="K28" s="3"/>
-      <c r="L28" s="3"/>
-    </row>
-    <row r="29" spans="7:12" x14ac:dyDescent="0.2">
+      <c r="J28" s="4"/>
+    </row>
+    <row r="29" spans="2:10" x14ac:dyDescent="0.2">
+      <c r="B29" s="3"/>
+      <c r="C29" s="3"/>
+      <c r="D29" s="3"/>
+      <c r="E29" s="3"/>
+      <c r="F29" s="3"/>
       <c r="G29" s="3"/>
-      <c r="H29" s="3"/>
-      <c r="I29" s="3"/>
-      <c r="J29" s="3"/>
-      <c r="K29" s="3"/>
-      <c r="L29" s="3"/>
-    </row>
-    <row r="30" spans="7:12" x14ac:dyDescent="0.2">
+      <c r="J29" s="4"/>
+    </row>
+    <row r="30" spans="2:10" x14ac:dyDescent="0.2">
+      <c r="B30" s="3"/>
+      <c r="C30" s="3"/>
+      <c r="D30" s="3"/>
+      <c r="E30" s="3"/>
+      <c r="F30" s="3"/>
       <c r="G30" s="3"/>
-      <c r="H30" s="3"/>
-      <c r="I30" s="3"/>
-      <c r="J30" s="3"/>
-      <c r="K30" s="3"/>
-      <c r="L30" s="3"/>
+      <c r="J30" s="4"/>
+    </row>
+    <row r="31" spans="2:10" x14ac:dyDescent="0.2">
+      <c r="B31" s="3"/>
+      <c r="C31" s="3"/>
+      <c r="D31" s="3"/>
+      <c r="E31" s="3"/>
+      <c r="F31" s="3"/>
+      <c r="G31" s="3"/>
+      <c r="J31" s="4"/>
+    </row>
+    <row r="32" spans="2:10" x14ac:dyDescent="0.2">
+      <c r="B32" s="3"/>
+      <c r="C32" s="3"/>
+      <c r="D32" s="3"/>
+      <c r="E32" s="3"/>
+      <c r="F32" s="3"/>
+      <c r="G32" s="3"/>
+      <c r="J32" s="4"/>
+    </row>
+    <row r="33" spans="2:10" x14ac:dyDescent="0.2">
+      <c r="B33" s="3"/>
+      <c r="C33" s="3"/>
+      <c r="D33" s="3"/>
+      <c r="E33" s="3"/>
+      <c r="F33" s="3"/>
+      <c r="G33" s="3"/>
+      <c r="J33" s="4"/>
+    </row>
+    <row r="34" spans="2:10" x14ac:dyDescent="0.2">
+      <c r="B34" s="3"/>
+      <c r="C34" s="3"/>
+      <c r="D34" s="3"/>
+      <c r="E34" s="3"/>
+      <c r="F34" s="3"/>
+      <c r="G34" s="3"/>
+      <c r="J34" s="4"/>
+    </row>
+    <row r="35" spans="2:10" x14ac:dyDescent="0.2">
+      <c r="B35" s="3"/>
+      <c r="C35" s="3"/>
+      <c r="D35" s="3"/>
+      <c r="E35" s="3"/>
+      <c r="F35" s="3"/>
+      <c r="G35" s="3"/>
+      <c r="J35" s="4"/>
+    </row>
+    <row r="36" spans="2:10" x14ac:dyDescent="0.2">
+      <c r="B36" s="3"/>
+      <c r="C36" s="3"/>
+      <c r="D36" s="3"/>
+      <c r="E36" s="3"/>
+      <c r="F36" s="3"/>
+      <c r="G36" s="3"/>
+      <c r="J36" s="4"/>
+    </row>
+    <row r="37" spans="2:10" x14ac:dyDescent="0.2">
+      <c r="B37" s="3"/>
+      <c r="C37" s="3"/>
+      <c r="D37" s="3"/>
+      <c r="E37" s="3"/>
+      <c r="F37" s="3"/>
+      <c r="G37" s="3"/>
+      <c r="J37" s="4"/>
+    </row>
+    <row r="38" spans="2:10" x14ac:dyDescent="0.2">
+      <c r="B38" s="3"/>
+      <c r="C38" s="3"/>
+      <c r="D38" s="3"/>
+      <c r="E38" s="3"/>
+      <c r="F38" s="3"/>
+      <c r="G38" s="3"/>
+      <c r="J38" s="4"/>
+    </row>
+    <row r="39" spans="2:10" x14ac:dyDescent="0.2">
+      <c r="B39" s="3"/>
+      <c r="C39" s="3"/>
+      <c r="D39" s="3"/>
+      <c r="E39" s="3"/>
+      <c r="F39" s="3"/>
+      <c r="G39" s="3"/>
+      <c r="J39" s="4"/>
+    </row>
+    <row r="40" spans="2:10" x14ac:dyDescent="0.2">
+      <c r="B40" s="3"/>
+      <c r="C40" s="3"/>
+      <c r="D40" s="3"/>
+      <c r="E40" s="3"/>
+      <c r="F40" s="3"/>
+      <c r="G40" s="3"/>
+      <c r="J40" s="4"/>
+    </row>
+    <row r="41" spans="2:10" x14ac:dyDescent="0.2">
+      <c r="B41" s="3"/>
+      <c r="C41" s="3"/>
+      <c r="D41" s="3"/>
+      <c r="E41" s="3"/>
+      <c r="F41" s="3"/>
+      <c r="G41" s="3"/>
+      <c r="J41" s="4"/>
+    </row>
+    <row r="42" spans="2:10" x14ac:dyDescent="0.2">
+      <c r="B42" s="3"/>
+      <c r="C42" s="3"/>
+      <c r="D42" s="3"/>
+      <c r="E42" s="3"/>
+      <c r="F42" s="3"/>
+      <c r="G42" s="3"/>
+      <c r="J42" s="4"/>
+    </row>
+    <row r="43" spans="2:10" x14ac:dyDescent="0.2">
+      <c r="B43" s="3"/>
+      <c r="C43" s="3"/>
+      <c r="D43" s="3"/>
+      <c r="E43" s="3"/>
+      <c r="F43" s="3"/>
+      <c r="G43" s="3"/>
+      <c r="J43" s="4"/>
+    </row>
+    <row r="44" spans="2:10" x14ac:dyDescent="0.2">
+      <c r="B44" s="3"/>
+      <c r="C44" s="3"/>
+      <c r="D44" s="3"/>
+      <c r="E44" s="3"/>
+      <c r="F44" s="3"/>
+      <c r="G44" s="3"/>
+      <c r="J44" s="4"/>
+    </row>
+    <row r="45" spans="2:10" x14ac:dyDescent="0.2">
+      <c r="B45" s="3"/>
+      <c r="C45" s="3"/>
+      <c r="D45" s="3"/>
+      <c r="E45" s="3"/>
+      <c r="F45" s="3"/>
+      <c r="G45" s="3"/>
+      <c r="J45" s="4"/>
+    </row>
+    <row r="46" spans="2:10" x14ac:dyDescent="0.2">
+      <c r="B46" s="3"/>
+      <c r="C46" s="3"/>
+      <c r="D46" s="3"/>
+      <c r="E46" s="3"/>
+      <c r="F46" s="3"/>
+      <c r="G46" s="3"/>
+      <c r="J46" s="4"/>
+    </row>
+    <row r="47" spans="2:10" x14ac:dyDescent="0.2">
+      <c r="B47" s="3"/>
+      <c r="C47" s="3"/>
+      <c r="D47" s="3"/>
+      <c r="E47" s="3"/>
+      <c r="F47" s="3"/>
+      <c r="G47" s="3"/>
+      <c r="J47" s="4"/>
+    </row>
+    <row r="48" spans="2:10" x14ac:dyDescent="0.2">
+      <c r="B48" s="3"/>
+      <c r="C48" s="3"/>
+      <c r="D48" s="3"/>
+      <c r="E48" s="3"/>
+      <c r="F48" s="3"/>
+      <c r="G48" s="3"/>
+      <c r="J48" s="4"/>
+    </row>
+    <row r="49" spans="2:10" x14ac:dyDescent="0.2">
+      <c r="B49" s="3"/>
+      <c r="C49" s="3"/>
+      <c r="D49" s="3"/>
+      <c r="E49" s="3"/>
+      <c r="F49" s="3"/>
+      <c r="G49" s="3"/>
+      <c r="J49" s="4"/>
+    </row>
+    <row r="50" spans="2:10" x14ac:dyDescent="0.2">
+      <c r="B50" s="3"/>
+      <c r="C50" s="3"/>
+      <c r="D50" s="3"/>
+      <c r="E50" s="3"/>
+      <c r="F50" s="3"/>
+      <c r="G50" s="3"/>
+      <c r="J50" s="4"/>
+    </row>
+    <row r="51" spans="2:10" x14ac:dyDescent="0.2">
+      <c r="B51" s="3"/>
+      <c r="C51" s="3"/>
+      <c r="D51" s="3"/>
+      <c r="E51" s="3"/>
+      <c r="F51" s="3"/>
+      <c r="G51" s="3"/>
+      <c r="J51" s="4"/>
+    </row>
+    <row r="52" spans="2:10" x14ac:dyDescent="0.2">
+      <c r="B52" s="3"/>
+      <c r="C52" s="3"/>
+      <c r="D52" s="3"/>
+      <c r="E52" s="3"/>
+      <c r="F52" s="3"/>
+      <c r="G52" s="3"/>
+      <c r="J52" s="4"/>
+    </row>
+    <row r="53" spans="2:10" x14ac:dyDescent="0.2">
+      <c r="B53" s="3"/>
+      <c r="C53" s="3"/>
+      <c r="D53" s="3"/>
+      <c r="E53" s="3"/>
+      <c r="F53" s="3"/>
+      <c r="G53" s="3"/>
+      <c r="J53" s="4"/>
+    </row>
+    <row r="54" spans="2:10" x14ac:dyDescent="0.2">
+      <c r="B54" s="3"/>
+      <c r="C54" s="3"/>
+      <c r="D54" s="3"/>
+      <c r="E54" s="3"/>
+      <c r="F54" s="3"/>
+      <c r="G54" s="3"/>
+      <c r="J54" s="4"/>
+    </row>
+    <row r="55" spans="2:10" x14ac:dyDescent="0.2">
+      <c r="B55" s="3"/>
+      <c r="C55" s="3"/>
+      <c r="D55" s="3"/>
+      <c r="E55" s="3"/>
+      <c r="F55" s="3"/>
+      <c r="G55" s="3"/>
+      <c r="J55" s="4"/>
+    </row>
+    <row r="56" spans="2:10" x14ac:dyDescent="0.2">
+      <c r="B56" s="3"/>
+      <c r="C56" s="3"/>
+      <c r="D56" s="3"/>
+      <c r="E56" s="3"/>
+      <c r="F56" s="3"/>
+      <c r="G56" s="3"/>
+      <c r="J56" s="4"/>
+    </row>
+    <row r="57" spans="2:10" x14ac:dyDescent="0.2">
+      <c r="B57" s="3"/>
+      <c r="C57" s="3"/>
+      <c r="D57" s="3"/>
+      <c r="E57" s="3"/>
+      <c r="F57" s="3"/>
+      <c r="G57" s="3"/>
+      <c r="J57" s="4"/>
+    </row>
+    <row r="58" spans="2:10" x14ac:dyDescent="0.2">
+      <c r="B58" s="3"/>
+      <c r="C58" s="3"/>
+      <c r="D58" s="3"/>
+      <c r="E58" s="3"/>
+      <c r="F58" s="3"/>
+      <c r="G58" s="3"/>
+      <c r="J58" s="4"/>
+    </row>
+    <row r="59" spans="2:10" x14ac:dyDescent="0.2">
+      <c r="B59" s="3"/>
+      <c r="C59" s="3"/>
+      <c r="D59" s="3"/>
+      <c r="E59" s="3"/>
+      <c r="F59" s="3"/>
+      <c r="G59" s="3"/>
+      <c r="J59" s="4"/>
+    </row>
+    <row r="60" spans="2:10" x14ac:dyDescent="0.2">
+      <c r="B60" s="3"/>
+      <c r="C60" s="3"/>
+      <c r="D60" s="3"/>
+      <c r="E60" s="3"/>
+      <c r="F60" s="3"/>
+      <c r="G60" s="3"/>
+      <c r="J60" s="4"/>
+    </row>
+    <row r="61" spans="2:10" x14ac:dyDescent="0.2">
+      <c r="B61" s="3"/>
+      <c r="C61" s="3"/>
+      <c r="D61" s="3"/>
+      <c r="E61" s="3"/>
+      <c r="F61" s="3"/>
+      <c r="G61" s="3"/>
+      <c r="J61" s="4"/>
+    </row>
+    <row r="62" spans="2:10" x14ac:dyDescent="0.2">
+      <c r="B62" s="3"/>
+      <c r="C62" s="3"/>
+      <c r="D62" s="3"/>
+      <c r="E62" s="3"/>
+      <c r="F62" s="3"/>
+      <c r="G62" s="3"/>
+      <c r="J62" s="4"/>
+    </row>
+    <row r="63" spans="2:10" x14ac:dyDescent="0.2">
+      <c r="B63" s="3"/>
+      <c r="C63" s="3"/>
+      <c r="D63" s="3"/>
+      <c r="E63" s="3"/>
+      <c r="F63" s="3"/>
+      <c r="G63" s="3"/>
+      <c r="J63" s="4"/>
+    </row>
+    <row r="64" spans="2:10" x14ac:dyDescent="0.2">
+      <c r="B64" s="3"/>
+      <c r="C64" s="3"/>
+      <c r="D64" s="3"/>
+      <c r="E64" s="3"/>
+      <c r="F64" s="3"/>
+      <c r="G64" s="3"/>
+      <c r="J64" s="4"/>
+    </row>
+    <row r="65" spans="2:10" x14ac:dyDescent="0.2">
+      <c r="B65" s="3"/>
+      <c r="C65" s="3"/>
+      <c r="D65" s="3"/>
+      <c r="E65" s="3"/>
+      <c r="F65" s="3"/>
+      <c r="G65" s="3"/>
+      <c r="J65" s="4"/>
+    </row>
+    <row r="66" spans="2:10" x14ac:dyDescent="0.2">
+      <c r="B66" s="3"/>
+      <c r="C66" s="3"/>
+      <c r="D66" s="3"/>
+      <c r="E66" s="3"/>
+      <c r="F66" s="3"/>
+      <c r="G66" s="3"/>
+      <c r="J66" s="4"/>
+    </row>
+    <row r="67" spans="2:10" x14ac:dyDescent="0.2">
+      <c r="B67" s="3"/>
+      <c r="C67" s="3"/>
+      <c r="D67" s="3"/>
+      <c r="E67" s="3"/>
+      <c r="F67" s="3"/>
+      <c r="G67" s="3"/>
+      <c r="J67" s="4"/>
+    </row>
+    <row r="68" spans="2:10" x14ac:dyDescent="0.2">
+      <c r="B68" s="3"/>
+      <c r="C68" s="3"/>
+      <c r="D68" s="3"/>
+      <c r="E68" s="3"/>
+      <c r="F68" s="3"/>
+      <c r="G68" s="3"/>
+      <c r="J68" s="4"/>
+    </row>
+    <row r="69" spans="2:10" x14ac:dyDescent="0.2">
+      <c r="B69" s="3"/>
+      <c r="C69" s="3"/>
+      <c r="D69" s="3"/>
+      <c r="E69" s="3"/>
+      <c r="F69" s="3"/>
+      <c r="G69" s="3"/>
+      <c r="J69" s="4"/>
+    </row>
+    <row r="70" spans="2:10" x14ac:dyDescent="0.2">
+      <c r="B70" s="3"/>
+      <c r="C70" s="3"/>
+      <c r="D70" s="3"/>
+      <c r="E70" s="3"/>
+      <c r="F70" s="3"/>
+      <c r="G70" s="3"/>
+      <c r="J70" s="4"/>
+    </row>
+    <row r="71" spans="2:10" x14ac:dyDescent="0.2">
+      <c r="B71" s="3"/>
+      <c r="C71" s="3"/>
+      <c r="D71" s="3"/>
+      <c r="E71" s="3"/>
+      <c r="F71" s="3"/>
+      <c r="G71" s="3"/>
+      <c r="J71" s="4"/>
+    </row>
+    <row r="72" spans="2:10" x14ac:dyDescent="0.2">
+      <c r="B72" s="3"/>
+      <c r="C72" s="3"/>
+      <c r="D72" s="3"/>
+      <c r="E72" s="3"/>
+      <c r="F72" s="3"/>
+      <c r="G72" s="3"/>
+      <c r="J72" s="4"/>
+    </row>
+    <row r="73" spans="2:10" x14ac:dyDescent="0.2">
+      <c r="B73" s="3"/>
+      <c r="C73" s="3"/>
+      <c r="D73" s="3"/>
+      <c r="E73" s="3"/>
+      <c r="F73" s="3"/>
+      <c r="G73" s="3"/>
+      <c r="J73" s="4"/>
+    </row>
+    <row r="74" spans="2:10" x14ac:dyDescent="0.2">
+      <c r="B74" s="3"/>
+      <c r="C74" s="3"/>
+      <c r="D74" s="3"/>
+      <c r="E74" s="3"/>
+      <c r="F74" s="3"/>
+      <c r="G74" s="3"/>
+      <c r="J74" s="4"/>
+    </row>
+    <row r="75" spans="2:10" x14ac:dyDescent="0.2">
+      <c r="B75" s="3"/>
+      <c r="C75" s="3"/>
+      <c r="D75" s="3"/>
+      <c r="E75" s="3"/>
+      <c r="F75" s="3"/>
+      <c r="G75" s="3"/>
+      <c r="J75" s="4"/>
+    </row>
+    <row r="76" spans="2:10" x14ac:dyDescent="0.2">
+      <c r="B76" s="3"/>
+      <c r="C76" s="3"/>
+      <c r="D76" s="3"/>
+      <c r="E76" s="3"/>
+      <c r="F76" s="3"/>
+      <c r="G76" s="3"/>
+      <c r="J76" s="4"/>
+    </row>
+    <row r="77" spans="2:10" x14ac:dyDescent="0.2">
+      <c r="B77" s="3"/>
+      <c r="C77" s="3"/>
+      <c r="D77" s="3"/>
+      <c r="E77" s="3"/>
+      <c r="F77" s="3"/>
+      <c r="G77" s="3"/>
+      <c r="J77" s="4"/>
+    </row>
+    <row r="78" spans="2:10" x14ac:dyDescent="0.2">
+      <c r="B78" s="3"/>
+      <c r="C78" s="3"/>
+      <c r="D78" s="3"/>
+      <c r="E78" s="3"/>
+      <c r="F78" s="3"/>
+      <c r="G78" s="3"/>
+      <c r="J78" s="4"/>
+    </row>
+    <row r="79" spans="2:10" x14ac:dyDescent="0.2">
+      <c r="B79" s="3"/>
+      <c r="C79" s="3"/>
+      <c r="D79" s="3"/>
+      <c r="E79" s="3"/>
+      <c r="F79" s="3"/>
+      <c r="G79" s="3"/>
+      <c r="J79" s="4"/>
+    </row>
+    <row r="80" spans="2:10" x14ac:dyDescent="0.2">
+      <c r="B80" s="3"/>
+      <c r="C80" s="3"/>
+      <c r="D80" s="3"/>
+      <c r="E80" s="3"/>
+      <c r="F80" s="3"/>
+      <c r="G80" s="3"/>
+      <c r="J80" s="4"/>
+    </row>
+    <row r="81" spans="2:10" x14ac:dyDescent="0.2">
+      <c r="B81" s="3"/>
+      <c r="C81" s="3"/>
+      <c r="D81" s="3"/>
+      <c r="E81" s="3"/>
+      <c r="F81" s="3"/>
+      <c r="G81" s="3"/>
+      <c r="J81" s="4"/>
+    </row>
+    <row r="82" spans="2:10" x14ac:dyDescent="0.2">
+      <c r="B82" s="3"/>
+      <c r="C82" s="3"/>
+      <c r="D82" s="3"/>
+      <c r="E82" s="3"/>
+      <c r="F82" s="3"/>
+      <c r="G82" s="3"/>
+      <c r="J82" s="4"/>
+    </row>
+    <row r="83" spans="2:10" x14ac:dyDescent="0.2">
+      <c r="B83" s="3"/>
+      <c r="C83" s="3"/>
+      <c r="D83" s="3"/>
+      <c r="E83" s="3"/>
+      <c r="F83" s="3"/>
+      <c r="G83" s="3"/>
+      <c r="J83" s="4"/>
+    </row>
+    <row r="84" spans="2:10" x14ac:dyDescent="0.2">
+      <c r="B84" s="3"/>
+      <c r="C84" s="3"/>
+      <c r="D84" s="3"/>
+      <c r="E84" s="3"/>
+      <c r="F84" s="3"/>
+      <c r="G84" s="3"/>
+      <c r="J84" s="4"/>
+    </row>
+    <row r="85" spans="2:10" x14ac:dyDescent="0.2">
+      <c r="B85" s="3"/>
+      <c r="C85" s="3"/>
+      <c r="D85" s="3"/>
+      <c r="E85" s="3"/>
+      <c r="F85" s="3"/>
+      <c r="G85" s="3"/>
+      <c r="J85" s="4"/>
+    </row>
+    <row r="86" spans="2:10" x14ac:dyDescent="0.2">
+      <c r="B86" s="3"/>
+      <c r="C86" s="3"/>
+      <c r="D86" s="3"/>
+      <c r="E86" s="3"/>
+      <c r="F86" s="3"/>
+      <c r="G86" s="3"/>
+      <c r="J86" s="4"/>
+    </row>
+    <row r="87" spans="2:10" x14ac:dyDescent="0.2">
+      <c r="B87" s="3"/>
+      <c r="C87" s="3"/>
+      <c r="D87" s="3"/>
+      <c r="E87" s="3"/>
+      <c r="F87" s="3"/>
+      <c r="G87" s="3"/>
+      <c r="J87" s="4"/>
+    </row>
+    <row r="88" spans="2:10" x14ac:dyDescent="0.2">
+      <c r="B88" s="3"/>
+      <c r="C88" s="3"/>
+      <c r="D88" s="3"/>
+      <c r="E88" s="3"/>
+      <c r="F88" s="3"/>
+      <c r="G88" s="3"/>
+      <c r="J88" s="4"/>
+    </row>
+    <row r="89" spans="2:10" x14ac:dyDescent="0.2">
+      <c r="B89" s="3"/>
+      <c r="C89" s="3"/>
+      <c r="D89" s="3"/>
+      <c r="E89" s="3"/>
+      <c r="F89" s="3"/>
+      <c r="G89" s="3"/>
+      <c r="J89" s="4"/>
+    </row>
+    <row r="90" spans="2:10" x14ac:dyDescent="0.2">
+      <c r="B90" s="3"/>
+      <c r="C90" s="3"/>
+      <c r="D90" s="3"/>
+      <c r="E90" s="3"/>
+      <c r="F90" s="3"/>
+      <c r="G90" s="3"/>
+      <c r="J90" s="4"/>
+    </row>
+    <row r="91" spans="2:10" x14ac:dyDescent="0.2">
+      <c r="B91" s="3"/>
+      <c r="C91" s="3"/>
+      <c r="D91" s="3"/>
+      <c r="E91" s="3"/>
+      <c r="F91" s="3"/>
+      <c r="G91" s="3"/>
+      <c r="J91" s="4"/>
+    </row>
+    <row r="92" spans="2:10" x14ac:dyDescent="0.2">
+      <c r="B92" s="3"/>
+      <c r="C92" s="3"/>
+      <c r="D92" s="3"/>
+      <c r="E92" s="3"/>
+      <c r="F92" s="3"/>
+      <c r="G92" s="3"/>
+      <c r="J92" s="4"/>
+    </row>
+    <row r="93" spans="2:10" x14ac:dyDescent="0.2">
+      <c r="B93" s="3"/>
+      <c r="C93" s="3"/>
+      <c r="D93" s="3"/>
+      <c r="E93" s="3"/>
+      <c r="F93" s="3"/>
+      <c r="G93" s="3"/>
+      <c r="J93" s="4"/>
+    </row>
+    <row r="94" spans="2:10" x14ac:dyDescent="0.2">
+      <c r="B94" s="3"/>
+      <c r="C94" s="3"/>
+      <c r="D94" s="3"/>
+      <c r="E94" s="3"/>
+      <c r="F94" s="3"/>
+      <c r="G94" s="3"/>
+      <c r="J94" s="4"/>
+    </row>
+    <row r="95" spans="2:10" x14ac:dyDescent="0.2">
+      <c r="B95" s="3"/>
+      <c r="C95" s="3"/>
+      <c r="D95" s="3"/>
+      <c r="E95" s="3"/>
+      <c r="F95" s="3"/>
+      <c r="G95" s="3"/>
+      <c r="J95" s="4"/>
+    </row>
+    <row r="96" spans="2:10" x14ac:dyDescent="0.2">
+      <c r="B96" s="3"/>
+      <c r="C96" s="3"/>
+      <c r="D96" s="3"/>
+      <c r="E96" s="3"/>
+      <c r="F96" s="3"/>
+      <c r="G96" s="3"/>
+      <c r="J96" s="4"/>
+    </row>
+    <row r="97" spans="2:10" x14ac:dyDescent="0.2">
+      <c r="B97" s="3"/>
+      <c r="C97" s="3"/>
+      <c r="D97" s="3"/>
+      <c r="E97" s="3"/>
+      <c r="F97" s="3"/>
+      <c r="G97" s="3"/>
+      <c r="J97" s="4"/>
+    </row>
+    <row r="98" spans="2:10" x14ac:dyDescent="0.2">
+      <c r="B98" s="3"/>
+      <c r="C98" s="3"/>
+      <c r="D98" s="3"/>
+      <c r="E98" s="3"/>
+      <c r="F98" s="3"/>
+      <c r="G98" s="3"/>
+      <c r="J98" s="4"/>
+    </row>
+    <row r="99" spans="2:10" x14ac:dyDescent="0.2">
+      <c r="B99" s="3"/>
+      <c r="C99" s="3"/>
+      <c r="D99" s="3"/>
+      <c r="E99" s="3"/>
+      <c r="F99" s="3"/>
+      <c r="G99" s="3"/>
+      <c r="J99" s="4"/>
+    </row>
+    <row r="100" spans="2:10" x14ac:dyDescent="0.2">
+      <c r="B100" s="3"/>
+      <c r="C100" s="3"/>
+      <c r="D100" s="3"/>
+      <c r="E100" s="3"/>
+      <c r="F100" s="3"/>
+      <c r="G100" s="3"/>
+      <c r="J100" s="4"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -16458,98 +17100,88 @@
     <mergeCell ref="AG9:AP9"/>
   </mergeCells>
   <conditionalFormatting sqref="F11:K52 AB11:AF52">
-    <cfRule type="expression" dxfId="22" priority="6">
+    <cfRule type="expression" dxfId="20" priority="6">
       <formula>$E11="hb"</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="21" priority="7">
+    <cfRule type="expression" dxfId="19" priority="7">
       <formula>$E11="pow"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="F11:L52">
-    <cfRule type="expression" dxfId="20" priority="19">
+    <cfRule type="expression" dxfId="18" priority="19">
       <formula>$E11="elastic"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="G11:G52">
-    <cfRule type="expression" dxfId="19" priority="8">
+    <cfRule type="expression" dxfId="17" priority="8">
       <formula>$E11="cp"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="H11:I52">
-    <cfRule type="expression" dxfId="18" priority="9">
+    <cfRule type="expression" dxfId="16" priority="9">
       <formula>$E11="mc"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="J11:K52">
-    <cfRule type="expression" dxfId="17" priority="10">
+    <cfRule type="expression" dxfId="15" priority="10">
       <formula>$E11="cp"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="O11:R52">
-    <cfRule type="expression" dxfId="16" priority="4">
+    <cfRule type="expression" dxfId="14" priority="4">
       <formula>$E11="elastic"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="P11:P52">
-    <cfRule type="expression" dxfId="15" priority="13">
+    <cfRule type="expression" dxfId="13" priority="13">
       <formula>AND($O11&lt;&gt;"",$O11&lt;&gt;"ru")</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="Q11:R52">
-    <cfRule type="expression" dxfId="14" priority="3">
+    <cfRule type="expression" dxfId="12" priority="3">
       <formula>$E11="cp"</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="13" priority="5">
+    <cfRule type="expression" dxfId="11" priority="5">
       <formula>AND($O11&lt;&gt;"",$O11&lt;&gt;"piezo",$O11&lt;&gt;"seep")</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="S11:V52">
-    <cfRule type="expression" dxfId="12" priority="11">
+    <cfRule type="expression" dxfId="10" priority="11">
       <formula>AND($E11&lt;&gt;"",$E11&lt;&gt;"pow")</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="W11:Z52">
-    <cfRule type="expression" dxfId="11" priority="12">
+    <cfRule type="expression" dxfId="9" priority="12">
       <formula>AND($E11&lt;&gt;"",$E11&lt;&gt;"hb")</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="AB11:AF52">
-    <cfRule type="expression" dxfId="10" priority="21">
+    <cfRule type="expression" dxfId="8" priority="21">
       <formula>$E11="elastic"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="AC11:AC52">
-    <cfRule type="expression" dxfId="9" priority="14">
+    <cfRule type="expression" dxfId="7" priority="14">
       <formula>$E11="cp"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="AD11:AD52">
-    <cfRule type="expression" dxfId="8" priority="15">
+    <cfRule type="expression" dxfId="6" priority="15">
       <formula>$E11="mc"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="AE11:AF52">
-    <cfRule type="expression" dxfId="7" priority="16">
+    <cfRule type="expression" dxfId="5" priority="16">
       <formula>$E11="cp"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="AK11:AL52">
-    <cfRule type="expression" dxfId="6" priority="17">
+    <cfRule type="expression" dxfId="4" priority="17">
       <formula>OR($AJ11="vg",$AJ11="gard")</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="AM11:AN52">
-    <cfRule type="expression" dxfId="5" priority="18">
-      <formula>$AJ11="lf"</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="AO11:AO52">
-    <cfRule type="expression" dxfId="1" priority="2">
-      <formula>$AJ11="lf"</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="AP11:AP52">
-    <cfRule type="expression" dxfId="0" priority="1">
+  <conditionalFormatting sqref="AM11:AP52">
+    <cfRule type="expression" dxfId="3" priority="1">
       <formula>$AJ11="lf"</formula>
     </cfRule>
   </conditionalFormatting>
@@ -16606,74 +17238,74 @@
       </c>
     </row>
     <row r="4" spans="1:44" x14ac:dyDescent="0.2">
-      <c r="A4" s="53" t="s">
+      <c r="A4" s="55" t="s">
         <v>2</v>
       </c>
-      <c r="B4" s="53"/>
-      <c r="D4" s="53" t="s">
+      <c r="B4" s="55"/>
+      <c r="D4" s="55" t="s">
         <v>5</v>
       </c>
-      <c r="E4" s="53"/>
-      <c r="G4" s="53" t="s">
+      <c r="E4" s="55"/>
+      <c r="G4" s="55" t="s">
         <v>6</v>
       </c>
-      <c r="H4" s="53"/>
-      <c r="J4" s="53" t="s">
+      <c r="H4" s="55"/>
+      <c r="J4" s="55" t="s">
         <v>7</v>
       </c>
-      <c r="K4" s="53"/>
-      <c r="M4" s="53" t="s">
+      <c r="K4" s="55"/>
+      <c r="M4" s="55" t="s">
         <v>8</v>
       </c>
-      <c r="N4" s="53"/>
-      <c r="P4" s="53" t="s">
+      <c r="N4" s="55"/>
+      <c r="P4" s="55" t="s">
         <v>9</v>
       </c>
-      <c r="Q4" s="53"/>
+      <c r="Q4" s="55"/>
       <c r="R4" s="1"/>
-      <c r="S4" s="53" t="s">
+      <c r="S4" s="55" t="s">
         <v>10</v>
       </c>
-      <c r="T4" s="53"/>
+      <c r="T4" s="55"/>
       <c r="U4" s="1"/>
-      <c r="V4" s="53" t="s">
+      <c r="V4" s="55" t="s">
         <v>11</v>
       </c>
-      <c r="W4" s="53"/>
+      <c r="W4" s="55"/>
       <c r="X4" s="1"/>
-      <c r="Y4" s="53" t="s">
+      <c r="Y4" s="55" t="s">
         <v>12</v>
       </c>
-      <c r="Z4" s="53"/>
+      <c r="Z4" s="55"/>
       <c r="AA4" s="1"/>
-      <c r="AB4" s="53" t="s">
+      <c r="AB4" s="55" t="s">
         <v>13</v>
       </c>
-      <c r="AC4" s="53"/>
-      <c r="AE4" s="53" t="s">
+      <c r="AC4" s="55"/>
+      <c r="AE4" s="55" t="s">
         <v>108</v>
       </c>
-      <c r="AF4" s="53"/>
+      <c r="AF4" s="55"/>
       <c r="AG4" s="1"/>
-      <c r="AH4" s="53" t="s">
+      <c r="AH4" s="55" t="s">
         <v>109</v>
       </c>
-      <c r="AI4" s="53"/>
+      <c r="AI4" s="55"/>
       <c r="AJ4" s="1"/>
-      <c r="AK4" s="53" t="s">
+      <c r="AK4" s="55" t="s">
         <v>110</v>
       </c>
-      <c r="AL4" s="53"/>
+      <c r="AL4" s="55"/>
       <c r="AM4" s="1"/>
-      <c r="AN4" s="53" t="s">
+      <c r="AN4" s="55" t="s">
         <v>111</v>
       </c>
-      <c r="AO4" s="53"/>
+      <c r="AO4" s="55"/>
       <c r="AP4" s="1"/>
-      <c r="AQ4" s="53" t="s">
+      <c r="AQ4" s="55" t="s">
         <v>112</v>
       </c>
-      <c r="AR4" s="53"/>
+      <c r="AR4" s="55"/>
     </row>
     <row r="5" spans="1:44" x14ac:dyDescent="0.2">
       <c r="A5" s="36" t="s">
@@ -16776,89 +17408,89 @@
       </c>
     </row>
     <row r="6" spans="1:44" x14ac:dyDescent="0.2">
-      <c r="A6" s="54" t="str">
+      <c r="A6" s="53" t="str">
         <f>_xlfn.XLOOKUP(B5,mat!$A:$A, mat!$B:$B,"") &amp; ""</f>
         <v/>
       </c>
-      <c r="B6" s="55"/>
-      <c r="D6" s="54" t="str">
+      <c r="B6" s="54"/>
+      <c r="D6" s="53" t="str">
         <f>_xlfn.XLOOKUP(E5,mat!$A:$A, mat!$B:$B,"") &amp; ""</f>
         <v/>
       </c>
-      <c r="E6" s="55"/>
-      <c r="G6" s="54" t="str">
+      <c r="E6" s="54"/>
+      <c r="G6" s="53" t="str">
         <f>_xlfn.XLOOKUP(H5,mat!$A:$A, mat!$B:$B,"") &amp; ""</f>
         <v/>
       </c>
-      <c r="H6" s="55"/>
-      <c r="J6" s="54" t="str">
+      <c r="H6" s="54"/>
+      <c r="J6" s="53" t="str">
         <f>_xlfn.XLOOKUP(K5,mat!$A:$A, mat!$B:$B,"") &amp; ""</f>
         <v/>
       </c>
-      <c r="K6" s="55"/>
-      <c r="M6" s="54" t="str">
+      <c r="K6" s="54"/>
+      <c r="M6" s="53" t="str">
         <f>_xlfn.XLOOKUP(N5,mat!$A:$A, mat!$B:$B,"") &amp; ""</f>
         <v/>
       </c>
-      <c r="N6" s="55"/>
-      <c r="P6" s="54" t="str">
+      <c r="N6" s="54"/>
+      <c r="P6" s="53" t="str">
         <f>_xlfn.XLOOKUP(Q5,mat!$A:$A, mat!$B:$B,"") &amp; ""</f>
         <v/>
       </c>
-      <c r="Q6" s="55"/>
+      <c r="Q6" s="54"/>
       <c r="R6" s="1"/>
-      <c r="S6" s="54" t="str">
+      <c r="S6" s="53" t="str">
         <f>_xlfn.XLOOKUP(T5,mat!$A:$A, mat!$B:$B,"") &amp; ""</f>
         <v/>
       </c>
-      <c r="T6" s="55"/>
+      <c r="T6" s="54"/>
       <c r="U6" s="1"/>
-      <c r="V6" s="54" t="str">
+      <c r="V6" s="53" t="str">
         <f>_xlfn.XLOOKUP(W5,mat!$A:$A, mat!$B:$B,"") &amp; ""</f>
         <v/>
       </c>
-      <c r="W6" s="55"/>
+      <c r="W6" s="54"/>
       <c r="X6" s="1"/>
-      <c r="Y6" s="54" t="str">
+      <c r="Y6" s="53" t="str">
         <f>_xlfn.XLOOKUP(Z5,mat!$A:$A, mat!$B:$B,"") &amp; ""</f>
         <v/>
       </c>
-      <c r="Z6" s="55"/>
+      <c r="Z6" s="54"/>
       <c r="AA6" s="1"/>
-      <c r="AB6" s="54" t="str">
+      <c r="AB6" s="53" t="str">
         <f>_xlfn.XLOOKUP(AC5,mat!$A:$A, mat!$B:$B,"") &amp; ""</f>
         <v/>
       </c>
-      <c r="AC6" s="55"/>
-      <c r="AE6" s="54" t="str">
+      <c r="AC6" s="54"/>
+      <c r="AE6" s="53" t="str">
         <f>_xlfn.XLOOKUP(AF5,mat!$A:$A, mat!$B:$B,"") &amp; ""</f>
         <v/>
       </c>
-      <c r="AF6" s="55"/>
+      <c r="AF6" s="54"/>
       <c r="AG6" s="1"/>
-      <c r="AH6" s="54" t="str">
+      <c r="AH6" s="53" t="str">
         <f>_xlfn.XLOOKUP(AI5,mat!$A:$A, mat!$B:$B,"") &amp; ""</f>
         <v/>
       </c>
-      <c r="AI6" s="55"/>
+      <c r="AI6" s="54"/>
       <c r="AJ6" s="1"/>
-      <c r="AK6" s="54" t="str">
+      <c r="AK6" s="53" t="str">
         <f>_xlfn.XLOOKUP(AL5,mat!$A:$A, mat!$B:$B,"") &amp; ""</f>
         <v/>
       </c>
-      <c r="AL6" s="55"/>
+      <c r="AL6" s="54"/>
       <c r="AM6" s="1"/>
-      <c r="AN6" s="54" t="str">
+      <c r="AN6" s="53" t="str">
         <f>_xlfn.XLOOKUP(AO5,mat!$A:$A, mat!$B:$B,"") &amp; ""</f>
         <v/>
       </c>
-      <c r="AO6" s="55"/>
+      <c r="AO6" s="54"/>
       <c r="AP6" s="1"/>
-      <c r="AQ6" s="54" t="str">
+      <c r="AQ6" s="53" t="str">
         <f>_xlfn.XLOOKUP(AR5,mat!$A:$A, mat!$B:$B,"") &amp; ""</f>
         <v/>
       </c>
-      <c r="AR6" s="55"/>
+      <c r="AR6" s="54"/>
     </row>
     <row r="7" spans="1:44" x14ac:dyDescent="0.2">
       <c r="A7" s="2" t="s">
@@ -17762,36 +18394,36 @@
     </row>
   </sheetData>
   <mergeCells count="30">
+    <mergeCell ref="A4:B4"/>
+    <mergeCell ref="D4:E4"/>
+    <mergeCell ref="G4:H4"/>
+    <mergeCell ref="J4:K4"/>
+    <mergeCell ref="M4:N4"/>
+    <mergeCell ref="P4:Q4"/>
+    <mergeCell ref="S4:T4"/>
+    <mergeCell ref="V4:W4"/>
+    <mergeCell ref="Y4:Z4"/>
+    <mergeCell ref="AB4:AC4"/>
+    <mergeCell ref="AE4:AF4"/>
+    <mergeCell ref="AH4:AI4"/>
+    <mergeCell ref="AK4:AL4"/>
+    <mergeCell ref="AN4:AO4"/>
+    <mergeCell ref="AQ4:AR4"/>
+    <mergeCell ref="A6:B6"/>
+    <mergeCell ref="D6:E6"/>
+    <mergeCell ref="G6:H6"/>
+    <mergeCell ref="J6:K6"/>
+    <mergeCell ref="M6:N6"/>
+    <mergeCell ref="P6:Q6"/>
+    <mergeCell ref="S6:T6"/>
+    <mergeCell ref="V6:W6"/>
+    <mergeCell ref="Y6:Z6"/>
+    <mergeCell ref="AB6:AC6"/>
     <mergeCell ref="AE6:AF6"/>
     <mergeCell ref="AH6:AI6"/>
     <mergeCell ref="AK6:AL6"/>
     <mergeCell ref="AN6:AO6"/>
     <mergeCell ref="AQ6:AR6"/>
-    <mergeCell ref="P6:Q6"/>
-    <mergeCell ref="S6:T6"/>
-    <mergeCell ref="V6:W6"/>
-    <mergeCell ref="Y6:Z6"/>
-    <mergeCell ref="AB6:AC6"/>
-    <mergeCell ref="A6:B6"/>
-    <mergeCell ref="D6:E6"/>
-    <mergeCell ref="G6:H6"/>
-    <mergeCell ref="J6:K6"/>
-    <mergeCell ref="M6:N6"/>
-    <mergeCell ref="AE4:AF4"/>
-    <mergeCell ref="AH4:AI4"/>
-    <mergeCell ref="AK4:AL4"/>
-    <mergeCell ref="AN4:AO4"/>
-    <mergeCell ref="AQ4:AR4"/>
-    <mergeCell ref="P4:Q4"/>
-    <mergeCell ref="S4:T4"/>
-    <mergeCell ref="V4:W4"/>
-    <mergeCell ref="Y4:Z4"/>
-    <mergeCell ref="AB4:AC4"/>
-    <mergeCell ref="A4:B4"/>
-    <mergeCell ref="D4:E4"/>
-    <mergeCell ref="G4:H4"/>
-    <mergeCell ref="J4:K4"/>
-    <mergeCell ref="M4:N4"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
@@ -17829,74 +18461,74 @@
       </c>
     </row>
     <row r="4" spans="1:44" x14ac:dyDescent="0.2">
-      <c r="A4" s="53" t="s">
+      <c r="A4" s="55" t="s">
         <v>137</v>
       </c>
-      <c r="B4" s="53"/>
-      <c r="D4" s="53" t="s">
+      <c r="B4" s="55"/>
+      <c r="D4" s="55" t="s">
         <v>138</v>
       </c>
-      <c r="E4" s="53"/>
-      <c r="G4" s="53" t="s">
+      <c r="E4" s="55"/>
+      <c r="G4" s="55" t="s">
         <v>139</v>
       </c>
-      <c r="H4" s="53"/>
-      <c r="J4" s="53" t="s">
+      <c r="H4" s="55"/>
+      <c r="J4" s="55" t="s">
         <v>140</v>
       </c>
-      <c r="K4" s="53"/>
-      <c r="M4" s="53" t="s">
+      <c r="K4" s="55"/>
+      <c r="M4" s="55" t="s">
         <v>141</v>
       </c>
-      <c r="N4" s="53"/>
-      <c r="P4" s="53" t="s">
+      <c r="N4" s="55"/>
+      <c r="P4" s="55" t="s">
         <v>142</v>
       </c>
-      <c r="Q4" s="53"/>
+      <c r="Q4" s="55"/>
       <c r="R4" s="1"/>
-      <c r="S4" s="53" t="s">
+      <c r="S4" s="55" t="s">
         <v>143</v>
       </c>
-      <c r="T4" s="53"/>
+      <c r="T4" s="55"/>
       <c r="U4" s="1"/>
-      <c r="V4" s="53" t="s">
+      <c r="V4" s="55" t="s">
         <v>144</v>
       </c>
-      <c r="W4" s="53"/>
+      <c r="W4" s="55"/>
       <c r="X4" s="1"/>
-      <c r="Y4" s="53" t="s">
+      <c r="Y4" s="55" t="s">
         <v>145</v>
       </c>
-      <c r="Z4" s="53"/>
+      <c r="Z4" s="55"/>
       <c r="AA4" s="1"/>
-      <c r="AB4" s="53" t="s">
+      <c r="AB4" s="55" t="s">
         <v>146</v>
       </c>
-      <c r="AC4" s="53"/>
-      <c r="AE4" s="53" t="s">
+      <c r="AC4" s="55"/>
+      <c r="AE4" s="55" t="s">
         <v>147</v>
       </c>
-      <c r="AF4" s="53"/>
+      <c r="AF4" s="55"/>
       <c r="AG4" s="1"/>
-      <c r="AH4" s="53" t="s">
+      <c r="AH4" s="55" t="s">
         <v>148</v>
       </c>
-      <c r="AI4" s="53"/>
+      <c r="AI4" s="55"/>
       <c r="AJ4" s="1"/>
-      <c r="AK4" s="53" t="s">
+      <c r="AK4" s="55" t="s">
         <v>149</v>
       </c>
-      <c r="AL4" s="53"/>
+      <c r="AL4" s="55"/>
       <c r="AM4" s="1"/>
-      <c r="AN4" s="53" t="s">
+      <c r="AN4" s="55" t="s">
         <v>150</v>
       </c>
-      <c r="AO4" s="53"/>
+      <c r="AO4" s="55"/>
       <c r="AP4" s="1"/>
-      <c r="AQ4" s="53" t="s">
+      <c r="AQ4" s="55" t="s">
         <v>151</v>
       </c>
-      <c r="AR4" s="53"/>
+      <c r="AR4" s="55"/>
     </row>
     <row r="5" spans="1:44" x14ac:dyDescent="0.2">
       <c r="A5" s="38" t="s">
@@ -18985,14 +19617,12 @@
     </row>
   </sheetData>
   <mergeCells count="30">
-    <mergeCell ref="AN6:AO6"/>
-    <mergeCell ref="AQ6:AR6"/>
-    <mergeCell ref="V6:W6"/>
-    <mergeCell ref="Y6:Z6"/>
-    <mergeCell ref="AB6:AC6"/>
-    <mergeCell ref="AE6:AF6"/>
-    <mergeCell ref="AH6:AI6"/>
-    <mergeCell ref="AK6:AL6"/>
+    <mergeCell ref="P4:Q4"/>
+    <mergeCell ref="A4:B4"/>
+    <mergeCell ref="D4:E4"/>
+    <mergeCell ref="G4:H4"/>
+    <mergeCell ref="J4:K4"/>
+    <mergeCell ref="M4:N4"/>
     <mergeCell ref="AK4:AL4"/>
     <mergeCell ref="AN4:AO4"/>
     <mergeCell ref="AQ4:AR4"/>
@@ -19009,12 +19639,14 @@
     <mergeCell ref="AB4:AC4"/>
     <mergeCell ref="AE4:AF4"/>
     <mergeCell ref="AH4:AI4"/>
-    <mergeCell ref="P4:Q4"/>
-    <mergeCell ref="A4:B4"/>
-    <mergeCell ref="D4:E4"/>
-    <mergeCell ref="G4:H4"/>
-    <mergeCell ref="J4:K4"/>
-    <mergeCell ref="M4:N4"/>
+    <mergeCell ref="AN6:AO6"/>
+    <mergeCell ref="AQ6:AR6"/>
+    <mergeCell ref="V6:W6"/>
+    <mergeCell ref="Y6:Z6"/>
+    <mergeCell ref="AB6:AC6"/>
+    <mergeCell ref="AE6:AF6"/>
+    <mergeCell ref="AH6:AI6"/>
+    <mergeCell ref="AK6:AL6"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
@@ -19405,17 +20037,17 @@
     </row>
   </sheetData>
   <conditionalFormatting sqref="E3:E42">
-    <cfRule type="expression" dxfId="4" priority="3">
+    <cfRule type="expression" dxfId="2" priority="3">
       <formula>OR($D3="Intercept", $D3="Radius")</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="F3:G42">
-    <cfRule type="expression" dxfId="3" priority="2">
+    <cfRule type="expression" dxfId="1" priority="2">
       <formula>OR($D3="Depth",$D3="Radius")</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="H3:H42">
-    <cfRule type="expression" dxfId="2" priority="1">
+    <cfRule type="expression" dxfId="0" priority="1">
       <formula>OR($D3="Depth",$D3="Intercept")</formula>
     </cfRule>
   </conditionalFormatting>

</xml_diff>

<commit_message>
template(v18): 'reservoir' joins the seep bc type dropdowns (both sheets)
Norm-approved Option B vocabulary: 'reservoir' will carry the submerged-only
falling-stage behavior; series-driven 'head' becomes a plain time-varying fixed
head. Dropdown item only in this commit — surgical XML edit (sheet14/15 T6 +
validation range + one shared string; byte-diff proven, all other members
byte-identical). Parser/solver/docs/Studio/corpus re-emit land as one batch
after the running verification wave releases the solver.

Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_0147GB4LGVZuqGHCRMVzZTsR
</commit_message>
<xml_diff>
--- a/docs/inputs/input_template.xlsx
+++ b/docs/inputs/input_template.xlsx
@@ -63,7 +63,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="478" uniqueCount="265">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="480" uniqueCount="266">
   <si>
     <t>X</t>
   </si>
@@ -1023,6 +1023,9 @@
   </si>
   <si>
     <t>save_times</t>
+  </si>
+  <si>
+    <t>reservoir</t>
   </si>
 </sst>
 </file>
@@ -13805,7 +13808,9 @@
       <c r="O6" s="3"/>
       <c r="Q6" s="3"/>
       <c r="R6" s="3"/>
-      <c r="T6" s="1"/>
+      <c r="T6" s="1" t="s">
+        <v>265</v>
+      </c>
       <c r="U6" s="9"/>
     </row>
     <row r="7" spans="2:21" x14ac:dyDescent="0.2">
@@ -14071,7 +14076,7 @@
   </mergeCells>
   <dataValidations count="1">
     <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="E3 H3 K3 N3 Q3" xr:uid="{21F200C9-4829-4345-9958-0F754F272AD0}">
-      <formula1>$T$4:$T$5</formula1>
+      <formula1>$T$4:$T$6</formula1>
     </dataValidation>
   </dataValidations>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -14221,6 +14226,9 @@
       <c r="O6" s="3"/>
       <c r="Q6" s="3"/>
       <c r="R6" s="3"/>
+      <c r="T6" s="1" t="s">
+        <v>265</v>
+      </c>
     </row>
     <row r="7" spans="2:21" x14ac:dyDescent="0.2">
       <c r="B7" s="3"/>
@@ -14485,7 +14493,7 @@
   </mergeCells>
   <dataValidations count="1">
     <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="E3 H3 K3 N3 Q3" xr:uid="{68C61D93-1721-F843-8E53-0F0E50006C65}">
-      <formula1>$T$4:$T$5</formula1>
+      <formula1>$T$4:$T$6</formula1>
     </dataValidation>
   </dataValidations>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>

<commit_message>
template(v18): seep bc (2) dropdown loses 'reservoir' — set 2 is the steady stage-2 drawdown set (Norm)
The second BC set exists solely for stage 2 of classic rapid drawdown, which is
by definition steady: no reservoir type, no series bindings. Surgical revert of
the T6 item + validation range on sheet15 only (byte-diff proven); the main
seep bc sheet keeps head/flux/reservoir. fileio-side loud validation lands with
the in-flight BC-symbology agent.

Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_0147GB4LGVZuqGHCRMVzZTsR
</commit_message>
<xml_diff>
--- a/docs/inputs/input_template.xlsx
+++ b/docs/inputs/input_template.xlsx
@@ -14226,9 +14226,6 @@
       <c r="O6" s="3"/>
       <c r="Q6" s="3"/>
       <c r="R6" s="3"/>
-      <c r="T6" s="1" t="s">
-        <v>265</v>
-      </c>
     </row>
     <row r="7" spans="2:21" x14ac:dyDescent="0.2">
       <c r="B7" s="3"/>
@@ -14493,7 +14490,7 @@
   </mergeCells>
   <dataValidations count="1">
     <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="E3 H3 K3 N3 Q3" xr:uid="{68C61D93-1721-F843-8E53-0F0E50006C65}">
-      <formula1>$T$4:$T$6</formula1>
+      <formula1>$T$4:$T$5</formula1>
     </dataValidation>
   </dataValidations>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>

<commit_message>
template(v20): SSR zones become polygon overlays — sentinel ids, mat flag retired (Norm)
Owner's edits: main!D5 = 20; mat column O (ssr_zone flag, v19, never released)
deleted — Excel re-merged the elastic graying into a two-range rule, all 18
v18 rule semantics verified present with ranges shifted back; polygon-sheet
row-6 echo formulas now display the sentinel codes (-1 'SSR reduce',
-2 'SSR hold', -3 'SSR elastic') and fall through to the material-name lookup
for positive ids. Zones are analysis overlays: never meshed, never material
regions — the design ruling that ends the zone question.

Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_0147GB4LGVZuqGHCRMVzZTsR
</commit_message>
<xml_diff>
--- a/docs/inputs/input_template.xlsx
+++ b/docs/inputs/input_template.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/njones/python_projects/xslope/docs/inputs/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{807E244B-733A-DD48-859C-6A1D7FF99A48}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CA8D9778-BA48-644C-980F-473DF9F954B0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="620" windowWidth="34200" windowHeight="19900" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -458,9 +458,6 @@
     <t>nu</t>
   </si>
   <si>
-    <t>ssr_zone</t>
-  </si>
-  <si>
     <t>u</t>
   </si>
   <si>
@@ -972,6 +969,9 @@
   </si>
   <si>
     <t>corps</t>
+  </si>
+  <si>
+    <t>Mat ID = -1 --&gt; SSR reduce, Mat ID = -2 --&gt; SSR hold, Mat ID = -3 --&gt; SSR elastic</t>
   </si>
 </sst>
 </file>
@@ -1479,11 +1479,18 @@
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="21">
+  <dxfs count="20">
     <dxf>
       <fill>
         <patternFill>
-          <bgColor theme="1" tint="0.499984740745262"/>
+          <bgColor theme="0" tint="-0.499984740745262"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="0" tint="-0.499984740745262"/>
         </patternFill>
       </fill>
     </dxf>
@@ -1504,21 +1511,7 @@
     <dxf>
       <fill>
         <patternFill>
-          <bgColor theme="0" tint="-0.499984740745262"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor theme="0" tint="-0.499984740745262"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor theme="0" tint="-0.499984740745262"/>
+          <bgColor theme="1" tint="0.499984740745262"/>
         </patternFill>
       </fill>
     </dxf>
@@ -8972,7 +8965,7 @@
         <v>13</v>
       </c>
       <c r="D5" s="30">
-        <v>19</v>
+        <v>20</v>
       </c>
     </row>
     <row r="7" spans="1:7" x14ac:dyDescent="0.2">
@@ -9256,7 +9249,7 @@
     </row>
     <row r="67" spans="4:4" x14ac:dyDescent="0.2">
       <c r="D67" s="1" t="s">
-        <v>303</v>
+        <v>302</v>
       </c>
     </row>
     <row r="68" spans="4:4" x14ac:dyDescent="0.2">
@@ -9355,90 +9348,90 @@
   <sheetData>
     <row r="2" spans="2:24" x14ac:dyDescent="0.2">
       <c r="B2" s="63" t="s">
-        <v>245</v>
+        <v>244</v>
       </c>
       <c r="C2" s="62"/>
       <c r="D2" s="62"/>
       <c r="F2" s="63" t="s">
-        <v>246</v>
+        <v>245</v>
       </c>
       <c r="G2" s="62"/>
       <c r="H2" s="62"/>
       <c r="J2" s="63" t="s">
-        <v>247</v>
+        <v>246</v>
       </c>
       <c r="K2" s="62"/>
       <c r="L2" s="62"/>
       <c r="N2" s="63" t="s">
-        <v>248</v>
+        <v>247</v>
       </c>
       <c r="O2" s="62"/>
       <c r="P2" s="62"/>
       <c r="R2" s="63" t="s">
-        <v>249</v>
+        <v>248</v>
       </c>
       <c r="S2" s="62"/>
       <c r="T2" s="62"/>
       <c r="V2" s="63" t="s">
-        <v>250</v>
+        <v>249</v>
       </c>
       <c r="W2" s="62"/>
       <c r="X2" s="62"/>
     </row>
     <row r="3" spans="2:24" x14ac:dyDescent="0.2">
       <c r="B3" s="2" t="s">
+        <v>228</v>
+      </c>
+      <c r="C3" s="2" t="s">
         <v>229</v>
       </c>
-      <c r="C3" s="2" t="s">
-        <v>230</v>
-      </c>
       <c r="D3" s="2" t="s">
-        <v>244</v>
+        <v>243</v>
       </c>
       <c r="F3" s="2" t="s">
+        <v>228</v>
+      </c>
+      <c r="G3" s="2" t="s">
         <v>229</v>
       </c>
-      <c r="G3" s="2" t="s">
-        <v>230</v>
-      </c>
       <c r="H3" s="2" t="s">
-        <v>244</v>
+        <v>243</v>
       </c>
       <c r="J3" s="2" t="s">
+        <v>228</v>
+      </c>
+      <c r="K3" s="2" t="s">
         <v>229</v>
       </c>
-      <c r="K3" s="2" t="s">
-        <v>230</v>
-      </c>
       <c r="L3" s="2" t="s">
-        <v>244</v>
+        <v>243</v>
       </c>
       <c r="N3" s="2" t="s">
+        <v>228</v>
+      </c>
+      <c r="O3" s="2" t="s">
         <v>229</v>
       </c>
-      <c r="O3" s="2" t="s">
-        <v>230</v>
-      </c>
       <c r="P3" s="2" t="s">
-        <v>244</v>
+        <v>243</v>
       </c>
       <c r="R3" s="2" t="s">
+        <v>228</v>
+      </c>
+      <c r="S3" s="2" t="s">
         <v>229</v>
       </c>
-      <c r="S3" s="2" t="s">
-        <v>230</v>
-      </c>
       <c r="T3" s="2" t="s">
-        <v>244</v>
+        <v>243</v>
       </c>
       <c r="V3" s="2" t="s">
+        <v>228</v>
+      </c>
+      <c r="W3" s="2" t="s">
         <v>229</v>
       </c>
-      <c r="W3" s="2" t="s">
-        <v>230</v>
-      </c>
       <c r="X3" s="2" t="s">
-        <v>244</v>
+        <v>243</v>
       </c>
     </row>
     <row r="4" spans="2:24" x14ac:dyDescent="0.2">
@@ -9823,12 +9816,12 @@
     </row>
   </sheetData>
   <mergeCells count="6">
+    <mergeCell ref="B2:D2"/>
     <mergeCell ref="V2:X2"/>
     <mergeCell ref="J2:L2"/>
     <mergeCell ref="N2:P2"/>
     <mergeCell ref="R2:T2"/>
     <mergeCell ref="F2:H2"/>
-    <mergeCell ref="B2:D2"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
@@ -9849,67 +9842,67 @@
   <sheetData>
     <row r="2" spans="1:28" x14ac:dyDescent="0.2">
       <c r="A2" s="12" t="s">
-        <v>204</v>
+        <v>203</v>
       </c>
       <c r="B2" s="12" t="s">
+        <v>250</v>
+      </c>
+      <c r="C2" s="12" t="s">
         <v>251</v>
       </c>
-      <c r="C2" s="12" t="s">
+      <c r="D2" s="12" t="s">
         <v>252</v>
       </c>
-      <c r="D2" s="12" t="s">
+      <c r="E2" s="12" t="s">
         <v>253</v>
       </c>
-      <c r="E2" s="12" t="s">
+      <c r="F2" s="12" t="s">
         <v>254</v>
       </c>
-      <c r="F2" s="12" t="s">
+      <c r="G2" s="40" t="s">
         <v>255</v>
       </c>
-      <c r="G2" s="40" t="s">
+      <c r="H2" s="40" t="s">
         <v>256</v>
       </c>
-      <c r="H2" s="40" t="s">
+      <c r="I2" s="40" t="s">
         <v>257</v>
       </c>
-      <c r="I2" s="40" t="s">
+      <c r="J2" s="27" t="s">
         <v>258</v>
       </c>
-      <c r="J2" s="27" t="s">
+      <c r="K2" s="27" t="s">
         <v>259</v>
       </c>
-      <c r="K2" s="27" t="s">
+      <c r="L2" s="27" t="s">
         <v>260</v>
       </c>
-      <c r="L2" s="27" t="s">
+      <c r="M2" s="27" t="s">
         <v>261</v>
       </c>
-      <c r="M2" s="27" t="s">
+      <c r="N2" s="27" t="s">
         <v>262</v>
       </c>
-      <c r="N2" s="27" t="s">
+      <c r="O2" s="27" t="s">
         <v>263</v>
       </c>
-      <c r="O2" s="27" t="s">
+      <c r="P2" s="28" t="s">
         <v>264</v>
-      </c>
-      <c r="P2" s="28" t="s">
-        <v>265</v>
       </c>
       <c r="Q2" s="28" t="s">
         <v>130</v>
       </c>
       <c r="R2" s="28" t="s">
+        <v>265</v>
+      </c>
+      <c r="Z2" t="s">
         <v>266</v>
       </c>
-      <c r="Z2" t="s">
+      <c r="AA2" t="s">
         <v>267</v>
       </c>
-      <c r="AA2" t="s">
+      <c r="AB2" t="s">
         <v>268</v>
-      </c>
-      <c r="AB2" t="s">
-        <v>269</v>
       </c>
     </row>
     <row r="3" spans="1:28" x14ac:dyDescent="0.2">
@@ -9940,13 +9933,13 @@
       <c r="Q3" s="3"/>
       <c r="R3" s="3"/>
       <c r="Z3" t="s">
+        <v>269</v>
+      </c>
+      <c r="AA3" t="s">
         <v>270</v>
       </c>
-      <c r="AA3" t="s">
+      <c r="AB3" t="s">
         <v>271</v>
-      </c>
-      <c r="AB3" t="s">
-        <v>272</v>
       </c>
     </row>
     <row r="4" spans="1:28" x14ac:dyDescent="0.2">
@@ -9977,7 +9970,7 @@
       <c r="Q4" s="3"/>
       <c r="R4" s="3"/>
       <c r="Z4" t="s">
-        <v>273</v>
+        <v>272</v>
       </c>
     </row>
     <row r="5" spans="1:28" x14ac:dyDescent="0.2">
@@ -10008,7 +10001,7 @@
       <c r="Q5" s="3"/>
       <c r="R5" s="3"/>
       <c r="Z5" t="s">
-        <v>274</v>
+        <v>273</v>
       </c>
     </row>
     <row r="6" spans="1:28" x14ac:dyDescent="0.2">
@@ -10095,13 +10088,13 @@
       <c r="Q8" s="3"/>
       <c r="R8" s="3"/>
       <c r="Z8" t="s">
+        <v>266</v>
+      </c>
+      <c r="AA8" t="s">
         <v>267</v>
       </c>
-      <c r="AA8" t="s">
+      <c r="AB8" t="s">
         <v>268</v>
-      </c>
-      <c r="AB8" t="s">
-        <v>269</v>
       </c>
     </row>
     <row r="9" spans="1:28" x14ac:dyDescent="0.2">
@@ -10132,13 +10125,13 @@
       <c r="Q9" s="3"/>
       <c r="R9" s="3"/>
       <c r="Z9" t="s">
+        <v>269</v>
+      </c>
+      <c r="AA9" t="s">
         <v>270</v>
       </c>
-      <c r="AA9" t="s">
+      <c r="AB9" t="s">
         <v>271</v>
-      </c>
-      <c r="AB9" t="s">
-        <v>272</v>
       </c>
     </row>
     <row r="10" spans="1:28" x14ac:dyDescent="0.2">
@@ -10169,13 +10162,13 @@
       <c r="Q10" s="3"/>
       <c r="R10" s="3"/>
       <c r="Z10" t="s">
-        <v>273</v>
+        <v>272</v>
       </c>
       <c r="AA10" t="s">
-        <v>271</v>
+        <v>270</v>
       </c>
       <c r="AB10" t="s">
-        <v>269</v>
+        <v>268</v>
       </c>
     </row>
     <row r="11" spans="1:28" x14ac:dyDescent="0.2">
@@ -10206,13 +10199,13 @@
       <c r="Q11" s="3"/>
       <c r="R11" s="3"/>
       <c r="Z11" t="s">
-        <v>274</v>
+        <v>273</v>
       </c>
       <c r="AA11" t="s">
-        <v>271</v>
+        <v>270</v>
       </c>
       <c r="AB11" t="s">
-        <v>269</v>
+        <v>268</v>
       </c>
     </row>
     <row r="12" spans="1:28" x14ac:dyDescent="0.2">
@@ -10576,61 +10569,61 @@
   <sheetData>
     <row r="2" spans="1:27" x14ac:dyDescent="0.2">
       <c r="A2" s="12" t="s">
-        <v>204</v>
+        <v>203</v>
       </c>
       <c r="B2" s="12" t="s">
+        <v>250</v>
+      </c>
+      <c r="C2" s="12" t="s">
         <v>251</v>
       </c>
-      <c r="C2" s="12" t="s">
+      <c r="D2" s="12" t="s">
         <v>252</v>
       </c>
-      <c r="D2" s="12" t="s">
+      <c r="E2" s="12" t="s">
         <v>253</v>
       </c>
-      <c r="E2" s="12" t="s">
+      <c r="F2" s="12" t="s">
         <v>254</v>
       </c>
-      <c r="F2" s="12" t="s">
-        <v>255</v>
-      </c>
       <c r="G2" s="40" t="s">
+        <v>274</v>
+      </c>
+      <c r="H2" s="40" t="s">
         <v>275</v>
       </c>
-      <c r="H2" s="40" t="s">
+      <c r="I2" s="40" t="s">
+        <v>257</v>
+      </c>
+      <c r="J2" s="27" t="s">
         <v>276</v>
       </c>
-      <c r="I2" s="40" t="s">
-        <v>258</v>
-      </c>
-      <c r="J2" s="27" t="s">
+      <c r="K2" s="27" t="s">
         <v>277</v>
       </c>
-      <c r="K2" s="27" t="s">
+      <c r="L2" s="41" t="s">
         <v>278</v>
       </c>
-      <c r="L2" s="41" t="s">
+      <c r="M2" s="41" t="s">
         <v>279</v>
-      </c>
-      <c r="M2" s="41" t="s">
-        <v>280</v>
       </c>
       <c r="N2" s="28" t="s">
         <v>130</v>
       </c>
       <c r="O2" s="28" t="s">
+        <v>280</v>
+      </c>
+      <c r="P2" s="28" t="s">
+        <v>265</v>
+      </c>
+      <c r="Q2" s="28" t="s">
         <v>281</v>
       </c>
-      <c r="P2" s="28" t="s">
-        <v>266</v>
-      </c>
-      <c r="Q2" s="28" t="s">
-        <v>282</v>
-      </c>
       <c r="Z2" t="s">
-        <v>232</v>
+        <v>231</v>
       </c>
       <c r="AA2" t="s">
-        <v>269</v>
+        <v>268</v>
       </c>
     </row>
     <row r="3" spans="1:27" x14ac:dyDescent="0.2">
@@ -10654,10 +10647,10 @@
       <c r="P3" s="3"/>
       <c r="Q3" s="3"/>
       <c r="Z3" t="s">
-        <v>236</v>
+        <v>235</v>
       </c>
       <c r="AA3" t="s">
-        <v>272</v>
+        <v>271</v>
       </c>
     </row>
     <row r="4" spans="1:27" x14ac:dyDescent="0.2">
@@ -10900,22 +10893,22 @@
   <sheetData>
     <row r="2" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A2" s="12" t="s">
-        <v>204</v>
+        <v>203</v>
       </c>
       <c r="B2" s="12" t="s">
-        <v>251</v>
+        <v>250</v>
       </c>
       <c r="C2" s="12" t="s">
+        <v>177</v>
+      </c>
+      <c r="D2" s="12" t="s">
         <v>178</v>
       </c>
-      <c r="D2" s="12" t="s">
-        <v>179</v>
-      </c>
       <c r="E2" s="12" t="s">
+        <v>282</v>
+      </c>
+      <c r="F2" s="12" t="s">
         <v>283</v>
-      </c>
-      <c r="F2" s="12" t="s">
-        <v>284</v>
       </c>
     </row>
     <row r="3" spans="1:6" x14ac:dyDescent="0.2">
@@ -11138,27 +11131,27 @@
   <sheetData>
     <row r="2" spans="2:21" x14ac:dyDescent="0.2">
       <c r="B2" s="64" t="s">
-        <v>285</v>
+        <v>284</v>
       </c>
       <c r="C2" s="65"/>
       <c r="E2" s="59" t="s">
-        <v>286</v>
+        <v>285</v>
       </c>
       <c r="F2" s="54"/>
       <c r="H2" s="59" t="s">
-        <v>287</v>
+        <v>286</v>
       </c>
       <c r="I2" s="54"/>
       <c r="K2" s="59" t="s">
-        <v>288</v>
+        <v>287</v>
       </c>
       <c r="L2" s="54"/>
       <c r="N2" s="59" t="s">
-        <v>289</v>
+        <v>288</v>
       </c>
       <c r="O2" s="54"/>
       <c r="Q2" s="59" t="s">
-        <v>290</v>
+        <v>289</v>
       </c>
       <c r="R2" s="54"/>
     </row>
@@ -11166,71 +11159,71 @@
       <c r="B3" s="66"/>
       <c r="C3" s="67"/>
       <c r="E3" s="32" t="s">
-        <v>291</v>
+        <v>290</v>
       </c>
       <c r="F3" s="33"/>
       <c r="H3" s="32" t="s">
-        <v>291</v>
+        <v>290</v>
       </c>
       <c r="I3" s="33"/>
       <c r="K3" s="32" t="s">
-        <v>291</v>
+        <v>290</v>
       </c>
       <c r="L3" s="33"/>
       <c r="N3" s="32" t="s">
-        <v>291</v>
+        <v>290</v>
       </c>
       <c r="O3" s="33"/>
       <c r="Q3" s="32" t="s">
-        <v>291</v>
+        <v>290</v>
       </c>
       <c r="R3" s="33"/>
       <c r="T3" s="6" t="s">
-        <v>292</v>
+        <v>291</v>
       </c>
     </row>
     <row r="4" spans="2:21" x14ac:dyDescent="0.2">
       <c r="B4" s="25" t="s">
+        <v>177</v>
+      </c>
+      <c r="C4" s="25" t="s">
         <v>178</v>
       </c>
-      <c r="C4" s="25" t="s">
-        <v>179</v>
-      </c>
       <c r="E4" s="25" t="s">
+        <v>177</v>
+      </c>
+      <c r="F4" s="25" t="s">
         <v>178</v>
       </c>
-      <c r="F4" s="25" t="s">
-        <v>179</v>
-      </c>
       <c r="H4" s="25" t="s">
+        <v>177</v>
+      </c>
+      <c r="I4" s="25" t="s">
         <v>178</v>
       </c>
-      <c r="I4" s="25" t="s">
-        <v>179</v>
-      </c>
       <c r="K4" s="25" t="s">
+        <v>177</v>
+      </c>
+      <c r="L4" s="25" t="s">
         <v>178</v>
       </c>
-      <c r="L4" s="25" t="s">
-        <v>179</v>
-      </c>
       <c r="N4" s="25" t="s">
+        <v>177</v>
+      </c>
+      <c r="O4" s="25" t="s">
         <v>178</v>
       </c>
-      <c r="O4" s="25" t="s">
-        <v>179</v>
-      </c>
       <c r="Q4" s="25" t="s">
+        <v>177</v>
+      </c>
+      <c r="R4" s="25" t="s">
         <v>178</v>
       </c>
-      <c r="R4" s="25" t="s">
-        <v>179</v>
-      </c>
       <c r="T4" s="1" t="s">
-        <v>291</v>
+        <v>290</v>
       </c>
       <c r="U4" t="s">
-        <v>293</v>
+        <v>292</v>
       </c>
     </row>
     <row r="5" spans="2:21" x14ac:dyDescent="0.2">
@@ -11247,10 +11240,10 @@
       <c r="Q5" s="3"/>
       <c r="R5" s="3"/>
       <c r="T5" s="1" t="s">
+        <v>293</v>
+      </c>
+      <c r="U5" t="s">
         <v>294</v>
-      </c>
-      <c r="U5" t="s">
-        <v>295</v>
       </c>
     </row>
     <row r="6" spans="2:21" x14ac:dyDescent="0.2">
@@ -11267,7 +11260,7 @@
       <c r="Q6" s="3"/>
       <c r="R6" s="3"/>
       <c r="T6" s="1" t="s">
-        <v>296</v>
+        <v>295</v>
       </c>
       <c r="U6" s="9"/>
     </row>
@@ -11556,27 +11549,27 @@
   <sheetData>
     <row r="2" spans="2:21" x14ac:dyDescent="0.2">
       <c r="B2" s="68" t="s">
-        <v>297</v>
+        <v>296</v>
       </c>
       <c r="C2" s="65"/>
       <c r="E2" s="60" t="s">
-        <v>298</v>
+        <v>297</v>
       </c>
       <c r="F2" s="54"/>
       <c r="H2" s="60" t="s">
-        <v>299</v>
+        <v>298</v>
       </c>
       <c r="I2" s="54"/>
       <c r="K2" s="60" t="s">
-        <v>300</v>
+        <v>299</v>
       </c>
       <c r="L2" s="54"/>
       <c r="N2" s="60" t="s">
-        <v>301</v>
+        <v>300</v>
       </c>
       <c r="O2" s="54"/>
       <c r="Q2" s="60" t="s">
-        <v>302</v>
+        <v>301</v>
       </c>
       <c r="R2" s="54"/>
     </row>
@@ -11584,71 +11577,71 @@
       <c r="B3" s="66"/>
       <c r="C3" s="67"/>
       <c r="E3" s="34" t="s">
-        <v>291</v>
+        <v>290</v>
       </c>
       <c r="F3" s="35"/>
       <c r="H3" s="34" t="s">
-        <v>291</v>
+        <v>290</v>
       </c>
       <c r="I3" s="35"/>
       <c r="K3" s="34" t="s">
-        <v>291</v>
+        <v>290</v>
       </c>
       <c r="L3" s="35"/>
       <c r="N3" s="34" t="s">
-        <v>291</v>
+        <v>290</v>
       </c>
       <c r="O3" s="35"/>
       <c r="Q3" s="34" t="s">
-        <v>291</v>
+        <v>290</v>
       </c>
       <c r="R3" s="35"/>
       <c r="T3" s="6" t="s">
-        <v>292</v>
+        <v>291</v>
       </c>
     </row>
     <row r="4" spans="2:21" x14ac:dyDescent="0.2">
       <c r="B4" s="25" t="s">
+        <v>177</v>
+      </c>
+      <c r="C4" s="25" t="s">
         <v>178</v>
       </c>
-      <c r="C4" s="25" t="s">
-        <v>179</v>
-      </c>
       <c r="E4" s="25" t="s">
+        <v>177</v>
+      </c>
+      <c r="F4" s="25" t="s">
         <v>178</v>
       </c>
-      <c r="F4" s="25" t="s">
-        <v>179</v>
-      </c>
       <c r="H4" s="25" t="s">
+        <v>177</v>
+      </c>
+      <c r="I4" s="25" t="s">
         <v>178</v>
       </c>
-      <c r="I4" s="25" t="s">
-        <v>179</v>
-      </c>
       <c r="K4" s="25" t="s">
+        <v>177</v>
+      </c>
+      <c r="L4" s="25" t="s">
         <v>178</v>
       </c>
-      <c r="L4" s="25" t="s">
-        <v>179</v>
-      </c>
       <c r="N4" s="25" t="s">
+        <v>177</v>
+      </c>
+      <c r="O4" s="25" t="s">
         <v>178</v>
       </c>
-      <c r="O4" s="25" t="s">
-        <v>179</v>
-      </c>
       <c r="Q4" s="25" t="s">
+        <v>177</v>
+      </c>
+      <c r="R4" s="25" t="s">
         <v>178</v>
       </c>
-      <c r="R4" s="25" t="s">
-        <v>179</v>
-      </c>
       <c r="T4" s="1" t="s">
-        <v>291</v>
+        <v>290</v>
       </c>
       <c r="U4" t="s">
-        <v>293</v>
+        <v>292</v>
       </c>
     </row>
     <row r="5" spans="2:21" x14ac:dyDescent="0.2">
@@ -11665,10 +11658,10 @@
       <c r="Q5" s="3"/>
       <c r="R5" s="3"/>
       <c r="T5" s="1" t="s">
+        <v>293</v>
+      </c>
+      <c r="U5" t="s">
         <v>294</v>
-      </c>
-      <c r="U5" t="s">
-        <v>295</v>
       </c>
     </row>
     <row r="6" spans="2:21" x14ac:dyDescent="0.2">
@@ -12900,52 +12893,52 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
-  <dimension ref="A2:AQ52"/>
+  <dimension ref="A2:AP52"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="7" style="1" customWidth="1"/>
     <col min="2" max="2" width="17.33203125" style="1" customWidth="1"/>
     <col min="3" max="10" width="8.5" style="1" customWidth="1"/>
-    <col min="11" max="42" width="8.5" customWidth="1"/>
+    <col min="11" max="41" width="8.5" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="2" spans="1:43" x14ac:dyDescent="0.2">
+    <row r="2" spans="1:42" x14ac:dyDescent="0.2">
       <c r="C2" s="6" t="s">
         <v>86</v>
       </c>
       <c r="L2" s="6" t="s">
         <v>87</v>
       </c>
-      <c r="P2" s="6" t="s">
+      <c r="O2" s="6" t="s">
         <v>88</v>
       </c>
-      <c r="AE2" s="6"/>
-      <c r="AK2" s="6" t="s">
+      <c r="AD2" s="6"/>
+      <c r="AJ2" s="6" t="s">
         <v>89</v>
       </c>
     </row>
-    <row r="3" spans="1:43" x14ac:dyDescent="0.2">
+    <row r="3" spans="1:42" x14ac:dyDescent="0.2">
       <c r="C3" s="1" t="s">
         <v>90</v>
       </c>
       <c r="D3" t="s">
         <v>91</v>
       </c>
-      <c r="P3" s="1" t="s">
+      <c r="O3" s="1" t="s">
         <v>92</v>
       </c>
-      <c r="Q3" t="s">
+      <c r="P3" t="s">
         <v>93</v>
       </c>
-      <c r="AE3" s="14"/>
-      <c r="AK3" s="1" t="s">
+      <c r="AD3" s="14"/>
+      <c r="AJ3" s="1" t="s">
         <v>94</v>
       </c>
-      <c r="AL3" t="s">
+      <c r="AK3" t="s">
         <v>95</v>
       </c>
     </row>
-    <row r="4" spans="1:43" x14ac:dyDescent="0.2">
+    <row r="4" spans="1:42" x14ac:dyDescent="0.2">
       <c r="C4" s="1" t="s">
         <v>96</v>
       </c>
@@ -12956,21 +12949,21 @@
       <c r="M4" t="s">
         <v>98</v>
       </c>
-      <c r="P4" s="1" t="s">
+      <c r="O4" s="1" t="s">
         <v>32</v>
       </c>
-      <c r="Q4" t="s">
+      <c r="P4" t="s">
         <v>99</v>
       </c>
-      <c r="AE4" s="14"/>
-      <c r="AK4" s="1" t="s">
+      <c r="AD4" s="14"/>
+      <c r="AJ4" s="1" t="s">
         <v>100</v>
       </c>
-      <c r="AL4" t="s">
+      <c r="AK4" t="s">
         <v>101</v>
       </c>
     </row>
-    <row r="5" spans="1:43" x14ac:dyDescent="0.2">
+    <row r="5" spans="1:42" x14ac:dyDescent="0.2">
       <c r="C5" s="1" t="s">
         <v>102</v>
       </c>
@@ -12981,21 +12974,21 @@
       <c r="M5" s="9" t="s">
         <v>104</v>
       </c>
-      <c r="P5" s="1" t="s">
+      <c r="O5" s="1" t="s">
         <v>105</v>
       </c>
-      <c r="Q5" s="9" t="s">
+      <c r="P5" s="9" t="s">
         <v>106</v>
       </c>
-      <c r="AE5" s="14"/>
-      <c r="AK5" s="1" t="s">
+      <c r="AD5" s="14"/>
+      <c r="AJ5" s="1" t="s">
         <v>107</v>
       </c>
-      <c r="AL5" s="9" t="s">
+      <c r="AK5" s="9" t="s">
         <v>108</v>
       </c>
     </row>
-    <row r="6" spans="1:43" x14ac:dyDescent="0.2">
+    <row r="6" spans="1:42" x14ac:dyDescent="0.2">
       <c r="C6" s="1" t="s">
         <v>109</v>
       </c>
@@ -13006,26 +12999,26 @@
       <c r="M6" s="9" t="s">
         <v>111</v>
       </c>
-      <c r="P6" s="1" t="s">
+      <c r="O6" s="1" t="s">
         <v>112</v>
       </c>
-      <c r="Q6" t="s">
+      <c r="P6" t="s">
         <v>113</v>
       </c>
+      <c r="AE6" s="1"/>
       <c r="AF6" s="1"/>
-      <c r="AG6" s="1"/>
-    </row>
-    <row r="7" spans="1:43" x14ac:dyDescent="0.2">
+    </row>
+    <row r="7" spans="1:42" x14ac:dyDescent="0.2">
       <c r="C7" s="1" t="s">
         <v>114</v>
       </c>
       <c r="D7" s="9" t="s">
         <v>115</v>
       </c>
+      <c r="AE7" s="1"/>
       <c r="AF7" s="1"/>
-      <c r="AG7" s="1"/>
-    </row>
-    <row r="9" spans="1:43" x14ac:dyDescent="0.2">
+    </row>
+    <row r="9" spans="1:42" x14ac:dyDescent="0.2">
       <c r="C9" s="53" t="s">
         <v>116</v>
       </c>
@@ -13052,18 +13045,18 @@
       <c r="X9" s="54"/>
       <c r="Y9" s="54"/>
       <c r="Z9" s="54"/>
-      <c r="AA9" s="54"/>
-      <c r="AB9" s="53" t="s">
+      <c r="AA9" s="53" t="s">
         <v>117</v>
       </c>
+      <c r="AB9" s="54"/>
       <c r="AC9" s="54"/>
       <c r="AD9" s="54"/>
       <c r="AE9" s="54"/>
       <c r="AF9" s="54"/>
-      <c r="AG9" s="54"/>
-      <c r="AH9" s="53" t="s">
+      <c r="AG9" s="53" t="s">
         <v>118</v>
       </c>
+      <c r="AH9" s="54"/>
       <c r="AI9" s="54"/>
       <c r="AJ9" s="54"/>
       <c r="AK9" s="54"/>
@@ -13072,9 +13065,8 @@
       <c r="AN9" s="54"/>
       <c r="AO9" s="54"/>
       <c r="AP9" s="54"/>
-      <c r="AQ9" s="54"/>
-    </row>
-    <row r="10" spans="1:43" ht="18" customHeight="1" x14ac:dyDescent="0.2">
+    </row>
+    <row r="10" spans="1:42" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A10" s="20" t="s">
         <v>23</v>
       </c>
@@ -13117,14 +13109,14 @@
       <c r="N10" s="43" t="s">
         <v>131</v>
       </c>
-      <c r="O10" s="43" t="s">
+      <c r="O10" s="44" t="s">
         <v>132</v>
       </c>
       <c r="P10" s="44" t="s">
+        <v>112</v>
+      </c>
+      <c r="Q10" s="44" t="s">
         <v>133</v>
-      </c>
-      <c r="Q10" s="44" t="s">
-        <v>112</v>
       </c>
       <c r="R10" s="44" t="s">
         <v>134</v>
@@ -13153,25 +13145,25 @@
       <c r="Z10" s="44" t="s">
         <v>142</v>
       </c>
-      <c r="AA10" s="44" t="s">
+      <c r="AA10" s="46" t="s">
         <v>143</v>
       </c>
       <c r="AB10" s="46" t="s">
         <v>144</v>
       </c>
-      <c r="AC10" s="46" t="s">
+      <c r="AC10" s="47" t="s">
         <v>145</v>
       </c>
-      <c r="AD10" s="47" t="s">
+      <c r="AD10" s="46" t="s">
         <v>146</v>
       </c>
       <c r="AE10" s="46" t="s">
         <v>147</v>
       </c>
-      <c r="AF10" s="46" t="s">
+      <c r="AF10" s="47" t="s">
         <v>148</v>
       </c>
-      <c r="AG10" s="47" t="s">
+      <c r="AG10" s="23" t="s">
         <v>149</v>
       </c>
       <c r="AH10" s="23" t="s">
@@ -13201,11 +13193,8 @@
       <c r="AP10" s="23" t="s">
         <v>158</v>
       </c>
-      <c r="AQ10" s="23" t="s">
-        <v>159</v>
-      </c>
-    </row>
-    <row r="11" spans="1:43" x14ac:dyDescent="0.2">
+    </row>
+    <row r="11" spans="1:42" x14ac:dyDescent="0.2">
       <c r="A11" s="3">
         <v>1</v>
       </c>
@@ -13250,9 +13239,8 @@
       <c r="AN11" s="3"/>
       <c r="AO11" s="3"/>
       <c r="AP11" s="3"/>
-      <c r="AQ11" s="3"/>
-    </row>
-    <row r="12" spans="1:43" x14ac:dyDescent="0.2">
+    </row>
+    <row r="12" spans="1:42" x14ac:dyDescent="0.2">
       <c r="A12" s="3">
         <v>2</v>
       </c>
@@ -13293,13 +13281,12 @@
       <c r="AJ12" s="3"/>
       <c r="AK12" s="3"/>
       <c r="AL12" s="3"/>
-      <c r="AM12" s="3"/>
-      <c r="AN12" s="18"/>
+      <c r="AM12" s="18"/>
+      <c r="AN12" s="19"/>
       <c r="AO12" s="19"/>
       <c r="AP12" s="19"/>
-      <c r="AQ12" s="19"/>
-    </row>
-    <row r="13" spans="1:43" x14ac:dyDescent="0.2">
+    </row>
+    <row r="13" spans="1:42" x14ac:dyDescent="0.2">
       <c r="A13" s="3">
         <v>3</v>
       </c>
@@ -13340,13 +13327,12 @@
       <c r="AJ13" s="3"/>
       <c r="AK13" s="3"/>
       <c r="AL13" s="3"/>
-      <c r="AM13" s="3"/>
-      <c r="AN13" s="18"/>
+      <c r="AM13" s="18"/>
+      <c r="AN13" s="19"/>
       <c r="AO13" s="19"/>
       <c r="AP13" s="19"/>
-      <c r="AQ13" s="19"/>
-    </row>
-    <row r="14" spans="1:43" x14ac:dyDescent="0.2">
+    </row>
+    <row r="14" spans="1:42" x14ac:dyDescent="0.2">
       <c r="A14" s="3">
         <v>4</v>
       </c>
@@ -13391,9 +13377,8 @@
       <c r="AN14" s="3"/>
       <c r="AO14" s="3"/>
       <c r="AP14" s="3"/>
-      <c r="AQ14" s="3"/>
-    </row>
-    <row r="15" spans="1:43" x14ac:dyDescent="0.2">
+    </row>
+    <row r="15" spans="1:42" x14ac:dyDescent="0.2">
       <c r="A15" s="3">
         <v>5</v>
       </c>
@@ -13438,9 +13423,8 @@
       <c r="AN15" s="3"/>
       <c r="AO15" s="3"/>
       <c r="AP15" s="3"/>
-      <c r="AQ15" s="3"/>
-    </row>
-    <row r="16" spans="1:43" x14ac:dyDescent="0.2">
+    </row>
+    <row r="16" spans="1:42" x14ac:dyDescent="0.2">
       <c r="A16" s="3">
         <v>6</v>
       </c>
@@ -13485,9 +13469,8 @@
       <c r="AN16" s="3"/>
       <c r="AO16" s="3"/>
       <c r="AP16" s="3"/>
-      <c r="AQ16" s="3"/>
-    </row>
-    <row r="17" spans="1:43" x14ac:dyDescent="0.2">
+    </row>
+    <row r="17" spans="1:42" x14ac:dyDescent="0.2">
       <c r="A17" s="3">
         <v>7</v>
       </c>
@@ -13532,9 +13515,8 @@
       <c r="AN17" s="3"/>
       <c r="AO17" s="3"/>
       <c r="AP17" s="3"/>
-      <c r="AQ17" s="3"/>
-    </row>
-    <row r="18" spans="1:43" x14ac:dyDescent="0.2">
+    </row>
+    <row r="18" spans="1:42" x14ac:dyDescent="0.2">
       <c r="A18" s="3">
         <v>8</v>
       </c>
@@ -13579,9 +13561,8 @@
       <c r="AN18" s="3"/>
       <c r="AO18" s="3"/>
       <c r="AP18" s="3"/>
-      <c r="AQ18" s="3"/>
-    </row>
-    <row r="19" spans="1:43" x14ac:dyDescent="0.2">
+    </row>
+    <row r="19" spans="1:42" x14ac:dyDescent="0.2">
       <c r="A19" s="3">
         <v>9</v>
       </c>
@@ -13626,9 +13607,8 @@
       <c r="AN19" s="3"/>
       <c r="AO19" s="3"/>
       <c r="AP19" s="3"/>
-      <c r="AQ19" s="3"/>
-    </row>
-    <row r="20" spans="1:43" x14ac:dyDescent="0.2">
+    </row>
+    <row r="20" spans="1:42" x14ac:dyDescent="0.2">
       <c r="A20" s="3">
         <v>10</v>
       </c>
@@ -13673,9 +13653,8 @@
       <c r="AN20" s="3"/>
       <c r="AO20" s="3"/>
       <c r="AP20" s="3"/>
-      <c r="AQ20" s="3"/>
-    </row>
-    <row r="21" spans="1:43" x14ac:dyDescent="0.2">
+    </row>
+    <row r="21" spans="1:42" x14ac:dyDescent="0.2">
       <c r="A21" s="3">
         <v>11</v>
       </c>
@@ -13720,9 +13699,8 @@
       <c r="AN21" s="3"/>
       <c r="AO21" s="3"/>
       <c r="AP21" s="3"/>
-      <c r="AQ21" s="3"/>
-    </row>
-    <row r="22" spans="1:43" x14ac:dyDescent="0.2">
+    </row>
+    <row r="22" spans="1:42" x14ac:dyDescent="0.2">
       <c r="A22" s="3">
         <v>12</v>
       </c>
@@ -13767,9 +13745,8 @@
       <c r="AN22" s="3"/>
       <c r="AO22" s="3"/>
       <c r="AP22" s="3"/>
-      <c r="AQ22" s="3"/>
-    </row>
-    <row r="23" spans="1:43" x14ac:dyDescent="0.2">
+    </row>
+    <row r="23" spans="1:42" x14ac:dyDescent="0.2">
       <c r="A23" s="3">
         <v>13</v>
       </c>
@@ -13814,9 +13791,8 @@
       <c r="AN23" s="3"/>
       <c r="AO23" s="3"/>
       <c r="AP23" s="3"/>
-      <c r="AQ23" s="3"/>
-    </row>
-    <row r="24" spans="1:43" x14ac:dyDescent="0.2">
+    </row>
+    <row r="24" spans="1:42" x14ac:dyDescent="0.2">
       <c r="A24" s="3">
         <v>14</v>
       </c>
@@ -13861,9 +13837,8 @@
       <c r="AN24" s="3"/>
       <c r="AO24" s="3"/>
       <c r="AP24" s="3"/>
-      <c r="AQ24" s="3"/>
-    </row>
-    <row r="25" spans="1:43" x14ac:dyDescent="0.2">
+    </row>
+    <row r="25" spans="1:42" x14ac:dyDescent="0.2">
       <c r="A25" s="3">
         <v>15</v>
       </c>
@@ -13908,9 +13883,8 @@
       <c r="AN25" s="3"/>
       <c r="AO25" s="3"/>
       <c r="AP25" s="3"/>
-      <c r="AQ25" s="3"/>
-    </row>
-    <row r="26" spans="1:43" x14ac:dyDescent="0.2">
+    </row>
+    <row r="26" spans="1:42" x14ac:dyDescent="0.2">
       <c r="K26" s="1"/>
       <c r="L26" s="1"/>
       <c r="M26" s="1"/>
@@ -13943,9 +13917,8 @@
       <c r="AN26" s="1"/>
       <c r="AO26" s="1"/>
       <c r="AP26" s="1"/>
-      <c r="AQ26" s="1"/>
-    </row>
-    <row r="27" spans="1:43" x14ac:dyDescent="0.2">
+    </row>
+    <row r="27" spans="1:42" x14ac:dyDescent="0.2">
       <c r="K27" s="1"/>
       <c r="L27" s="1"/>
       <c r="M27" s="1"/>
@@ -13968,9 +13941,8 @@
       <c r="AD27" s="1"/>
       <c r="AE27" s="1"/>
       <c r="AF27" s="1"/>
-      <c r="AG27" s="1"/>
-    </row>
-    <row r="28" spans="1:43" x14ac:dyDescent="0.2">
+    </row>
+    <row r="28" spans="1:42" x14ac:dyDescent="0.2">
       <c r="K28" s="1"/>
       <c r="L28" s="1"/>
       <c r="M28" s="1"/>
@@ -13993,9 +13965,8 @@
       <c r="AD28" s="1"/>
       <c r="AE28" s="1"/>
       <c r="AF28" s="1"/>
-      <c r="AG28" s="1"/>
-    </row>
-    <row r="29" spans="1:43" x14ac:dyDescent="0.2">
+    </row>
+    <row r="29" spans="1:42" x14ac:dyDescent="0.2">
       <c r="K29" s="1"/>
       <c r="L29" s="1"/>
       <c r="M29" s="1"/>
@@ -14018,9 +13989,8 @@
       <c r="AD29" s="1"/>
       <c r="AE29" s="1"/>
       <c r="AF29" s="1"/>
-      <c r="AG29" s="1"/>
-    </row>
-    <row r="30" spans="1:43" x14ac:dyDescent="0.2">
+    </row>
+    <row r="30" spans="1:42" x14ac:dyDescent="0.2">
       <c r="K30" s="1"/>
       <c r="L30" s="1"/>
       <c r="M30" s="1"/>
@@ -14043,9 +14013,8 @@
       <c r="AD30" s="1"/>
       <c r="AE30" s="1"/>
       <c r="AF30" s="1"/>
-      <c r="AG30" s="1"/>
-    </row>
-    <row r="31" spans="1:43" x14ac:dyDescent="0.2">
+    </row>
+    <row r="31" spans="1:42" x14ac:dyDescent="0.2">
       <c r="K31" s="1"/>
       <c r="L31" s="1"/>
       <c r="M31" s="1"/>
@@ -14068,9 +14037,8 @@
       <c r="AD31" s="1"/>
       <c r="AE31" s="1"/>
       <c r="AF31" s="1"/>
-      <c r="AG31" s="1"/>
-    </row>
-    <row r="32" spans="1:43" x14ac:dyDescent="0.2">
+    </row>
+    <row r="32" spans="1:42" x14ac:dyDescent="0.2">
       <c r="K32" s="1"/>
       <c r="L32" s="1"/>
       <c r="M32" s="1"/>
@@ -14093,9 +14061,8 @@
       <c r="AD32" s="1"/>
       <c r="AE32" s="1"/>
       <c r="AF32" s="1"/>
-      <c r="AG32" s="1"/>
-    </row>
-    <row r="33" spans="11:33" x14ac:dyDescent="0.2">
+    </row>
+    <row r="33" spans="11:32" x14ac:dyDescent="0.2">
       <c r="K33" s="1"/>
       <c r="L33" s="1"/>
       <c r="M33" s="1"/>
@@ -14118,9 +14085,8 @@
       <c r="AD33" s="1"/>
       <c r="AE33" s="1"/>
       <c r="AF33" s="1"/>
-      <c r="AG33" s="1"/>
-    </row>
-    <row r="34" spans="11:33" x14ac:dyDescent="0.2">
+    </row>
+    <row r="34" spans="11:32" x14ac:dyDescent="0.2">
       <c r="K34" s="1"/>
       <c r="L34" s="1"/>
       <c r="M34" s="1"/>
@@ -14143,9 +14109,8 @@
       <c r="AD34" s="1"/>
       <c r="AE34" s="1"/>
       <c r="AF34" s="1"/>
-      <c r="AG34" s="1"/>
-    </row>
-    <row r="35" spans="11:33" x14ac:dyDescent="0.2">
+    </row>
+    <row r="35" spans="11:32" x14ac:dyDescent="0.2">
       <c r="K35" s="1"/>
       <c r="L35" s="1"/>
       <c r="M35" s="1"/>
@@ -14168,9 +14133,8 @@
       <c r="AD35" s="1"/>
       <c r="AE35" s="1"/>
       <c r="AF35" s="1"/>
-      <c r="AG35" s="1"/>
-    </row>
-    <row r="36" spans="11:33" x14ac:dyDescent="0.2">
+    </row>
+    <row r="36" spans="11:32" x14ac:dyDescent="0.2">
       <c r="K36" s="1"/>
       <c r="L36" s="1"/>
       <c r="M36" s="1"/>
@@ -14193,9 +14157,8 @@
       <c r="AD36" s="1"/>
       <c r="AE36" s="1"/>
       <c r="AF36" s="1"/>
-      <c r="AG36" s="1"/>
-    </row>
-    <row r="37" spans="11:33" x14ac:dyDescent="0.2">
+    </row>
+    <row r="37" spans="11:32" x14ac:dyDescent="0.2">
       <c r="K37" s="1"/>
       <c r="L37" s="1"/>
       <c r="M37" s="1"/>
@@ -14218,9 +14181,8 @@
       <c r="AD37" s="1"/>
       <c r="AE37" s="1"/>
       <c r="AF37" s="1"/>
-      <c r="AG37" s="1"/>
-    </row>
-    <row r="38" spans="11:33" x14ac:dyDescent="0.2">
+    </row>
+    <row r="38" spans="11:32" x14ac:dyDescent="0.2">
       <c r="K38" s="1"/>
       <c r="L38" s="1"/>
       <c r="M38" s="1"/>
@@ -14243,9 +14205,8 @@
       <c r="AD38" s="1"/>
       <c r="AE38" s="1"/>
       <c r="AF38" s="1"/>
-      <c r="AG38" s="1"/>
-    </row>
-    <row r="39" spans="11:33" x14ac:dyDescent="0.2">
+    </row>
+    <row r="39" spans="11:32" x14ac:dyDescent="0.2">
       <c r="K39" s="1"/>
       <c r="L39" s="1"/>
       <c r="M39" s="1"/>
@@ -14268,9 +14229,8 @@
       <c r="AD39" s="1"/>
       <c r="AE39" s="1"/>
       <c r="AF39" s="1"/>
-      <c r="AG39" s="1"/>
-    </row>
-    <row r="40" spans="11:33" x14ac:dyDescent="0.2">
+    </row>
+    <row r="40" spans="11:32" x14ac:dyDescent="0.2">
       <c r="K40" s="1"/>
       <c r="L40" s="1"/>
       <c r="M40" s="1"/>
@@ -14293,9 +14253,8 @@
       <c r="AD40" s="1"/>
       <c r="AE40" s="1"/>
       <c r="AF40" s="1"/>
-      <c r="AG40" s="1"/>
-    </row>
-    <row r="41" spans="11:33" x14ac:dyDescent="0.2">
+    </row>
+    <row r="41" spans="11:32" x14ac:dyDescent="0.2">
       <c r="K41" s="1"/>
       <c r="L41" s="1"/>
       <c r="M41" s="1"/>
@@ -14318,9 +14277,8 @@
       <c r="AD41" s="1"/>
       <c r="AE41" s="1"/>
       <c r="AF41" s="1"/>
-      <c r="AG41" s="1"/>
-    </row>
-    <row r="42" spans="11:33" x14ac:dyDescent="0.2">
+    </row>
+    <row r="42" spans="11:32" x14ac:dyDescent="0.2">
       <c r="K42" s="1"/>
       <c r="L42" s="1"/>
       <c r="M42" s="1"/>
@@ -14343,9 +14301,8 @@
       <c r="AD42" s="1"/>
       <c r="AE42" s="1"/>
       <c r="AF42" s="1"/>
-      <c r="AG42" s="1"/>
-    </row>
-    <row r="43" spans="11:33" x14ac:dyDescent="0.2">
+    </row>
+    <row r="43" spans="11:32" x14ac:dyDescent="0.2">
       <c r="K43" s="1"/>
       <c r="L43" s="1"/>
       <c r="M43" s="1"/>
@@ -14368,9 +14325,8 @@
       <c r="AD43" s="1"/>
       <c r="AE43" s="1"/>
       <c r="AF43" s="1"/>
-      <c r="AG43" s="1"/>
-    </row>
-    <row r="44" spans="11:33" x14ac:dyDescent="0.2">
+    </row>
+    <row r="44" spans="11:32" x14ac:dyDescent="0.2">
       <c r="K44" s="1"/>
       <c r="L44" s="1"/>
       <c r="M44" s="1"/>
@@ -14393,9 +14349,8 @@
       <c r="AD44" s="1"/>
       <c r="AE44" s="1"/>
       <c r="AF44" s="1"/>
-      <c r="AG44" s="1"/>
-    </row>
-    <row r="45" spans="11:33" x14ac:dyDescent="0.2">
+    </row>
+    <row r="45" spans="11:32" x14ac:dyDescent="0.2">
       <c r="K45" s="1"/>
       <c r="L45" s="1"/>
       <c r="M45" s="1"/>
@@ -14418,9 +14373,8 @@
       <c r="AD45" s="1"/>
       <c r="AE45" s="1"/>
       <c r="AF45" s="1"/>
-      <c r="AG45" s="1"/>
-    </row>
-    <row r="46" spans="11:33" x14ac:dyDescent="0.2">
+    </row>
+    <row r="46" spans="11:32" x14ac:dyDescent="0.2">
       <c r="K46" s="1"/>
       <c r="L46" s="1"/>
       <c r="M46" s="1"/>
@@ -14443,9 +14397,8 @@
       <c r="AD46" s="1"/>
       <c r="AE46" s="1"/>
       <c r="AF46" s="1"/>
-      <c r="AG46" s="1"/>
-    </row>
-    <row r="47" spans="11:33" x14ac:dyDescent="0.2">
+    </row>
+    <row r="47" spans="11:32" x14ac:dyDescent="0.2">
       <c r="K47" s="1"/>
       <c r="L47" s="1"/>
       <c r="M47" s="1"/>
@@ -14468,9 +14421,8 @@
       <c r="AD47" s="1"/>
       <c r="AE47" s="1"/>
       <c r="AF47" s="1"/>
-      <c r="AG47" s="1"/>
-    </row>
-    <row r="48" spans="11:33" x14ac:dyDescent="0.2">
+    </row>
+    <row r="48" spans="11:32" x14ac:dyDescent="0.2">
       <c r="K48" s="1"/>
       <c r="L48" s="1"/>
       <c r="M48" s="1"/>
@@ -14493,9 +14445,8 @@
       <c r="AD48" s="1"/>
       <c r="AE48" s="1"/>
       <c r="AF48" s="1"/>
-      <c r="AG48" s="1"/>
-    </row>
-    <row r="49" spans="11:33" x14ac:dyDescent="0.2">
+    </row>
+    <row r="49" spans="11:32" x14ac:dyDescent="0.2">
       <c r="K49" s="1"/>
       <c r="L49" s="1"/>
       <c r="M49" s="1"/>
@@ -14518,9 +14469,8 @@
       <c r="AD49" s="1"/>
       <c r="AE49" s="1"/>
       <c r="AF49" s="1"/>
-      <c r="AG49" s="1"/>
-    </row>
-    <row r="50" spans="11:33" x14ac:dyDescent="0.2">
+    </row>
+    <row r="50" spans="11:32" x14ac:dyDescent="0.2">
       <c r="K50" s="1"/>
       <c r="L50" s="1"/>
       <c r="M50" s="1"/>
@@ -14543,9 +14493,8 @@
       <c r="AD50" s="1"/>
       <c r="AE50" s="1"/>
       <c r="AF50" s="1"/>
-      <c r="AG50" s="1"/>
-    </row>
-    <row r="51" spans="11:33" x14ac:dyDescent="0.2">
+    </row>
+    <row r="51" spans="11:32" x14ac:dyDescent="0.2">
       <c r="K51" s="1"/>
       <c r="L51" s="1"/>
       <c r="M51" s="1"/>
@@ -14568,9 +14517,8 @@
       <c r="AD51" s="1"/>
       <c r="AE51" s="1"/>
       <c r="AF51" s="1"/>
-      <c r="AG51" s="1"/>
-    </row>
-    <row r="52" spans="11:33" x14ac:dyDescent="0.2">
+    </row>
+    <row r="52" spans="11:32" x14ac:dyDescent="0.2">
       <c r="K52" s="1"/>
       <c r="L52" s="1"/>
       <c r="M52" s="1"/>
@@ -14593,109 +14541,103 @@
       <c r="AD52" s="1"/>
       <c r="AE52" s="1"/>
       <c r="AF52" s="1"/>
-      <c r="AG52" s="1"/>
     </row>
   </sheetData>
   <mergeCells count="3">
-    <mergeCell ref="C9:AA9"/>
-    <mergeCell ref="AB9:AG9"/>
-    <mergeCell ref="AH9:AQ9"/>
+    <mergeCell ref="C9:Z9"/>
+    <mergeCell ref="AA9:AF9"/>
+    <mergeCell ref="AG9:AP9"/>
   </mergeCells>
-  <conditionalFormatting sqref="F11:K52 AC11:AG52">
-    <cfRule type="expression" dxfId="20" priority="6">
+  <conditionalFormatting sqref="F11:K52 AB11:AF52">
+    <cfRule type="expression" dxfId="19" priority="6">
       <formula>$E11="hb"</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="19" priority="7">
+    <cfRule type="expression" dxfId="18" priority="7">
       <formula>$E11="pow"</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="F11:L52">
-    <cfRule type="expression" dxfId="18" priority="19">
+  <conditionalFormatting sqref="F11:L52 O11:R52">
+    <cfRule type="expression" dxfId="17" priority="19">
       <formula>$E11="elastic"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="G11:G52">
-    <cfRule type="expression" dxfId="17" priority="8">
+    <cfRule type="expression" dxfId="16" priority="8">
       <formula>$E11="cp"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="H11:I52">
-    <cfRule type="expression" dxfId="16" priority="9">
+    <cfRule type="expression" dxfId="15" priority="9">
       <formula>$E11="mc"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="J11:K52">
-    <cfRule type="expression" dxfId="15" priority="10">
+    <cfRule type="expression" dxfId="14" priority="10">
       <formula>$E11="cp"</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="O11:S52">
-    <cfRule type="expression" dxfId="14" priority="4">
+  <conditionalFormatting sqref="P11:P52">
+    <cfRule type="expression" dxfId="13" priority="13">
+      <formula>AND($O11&lt;&gt;"",$O11&lt;&gt;"ru")</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="S11:V52">
+    <cfRule type="expression" dxfId="12" priority="11">
+      <formula>AND($E11&lt;&gt;"",$E11&lt;&gt;"pow")</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="W11:Z52">
+    <cfRule type="expression" dxfId="11" priority="12">
+      <formula>AND($E11&lt;&gt;"",$E11&lt;&gt;"hb")</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="AB11:AF52">
+    <cfRule type="expression" dxfId="10" priority="21">
       <formula>$E11="elastic"</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="Q11:Q52">
-    <cfRule type="expression" dxfId="13" priority="13">
-      <formula>AND($P11&lt;&gt;"",$P11&lt;&gt;"ru")</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="R11:S52">
-    <cfRule type="expression" dxfId="12" priority="3">
+  <conditionalFormatting sqref="AC11:AC52">
+    <cfRule type="expression" dxfId="9" priority="14">
       <formula>$E11="cp"</formula>
-    </cfRule>
-    <cfRule type="expression" dxfId="11" priority="5">
-      <formula>AND($P11&lt;&gt;"",$P11&lt;&gt;"piezo",$P11&lt;&gt;"seep")</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="T11:W52">
-    <cfRule type="expression" dxfId="10" priority="11">
-      <formula>AND($E11&lt;&gt;"",$E11&lt;&gt;"pow")</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="X11:AA52">
-    <cfRule type="expression" dxfId="9" priority="12">
-      <formula>AND($E11&lt;&gt;"",$E11&lt;&gt;"hb")</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="AC11:AG52">
-    <cfRule type="expression" dxfId="8" priority="21">
-      <formula>$E11="elastic"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="AD11:AD52">
-    <cfRule type="expression" dxfId="7" priority="14">
+    <cfRule type="expression" dxfId="8" priority="15">
+      <formula>$E11="mc"</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="AE11:AF52">
+    <cfRule type="expression" dxfId="7" priority="16">
       <formula>$E11="cp"</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="AE11:AE52">
-    <cfRule type="expression" dxfId="6" priority="15">
-      <formula>$E11="mc"</formula>
+  <conditionalFormatting sqref="AK11:AL52">
+    <cfRule type="expression" dxfId="6" priority="17">
+      <formula>OR($AJ11="vg",$AJ11="gard")</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="AF11:AG52">
-    <cfRule type="expression" dxfId="5" priority="16">
+  <conditionalFormatting sqref="AM11:AN52">
+    <cfRule type="expression" dxfId="5" priority="1">
+      <formula>$AJ11="lf"</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="Q11:R52">
+    <cfRule type="expression" dxfId="1" priority="23">
       <formula>$E11="cp"</formula>
     </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="AL11:AM52">
-    <cfRule type="expression" dxfId="4" priority="17">
-      <formula>OR($AK11="vg",$AK11="gard")</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="AN11:AO52">
-    <cfRule type="expression" dxfId="3" priority="1">
-      <formula>$AK11="lf"</formula>
+    <cfRule type="expression" dxfId="0" priority="24">
+      <formula>AND($O11&lt;&gt;"",$O11&lt;&gt;"piezo",$O11&lt;&gt;"seep")</formula>
     </cfRule>
   </conditionalFormatting>
   <dataValidations count="3">
     <dataValidation type="list" allowBlank="1" sqref="E11:E52" xr:uid="{00000000-0002-0000-0200-000000000000}">
       <formula1>$C$3:$C$7</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" sqref="AK11:AK102" xr:uid="{00000000-0002-0000-0200-000001000000}">
-      <formula1>$AK$3:$AK$5</formula1>
+    <dataValidation type="list" allowBlank="1" sqref="AJ11:AJ102" xr:uid="{00000000-0002-0000-0200-000001000000}">
+      <formula1>$AJ$3:$AJ$5</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" sqref="P11:P52" xr:uid="{00000000-0002-0000-0200-000002000000}">
-      <formula1>$P$3:$P$6</formula1>
+    <dataValidation type="list" allowBlank="1" sqref="O11:O52" xr:uid="{00000000-0002-0000-0200-000002000000}">
+      <formula1>$O$3:$O$6</formula1>
     </dataValidation>
   </dataValidations>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -14730,180 +14672,180 @@
   <sheetData>
     <row r="2" spans="1:44" x14ac:dyDescent="0.2">
       <c r="A2" s="5" t="s">
-        <v>160</v>
+        <v>159</v>
       </c>
       <c r="B2" s="3">
         <v>0</v>
       </c>
       <c r="D2" s="24" t="s">
-        <v>161</v>
+        <v>160</v>
       </c>
     </row>
     <row r="4" spans="1:44" x14ac:dyDescent="0.2">
       <c r="A4" s="55" t="s">
-        <v>162</v>
+        <v>161</v>
       </c>
       <c r="B4" s="52"/>
       <c r="D4" s="55" t="s">
-        <v>163</v>
+        <v>162</v>
       </c>
       <c r="E4" s="52"/>
       <c r="G4" s="55" t="s">
-        <v>164</v>
+        <v>163</v>
       </c>
       <c r="H4" s="52"/>
       <c r="J4" s="55" t="s">
-        <v>165</v>
+        <v>164</v>
       </c>
       <c r="K4" s="52"/>
       <c r="M4" s="55" t="s">
-        <v>166</v>
+        <v>165</v>
       </c>
       <c r="N4" s="52"/>
       <c r="P4" s="55" t="s">
-        <v>167</v>
+        <v>166</v>
       </c>
       <c r="Q4" s="54"/>
       <c r="R4" s="1"/>
       <c r="S4" s="55" t="s">
-        <v>168</v>
+        <v>167</v>
       </c>
       <c r="T4" s="54"/>
       <c r="U4" s="1"/>
       <c r="V4" s="55" t="s">
-        <v>169</v>
+        <v>168</v>
       </c>
       <c r="W4" s="54"/>
       <c r="X4" s="1"/>
       <c r="Y4" s="55" t="s">
-        <v>170</v>
+        <v>169</v>
       </c>
       <c r="Z4" s="54"/>
       <c r="AA4" s="1"/>
       <c r="AB4" s="55" t="s">
-        <v>171</v>
+        <v>170</v>
       </c>
       <c r="AC4" s="54"/>
       <c r="AE4" s="55" t="s">
-        <v>172</v>
+        <v>171</v>
       </c>
       <c r="AF4" s="54"/>
       <c r="AG4" s="1"/>
       <c r="AH4" s="55" t="s">
-        <v>173</v>
+        <v>172</v>
       </c>
       <c r="AI4" s="54"/>
       <c r="AJ4" s="1"/>
       <c r="AK4" s="55" t="s">
-        <v>174</v>
+        <v>173</v>
       </c>
       <c r="AL4" s="54"/>
       <c r="AM4" s="1"/>
       <c r="AN4" s="55" t="s">
-        <v>175</v>
+        <v>174</v>
       </c>
       <c r="AO4" s="54"/>
       <c r="AP4" s="1"/>
       <c r="AQ4" s="55" t="s">
-        <v>176</v>
+        <v>175</v>
       </c>
       <c r="AR4" s="54"/>
     </row>
     <row r="5" spans="1:44" x14ac:dyDescent="0.2">
       <c r="A5" s="36" t="s">
-        <v>177</v>
+        <v>176</v>
       </c>
       <c r="B5" s="37">
         <v>1</v>
       </c>
       <c r="D5" s="36" t="s">
-        <v>177</v>
+        <v>176</v>
       </c>
       <c r="E5" s="37">
         <v>2</v>
       </c>
       <c r="G5" s="36" t="s">
-        <v>177</v>
+        <v>176</v>
       </c>
       <c r="H5" s="37">
         <v>3</v>
       </c>
       <c r="J5" s="36" t="s">
-        <v>177</v>
+        <v>176</v>
       </c>
       <c r="K5" s="37">
         <v>4</v>
       </c>
       <c r="M5" s="36" t="s">
-        <v>177</v>
+        <v>176</v>
       </c>
       <c r="N5" s="37">
         <v>5</v>
       </c>
       <c r="P5" s="36" t="s">
-        <v>177</v>
+        <v>176</v>
       </c>
       <c r="Q5" s="37">
         <v>6</v>
       </c>
       <c r="R5" s="1"/>
       <c r="S5" s="36" t="s">
-        <v>177</v>
+        <v>176</v>
       </c>
       <c r="T5" s="37">
         <v>7</v>
       </c>
       <c r="U5" s="1"/>
       <c r="V5" s="36" t="s">
-        <v>177</v>
+        <v>176</v>
       </c>
       <c r="W5" s="37">
         <v>8</v>
       </c>
       <c r="X5" s="1"/>
       <c r="Y5" s="36" t="s">
-        <v>177</v>
+        <v>176</v>
       </c>
       <c r="Z5" s="37">
         <v>9</v>
       </c>
       <c r="AA5" s="1"/>
       <c r="AB5" s="36" t="s">
-        <v>177</v>
+        <v>176</v>
       </c>
       <c r="AC5" s="37">
         <v>10</v>
       </c>
       <c r="AE5" s="36" t="s">
-        <v>177</v>
+        <v>176</v>
       </c>
       <c r="AF5" s="37">
         <v>11</v>
       </c>
       <c r="AG5" s="1"/>
       <c r="AH5" s="36" t="s">
-        <v>177</v>
+        <v>176</v>
       </c>
       <c r="AI5" s="37">
         <v>12</v>
       </c>
       <c r="AJ5" s="1"/>
       <c r="AK5" s="36" t="s">
-        <v>177</v>
+        <v>176</v>
       </c>
       <c r="AL5" s="37">
         <v>13</v>
       </c>
       <c r="AM5" s="1"/>
       <c r="AN5" s="36" t="s">
-        <v>177</v>
+        <v>176</v>
       </c>
       <c r="AO5" s="37">
         <v>14</v>
       </c>
       <c r="AP5" s="1"/>
       <c r="AQ5" s="36" t="s">
-        <v>177</v>
+        <v>176</v>
       </c>
       <c r="AR5" s="37">
         <v>15</v>
@@ -14996,102 +14938,102 @@
     </row>
     <row r="7" spans="1:44" x14ac:dyDescent="0.2">
       <c r="A7" s="2" t="s">
+        <v>177</v>
+      </c>
+      <c r="B7" s="2" t="s">
         <v>178</v>
       </c>
-      <c r="B7" s="2" t="s">
-        <v>179</v>
-      </c>
       <c r="D7" s="2" t="s">
+        <v>177</v>
+      </c>
+      <c r="E7" s="2" t="s">
         <v>178</v>
       </c>
-      <c r="E7" s="2" t="s">
-        <v>179</v>
-      </c>
       <c r="G7" s="2" t="s">
+        <v>177</v>
+      </c>
+      <c r="H7" s="2" t="s">
         <v>178</v>
       </c>
-      <c r="H7" s="2" t="s">
-        <v>179</v>
-      </c>
       <c r="J7" s="2" t="s">
+        <v>177</v>
+      </c>
+      <c r="K7" s="2" t="s">
         <v>178</v>
       </c>
-      <c r="K7" s="2" t="s">
-        <v>179</v>
-      </c>
       <c r="M7" s="2" t="s">
+        <v>177</v>
+      </c>
+      <c r="N7" s="2" t="s">
         <v>178</v>
       </c>
-      <c r="N7" s="2" t="s">
-        <v>179</v>
-      </c>
       <c r="P7" s="2" t="s">
+        <v>177</v>
+      </c>
+      <c r="Q7" s="2" t="s">
         <v>178</v>
-      </c>
-      <c r="Q7" s="2" t="s">
-        <v>179</v>
       </c>
       <c r="R7" s="1"/>
       <c r="S7" s="2" t="s">
+        <v>177</v>
+      </c>
+      <c r="T7" s="2" t="s">
         <v>178</v>
-      </c>
-      <c r="T7" s="2" t="s">
-        <v>179</v>
       </c>
       <c r="U7" s="1"/>
       <c r="V7" s="2" t="s">
+        <v>177</v>
+      </c>
+      <c r="W7" s="2" t="s">
         <v>178</v>
-      </c>
-      <c r="W7" s="2" t="s">
-        <v>179</v>
       </c>
       <c r="X7" s="1"/>
       <c r="Y7" s="2" t="s">
+        <v>177</v>
+      </c>
+      <c r="Z7" s="2" t="s">
         <v>178</v>
-      </c>
-      <c r="Z7" s="2" t="s">
-        <v>179</v>
       </c>
       <c r="AA7" s="1"/>
       <c r="AB7" s="2" t="s">
+        <v>177</v>
+      </c>
+      <c r="AC7" s="2" t="s">
         <v>178</v>
       </c>
-      <c r="AC7" s="2" t="s">
-        <v>179</v>
-      </c>
       <c r="AE7" s="2" t="s">
+        <v>177</v>
+      </c>
+      <c r="AF7" s="2" t="s">
         <v>178</v>
-      </c>
-      <c r="AF7" s="2" t="s">
-        <v>179</v>
       </c>
       <c r="AG7" s="1"/>
       <c r="AH7" s="2" t="s">
+        <v>177</v>
+      </c>
+      <c r="AI7" s="2" t="s">
         <v>178</v>
-      </c>
-      <c r="AI7" s="2" t="s">
-        <v>179</v>
       </c>
       <c r="AJ7" s="1"/>
       <c r="AK7" s="2" t="s">
+        <v>177</v>
+      </c>
+      <c r="AL7" s="2" t="s">
         <v>178</v>
-      </c>
-      <c r="AL7" s="2" t="s">
-        <v>179</v>
       </c>
       <c r="AM7" s="1"/>
       <c r="AN7" s="2" t="s">
+        <v>177</v>
+      </c>
+      <c r="AO7" s="2" t="s">
         <v>178</v>
-      </c>
-      <c r="AO7" s="2" t="s">
-        <v>179</v>
       </c>
       <c r="AP7" s="1"/>
       <c r="AQ7" s="2" t="s">
+        <v>177</v>
+      </c>
+      <c r="AR7" s="2" t="s">
         <v>178</v>
-      </c>
-      <c r="AR7" s="2" t="s">
-        <v>179</v>
       </c>
     </row>
     <row r="8" spans="1:44" x14ac:dyDescent="0.2">
@@ -15896,6 +15838,20 @@
     </row>
   </sheetData>
   <mergeCells count="30">
+    <mergeCell ref="D4:E4"/>
+    <mergeCell ref="P4:Q4"/>
+    <mergeCell ref="Y4:Z4"/>
+    <mergeCell ref="AB6:AC6"/>
+    <mergeCell ref="AN6:AO6"/>
+    <mergeCell ref="AB4:AC4"/>
+    <mergeCell ref="AN4:AO4"/>
+    <mergeCell ref="G6:H6"/>
+    <mergeCell ref="J4:K4"/>
+    <mergeCell ref="V6:W6"/>
+    <mergeCell ref="M6:N6"/>
+    <mergeCell ref="AH6:AI6"/>
+    <mergeCell ref="S6:T6"/>
+    <mergeCell ref="Y6:Z6"/>
     <mergeCell ref="AQ4:AR4"/>
     <mergeCell ref="A4:B4"/>
     <mergeCell ref="G4:H4"/>
@@ -15912,20 +15868,6 @@
     <mergeCell ref="AH4:AI4"/>
     <mergeCell ref="J6:K6"/>
     <mergeCell ref="P6:Q6"/>
-    <mergeCell ref="G6:H6"/>
-    <mergeCell ref="J4:K4"/>
-    <mergeCell ref="V6:W6"/>
-    <mergeCell ref="M6:N6"/>
-    <mergeCell ref="AH6:AI6"/>
-    <mergeCell ref="S6:T6"/>
-    <mergeCell ref="Y6:Z6"/>
-    <mergeCell ref="D4:E4"/>
-    <mergeCell ref="P4:Q4"/>
-    <mergeCell ref="Y4:Z4"/>
-    <mergeCell ref="AB6:AC6"/>
-    <mergeCell ref="AN6:AO6"/>
-    <mergeCell ref="AB4:AC4"/>
-    <mergeCell ref="AN4:AO4"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
@@ -15959,174 +15901,177 @@
   <sheetData>
     <row r="2" spans="1:44" x14ac:dyDescent="0.2">
       <c r="A2" s="24" t="s">
-        <v>180</v>
+        <v>179</v>
+      </c>
+      <c r="G2" s="9" t="s">
+        <v>303</v>
       </c>
     </row>
     <row r="4" spans="1:44" x14ac:dyDescent="0.2">
       <c r="A4" s="55" t="s">
-        <v>181</v>
+        <v>180</v>
       </c>
       <c r="B4" s="52"/>
       <c r="D4" s="55" t="s">
-        <v>182</v>
+        <v>181</v>
       </c>
       <c r="E4" s="52"/>
       <c r="G4" s="55" t="s">
-        <v>183</v>
+        <v>182</v>
       </c>
       <c r="H4" s="52"/>
       <c r="J4" s="55" t="s">
-        <v>184</v>
+        <v>183</v>
       </c>
       <c r="K4" s="52"/>
       <c r="M4" s="55" t="s">
-        <v>185</v>
+        <v>184</v>
       </c>
       <c r="N4" s="52"/>
       <c r="P4" s="55" t="s">
-        <v>186</v>
+        <v>185</v>
       </c>
       <c r="Q4" s="54"/>
       <c r="R4" s="1"/>
       <c r="S4" s="55" t="s">
-        <v>187</v>
+        <v>186</v>
       </c>
       <c r="T4" s="54"/>
       <c r="U4" s="1"/>
       <c r="V4" s="55" t="s">
-        <v>188</v>
+        <v>187</v>
       </c>
       <c r="W4" s="54"/>
       <c r="X4" s="1"/>
       <c r="Y4" s="55" t="s">
-        <v>189</v>
+        <v>188</v>
       </c>
       <c r="Z4" s="54"/>
       <c r="AA4" s="1"/>
       <c r="AB4" s="55" t="s">
-        <v>190</v>
+        <v>189</v>
       </c>
       <c r="AC4" s="54"/>
       <c r="AE4" s="55" t="s">
-        <v>191</v>
+        <v>190</v>
       </c>
       <c r="AF4" s="54"/>
       <c r="AG4" s="1"/>
       <c r="AH4" s="55" t="s">
-        <v>192</v>
+        <v>191</v>
       </c>
       <c r="AI4" s="54"/>
       <c r="AJ4" s="1"/>
       <c r="AK4" s="55" t="s">
-        <v>193</v>
+        <v>192</v>
       </c>
       <c r="AL4" s="54"/>
       <c r="AM4" s="1"/>
       <c r="AN4" s="55" t="s">
-        <v>194</v>
+        <v>193</v>
       </c>
       <c r="AO4" s="54"/>
       <c r="AP4" s="1"/>
       <c r="AQ4" s="55" t="s">
-        <v>195</v>
+        <v>194</v>
       </c>
       <c r="AR4" s="54"/>
     </row>
     <row r="5" spans="1:44" x14ac:dyDescent="0.2">
       <c r="A5" s="38" t="s">
-        <v>177</v>
+        <v>176</v>
       </c>
       <c r="B5" s="39">
         <v>1</v>
       </c>
       <c r="D5" s="38" t="s">
-        <v>177</v>
+        <v>176</v>
       </c>
       <c r="E5" s="39">
         <v>2</v>
       </c>
       <c r="G5" s="38" t="s">
-        <v>177</v>
+        <v>176</v>
       </c>
       <c r="H5" s="39">
         <v>3</v>
       </c>
       <c r="J5" s="38" t="s">
-        <v>177</v>
+        <v>176</v>
       </c>
       <c r="K5" s="39">
         <v>4</v>
       </c>
       <c r="M5" s="38" t="s">
-        <v>177</v>
+        <v>176</v>
       </c>
       <c r="N5" s="39">
         <v>5</v>
       </c>
       <c r="P5" s="38" t="s">
-        <v>177</v>
+        <v>176</v>
       </c>
       <c r="Q5" s="39">
         <v>6</v>
       </c>
       <c r="R5" s="1"/>
       <c r="S5" s="38" t="s">
-        <v>177</v>
+        <v>176</v>
       </c>
       <c r="T5" s="39">
         <v>7</v>
       </c>
       <c r="U5" s="1"/>
       <c r="V5" s="38" t="s">
-        <v>177</v>
+        <v>176</v>
       </c>
       <c r="W5" s="39">
         <v>8</v>
       </c>
       <c r="X5" s="1"/>
       <c r="Y5" s="38" t="s">
-        <v>177</v>
+        <v>176</v>
       </c>
       <c r="Z5" s="39">
         <v>9</v>
       </c>
       <c r="AA5" s="1"/>
       <c r="AB5" s="38" t="s">
-        <v>177</v>
+        <v>176</v>
       </c>
       <c r="AC5" s="39">
         <v>10</v>
       </c>
       <c r="AE5" s="38" t="s">
-        <v>177</v>
+        <v>176</v>
       </c>
       <c r="AF5" s="39">
         <v>11</v>
       </c>
       <c r="AG5" s="1"/>
       <c r="AH5" s="38" t="s">
-        <v>177</v>
+        <v>176</v>
       </c>
       <c r="AI5" s="39">
         <v>12</v>
       </c>
       <c r="AJ5" s="1"/>
       <c r="AK5" s="38" t="s">
-        <v>177</v>
+        <v>176</v>
       </c>
       <c r="AL5" s="39">
         <v>13</v>
       </c>
       <c r="AM5" s="1"/>
       <c r="AN5" s="38" t="s">
-        <v>177</v>
+        <v>176</v>
       </c>
       <c r="AO5" s="39">
         <v>14</v>
       </c>
       <c r="AP5" s="1"/>
       <c r="AQ5" s="38" t="s">
-        <v>177</v>
+        <v>176</v>
       </c>
       <c r="AR5" s="39">
         <v>15</v>
@@ -16134,187 +16079,187 @@
     </row>
     <row r="6" spans="1:44" x14ac:dyDescent="0.2">
       <c r="A6" s="58" t="str">
-        <f>_xlfn.XLOOKUP(B5,mat!$A:$A, mat!$B:$B,"") &amp; ""</f>
+        <f>IF(B5=-1,"SSR reduce",IF(B5=-2,"SSR hold",IF(B5=-3,"SSR elastic",_xlfn.XLOOKUP(B5,mat!$A:$A, mat!$B:$B,"") &amp; "")))</f>
         <v/>
       </c>
       <c r="B6" s="57"/>
       <c r="D6" s="58" t="str">
-        <f>_xlfn.XLOOKUP(E5,mat!$A:$A, mat!$B:$B,"") &amp; ""</f>
+        <f>IF(E5=-1,"SSR reduce",IF(E5=-2,"SSR hold",IF(E5=-3,"SSR elastic",_xlfn.XLOOKUP(E5,mat!$A:$A, mat!$B:$B,"") &amp; "")))</f>
         <v/>
       </c>
       <c r="E6" s="57"/>
       <c r="G6" s="58" t="str">
-        <f>_xlfn.XLOOKUP(H5,mat!$A:$A, mat!$B:$B,"") &amp; ""</f>
+        <f>IF(H5=-1,"SSR reduce",IF(H5=-2,"SSR hold",IF(H5=-3,"SSR elastic",_xlfn.XLOOKUP(H5,mat!$A:$A, mat!$B:$B,"") &amp; "")))</f>
         <v/>
       </c>
       <c r="H6" s="57"/>
       <c r="J6" s="58" t="str">
-        <f>_xlfn.XLOOKUP(K5,mat!$A:$A, mat!$B:$B,"") &amp; ""</f>
+        <f>IF(K5=-1,"SSR reduce",IF(K5=-2,"SSR hold",IF(K5=-3,"SSR elastic",_xlfn.XLOOKUP(K5,mat!$A:$A, mat!$B:$B,"") &amp; "")))</f>
         <v/>
       </c>
       <c r="K6" s="57"/>
       <c r="M6" s="58" t="str">
-        <f>_xlfn.XLOOKUP(N5,mat!$A:$A, mat!$B:$B,"") &amp; ""</f>
+        <f>IF(N5=-1,"SSR reduce",IF(N5=-2,"SSR hold",IF(N5=-3,"SSR elastic",_xlfn.XLOOKUP(N5,mat!$A:$A, mat!$B:$B,"") &amp; "")))</f>
         <v/>
       </c>
       <c r="N6" s="57"/>
       <c r="P6" s="58" t="str">
-        <f>_xlfn.XLOOKUP(Q5,mat!$A:$A, mat!$B:$B,"") &amp; ""</f>
+        <f>IF(Q5=-1,"SSR reduce",IF(Q5=-2,"SSR hold",IF(Q5=-3,"SSR elastic",_xlfn.XLOOKUP(Q5,mat!$A:$A, mat!$B:$B,"") &amp; "")))</f>
         <v/>
       </c>
       <c r="Q6" s="57"/>
       <c r="R6" s="1"/>
       <c r="S6" s="58" t="str">
-        <f>_xlfn.XLOOKUP(T5,mat!$A:$A, mat!$B:$B,"") &amp; ""</f>
+        <f>IF(T5=-1,"SSR reduce",IF(T5=-2,"SSR hold",IF(T5=-3,"SSR elastic",_xlfn.XLOOKUP(T5,mat!$A:$A, mat!$B:$B,"") &amp; "")))</f>
         <v/>
       </c>
       <c r="T6" s="57"/>
       <c r="U6" s="1"/>
       <c r="V6" s="58" t="str">
-        <f>_xlfn.XLOOKUP(W5,mat!$A:$A, mat!$B:$B,"") &amp; ""</f>
+        <f>IF(W5=-1,"SSR reduce",IF(W5=-2,"SSR hold",IF(W5=-3,"SSR elastic",_xlfn.XLOOKUP(W5,mat!$A:$A, mat!$B:$B,"") &amp; "")))</f>
         <v/>
       </c>
       <c r="W6" s="57"/>
       <c r="X6" s="1"/>
       <c r="Y6" s="58" t="str">
-        <f>_xlfn.XLOOKUP(Z5,mat!$A:$A, mat!$B:$B,"") &amp; ""</f>
+        <f>IF(Z5=-1,"SSR reduce",IF(Z5=-2,"SSR hold",IF(Z5=-3,"SSR elastic",_xlfn.XLOOKUP(Z5,mat!$A:$A, mat!$B:$B,"") &amp; "")))</f>
         <v/>
       </c>
       <c r="Z6" s="57"/>
       <c r="AA6" s="1"/>
       <c r="AB6" s="58" t="str">
-        <f>_xlfn.XLOOKUP(AC5,mat!$A:$A, mat!$B:$B,"") &amp; ""</f>
+        <f>IF(AC5=-1,"SSR reduce",IF(AC5=-2,"SSR hold",IF(AC5=-3,"SSR elastic",_xlfn.XLOOKUP(AC5,mat!$A:$A, mat!$B:$B,"") &amp; "")))</f>
         <v/>
       </c>
       <c r="AC6" s="57"/>
       <c r="AE6" s="58" t="str">
-        <f>_xlfn.XLOOKUP(AF5,mat!$A:$A, mat!$B:$B,"") &amp; ""</f>
+        <f>IF(AF5=-1,"SSR reduce",IF(AF5=-2,"SSR hold",IF(AF5=-3,"SSR elastic",_xlfn.XLOOKUP(AF5,mat!$A:$A, mat!$B:$B,"") &amp; "")))</f>
         <v/>
       </c>
       <c r="AF6" s="57"/>
       <c r="AG6" s="1"/>
       <c r="AH6" s="58" t="str">
-        <f>_xlfn.XLOOKUP(AI5,mat!$A:$A, mat!$B:$B,"") &amp; ""</f>
+        <f>IF(AI5=-1,"SSR reduce",IF(AI5=-2,"SSR hold",IF(AI5=-3,"SSR elastic",_xlfn.XLOOKUP(AI5,mat!$A:$A, mat!$B:$B,"") &amp; "")))</f>
         <v/>
       </c>
       <c r="AI6" s="57"/>
       <c r="AJ6" s="1"/>
       <c r="AK6" s="58" t="str">
-        <f>_xlfn.XLOOKUP(AL5,mat!$A:$A, mat!$B:$B,"") &amp; ""</f>
+        <f>IF(AL5=-1,"SSR reduce",IF(AL5=-2,"SSR hold",IF(AL5=-3,"SSR elastic",_xlfn.XLOOKUP(AL5,mat!$A:$A, mat!$B:$B,"") &amp; "")))</f>
         <v/>
       </c>
       <c r="AL6" s="57"/>
       <c r="AM6" s="1"/>
       <c r="AN6" s="58" t="str">
-        <f>_xlfn.XLOOKUP(AO5,mat!$A:$A, mat!$B:$B,"") &amp; ""</f>
+        <f>IF(AO5=-1,"SSR reduce",IF(AO5=-2,"SSR hold",IF(AO5=-3,"SSR elastic",_xlfn.XLOOKUP(AO5,mat!$A:$A, mat!$B:$B,"") &amp; "")))</f>
         <v/>
       </c>
       <c r="AO6" s="57"/>
       <c r="AP6" s="1"/>
       <c r="AQ6" s="58" t="str">
-        <f>_xlfn.XLOOKUP(AR5,mat!$A:$A, mat!$B:$B,"") &amp; ""</f>
+        <f>IF(AR5=-1,"SSR reduce",IF(AR5=-2,"SSR hold",IF(AR5=-3,"SSR elastic",_xlfn.XLOOKUP(AR5,mat!$A:$A, mat!$B:$B,"") &amp; "")))</f>
         <v/>
       </c>
       <c r="AR6" s="57"/>
     </row>
     <row r="7" spans="1:44" x14ac:dyDescent="0.2">
       <c r="A7" s="2" t="s">
+        <v>177</v>
+      </c>
+      <c r="B7" s="2" t="s">
         <v>178</v>
       </c>
-      <c r="B7" s="2" t="s">
-        <v>179</v>
-      </c>
       <c r="D7" s="2" t="s">
+        <v>177</v>
+      </c>
+      <c r="E7" s="2" t="s">
         <v>178</v>
       </c>
-      <c r="E7" s="2" t="s">
-        <v>179</v>
-      </c>
       <c r="G7" s="2" t="s">
+        <v>177</v>
+      </c>
+      <c r="H7" s="2" t="s">
         <v>178</v>
       </c>
-      <c r="H7" s="2" t="s">
-        <v>179</v>
-      </c>
       <c r="J7" s="2" t="s">
+        <v>177</v>
+      </c>
+      <c r="K7" s="2" t="s">
         <v>178</v>
       </c>
-      <c r="K7" s="2" t="s">
-        <v>179</v>
-      </c>
       <c r="M7" s="2" t="s">
+        <v>177</v>
+      </c>
+      <c r="N7" s="2" t="s">
         <v>178</v>
       </c>
-      <c r="N7" s="2" t="s">
-        <v>179</v>
-      </c>
       <c r="P7" s="2" t="s">
+        <v>177</v>
+      </c>
+      <c r="Q7" s="2" t="s">
         <v>178</v>
-      </c>
-      <c r="Q7" s="2" t="s">
-        <v>179</v>
       </c>
       <c r="R7" s="1"/>
       <c r="S7" s="2" t="s">
+        <v>177</v>
+      </c>
+      <c r="T7" s="2" t="s">
         <v>178</v>
-      </c>
-      <c r="T7" s="2" t="s">
-        <v>179</v>
       </c>
       <c r="U7" s="1"/>
       <c r="V7" s="2" t="s">
+        <v>177</v>
+      </c>
+      <c r="W7" s="2" t="s">
         <v>178</v>
-      </c>
-      <c r="W7" s="2" t="s">
-        <v>179</v>
       </c>
       <c r="X7" s="1"/>
       <c r="Y7" s="2" t="s">
+        <v>177</v>
+      </c>
+      <c r="Z7" s="2" t="s">
         <v>178</v>
-      </c>
-      <c r="Z7" s="2" t="s">
-        <v>179</v>
       </c>
       <c r="AA7" s="1"/>
       <c r="AB7" s="2" t="s">
+        <v>177</v>
+      </c>
+      <c r="AC7" s="2" t="s">
         <v>178</v>
       </c>
-      <c r="AC7" s="2" t="s">
-        <v>179</v>
-      </c>
       <c r="AE7" s="2" t="s">
+        <v>177</v>
+      </c>
+      <c r="AF7" s="2" t="s">
         <v>178</v>
-      </c>
-      <c r="AF7" s="2" t="s">
-        <v>179</v>
       </c>
       <c r="AG7" s="1"/>
       <c r="AH7" s="2" t="s">
+        <v>177</v>
+      </c>
+      <c r="AI7" s="2" t="s">
         <v>178</v>
-      </c>
-      <c r="AI7" s="2" t="s">
-        <v>179</v>
       </c>
       <c r="AJ7" s="1"/>
       <c r="AK7" s="2" t="s">
+        <v>177</v>
+      </c>
+      <c r="AL7" s="2" t="s">
         <v>178</v>
-      </c>
-      <c r="AL7" s="2" t="s">
-        <v>179</v>
       </c>
       <c r="AM7" s="1"/>
       <c r="AN7" s="2" t="s">
+        <v>177</v>
+      </c>
+      <c r="AO7" s="2" t="s">
         <v>178</v>
-      </c>
-      <c r="AO7" s="2" t="s">
-        <v>179</v>
       </c>
       <c r="AP7" s="1"/>
       <c r="AQ7" s="2" t="s">
+        <v>177</v>
+      </c>
+      <c r="AR7" s="2" t="s">
         <v>178</v>
-      </c>
-      <c r="AR7" s="2" t="s">
-        <v>179</v>
       </c>
     </row>
     <row r="8" spans="1:44" x14ac:dyDescent="0.2">
@@ -17119,6 +17064,20 @@
     </row>
   </sheetData>
   <mergeCells count="30">
+    <mergeCell ref="D4:E4"/>
+    <mergeCell ref="P4:Q4"/>
+    <mergeCell ref="Y4:Z4"/>
+    <mergeCell ref="AB6:AC6"/>
+    <mergeCell ref="AN6:AO6"/>
+    <mergeCell ref="AB4:AC4"/>
+    <mergeCell ref="AN4:AO4"/>
+    <mergeCell ref="G6:H6"/>
+    <mergeCell ref="J4:K4"/>
+    <mergeCell ref="V6:W6"/>
+    <mergeCell ref="M6:N6"/>
+    <mergeCell ref="AH6:AI6"/>
+    <mergeCell ref="S6:T6"/>
+    <mergeCell ref="Y6:Z6"/>
     <mergeCell ref="AQ4:AR4"/>
     <mergeCell ref="A4:B4"/>
     <mergeCell ref="G4:H4"/>
@@ -17135,20 +17094,6 @@
     <mergeCell ref="AH4:AI4"/>
     <mergeCell ref="J6:K6"/>
     <mergeCell ref="P6:Q6"/>
-    <mergeCell ref="G6:H6"/>
-    <mergeCell ref="J4:K4"/>
-    <mergeCell ref="V6:W6"/>
-    <mergeCell ref="M6:N6"/>
-    <mergeCell ref="AH6:AI6"/>
-    <mergeCell ref="S6:T6"/>
-    <mergeCell ref="Y6:Z6"/>
-    <mergeCell ref="D4:E4"/>
-    <mergeCell ref="P4:Q4"/>
-    <mergeCell ref="Y4:Z4"/>
-    <mergeCell ref="AB6:AC6"/>
-    <mergeCell ref="AN6:AO6"/>
-    <mergeCell ref="AB4:AC4"/>
-    <mergeCell ref="AN4:AO4"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
@@ -17165,43 +17110,43 @@
   <sheetData>
     <row r="2" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A2" s="59" t="s">
-        <v>196</v>
+        <v>195</v>
       </c>
       <c r="B2" s="54"/>
       <c r="D2" s="60" t="s">
-        <v>197</v>
+        <v>196</v>
       </c>
       <c r="E2" s="54"/>
       <c r="G2" s="22" t="s">
-        <v>198</v>
+        <v>197</v>
       </c>
     </row>
     <row r="3" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A3" s="32" t="s">
-        <v>199</v>
+        <v>198</v>
       </c>
       <c r="B3" s="33"/>
       <c r="D3" s="34" t="s">
-        <v>199</v>
+        <v>198</v>
       </c>
       <c r="E3" s="35"/>
       <c r="G3" s="22"/>
     </row>
     <row r="4" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A4" s="2" t="s">
+        <v>177</v>
+      </c>
+      <c r="B4" s="2" t="s">
         <v>178</v>
       </c>
-      <c r="B4" s="2" t="s">
-        <v>179</v>
-      </c>
       <c r="D4" s="2" t="s">
+        <v>177</v>
+      </c>
+      <c r="E4" s="2" t="s">
         <v>178</v>
       </c>
-      <c r="E4" s="2" t="s">
-        <v>179</v>
-      </c>
       <c r="G4" s="6" t="s">
-        <v>200</v>
+        <v>199</v>
       </c>
       <c r="H4" s="1"/>
     </row>
@@ -17214,7 +17159,7 @@
         <v>32</v>
       </c>
       <c r="H5" t="s">
-        <v>201</v>
+        <v>200</v>
       </c>
     </row>
     <row r="6" spans="1:8" x14ac:dyDescent="0.2">
@@ -17223,10 +17168,10 @@
       <c r="D6" s="3"/>
       <c r="E6" s="3"/>
       <c r="G6" s="1" t="s">
+        <v>201</v>
+      </c>
+      <c r="H6" t="s">
         <v>202</v>
-      </c>
-      <c r="H6" t="s">
-        <v>203</v>
       </c>
     </row>
     <row r="7" spans="1:8" x14ac:dyDescent="0.2">
@@ -17363,31 +17308,31 @@
   <sheetData>
     <row r="2" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A2" s="13" t="s">
+        <v>203</v>
+      </c>
+      <c r="B2" s="13" t="s">
         <v>204</v>
       </c>
-      <c r="B2" s="13" t="s">
+      <c r="C2" s="13" t="s">
         <v>205</v>
       </c>
-      <c r="C2" s="13" t="s">
+      <c r="D2" s="13" t="s">
         <v>206</v>
       </c>
-      <c r="D2" s="13" t="s">
+      <c r="E2" s="13" t="s">
         <v>207</v>
       </c>
-      <c r="E2" s="13" t="s">
+      <c r="F2" s="13" t="s">
         <v>208</v>
       </c>
-      <c r="F2" s="13" t="s">
+      <c r="G2" s="13" t="s">
         <v>209</v>
       </c>
-      <c r="G2" s="13" t="s">
+      <c r="H2" s="13" t="s">
         <v>210</v>
       </c>
-      <c r="H2" s="13" t="s">
+      <c r="J2" s="5" t="s">
         <v>211</v>
-      </c>
-      <c r="J2" s="5" t="s">
-        <v>212</v>
       </c>
       <c r="K2" s="10" t="s">
         <v>16</v>
@@ -17405,10 +17350,10 @@
       <c r="G3" s="3"/>
       <c r="H3" s="3"/>
       <c r="J3" s="1" t="s">
-        <v>208</v>
+        <v>207</v>
       </c>
       <c r="K3" s="9" t="s">
-        <v>213</v>
+        <v>212</v>
       </c>
     </row>
     <row r="4" spans="1:14" x14ac:dyDescent="0.2">
@@ -17423,10 +17368,10 @@
       <c r="G4" s="3"/>
       <c r="H4" s="3"/>
       <c r="J4" s="1" t="s">
+        <v>213</v>
+      </c>
+      <c r="K4" s="9" t="s">
         <v>214</v>
-      </c>
-      <c r="K4" s="9" t="s">
-        <v>215</v>
       </c>
     </row>
     <row r="5" spans="1:14" x14ac:dyDescent="0.2">
@@ -17441,10 +17386,10 @@
       <c r="G5" s="3"/>
       <c r="H5" s="3"/>
       <c r="J5" s="1" t="s">
+        <v>215</v>
+      </c>
+      <c r="K5" t="s">
         <v>216</v>
-      </c>
-      <c r="K5" t="s">
-        <v>217</v>
       </c>
     </row>
     <row r="6" spans="1:14" x14ac:dyDescent="0.2">
@@ -17471,7 +17416,7 @@
       <c r="G7" s="3"/>
       <c r="H7" s="3"/>
       <c r="J7" s="5" t="s">
-        <v>218</v>
+        <v>217</v>
       </c>
     </row>
     <row r="8" spans="1:14" x14ac:dyDescent="0.2">
@@ -17486,7 +17431,7 @@
       <c r="G8" s="3"/>
       <c r="H8" s="3"/>
       <c r="J8" s="14" t="s">
-        <v>219</v>
+        <v>218</v>
       </c>
     </row>
     <row r="9" spans="1:14" x14ac:dyDescent="0.2">
@@ -17501,7 +17446,7 @@
       <c r="G9" s="3"/>
       <c r="H9" s="3"/>
       <c r="J9" s="14" t="s">
-        <v>220</v>
+        <v>219</v>
       </c>
     </row>
     <row r="10" spans="1:14" x14ac:dyDescent="0.2">
@@ -17516,7 +17461,7 @@
       <c r="G10" s="3"/>
       <c r="H10" s="3"/>
       <c r="J10" s="14" t="s">
-        <v>221</v>
+        <v>220</v>
       </c>
     </row>
     <row r="11" spans="1:14" x14ac:dyDescent="0.2">
@@ -17531,7 +17476,7 @@
       <c r="G11" s="3"/>
       <c r="H11" s="3"/>
       <c r="J11" s="14" t="s">
-        <v>222</v>
+        <v>221</v>
       </c>
     </row>
     <row r="12" spans="1:14" x14ac:dyDescent="0.2">
@@ -17546,27 +17491,27 @@
       <c r="G12" s="3"/>
       <c r="H12" s="3"/>
       <c r="J12" s="14" t="s">
-        <v>223</v>
+        <v>222</v>
       </c>
     </row>
     <row r="13" spans="1:14" x14ac:dyDescent="0.2">
       <c r="J13" s="14" t="s">
-        <v>224</v>
+        <v>223</v>
       </c>
     </row>
     <row r="14" spans="1:14" x14ac:dyDescent="0.2">
       <c r="J14" s="14" t="s">
-        <v>225</v>
+        <v>224</v>
       </c>
     </row>
     <row r="15" spans="1:14" x14ac:dyDescent="0.2">
       <c r="J15" s="14" t="s">
-        <v>226</v>
+        <v>225</v>
       </c>
     </row>
     <row r="16" spans="1:14" x14ac:dyDescent="0.2">
       <c r="J16" s="14" t="s">
-        <v>227</v>
+        <v>226</v>
       </c>
       <c r="K16" s="1"/>
       <c r="L16" s="1"/>
@@ -17575,22 +17520,22 @@
     </row>
     <row r="17" spans="10:10" x14ac:dyDescent="0.2">
       <c r="J17" s="14" t="s">
-        <v>228</v>
+        <v>227</v>
       </c>
     </row>
   </sheetData>
   <conditionalFormatting sqref="E3:E42">
-    <cfRule type="expression" dxfId="2" priority="3">
+    <cfRule type="expression" dxfId="4" priority="3">
       <formula>OR($D3="Intercept", $D3="Radius")</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="F3:G42">
-    <cfRule type="expression" dxfId="1" priority="2">
+    <cfRule type="expression" dxfId="3" priority="2">
       <formula>OR($D3="Depth",$D3="Radius")</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="H3:H42">
-    <cfRule type="expression" dxfId="0" priority="1">
+    <cfRule type="expression" dxfId="2" priority="1">
       <formula>OR($D3="Depth",$D3="Intercept")</formula>
     </cfRule>
   </conditionalFormatting>
@@ -17615,16 +17560,16 @@
   <sheetData>
     <row r="2" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A2" s="11" t="s">
+        <v>228</v>
+      </c>
+      <c r="B2" s="11" t="s">
         <v>229</v>
       </c>
-      <c r="B2" s="11" t="s">
+      <c r="C2" s="12" t="s">
         <v>230</v>
       </c>
-      <c r="C2" s="12" t="s">
-        <v>231</v>
-      </c>
       <c r="E2" s="6" t="s">
-        <v>212</v>
+        <v>211</v>
       </c>
       <c r="F2" s="6" t="s">
         <v>16</v>
@@ -17635,10 +17580,10 @@
       <c r="B3" s="3"/>
       <c r="C3" s="3"/>
       <c r="E3" t="s">
+        <v>231</v>
+      </c>
+      <c r="F3" t="s">
         <v>232</v>
-      </c>
-      <c r="F3" t="s">
-        <v>233</v>
       </c>
     </row>
     <row r="4" spans="1:6" x14ac:dyDescent="0.2">
@@ -17646,10 +17591,10 @@
       <c r="B4" s="3"/>
       <c r="C4" s="3"/>
       <c r="E4" t="s">
+        <v>233</v>
+      </c>
+      <c r="F4" t="s">
         <v>234</v>
-      </c>
-      <c r="F4" t="s">
-        <v>235</v>
       </c>
     </row>
     <row r="5" spans="1:6" x14ac:dyDescent="0.2">
@@ -17657,10 +17602,10 @@
       <c r="B5" s="3"/>
       <c r="C5" s="3"/>
       <c r="E5" t="s">
+        <v>235</v>
+      </c>
+      <c r="F5" t="s">
         <v>236</v>
-      </c>
-      <c r="F5" t="s">
-        <v>237</v>
       </c>
     </row>
     <row r="6" spans="1:6" x14ac:dyDescent="0.2">
@@ -17784,90 +17729,90 @@
   <sheetData>
     <row r="2" spans="2:24" x14ac:dyDescent="0.2">
       <c r="B2" s="61" t="s">
-        <v>238</v>
+        <v>237</v>
       </c>
       <c r="C2" s="62"/>
       <c r="D2" s="62"/>
       <c r="F2" s="61" t="s">
-        <v>239</v>
+        <v>238</v>
       </c>
       <c r="G2" s="62"/>
       <c r="H2" s="62"/>
       <c r="J2" s="61" t="s">
-        <v>240</v>
+        <v>239</v>
       </c>
       <c r="K2" s="62"/>
       <c r="L2" s="62"/>
       <c r="N2" s="61" t="s">
-        <v>241</v>
+        <v>240</v>
       </c>
       <c r="O2" s="62"/>
       <c r="P2" s="62"/>
       <c r="R2" s="61" t="s">
-        <v>242</v>
+        <v>241</v>
       </c>
       <c r="S2" s="62"/>
       <c r="T2" s="62"/>
       <c r="V2" s="61" t="s">
-        <v>243</v>
+        <v>242</v>
       </c>
       <c r="W2" s="62"/>
       <c r="X2" s="62"/>
     </row>
     <row r="3" spans="2:24" x14ac:dyDescent="0.2">
       <c r="B3" s="2" t="s">
+        <v>228</v>
+      </c>
+      <c r="C3" s="2" t="s">
         <v>229</v>
       </c>
-      <c r="C3" s="2" t="s">
-        <v>230</v>
-      </c>
       <c r="D3" s="2" t="s">
-        <v>244</v>
+        <v>243</v>
       </c>
       <c r="F3" s="2" t="s">
+        <v>228</v>
+      </c>
+      <c r="G3" s="2" t="s">
         <v>229</v>
       </c>
-      <c r="G3" s="2" t="s">
-        <v>230</v>
-      </c>
       <c r="H3" s="2" t="s">
-        <v>244</v>
+        <v>243</v>
       </c>
       <c r="J3" s="2" t="s">
+        <v>228</v>
+      </c>
+      <c r="K3" s="2" t="s">
         <v>229</v>
       </c>
-      <c r="K3" s="2" t="s">
-        <v>230</v>
-      </c>
       <c r="L3" s="2" t="s">
-        <v>244</v>
+        <v>243</v>
       </c>
       <c r="N3" s="2" t="s">
+        <v>228</v>
+      </c>
+      <c r="O3" s="2" t="s">
         <v>229</v>
       </c>
-      <c r="O3" s="2" t="s">
-        <v>230</v>
-      </c>
       <c r="P3" s="2" t="s">
-        <v>244</v>
+        <v>243</v>
       </c>
       <c r="R3" s="2" t="s">
+        <v>228</v>
+      </c>
+      <c r="S3" s="2" t="s">
         <v>229</v>
       </c>
-      <c r="S3" s="2" t="s">
-        <v>230</v>
-      </c>
       <c r="T3" s="2" t="s">
-        <v>244</v>
+        <v>243</v>
       </c>
       <c r="V3" s="2" t="s">
+        <v>228</v>
+      </c>
+      <c r="W3" s="2" t="s">
         <v>229</v>
       </c>
-      <c r="W3" s="2" t="s">
-        <v>230</v>
-      </c>
       <c r="X3" s="2" t="s">
-        <v>244</v>
+        <v>243</v>
       </c>
     </row>
     <row r="4" spans="2:24" x14ac:dyDescent="0.2">
@@ -18252,12 +18197,12 @@
     </row>
   </sheetData>
   <mergeCells count="6">
+    <mergeCell ref="B2:D2"/>
     <mergeCell ref="V2:X2"/>
     <mergeCell ref="J2:L2"/>
     <mergeCell ref="N2:P2"/>
     <mergeCell ref="R2:T2"/>
     <mergeCell ref="F2:H2"/>
-    <mergeCell ref="B2:D2"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>

<commit_message>
feat(template): v21 — polygon Type/Size overlay rows + dload Direction (phase one, pending owner review)
Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_0147GB4LGVZuqGHCRMVzZTsR
</commit_message>
<xml_diff>
--- a/docs/inputs/input_template.xlsx
+++ b/docs/inputs/input_template.xlsx
@@ -42,7 +42,7 @@
     <definedName name="solution2">mat!#REF!</definedName>
     <definedName name="version">main!$D$5</definedName>
   </definedNames>
-  <calcPr calcId="191029"/>
+  <calcPr calcId="191029" fullCalcOnLoad="1"/>
   <extLst>
     <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
       <xcalcf:calcFeatures>
@@ -60,7 +60,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="518" uniqueCount="304">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="575" uniqueCount="308">
   <si>
     <t>time</t>
   </si>
@@ -972,6 +972,18 @@
   </si>
   <si>
     <t>Mat ID = -1 --&gt; SSR reduce, Mat ID = -2 --&gt; SSR hold, Mat ID = -3 --&gt; SSR elastic</t>
+  </si>
+  <si>
+    <t>Size:</t>
+  </si>
+  <si>
+    <t>Direction:</t>
+  </si>
+  <si>
+    <t>material</t>
+  </si>
+  <si>
+    <t>Type: material zone (default), an SSR analysis overlay, or a mesh refinement region.   Size: optional target mesh element size inside the polygon (blank = global size).</t>
   </si>
 </sst>
 </file>
@@ -2879,7 +2891,7 @@
           </c:marker>
           <c:xVal>
             <c:numRef>
-              <c:f>dloads!$B$4:$B$13</c:f>
+              <c:f>dloads!$B$5:$B$14</c:f>
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="10"/>
@@ -2888,7 +2900,7 @@
           </c:xVal>
           <c:yVal>
             <c:numRef>
-              <c:f>dloads!$C$4:$C$13</c:f>
+              <c:f>dloads!$C$5:$C$14</c:f>
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="10"/>
@@ -2951,7 +2963,7 @@
           </c:marker>
           <c:xVal>
             <c:numRef>
-              <c:f>dloads!$F$4:$F$13</c:f>
+              <c:f>dloads!$F$5:$F$14</c:f>
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="10"/>
@@ -2960,7 +2972,7 @@
           </c:xVal>
           <c:yVal>
             <c:numRef>
-              <c:f>dloads!$G$4:$G$13</c:f>
+              <c:f>dloads!$G$5:$G$14</c:f>
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="10"/>
@@ -3023,7 +3035,7 @@
           </c:marker>
           <c:xVal>
             <c:numRef>
-              <c:f>dloads!$J$4:$J$13</c:f>
+              <c:f>dloads!$J$5:$J$14</c:f>
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="10"/>
@@ -3032,7 +3044,7 @@
           </c:xVal>
           <c:yVal>
             <c:numRef>
-              <c:f>dloads!$K$4:$K$13</c:f>
+              <c:f>dloads!$K$5:$K$14</c:f>
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="10"/>
@@ -3095,7 +3107,7 @@
           </c:marker>
           <c:xVal>
             <c:numRef>
-              <c:f>dloads!$N$4:$N$13</c:f>
+              <c:f>dloads!$N$5:$N$14</c:f>
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="10"/>
@@ -3104,7 +3116,7 @@
           </c:xVal>
           <c:yVal>
             <c:numRef>
-              <c:f>dloads!$O$4:$O$13</c:f>
+              <c:f>dloads!$O$5:$O$14</c:f>
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="10"/>
@@ -3167,7 +3179,7 @@
           </c:marker>
           <c:xVal>
             <c:numRef>
-              <c:f>dloads!$R$4:$R$22</c:f>
+              <c:f>dloads!$R$5:$R$23</c:f>
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="19"/>
@@ -3176,7 +3188,7 @@
           </c:xVal>
           <c:yVal>
             <c:numRef>
-              <c:f>dloads!$S$4:$S$22</c:f>
+              <c:f>dloads!$S$5:$S$23</c:f>
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="19"/>
@@ -3239,7 +3251,7 @@
           </c:marker>
           <c:xVal>
             <c:numRef>
-              <c:f>dloads!$V$4:$V$22</c:f>
+              <c:f>dloads!$V$5:$V$23</c:f>
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="19"/>
@@ -3248,7 +3260,7 @@
           </c:xVal>
           <c:yVal>
             <c:numRef>
-              <c:f>dloads!$W$4:$W$22</c:f>
+              <c:f>dloads!$W$5:$W$23</c:f>
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="19"/>
@@ -3496,7 +3508,7 @@
           </c:dPt>
           <c:xVal>
             <c:numRef>
-              <c:f>'dloads (2)'!$B$4:$B$22</c:f>
+              <c:f>'dloads (2)'!$B$5:$B$23</c:f>
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="19"/>
@@ -3505,7 +3517,7 @@
           </c:xVal>
           <c:yVal>
             <c:numRef>
-              <c:f>'dloads (2)'!$C$4:$C$22</c:f>
+              <c:f>'dloads (2)'!$C$5:$C$23</c:f>
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="19"/>
@@ -3565,7 +3577,7 @@
           </c:marker>
           <c:xVal>
             <c:numRef>
-              <c:f>'dloads (2)'!$F$4:$F$22</c:f>
+              <c:f>'dloads (2)'!$F$5:$F$23</c:f>
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="19"/>
@@ -3574,7 +3586,7 @@
           </c:xVal>
           <c:yVal>
             <c:numRef>
-              <c:f>'dloads (2)'!$G$4:$G$22</c:f>
+              <c:f>'dloads (2)'!$G$5:$G$23</c:f>
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="19"/>
@@ -3628,7 +3640,7 @@
           </c:marker>
           <c:xVal>
             <c:numRef>
-              <c:f>'dloads (2)'!$J$4:$J$22</c:f>
+              <c:f>'dloads (2)'!$J$5:$J$23</c:f>
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="19"/>
@@ -3637,7 +3649,7 @@
           </c:xVal>
           <c:yVal>
             <c:numRef>
-              <c:f>'dloads (2)'!$K$4:$K$22</c:f>
+              <c:f>'dloads (2)'!$K$5:$K$23</c:f>
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="19"/>
@@ -3691,7 +3703,7 @@
           </c:marker>
           <c:xVal>
             <c:numRef>
-              <c:f>'dloads (2)'!$N$4:$N$22</c:f>
+              <c:f>'dloads (2)'!$N$5:$N$23</c:f>
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="19"/>
@@ -3700,7 +3712,7 @@
           </c:xVal>
           <c:yVal>
             <c:numRef>
-              <c:f>'dloads (2)'!$O$4:$O$22</c:f>
+              <c:f>'dloads (2)'!$O$5:$O$23</c:f>
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="19"/>
@@ -3754,7 +3766,7 @@
           </c:marker>
           <c:xVal>
             <c:numRef>
-              <c:f>'dloads (2)'!$R$4:$R$22</c:f>
+              <c:f>'dloads (2)'!$R$5:$R$23</c:f>
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="19"/>
@@ -3763,7 +3775,7 @@
           </c:xVal>
           <c:yVal>
             <c:numRef>
-              <c:f>'dloads (2)'!$S$4:$S$22</c:f>
+              <c:f>'dloads (2)'!$S$5:$S$23</c:f>
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="19"/>
@@ -3817,7 +3829,7 @@
           </c:marker>
           <c:xVal>
             <c:numRef>
-              <c:f>'dloads (2)'!$V$4:$V$22</c:f>
+              <c:f>'dloads (2)'!$V$5:$V$23</c:f>
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="19"/>
@@ -3826,7 +3838,7 @@
           </c:xVal>
           <c:yVal>
             <c:numRef>
-              <c:f>'dloads (2)'!$W$4:$W$22</c:f>
+              <c:f>'dloads (2)'!$W$5:$W$23</c:f>
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="19"/>
@@ -6241,7 +6253,7 @@
           </c:marker>
           <c:xVal>
             <c:numRef>
-              <c:f>polygon!$A$8:$A$27</c:f>
+              <c:f>polygon!$A$10:$A$29</c:f>
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="20"/>
@@ -6250,7 +6262,7 @@
           </c:xVal>
           <c:yVal>
             <c:numRef>
-              <c:f>polygon!$B$8:$B$27</c:f>
+              <c:f>polygon!$B$10:$B$29</c:f>
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="20"/>
@@ -6310,7 +6322,7 @@
           </c:marker>
           <c:xVal>
             <c:numRef>
-              <c:f>polygon!$D$8:$D$27</c:f>
+              <c:f>polygon!$D$10:$D$29</c:f>
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="20"/>
@@ -6319,7 +6331,7 @@
           </c:xVal>
           <c:yVal>
             <c:numRef>
-              <c:f>polygon!$E$8:$E$27</c:f>
+              <c:f>polygon!$E$10:$E$29</c:f>
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="20"/>
@@ -6379,7 +6391,7 @@
           </c:marker>
           <c:xVal>
             <c:numRef>
-              <c:f>polygon!$G$8:$G$27</c:f>
+              <c:f>polygon!$G$10:$G$29</c:f>
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="20"/>
@@ -6388,7 +6400,7 @@
           </c:xVal>
           <c:yVal>
             <c:numRef>
-              <c:f>polygon!$H$8:$H$27</c:f>
+              <c:f>polygon!$H$10:$H$29</c:f>
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="20"/>
@@ -6448,7 +6460,7 @@
           </c:marker>
           <c:xVal>
             <c:numRef>
-              <c:f>polygon!$J$8:$J$27</c:f>
+              <c:f>polygon!$J$10:$J$29</c:f>
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="20"/>
@@ -6457,7 +6469,7 @@
           </c:xVal>
           <c:yVal>
             <c:numRef>
-              <c:f>polygon!$K$8:$K$27</c:f>
+              <c:f>polygon!$K$10:$K$29</c:f>
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="20"/>
@@ -6520,7 +6532,7 @@
           </c:marker>
           <c:xVal>
             <c:numRef>
-              <c:f>polygon!$M$8:$M$27</c:f>
+              <c:f>polygon!$M$10:$M$29</c:f>
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="20"/>
@@ -6529,7 +6541,7 @@
           </c:xVal>
           <c:yVal>
             <c:numRef>
-              <c:f>polygon!$N$8:$N$27</c:f>
+              <c:f>polygon!$N$10:$N$29</c:f>
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="20"/>
@@ -6592,7 +6604,7 @@
           </c:marker>
           <c:xVal>
             <c:numRef>
-              <c:f>polygon!$P$8:$P$27</c:f>
+              <c:f>polygon!$P$10:$P$29</c:f>
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="20"/>
@@ -6601,7 +6613,7 @@
           </c:xVal>
           <c:yVal>
             <c:numRef>
-              <c:f>polygon!$Q$8:$Q$27</c:f>
+              <c:f>polygon!$Q$10:$Q$29</c:f>
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="20"/>
@@ -6664,7 +6676,7 @@
           </c:marker>
           <c:xVal>
             <c:numRef>
-              <c:f>polygon!$S$8:$S$27</c:f>
+              <c:f>polygon!$S$10:$S$29</c:f>
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="20"/>
@@ -6673,7 +6685,7 @@
           </c:xVal>
           <c:yVal>
             <c:numRef>
-              <c:f>polygon!$T$8:$T$27</c:f>
+              <c:f>polygon!$T$10:$T$29</c:f>
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="20"/>
@@ -6736,7 +6748,7 @@
           </c:marker>
           <c:xVal>
             <c:numRef>
-              <c:f>polygon!$V$8:$V$27</c:f>
+              <c:f>polygon!$V$10:$V$29</c:f>
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="20"/>
@@ -6745,7 +6757,7 @@
           </c:xVal>
           <c:yVal>
             <c:numRef>
-              <c:f>polygon!$W$8:$W$27</c:f>
+              <c:f>polygon!$W$10:$W$29</c:f>
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="20"/>
@@ -6808,7 +6820,7 @@
           </c:marker>
           <c:xVal>
             <c:numRef>
-              <c:f>polygon!$Y$8:$Y$27</c:f>
+              <c:f>polygon!$Y$10:$Y$29</c:f>
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="20"/>
@@ -6817,7 +6829,7 @@
           </c:xVal>
           <c:yVal>
             <c:numRef>
-              <c:f>polygon!$Z$8:$Z$27</c:f>
+              <c:f>polygon!$Z$10:$Z$29</c:f>
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="20"/>
@@ -6880,7 +6892,7 @@
           </c:marker>
           <c:xVal>
             <c:numRef>
-              <c:f>polygon!$AB$8:$AB$27</c:f>
+              <c:f>polygon!$AB$10:$AB$29</c:f>
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="20"/>
@@ -6889,7 +6901,7 @@
           </c:xVal>
           <c:yVal>
             <c:numRef>
-              <c:f>polygon!$AC$8:$AC$27</c:f>
+              <c:f>polygon!$AC$10:$AC$29</c:f>
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="20"/>
@@ -6949,7 +6961,7 @@
           </c:marker>
           <c:xVal>
             <c:numRef>
-              <c:f>polygon!$AE$8:$AE$27</c:f>
+              <c:f>polygon!$AE$10:$AE$29</c:f>
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="20"/>
@@ -6958,7 +6970,7 @@
           </c:xVal>
           <c:yVal>
             <c:numRef>
-              <c:f>polygon!$AF$8:$AF$27</c:f>
+              <c:f>polygon!$AF$10:$AF$29</c:f>
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="20"/>
@@ -7018,7 +7030,7 @@
           </c:marker>
           <c:xVal>
             <c:numRef>
-              <c:f>polygon!$AH$8:$AH$27</c:f>
+              <c:f>polygon!$AH$10:$AH$29</c:f>
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="20"/>
@@ -7027,7 +7039,7 @@
           </c:xVal>
           <c:yVal>
             <c:numRef>
-              <c:f>polygon!$AI$8:$AI$27</c:f>
+              <c:f>polygon!$AI$10:$AI$29</c:f>
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="20"/>
@@ -7087,7 +7099,7 @@
           </c:marker>
           <c:xVal>
             <c:numRef>
-              <c:f>polygon!$AK$8:$AK$27</c:f>
+              <c:f>polygon!$AK$10:$AK$29</c:f>
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="20"/>
@@ -7096,7 +7108,7 @@
           </c:xVal>
           <c:yVal>
             <c:numRef>
-              <c:f>polygon!$AL$8:$AL$27</c:f>
+              <c:f>polygon!$AL$10:$AL$29</c:f>
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="20"/>
@@ -7156,7 +7168,7 @@
           </c:marker>
           <c:xVal>
             <c:numRef>
-              <c:f>polygon!$AN$8:$AN$27</c:f>
+              <c:f>polygon!$AN$10:$AN$29</c:f>
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="20"/>
@@ -7165,7 +7177,7 @@
           </c:xVal>
           <c:yVal>
             <c:numRef>
-              <c:f>polygon!$AO$8:$AO$27</c:f>
+              <c:f>polygon!$AO$10:$AO$29</c:f>
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="20"/>
@@ -7225,7 +7237,7 @@
           </c:marker>
           <c:xVal>
             <c:numRef>
-              <c:f>polygon!$AQ$8:$AQ$27</c:f>
+              <c:f>polygon!$AQ$10:$AQ$29</c:f>
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="20"/>
@@ -7234,7 +7246,7 @@
           </c:xVal>
           <c:yVal>
             <c:numRef>
-              <c:f>polygon!$AR$8:$AR$27</c:f>
+              <c:f>polygon!$AR$10:$AR$29</c:f>
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="20"/>
@@ -8965,7 +8977,7 @@
         <v>13</v>
       </c>
       <c r="D5" s="30">
-        <v>20</v>
+        <v>21</v>
       </c>
     </row>
     <row r="7" spans="1:7" x14ac:dyDescent="0.2">
@@ -9329,7 +9341,7 @@
 
 <file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0900-000000000000}">
-  <dimension ref="B2:X22"/>
+  <dimension ref="B2:X23"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="3" customWidth="1"/>
@@ -9379,80 +9391,92 @@
       <c r="X2" s="62"/>
     </row>
     <row r="3" spans="2:24" x14ac:dyDescent="0.2">
-      <c r="B3" s="2" t="s">
+      <c r="B3" s="38" t="s">
+        <v>305</v>
+      </c>
+      <c r="C3" s="38"/>
+      <c r="D3" s="39"/>
+      <c r="F3" s="38" t="s">
+        <v>305</v>
+      </c>
+      <c r="G3" s="38"/>
+      <c r="H3" s="39"/>
+      <c r="J3" s="38" t="s">
+        <v>305</v>
+      </c>
+      <c r="K3" s="38"/>
+      <c r="L3" s="39"/>
+      <c r="N3" s="38" t="s">
+        <v>305</v>
+      </c>
+      <c r="O3" s="38"/>
+      <c r="P3" s="39"/>
+      <c r="R3" s="38" t="s">
+        <v>305</v>
+      </c>
+      <c r="S3" s="38"/>
+      <c r="T3" s="39"/>
+      <c r="V3" s="38" t="s">
+        <v>305</v>
+      </c>
+      <c r="W3" s="38"/>
+      <c r="X3" s="39"/>
+    </row>
+    <row r="4" spans="2:24" x14ac:dyDescent="0.2">
+      <c r="B4" s="2" t="s">
         <v>228</v>
       </c>
-      <c r="C3" s="2" t="s">
+      <c r="C4" s="2" t="s">
         <v>229</v>
       </c>
-      <c r="D3" s="2" t="s">
+      <c r="D4" s="2" t="s">
         <v>243</v>
       </c>
-      <c r="F3" s="2" t="s">
+      <c r="F4" s="2" t="s">
         <v>228</v>
       </c>
-      <c r="G3" s="2" t="s">
+      <c r="G4" s="2" t="s">
         <v>229</v>
       </c>
-      <c r="H3" s="2" t="s">
+      <c r="H4" s="2" t="s">
         <v>243</v>
       </c>
-      <c r="J3" s="2" t="s">
+      <c r="J4" s="2" t="s">
         <v>228</v>
       </c>
-      <c r="K3" s="2" t="s">
+      <c r="K4" s="2" t="s">
         <v>229</v>
       </c>
-      <c r="L3" s="2" t="s">
+      <c r="L4" s="2" t="s">
         <v>243</v>
       </c>
-      <c r="N3" s="2" t="s">
+      <c r="N4" s="2" t="s">
         <v>228</v>
       </c>
-      <c r="O3" s="2" t="s">
+      <c r="O4" s="2" t="s">
         <v>229</v>
       </c>
-      <c r="P3" s="2" t="s">
+      <c r="P4" s="2" t="s">
         <v>243</v>
       </c>
-      <c r="R3" s="2" t="s">
+      <c r="R4" s="2" t="s">
         <v>228</v>
       </c>
-      <c r="S3" s="2" t="s">
+      <c r="S4" s="2" t="s">
         <v>229</v>
       </c>
-      <c r="T3" s="2" t="s">
+      <c r="T4" s="2" t="s">
         <v>243</v>
       </c>
-      <c r="V3" s="2" t="s">
+      <c r="V4" s="2" t="s">
         <v>228</v>
       </c>
-      <c r="W3" s="2" t="s">
+      <c r="W4" s="2" t="s">
         <v>229</v>
       </c>
-      <c r="X3" s="2" t="s">
+      <c r="X4" s="2" t="s">
         <v>243</v>
       </c>
-    </row>
-    <row r="4" spans="2:24" x14ac:dyDescent="0.2">
-      <c r="B4" s="3"/>
-      <c r="C4" s="3"/>
-      <c r="D4" s="3"/>
-      <c r="F4" s="3"/>
-      <c r="G4" s="3"/>
-      <c r="H4" s="3"/>
-      <c r="J4" s="3"/>
-      <c r="K4" s="3"/>
-      <c r="L4" s="3"/>
-      <c r="N4" s="3"/>
-      <c r="O4" s="3"/>
-      <c r="P4" s="3"/>
-      <c r="R4" s="3"/>
-      <c r="S4" s="3"/>
-      <c r="T4" s="3"/>
-      <c r="V4" s="3"/>
-      <c r="W4" s="3"/>
-      <c r="X4" s="3"/>
     </row>
     <row r="5" spans="2:24" x14ac:dyDescent="0.2">
       <c r="B5" s="3"/>
@@ -9814,15 +9838,46 @@
       <c r="W22" s="3"/>
       <c r="X22" s="3"/>
     </row>
+    <row r="23" spans="2:24" x14ac:dyDescent="0.2">
+      <c r="B23" s="3"/>
+      <c r="C23" s="3"/>
+      <c r="D23" s="3"/>
+      <c r="F23" s="3"/>
+      <c r="G23" s="3"/>
+      <c r="H23" s="3"/>
+      <c r="J23" s="3"/>
+      <c r="K23" s="3"/>
+      <c r="L23" s="3"/>
+      <c r="N23" s="3"/>
+      <c r="O23" s="3"/>
+      <c r="P23" s="3"/>
+      <c r="R23" s="3"/>
+      <c r="S23" s="3"/>
+      <c r="T23" s="3"/>
+      <c r="V23" s="3"/>
+      <c r="W23" s="3"/>
+      <c r="X23" s="3"/>
+    </row>
   </sheetData>
-  <mergeCells count="6">
+  <mergeCells count="12">
     <mergeCell ref="B2:D2"/>
     <mergeCell ref="V2:X2"/>
     <mergeCell ref="J2:L2"/>
     <mergeCell ref="N2:P2"/>
     <mergeCell ref="R2:T2"/>
     <mergeCell ref="F2:H2"/>
+    <mergeCell ref="B3:C3"/>
+    <mergeCell ref="F3:G3"/>
+    <mergeCell ref="J3:K3"/>
+    <mergeCell ref="N3:O3"/>
+    <mergeCell ref="R3:S3"/>
+    <mergeCell ref="V3:W3"/>
   </mergeCells>
+  <dataValidations count="1">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="D3 H3 L3 P3 T3 X3">
+      <formula1>"normal,vertical"</formula1>
+    </dataValidation>
+  </dataValidations>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
@@ -15875,7 +15930,7 @@
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0400-000000000000}">
-  <dimension ref="A2:AR27"/>
+  <dimension ref="A2:AR29"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="2" width="10.83203125" style="1" customWidth="1"/>
@@ -15904,7 +15959,7 @@
         <v>179</v>
       </c>
       <c r="G2" s="9" t="s">
-        <v>303</v>
+        <v>307</v>
       </c>
     </row>
     <row r="4" spans="1:44" x14ac:dyDescent="0.2">
@@ -15979,368 +16034,458 @@
     </row>
     <row r="5" spans="1:44" x14ac:dyDescent="0.2">
       <c r="A5" s="38" t="s">
-        <v>176</v>
-      </c>
-      <c r="B5" s="39">
-        <v>1</v>
+        <v>198</v>
+      </c>
+      <c r="B5" s="39" t="s">
+        <v>306</v>
       </c>
       <c r="D5" s="38" t="s">
-        <v>176</v>
-      </c>
-      <c r="E5" s="39">
-        <v>2</v>
+        <v>198</v>
+      </c>
+      <c r="E5" s="39" t="s">
+        <v>306</v>
       </c>
       <c r="G5" s="38" t="s">
-        <v>176</v>
-      </c>
-      <c r="H5" s="39">
-        <v>3</v>
+        <v>198</v>
+      </c>
+      <c r="H5" s="39" t="s">
+        <v>306</v>
       </c>
       <c r="J5" s="38" t="s">
-        <v>176</v>
-      </c>
-      <c r="K5" s="39">
-        <v>4</v>
+        <v>198</v>
+      </c>
+      <c r="K5" s="39" t="s">
+        <v>306</v>
       </c>
       <c r="M5" s="38" t="s">
-        <v>176</v>
-      </c>
-      <c r="N5" s="39">
-        <v>5</v>
+        <v>198</v>
+      </c>
+      <c r="N5" s="39" t="s">
+        <v>306</v>
       </c>
       <c r="P5" s="38" t="s">
-        <v>176</v>
-      </c>
-      <c r="Q5" s="39">
-        <v>6</v>
+        <v>198</v>
+      </c>
+      <c r="Q5" s="39" t="s">
+        <v>306</v>
       </c>
       <c r="R5" s="1"/>
       <c r="S5" s="38" t="s">
-        <v>176</v>
-      </c>
-      <c r="T5" s="39">
-        <v>7</v>
+        <v>198</v>
+      </c>
+      <c r="T5" s="39" t="s">
+        <v>306</v>
       </c>
       <c r="U5" s="1"/>
       <c r="V5" s="38" t="s">
-        <v>176</v>
-      </c>
-      <c r="W5" s="39">
-        <v>8</v>
+        <v>198</v>
+      </c>
+      <c r="W5" s="39" t="s">
+        <v>306</v>
       </c>
       <c r="X5" s="1"/>
       <c r="Y5" s="38" t="s">
-        <v>176</v>
-      </c>
-      <c r="Z5" s="39">
-        <v>9</v>
+        <v>198</v>
+      </c>
+      <c r="Z5" s="39" t="s">
+        <v>306</v>
       </c>
       <c r="AA5" s="1"/>
       <c r="AB5" s="38" t="s">
-        <v>176</v>
-      </c>
-      <c r="AC5" s="39">
-        <v>10</v>
+        <v>198</v>
+      </c>
+      <c r="AC5" s="39" t="s">
+        <v>306</v>
       </c>
       <c r="AE5" s="38" t="s">
-        <v>176</v>
-      </c>
-      <c r="AF5" s="39">
-        <v>11</v>
+        <v>198</v>
+      </c>
+      <c r="AF5" s="39" t="s">
+        <v>306</v>
       </c>
       <c r="AG5" s="1"/>
       <c r="AH5" s="38" t="s">
-        <v>176</v>
-      </c>
-      <c r="AI5" s="39">
-        <v>12</v>
+        <v>198</v>
+      </c>
+      <c r="AI5" s="39" t="s">
+        <v>306</v>
       </c>
       <c r="AJ5" s="1"/>
       <c r="AK5" s="38" t="s">
-        <v>176</v>
-      </c>
-      <c r="AL5" s="39">
-        <v>13</v>
+        <v>198</v>
+      </c>
+      <c r="AL5" s="39" t="s">
+        <v>306</v>
       </c>
       <c r="AM5" s="1"/>
       <c r="AN5" s="38" t="s">
-        <v>176</v>
-      </c>
-      <c r="AO5" s="39">
-        <v>14</v>
+        <v>198</v>
+      </c>
+      <c r="AO5" s="39" t="s">
+        <v>306</v>
       </c>
       <c r="AP5" s="1"/>
       <c r="AQ5" s="38" t="s">
+        <v>198</v>
+      </c>
+      <c r="AR5" s="39" t="s">
+        <v>306</v>
+      </c>
+    </row>
+    <row r="6" spans="1:44" x14ac:dyDescent="0.2">
+      <c r="A6" s="38" t="s">
         <v>176</v>
       </c>
-      <c r="AR5" s="39">
+      <c r="B6" s="39">
+        <v>1</v>
+      </c>
+      <c r="D6" s="38" t="s">
+        <v>176</v>
+      </c>
+      <c r="E6" s="39">
+        <v>2</v>
+      </c>
+      <c r="G6" s="38" t="s">
+        <v>176</v>
+      </c>
+      <c r="H6" s="39">
+        <v>3</v>
+      </c>
+      <c r="J6" s="38" t="s">
+        <v>176</v>
+      </c>
+      <c r="K6" s="39">
+        <v>4</v>
+      </c>
+      <c r="M6" s="38" t="s">
+        <v>176</v>
+      </c>
+      <c r="N6" s="39">
+        <v>5</v>
+      </c>
+      <c r="P6" s="38" t="s">
+        <v>176</v>
+      </c>
+      <c r="Q6" s="39">
+        <v>6</v>
+      </c>
+      <c r="R6" s="1"/>
+      <c r="S6" s="38" t="s">
+        <v>176</v>
+      </c>
+      <c r="T6" s="39">
+        <v>7</v>
+      </c>
+      <c r="U6" s="1"/>
+      <c r="V6" s="38" t="s">
+        <v>176</v>
+      </c>
+      <c r="W6" s="39">
+        <v>8</v>
+      </c>
+      <c r="X6" s="1"/>
+      <c r="Y6" s="38" t="s">
+        <v>176</v>
+      </c>
+      <c r="Z6" s="39">
+        <v>9</v>
+      </c>
+      <c r="AA6" s="1"/>
+      <c r="AB6" s="38" t="s">
+        <v>176</v>
+      </c>
+      <c r="AC6" s="39">
+        <v>10</v>
+      </c>
+      <c r="AE6" s="38" t="s">
+        <v>176</v>
+      </c>
+      <c r="AF6" s="39">
+        <v>11</v>
+      </c>
+      <c r="AG6" s="1"/>
+      <c r="AH6" s="38" t="s">
+        <v>176</v>
+      </c>
+      <c r="AI6" s="39">
+        <v>12</v>
+      </c>
+      <c r="AJ6" s="1"/>
+      <c r="AK6" s="38" t="s">
+        <v>176</v>
+      </c>
+      <c r="AL6" s="39">
+        <v>13</v>
+      </c>
+      <c r="AM6" s="1"/>
+      <c r="AN6" s="38" t="s">
+        <v>176</v>
+      </c>
+      <c r="AO6" s="39">
+        <v>14</v>
+      </c>
+      <c r="AP6" s="1"/>
+      <c r="AQ6" s="38" t="s">
+        <v>176</v>
+      </c>
+      <c r="AR6" s="39">
         <v>15</v>
       </c>
     </row>
-    <row r="6" spans="1:44" x14ac:dyDescent="0.2">
-      <c r="A6" s="58" t="str">
-        <f>IF(B5=-1,"SSR reduce",IF(B5=-2,"SSR hold",IF(B5=-3,"SSR elastic",_xlfn.XLOOKUP(B5,mat!$A:$A, mat!$B:$B,"") &amp; "")))</f>
+    <row r="7" spans="1:44" x14ac:dyDescent="0.2">
+      <c r="A7" s="58" t="str">
+        <f>IF(OR(B5="",B5="material"),_xlfn.XLOOKUP(B6,mat!$A:$A, mat!$B:$B,"") &amp; "",B5)</f>
         <v/>
       </c>
-      <c r="B6" s="57"/>
-      <c r="D6" s="58" t="str">
-        <f>IF(E5=-1,"SSR reduce",IF(E5=-2,"SSR hold",IF(E5=-3,"SSR elastic",_xlfn.XLOOKUP(E5,mat!$A:$A, mat!$B:$B,"") &amp; "")))</f>
+      <c r="B7" s="57"/>
+      <c r="D7" s="58" t="str">
+        <f>IF(OR(E5="",E5="material"),_xlfn.XLOOKUP(E6,mat!$A:$A, mat!$B:$B,"") &amp; "",E5)</f>
         <v/>
       </c>
-      <c r="E6" s="57"/>
-      <c r="G6" s="58" t="str">
-        <f>IF(H5=-1,"SSR reduce",IF(H5=-2,"SSR hold",IF(H5=-3,"SSR elastic",_xlfn.XLOOKUP(H5,mat!$A:$A, mat!$B:$B,"") &amp; "")))</f>
+      <c r="E7" s="57"/>
+      <c r="G7" s="58" t="str">
+        <f>IF(OR(H5="",H5="material"),_xlfn.XLOOKUP(H6,mat!$A:$A, mat!$B:$B,"") &amp; "",H5)</f>
         <v/>
       </c>
-      <c r="H6" s="57"/>
-      <c r="J6" s="58" t="str">
-        <f>IF(K5=-1,"SSR reduce",IF(K5=-2,"SSR hold",IF(K5=-3,"SSR elastic",_xlfn.XLOOKUP(K5,mat!$A:$A, mat!$B:$B,"") &amp; "")))</f>
+      <c r="H7" s="57"/>
+      <c r="J7" s="58" t="str">
+        <f>IF(OR(K5="",K5="material"),_xlfn.XLOOKUP(K6,mat!$A:$A, mat!$B:$B,"") &amp; "",K5)</f>
         <v/>
       </c>
-      <c r="K6" s="57"/>
-      <c r="M6" s="58" t="str">
-        <f>IF(N5=-1,"SSR reduce",IF(N5=-2,"SSR hold",IF(N5=-3,"SSR elastic",_xlfn.XLOOKUP(N5,mat!$A:$A, mat!$B:$B,"") &amp; "")))</f>
+      <c r="K7" s="57"/>
+      <c r="M7" s="58" t="str">
+        <f>IF(OR(N5="",N5="material"),_xlfn.XLOOKUP(N6,mat!$A:$A, mat!$B:$B,"") &amp; "",N5)</f>
         <v/>
       </c>
-      <c r="N6" s="57"/>
-      <c r="P6" s="58" t="str">
-        <f>IF(Q5=-1,"SSR reduce",IF(Q5=-2,"SSR hold",IF(Q5=-3,"SSR elastic",_xlfn.XLOOKUP(Q5,mat!$A:$A, mat!$B:$B,"") &amp; "")))</f>
+      <c r="N7" s="57"/>
+      <c r="P7" s="58" t="str">
+        <f>IF(OR(Q5="",Q5="material"),_xlfn.XLOOKUP(Q6,mat!$A:$A, mat!$B:$B,"") &amp; "",Q5)</f>
         <v/>
       </c>
-      <c r="Q6" s="57"/>
-      <c r="R6" s="1"/>
-      <c r="S6" s="58" t="str">
-        <f>IF(T5=-1,"SSR reduce",IF(T5=-2,"SSR hold",IF(T5=-3,"SSR elastic",_xlfn.XLOOKUP(T5,mat!$A:$A, mat!$B:$B,"") &amp; "")))</f>
+      <c r="Q7" s="57"/>
+      <c r="R7" s="1"/>
+      <c r="S7" s="58" t="str">
+        <f>IF(OR(T5="",T5="material"),_xlfn.XLOOKUP(T6,mat!$A:$A, mat!$B:$B,"") &amp; "",T5)</f>
         <v/>
       </c>
-      <c r="T6" s="57"/>
-      <c r="U6" s="1"/>
-      <c r="V6" s="58" t="str">
-        <f>IF(W5=-1,"SSR reduce",IF(W5=-2,"SSR hold",IF(W5=-3,"SSR elastic",_xlfn.XLOOKUP(W5,mat!$A:$A, mat!$B:$B,"") &amp; "")))</f>
+      <c r="T7" s="57"/>
+      <c r="U7" s="1"/>
+      <c r="V7" s="58" t="str">
+        <f>IF(OR(W5="",W5="material"),_xlfn.XLOOKUP(W6,mat!$A:$A, mat!$B:$B,"") &amp; "",W5)</f>
         <v/>
       </c>
-      <c r="W6" s="57"/>
-      <c r="X6" s="1"/>
-      <c r="Y6" s="58" t="str">
-        <f>IF(Z5=-1,"SSR reduce",IF(Z5=-2,"SSR hold",IF(Z5=-3,"SSR elastic",_xlfn.XLOOKUP(Z5,mat!$A:$A, mat!$B:$B,"") &amp; "")))</f>
+      <c r="W7" s="57"/>
+      <c r="X7" s="1"/>
+      <c r="Y7" s="58" t="str">
+        <f>IF(OR(Z5="",Z5="material"),_xlfn.XLOOKUP(Z6,mat!$A:$A, mat!$B:$B,"") &amp; "",Z5)</f>
         <v/>
       </c>
-      <c r="Z6" s="57"/>
-      <c r="AA6" s="1"/>
-      <c r="AB6" s="58" t="str">
-        <f>IF(AC5=-1,"SSR reduce",IF(AC5=-2,"SSR hold",IF(AC5=-3,"SSR elastic",_xlfn.XLOOKUP(AC5,mat!$A:$A, mat!$B:$B,"") &amp; "")))</f>
+      <c r="Z7" s="57"/>
+      <c r="AA7" s="1"/>
+      <c r="AB7" s="58" t="str">
+        <f>IF(OR(AC5="",AC5="material"),_xlfn.XLOOKUP(AC6,mat!$A:$A, mat!$B:$B,"") &amp; "",AC5)</f>
         <v/>
       </c>
-      <c r="AC6" s="57"/>
-      <c r="AE6" s="58" t="str">
-        <f>IF(AF5=-1,"SSR reduce",IF(AF5=-2,"SSR hold",IF(AF5=-3,"SSR elastic",_xlfn.XLOOKUP(AF5,mat!$A:$A, mat!$B:$B,"") &amp; "")))</f>
+      <c r="AC7" s="57"/>
+      <c r="AE7" s="58" t="str">
+        <f>IF(OR(AF5="",AF5="material"),_xlfn.XLOOKUP(AF6,mat!$A:$A, mat!$B:$B,"") &amp; "",AF5)</f>
         <v/>
       </c>
-      <c r="AF6" s="57"/>
-      <c r="AG6" s="1"/>
-      <c r="AH6" s="58" t="str">
-        <f>IF(AI5=-1,"SSR reduce",IF(AI5=-2,"SSR hold",IF(AI5=-3,"SSR elastic",_xlfn.XLOOKUP(AI5,mat!$A:$A, mat!$B:$B,"") &amp; "")))</f>
+      <c r="AF7" s="57"/>
+      <c r="AG7" s="1"/>
+      <c r="AH7" s="58" t="str">
+        <f>IF(OR(AI5="",AI5="material"),_xlfn.XLOOKUP(AI6,mat!$A:$A, mat!$B:$B,"") &amp; "",AI5)</f>
         <v/>
       </c>
-      <c r="AI6" s="57"/>
-      <c r="AJ6" s="1"/>
-      <c r="AK6" s="58" t="str">
-        <f>IF(AL5=-1,"SSR reduce",IF(AL5=-2,"SSR hold",IF(AL5=-3,"SSR elastic",_xlfn.XLOOKUP(AL5,mat!$A:$A, mat!$B:$B,"") &amp; "")))</f>
+      <c r="AI7" s="57"/>
+      <c r="AJ7" s="1"/>
+      <c r="AK7" s="58" t="str">
+        <f>IF(OR(AL5="",AL5="material"),_xlfn.XLOOKUP(AL6,mat!$A:$A, mat!$B:$B,"") &amp; "",AL5)</f>
         <v/>
       </c>
-      <c r="AL6" s="57"/>
-      <c r="AM6" s="1"/>
-      <c r="AN6" s="58" t="str">
-        <f>IF(AO5=-1,"SSR reduce",IF(AO5=-2,"SSR hold",IF(AO5=-3,"SSR elastic",_xlfn.XLOOKUP(AO5,mat!$A:$A, mat!$B:$B,"") &amp; "")))</f>
+      <c r="AL7" s="57"/>
+      <c r="AM7" s="1"/>
+      <c r="AN7" s="58" t="str">
+        <f>IF(OR(AO5="",AO5="material"),_xlfn.XLOOKUP(AO6,mat!$A:$A, mat!$B:$B,"") &amp; "",AO5)</f>
         <v/>
       </c>
-      <c r="AO6" s="57"/>
-      <c r="AP6" s="1"/>
-      <c r="AQ6" s="58" t="str">
-        <f>IF(AR5=-1,"SSR reduce",IF(AR5=-2,"SSR hold",IF(AR5=-3,"SSR elastic",_xlfn.XLOOKUP(AR5,mat!$A:$A, mat!$B:$B,"") &amp; "")))</f>
+      <c r="AO7" s="57"/>
+      <c r="AP7" s="1"/>
+      <c r="AQ7" s="58" t="str">
+        <f>IF(OR(AR5="",AR5="material"),_xlfn.XLOOKUP(AR6,mat!$A:$A, mat!$B:$B,"") &amp; "",AR5)</f>
         <v/>
       </c>
-      <c r="AR6" s="57"/>
-    </row>
-    <row r="7" spans="1:44" x14ac:dyDescent="0.2">
-      <c r="A7" s="2" t="s">
+      <c r="AR7" s="57"/>
+    </row>
+    <row r="8" spans="1:44" x14ac:dyDescent="0.2">
+      <c r="A8" s="38" t="s">
+        <v>304</v>
+      </c>
+      <c r="B8" s="39"/>
+      <c r="D8" s="38" t="s">
+        <v>304</v>
+      </c>
+      <c r="E8" s="39"/>
+      <c r="G8" s="38" t="s">
+        <v>304</v>
+      </c>
+      <c r="H8" s="39"/>
+      <c r="J8" s="38" t="s">
+        <v>304</v>
+      </c>
+      <c r="K8" s="39"/>
+      <c r="M8" s="38" t="s">
+        <v>304</v>
+      </c>
+      <c r="N8" s="39"/>
+      <c r="P8" s="38" t="s">
+        <v>304</v>
+      </c>
+      <c r="Q8" s="39"/>
+      <c r="R8" s="1"/>
+      <c r="S8" s="38" t="s">
+        <v>304</v>
+      </c>
+      <c r="T8" s="39"/>
+      <c r="U8" s="1"/>
+      <c r="V8" s="38" t="s">
+        <v>304</v>
+      </c>
+      <c r="W8" s="39"/>
+      <c r="X8" s="1"/>
+      <c r="Y8" s="38" t="s">
+        <v>304</v>
+      </c>
+      <c r="Z8" s="39"/>
+      <c r="AA8" s="1"/>
+      <c r="AB8" s="38" t="s">
+        <v>304</v>
+      </c>
+      <c r="AC8" s="39"/>
+      <c r="AE8" s="38" t="s">
+        <v>304</v>
+      </c>
+      <c r="AF8" s="39"/>
+      <c r="AG8" s="1"/>
+      <c r="AH8" s="38" t="s">
+        <v>304</v>
+      </c>
+      <c r="AI8" s="39"/>
+      <c r="AJ8" s="1"/>
+      <c r="AK8" s="38" t="s">
+        <v>304</v>
+      </c>
+      <c r="AL8" s="39"/>
+      <c r="AM8" s="1"/>
+      <c r="AN8" s="38" t="s">
+        <v>304</v>
+      </c>
+      <c r="AO8" s="39"/>
+      <c r="AP8" s="1"/>
+      <c r="AQ8" s="38" t="s">
+        <v>304</v>
+      </c>
+      <c r="AR8" s="39"/>
+    </row>
+    <row r="9" spans="1:44" x14ac:dyDescent="0.2">
+      <c r="A9" s="2" t="s">
         <v>177</v>
       </c>
-      <c r="B7" s="2" t="s">
+      <c r="B9" s="2" t="s">
         <v>178</v>
       </c>
-      <c r="D7" s="2" t="s">
+      <c r="D9" s="2" t="s">
         <v>177</v>
       </c>
-      <c r="E7" s="2" t="s">
+      <c r="E9" s="2" t="s">
         <v>178</v>
       </c>
-      <c r="G7" s="2" t="s">
+      <c r="G9" s="2" t="s">
         <v>177</v>
       </c>
-      <c r="H7" s="2" t="s">
+      <c r="H9" s="2" t="s">
         <v>178</v>
       </c>
-      <c r="J7" s="2" t="s">
+      <c r="J9" s="2" t="s">
         <v>177</v>
       </c>
-      <c r="K7" s="2" t="s">
+      <c r="K9" s="2" t="s">
         <v>178</v>
       </c>
-      <c r="M7" s="2" t="s">
+      <c r="M9" s="2" t="s">
         <v>177</v>
       </c>
-      <c r="N7" s="2" t="s">
+      <c r="N9" s="2" t="s">
         <v>178</v>
       </c>
-      <c r="P7" s="2" t="s">
+      <c r="P9" s="2" t="s">
         <v>177</v>
       </c>
-      <c r="Q7" s="2" t="s">
+      <c r="Q9" s="2" t="s">
         <v>178</v>
       </c>
-      <c r="R7" s="1"/>
-      <c r="S7" s="2" t="s">
+      <c r="R9" s="1"/>
+      <c r="S9" s="2" t="s">
         <v>177</v>
       </c>
-      <c r="T7" s="2" t="s">
+      <c r="T9" s="2" t="s">
         <v>178</v>
       </c>
-      <c r="U7" s="1"/>
-      <c r="V7" s="2" t="s">
+      <c r="U9" s="1"/>
+      <c r="V9" s="2" t="s">
         <v>177</v>
       </c>
-      <c r="W7" s="2" t="s">
+      <c r="W9" s="2" t="s">
         <v>178</v>
       </c>
-      <c r="X7" s="1"/>
-      <c r="Y7" s="2" t="s">
+      <c r="X9" s="1"/>
+      <c r="Y9" s="2" t="s">
         <v>177</v>
       </c>
-      <c r="Z7" s="2" t="s">
+      <c r="Z9" s="2" t="s">
         <v>178</v>
       </c>
-      <c r="AA7" s="1"/>
-      <c r="AB7" s="2" t="s">
+      <c r="AA9" s="1"/>
+      <c r="AB9" s="2" t="s">
         <v>177</v>
       </c>
-      <c r="AC7" s="2" t="s">
+      <c r="AC9" s="2" t="s">
         <v>178</v>
       </c>
-      <c r="AE7" s="2" t="s">
+      <c r="AE9" s="2" t="s">
         <v>177</v>
       </c>
-      <c r="AF7" s="2" t="s">
+      <c r="AF9" s="2" t="s">
         <v>178</v>
       </c>
-      <c r="AG7" s="1"/>
-      <c r="AH7" s="2" t="s">
+      <c r="AG9" s="1"/>
+      <c r="AH9" s="2" t="s">
         <v>177</v>
       </c>
-      <c r="AI7" s="2" t="s">
+      <c r="AI9" s="2" t="s">
         <v>178</v>
       </c>
-      <c r="AJ7" s="1"/>
-      <c r="AK7" s="2" t="s">
+      <c r="AJ9" s="1"/>
+      <c r="AK9" s="2" t="s">
         <v>177</v>
       </c>
-      <c r="AL7" s="2" t="s">
+      <c r="AL9" s="2" t="s">
         <v>178</v>
       </c>
-      <c r="AM7" s="1"/>
-      <c r="AN7" s="2" t="s">
+      <c r="AM9" s="1"/>
+      <c r="AN9" s="2" t="s">
         <v>177</v>
       </c>
-      <c r="AO7" s="2" t="s">
+      <c r="AO9" s="2" t="s">
         <v>178</v>
       </c>
-      <c r="AP7" s="1"/>
-      <c r="AQ7" s="2" t="s">
+      <c r="AP9" s="1"/>
+      <c r="AQ9" s="2" t="s">
         <v>177</v>
       </c>
-      <c r="AR7" s="2" t="s">
+      <c r="AR9" s="2" t="s">
         <v>178</v>
       </c>
-    </row>
-    <row r="8" spans="1:44" x14ac:dyDescent="0.2">
-      <c r="A8" s="3"/>
-      <c r="B8" s="3"/>
-      <c r="D8" s="3"/>
-      <c r="E8" s="3"/>
-      <c r="G8" s="3"/>
-      <c r="H8" s="3"/>
-      <c r="J8" s="3"/>
-      <c r="K8" s="3"/>
-      <c r="M8" s="3"/>
-      <c r="N8" s="3"/>
-      <c r="P8" s="3"/>
-      <c r="Q8" s="3"/>
-      <c r="R8" s="1"/>
-      <c r="S8" s="3"/>
-      <c r="T8" s="3"/>
-      <c r="U8" s="1"/>
-      <c r="V8" s="3"/>
-      <c r="W8" s="3"/>
-      <c r="X8" s="1"/>
-      <c r="Y8" s="3"/>
-      <c r="Z8" s="3"/>
-      <c r="AA8" s="1"/>
-      <c r="AB8" s="3"/>
-      <c r="AC8" s="3"/>
-      <c r="AE8" s="3"/>
-      <c r="AF8" s="3"/>
-      <c r="AG8" s="1"/>
-      <c r="AH8" s="3"/>
-      <c r="AI8" s="3"/>
-      <c r="AJ8" s="1"/>
-      <c r="AK8" s="3"/>
-      <c r="AL8" s="3"/>
-      <c r="AM8" s="1"/>
-      <c r="AN8" s="3"/>
-      <c r="AO8" s="3"/>
-      <c r="AP8" s="1"/>
-      <c r="AQ8" s="3"/>
-      <c r="AR8" s="3"/>
-    </row>
-    <row r="9" spans="1:44" x14ac:dyDescent="0.2">
-      <c r="A9" s="3"/>
-      <c r="B9" s="3"/>
-      <c r="D9" s="3"/>
-      <c r="E9" s="3"/>
-      <c r="G9" s="3"/>
-      <c r="H9" s="3"/>
-      <c r="J9" s="3"/>
-      <c r="K9" s="3"/>
-      <c r="M9" s="3"/>
-      <c r="N9" s="3"/>
-      <c r="P9" s="3"/>
-      <c r="Q9" s="3"/>
-      <c r="R9" s="1"/>
-      <c r="S9" s="3"/>
-      <c r="T9" s="3"/>
-      <c r="U9" s="1"/>
-      <c r="V9" s="3"/>
-      <c r="W9" s="3"/>
-      <c r="X9" s="1"/>
-      <c r="Y9" s="3"/>
-      <c r="Z9" s="3"/>
-      <c r="AA9" s="1"/>
-      <c r="AB9" s="3"/>
-      <c r="AC9" s="3"/>
-      <c r="AE9" s="3"/>
-      <c r="AF9" s="3"/>
-      <c r="AG9" s="1"/>
-      <c r="AH9" s="3"/>
-      <c r="AI9" s="3"/>
-      <c r="AJ9" s="1"/>
-      <c r="AK9" s="3"/>
-      <c r="AL9" s="3"/>
-      <c r="AM9" s="1"/>
-      <c r="AN9" s="3"/>
-      <c r="AO9" s="3"/>
-      <c r="AP9" s="1"/>
-      <c r="AQ9" s="3"/>
-      <c r="AR9" s="3"/>
     </row>
     <row r="10" spans="1:44" x14ac:dyDescent="0.2">
       <c r="A10" s="3"/>
@@ -17062,39 +17207,199 @@
       <c r="AQ27" s="3"/>
       <c r="AR27" s="3"/>
     </row>
+    <row r="28" spans="1:44" x14ac:dyDescent="0.2">
+      <c r="A28" s="3"/>
+      <c r="B28" s="3"/>
+      <c r="D28" s="3"/>
+      <c r="E28" s="3"/>
+      <c r="G28" s="3"/>
+      <c r="H28" s="3"/>
+      <c r="J28" s="3"/>
+      <c r="K28" s="3"/>
+      <c r="M28" s="3"/>
+      <c r="N28" s="3"/>
+      <c r="P28" s="3"/>
+      <c r="Q28" s="3"/>
+      <c r="R28" s="1"/>
+      <c r="S28" s="3"/>
+      <c r="T28" s="3"/>
+      <c r="U28" s="1"/>
+      <c r="V28" s="3"/>
+      <c r="W28" s="3"/>
+      <c r="X28" s="1"/>
+      <c r="Y28" s="3"/>
+      <c r="Z28" s="3"/>
+      <c r="AA28" s="1"/>
+      <c r="AB28" s="3"/>
+      <c r="AC28" s="3"/>
+      <c r="AE28" s="3"/>
+      <c r="AF28" s="3"/>
+      <c r="AG28" s="1"/>
+      <c r="AH28" s="3"/>
+      <c r="AI28" s="3"/>
+      <c r="AJ28" s="1"/>
+      <c r="AK28" s="3"/>
+      <c r="AL28" s="3"/>
+      <c r="AM28" s="1"/>
+      <c r="AN28" s="3"/>
+      <c r="AO28" s="3"/>
+      <c r="AP28" s="1"/>
+      <c r="AQ28" s="3"/>
+      <c r="AR28" s="3"/>
+    </row>
+    <row r="29" spans="1:44" x14ac:dyDescent="0.2">
+      <c r="A29" s="3"/>
+      <c r="B29" s="3"/>
+      <c r="D29" s="3"/>
+      <c r="E29" s="3"/>
+      <c r="G29" s="3"/>
+      <c r="H29" s="3"/>
+      <c r="J29" s="3"/>
+      <c r="K29" s="3"/>
+      <c r="M29" s="3"/>
+      <c r="N29" s="3"/>
+      <c r="P29" s="3"/>
+      <c r="Q29" s="3"/>
+      <c r="R29" s="1"/>
+      <c r="S29" s="3"/>
+      <c r="T29" s="3"/>
+      <c r="U29" s="1"/>
+      <c r="V29" s="3"/>
+      <c r="W29" s="3"/>
+      <c r="X29" s="1"/>
+      <c r="Y29" s="3"/>
+      <c r="Z29" s="3"/>
+      <c r="AA29" s="1"/>
+      <c r="AB29" s="3"/>
+      <c r="AC29" s="3"/>
+      <c r="AE29" s="3"/>
+      <c r="AF29" s="3"/>
+      <c r="AG29" s="1"/>
+      <c r="AH29" s="3"/>
+      <c r="AI29" s="3"/>
+      <c r="AJ29" s="1"/>
+      <c r="AK29" s="3"/>
+      <c r="AL29" s="3"/>
+      <c r="AM29" s="1"/>
+      <c r="AN29" s="3"/>
+      <c r="AO29" s="3"/>
+      <c r="AP29" s="1"/>
+      <c r="AQ29" s="3"/>
+      <c r="AR29" s="3"/>
+    </row>
   </sheetData>
   <mergeCells count="30">
     <mergeCell ref="D4:E4"/>
     <mergeCell ref="P4:Q4"/>
     <mergeCell ref="Y4:Z4"/>
-    <mergeCell ref="AB6:AC6"/>
-    <mergeCell ref="AN6:AO6"/>
+    <mergeCell ref="AB7:AC7"/>
+    <mergeCell ref="AN7:AO7"/>
     <mergeCell ref="AB4:AC4"/>
     <mergeCell ref="AN4:AO4"/>
-    <mergeCell ref="G6:H6"/>
+    <mergeCell ref="G7:H7"/>
     <mergeCell ref="J4:K4"/>
-    <mergeCell ref="V6:W6"/>
-    <mergeCell ref="M6:N6"/>
-    <mergeCell ref="AH6:AI6"/>
-    <mergeCell ref="S6:T6"/>
-    <mergeCell ref="Y6:Z6"/>
+    <mergeCell ref="V7:W7"/>
+    <mergeCell ref="M7:N7"/>
+    <mergeCell ref="AH7:AI7"/>
+    <mergeCell ref="S7:T7"/>
+    <mergeCell ref="Y7:Z7"/>
     <mergeCell ref="AQ4:AR4"/>
     <mergeCell ref="A4:B4"/>
     <mergeCell ref="G4:H4"/>
-    <mergeCell ref="AK6:AL6"/>
-    <mergeCell ref="AE6:AF6"/>
-    <mergeCell ref="AQ6:AR6"/>
+    <mergeCell ref="AK7:AL7"/>
+    <mergeCell ref="AE7:AF7"/>
+    <mergeCell ref="AQ7:AR7"/>
     <mergeCell ref="M4:N4"/>
     <mergeCell ref="S4:T4"/>
     <mergeCell ref="AE4:AF4"/>
-    <mergeCell ref="A6:B6"/>
+    <mergeCell ref="A7:B7"/>
     <mergeCell ref="AK4:AL4"/>
-    <mergeCell ref="D6:E6"/>
+    <mergeCell ref="D7:E7"/>
     <mergeCell ref="V4:W4"/>
     <mergeCell ref="AH4:AI4"/>
-    <mergeCell ref="J6:K6"/>
-    <mergeCell ref="P6:Q6"/>
+    <mergeCell ref="J7:K7"/>
+    <mergeCell ref="P7:Q7"/>
   </mergeCells>
+  <conditionalFormatting sqref="B6 A7:B7">
+    <cfRule type="expression" dxfId="0" priority="1">
+      <formula>AND($B$5&lt;&gt;"",$B$5&lt;&gt;"material")</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="E6 D7:E7">
+    <cfRule type="expression" dxfId="0" priority="2">
+      <formula>AND($E$5&lt;&gt;"",$E$5&lt;&gt;"material")</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="H6 G7:H7">
+    <cfRule type="expression" dxfId="0" priority="3">
+      <formula>AND($H$5&lt;&gt;"",$H$5&lt;&gt;"material")</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="K6 J7:K7">
+    <cfRule type="expression" dxfId="0" priority="4">
+      <formula>AND($K$5&lt;&gt;"",$K$5&lt;&gt;"material")</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="N6 M7:N7">
+    <cfRule type="expression" dxfId="0" priority="5">
+      <formula>AND($N$5&lt;&gt;"",$N$5&lt;&gt;"material")</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="Q6 P7:Q7">
+    <cfRule type="expression" dxfId="0" priority="6">
+      <formula>AND($Q$5&lt;&gt;"",$Q$5&lt;&gt;"material")</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="T6 S7:T7">
+    <cfRule type="expression" dxfId="0" priority="7">
+      <formula>AND($T$5&lt;&gt;"",$T$5&lt;&gt;"material")</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="W6 V7:W7">
+    <cfRule type="expression" dxfId="0" priority="8">
+      <formula>AND($W$5&lt;&gt;"",$W$5&lt;&gt;"material")</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="Z6 Y7:Z7">
+    <cfRule type="expression" dxfId="0" priority="9">
+      <formula>AND($Z$5&lt;&gt;"",$Z$5&lt;&gt;"material")</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="AC6 AB7:AC7">
+    <cfRule type="expression" dxfId="0" priority="10">
+      <formula>AND($AC$5&lt;&gt;"",$AC$5&lt;&gt;"material")</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="AF6 AE7:AF7">
+    <cfRule type="expression" dxfId="0" priority="11">
+      <formula>AND($AF$5&lt;&gt;"",$AF$5&lt;&gt;"material")</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="AI6 AH7:AI7">
+    <cfRule type="expression" dxfId="0" priority="12">
+      <formula>AND($AI$5&lt;&gt;"",$AI$5&lt;&gt;"material")</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="AL6 AK7:AL7">
+    <cfRule type="expression" dxfId="0" priority="13">
+      <formula>AND($AL$5&lt;&gt;"",$AL$5&lt;&gt;"material")</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="AO6 AN7:AO7">
+    <cfRule type="expression" dxfId="0" priority="14">
+      <formula>AND($AO$5&lt;&gt;"",$AO$5&lt;&gt;"material")</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="AR6 AQ7:AR7">
+    <cfRule type="expression" dxfId="0" priority="15">
+      <formula>AND($AR$5&lt;&gt;"",$AR$5&lt;&gt;"material")</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <dataValidations count="1">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="B5 E5 H5 K5 N5 Q5 T5 W5 Z5 AC5 AF5 AI5 AL5 AO5 AR5">
+      <formula1>"material,ssr reduce,ssr hold,ssr elastic,refine"</formula1>
+    </dataValidation>
+  </dataValidations>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
@@ -17710,7 +18015,7 @@
 
 <file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0800-000000000000}">
-  <dimension ref="B2:X22"/>
+  <dimension ref="B2:X23"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="3" customWidth="1"/>
@@ -17760,80 +18065,92 @@
       <c r="X2" s="62"/>
     </row>
     <row r="3" spans="2:24" x14ac:dyDescent="0.2">
-      <c r="B3" s="2" t="s">
+      <c r="B3" s="38" t="s">
+        <v>305</v>
+      </c>
+      <c r="C3" s="38"/>
+      <c r="D3" s="39"/>
+      <c r="F3" s="38" t="s">
+        <v>305</v>
+      </c>
+      <c r="G3" s="38"/>
+      <c r="H3" s="39"/>
+      <c r="J3" s="38" t="s">
+        <v>305</v>
+      </c>
+      <c r="K3" s="38"/>
+      <c r="L3" s="39"/>
+      <c r="N3" s="38" t="s">
+        <v>305</v>
+      </c>
+      <c r="O3" s="38"/>
+      <c r="P3" s="39"/>
+      <c r="R3" s="38" t="s">
+        <v>305</v>
+      </c>
+      <c r="S3" s="38"/>
+      <c r="T3" s="39"/>
+      <c r="V3" s="38" t="s">
+        <v>305</v>
+      </c>
+      <c r="W3" s="38"/>
+      <c r="X3" s="39"/>
+    </row>
+    <row r="4" spans="2:24" x14ac:dyDescent="0.2">
+      <c r="B4" s="2" t="s">
         <v>228</v>
       </c>
-      <c r="C3" s="2" t="s">
+      <c r="C4" s="2" t="s">
         <v>229</v>
       </c>
-      <c r="D3" s="2" t="s">
+      <c r="D4" s="2" t="s">
         <v>243</v>
       </c>
-      <c r="F3" s="2" t="s">
+      <c r="F4" s="2" t="s">
         <v>228</v>
       </c>
-      <c r="G3" s="2" t="s">
+      <c r="G4" s="2" t="s">
         <v>229</v>
       </c>
-      <c r="H3" s="2" t="s">
+      <c r="H4" s="2" t="s">
         <v>243</v>
       </c>
-      <c r="J3" s="2" t="s">
+      <c r="J4" s="2" t="s">
         <v>228</v>
       </c>
-      <c r="K3" s="2" t="s">
+      <c r="K4" s="2" t="s">
         <v>229</v>
       </c>
-      <c r="L3" s="2" t="s">
+      <c r="L4" s="2" t="s">
         <v>243</v>
       </c>
-      <c r="N3" s="2" t="s">
+      <c r="N4" s="2" t="s">
         <v>228</v>
       </c>
-      <c r="O3" s="2" t="s">
+      <c r="O4" s="2" t="s">
         <v>229</v>
       </c>
-      <c r="P3" s="2" t="s">
+      <c r="P4" s="2" t="s">
         <v>243</v>
       </c>
-      <c r="R3" s="2" t="s">
+      <c r="R4" s="2" t="s">
         <v>228</v>
       </c>
-      <c r="S3" s="2" t="s">
+      <c r="S4" s="2" t="s">
         <v>229</v>
       </c>
-      <c r="T3" s="2" t="s">
+      <c r="T4" s="2" t="s">
         <v>243</v>
       </c>
-      <c r="V3" s="2" t="s">
+      <c r="V4" s="2" t="s">
         <v>228</v>
       </c>
-      <c r="W3" s="2" t="s">
+      <c r="W4" s="2" t="s">
         <v>229</v>
       </c>
-      <c r="X3" s="2" t="s">
+      <c r="X4" s="2" t="s">
         <v>243</v>
       </c>
-    </row>
-    <row r="4" spans="2:24" x14ac:dyDescent="0.2">
-      <c r="B4" s="3"/>
-      <c r="C4" s="3"/>
-      <c r="D4" s="3"/>
-      <c r="F4" s="3"/>
-      <c r="G4" s="3"/>
-      <c r="H4" s="3"/>
-      <c r="J4" s="3"/>
-      <c r="K4" s="3"/>
-      <c r="L4" s="3"/>
-      <c r="N4" s="3"/>
-      <c r="O4" s="3"/>
-      <c r="P4" s="3"/>
-      <c r="R4" s="3"/>
-      <c r="S4" s="3"/>
-      <c r="T4" s="3"/>
-      <c r="V4" s="3"/>
-      <c r="W4" s="3"/>
-      <c r="X4" s="3"/>
     </row>
     <row r="5" spans="2:24" x14ac:dyDescent="0.2">
       <c r="B5" s="3"/>
@@ -18195,15 +18512,46 @@
       <c r="W22" s="3"/>
       <c r="X22" s="3"/>
     </row>
+    <row r="23" spans="2:24" x14ac:dyDescent="0.2">
+      <c r="B23" s="3"/>
+      <c r="C23" s="3"/>
+      <c r="D23" s="3"/>
+      <c r="F23" s="3"/>
+      <c r="G23" s="3"/>
+      <c r="H23" s="3"/>
+      <c r="J23" s="3"/>
+      <c r="K23" s="3"/>
+      <c r="L23" s="3"/>
+      <c r="N23" s="3"/>
+      <c r="O23" s="3"/>
+      <c r="P23" s="3"/>
+      <c r="R23" s="3"/>
+      <c r="S23" s="3"/>
+      <c r="T23" s="3"/>
+      <c r="V23" s="3"/>
+      <c r="W23" s="3"/>
+      <c r="X23" s="3"/>
+    </row>
   </sheetData>
-  <mergeCells count="6">
+  <mergeCells count="12">
     <mergeCell ref="B2:D2"/>
     <mergeCell ref="V2:X2"/>
     <mergeCell ref="J2:L2"/>
     <mergeCell ref="N2:P2"/>
     <mergeCell ref="R2:T2"/>
     <mergeCell ref="F2:H2"/>
+    <mergeCell ref="B3:C3"/>
+    <mergeCell ref="F3:G3"/>
+    <mergeCell ref="J3:K3"/>
+    <mergeCell ref="N3:O3"/>
+    <mergeCell ref="R3:S3"/>
+    <mergeCell ref="V3:W3"/>
   </mergeCells>
+  <dataValidations count="1">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="D3 H3 L3 P3 T3 X3">
+      <formula1>"normal,vertical"</formula1>
+    </dataValidation>
+  </dataValidations>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
feat(template): v21 review revisions — blank name echo for overlays, profile Size row, main Side BC
Owner's phase-one review: the polygon name echo now shows nothing (still
dimmed) when Type is not a material zone, since the Type dropdown directly
above already names the overlay; profile-line blocks gain the same optional
Size row as polygons, since profile lines build material zones and carry the
same local-mesh-size option; and the main sheet gains a global Side BC setting
(rollers | fixed, shipping rollers = today's behavior), inert until fem.py's
side-BC assignment reads it.

Built on the owner's Excel-saved master, so his round-trip through Excel is
preserved; calcChain dropped and fullCalcOnLoad restored after it.

Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_0147GB4LGVZuqGHCRMVzZTsR
</commit_message>
<xml_diff>
--- a/docs/inputs/input_template.xlsx
+++ b/docs/inputs/input_template.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/njones/python_projects/xslope/docs/inputs/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CA8D9778-BA48-644C-980F-473DF9F954B0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D0BA7854-5540-8340-8930-9B54C7224615}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="620" windowWidth="34200" windowHeight="19900" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -60,7 +60,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="575" uniqueCount="308">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="593" uniqueCount="310">
   <si>
     <t>time</t>
   </si>
@@ -971,9 +971,6 @@
     <t>corps</t>
   </si>
   <si>
-    <t>Mat ID = -1 --&gt; SSR reduce, Mat ID = -2 --&gt; SSR hold, Mat ID = -3 --&gt; SSR elastic</t>
-  </si>
-  <si>
     <t>Size:</t>
   </si>
   <si>
@@ -984,6 +981,15 @@
   </si>
   <si>
     <t>Type: material zone (default), an SSR analysis overlay, or a mesh refinement region.   Size: optional target mesh element size inside the polygon (blank = global size).</t>
+  </si>
+  <si>
+    <t>Side BC:</t>
+  </si>
+  <si>
+    <t>rollers</t>
+  </si>
+  <si>
+    <t>Size: optional target mesh element size inside this line's material zone (blank = global size).</t>
   </si>
 </sst>
 </file>
@@ -1491,18 +1497,11 @@
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="20">
+  <dxfs count="35">
     <dxf>
       <fill>
         <patternFill>
-          <bgColor theme="0" tint="-0.499984740745262"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor theme="0" tint="-0.499984740745262"/>
+          <bgColor theme="1" tint="0.499984740745262"/>
         </patternFill>
       </fill>
     </dxf>
@@ -1523,7 +1522,119 @@
     <dxf>
       <fill>
         <patternFill>
-          <bgColor theme="1" tint="0.499984740745262"/>
+          <bgColor theme="0" tint="-0.499984740745262"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="0" tint="-0.499984740745262"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="0" tint="-0.499984740745262"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="0" tint="-0.499984740745262"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="0" tint="-0.499984740745262"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="0" tint="-0.499984740745262"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="0" tint="-0.499984740745262"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="0" tint="-0.499984740745262"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="0" tint="-0.499984740745262"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="0" tint="-0.499984740745262"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="0" tint="-0.499984740745262"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="0" tint="-0.499984740745262"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="0" tint="-0.499984740745262"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="0" tint="-0.499984740745262"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="0" tint="-0.499984740745262"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="0" tint="-0.499984740745262"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="0" tint="-0.499984740745262"/>
         </patternFill>
       </fill>
     </dxf>
@@ -1698,7 +1809,7 @@
           </c:marker>
           <c:xVal>
             <c:numRef>
-              <c:f>profile!$A$8:$A$27</c:f>
+              <c:f>profile!$A$9:$A$28</c:f>
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="20"/>
@@ -1707,7 +1818,7 @@
           </c:xVal>
           <c:yVal>
             <c:numRef>
-              <c:f>profile!$B$8:$B$27</c:f>
+              <c:f>profile!$B$9:$B$28</c:f>
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="20"/>
@@ -1761,7 +1872,7 @@
           </c:marker>
           <c:xVal>
             <c:numRef>
-              <c:f>profile!$D$8:$D$27</c:f>
+              <c:f>profile!$D$9:$D$28</c:f>
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="20"/>
@@ -1770,7 +1881,7 @@
           </c:xVal>
           <c:yVal>
             <c:numRef>
-              <c:f>profile!$E$8:$E$27</c:f>
+              <c:f>profile!$E$9:$E$28</c:f>
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="20"/>
@@ -1824,7 +1935,7 @@
           </c:marker>
           <c:xVal>
             <c:numRef>
-              <c:f>profile!$G$8:$G$27</c:f>
+              <c:f>profile!$G$9:$G$28</c:f>
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="20"/>
@@ -1833,7 +1944,7 @@
           </c:xVal>
           <c:yVal>
             <c:numRef>
-              <c:f>profile!$H$8:$H$27</c:f>
+              <c:f>profile!$H$9:$H$28</c:f>
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="20"/>
@@ -1887,7 +1998,7 @@
           </c:marker>
           <c:xVal>
             <c:numRef>
-              <c:f>profile!$J$8:$J$27</c:f>
+              <c:f>profile!$J$9:$J$28</c:f>
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="20"/>
@@ -1896,7 +2007,7 @@
           </c:xVal>
           <c:yVal>
             <c:numRef>
-              <c:f>profile!$K$8:$K$27</c:f>
+              <c:f>profile!$K$9:$K$28</c:f>
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="20"/>
@@ -1950,7 +2061,7 @@
           </c:marker>
           <c:xVal>
             <c:numRef>
-              <c:f>profile!$M$8:$M$27</c:f>
+              <c:f>profile!$M$9:$M$28</c:f>
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="20"/>
@@ -1959,7 +2070,7 @@
           </c:xVal>
           <c:yVal>
             <c:numRef>
-              <c:f>profile!$N$8:$N$27</c:f>
+              <c:f>profile!$N$9:$N$28</c:f>
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="20"/>
@@ -2013,7 +2124,7 @@
           </c:marker>
           <c:xVal>
             <c:numRef>
-              <c:f>profile!$P$8:$P$27</c:f>
+              <c:f>profile!$P$9:$P$28</c:f>
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="20"/>
@@ -2022,7 +2133,7 @@
           </c:xVal>
           <c:yVal>
             <c:numRef>
-              <c:f>profile!$Q$8:$Q$27</c:f>
+              <c:f>profile!$Q$9:$Q$28</c:f>
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="20"/>
@@ -2082,7 +2193,7 @@
           </c:marker>
           <c:xVal>
             <c:numRef>
-              <c:f>profile!$S$8:$S$27</c:f>
+              <c:f>profile!$S$9:$S$28</c:f>
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="20"/>
@@ -2091,7 +2202,7 @@
           </c:xVal>
           <c:yVal>
             <c:numRef>
-              <c:f>profile!$T$8:$T$27</c:f>
+              <c:f>profile!$T$9:$T$28</c:f>
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="20"/>
@@ -2151,7 +2262,7 @@
           </c:marker>
           <c:xVal>
             <c:numRef>
-              <c:f>profile!$V$8:$V$27</c:f>
+              <c:f>profile!$V$9:$V$28</c:f>
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="20"/>
@@ -2160,7 +2271,7 @@
           </c:xVal>
           <c:yVal>
             <c:numRef>
-              <c:f>profile!$W$8:$W$27</c:f>
+              <c:f>profile!$W$9:$W$28</c:f>
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="20"/>
@@ -2220,7 +2331,7 @@
           </c:marker>
           <c:xVal>
             <c:numRef>
-              <c:f>profile!$Y$8:$Y$27</c:f>
+              <c:f>profile!$Y$9:$Y$28</c:f>
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="20"/>
@@ -2229,7 +2340,7 @@
           </c:xVal>
           <c:yVal>
             <c:numRef>
-              <c:f>profile!$Z$8:$Z$27</c:f>
+              <c:f>profile!$Z$9:$Z$28</c:f>
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="20"/>
@@ -2289,7 +2400,7 @@
           </c:marker>
           <c:xVal>
             <c:numRef>
-              <c:f>profile!$AB$8:$AB$27</c:f>
+              <c:f>profile!$AB$9:$AB$28</c:f>
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="20"/>
@@ -2298,7 +2409,7 @@
           </c:xVal>
           <c:yVal>
             <c:numRef>
-              <c:f>profile!$AC$8:$AC$27</c:f>
+              <c:f>profile!$AC$9:$AC$28</c:f>
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="20"/>
@@ -2358,7 +2469,7 @@
           </c:marker>
           <c:xVal>
             <c:numRef>
-              <c:f>profile!$AE$8:$AE$27</c:f>
+              <c:f>profile!$AE$9:$AE$28</c:f>
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="20"/>
@@ -2367,7 +2478,7 @@
           </c:xVal>
           <c:yVal>
             <c:numRef>
-              <c:f>profile!$AF$8:$AF$27</c:f>
+              <c:f>profile!$AF$9:$AF$28</c:f>
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="20"/>
@@ -2427,7 +2538,7 @@
           </c:marker>
           <c:xVal>
             <c:numRef>
-              <c:f>profile!$AH$8:$AH$27</c:f>
+              <c:f>profile!$AH$9:$AH$28</c:f>
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="20"/>
@@ -2436,7 +2547,7 @@
           </c:xVal>
           <c:yVal>
             <c:numRef>
-              <c:f>profile!$AI$8:$AI$27</c:f>
+              <c:f>profile!$AI$9:$AI$28</c:f>
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="20"/>
@@ -2496,7 +2607,7 @@
           </c:marker>
           <c:xVal>
             <c:numRef>
-              <c:f>profile!$AK$8:$AK$27</c:f>
+              <c:f>profile!$AK$9:$AK$28</c:f>
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="20"/>
@@ -2505,7 +2616,7 @@
           </c:xVal>
           <c:yVal>
             <c:numRef>
-              <c:f>profile!$AL$8:$AL$27</c:f>
+              <c:f>profile!$AL$9:$AL$28</c:f>
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="20"/>
@@ -2568,7 +2679,7 @@
           </c:marker>
           <c:xVal>
             <c:numRef>
-              <c:f>profile!$AN$8:$AN$27</c:f>
+              <c:f>profile!$AN$9:$AN$28</c:f>
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="20"/>
@@ -2577,7 +2688,7 @@
           </c:xVal>
           <c:yVal>
             <c:numRef>
-              <c:f>profile!$AO$8:$AO$27</c:f>
+              <c:f>profile!$AO$9:$AO$28</c:f>
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="20"/>
@@ -2640,7 +2751,7 @@
           </c:marker>
           <c:xVal>
             <c:numRef>
-              <c:f>profile!$AQ$8:$AQ$27</c:f>
+              <c:f>profile!$AQ$9:$AQ$28</c:f>
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="20"/>
@@ -2649,7 +2760,7 @@
           </c:xVal>
           <c:yVal>
             <c:numRef>
-              <c:f>profile!$AR$8:$AR$27</c:f>
+              <c:f>profile!$AR$9:$AR$28</c:f>
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="20"/>
@@ -9171,6 +9282,12 @@
       </c>
     </row>
     <row r="22" spans="2:7" x14ac:dyDescent="0.2">
+      <c r="C22" s="14" t="s">
+        <v>307</v>
+      </c>
+      <c r="D22" s="1" t="s">
+        <v>308</v>
+      </c>
       <c r="F22" s="1" t="s">
         <v>62</v>
       </c>
@@ -9318,7 +9435,10 @@
   <mergeCells count="1">
     <mergeCell ref="B7:D7"/>
   </mergeCells>
-  <dataValidations count="5">
+  <dataValidations count="6">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="D22">
+      <formula1>"rollers,fixed"</formula1>
+    </dataValidation>
     <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="D8" xr:uid="{00000000-0002-0000-0000-000000000000}">
       <formula1>$D$50:$D$51</formula1>
     </dataValidation>
@@ -9391,35 +9511,35 @@
       <c r="X2" s="62"/>
     </row>
     <row r="3" spans="2:24" x14ac:dyDescent="0.2">
-      <c r="B3" s="38" t="s">
-        <v>305</v>
-      </c>
-      <c r="C3" s="38"/>
+      <c r="B3" s="58" t="s">
+        <v>304</v>
+      </c>
+      <c r="C3" s="58"/>
       <c r="D3" s="39"/>
-      <c r="F3" s="38" t="s">
-        <v>305</v>
-      </c>
-      <c r="G3" s="38"/>
+      <c r="F3" s="58" t="s">
+        <v>304</v>
+      </c>
+      <c r="G3" s="58"/>
       <c r="H3" s="39"/>
-      <c r="J3" s="38" t="s">
-        <v>305</v>
-      </c>
-      <c r="K3" s="38"/>
+      <c r="J3" s="58" t="s">
+        <v>304</v>
+      </c>
+      <c r="K3" s="58"/>
       <c r="L3" s="39"/>
-      <c r="N3" s="38" t="s">
-        <v>305</v>
-      </c>
-      <c r="O3" s="38"/>
+      <c r="N3" s="58" t="s">
+        <v>304</v>
+      </c>
+      <c r="O3" s="58"/>
       <c r="P3" s="39"/>
-      <c r="R3" s="38" t="s">
-        <v>305</v>
-      </c>
-      <c r="S3" s="38"/>
+      <c r="R3" s="58" t="s">
+        <v>304</v>
+      </c>
+      <c r="S3" s="58"/>
       <c r="T3" s="39"/>
-      <c r="V3" s="38" t="s">
-        <v>305</v>
-      </c>
-      <c r="W3" s="38"/>
+      <c r="V3" s="58" t="s">
+        <v>304</v>
+      </c>
+      <c r="W3" s="58"/>
       <c r="X3" s="39"/>
     </row>
     <row r="4" spans="2:24" x14ac:dyDescent="0.2">
@@ -9860,21 +9980,21 @@
     </row>
   </sheetData>
   <mergeCells count="12">
+    <mergeCell ref="V3:W3"/>
+    <mergeCell ref="B3:C3"/>
+    <mergeCell ref="F3:G3"/>
+    <mergeCell ref="J3:K3"/>
+    <mergeCell ref="N3:O3"/>
+    <mergeCell ref="R3:S3"/>
     <mergeCell ref="B2:D2"/>
     <mergeCell ref="V2:X2"/>
     <mergeCell ref="J2:L2"/>
     <mergeCell ref="N2:P2"/>
     <mergeCell ref="R2:T2"/>
     <mergeCell ref="F2:H2"/>
-    <mergeCell ref="B3:C3"/>
-    <mergeCell ref="F3:G3"/>
-    <mergeCell ref="J3:K3"/>
-    <mergeCell ref="N3:O3"/>
-    <mergeCell ref="R3:S3"/>
-    <mergeCell ref="V3:W3"/>
   </mergeCells>
   <dataValidations count="1">
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="D3 H3 L3 P3 T3 X3">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="D3 H3 L3 P3 T3 X3" xr:uid="{00000000-0002-0000-0900-000000000000}">
       <formula1>"normal,vertical"</formula1>
     </dataValidation>
   </dataValidations>
@@ -14604,84 +14724,84 @@
     <mergeCell ref="AG9:AP9"/>
   </mergeCells>
   <conditionalFormatting sqref="F11:K52 AB11:AF52">
-    <cfRule type="expression" dxfId="19" priority="6">
+    <cfRule type="expression" dxfId="34" priority="6">
       <formula>$E11="hb"</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="18" priority="7">
+    <cfRule type="expression" dxfId="33" priority="7">
       <formula>$E11="pow"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="F11:L52 O11:R52">
-    <cfRule type="expression" dxfId="17" priority="19">
+    <cfRule type="expression" dxfId="32" priority="19">
       <formula>$E11="elastic"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="G11:G52">
-    <cfRule type="expression" dxfId="16" priority="8">
+    <cfRule type="expression" dxfId="31" priority="8">
       <formula>$E11="cp"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="H11:I52">
-    <cfRule type="expression" dxfId="15" priority="9">
+    <cfRule type="expression" dxfId="30" priority="9">
       <formula>$E11="mc"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="J11:K52">
-    <cfRule type="expression" dxfId="14" priority="10">
+    <cfRule type="expression" dxfId="29" priority="10">
       <formula>$E11="cp"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="P11:P52">
-    <cfRule type="expression" dxfId="13" priority="13">
+    <cfRule type="expression" dxfId="28" priority="13">
       <formula>AND($O11&lt;&gt;"",$O11&lt;&gt;"ru")</formula>
     </cfRule>
   </conditionalFormatting>
+  <conditionalFormatting sqref="Q11:R52">
+    <cfRule type="expression" dxfId="27" priority="23">
+      <formula>$E11="cp"</formula>
+    </cfRule>
+    <cfRule type="expression" dxfId="26" priority="24">
+      <formula>AND($O11&lt;&gt;"",$O11&lt;&gt;"piezo",$O11&lt;&gt;"seep")</formula>
+    </cfRule>
+  </conditionalFormatting>
   <conditionalFormatting sqref="S11:V52">
-    <cfRule type="expression" dxfId="12" priority="11">
+    <cfRule type="expression" dxfId="25" priority="11">
       <formula>AND($E11&lt;&gt;"",$E11&lt;&gt;"pow")</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="W11:Z52">
-    <cfRule type="expression" dxfId="11" priority="12">
+    <cfRule type="expression" dxfId="24" priority="12">
       <formula>AND($E11&lt;&gt;"",$E11&lt;&gt;"hb")</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="AB11:AF52">
-    <cfRule type="expression" dxfId="10" priority="21">
+    <cfRule type="expression" dxfId="23" priority="21">
       <formula>$E11="elastic"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="AC11:AC52">
-    <cfRule type="expression" dxfId="9" priority="14">
+    <cfRule type="expression" dxfId="22" priority="14">
       <formula>$E11="cp"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="AD11:AD52">
-    <cfRule type="expression" dxfId="8" priority="15">
+    <cfRule type="expression" dxfId="21" priority="15">
       <formula>$E11="mc"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="AE11:AF52">
-    <cfRule type="expression" dxfId="7" priority="16">
+    <cfRule type="expression" dxfId="20" priority="16">
       <formula>$E11="cp"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="AK11:AL52">
-    <cfRule type="expression" dxfId="6" priority="17">
+    <cfRule type="expression" dxfId="19" priority="17">
       <formula>OR($AJ11="vg",$AJ11="gard")</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="AM11:AN52">
-    <cfRule type="expression" dxfId="5" priority="1">
+    <cfRule type="expression" dxfId="18" priority="1">
       <formula>$AJ11="lf"</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="Q11:R52">
-    <cfRule type="expression" dxfId="1" priority="23">
-      <formula>$E11="cp"</formula>
-    </cfRule>
-    <cfRule type="expression" dxfId="0" priority="24">
-      <formula>AND($O11&lt;&gt;"",$O11&lt;&gt;"piezo",$O11&lt;&gt;"seep")</formula>
     </cfRule>
   </conditionalFormatting>
   <dataValidations count="3">
@@ -14701,7 +14821,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0300-000000000000}">
-  <dimension ref="A2:AR27"/>
+  <dimension ref="A2:AR28"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="2" width="10.83203125" style="1" customWidth="1"/>
@@ -14736,6 +14856,11 @@
         <v>160</v>
       </c>
     </row>
+    <row r="3" spans="1:44" x14ac:dyDescent="0.2">
+      <c r="D3" s="24" t="s">
+        <v>309</v>
+      </c>
+    </row>
     <row r="4" spans="1:44" x14ac:dyDescent="0.2">
       <c r="A4" s="55" t="s">
         <v>161</v>
@@ -14992,144 +15117,174 @@
       <c r="AR6" s="57"/>
     </row>
     <row r="7" spans="1:44" x14ac:dyDescent="0.2">
-      <c r="A7" s="2" t="s">
+      <c r="A7" s="36" t="s">
+        <v>303</v>
+      </c>
+      <c r="B7" s="37"/>
+      <c r="D7" s="36" t="s">
+        <v>303</v>
+      </c>
+      <c r="E7" s="37"/>
+      <c r="G7" s="36" t="s">
+        <v>303</v>
+      </c>
+      <c r="H7" s="37"/>
+      <c r="J7" s="36" t="s">
+        <v>303</v>
+      </c>
+      <c r="K7" s="37"/>
+      <c r="M7" s="36" t="s">
+        <v>303</v>
+      </c>
+      <c r="N7" s="37"/>
+      <c r="P7" s="36" t="s">
+        <v>303</v>
+      </c>
+      <c r="Q7" s="37"/>
+      <c r="R7" s="1"/>
+      <c r="S7" s="36" t="s">
+        <v>303</v>
+      </c>
+      <c r="T7" s="37"/>
+      <c r="U7" s="1"/>
+      <c r="V7" s="36" t="s">
+        <v>303</v>
+      </c>
+      <c r="W7" s="37"/>
+      <c r="X7" s="1"/>
+      <c r="Y7" s="36" t="s">
+        <v>303</v>
+      </c>
+      <c r="Z7" s="37"/>
+      <c r="AA7" s="1"/>
+      <c r="AB7" s="36" t="s">
+        <v>303</v>
+      </c>
+      <c r="AC7" s="37"/>
+      <c r="AE7" s="36" t="s">
+        <v>303</v>
+      </c>
+      <c r="AF7" s="37"/>
+      <c r="AG7" s="1"/>
+      <c r="AH7" s="36" t="s">
+        <v>303</v>
+      </c>
+      <c r="AI7" s="37"/>
+      <c r="AJ7" s="1"/>
+      <c r="AK7" s="36" t="s">
+        <v>303</v>
+      </c>
+      <c r="AL7" s="37"/>
+      <c r="AM7" s="1"/>
+      <c r="AN7" s="36" t="s">
+        <v>303</v>
+      </c>
+      <c r="AO7" s="37"/>
+      <c r="AP7" s="1"/>
+      <c r="AQ7" s="36" t="s">
+        <v>303</v>
+      </c>
+      <c r="AR7" s="37"/>
+    </row>
+    <row r="8" spans="1:44" x14ac:dyDescent="0.2">
+      <c r="A8" s="2" t="s">
         <v>177</v>
       </c>
-      <c r="B7" s="2" t="s">
+      <c r="B8" s="2" t="s">
         <v>178</v>
       </c>
-      <c r="D7" s="2" t="s">
+      <c r="D8" s="2" t="s">
         <v>177</v>
       </c>
-      <c r="E7" s="2" t="s">
+      <c r="E8" s="2" t="s">
         <v>178</v>
       </c>
-      <c r="G7" s="2" t="s">
+      <c r="G8" s="2" t="s">
         <v>177</v>
       </c>
-      <c r="H7" s="2" t="s">
+      <c r="H8" s="2" t="s">
         <v>178</v>
       </c>
-      <c r="J7" s="2" t="s">
+      <c r="J8" s="2" t="s">
         <v>177</v>
       </c>
-      <c r="K7" s="2" t="s">
+      <c r="K8" s="2" t="s">
         <v>178</v>
       </c>
-      <c r="M7" s="2" t="s">
+      <c r="M8" s="2" t="s">
         <v>177</v>
       </c>
-      <c r="N7" s="2" t="s">
+      <c r="N8" s="2" t="s">
         <v>178</v>
       </c>
-      <c r="P7" s="2" t="s">
+      <c r="P8" s="2" t="s">
         <v>177</v>
       </c>
-      <c r="Q7" s="2" t="s">
+      <c r="Q8" s="2" t="s">
         <v>178</v>
       </c>
-      <c r="R7" s="1"/>
-      <c r="S7" s="2" t="s">
+      <c r="R8" s="1"/>
+      <c r="S8" s="2" t="s">
         <v>177</v>
       </c>
-      <c r="T7" s="2" t="s">
+      <c r="T8" s="2" t="s">
         <v>178</v>
       </c>
-      <c r="U7" s="1"/>
-      <c r="V7" s="2" t="s">
+      <c r="U8" s="1"/>
+      <c r="V8" s="2" t="s">
         <v>177</v>
       </c>
-      <c r="W7" s="2" t="s">
+      <c r="W8" s="2" t="s">
         <v>178</v>
       </c>
-      <c r="X7" s="1"/>
-      <c r="Y7" s="2" t="s">
+      <c r="X8" s="1"/>
+      <c r="Y8" s="2" t="s">
         <v>177</v>
       </c>
-      <c r="Z7" s="2" t="s">
+      <c r="Z8" s="2" t="s">
         <v>178</v>
       </c>
-      <c r="AA7" s="1"/>
-      <c r="AB7" s="2" t="s">
+      <c r="AA8" s="1"/>
+      <c r="AB8" s="2" t="s">
         <v>177</v>
       </c>
-      <c r="AC7" s="2" t="s">
+      <c r="AC8" s="2" t="s">
         <v>178</v>
       </c>
-      <c r="AE7" s="2" t="s">
+      <c r="AE8" s="2" t="s">
         <v>177</v>
       </c>
-      <c r="AF7" s="2" t="s">
+      <c r="AF8" s="2" t="s">
         <v>178</v>
       </c>
-      <c r="AG7" s="1"/>
-      <c r="AH7" s="2" t="s">
+      <c r="AG8" s="1"/>
+      <c r="AH8" s="2" t="s">
         <v>177</v>
       </c>
-      <c r="AI7" s="2" t="s">
+      <c r="AI8" s="2" t="s">
         <v>178</v>
       </c>
-      <c r="AJ7" s="1"/>
-      <c r="AK7" s="2" t="s">
+      <c r="AJ8" s="1"/>
+      <c r="AK8" s="2" t="s">
         <v>177</v>
       </c>
-      <c r="AL7" s="2" t="s">
+      <c r="AL8" s="2" t="s">
         <v>178</v>
       </c>
-      <c r="AM7" s="1"/>
-      <c r="AN7" s="2" t="s">
+      <c r="AM8" s="1"/>
+      <c r="AN8" s="2" t="s">
         <v>177</v>
       </c>
-      <c r="AO7" s="2" t="s">
+      <c r="AO8" s="2" t="s">
         <v>178</v>
       </c>
-      <c r="AP7" s="1"/>
-      <c r="AQ7" s="2" t="s">
+      <c r="AP8" s="1"/>
+      <c r="AQ8" s="2" t="s">
         <v>177</v>
       </c>
-      <c r="AR7" s="2" t="s">
+      <c r="AR8" s="2" t="s">
         <v>178</v>
       </c>
-    </row>
-    <row r="8" spans="1:44" x14ac:dyDescent="0.2">
-      <c r="A8" s="3"/>
-      <c r="B8" s="3"/>
-      <c r="D8" s="3"/>
-      <c r="E8" s="3"/>
-      <c r="G8" s="3"/>
-      <c r="H8" s="3"/>
-      <c r="J8" s="3"/>
-      <c r="K8" s="3"/>
-      <c r="M8" s="3"/>
-      <c r="N8" s="3"/>
-      <c r="P8" s="3"/>
-      <c r="Q8" s="3"/>
-      <c r="R8" s="1"/>
-      <c r="S8" s="16"/>
-      <c r="T8" s="17"/>
-      <c r="U8" s="1"/>
-      <c r="V8" s="16"/>
-      <c r="W8" s="17"/>
-      <c r="X8" s="1"/>
-      <c r="Y8" s="16"/>
-      <c r="Z8" s="17"/>
-      <c r="AA8" s="1"/>
-      <c r="AB8" s="16"/>
-      <c r="AC8" s="17"/>
-      <c r="AE8" s="3"/>
-      <c r="AF8" s="3"/>
-      <c r="AG8" s="1"/>
-      <c r="AH8" s="16"/>
-      <c r="AI8" s="17"/>
-      <c r="AJ8" s="1"/>
-      <c r="AK8" s="16"/>
-      <c r="AL8" s="17"/>
-      <c r="AM8" s="1"/>
-      <c r="AN8" s="16"/>
-      <c r="AO8" s="17"/>
-      <c r="AP8" s="1"/>
-      <c r="AQ8" s="16"/>
-      <c r="AR8" s="17"/>
     </row>
     <row r="9" spans="1:44" x14ac:dyDescent="0.2">
       <c r="A9" s="3"/>
@@ -15145,31 +15300,31 @@
       <c r="P9" s="3"/>
       <c r="Q9" s="3"/>
       <c r="R9" s="1"/>
-      <c r="S9" s="18"/>
-      <c r="T9" s="19"/>
+      <c r="S9" s="16"/>
+      <c r="T9" s="17"/>
       <c r="U9" s="1"/>
-      <c r="V9" s="18"/>
-      <c r="W9" s="19"/>
+      <c r="V9" s="16"/>
+      <c r="W9" s="17"/>
       <c r="X9" s="1"/>
-      <c r="Y9" s="18"/>
-      <c r="Z9" s="19"/>
+      <c r="Y9" s="16"/>
+      <c r="Z9" s="17"/>
       <c r="AA9" s="1"/>
-      <c r="AB9" s="18"/>
-      <c r="AC9" s="19"/>
+      <c r="AB9" s="16"/>
+      <c r="AC9" s="17"/>
       <c r="AE9" s="3"/>
       <c r="AF9" s="3"/>
       <c r="AG9" s="1"/>
-      <c r="AH9" s="18"/>
-      <c r="AI9" s="19"/>
+      <c r="AH9" s="16"/>
+      <c r="AI9" s="17"/>
       <c r="AJ9" s="1"/>
-      <c r="AK9" s="18"/>
-      <c r="AL9" s="19"/>
+      <c r="AK9" s="16"/>
+      <c r="AL9" s="17"/>
       <c r="AM9" s="1"/>
-      <c r="AN9" s="18"/>
-      <c r="AO9" s="19"/>
+      <c r="AN9" s="16"/>
+      <c r="AO9" s="17"/>
       <c r="AP9" s="1"/>
-      <c r="AQ9" s="18"/>
-      <c r="AR9" s="19"/>
+      <c r="AQ9" s="16"/>
+      <c r="AR9" s="17"/>
     </row>
     <row r="10" spans="1:44" x14ac:dyDescent="0.2">
       <c r="A10" s="3"/>
@@ -15228,8 +15383,8 @@
       <c r="S11" s="18"/>
       <c r="T11" s="19"/>
       <c r="U11" s="1"/>
-      <c r="V11" s="16"/>
-      <c r="W11" s="17"/>
+      <c r="V11" s="18"/>
+      <c r="W11" s="19"/>
       <c r="X11" s="1"/>
       <c r="Y11" s="18"/>
       <c r="Z11" s="19"/>
@@ -15250,6 +15405,1362 @@
       <c r="AP11" s="1"/>
       <c r="AQ11" s="18"/>
       <c r="AR11" s="19"/>
+    </row>
+    <row r="12" spans="1:44" x14ac:dyDescent="0.2">
+      <c r="A12" s="3"/>
+      <c r="B12" s="3"/>
+      <c r="D12" s="3"/>
+      <c r="E12" s="3"/>
+      <c r="G12" s="3"/>
+      <c r="H12" s="3"/>
+      <c r="J12" s="3"/>
+      <c r="K12" s="3"/>
+      <c r="M12" s="3"/>
+      <c r="N12" s="3"/>
+      <c r="P12" s="3"/>
+      <c r="Q12" s="3"/>
+      <c r="R12" s="1"/>
+      <c r="S12" s="18"/>
+      <c r="T12" s="19"/>
+      <c r="U12" s="1"/>
+      <c r="V12" s="16"/>
+      <c r="W12" s="17"/>
+      <c r="X12" s="1"/>
+      <c r="Y12" s="18"/>
+      <c r="Z12" s="19"/>
+      <c r="AA12" s="1"/>
+      <c r="AB12" s="18"/>
+      <c r="AC12" s="19"/>
+      <c r="AE12" s="3"/>
+      <c r="AF12" s="3"/>
+      <c r="AG12" s="1"/>
+      <c r="AH12" s="18"/>
+      <c r="AI12" s="19"/>
+      <c r="AJ12" s="1"/>
+      <c r="AK12" s="18"/>
+      <c r="AL12" s="19"/>
+      <c r="AM12" s="1"/>
+      <c r="AN12" s="18"/>
+      <c r="AO12" s="19"/>
+      <c r="AP12" s="1"/>
+      <c r="AQ12" s="18"/>
+      <c r="AR12" s="19"/>
+    </row>
+    <row r="13" spans="1:44" x14ac:dyDescent="0.2">
+      <c r="A13" s="3"/>
+      <c r="B13" s="3"/>
+      <c r="D13" s="3"/>
+      <c r="E13" s="3"/>
+      <c r="G13" s="3"/>
+      <c r="H13" s="3"/>
+      <c r="J13" s="3"/>
+      <c r="K13" s="3"/>
+      <c r="M13" s="3"/>
+      <c r="N13" s="3"/>
+      <c r="P13" s="3"/>
+      <c r="Q13" s="3"/>
+      <c r="R13" s="1"/>
+      <c r="S13" s="3"/>
+      <c r="T13" s="3"/>
+      <c r="U13" s="1"/>
+      <c r="V13" s="3"/>
+      <c r="W13" s="3"/>
+      <c r="X13" s="1"/>
+      <c r="Y13" s="3"/>
+      <c r="Z13" s="3"/>
+      <c r="AA13" s="1"/>
+      <c r="AB13" s="3"/>
+      <c r="AC13" s="3"/>
+      <c r="AE13" s="3"/>
+      <c r="AF13" s="3"/>
+      <c r="AG13" s="1"/>
+      <c r="AH13" s="3"/>
+      <c r="AI13" s="3"/>
+      <c r="AJ13" s="1"/>
+      <c r="AK13" s="3"/>
+      <c r="AL13" s="3"/>
+      <c r="AM13" s="1"/>
+      <c r="AN13" s="3"/>
+      <c r="AO13" s="3"/>
+      <c r="AP13" s="1"/>
+      <c r="AQ13" s="3"/>
+      <c r="AR13" s="3"/>
+    </row>
+    <row r="14" spans="1:44" x14ac:dyDescent="0.2">
+      <c r="A14" s="3"/>
+      <c r="B14" s="3"/>
+      <c r="D14" s="3"/>
+      <c r="E14" s="3"/>
+      <c r="G14" s="3"/>
+      <c r="H14" s="3"/>
+      <c r="J14" s="3"/>
+      <c r="K14" s="3"/>
+      <c r="M14" s="3"/>
+      <c r="N14" s="3"/>
+      <c r="P14" s="3"/>
+      <c r="Q14" s="3"/>
+      <c r="R14" s="1"/>
+      <c r="S14" s="3"/>
+      <c r="T14" s="3"/>
+      <c r="U14" s="1"/>
+      <c r="V14" s="3"/>
+      <c r="W14" s="3"/>
+      <c r="X14" s="1"/>
+      <c r="Y14" s="3"/>
+      <c r="Z14" s="3"/>
+      <c r="AA14" s="1"/>
+      <c r="AB14" s="3"/>
+      <c r="AC14" s="3"/>
+      <c r="AE14" s="3"/>
+      <c r="AF14" s="3"/>
+      <c r="AG14" s="1"/>
+      <c r="AH14" s="3"/>
+      <c r="AI14" s="3"/>
+      <c r="AJ14" s="1"/>
+      <c r="AK14" s="3"/>
+      <c r="AL14" s="3"/>
+      <c r="AM14" s="1"/>
+      <c r="AN14" s="3"/>
+      <c r="AO14" s="3"/>
+      <c r="AP14" s="1"/>
+      <c r="AQ14" s="3"/>
+      <c r="AR14" s="3"/>
+    </row>
+    <row r="15" spans="1:44" x14ac:dyDescent="0.2">
+      <c r="A15" s="3"/>
+      <c r="B15" s="3"/>
+      <c r="D15" s="3"/>
+      <c r="E15" s="3"/>
+      <c r="G15" s="3"/>
+      <c r="H15" s="3"/>
+      <c r="J15" s="3"/>
+      <c r="K15" s="3"/>
+      <c r="M15" s="3"/>
+      <c r="N15" s="3"/>
+      <c r="P15" s="3"/>
+      <c r="Q15" s="3"/>
+      <c r="R15" s="1"/>
+      <c r="S15" s="3"/>
+      <c r="T15" s="3"/>
+      <c r="U15" s="1"/>
+      <c r="V15" s="3"/>
+      <c r="W15" s="3"/>
+      <c r="X15" s="1"/>
+      <c r="Y15" s="3"/>
+      <c r="Z15" s="3"/>
+      <c r="AA15" s="1"/>
+      <c r="AB15" s="3"/>
+      <c r="AC15" s="3"/>
+      <c r="AE15" s="3"/>
+      <c r="AF15" s="3"/>
+      <c r="AG15" s="1"/>
+      <c r="AH15" s="3"/>
+      <c r="AI15" s="3"/>
+      <c r="AJ15" s="1"/>
+      <c r="AK15" s="3"/>
+      <c r="AL15" s="3"/>
+      <c r="AM15" s="1"/>
+      <c r="AN15" s="3"/>
+      <c r="AO15" s="3"/>
+      <c r="AP15" s="1"/>
+      <c r="AQ15" s="3"/>
+      <c r="AR15" s="3"/>
+    </row>
+    <row r="16" spans="1:44" x14ac:dyDescent="0.2">
+      <c r="A16" s="3"/>
+      <c r="B16" s="3"/>
+      <c r="D16" s="3"/>
+      <c r="E16" s="3"/>
+      <c r="G16" s="3"/>
+      <c r="H16" s="3"/>
+      <c r="J16" s="3"/>
+      <c r="K16" s="3"/>
+      <c r="M16" s="3"/>
+      <c r="N16" s="3"/>
+      <c r="P16" s="3"/>
+      <c r="Q16" s="3"/>
+      <c r="R16" s="1"/>
+      <c r="S16" s="3"/>
+      <c r="T16" s="3"/>
+      <c r="U16" s="1"/>
+      <c r="V16" s="3"/>
+      <c r="W16" s="3"/>
+      <c r="X16" s="1"/>
+      <c r="Y16" s="3"/>
+      <c r="Z16" s="3"/>
+      <c r="AA16" s="1"/>
+      <c r="AB16" s="3"/>
+      <c r="AC16" s="3"/>
+      <c r="AE16" s="3"/>
+      <c r="AF16" s="3"/>
+      <c r="AG16" s="1"/>
+      <c r="AH16" s="3"/>
+      <c r="AI16" s="3"/>
+      <c r="AJ16" s="1"/>
+      <c r="AK16" s="3"/>
+      <c r="AL16" s="3"/>
+      <c r="AM16" s="1"/>
+      <c r="AN16" s="3"/>
+      <c r="AO16" s="3"/>
+      <c r="AP16" s="1"/>
+      <c r="AQ16" s="3"/>
+      <c r="AR16" s="3"/>
+    </row>
+    <row r="17" spans="1:44" x14ac:dyDescent="0.2">
+      <c r="A17" s="3"/>
+      <c r="B17" s="3"/>
+      <c r="D17" s="3"/>
+      <c r="E17" s="3"/>
+      <c r="G17" s="3"/>
+      <c r="H17" s="3"/>
+      <c r="J17" s="3"/>
+      <c r="K17" s="3"/>
+      <c r="M17" s="3"/>
+      <c r="N17" s="3"/>
+      <c r="P17" s="3"/>
+      <c r="Q17" s="3"/>
+      <c r="R17" s="1"/>
+      <c r="S17" s="3"/>
+      <c r="T17" s="3"/>
+      <c r="U17" s="1"/>
+      <c r="V17" s="3"/>
+      <c r="W17" s="3"/>
+      <c r="X17" s="1"/>
+      <c r="Y17" s="3"/>
+      <c r="Z17" s="3"/>
+      <c r="AA17" s="1"/>
+      <c r="AB17" s="3"/>
+      <c r="AC17" s="3"/>
+      <c r="AE17" s="3"/>
+      <c r="AF17" s="3"/>
+      <c r="AG17" s="1"/>
+      <c r="AH17" s="3"/>
+      <c r="AI17" s="3"/>
+      <c r="AJ17" s="1"/>
+      <c r="AK17" s="3"/>
+      <c r="AL17" s="3"/>
+      <c r="AM17" s="1"/>
+      <c r="AN17" s="3"/>
+      <c r="AO17" s="3"/>
+      <c r="AP17" s="1"/>
+      <c r="AQ17" s="3"/>
+      <c r="AR17" s="3"/>
+    </row>
+    <row r="18" spans="1:44" x14ac:dyDescent="0.2">
+      <c r="A18" s="3"/>
+      <c r="B18" s="3"/>
+      <c r="D18" s="3"/>
+      <c r="E18" s="3"/>
+      <c r="G18" s="3"/>
+      <c r="H18" s="3"/>
+      <c r="J18" s="3"/>
+      <c r="K18" s="3"/>
+      <c r="M18" s="3"/>
+      <c r="N18" s="3"/>
+      <c r="P18" s="3"/>
+      <c r="Q18" s="3"/>
+      <c r="R18" s="1"/>
+      <c r="S18" s="3"/>
+      <c r="T18" s="3"/>
+      <c r="U18" s="1"/>
+      <c r="V18" s="3"/>
+      <c r="W18" s="3"/>
+      <c r="X18" s="1"/>
+      <c r="Y18" s="3"/>
+      <c r="Z18" s="3"/>
+      <c r="AA18" s="1"/>
+      <c r="AB18" s="3"/>
+      <c r="AC18" s="3"/>
+      <c r="AE18" s="3"/>
+      <c r="AF18" s="3"/>
+      <c r="AG18" s="1"/>
+      <c r="AH18" s="3"/>
+      <c r="AI18" s="3"/>
+      <c r="AJ18" s="1"/>
+      <c r="AK18" s="3"/>
+      <c r="AL18" s="3"/>
+      <c r="AM18" s="1"/>
+      <c r="AN18" s="3"/>
+      <c r="AO18" s="3"/>
+      <c r="AP18" s="1"/>
+      <c r="AQ18" s="3"/>
+      <c r="AR18" s="3"/>
+    </row>
+    <row r="19" spans="1:44" x14ac:dyDescent="0.2">
+      <c r="A19" s="3"/>
+      <c r="B19" s="3"/>
+      <c r="D19" s="3"/>
+      <c r="E19" s="3"/>
+      <c r="G19" s="3"/>
+      <c r="H19" s="3"/>
+      <c r="J19" s="3"/>
+      <c r="K19" s="3"/>
+      <c r="M19" s="3"/>
+      <c r="N19" s="3"/>
+      <c r="P19" s="3"/>
+      <c r="Q19" s="3"/>
+      <c r="R19" s="1"/>
+      <c r="S19" s="3"/>
+      <c r="T19" s="3"/>
+      <c r="U19" s="1"/>
+      <c r="V19" s="3"/>
+      <c r="W19" s="3"/>
+      <c r="X19" s="1"/>
+      <c r="Y19" s="3"/>
+      <c r="Z19" s="3"/>
+      <c r="AA19" s="1"/>
+      <c r="AB19" s="3"/>
+      <c r="AC19" s="3"/>
+      <c r="AE19" s="3"/>
+      <c r="AF19" s="3"/>
+      <c r="AG19" s="1"/>
+      <c r="AH19" s="3"/>
+      <c r="AI19" s="3"/>
+      <c r="AJ19" s="1"/>
+      <c r="AK19" s="3"/>
+      <c r="AL19" s="3"/>
+      <c r="AM19" s="1"/>
+      <c r="AN19" s="3"/>
+      <c r="AO19" s="3"/>
+      <c r="AP19" s="1"/>
+      <c r="AQ19" s="3"/>
+      <c r="AR19" s="3"/>
+    </row>
+    <row r="20" spans="1:44" x14ac:dyDescent="0.2">
+      <c r="A20" s="3"/>
+      <c r="B20" s="3"/>
+      <c r="D20" s="3"/>
+      <c r="E20" s="3"/>
+      <c r="G20" s="3"/>
+      <c r="H20" s="3"/>
+      <c r="J20" s="3"/>
+      <c r="K20" s="3"/>
+      <c r="M20" s="3"/>
+      <c r="N20" s="3"/>
+      <c r="P20" s="3"/>
+      <c r="Q20" s="3"/>
+      <c r="R20" s="1"/>
+      <c r="S20" s="3"/>
+      <c r="T20" s="3"/>
+      <c r="U20" s="1"/>
+      <c r="V20" s="3"/>
+      <c r="W20" s="3"/>
+      <c r="X20" s="1"/>
+      <c r="Y20" s="3"/>
+      <c r="Z20" s="3"/>
+      <c r="AA20" s="1"/>
+      <c r="AB20" s="3"/>
+      <c r="AC20" s="3"/>
+      <c r="AE20" s="3"/>
+      <c r="AF20" s="3"/>
+      <c r="AG20" s="1"/>
+      <c r="AH20" s="3"/>
+      <c r="AI20" s="3"/>
+      <c r="AJ20" s="1"/>
+      <c r="AK20" s="3"/>
+      <c r="AL20" s="3"/>
+      <c r="AM20" s="1"/>
+      <c r="AN20" s="3"/>
+      <c r="AO20" s="3"/>
+      <c r="AP20" s="1"/>
+      <c r="AQ20" s="3"/>
+      <c r="AR20" s="3"/>
+    </row>
+    <row r="21" spans="1:44" x14ac:dyDescent="0.2">
+      <c r="A21" s="3"/>
+      <c r="B21" s="3"/>
+      <c r="D21" s="3"/>
+      <c r="E21" s="3"/>
+      <c r="G21" s="3"/>
+      <c r="H21" s="3"/>
+      <c r="J21" s="3"/>
+      <c r="K21" s="3"/>
+      <c r="M21" s="3"/>
+      <c r="N21" s="3"/>
+      <c r="P21" s="3"/>
+      <c r="Q21" s="3"/>
+      <c r="R21" s="1"/>
+      <c r="S21" s="3"/>
+      <c r="T21" s="3"/>
+      <c r="U21" s="1"/>
+      <c r="V21" s="3"/>
+      <c r="W21" s="3"/>
+      <c r="X21" s="1"/>
+      <c r="Y21" s="3"/>
+      <c r="Z21" s="3"/>
+      <c r="AA21" s="1"/>
+      <c r="AB21" s="3"/>
+      <c r="AC21" s="3"/>
+      <c r="AE21" s="3"/>
+      <c r="AF21" s="3"/>
+      <c r="AG21" s="1"/>
+      <c r="AH21" s="3"/>
+      <c r="AI21" s="3"/>
+      <c r="AJ21" s="1"/>
+      <c r="AK21" s="3"/>
+      <c r="AL21" s="3"/>
+      <c r="AM21" s="1"/>
+      <c r="AN21" s="3"/>
+      <c r="AO21" s="3"/>
+      <c r="AP21" s="1"/>
+      <c r="AQ21" s="3"/>
+      <c r="AR21" s="3"/>
+    </row>
+    <row r="22" spans="1:44" x14ac:dyDescent="0.2">
+      <c r="A22" s="3"/>
+      <c r="B22" s="3"/>
+      <c r="D22" s="3"/>
+      <c r="E22" s="3"/>
+      <c r="G22" s="3"/>
+      <c r="H22" s="3"/>
+      <c r="J22" s="3"/>
+      <c r="K22" s="3"/>
+      <c r="M22" s="3"/>
+      <c r="N22" s="3"/>
+      <c r="P22" s="3"/>
+      <c r="Q22" s="3"/>
+      <c r="R22" s="1"/>
+      <c r="S22" s="3"/>
+      <c r="T22" s="3"/>
+      <c r="U22" s="1"/>
+      <c r="V22" s="3"/>
+      <c r="W22" s="3"/>
+      <c r="X22" s="1"/>
+      <c r="Y22" s="3"/>
+      <c r="Z22" s="3"/>
+      <c r="AA22" s="1"/>
+      <c r="AB22" s="3"/>
+      <c r="AC22" s="3"/>
+      <c r="AE22" s="3"/>
+      <c r="AF22" s="3"/>
+      <c r="AG22" s="1"/>
+      <c r="AH22" s="3"/>
+      <c r="AI22" s="3"/>
+      <c r="AJ22" s="1"/>
+      <c r="AK22" s="3"/>
+      <c r="AL22" s="3"/>
+      <c r="AM22" s="1"/>
+      <c r="AN22" s="3"/>
+      <c r="AO22" s="3"/>
+      <c r="AP22" s="1"/>
+      <c r="AQ22" s="3"/>
+      <c r="AR22" s="3"/>
+    </row>
+    <row r="23" spans="1:44" x14ac:dyDescent="0.2">
+      <c r="A23" s="3"/>
+      <c r="B23" s="3"/>
+      <c r="D23" s="3"/>
+      <c r="E23" s="3"/>
+      <c r="G23" s="3"/>
+      <c r="H23" s="3"/>
+      <c r="J23" s="3"/>
+      <c r="K23" s="3"/>
+      <c r="M23" s="3"/>
+      <c r="N23" s="3"/>
+      <c r="P23" s="3"/>
+      <c r="Q23" s="3"/>
+      <c r="R23" s="1"/>
+      <c r="S23" s="3"/>
+      <c r="T23" s="3"/>
+      <c r="U23" s="1"/>
+      <c r="V23" s="3"/>
+      <c r="W23" s="3"/>
+      <c r="X23" s="1"/>
+      <c r="Y23" s="3"/>
+      <c r="Z23" s="3"/>
+      <c r="AA23" s="1"/>
+      <c r="AB23" s="3"/>
+      <c r="AC23" s="3"/>
+      <c r="AE23" s="3"/>
+      <c r="AF23" s="3"/>
+      <c r="AG23" s="1"/>
+      <c r="AH23" s="3"/>
+      <c r="AI23" s="3"/>
+      <c r="AJ23" s="1"/>
+      <c r="AK23" s="3"/>
+      <c r="AL23" s="3"/>
+      <c r="AM23" s="1"/>
+      <c r="AN23" s="3"/>
+      <c r="AO23" s="3"/>
+      <c r="AP23" s="1"/>
+      <c r="AQ23" s="3"/>
+      <c r="AR23" s="3"/>
+    </row>
+    <row r="24" spans="1:44" x14ac:dyDescent="0.2">
+      <c r="A24" s="3"/>
+      <c r="B24" s="3"/>
+      <c r="D24" s="3"/>
+      <c r="E24" s="3"/>
+      <c r="G24" s="3"/>
+      <c r="H24" s="3"/>
+      <c r="J24" s="3"/>
+      <c r="K24" s="3"/>
+      <c r="M24" s="3"/>
+      <c r="N24" s="3"/>
+      <c r="P24" s="3"/>
+      <c r="Q24" s="3"/>
+      <c r="R24" s="1"/>
+      <c r="S24" s="3"/>
+      <c r="T24" s="3"/>
+      <c r="U24" s="1"/>
+      <c r="V24" s="3"/>
+      <c r="W24" s="3"/>
+      <c r="X24" s="1"/>
+      <c r="Y24" s="3"/>
+      <c r="Z24" s="3"/>
+      <c r="AA24" s="1"/>
+      <c r="AB24" s="3"/>
+      <c r="AC24" s="3"/>
+      <c r="AE24" s="3"/>
+      <c r="AF24" s="3"/>
+      <c r="AG24" s="1"/>
+      <c r="AH24" s="3"/>
+      <c r="AI24" s="3"/>
+      <c r="AJ24" s="1"/>
+      <c r="AK24" s="3"/>
+      <c r="AL24" s="3"/>
+      <c r="AM24" s="1"/>
+      <c r="AN24" s="3"/>
+      <c r="AO24" s="3"/>
+      <c r="AP24" s="1"/>
+      <c r="AQ24" s="3"/>
+      <c r="AR24" s="3"/>
+    </row>
+    <row r="25" spans="1:44" x14ac:dyDescent="0.2">
+      <c r="A25" s="3"/>
+      <c r="B25" s="3"/>
+      <c r="D25" s="3"/>
+      <c r="E25" s="3"/>
+      <c r="G25" s="3"/>
+      <c r="H25" s="3"/>
+      <c r="J25" s="3"/>
+      <c r="K25" s="3"/>
+      <c r="M25" s="3"/>
+      <c r="N25" s="3"/>
+      <c r="P25" s="3"/>
+      <c r="Q25" s="3"/>
+      <c r="R25" s="1"/>
+      <c r="S25" s="3"/>
+      <c r="T25" s="3"/>
+      <c r="U25" s="1"/>
+      <c r="V25" s="3"/>
+      <c r="W25" s="3"/>
+      <c r="X25" s="1"/>
+      <c r="Y25" s="3"/>
+      <c r="Z25" s="3"/>
+      <c r="AA25" s="1"/>
+      <c r="AB25" s="3"/>
+      <c r="AC25" s="3"/>
+      <c r="AE25" s="3"/>
+      <c r="AF25" s="3"/>
+      <c r="AG25" s="1"/>
+      <c r="AH25" s="3"/>
+      <c r="AI25" s="3"/>
+      <c r="AJ25" s="1"/>
+      <c r="AK25" s="3"/>
+      <c r="AL25" s="3"/>
+      <c r="AM25" s="1"/>
+      <c r="AN25" s="3"/>
+      <c r="AO25" s="3"/>
+      <c r="AP25" s="1"/>
+      <c r="AQ25" s="3"/>
+      <c r="AR25" s="3"/>
+    </row>
+    <row r="26" spans="1:44" x14ac:dyDescent="0.2">
+      <c r="A26" s="3"/>
+      <c r="B26" s="3"/>
+      <c r="D26" s="3"/>
+      <c r="E26" s="3"/>
+      <c r="G26" s="3"/>
+      <c r="H26" s="3"/>
+      <c r="J26" s="3"/>
+      <c r="K26" s="3"/>
+      <c r="M26" s="3"/>
+      <c r="N26" s="3"/>
+      <c r="P26" s="3"/>
+      <c r="Q26" s="3"/>
+      <c r="R26" s="1"/>
+      <c r="S26" s="3"/>
+      <c r="T26" s="3"/>
+      <c r="U26" s="1"/>
+      <c r="V26" s="3"/>
+      <c r="W26" s="3"/>
+      <c r="X26" s="1"/>
+      <c r="Y26" s="3"/>
+      <c r="Z26" s="3"/>
+      <c r="AA26" s="1"/>
+      <c r="AB26" s="3"/>
+      <c r="AC26" s="3"/>
+      <c r="AE26" s="3"/>
+      <c r="AF26" s="3"/>
+      <c r="AG26" s="1"/>
+      <c r="AH26" s="3"/>
+      <c r="AI26" s="3"/>
+      <c r="AJ26" s="1"/>
+      <c r="AK26" s="3"/>
+      <c r="AL26" s="3"/>
+      <c r="AM26" s="1"/>
+      <c r="AN26" s="3"/>
+      <c r="AO26" s="3"/>
+      <c r="AP26" s="1"/>
+      <c r="AQ26" s="3"/>
+      <c r="AR26" s="3"/>
+    </row>
+    <row r="27" spans="1:44" x14ac:dyDescent="0.2">
+      <c r="A27" s="3"/>
+      <c r="B27" s="3"/>
+      <c r="D27" s="3"/>
+      <c r="E27" s="3"/>
+      <c r="G27" s="3"/>
+      <c r="H27" s="3"/>
+      <c r="J27" s="3"/>
+      <c r="K27" s="3"/>
+      <c r="M27" s="3"/>
+      <c r="N27" s="3"/>
+      <c r="P27" s="3"/>
+      <c r="Q27" s="3"/>
+      <c r="R27" s="1"/>
+      <c r="S27" s="3"/>
+      <c r="T27" s="3"/>
+      <c r="U27" s="1"/>
+      <c r="V27" s="3"/>
+      <c r="W27" s="3"/>
+      <c r="X27" s="1"/>
+      <c r="Y27" s="3"/>
+      <c r="Z27" s="3"/>
+      <c r="AA27" s="1"/>
+      <c r="AB27" s="3"/>
+      <c r="AC27" s="3"/>
+      <c r="AE27" s="3"/>
+      <c r="AF27" s="3"/>
+      <c r="AG27" s="1"/>
+      <c r="AH27" s="3"/>
+      <c r="AI27" s="3"/>
+      <c r="AJ27" s="1"/>
+      <c r="AK27" s="3"/>
+      <c r="AL27" s="3"/>
+      <c r="AM27" s="1"/>
+      <c r="AN27" s="3"/>
+      <c r="AO27" s="3"/>
+      <c r="AP27" s="1"/>
+      <c r="AQ27" s="3"/>
+      <c r="AR27" s="3"/>
+    </row>
+    <row r="28" spans="1:44" x14ac:dyDescent="0.2">
+      <c r="A28" s="3"/>
+      <c r="B28" s="3"/>
+      <c r="D28" s="3"/>
+      <c r="E28" s="3"/>
+      <c r="G28" s="3"/>
+      <c r="H28" s="3"/>
+      <c r="J28" s="3"/>
+      <c r="K28" s="3"/>
+      <c r="M28" s="3"/>
+      <c r="N28" s="3"/>
+      <c r="P28" s="3"/>
+      <c r="Q28" s="3"/>
+      <c r="R28" s="1"/>
+      <c r="S28" s="3"/>
+      <c r="T28" s="3"/>
+      <c r="U28" s="1"/>
+      <c r="V28" s="3"/>
+      <c r="W28" s="3"/>
+      <c r="X28" s="1"/>
+      <c r="Y28" s="3"/>
+      <c r="Z28" s="3"/>
+      <c r="AA28" s="1"/>
+      <c r="AB28" s="3"/>
+      <c r="AC28" s="3"/>
+      <c r="AE28" s="3"/>
+      <c r="AF28" s="3"/>
+      <c r="AG28" s="1"/>
+      <c r="AH28" s="3"/>
+      <c r="AI28" s="3"/>
+      <c r="AJ28" s="1"/>
+      <c r="AK28" s="3"/>
+      <c r="AL28" s="3"/>
+      <c r="AM28" s="1"/>
+      <c r="AN28" s="3"/>
+      <c r="AO28" s="3"/>
+      <c r="AP28" s="1"/>
+      <c r="AQ28" s="3"/>
+      <c r="AR28" s="3"/>
+    </row>
+  </sheetData>
+  <mergeCells count="30">
+    <mergeCell ref="AQ4:AR4"/>
+    <mergeCell ref="A4:B4"/>
+    <mergeCell ref="G4:H4"/>
+    <mergeCell ref="AK6:AL6"/>
+    <mergeCell ref="AE6:AF6"/>
+    <mergeCell ref="AQ6:AR6"/>
+    <mergeCell ref="M4:N4"/>
+    <mergeCell ref="S4:T4"/>
+    <mergeCell ref="AE4:AF4"/>
+    <mergeCell ref="A6:B6"/>
+    <mergeCell ref="AK4:AL4"/>
+    <mergeCell ref="D6:E6"/>
+    <mergeCell ref="V4:W4"/>
+    <mergeCell ref="AH4:AI4"/>
+    <mergeCell ref="J6:K6"/>
+    <mergeCell ref="P6:Q6"/>
+    <mergeCell ref="D4:E4"/>
+    <mergeCell ref="P4:Q4"/>
+    <mergeCell ref="Y4:Z4"/>
+    <mergeCell ref="AB6:AC6"/>
+    <mergeCell ref="AN6:AO6"/>
+    <mergeCell ref="AB4:AC4"/>
+    <mergeCell ref="AN4:AO4"/>
+    <mergeCell ref="G6:H6"/>
+    <mergeCell ref="J4:K4"/>
+    <mergeCell ref="V6:W6"/>
+    <mergeCell ref="M6:N6"/>
+    <mergeCell ref="AH6:AI6"/>
+    <mergeCell ref="S6:T6"/>
+    <mergeCell ref="Y6:Z6"/>
+  </mergeCells>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0400-000000000000}">
+  <dimension ref="A2:AR29"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
+  <cols>
+    <col min="1" max="2" width="10.83203125" style="1" customWidth="1"/>
+    <col min="3" max="3" width="3.83203125" style="1" customWidth="1"/>
+    <col min="4" max="5" width="10.83203125" style="1" customWidth="1"/>
+    <col min="6" max="6" width="3.83203125" style="1" customWidth="1"/>
+    <col min="7" max="8" width="10.83203125" style="1" customWidth="1"/>
+    <col min="9" max="9" width="3.83203125" style="1" customWidth="1"/>
+    <col min="10" max="11" width="10.83203125" style="1" customWidth="1"/>
+    <col min="12" max="12" width="3.83203125" style="1" customWidth="1"/>
+    <col min="13" max="14" width="10.83203125" style="1" customWidth="1"/>
+    <col min="15" max="15" width="3.83203125" customWidth="1"/>
+    <col min="18" max="18" width="3.83203125" customWidth="1"/>
+    <col min="21" max="21" width="3.83203125" customWidth="1"/>
+    <col min="24" max="24" width="3.83203125" customWidth="1"/>
+    <col min="27" max="27" width="3.83203125" customWidth="1"/>
+    <col min="30" max="30" width="3.83203125" customWidth="1"/>
+    <col min="33" max="33" width="3.83203125" customWidth="1"/>
+    <col min="36" max="36" width="3.83203125" customWidth="1"/>
+    <col min="39" max="39" width="3.83203125" customWidth="1"/>
+    <col min="42" max="42" width="3.83203125" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="2" spans="1:44" x14ac:dyDescent="0.2">
+      <c r="A2" s="24" t="s">
+        <v>179</v>
+      </c>
+      <c r="G2" s="9" t="s">
+        <v>306</v>
+      </c>
+    </row>
+    <row r="4" spans="1:44" x14ac:dyDescent="0.2">
+      <c r="A4" s="55" t="s">
+        <v>180</v>
+      </c>
+      <c r="B4" s="52"/>
+      <c r="D4" s="55" t="s">
+        <v>181</v>
+      </c>
+      <c r="E4" s="52"/>
+      <c r="G4" s="55" t="s">
+        <v>182</v>
+      </c>
+      <c r="H4" s="52"/>
+      <c r="J4" s="55" t="s">
+        <v>183</v>
+      </c>
+      <c r="K4" s="52"/>
+      <c r="M4" s="55" t="s">
+        <v>184</v>
+      </c>
+      <c r="N4" s="52"/>
+      <c r="P4" s="55" t="s">
+        <v>185</v>
+      </c>
+      <c r="Q4" s="54"/>
+      <c r="R4" s="1"/>
+      <c r="S4" s="55" t="s">
+        <v>186</v>
+      </c>
+      <c r="T4" s="54"/>
+      <c r="U4" s="1"/>
+      <c r="V4" s="55" t="s">
+        <v>187</v>
+      </c>
+      <c r="W4" s="54"/>
+      <c r="X4" s="1"/>
+      <c r="Y4" s="55" t="s">
+        <v>188</v>
+      </c>
+      <c r="Z4" s="54"/>
+      <c r="AA4" s="1"/>
+      <c r="AB4" s="55" t="s">
+        <v>189</v>
+      </c>
+      <c r="AC4" s="54"/>
+      <c r="AE4" s="55" t="s">
+        <v>190</v>
+      </c>
+      <c r="AF4" s="54"/>
+      <c r="AG4" s="1"/>
+      <c r="AH4" s="55" t="s">
+        <v>191</v>
+      </c>
+      <c r="AI4" s="54"/>
+      <c r="AJ4" s="1"/>
+      <c r="AK4" s="55" t="s">
+        <v>192</v>
+      </c>
+      <c r="AL4" s="54"/>
+      <c r="AM4" s="1"/>
+      <c r="AN4" s="55" t="s">
+        <v>193</v>
+      </c>
+      <c r="AO4" s="54"/>
+      <c r="AP4" s="1"/>
+      <c r="AQ4" s="55" t="s">
+        <v>194</v>
+      </c>
+      <c r="AR4" s="54"/>
+    </row>
+    <row r="5" spans="1:44" x14ac:dyDescent="0.2">
+      <c r="A5" s="38" t="s">
+        <v>198</v>
+      </c>
+      <c r="B5" s="39" t="s">
+        <v>305</v>
+      </c>
+      <c r="D5" s="38" t="s">
+        <v>198</v>
+      </c>
+      <c r="E5" s="39" t="s">
+        <v>305</v>
+      </c>
+      <c r="G5" s="38" t="s">
+        <v>198</v>
+      </c>
+      <c r="H5" s="39" t="s">
+        <v>305</v>
+      </c>
+      <c r="J5" s="38" t="s">
+        <v>198</v>
+      </c>
+      <c r="K5" s="39" t="s">
+        <v>305</v>
+      </c>
+      <c r="M5" s="38" t="s">
+        <v>198</v>
+      </c>
+      <c r="N5" s="39" t="s">
+        <v>305</v>
+      </c>
+      <c r="P5" s="38" t="s">
+        <v>198</v>
+      </c>
+      <c r="Q5" s="39" t="s">
+        <v>305</v>
+      </c>
+      <c r="R5" s="1"/>
+      <c r="S5" s="38" t="s">
+        <v>198</v>
+      </c>
+      <c r="T5" s="39" t="s">
+        <v>305</v>
+      </c>
+      <c r="U5" s="1"/>
+      <c r="V5" s="38" t="s">
+        <v>198</v>
+      </c>
+      <c r="W5" s="39" t="s">
+        <v>305</v>
+      </c>
+      <c r="X5" s="1"/>
+      <c r="Y5" s="38" t="s">
+        <v>198</v>
+      </c>
+      <c r="Z5" s="39" t="s">
+        <v>305</v>
+      </c>
+      <c r="AA5" s="1"/>
+      <c r="AB5" s="38" t="s">
+        <v>198</v>
+      </c>
+      <c r="AC5" s="39" t="s">
+        <v>305</v>
+      </c>
+      <c r="AE5" s="38" t="s">
+        <v>198</v>
+      </c>
+      <c r="AF5" s="39" t="s">
+        <v>305</v>
+      </c>
+      <c r="AG5" s="1"/>
+      <c r="AH5" s="38" t="s">
+        <v>198</v>
+      </c>
+      <c r="AI5" s="39" t="s">
+        <v>305</v>
+      </c>
+      <c r="AJ5" s="1"/>
+      <c r="AK5" s="38" t="s">
+        <v>198</v>
+      </c>
+      <c r="AL5" s="39" t="s">
+        <v>305</v>
+      </c>
+      <c r="AM5" s="1"/>
+      <c r="AN5" s="38" t="s">
+        <v>198</v>
+      </c>
+      <c r="AO5" s="39" t="s">
+        <v>305</v>
+      </c>
+      <c r="AP5" s="1"/>
+      <c r="AQ5" s="38" t="s">
+        <v>198</v>
+      </c>
+      <c r="AR5" s="39" t="s">
+        <v>305</v>
+      </c>
+    </row>
+    <row r="6" spans="1:44" x14ac:dyDescent="0.2">
+      <c r="A6" s="38" t="s">
+        <v>176</v>
+      </c>
+      <c r="B6" s="39">
+        <v>1</v>
+      </c>
+      <c r="D6" s="38" t="s">
+        <v>176</v>
+      </c>
+      <c r="E6" s="39">
+        <v>2</v>
+      </c>
+      <c r="G6" s="38" t="s">
+        <v>176</v>
+      </c>
+      <c r="H6" s="39">
+        <v>3</v>
+      </c>
+      <c r="J6" s="38" t="s">
+        <v>176</v>
+      </c>
+      <c r="K6" s="39">
+        <v>4</v>
+      </c>
+      <c r="M6" s="38" t="s">
+        <v>176</v>
+      </c>
+      <c r="N6" s="39">
+        <v>5</v>
+      </c>
+      <c r="P6" s="38" t="s">
+        <v>176</v>
+      </c>
+      <c r="Q6" s="39">
+        <v>6</v>
+      </c>
+      <c r="R6" s="1"/>
+      <c r="S6" s="38" t="s">
+        <v>176</v>
+      </c>
+      <c r="T6" s="39">
+        <v>7</v>
+      </c>
+      <c r="U6" s="1"/>
+      <c r="V6" s="38" t="s">
+        <v>176</v>
+      </c>
+      <c r="W6" s="39">
+        <v>8</v>
+      </c>
+      <c r="X6" s="1"/>
+      <c r="Y6" s="38" t="s">
+        <v>176</v>
+      </c>
+      <c r="Z6" s="39">
+        <v>9</v>
+      </c>
+      <c r="AA6" s="1"/>
+      <c r="AB6" s="38" t="s">
+        <v>176</v>
+      </c>
+      <c r="AC6" s="39">
+        <v>10</v>
+      </c>
+      <c r="AE6" s="38" t="s">
+        <v>176</v>
+      </c>
+      <c r="AF6" s="39">
+        <v>11</v>
+      </c>
+      <c r="AG6" s="1"/>
+      <c r="AH6" s="38" t="s">
+        <v>176</v>
+      </c>
+      <c r="AI6" s="39">
+        <v>12</v>
+      </c>
+      <c r="AJ6" s="1"/>
+      <c r="AK6" s="38" t="s">
+        <v>176</v>
+      </c>
+      <c r="AL6" s="39">
+        <v>13</v>
+      </c>
+      <c r="AM6" s="1"/>
+      <c r="AN6" s="38" t="s">
+        <v>176</v>
+      </c>
+      <c r="AO6" s="39">
+        <v>14</v>
+      </c>
+      <c r="AP6" s="1"/>
+      <c r="AQ6" s="38" t="s">
+        <v>176</v>
+      </c>
+      <c r="AR6" s="39">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="7" spans="1:44" x14ac:dyDescent="0.2">
+      <c r="A7" s="58" t="str">
+        <f>IF(OR(B5="",B5="material"),_xlfn.XLOOKUP(B6,mat!$A:$A, mat!$B:$B,"") &amp; "","")</f>
+        <v/>
+      </c>
+      <c r="B7" s="57"/>
+      <c r="D7" s="58" t="str">
+        <f>IF(OR(E5="",E5="material"),_xlfn.XLOOKUP(E6,mat!$A:$A, mat!$B:$B,"") &amp; "","")</f>
+        <v/>
+      </c>
+      <c r="E7" s="57"/>
+      <c r="G7" s="58" t="str">
+        <f>IF(OR(H5="",H5="material"),_xlfn.XLOOKUP(H6,mat!$A:$A, mat!$B:$B,"") &amp; "","")</f>
+        <v/>
+      </c>
+      <c r="H7" s="57"/>
+      <c r="J7" s="58" t="str">
+        <f>IF(OR(K5="",K5="material"),_xlfn.XLOOKUP(K6,mat!$A:$A, mat!$B:$B,"") &amp; "","")</f>
+        <v/>
+      </c>
+      <c r="K7" s="57"/>
+      <c r="M7" s="58" t="str">
+        <f>IF(OR(N5="",N5="material"),_xlfn.XLOOKUP(N6,mat!$A:$A, mat!$B:$B,"") &amp; "","")</f>
+        <v/>
+      </c>
+      <c r="N7" s="57"/>
+      <c r="P7" s="58" t="str">
+        <f>IF(OR(Q5="",Q5="material"),_xlfn.XLOOKUP(Q6,mat!$A:$A, mat!$B:$B,"") &amp; "","")</f>
+        <v/>
+      </c>
+      <c r="Q7" s="57"/>
+      <c r="R7" s="1"/>
+      <c r="S7" s="58" t="str">
+        <f>IF(OR(T5="",T5="material"),_xlfn.XLOOKUP(T6,mat!$A:$A, mat!$B:$B,"") &amp; "","")</f>
+        <v/>
+      </c>
+      <c r="T7" s="57"/>
+      <c r="U7" s="1"/>
+      <c r="V7" s="58" t="str">
+        <f>IF(OR(W5="",W5="material"),_xlfn.XLOOKUP(W6,mat!$A:$A, mat!$B:$B,"") &amp; "","")</f>
+        <v/>
+      </c>
+      <c r="W7" s="57"/>
+      <c r="X7" s="1"/>
+      <c r="Y7" s="58" t="str">
+        <f>IF(OR(Z5="",Z5="material"),_xlfn.XLOOKUP(Z6,mat!$A:$A, mat!$B:$B,"") &amp; "","")</f>
+        <v/>
+      </c>
+      <c r="Z7" s="57"/>
+      <c r="AA7" s="1"/>
+      <c r="AB7" s="58" t="str">
+        <f>IF(OR(AC5="",AC5="material"),_xlfn.XLOOKUP(AC6,mat!$A:$A, mat!$B:$B,"") &amp; "","")</f>
+        <v/>
+      </c>
+      <c r="AC7" s="57"/>
+      <c r="AE7" s="58" t="str">
+        <f>IF(OR(AF5="",AF5="material"),_xlfn.XLOOKUP(AF6,mat!$A:$A, mat!$B:$B,"") &amp; "","")</f>
+        <v/>
+      </c>
+      <c r="AF7" s="57"/>
+      <c r="AG7" s="1"/>
+      <c r="AH7" s="58" t="str">
+        <f>IF(OR(AI5="",AI5="material"),_xlfn.XLOOKUP(AI6,mat!$A:$A, mat!$B:$B,"") &amp; "","")</f>
+        <v/>
+      </c>
+      <c r="AI7" s="57"/>
+      <c r="AJ7" s="1"/>
+      <c r="AK7" s="58" t="str">
+        <f>IF(OR(AL5="",AL5="material"),_xlfn.XLOOKUP(AL6,mat!$A:$A, mat!$B:$B,"") &amp; "","")</f>
+        <v/>
+      </c>
+      <c r="AL7" s="57"/>
+      <c r="AM7" s="1"/>
+      <c r="AN7" s="58" t="str">
+        <f>IF(OR(AO5="",AO5="material"),_xlfn.XLOOKUP(AO6,mat!$A:$A, mat!$B:$B,"") &amp; "","")</f>
+        <v/>
+      </c>
+      <c r="AO7" s="57"/>
+      <c r="AP7" s="1"/>
+      <c r="AQ7" s="58" t="str">
+        <f>IF(OR(AR5="",AR5="material"),_xlfn.XLOOKUP(AR6,mat!$A:$A, mat!$B:$B,"") &amp; "","")</f>
+        <v/>
+      </c>
+      <c r="AR7" s="57"/>
+    </row>
+    <row r="8" spans="1:44" x14ac:dyDescent="0.2">
+      <c r="A8" s="38" t="s">
+        <v>303</v>
+      </c>
+      <c r="B8" s="39"/>
+      <c r="D8" s="38" t="s">
+        <v>303</v>
+      </c>
+      <c r="E8" s="39"/>
+      <c r="G8" s="38" t="s">
+        <v>303</v>
+      </c>
+      <c r="H8" s="39"/>
+      <c r="J8" s="38" t="s">
+        <v>303</v>
+      </c>
+      <c r="K8" s="39"/>
+      <c r="M8" s="38" t="s">
+        <v>303</v>
+      </c>
+      <c r="N8" s="39"/>
+      <c r="P8" s="38" t="s">
+        <v>303</v>
+      </c>
+      <c r="Q8" s="39"/>
+      <c r="R8" s="1"/>
+      <c r="S8" s="38" t="s">
+        <v>303</v>
+      </c>
+      <c r="T8" s="39"/>
+      <c r="U8" s="1"/>
+      <c r="V8" s="38" t="s">
+        <v>303</v>
+      </c>
+      <c r="W8" s="39"/>
+      <c r="X8" s="1"/>
+      <c r="Y8" s="38" t="s">
+        <v>303</v>
+      </c>
+      <c r="Z8" s="39"/>
+      <c r="AA8" s="1"/>
+      <c r="AB8" s="38" t="s">
+        <v>303</v>
+      </c>
+      <c r="AC8" s="39"/>
+      <c r="AE8" s="38" t="s">
+        <v>303</v>
+      </c>
+      <c r="AF8" s="39"/>
+      <c r="AG8" s="1"/>
+      <c r="AH8" s="38" t="s">
+        <v>303</v>
+      </c>
+      <c r="AI8" s="39"/>
+      <c r="AJ8" s="1"/>
+      <c r="AK8" s="38" t="s">
+        <v>303</v>
+      </c>
+      <c r="AL8" s="39"/>
+      <c r="AM8" s="1"/>
+      <c r="AN8" s="38" t="s">
+        <v>303</v>
+      </c>
+      <c r="AO8" s="39"/>
+      <c r="AP8" s="1"/>
+      <c r="AQ8" s="38" t="s">
+        <v>303</v>
+      </c>
+      <c r="AR8" s="39"/>
+    </row>
+    <row r="9" spans="1:44" x14ac:dyDescent="0.2">
+      <c r="A9" s="2" t="s">
+        <v>177</v>
+      </c>
+      <c r="B9" s="2" t="s">
+        <v>178</v>
+      </c>
+      <c r="D9" s="2" t="s">
+        <v>177</v>
+      </c>
+      <c r="E9" s="2" t="s">
+        <v>178</v>
+      </c>
+      <c r="G9" s="2" t="s">
+        <v>177</v>
+      </c>
+      <c r="H9" s="2" t="s">
+        <v>178</v>
+      </c>
+      <c r="J9" s="2" t="s">
+        <v>177</v>
+      </c>
+      <c r="K9" s="2" t="s">
+        <v>178</v>
+      </c>
+      <c r="M9" s="2" t="s">
+        <v>177</v>
+      </c>
+      <c r="N9" s="2" t="s">
+        <v>178</v>
+      </c>
+      <c r="P9" s="2" t="s">
+        <v>177</v>
+      </c>
+      <c r="Q9" s="2" t="s">
+        <v>178</v>
+      </c>
+      <c r="R9" s="1"/>
+      <c r="S9" s="2" t="s">
+        <v>177</v>
+      </c>
+      <c r="T9" s="2" t="s">
+        <v>178</v>
+      </c>
+      <c r="U9" s="1"/>
+      <c r="V9" s="2" t="s">
+        <v>177</v>
+      </c>
+      <c r="W9" s="2" t="s">
+        <v>178</v>
+      </c>
+      <c r="X9" s="1"/>
+      <c r="Y9" s="2" t="s">
+        <v>177</v>
+      </c>
+      <c r="Z9" s="2" t="s">
+        <v>178</v>
+      </c>
+      <c r="AA9" s="1"/>
+      <c r="AB9" s="2" t="s">
+        <v>177</v>
+      </c>
+      <c r="AC9" s="2" t="s">
+        <v>178</v>
+      </c>
+      <c r="AE9" s="2" t="s">
+        <v>177</v>
+      </c>
+      <c r="AF9" s="2" t="s">
+        <v>178</v>
+      </c>
+      <c r="AG9" s="1"/>
+      <c r="AH9" s="2" t="s">
+        <v>177</v>
+      </c>
+      <c r="AI9" s="2" t="s">
+        <v>178</v>
+      </c>
+      <c r="AJ9" s="1"/>
+      <c r="AK9" s="2" t="s">
+        <v>177</v>
+      </c>
+      <c r="AL9" s="2" t="s">
+        <v>178</v>
+      </c>
+      <c r="AM9" s="1"/>
+      <c r="AN9" s="2" t="s">
+        <v>177</v>
+      </c>
+      <c r="AO9" s="2" t="s">
+        <v>178</v>
+      </c>
+      <c r="AP9" s="1"/>
+      <c r="AQ9" s="2" t="s">
+        <v>177</v>
+      </c>
+      <c r="AR9" s="2" t="s">
+        <v>178</v>
+      </c>
+    </row>
+    <row r="10" spans="1:44" x14ac:dyDescent="0.2">
+      <c r="A10" s="3"/>
+      <c r="B10" s="3"/>
+      <c r="D10" s="3"/>
+      <c r="E10" s="3"/>
+      <c r="G10" s="3"/>
+      <c r="H10" s="3"/>
+      <c r="J10" s="3"/>
+      <c r="K10" s="3"/>
+      <c r="M10" s="3"/>
+      <c r="N10" s="3"/>
+      <c r="P10" s="3"/>
+      <c r="Q10" s="3"/>
+      <c r="R10" s="1"/>
+      <c r="S10" s="3"/>
+      <c r="T10" s="3"/>
+      <c r="U10" s="1"/>
+      <c r="V10" s="3"/>
+      <c r="W10" s="3"/>
+      <c r="X10" s="1"/>
+      <c r="Y10" s="3"/>
+      <c r="Z10" s="3"/>
+      <c r="AA10" s="1"/>
+      <c r="AB10" s="3"/>
+      <c r="AC10" s="3"/>
+      <c r="AE10" s="3"/>
+      <c r="AF10" s="3"/>
+      <c r="AG10" s="1"/>
+      <c r="AH10" s="3"/>
+      <c r="AI10" s="3"/>
+      <c r="AJ10" s="1"/>
+      <c r="AK10" s="3"/>
+      <c r="AL10" s="3"/>
+      <c r="AM10" s="1"/>
+      <c r="AN10" s="3"/>
+      <c r="AO10" s="3"/>
+      <c r="AP10" s="1"/>
+      <c r="AQ10" s="3"/>
+      <c r="AR10" s="3"/>
+    </row>
+    <row r="11" spans="1:44" x14ac:dyDescent="0.2">
+      <c r="A11" s="3"/>
+      <c r="B11" s="3"/>
+      <c r="D11" s="3"/>
+      <c r="E11" s="3"/>
+      <c r="G11" s="3"/>
+      <c r="H11" s="3"/>
+      <c r="J11" s="3"/>
+      <c r="K11" s="3"/>
+      <c r="M11" s="3"/>
+      <c r="N11" s="3"/>
+      <c r="P11" s="3"/>
+      <c r="Q11" s="3"/>
+      <c r="R11" s="1"/>
+      <c r="S11" s="3"/>
+      <c r="T11" s="3"/>
+      <c r="U11" s="1"/>
+      <c r="V11" s="3"/>
+      <c r="W11" s="3"/>
+      <c r="X11" s="1"/>
+      <c r="Y11" s="3"/>
+      <c r="Z11" s="3"/>
+      <c r="AA11" s="1"/>
+      <c r="AB11" s="3"/>
+      <c r="AC11" s="3"/>
+      <c r="AE11" s="3"/>
+      <c r="AF11" s="3"/>
+      <c r="AG11" s="1"/>
+      <c r="AH11" s="3"/>
+      <c r="AI11" s="3"/>
+      <c r="AJ11" s="1"/>
+      <c r="AK11" s="3"/>
+      <c r="AL11" s="3"/>
+      <c r="AM11" s="1"/>
+      <c r="AN11" s="3"/>
+      <c r="AO11" s="3"/>
+      <c r="AP11" s="1"/>
+      <c r="AQ11" s="3"/>
+      <c r="AR11" s="3"/>
     </row>
     <row r="12" spans="1:44" x14ac:dyDescent="0.2">
       <c r="A12" s="3"/>
@@ -15891,1322 +17402,6 @@
       <c r="AQ27" s="3"/>
       <c r="AR27" s="3"/>
     </row>
-  </sheetData>
-  <mergeCells count="30">
-    <mergeCell ref="D4:E4"/>
-    <mergeCell ref="P4:Q4"/>
-    <mergeCell ref="Y4:Z4"/>
-    <mergeCell ref="AB6:AC6"/>
-    <mergeCell ref="AN6:AO6"/>
-    <mergeCell ref="AB4:AC4"/>
-    <mergeCell ref="AN4:AO4"/>
-    <mergeCell ref="G6:H6"/>
-    <mergeCell ref="J4:K4"/>
-    <mergeCell ref="V6:W6"/>
-    <mergeCell ref="M6:N6"/>
-    <mergeCell ref="AH6:AI6"/>
-    <mergeCell ref="S6:T6"/>
-    <mergeCell ref="Y6:Z6"/>
-    <mergeCell ref="AQ4:AR4"/>
-    <mergeCell ref="A4:B4"/>
-    <mergeCell ref="G4:H4"/>
-    <mergeCell ref="AK6:AL6"/>
-    <mergeCell ref="AE6:AF6"/>
-    <mergeCell ref="AQ6:AR6"/>
-    <mergeCell ref="M4:N4"/>
-    <mergeCell ref="S4:T4"/>
-    <mergeCell ref="AE4:AF4"/>
-    <mergeCell ref="A6:B6"/>
-    <mergeCell ref="AK4:AL4"/>
-    <mergeCell ref="D6:E6"/>
-    <mergeCell ref="V4:W4"/>
-    <mergeCell ref="AH4:AI4"/>
-    <mergeCell ref="J6:K6"/>
-    <mergeCell ref="P6:Q6"/>
-  </mergeCells>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0400-000000000000}">
-  <dimension ref="A2:AR29"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
-  <cols>
-    <col min="1" max="2" width="10.83203125" style="1" customWidth="1"/>
-    <col min="3" max="3" width="3.83203125" style="1" customWidth="1"/>
-    <col min="4" max="5" width="10.83203125" style="1" customWidth="1"/>
-    <col min="6" max="6" width="3.83203125" style="1" customWidth="1"/>
-    <col min="7" max="8" width="10.83203125" style="1" customWidth="1"/>
-    <col min="9" max="9" width="3.83203125" style="1" customWidth="1"/>
-    <col min="10" max="11" width="10.83203125" style="1" customWidth="1"/>
-    <col min="12" max="12" width="3.83203125" style="1" customWidth="1"/>
-    <col min="13" max="14" width="10.83203125" style="1" customWidth="1"/>
-    <col min="15" max="15" width="3.83203125" customWidth="1"/>
-    <col min="18" max="18" width="3.83203125" customWidth="1"/>
-    <col min="21" max="21" width="3.83203125" customWidth="1"/>
-    <col min="24" max="24" width="3.83203125" customWidth="1"/>
-    <col min="27" max="27" width="3.83203125" customWidth="1"/>
-    <col min="30" max="30" width="3.83203125" customWidth="1"/>
-    <col min="33" max="33" width="3.83203125" customWidth="1"/>
-    <col min="36" max="36" width="3.83203125" customWidth="1"/>
-    <col min="39" max="39" width="3.83203125" customWidth="1"/>
-    <col min="42" max="42" width="3.83203125" customWidth="1"/>
-  </cols>
-  <sheetData>
-    <row r="2" spans="1:44" x14ac:dyDescent="0.2">
-      <c r="A2" s="24" t="s">
-        <v>179</v>
-      </c>
-      <c r="G2" s="9" t="s">
-        <v>307</v>
-      </c>
-    </row>
-    <row r="4" spans="1:44" x14ac:dyDescent="0.2">
-      <c r="A4" s="55" t="s">
-        <v>180</v>
-      </c>
-      <c r="B4" s="52"/>
-      <c r="D4" s="55" t="s">
-        <v>181</v>
-      </c>
-      <c r="E4" s="52"/>
-      <c r="G4" s="55" t="s">
-        <v>182</v>
-      </c>
-      <c r="H4" s="52"/>
-      <c r="J4" s="55" t="s">
-        <v>183</v>
-      </c>
-      <c r="K4" s="52"/>
-      <c r="M4" s="55" t="s">
-        <v>184</v>
-      </c>
-      <c r="N4" s="52"/>
-      <c r="P4" s="55" t="s">
-        <v>185</v>
-      </c>
-      <c r="Q4" s="54"/>
-      <c r="R4" s="1"/>
-      <c r="S4" s="55" t="s">
-        <v>186</v>
-      </c>
-      <c r="T4" s="54"/>
-      <c r="U4" s="1"/>
-      <c r="V4" s="55" t="s">
-        <v>187</v>
-      </c>
-      <c r="W4" s="54"/>
-      <c r="X4" s="1"/>
-      <c r="Y4" s="55" t="s">
-        <v>188</v>
-      </c>
-      <c r="Z4" s="54"/>
-      <c r="AA4" s="1"/>
-      <c r="AB4" s="55" t="s">
-        <v>189</v>
-      </c>
-      <c r="AC4" s="54"/>
-      <c r="AE4" s="55" t="s">
-        <v>190</v>
-      </c>
-      <c r="AF4" s="54"/>
-      <c r="AG4" s="1"/>
-      <c r="AH4" s="55" t="s">
-        <v>191</v>
-      </c>
-      <c r="AI4" s="54"/>
-      <c r="AJ4" s="1"/>
-      <c r="AK4" s="55" t="s">
-        <v>192</v>
-      </c>
-      <c r="AL4" s="54"/>
-      <c r="AM4" s="1"/>
-      <c r="AN4" s="55" t="s">
-        <v>193</v>
-      </c>
-      <c r="AO4" s="54"/>
-      <c r="AP4" s="1"/>
-      <c r="AQ4" s="55" t="s">
-        <v>194</v>
-      </c>
-      <c r="AR4" s="54"/>
-    </row>
-    <row r="5" spans="1:44" x14ac:dyDescent="0.2">
-      <c r="A5" s="38" t="s">
-        <v>198</v>
-      </c>
-      <c r="B5" s="39" t="s">
-        <v>306</v>
-      </c>
-      <c r="D5" s="38" t="s">
-        <v>198</v>
-      </c>
-      <c r="E5" s="39" t="s">
-        <v>306</v>
-      </c>
-      <c r="G5" s="38" t="s">
-        <v>198</v>
-      </c>
-      <c r="H5" s="39" t="s">
-        <v>306</v>
-      </c>
-      <c r="J5" s="38" t="s">
-        <v>198</v>
-      </c>
-      <c r="K5" s="39" t="s">
-        <v>306</v>
-      </c>
-      <c r="M5" s="38" t="s">
-        <v>198</v>
-      </c>
-      <c r="N5" s="39" t="s">
-        <v>306</v>
-      </c>
-      <c r="P5" s="38" t="s">
-        <v>198</v>
-      </c>
-      <c r="Q5" s="39" t="s">
-        <v>306</v>
-      </c>
-      <c r="R5" s="1"/>
-      <c r="S5" s="38" t="s">
-        <v>198</v>
-      </c>
-      <c r="T5" s="39" t="s">
-        <v>306</v>
-      </c>
-      <c r="U5" s="1"/>
-      <c r="V5" s="38" t="s">
-        <v>198</v>
-      </c>
-      <c r="W5" s="39" t="s">
-        <v>306</v>
-      </c>
-      <c r="X5" s="1"/>
-      <c r="Y5" s="38" t="s">
-        <v>198</v>
-      </c>
-      <c r="Z5" s="39" t="s">
-        <v>306</v>
-      </c>
-      <c r="AA5" s="1"/>
-      <c r="AB5" s="38" t="s">
-        <v>198</v>
-      </c>
-      <c r="AC5" s="39" t="s">
-        <v>306</v>
-      </c>
-      <c r="AE5" s="38" t="s">
-        <v>198</v>
-      </c>
-      <c r="AF5" s="39" t="s">
-        <v>306</v>
-      </c>
-      <c r="AG5" s="1"/>
-      <c r="AH5" s="38" t="s">
-        <v>198</v>
-      </c>
-      <c r="AI5" s="39" t="s">
-        <v>306</v>
-      </c>
-      <c r="AJ5" s="1"/>
-      <c r="AK5" s="38" t="s">
-        <v>198</v>
-      </c>
-      <c r="AL5" s="39" t="s">
-        <v>306</v>
-      </c>
-      <c r="AM5" s="1"/>
-      <c r="AN5" s="38" t="s">
-        <v>198</v>
-      </c>
-      <c r="AO5" s="39" t="s">
-        <v>306</v>
-      </c>
-      <c r="AP5" s="1"/>
-      <c r="AQ5" s="38" t="s">
-        <v>198</v>
-      </c>
-      <c r="AR5" s="39" t="s">
-        <v>306</v>
-      </c>
-    </row>
-    <row r="6" spans="1:44" x14ac:dyDescent="0.2">
-      <c r="A6" s="38" t="s">
-        <v>176</v>
-      </c>
-      <c r="B6" s="39">
-        <v>1</v>
-      </c>
-      <c r="D6" s="38" t="s">
-        <v>176</v>
-      </c>
-      <c r="E6" s="39">
-        <v>2</v>
-      </c>
-      <c r="G6" s="38" t="s">
-        <v>176</v>
-      </c>
-      <c r="H6" s="39">
-        <v>3</v>
-      </c>
-      <c r="J6" s="38" t="s">
-        <v>176</v>
-      </c>
-      <c r="K6" s="39">
-        <v>4</v>
-      </c>
-      <c r="M6" s="38" t="s">
-        <v>176</v>
-      </c>
-      <c r="N6" s="39">
-        <v>5</v>
-      </c>
-      <c r="P6" s="38" t="s">
-        <v>176</v>
-      </c>
-      <c r="Q6" s="39">
-        <v>6</v>
-      </c>
-      <c r="R6" s="1"/>
-      <c r="S6" s="38" t="s">
-        <v>176</v>
-      </c>
-      <c r="T6" s="39">
-        <v>7</v>
-      </c>
-      <c r="U6" s="1"/>
-      <c r="V6" s="38" t="s">
-        <v>176</v>
-      </c>
-      <c r="W6" s="39">
-        <v>8</v>
-      </c>
-      <c r="X6" s="1"/>
-      <c r="Y6" s="38" t="s">
-        <v>176</v>
-      </c>
-      <c r="Z6" s="39">
-        <v>9</v>
-      </c>
-      <c r="AA6" s="1"/>
-      <c r="AB6" s="38" t="s">
-        <v>176</v>
-      </c>
-      <c r="AC6" s="39">
-        <v>10</v>
-      </c>
-      <c r="AE6" s="38" t="s">
-        <v>176</v>
-      </c>
-      <c r="AF6" s="39">
-        <v>11</v>
-      </c>
-      <c r="AG6" s="1"/>
-      <c r="AH6" s="38" t="s">
-        <v>176</v>
-      </c>
-      <c r="AI6" s="39">
-        <v>12</v>
-      </c>
-      <c r="AJ6" s="1"/>
-      <c r="AK6" s="38" t="s">
-        <v>176</v>
-      </c>
-      <c r="AL6" s="39">
-        <v>13</v>
-      </c>
-      <c r="AM6" s="1"/>
-      <c r="AN6" s="38" t="s">
-        <v>176</v>
-      </c>
-      <c r="AO6" s="39">
-        <v>14</v>
-      </c>
-      <c r="AP6" s="1"/>
-      <c r="AQ6" s="38" t="s">
-        <v>176</v>
-      </c>
-      <c r="AR6" s="39">
-        <v>15</v>
-      </c>
-    </row>
-    <row r="7" spans="1:44" x14ac:dyDescent="0.2">
-      <c r="A7" s="58" t="str">
-        <f>IF(OR(B5="",B5="material"),_xlfn.XLOOKUP(B6,mat!$A:$A, mat!$B:$B,"") &amp; "",B5)</f>
-        <v/>
-      </c>
-      <c r="B7" s="57"/>
-      <c r="D7" s="58" t="str">
-        <f>IF(OR(E5="",E5="material"),_xlfn.XLOOKUP(E6,mat!$A:$A, mat!$B:$B,"") &amp; "",E5)</f>
-        <v/>
-      </c>
-      <c r="E7" s="57"/>
-      <c r="G7" s="58" t="str">
-        <f>IF(OR(H5="",H5="material"),_xlfn.XLOOKUP(H6,mat!$A:$A, mat!$B:$B,"") &amp; "",H5)</f>
-        <v/>
-      </c>
-      <c r="H7" s="57"/>
-      <c r="J7" s="58" t="str">
-        <f>IF(OR(K5="",K5="material"),_xlfn.XLOOKUP(K6,mat!$A:$A, mat!$B:$B,"") &amp; "",K5)</f>
-        <v/>
-      </c>
-      <c r="K7" s="57"/>
-      <c r="M7" s="58" t="str">
-        <f>IF(OR(N5="",N5="material"),_xlfn.XLOOKUP(N6,mat!$A:$A, mat!$B:$B,"") &amp; "",N5)</f>
-        <v/>
-      </c>
-      <c r="N7" s="57"/>
-      <c r="P7" s="58" t="str">
-        <f>IF(OR(Q5="",Q5="material"),_xlfn.XLOOKUP(Q6,mat!$A:$A, mat!$B:$B,"") &amp; "",Q5)</f>
-        <v/>
-      </c>
-      <c r="Q7" s="57"/>
-      <c r="R7" s="1"/>
-      <c r="S7" s="58" t="str">
-        <f>IF(OR(T5="",T5="material"),_xlfn.XLOOKUP(T6,mat!$A:$A, mat!$B:$B,"") &amp; "",T5)</f>
-        <v/>
-      </c>
-      <c r="T7" s="57"/>
-      <c r="U7" s="1"/>
-      <c r="V7" s="58" t="str">
-        <f>IF(OR(W5="",W5="material"),_xlfn.XLOOKUP(W6,mat!$A:$A, mat!$B:$B,"") &amp; "",W5)</f>
-        <v/>
-      </c>
-      <c r="W7" s="57"/>
-      <c r="X7" s="1"/>
-      <c r="Y7" s="58" t="str">
-        <f>IF(OR(Z5="",Z5="material"),_xlfn.XLOOKUP(Z6,mat!$A:$A, mat!$B:$B,"") &amp; "",Z5)</f>
-        <v/>
-      </c>
-      <c r="Z7" s="57"/>
-      <c r="AA7" s="1"/>
-      <c r="AB7" s="58" t="str">
-        <f>IF(OR(AC5="",AC5="material"),_xlfn.XLOOKUP(AC6,mat!$A:$A, mat!$B:$B,"") &amp; "",AC5)</f>
-        <v/>
-      </c>
-      <c r="AC7" s="57"/>
-      <c r="AE7" s="58" t="str">
-        <f>IF(OR(AF5="",AF5="material"),_xlfn.XLOOKUP(AF6,mat!$A:$A, mat!$B:$B,"") &amp; "",AF5)</f>
-        <v/>
-      </c>
-      <c r="AF7" s="57"/>
-      <c r="AG7" s="1"/>
-      <c r="AH7" s="58" t="str">
-        <f>IF(OR(AI5="",AI5="material"),_xlfn.XLOOKUP(AI6,mat!$A:$A, mat!$B:$B,"") &amp; "",AI5)</f>
-        <v/>
-      </c>
-      <c r="AI7" s="57"/>
-      <c r="AJ7" s="1"/>
-      <c r="AK7" s="58" t="str">
-        <f>IF(OR(AL5="",AL5="material"),_xlfn.XLOOKUP(AL6,mat!$A:$A, mat!$B:$B,"") &amp; "",AL5)</f>
-        <v/>
-      </c>
-      <c r="AL7" s="57"/>
-      <c r="AM7" s="1"/>
-      <c r="AN7" s="58" t="str">
-        <f>IF(OR(AO5="",AO5="material"),_xlfn.XLOOKUP(AO6,mat!$A:$A, mat!$B:$B,"") &amp; "",AO5)</f>
-        <v/>
-      </c>
-      <c r="AO7" s="57"/>
-      <c r="AP7" s="1"/>
-      <c r="AQ7" s="58" t="str">
-        <f>IF(OR(AR5="",AR5="material"),_xlfn.XLOOKUP(AR6,mat!$A:$A, mat!$B:$B,"") &amp; "",AR5)</f>
-        <v/>
-      </c>
-      <c r="AR7" s="57"/>
-    </row>
-    <row r="8" spans="1:44" x14ac:dyDescent="0.2">
-      <c r="A8" s="38" t="s">
-        <v>304</v>
-      </c>
-      <c r="B8" s="39"/>
-      <c r="D8" s="38" t="s">
-        <v>304</v>
-      </c>
-      <c r="E8" s="39"/>
-      <c r="G8" s="38" t="s">
-        <v>304</v>
-      </c>
-      <c r="H8" s="39"/>
-      <c r="J8" s="38" t="s">
-        <v>304</v>
-      </c>
-      <c r="K8" s="39"/>
-      <c r="M8" s="38" t="s">
-        <v>304</v>
-      </c>
-      <c r="N8" s="39"/>
-      <c r="P8" s="38" t="s">
-        <v>304</v>
-      </c>
-      <c r="Q8" s="39"/>
-      <c r="R8" s="1"/>
-      <c r="S8" s="38" t="s">
-        <v>304</v>
-      </c>
-      <c r="T8" s="39"/>
-      <c r="U8" s="1"/>
-      <c r="V8" s="38" t="s">
-        <v>304</v>
-      </c>
-      <c r="W8" s="39"/>
-      <c r="X8" s="1"/>
-      <c r="Y8" s="38" t="s">
-        <v>304</v>
-      </c>
-      <c r="Z8" s="39"/>
-      <c r="AA8" s="1"/>
-      <c r="AB8" s="38" t="s">
-        <v>304</v>
-      </c>
-      <c r="AC8" s="39"/>
-      <c r="AE8" s="38" t="s">
-        <v>304</v>
-      </c>
-      <c r="AF8" s="39"/>
-      <c r="AG8" s="1"/>
-      <c r="AH8" s="38" t="s">
-        <v>304</v>
-      </c>
-      <c r="AI8" s="39"/>
-      <c r="AJ8" s="1"/>
-      <c r="AK8" s="38" t="s">
-        <v>304</v>
-      </c>
-      <c r="AL8" s="39"/>
-      <c r="AM8" s="1"/>
-      <c r="AN8" s="38" t="s">
-        <v>304</v>
-      </c>
-      <c r="AO8" s="39"/>
-      <c r="AP8" s="1"/>
-      <c r="AQ8" s="38" t="s">
-        <v>304</v>
-      </c>
-      <c r="AR8" s="39"/>
-    </row>
-    <row r="9" spans="1:44" x14ac:dyDescent="0.2">
-      <c r="A9" s="2" t="s">
-        <v>177</v>
-      </c>
-      <c r="B9" s="2" t="s">
-        <v>178</v>
-      </c>
-      <c r="D9" s="2" t="s">
-        <v>177</v>
-      </c>
-      <c r="E9" s="2" t="s">
-        <v>178</v>
-      </c>
-      <c r="G9" s="2" t="s">
-        <v>177</v>
-      </c>
-      <c r="H9" s="2" t="s">
-        <v>178</v>
-      </c>
-      <c r="J9" s="2" t="s">
-        <v>177</v>
-      </c>
-      <c r="K9" s="2" t="s">
-        <v>178</v>
-      </c>
-      <c r="M9" s="2" t="s">
-        <v>177</v>
-      </c>
-      <c r="N9" s="2" t="s">
-        <v>178</v>
-      </c>
-      <c r="P9" s="2" t="s">
-        <v>177</v>
-      </c>
-      <c r="Q9" s="2" t="s">
-        <v>178</v>
-      </c>
-      <c r="R9" s="1"/>
-      <c r="S9" s="2" t="s">
-        <v>177</v>
-      </c>
-      <c r="T9" s="2" t="s">
-        <v>178</v>
-      </c>
-      <c r="U9" s="1"/>
-      <c r="V9" s="2" t="s">
-        <v>177</v>
-      </c>
-      <c r="W9" s="2" t="s">
-        <v>178</v>
-      </c>
-      <c r="X9" s="1"/>
-      <c r="Y9" s="2" t="s">
-        <v>177</v>
-      </c>
-      <c r="Z9" s="2" t="s">
-        <v>178</v>
-      </c>
-      <c r="AA9" s="1"/>
-      <c r="AB9" s="2" t="s">
-        <v>177</v>
-      </c>
-      <c r="AC9" s="2" t="s">
-        <v>178</v>
-      </c>
-      <c r="AE9" s="2" t="s">
-        <v>177</v>
-      </c>
-      <c r="AF9" s="2" t="s">
-        <v>178</v>
-      </c>
-      <c r="AG9" s="1"/>
-      <c r="AH9" s="2" t="s">
-        <v>177</v>
-      </c>
-      <c r="AI9" s="2" t="s">
-        <v>178</v>
-      </c>
-      <c r="AJ9" s="1"/>
-      <c r="AK9" s="2" t="s">
-        <v>177</v>
-      </c>
-      <c r="AL9" s="2" t="s">
-        <v>178</v>
-      </c>
-      <c r="AM9" s="1"/>
-      <c r="AN9" s="2" t="s">
-        <v>177</v>
-      </c>
-      <c r="AO9" s="2" t="s">
-        <v>178</v>
-      </c>
-      <c r="AP9" s="1"/>
-      <c r="AQ9" s="2" t="s">
-        <v>177</v>
-      </c>
-      <c r="AR9" s="2" t="s">
-        <v>178</v>
-      </c>
-    </row>
-    <row r="10" spans="1:44" x14ac:dyDescent="0.2">
-      <c r="A10" s="3"/>
-      <c r="B10" s="3"/>
-      <c r="D10" s="3"/>
-      <c r="E10" s="3"/>
-      <c r="G10" s="3"/>
-      <c r="H10" s="3"/>
-      <c r="J10" s="3"/>
-      <c r="K10" s="3"/>
-      <c r="M10" s="3"/>
-      <c r="N10" s="3"/>
-      <c r="P10" s="3"/>
-      <c r="Q10" s="3"/>
-      <c r="R10" s="1"/>
-      <c r="S10" s="3"/>
-      <c r="T10" s="3"/>
-      <c r="U10" s="1"/>
-      <c r="V10" s="3"/>
-      <c r="W10" s="3"/>
-      <c r="X10" s="1"/>
-      <c r="Y10" s="3"/>
-      <c r="Z10" s="3"/>
-      <c r="AA10" s="1"/>
-      <c r="AB10" s="3"/>
-      <c r="AC10" s="3"/>
-      <c r="AE10" s="3"/>
-      <c r="AF10" s="3"/>
-      <c r="AG10" s="1"/>
-      <c r="AH10" s="3"/>
-      <c r="AI10" s="3"/>
-      <c r="AJ10" s="1"/>
-      <c r="AK10" s="3"/>
-      <c r="AL10" s="3"/>
-      <c r="AM10" s="1"/>
-      <c r="AN10" s="3"/>
-      <c r="AO10" s="3"/>
-      <c r="AP10" s="1"/>
-      <c r="AQ10" s="3"/>
-      <c r="AR10" s="3"/>
-    </row>
-    <row r="11" spans="1:44" x14ac:dyDescent="0.2">
-      <c r="A11" s="3"/>
-      <c r="B11" s="3"/>
-      <c r="D11" s="3"/>
-      <c r="E11" s="3"/>
-      <c r="G11" s="3"/>
-      <c r="H11" s="3"/>
-      <c r="J11" s="3"/>
-      <c r="K11" s="3"/>
-      <c r="M11" s="3"/>
-      <c r="N11" s="3"/>
-      <c r="P11" s="3"/>
-      <c r="Q11" s="3"/>
-      <c r="R11" s="1"/>
-      <c r="S11" s="3"/>
-      <c r="T11" s="3"/>
-      <c r="U11" s="1"/>
-      <c r="V11" s="3"/>
-      <c r="W11" s="3"/>
-      <c r="X11" s="1"/>
-      <c r="Y11" s="3"/>
-      <c r="Z11" s="3"/>
-      <c r="AA11" s="1"/>
-      <c r="AB11" s="3"/>
-      <c r="AC11" s="3"/>
-      <c r="AE11" s="3"/>
-      <c r="AF11" s="3"/>
-      <c r="AG11" s="1"/>
-      <c r="AH11" s="3"/>
-      <c r="AI11" s="3"/>
-      <c r="AJ11" s="1"/>
-      <c r="AK11" s="3"/>
-      <c r="AL11" s="3"/>
-      <c r="AM11" s="1"/>
-      <c r="AN11" s="3"/>
-      <c r="AO11" s="3"/>
-      <c r="AP11" s="1"/>
-      <c r="AQ11" s="3"/>
-      <c r="AR11" s="3"/>
-    </row>
-    <row r="12" spans="1:44" x14ac:dyDescent="0.2">
-      <c r="A12" s="3"/>
-      <c r="B12" s="3"/>
-      <c r="D12" s="3"/>
-      <c r="E12" s="3"/>
-      <c r="G12" s="3"/>
-      <c r="H12" s="3"/>
-      <c r="J12" s="3"/>
-      <c r="K12" s="3"/>
-      <c r="M12" s="3"/>
-      <c r="N12" s="3"/>
-      <c r="P12" s="3"/>
-      <c r="Q12" s="3"/>
-      <c r="R12" s="1"/>
-      <c r="S12" s="3"/>
-      <c r="T12" s="3"/>
-      <c r="U12" s="1"/>
-      <c r="V12" s="3"/>
-      <c r="W12" s="3"/>
-      <c r="X12" s="1"/>
-      <c r="Y12" s="3"/>
-      <c r="Z12" s="3"/>
-      <c r="AA12" s="1"/>
-      <c r="AB12" s="3"/>
-      <c r="AC12" s="3"/>
-      <c r="AE12" s="3"/>
-      <c r="AF12" s="3"/>
-      <c r="AG12" s="1"/>
-      <c r="AH12" s="3"/>
-      <c r="AI12" s="3"/>
-      <c r="AJ12" s="1"/>
-      <c r="AK12" s="3"/>
-      <c r="AL12" s="3"/>
-      <c r="AM12" s="1"/>
-      <c r="AN12" s="3"/>
-      <c r="AO12" s="3"/>
-      <c r="AP12" s="1"/>
-      <c r="AQ12" s="3"/>
-      <c r="AR12" s="3"/>
-    </row>
-    <row r="13" spans="1:44" x14ac:dyDescent="0.2">
-      <c r="A13" s="3"/>
-      <c r="B13" s="3"/>
-      <c r="D13" s="3"/>
-      <c r="E13" s="3"/>
-      <c r="G13" s="3"/>
-      <c r="H13" s="3"/>
-      <c r="J13" s="3"/>
-      <c r="K13" s="3"/>
-      <c r="M13" s="3"/>
-      <c r="N13" s="3"/>
-      <c r="P13" s="3"/>
-      <c r="Q13" s="3"/>
-      <c r="R13" s="1"/>
-      <c r="S13" s="3"/>
-      <c r="T13" s="3"/>
-      <c r="U13" s="1"/>
-      <c r="V13" s="3"/>
-      <c r="W13" s="3"/>
-      <c r="X13" s="1"/>
-      <c r="Y13" s="3"/>
-      <c r="Z13" s="3"/>
-      <c r="AA13" s="1"/>
-      <c r="AB13" s="3"/>
-      <c r="AC13" s="3"/>
-      <c r="AE13" s="3"/>
-      <c r="AF13" s="3"/>
-      <c r="AG13" s="1"/>
-      <c r="AH13" s="3"/>
-      <c r="AI13" s="3"/>
-      <c r="AJ13" s="1"/>
-      <c r="AK13" s="3"/>
-      <c r="AL13" s="3"/>
-      <c r="AM13" s="1"/>
-      <c r="AN13" s="3"/>
-      <c r="AO13" s="3"/>
-      <c r="AP13" s="1"/>
-      <c r="AQ13" s="3"/>
-      <c r="AR13" s="3"/>
-    </row>
-    <row r="14" spans="1:44" x14ac:dyDescent="0.2">
-      <c r="A14" s="3"/>
-      <c r="B14" s="3"/>
-      <c r="D14" s="3"/>
-      <c r="E14" s="3"/>
-      <c r="G14" s="3"/>
-      <c r="H14" s="3"/>
-      <c r="J14" s="3"/>
-      <c r="K14" s="3"/>
-      <c r="M14" s="3"/>
-      <c r="N14" s="3"/>
-      <c r="P14" s="3"/>
-      <c r="Q14" s="3"/>
-      <c r="R14" s="1"/>
-      <c r="S14" s="3"/>
-      <c r="T14" s="3"/>
-      <c r="U14" s="1"/>
-      <c r="V14" s="3"/>
-      <c r="W14" s="3"/>
-      <c r="X14" s="1"/>
-      <c r="Y14" s="3"/>
-      <c r="Z14" s="3"/>
-      <c r="AA14" s="1"/>
-      <c r="AB14" s="3"/>
-      <c r="AC14" s="3"/>
-      <c r="AE14" s="3"/>
-      <c r="AF14" s="3"/>
-      <c r="AG14" s="1"/>
-      <c r="AH14" s="3"/>
-      <c r="AI14" s="3"/>
-      <c r="AJ14" s="1"/>
-      <c r="AK14" s="3"/>
-      <c r="AL14" s="3"/>
-      <c r="AM14" s="1"/>
-      <c r="AN14" s="3"/>
-      <c r="AO14" s="3"/>
-      <c r="AP14" s="1"/>
-      <c r="AQ14" s="3"/>
-      <c r="AR14" s="3"/>
-    </row>
-    <row r="15" spans="1:44" x14ac:dyDescent="0.2">
-      <c r="A15" s="3"/>
-      <c r="B15" s="3"/>
-      <c r="D15" s="3"/>
-      <c r="E15" s="3"/>
-      <c r="G15" s="3"/>
-      <c r="H15" s="3"/>
-      <c r="J15" s="3"/>
-      <c r="K15" s="3"/>
-      <c r="M15" s="3"/>
-      <c r="N15" s="3"/>
-      <c r="P15" s="3"/>
-      <c r="Q15" s="3"/>
-      <c r="R15" s="1"/>
-      <c r="S15" s="3"/>
-      <c r="T15" s="3"/>
-      <c r="U15" s="1"/>
-      <c r="V15" s="3"/>
-      <c r="W15" s="3"/>
-      <c r="X15" s="1"/>
-      <c r="Y15" s="3"/>
-      <c r="Z15" s="3"/>
-      <c r="AA15" s="1"/>
-      <c r="AB15" s="3"/>
-      <c r="AC15" s="3"/>
-      <c r="AE15" s="3"/>
-      <c r="AF15" s="3"/>
-      <c r="AG15" s="1"/>
-      <c r="AH15" s="3"/>
-      <c r="AI15" s="3"/>
-      <c r="AJ15" s="1"/>
-      <c r="AK15" s="3"/>
-      <c r="AL15" s="3"/>
-      <c r="AM15" s="1"/>
-      <c r="AN15" s="3"/>
-      <c r="AO15" s="3"/>
-      <c r="AP15" s="1"/>
-      <c r="AQ15" s="3"/>
-      <c r="AR15" s="3"/>
-    </row>
-    <row r="16" spans="1:44" x14ac:dyDescent="0.2">
-      <c r="A16" s="3"/>
-      <c r="B16" s="3"/>
-      <c r="D16" s="3"/>
-      <c r="E16" s="3"/>
-      <c r="G16" s="3"/>
-      <c r="H16" s="3"/>
-      <c r="J16" s="3"/>
-      <c r="K16" s="3"/>
-      <c r="M16" s="3"/>
-      <c r="N16" s="3"/>
-      <c r="P16" s="3"/>
-      <c r="Q16" s="3"/>
-      <c r="R16" s="1"/>
-      <c r="S16" s="3"/>
-      <c r="T16" s="3"/>
-      <c r="U16" s="1"/>
-      <c r="V16" s="3"/>
-      <c r="W16" s="3"/>
-      <c r="X16" s="1"/>
-      <c r="Y16" s="3"/>
-      <c r="Z16" s="3"/>
-      <c r="AA16" s="1"/>
-      <c r="AB16" s="3"/>
-      <c r="AC16" s="3"/>
-      <c r="AE16" s="3"/>
-      <c r="AF16" s="3"/>
-      <c r="AG16" s="1"/>
-      <c r="AH16" s="3"/>
-      <c r="AI16" s="3"/>
-      <c r="AJ16" s="1"/>
-      <c r="AK16" s="3"/>
-      <c r="AL16" s="3"/>
-      <c r="AM16" s="1"/>
-      <c r="AN16" s="3"/>
-      <c r="AO16" s="3"/>
-      <c r="AP16" s="1"/>
-      <c r="AQ16" s="3"/>
-      <c r="AR16" s="3"/>
-    </row>
-    <row r="17" spans="1:44" x14ac:dyDescent="0.2">
-      <c r="A17" s="3"/>
-      <c r="B17" s="3"/>
-      <c r="D17" s="3"/>
-      <c r="E17" s="3"/>
-      <c r="G17" s="3"/>
-      <c r="H17" s="3"/>
-      <c r="J17" s="3"/>
-      <c r="K17" s="3"/>
-      <c r="M17" s="3"/>
-      <c r="N17" s="3"/>
-      <c r="P17" s="3"/>
-      <c r="Q17" s="3"/>
-      <c r="R17" s="1"/>
-      <c r="S17" s="3"/>
-      <c r="T17" s="3"/>
-      <c r="U17" s="1"/>
-      <c r="V17" s="3"/>
-      <c r="W17" s="3"/>
-      <c r="X17" s="1"/>
-      <c r="Y17" s="3"/>
-      <c r="Z17" s="3"/>
-      <c r="AA17" s="1"/>
-      <c r="AB17" s="3"/>
-      <c r="AC17" s="3"/>
-      <c r="AE17" s="3"/>
-      <c r="AF17" s="3"/>
-      <c r="AG17" s="1"/>
-      <c r="AH17" s="3"/>
-      <c r="AI17" s="3"/>
-      <c r="AJ17" s="1"/>
-      <c r="AK17" s="3"/>
-      <c r="AL17" s="3"/>
-      <c r="AM17" s="1"/>
-      <c r="AN17" s="3"/>
-      <c r="AO17" s="3"/>
-      <c r="AP17" s="1"/>
-      <c r="AQ17" s="3"/>
-      <c r="AR17" s="3"/>
-    </row>
-    <row r="18" spans="1:44" x14ac:dyDescent="0.2">
-      <c r="A18" s="3"/>
-      <c r="B18" s="3"/>
-      <c r="D18" s="3"/>
-      <c r="E18" s="3"/>
-      <c r="G18" s="3"/>
-      <c r="H18" s="3"/>
-      <c r="J18" s="3"/>
-      <c r="K18" s="3"/>
-      <c r="M18" s="3"/>
-      <c r="N18" s="3"/>
-      <c r="P18" s="3"/>
-      <c r="Q18" s="3"/>
-      <c r="R18" s="1"/>
-      <c r="S18" s="3"/>
-      <c r="T18" s="3"/>
-      <c r="U18" s="1"/>
-      <c r="V18" s="3"/>
-      <c r="W18" s="3"/>
-      <c r="X18" s="1"/>
-      <c r="Y18" s="3"/>
-      <c r="Z18" s="3"/>
-      <c r="AA18" s="1"/>
-      <c r="AB18" s="3"/>
-      <c r="AC18" s="3"/>
-      <c r="AE18" s="3"/>
-      <c r="AF18" s="3"/>
-      <c r="AG18" s="1"/>
-      <c r="AH18" s="3"/>
-      <c r="AI18" s="3"/>
-      <c r="AJ18" s="1"/>
-      <c r="AK18" s="3"/>
-      <c r="AL18" s="3"/>
-      <c r="AM18" s="1"/>
-      <c r="AN18" s="3"/>
-      <c r="AO18" s="3"/>
-      <c r="AP18" s="1"/>
-      <c r="AQ18" s="3"/>
-      <c r="AR18" s="3"/>
-    </row>
-    <row r="19" spans="1:44" x14ac:dyDescent="0.2">
-      <c r="A19" s="3"/>
-      <c r="B19" s="3"/>
-      <c r="D19" s="3"/>
-      <c r="E19" s="3"/>
-      <c r="G19" s="3"/>
-      <c r="H19" s="3"/>
-      <c r="J19" s="3"/>
-      <c r="K19" s="3"/>
-      <c r="M19" s="3"/>
-      <c r="N19" s="3"/>
-      <c r="P19" s="3"/>
-      <c r="Q19" s="3"/>
-      <c r="R19" s="1"/>
-      <c r="S19" s="3"/>
-      <c r="T19" s="3"/>
-      <c r="U19" s="1"/>
-      <c r="V19" s="3"/>
-      <c r="W19" s="3"/>
-      <c r="X19" s="1"/>
-      <c r="Y19" s="3"/>
-      <c r="Z19" s="3"/>
-      <c r="AA19" s="1"/>
-      <c r="AB19" s="3"/>
-      <c r="AC19" s="3"/>
-      <c r="AE19" s="3"/>
-      <c r="AF19" s="3"/>
-      <c r="AG19" s="1"/>
-      <c r="AH19" s="3"/>
-      <c r="AI19" s="3"/>
-      <c r="AJ19" s="1"/>
-      <c r="AK19" s="3"/>
-      <c r="AL19" s="3"/>
-      <c r="AM19" s="1"/>
-      <c r="AN19" s="3"/>
-      <c r="AO19" s="3"/>
-      <c r="AP19" s="1"/>
-      <c r="AQ19" s="3"/>
-      <c r="AR19" s="3"/>
-    </row>
-    <row r="20" spans="1:44" x14ac:dyDescent="0.2">
-      <c r="A20" s="3"/>
-      <c r="B20" s="3"/>
-      <c r="D20" s="3"/>
-      <c r="E20" s="3"/>
-      <c r="G20" s="3"/>
-      <c r="H20" s="3"/>
-      <c r="J20" s="3"/>
-      <c r="K20" s="3"/>
-      <c r="M20" s="3"/>
-      <c r="N20" s="3"/>
-      <c r="P20" s="3"/>
-      <c r="Q20" s="3"/>
-      <c r="R20" s="1"/>
-      <c r="S20" s="3"/>
-      <c r="T20" s="3"/>
-      <c r="U20" s="1"/>
-      <c r="V20" s="3"/>
-      <c r="W20" s="3"/>
-      <c r="X20" s="1"/>
-      <c r="Y20" s="3"/>
-      <c r="Z20" s="3"/>
-      <c r="AA20" s="1"/>
-      <c r="AB20" s="3"/>
-      <c r="AC20" s="3"/>
-      <c r="AE20" s="3"/>
-      <c r="AF20" s="3"/>
-      <c r="AG20" s="1"/>
-      <c r="AH20" s="3"/>
-      <c r="AI20" s="3"/>
-      <c r="AJ20" s="1"/>
-      <c r="AK20" s="3"/>
-      <c r="AL20" s="3"/>
-      <c r="AM20" s="1"/>
-      <c r="AN20" s="3"/>
-      <c r="AO20" s="3"/>
-      <c r="AP20" s="1"/>
-      <c r="AQ20" s="3"/>
-      <c r="AR20" s="3"/>
-    </row>
-    <row r="21" spans="1:44" x14ac:dyDescent="0.2">
-      <c r="A21" s="3"/>
-      <c r="B21" s="3"/>
-      <c r="D21" s="3"/>
-      <c r="E21" s="3"/>
-      <c r="G21" s="3"/>
-      <c r="H21" s="3"/>
-      <c r="J21" s="3"/>
-      <c r="K21" s="3"/>
-      <c r="M21" s="3"/>
-      <c r="N21" s="3"/>
-      <c r="P21" s="3"/>
-      <c r="Q21" s="3"/>
-      <c r="R21" s="1"/>
-      <c r="S21" s="3"/>
-      <c r="T21" s="3"/>
-      <c r="U21" s="1"/>
-      <c r="V21" s="3"/>
-      <c r="W21" s="3"/>
-      <c r="X21" s="1"/>
-      <c r="Y21" s="3"/>
-      <c r="Z21" s="3"/>
-      <c r="AA21" s="1"/>
-      <c r="AB21" s="3"/>
-      <c r="AC21" s="3"/>
-      <c r="AE21" s="3"/>
-      <c r="AF21" s="3"/>
-      <c r="AG21" s="1"/>
-      <c r="AH21" s="3"/>
-      <c r="AI21" s="3"/>
-      <c r="AJ21" s="1"/>
-      <c r="AK21" s="3"/>
-      <c r="AL21" s="3"/>
-      <c r="AM21" s="1"/>
-      <c r="AN21" s="3"/>
-      <c r="AO21" s="3"/>
-      <c r="AP21" s="1"/>
-      <c r="AQ21" s="3"/>
-      <c r="AR21" s="3"/>
-    </row>
-    <row r="22" spans="1:44" x14ac:dyDescent="0.2">
-      <c r="A22" s="3"/>
-      <c r="B22" s="3"/>
-      <c r="D22" s="3"/>
-      <c r="E22" s="3"/>
-      <c r="G22" s="3"/>
-      <c r="H22" s="3"/>
-      <c r="J22" s="3"/>
-      <c r="K22" s="3"/>
-      <c r="M22" s="3"/>
-      <c r="N22" s="3"/>
-      <c r="P22" s="3"/>
-      <c r="Q22" s="3"/>
-      <c r="R22" s="1"/>
-      <c r="S22" s="3"/>
-      <c r="T22" s="3"/>
-      <c r="U22" s="1"/>
-      <c r="V22" s="3"/>
-      <c r="W22" s="3"/>
-      <c r="X22" s="1"/>
-      <c r="Y22" s="3"/>
-      <c r="Z22" s="3"/>
-      <c r="AA22" s="1"/>
-      <c r="AB22" s="3"/>
-      <c r="AC22" s="3"/>
-      <c r="AE22" s="3"/>
-      <c r="AF22" s="3"/>
-      <c r="AG22" s="1"/>
-      <c r="AH22" s="3"/>
-      <c r="AI22" s="3"/>
-      <c r="AJ22" s="1"/>
-      <c r="AK22" s="3"/>
-      <c r="AL22" s="3"/>
-      <c r="AM22" s="1"/>
-      <c r="AN22" s="3"/>
-      <c r="AO22" s="3"/>
-      <c r="AP22" s="1"/>
-      <c r="AQ22" s="3"/>
-      <c r="AR22" s="3"/>
-    </row>
-    <row r="23" spans="1:44" x14ac:dyDescent="0.2">
-      <c r="A23" s="3"/>
-      <c r="B23" s="3"/>
-      <c r="D23" s="3"/>
-      <c r="E23" s="3"/>
-      <c r="G23" s="3"/>
-      <c r="H23" s="3"/>
-      <c r="J23" s="3"/>
-      <c r="K23" s="3"/>
-      <c r="M23" s="3"/>
-      <c r="N23" s="3"/>
-      <c r="P23" s="3"/>
-      <c r="Q23" s="3"/>
-      <c r="R23" s="1"/>
-      <c r="S23" s="3"/>
-      <c r="T23" s="3"/>
-      <c r="U23" s="1"/>
-      <c r="V23" s="3"/>
-      <c r="W23" s="3"/>
-      <c r="X23" s="1"/>
-      <c r="Y23" s="3"/>
-      <c r="Z23" s="3"/>
-      <c r="AA23" s="1"/>
-      <c r="AB23" s="3"/>
-      <c r="AC23" s="3"/>
-      <c r="AE23" s="3"/>
-      <c r="AF23" s="3"/>
-      <c r="AG23" s="1"/>
-      <c r="AH23" s="3"/>
-      <c r="AI23" s="3"/>
-      <c r="AJ23" s="1"/>
-      <c r="AK23" s="3"/>
-      <c r="AL23" s="3"/>
-      <c r="AM23" s="1"/>
-      <c r="AN23" s="3"/>
-      <c r="AO23" s="3"/>
-      <c r="AP23" s="1"/>
-      <c r="AQ23" s="3"/>
-      <c r="AR23" s="3"/>
-    </row>
-    <row r="24" spans="1:44" x14ac:dyDescent="0.2">
-      <c r="A24" s="3"/>
-      <c r="B24" s="3"/>
-      <c r="D24" s="3"/>
-      <c r="E24" s="3"/>
-      <c r="G24" s="3"/>
-      <c r="H24" s="3"/>
-      <c r="J24" s="3"/>
-      <c r="K24" s="3"/>
-      <c r="M24" s="3"/>
-      <c r="N24" s="3"/>
-      <c r="P24" s="3"/>
-      <c r="Q24" s="3"/>
-      <c r="R24" s="1"/>
-      <c r="S24" s="3"/>
-      <c r="T24" s="3"/>
-      <c r="U24" s="1"/>
-      <c r="V24" s="3"/>
-      <c r="W24" s="3"/>
-      <c r="X24" s="1"/>
-      <c r="Y24" s="3"/>
-      <c r="Z24" s="3"/>
-      <c r="AA24" s="1"/>
-      <c r="AB24" s="3"/>
-      <c r="AC24" s="3"/>
-      <c r="AE24" s="3"/>
-      <c r="AF24" s="3"/>
-      <c r="AG24" s="1"/>
-      <c r="AH24" s="3"/>
-      <c r="AI24" s="3"/>
-      <c r="AJ24" s="1"/>
-      <c r="AK24" s="3"/>
-      <c r="AL24" s="3"/>
-      <c r="AM24" s="1"/>
-      <c r="AN24" s="3"/>
-      <c r="AO24" s="3"/>
-      <c r="AP24" s="1"/>
-      <c r="AQ24" s="3"/>
-      <c r="AR24" s="3"/>
-    </row>
-    <row r="25" spans="1:44" x14ac:dyDescent="0.2">
-      <c r="A25" s="3"/>
-      <c r="B25" s="3"/>
-      <c r="D25" s="3"/>
-      <c r="E25" s="3"/>
-      <c r="G25" s="3"/>
-      <c r="H25" s="3"/>
-      <c r="J25" s="3"/>
-      <c r="K25" s="3"/>
-      <c r="M25" s="3"/>
-      <c r="N25" s="3"/>
-      <c r="P25" s="3"/>
-      <c r="Q25" s="3"/>
-      <c r="R25" s="1"/>
-      <c r="S25" s="3"/>
-      <c r="T25" s="3"/>
-      <c r="U25" s="1"/>
-      <c r="V25" s="3"/>
-      <c r="W25" s="3"/>
-      <c r="X25" s="1"/>
-      <c r="Y25" s="3"/>
-      <c r="Z25" s="3"/>
-      <c r="AA25" s="1"/>
-      <c r="AB25" s="3"/>
-      <c r="AC25" s="3"/>
-      <c r="AE25" s="3"/>
-      <c r="AF25" s="3"/>
-      <c r="AG25" s="1"/>
-      <c r="AH25" s="3"/>
-      <c r="AI25" s="3"/>
-      <c r="AJ25" s="1"/>
-      <c r="AK25" s="3"/>
-      <c r="AL25" s="3"/>
-      <c r="AM25" s="1"/>
-      <c r="AN25" s="3"/>
-      <c r="AO25" s="3"/>
-      <c r="AP25" s="1"/>
-      <c r="AQ25" s="3"/>
-      <c r="AR25" s="3"/>
-    </row>
-    <row r="26" spans="1:44" x14ac:dyDescent="0.2">
-      <c r="A26" s="3"/>
-      <c r="B26" s="3"/>
-      <c r="D26" s="3"/>
-      <c r="E26" s="3"/>
-      <c r="G26" s="3"/>
-      <c r="H26" s="3"/>
-      <c r="J26" s="3"/>
-      <c r="K26" s="3"/>
-      <c r="M26" s="3"/>
-      <c r="N26" s="3"/>
-      <c r="P26" s="3"/>
-      <c r="Q26" s="3"/>
-      <c r="R26" s="1"/>
-      <c r="S26" s="3"/>
-      <c r="T26" s="3"/>
-      <c r="U26" s="1"/>
-      <c r="V26" s="3"/>
-      <c r="W26" s="3"/>
-      <c r="X26" s="1"/>
-      <c r="Y26" s="3"/>
-      <c r="Z26" s="3"/>
-      <c r="AA26" s="1"/>
-      <c r="AB26" s="3"/>
-      <c r="AC26" s="3"/>
-      <c r="AE26" s="3"/>
-      <c r="AF26" s="3"/>
-      <c r="AG26" s="1"/>
-      <c r="AH26" s="3"/>
-      <c r="AI26" s="3"/>
-      <c r="AJ26" s="1"/>
-      <c r="AK26" s="3"/>
-      <c r="AL26" s="3"/>
-      <c r="AM26" s="1"/>
-      <c r="AN26" s="3"/>
-      <c r="AO26" s="3"/>
-      <c r="AP26" s="1"/>
-      <c r="AQ26" s="3"/>
-      <c r="AR26" s="3"/>
-    </row>
-    <row r="27" spans="1:44" x14ac:dyDescent="0.2">
-      <c r="A27" s="3"/>
-      <c r="B27" s="3"/>
-      <c r="D27" s="3"/>
-      <c r="E27" s="3"/>
-      <c r="G27" s="3"/>
-      <c r="H27" s="3"/>
-      <c r="J27" s="3"/>
-      <c r="K27" s="3"/>
-      <c r="M27" s="3"/>
-      <c r="N27" s="3"/>
-      <c r="P27" s="3"/>
-      <c r="Q27" s="3"/>
-      <c r="R27" s="1"/>
-      <c r="S27" s="3"/>
-      <c r="T27" s="3"/>
-      <c r="U27" s="1"/>
-      <c r="V27" s="3"/>
-      <c r="W27" s="3"/>
-      <c r="X27" s="1"/>
-      <c r="Y27" s="3"/>
-      <c r="Z27" s="3"/>
-      <c r="AA27" s="1"/>
-      <c r="AB27" s="3"/>
-      <c r="AC27" s="3"/>
-      <c r="AE27" s="3"/>
-      <c r="AF27" s="3"/>
-      <c r="AG27" s="1"/>
-      <c r="AH27" s="3"/>
-      <c r="AI27" s="3"/>
-      <c r="AJ27" s="1"/>
-      <c r="AK27" s="3"/>
-      <c r="AL27" s="3"/>
-      <c r="AM27" s="1"/>
-      <c r="AN27" s="3"/>
-      <c r="AO27" s="3"/>
-      <c r="AP27" s="1"/>
-      <c r="AQ27" s="3"/>
-      <c r="AR27" s="3"/>
-    </row>
     <row r="28" spans="1:44" x14ac:dyDescent="0.2">
       <c r="A28" s="3"/>
       <c r="B28" s="3"/>
@@ -17289,20 +17484,6 @@
     </row>
   </sheetData>
   <mergeCells count="30">
-    <mergeCell ref="D4:E4"/>
-    <mergeCell ref="P4:Q4"/>
-    <mergeCell ref="Y4:Z4"/>
-    <mergeCell ref="AB7:AC7"/>
-    <mergeCell ref="AN7:AO7"/>
-    <mergeCell ref="AB4:AC4"/>
-    <mergeCell ref="AN4:AO4"/>
-    <mergeCell ref="G7:H7"/>
-    <mergeCell ref="J4:K4"/>
-    <mergeCell ref="V7:W7"/>
-    <mergeCell ref="M7:N7"/>
-    <mergeCell ref="AH7:AI7"/>
-    <mergeCell ref="S7:T7"/>
-    <mergeCell ref="Y7:Z7"/>
     <mergeCell ref="AQ4:AR4"/>
     <mergeCell ref="A4:B4"/>
     <mergeCell ref="G4:H4"/>
@@ -17319,84 +17500,98 @@
     <mergeCell ref="AH4:AI4"/>
     <mergeCell ref="J7:K7"/>
     <mergeCell ref="P7:Q7"/>
+    <mergeCell ref="D4:E4"/>
+    <mergeCell ref="P4:Q4"/>
+    <mergeCell ref="Y4:Z4"/>
+    <mergeCell ref="AB7:AC7"/>
+    <mergeCell ref="AN7:AO7"/>
+    <mergeCell ref="AB4:AC4"/>
+    <mergeCell ref="AN4:AO4"/>
+    <mergeCell ref="G7:H7"/>
+    <mergeCell ref="J4:K4"/>
+    <mergeCell ref="V7:W7"/>
+    <mergeCell ref="M7:N7"/>
+    <mergeCell ref="AH7:AI7"/>
+    <mergeCell ref="S7:T7"/>
+    <mergeCell ref="Y7:Z7"/>
   </mergeCells>
   <conditionalFormatting sqref="B6 A7:B7">
-    <cfRule type="expression" dxfId="0" priority="1">
+    <cfRule type="expression" dxfId="17" priority="1">
       <formula>AND($B$5&lt;&gt;"",$B$5&lt;&gt;"material")</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="E6 D7:E7">
-    <cfRule type="expression" dxfId="0" priority="2">
+    <cfRule type="expression" dxfId="16" priority="2">
       <formula>AND($E$5&lt;&gt;"",$E$5&lt;&gt;"material")</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="H6 G7:H7">
-    <cfRule type="expression" dxfId="0" priority="3">
+    <cfRule type="expression" dxfId="15" priority="3">
       <formula>AND($H$5&lt;&gt;"",$H$5&lt;&gt;"material")</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="K6 J7:K7">
-    <cfRule type="expression" dxfId="0" priority="4">
+    <cfRule type="expression" dxfId="14" priority="4">
       <formula>AND($K$5&lt;&gt;"",$K$5&lt;&gt;"material")</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="N6 M7:N7">
-    <cfRule type="expression" dxfId="0" priority="5">
+    <cfRule type="expression" dxfId="13" priority="5">
       <formula>AND($N$5&lt;&gt;"",$N$5&lt;&gt;"material")</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="Q6 P7:Q7">
-    <cfRule type="expression" dxfId="0" priority="6">
+    <cfRule type="expression" dxfId="12" priority="6">
       <formula>AND($Q$5&lt;&gt;"",$Q$5&lt;&gt;"material")</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="T6 S7:T7">
-    <cfRule type="expression" dxfId="0" priority="7">
+    <cfRule type="expression" dxfId="11" priority="7">
       <formula>AND($T$5&lt;&gt;"",$T$5&lt;&gt;"material")</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="W6 V7:W7">
-    <cfRule type="expression" dxfId="0" priority="8">
+    <cfRule type="expression" dxfId="10" priority="8">
       <formula>AND($W$5&lt;&gt;"",$W$5&lt;&gt;"material")</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="Z6 Y7:Z7">
-    <cfRule type="expression" dxfId="0" priority="9">
+    <cfRule type="expression" dxfId="9" priority="9">
       <formula>AND($Z$5&lt;&gt;"",$Z$5&lt;&gt;"material")</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="AC6 AB7:AC7">
-    <cfRule type="expression" dxfId="0" priority="10">
+    <cfRule type="expression" dxfId="8" priority="10">
       <formula>AND($AC$5&lt;&gt;"",$AC$5&lt;&gt;"material")</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="AF6 AE7:AF7">
-    <cfRule type="expression" dxfId="0" priority="11">
+    <cfRule type="expression" dxfId="7" priority="11">
       <formula>AND($AF$5&lt;&gt;"",$AF$5&lt;&gt;"material")</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="AI6 AH7:AI7">
-    <cfRule type="expression" dxfId="0" priority="12">
+    <cfRule type="expression" dxfId="6" priority="12">
       <formula>AND($AI$5&lt;&gt;"",$AI$5&lt;&gt;"material")</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="AL6 AK7:AL7">
-    <cfRule type="expression" dxfId="0" priority="13">
+    <cfRule type="expression" dxfId="5" priority="13">
       <formula>AND($AL$5&lt;&gt;"",$AL$5&lt;&gt;"material")</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="AO6 AN7:AO7">
-    <cfRule type="expression" dxfId="0" priority="14">
+    <cfRule type="expression" dxfId="4" priority="14">
       <formula>AND($AO$5&lt;&gt;"",$AO$5&lt;&gt;"material")</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="AR6 AQ7:AR7">
-    <cfRule type="expression" dxfId="0" priority="15">
+    <cfRule type="expression" dxfId="3" priority="15">
       <formula>AND($AR$5&lt;&gt;"",$AR$5&lt;&gt;"material")</formula>
     </cfRule>
   </conditionalFormatting>
   <dataValidations count="1">
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="B5 E5 H5 K5 N5 Q5 T5 W5 Z5 AC5 AF5 AI5 AL5 AO5 AR5">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="B5 E5 H5 K5 N5 Q5 T5 W5 Z5 AC5 AF5 AI5 AL5 AO5 AR5" xr:uid="{00000000-0002-0000-0400-000000000000}">
       <formula1>"material,ssr reduce,ssr hold,ssr elastic,refine"</formula1>
     </dataValidation>
   </dataValidations>
@@ -17830,17 +18025,17 @@
     </row>
   </sheetData>
   <conditionalFormatting sqref="E3:E42">
-    <cfRule type="expression" dxfId="4" priority="3">
+    <cfRule type="expression" dxfId="2" priority="3">
       <formula>OR($D3="Intercept", $D3="Radius")</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="F3:G42">
-    <cfRule type="expression" dxfId="3" priority="2">
+    <cfRule type="expression" dxfId="1" priority="2">
       <formula>OR($D3="Depth",$D3="Radius")</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="H3:H42">
-    <cfRule type="expression" dxfId="2" priority="1">
+    <cfRule type="expression" dxfId="0" priority="1">
       <formula>OR($D3="Depth",$D3="Intercept")</formula>
     </cfRule>
   </conditionalFormatting>
@@ -18065,35 +18260,35 @@
       <c r="X2" s="62"/>
     </row>
     <row r="3" spans="2:24" x14ac:dyDescent="0.2">
-      <c r="B3" s="38" t="s">
-        <v>305</v>
-      </c>
-      <c r="C3" s="38"/>
+      <c r="B3" s="58" t="s">
+        <v>304</v>
+      </c>
+      <c r="C3" s="58"/>
       <c r="D3" s="39"/>
-      <c r="F3" s="38" t="s">
-        <v>305</v>
-      </c>
-      <c r="G3" s="38"/>
+      <c r="F3" s="58" t="s">
+        <v>304</v>
+      </c>
+      <c r="G3" s="58"/>
       <c r="H3" s="39"/>
-      <c r="J3" s="38" t="s">
-        <v>305</v>
-      </c>
-      <c r="K3" s="38"/>
+      <c r="J3" s="58" t="s">
+        <v>304</v>
+      </c>
+      <c r="K3" s="58"/>
       <c r="L3" s="39"/>
-      <c r="N3" s="38" t="s">
-        <v>305</v>
-      </c>
-      <c r="O3" s="38"/>
+      <c r="N3" s="58" t="s">
+        <v>304</v>
+      </c>
+      <c r="O3" s="58"/>
       <c r="P3" s="39"/>
-      <c r="R3" s="38" t="s">
-        <v>305</v>
-      </c>
-      <c r="S3" s="38"/>
+      <c r="R3" s="58" t="s">
+        <v>304</v>
+      </c>
+      <c r="S3" s="58"/>
       <c r="T3" s="39"/>
-      <c r="V3" s="38" t="s">
-        <v>305</v>
-      </c>
-      <c r="W3" s="38"/>
+      <c r="V3" s="58" t="s">
+        <v>304</v>
+      </c>
+      <c r="W3" s="58"/>
       <c r="X3" s="39"/>
     </row>
     <row r="4" spans="2:24" x14ac:dyDescent="0.2">
@@ -18534,21 +18729,21 @@
     </row>
   </sheetData>
   <mergeCells count="12">
+    <mergeCell ref="V3:W3"/>
+    <mergeCell ref="B3:C3"/>
+    <mergeCell ref="F3:G3"/>
+    <mergeCell ref="J3:K3"/>
+    <mergeCell ref="N3:O3"/>
+    <mergeCell ref="R3:S3"/>
     <mergeCell ref="B2:D2"/>
     <mergeCell ref="V2:X2"/>
     <mergeCell ref="J2:L2"/>
     <mergeCell ref="N2:P2"/>
     <mergeCell ref="R2:T2"/>
     <mergeCell ref="F2:H2"/>
-    <mergeCell ref="B3:C3"/>
-    <mergeCell ref="F3:G3"/>
-    <mergeCell ref="J3:K3"/>
-    <mergeCell ref="N3:O3"/>
-    <mergeCell ref="R3:S3"/>
-    <mergeCell ref="V3:W3"/>
   </mergeCells>
   <dataValidations count="1">
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="D3 H3 L3 P3 T3 X3">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="D3 H3 L3 P3 T3 X3" xr:uid="{00000000-0002-0000-0800-000000000000}">
       <formula1>"normal,vertical"</formula1>
     </dataValidation>
   </dataValidations>

</xml_diff>

<commit_message>
feat(template): v21 approved — owner review pass, profile-sheet help note repositioned
Owner-edited in Excel and approved; phase two (reader/writer branch, packaged
copy sync, builder migration, load-direction and side-BC wiring) proceeds on
this file.

Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_0147GB4LGVZuqGHCRMVzZTsR
</commit_message>
<xml_diff>
--- a/docs/inputs/input_template.xlsx
+++ b/docs/inputs/input_template.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/njones/python_projects/xslope/docs/inputs/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D0BA7854-5540-8340-8930-9B54C7224615}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8EEB53F3-5E86-5B42-A7B6-55B20E1E8D9A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="620" windowWidth="34200" windowHeight="19900" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -42,7 +42,7 @@
     <definedName name="solution2">mat!#REF!</definedName>
     <definedName name="version">main!$D$5</definedName>
   </definedNames>
-  <calcPr calcId="191029" fullCalcOnLoad="1"/>
+  <calcPr calcId="191029"/>
   <extLst>
     <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
       <xcalcf:calcFeatures>
@@ -9436,22 +9436,22 @@
     <mergeCell ref="B7:D7"/>
   </mergeCells>
   <dataValidations count="6">
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="D22">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="D22" xr:uid="{4E2B12C7-FE67-3B4F-885D-33F99F4A0D82}">
       <formula1>"rollers,fixed"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="D8" xr:uid="{00000000-0002-0000-0000-000000000000}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="D8" xr:uid="{0D3EDF25-93C5-C944-8126-8CC9B17A21FC}">
       <formula1>$D$50:$D$51</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="D9" xr:uid="{00000000-0002-0000-0000-000001000000}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="D9" xr:uid="{4694A1A0-8B80-B646-8FBE-EF2E498B980D}">
       <formula1>$D$54:$D$57</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" sqref="D17" xr:uid="{00000000-0002-0000-0000-000002000000}">
+    <dataValidation type="list" allowBlank="1" sqref="D17" xr:uid="{0356D3C6-ECF7-2D4C-8DB0-E3BFC9D663DB}">
       <formula1>$D$60:$D$61</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" sqref="D14" xr:uid="{00000000-0002-0000-0000-000003000000}">
+    <dataValidation type="list" allowBlank="1" sqref="D14" xr:uid="{BDB1B4FF-9C3D-5F43-BB1B-429406E4C3E1}">
       <formula1>$D$64:$D$71</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" sqref="D18" xr:uid="{00000000-0002-0000-0000-000004000000}">
+    <dataValidation type="list" allowBlank="1" sqref="D18" xr:uid="{8A75E61B-C3DC-0F4A-869A-1DA1855E5B34}">
       <formula1>$D$74:$D$78</formula1>
     </dataValidation>
   </dataValidations>
@@ -9980,18 +9980,18 @@
     </row>
   </sheetData>
   <mergeCells count="12">
+    <mergeCell ref="B2:D2"/>
+    <mergeCell ref="V2:X2"/>
+    <mergeCell ref="J2:L2"/>
+    <mergeCell ref="N2:P2"/>
+    <mergeCell ref="R2:T2"/>
+    <mergeCell ref="F2:H2"/>
     <mergeCell ref="V3:W3"/>
     <mergeCell ref="B3:C3"/>
     <mergeCell ref="F3:G3"/>
     <mergeCell ref="J3:K3"/>
     <mergeCell ref="N3:O3"/>
     <mergeCell ref="R3:S3"/>
-    <mergeCell ref="B2:D2"/>
-    <mergeCell ref="V2:X2"/>
-    <mergeCell ref="J2:L2"/>
-    <mergeCell ref="N2:P2"/>
-    <mergeCell ref="R2:T2"/>
-    <mergeCell ref="F2:H2"/>
   </mergeCells>
   <dataValidations count="1">
     <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="D3 H3 L3 P3 T3 X3" xr:uid="{00000000-0002-0000-0900-000000000000}">
@@ -14855,9 +14855,7 @@
       <c r="D2" s="24" t="s">
         <v>160</v>
       </c>
-    </row>
-    <row r="3" spans="1:44" x14ac:dyDescent="0.2">
-      <c r="D3" s="24" t="s">
+      <c r="N2" s="24" t="s">
         <v>309</v>
       </c>
     </row>
@@ -16088,6 +16086,20 @@
     </row>
   </sheetData>
   <mergeCells count="30">
+    <mergeCell ref="D4:E4"/>
+    <mergeCell ref="P4:Q4"/>
+    <mergeCell ref="Y4:Z4"/>
+    <mergeCell ref="AB6:AC6"/>
+    <mergeCell ref="AN6:AO6"/>
+    <mergeCell ref="AB4:AC4"/>
+    <mergeCell ref="AN4:AO4"/>
+    <mergeCell ref="G6:H6"/>
+    <mergeCell ref="J4:K4"/>
+    <mergeCell ref="V6:W6"/>
+    <mergeCell ref="M6:N6"/>
+    <mergeCell ref="AH6:AI6"/>
+    <mergeCell ref="S6:T6"/>
+    <mergeCell ref="Y6:Z6"/>
     <mergeCell ref="AQ4:AR4"/>
     <mergeCell ref="A4:B4"/>
     <mergeCell ref="G4:H4"/>
@@ -16104,20 +16116,6 @@
     <mergeCell ref="AH4:AI4"/>
     <mergeCell ref="J6:K6"/>
     <mergeCell ref="P6:Q6"/>
-    <mergeCell ref="D4:E4"/>
-    <mergeCell ref="P4:Q4"/>
-    <mergeCell ref="Y4:Z4"/>
-    <mergeCell ref="AB6:AC6"/>
-    <mergeCell ref="AN6:AO6"/>
-    <mergeCell ref="AB4:AC4"/>
-    <mergeCell ref="AN4:AO4"/>
-    <mergeCell ref="G6:H6"/>
-    <mergeCell ref="J4:K4"/>
-    <mergeCell ref="V6:W6"/>
-    <mergeCell ref="M6:N6"/>
-    <mergeCell ref="AH6:AI6"/>
-    <mergeCell ref="S6:T6"/>
-    <mergeCell ref="Y6:Z6"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
@@ -17484,6 +17482,20 @@
     </row>
   </sheetData>
   <mergeCells count="30">
+    <mergeCell ref="D4:E4"/>
+    <mergeCell ref="P4:Q4"/>
+    <mergeCell ref="Y4:Z4"/>
+    <mergeCell ref="AB7:AC7"/>
+    <mergeCell ref="AN7:AO7"/>
+    <mergeCell ref="AB4:AC4"/>
+    <mergeCell ref="AN4:AO4"/>
+    <mergeCell ref="G7:H7"/>
+    <mergeCell ref="J4:K4"/>
+    <mergeCell ref="V7:W7"/>
+    <mergeCell ref="M7:N7"/>
+    <mergeCell ref="AH7:AI7"/>
+    <mergeCell ref="S7:T7"/>
+    <mergeCell ref="Y7:Z7"/>
     <mergeCell ref="AQ4:AR4"/>
     <mergeCell ref="A4:B4"/>
     <mergeCell ref="G4:H4"/>
@@ -17500,20 +17512,6 @@
     <mergeCell ref="AH4:AI4"/>
     <mergeCell ref="J7:K7"/>
     <mergeCell ref="P7:Q7"/>
-    <mergeCell ref="D4:E4"/>
-    <mergeCell ref="P4:Q4"/>
-    <mergeCell ref="Y4:Z4"/>
-    <mergeCell ref="AB7:AC7"/>
-    <mergeCell ref="AN7:AO7"/>
-    <mergeCell ref="AB4:AC4"/>
-    <mergeCell ref="AN4:AO4"/>
-    <mergeCell ref="G7:H7"/>
-    <mergeCell ref="J4:K4"/>
-    <mergeCell ref="V7:W7"/>
-    <mergeCell ref="M7:N7"/>
-    <mergeCell ref="AH7:AI7"/>
-    <mergeCell ref="S7:T7"/>
-    <mergeCell ref="Y7:Z7"/>
   </mergeCells>
   <conditionalFormatting sqref="B6 A7:B7">
     <cfRule type="expression" dxfId="17" priority="1">
@@ -18729,18 +18727,18 @@
     </row>
   </sheetData>
   <mergeCells count="12">
+    <mergeCell ref="B2:D2"/>
+    <mergeCell ref="V2:X2"/>
+    <mergeCell ref="J2:L2"/>
+    <mergeCell ref="N2:P2"/>
+    <mergeCell ref="R2:T2"/>
+    <mergeCell ref="F2:H2"/>
     <mergeCell ref="V3:W3"/>
     <mergeCell ref="B3:C3"/>
     <mergeCell ref="F3:G3"/>
     <mergeCell ref="J3:K3"/>
     <mergeCell ref="N3:O3"/>
     <mergeCell ref="R3:S3"/>
-    <mergeCell ref="B2:D2"/>
-    <mergeCell ref="V2:X2"/>
-    <mergeCell ref="J2:L2"/>
-    <mergeCell ref="N2:P2"/>
-    <mergeCell ref="R2:T2"/>
-    <mergeCell ref="F2:H2"/>
   </mergeCells>
   <dataValidations count="1">
     <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="D3 H3 L3 P3 T3 X3" xr:uid="{00000000-0002-0000-0800-000000000000}">

</xml_diff>

<commit_message>
template: the sigma headers come back as mixed-font runs
Owner's fix — Symbol-font sigma with regular parentheses per header;
resources copy synced byte-identical.

Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01XjjT2aBxw8gY7EFdpoUcpj
</commit_message>
<xml_diff>
--- a/docs/inputs/input_template.xlsx
+++ b/docs/inputs/input_template.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/njones/python_projects/xslope/docs/inputs/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{19FD11EF-E78F-0F4F-A3B9-EC76A92B0151}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FD1DA693-1E25-A64A-9652-172751DD72EE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="6420" yWindow="600" windowWidth="44060" windowHeight="18400" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="660" yWindow="600" windowWidth="44060" windowHeight="18400" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="main" sheetId="1" r:id="rId1"/>
@@ -472,15 +472,6 @@
     <t>s(f)</t>
   </si>
   <si>
-    <t>s(c/p)</t>
-  </si>
-  <si>
-    <t>s(d)</t>
-  </si>
-  <si>
-    <t>s(psi)</t>
-  </si>
-  <si>
     <t>k1</t>
   </si>
   <si>
@@ -1026,7 +1017,7 @@
         <rFont val="Aptos Narrow"/>
         <scheme val="minor"/>
       </rPr>
-      <t>(g)</t>
+      <t>(c)</t>
     </r>
   </si>
   <si>
@@ -1046,7 +1037,87 @@
         <rFont val="Aptos Narrow"/>
         <scheme val="minor"/>
       </rPr>
-      <t>(c)</t>
+      <t>(</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color theme="0"/>
+        <rFont val="Symbol"/>
+        <charset val="2"/>
+      </rPr>
+      <t>g</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color theme="0"/>
+        <rFont val="Aptos Narrow"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>)</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color theme="0"/>
+        <rFont val="Symbol"/>
+        <charset val="2"/>
+      </rPr>
+      <t>s</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color theme="0"/>
+        <rFont val="Aptos Narrow"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>(c/p)</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color theme="0"/>
+        <rFont val="Symbol"/>
+        <charset val="2"/>
+      </rPr>
+      <t>s</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color theme="0"/>
+        <rFont val="Aptos Narrow"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>(d)</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t>s(</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color theme="0"/>
+        <rFont val="Aptos Narrow"/>
+      </rPr>
+      <t>psi</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color theme="0"/>
+        <rFont val="Symbol"/>
+        <charset val="2"/>
+      </rPr>
+      <t>)</t>
     </r>
   </si>
 </sst>
@@ -3142,67 +3213,67 @@
   <sheetData>
     <row r="2" spans="1:28" x14ac:dyDescent="0.2">
       <c r="A2" s="12" t="s">
-        <v>198</v>
+        <v>195</v>
       </c>
       <c r="B2" s="12" t="s">
+        <v>243</v>
+      </c>
+      <c r="C2" s="12" t="s">
+        <v>244</v>
+      </c>
+      <c r="D2" s="12" t="s">
+        <v>245</v>
+      </c>
+      <c r="E2" s="12" t="s">
         <v>246</v>
       </c>
-      <c r="C2" s="12" t="s">
+      <c r="F2" s="12" t="s">
         <v>247</v>
       </c>
-      <c r="D2" s="12" t="s">
+      <c r="G2" s="40" t="s">
         <v>248</v>
       </c>
-      <c r="E2" s="12" t="s">
+      <c r="H2" s="40" t="s">
         <v>249</v>
       </c>
-      <c r="F2" s="12" t="s">
+      <c r="I2" s="40" t="s">
         <v>250</v>
       </c>
-      <c r="G2" s="40" t="s">
+      <c r="J2" s="27" t="s">
         <v>251</v>
       </c>
-      <c r="H2" s="40" t="s">
+      <c r="K2" s="27" t="s">
         <v>252</v>
       </c>
-      <c r="I2" s="40" t="s">
+      <c r="L2" s="27" t="s">
         <v>253</v>
       </c>
-      <c r="J2" s="27" t="s">
+      <c r="M2" s="27" t="s">
         <v>254</v>
       </c>
-      <c r="K2" s="27" t="s">
+      <c r="N2" s="27" t="s">
         <v>255</v>
       </c>
-      <c r="L2" s="27" t="s">
+      <c r="O2" s="27" t="s">
         <v>256</v>
       </c>
-      <c r="M2" s="27" t="s">
+      <c r="P2" s="28" t="s">
         <v>257</v>
-      </c>
-      <c r="N2" s="27" t="s">
-        <v>258</v>
-      </c>
-      <c r="O2" s="27" t="s">
-        <v>259</v>
-      </c>
-      <c r="P2" s="28" t="s">
-        <v>260</v>
       </c>
       <c r="Q2" s="28" t="s">
         <v>123</v>
       </c>
       <c r="R2" s="28" t="s">
+        <v>258</v>
+      </c>
+      <c r="Z2" t="s">
+        <v>259</v>
+      </c>
+      <c r="AA2" t="s">
+        <v>260</v>
+      </c>
+      <c r="AB2" t="s">
         <v>261</v>
-      </c>
-      <c r="Z2" t="s">
-        <v>262</v>
-      </c>
-      <c r="AA2" t="s">
-        <v>263</v>
-      </c>
-      <c r="AB2" t="s">
-        <v>264</v>
       </c>
     </row>
     <row r="3" spans="1:28" x14ac:dyDescent="0.2">
@@ -3233,13 +3304,13 @@
       <c r="Q3" s="3"/>
       <c r="R3" s="3"/>
       <c r="Z3" t="s">
-        <v>265</v>
+        <v>262</v>
       </c>
       <c r="AA3" t="s">
-        <v>266</v>
+        <v>263</v>
       </c>
       <c r="AB3" t="s">
-        <v>267</v>
+        <v>264</v>
       </c>
     </row>
     <row r="4" spans="1:28" x14ac:dyDescent="0.2">
@@ -3270,7 +3341,7 @@
       <c r="Q4" s="3"/>
       <c r="R4" s="3"/>
       <c r="Z4" t="s">
-        <v>268</v>
+        <v>265</v>
       </c>
     </row>
     <row r="5" spans="1:28" x14ac:dyDescent="0.2">
@@ -3301,7 +3372,7 @@
       <c r="Q5" s="3"/>
       <c r="R5" s="3"/>
       <c r="Z5" t="s">
-        <v>269</v>
+        <v>266</v>
       </c>
     </row>
     <row r="6" spans="1:28" x14ac:dyDescent="0.2">
@@ -3388,13 +3459,13 @@
       <c r="Q8" s="3"/>
       <c r="R8" s="3"/>
       <c r="Z8" t="s">
-        <v>262</v>
+        <v>259</v>
       </c>
       <c r="AA8" t="s">
-        <v>263</v>
+        <v>260</v>
       </c>
       <c r="AB8" t="s">
-        <v>264</v>
+        <v>261</v>
       </c>
     </row>
     <row r="9" spans="1:28" x14ac:dyDescent="0.2">
@@ -3425,13 +3496,13 @@
       <c r="Q9" s="3"/>
       <c r="R9" s="3"/>
       <c r="Z9" t="s">
-        <v>265</v>
+        <v>262</v>
       </c>
       <c r="AA9" t="s">
-        <v>266</v>
+        <v>263</v>
       </c>
       <c r="AB9" t="s">
-        <v>267</v>
+        <v>264</v>
       </c>
     </row>
     <row r="10" spans="1:28" x14ac:dyDescent="0.2">
@@ -3462,13 +3533,13 @@
       <c r="Q10" s="3"/>
       <c r="R10" s="3"/>
       <c r="Z10" t="s">
-        <v>268</v>
+        <v>265</v>
       </c>
       <c r="AA10" t="s">
-        <v>266</v>
+        <v>263</v>
       </c>
       <c r="AB10" t="s">
-        <v>264</v>
+        <v>261</v>
       </c>
     </row>
     <row r="11" spans="1:28" x14ac:dyDescent="0.2">
@@ -3499,13 +3570,13 @@
       <c r="Q11" s="3"/>
       <c r="R11" s="3"/>
       <c r="Z11" t="s">
-        <v>269</v>
+        <v>266</v>
       </c>
       <c r="AA11" t="s">
-        <v>266</v>
+        <v>263</v>
       </c>
       <c r="AB11" t="s">
-        <v>264</v>
+        <v>261</v>
       </c>
     </row>
     <row r="12" spans="1:28" x14ac:dyDescent="0.2">
@@ -3870,61 +3941,61 @@
   <sheetData>
     <row r="2" spans="1:27" x14ac:dyDescent="0.2">
       <c r="A2" s="12" t="s">
-        <v>198</v>
+        <v>195</v>
       </c>
       <c r="B2" s="12" t="s">
+        <v>243</v>
+      </c>
+      <c r="C2" s="12" t="s">
+        <v>244</v>
+      </c>
+      <c r="D2" s="12" t="s">
+        <v>245</v>
+      </c>
+      <c r="E2" s="12" t="s">
         <v>246</v>
       </c>
-      <c r="C2" s="12" t="s">
+      <c r="F2" s="12" t="s">
         <v>247</v>
       </c>
-      <c r="D2" s="12" t="s">
-        <v>248</v>
-      </c>
-      <c r="E2" s="12" t="s">
-        <v>249</v>
-      </c>
-      <c r="F2" s="12" t="s">
+      <c r="G2" s="40" t="s">
+        <v>267</v>
+      </c>
+      <c r="H2" s="40" t="s">
+        <v>306</v>
+      </c>
+      <c r="I2" s="40" t="s">
         <v>250</v>
       </c>
-      <c r="G2" s="40" t="s">
+      <c r="J2" s="27" t="s">
+        <v>268</v>
+      </c>
+      <c r="K2" s="27" t="s">
+        <v>269</v>
+      </c>
+      <c r="L2" s="41" t="s">
         <v>270</v>
       </c>
-      <c r="H2" s="40" t="s">
-        <v>309</v>
-      </c>
-      <c r="I2" s="40" t="s">
-        <v>253</v>
-      </c>
-      <c r="J2" s="27" t="s">
+      <c r="M2" s="41" t="s">
         <v>271</v>
-      </c>
-      <c r="K2" s="27" t="s">
-        <v>272</v>
-      </c>
-      <c r="L2" s="41" t="s">
-        <v>273</v>
-      </c>
-      <c r="M2" s="41" t="s">
-        <v>274</v>
       </c>
       <c r="N2" s="28" t="s">
         <v>123</v>
       </c>
       <c r="O2" s="28" t="s">
-        <v>275</v>
+        <v>272</v>
       </c>
       <c r="P2" s="28" t="s">
+        <v>258</v>
+      </c>
+      <c r="Q2" s="28" t="s">
+        <v>273</v>
+      </c>
+      <c r="Z2" t="s">
+        <v>223</v>
+      </c>
+      <c r="AA2" t="s">
         <v>261</v>
-      </c>
-      <c r="Q2" s="28" t="s">
-        <v>276</v>
-      </c>
-      <c r="Z2" t="s">
-        <v>226</v>
-      </c>
-      <c r="AA2" t="s">
-        <v>264</v>
       </c>
     </row>
     <row r="3" spans="1:27" x14ac:dyDescent="0.2">
@@ -3948,10 +4019,10 @@
       <c r="P3" s="3"/>
       <c r="Q3" s="3"/>
       <c r="Z3" t="s">
-        <v>230</v>
+        <v>227</v>
       </c>
       <c r="AA3" t="s">
-        <v>267</v>
+        <v>264</v>
       </c>
     </row>
     <row r="4" spans="1:27" x14ac:dyDescent="0.2">
@@ -4195,22 +4266,22 @@
   <sheetData>
     <row r="2" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A2" s="12" t="s">
-        <v>198</v>
+        <v>195</v>
       </c>
       <c r="B2" s="12" t="s">
-        <v>246</v>
+        <v>243</v>
       </c>
       <c r="C2" s="12" t="s">
-        <v>170</v>
+        <v>167</v>
       </c>
       <c r="D2" s="12" t="s">
-        <v>171</v>
+        <v>168</v>
       </c>
       <c r="E2" s="12" t="s">
-        <v>277</v>
+        <v>274</v>
       </c>
       <c r="F2" s="12" t="s">
-        <v>278</v>
+        <v>275</v>
       </c>
     </row>
     <row r="3" spans="1:6" x14ac:dyDescent="0.2">
@@ -4433,27 +4504,27 @@
   <sheetData>
     <row r="2" spans="2:21" x14ac:dyDescent="0.2">
       <c r="B2" s="64" t="s">
-        <v>279</v>
+        <v>276</v>
       </c>
       <c r="C2" s="65"/>
       <c r="E2" s="59" t="s">
-        <v>280</v>
+        <v>277</v>
       </c>
       <c r="F2" s="54"/>
       <c r="H2" s="59" t="s">
-        <v>281</v>
+        <v>278</v>
       </c>
       <c r="I2" s="54"/>
       <c r="K2" s="59" t="s">
-        <v>282</v>
+        <v>279</v>
       </c>
       <c r="L2" s="54"/>
       <c r="N2" s="59" t="s">
-        <v>283</v>
+        <v>280</v>
       </c>
       <c r="O2" s="54"/>
       <c r="Q2" s="59" t="s">
-        <v>284</v>
+        <v>281</v>
       </c>
       <c r="R2" s="54"/>
     </row>
@@ -4461,71 +4532,71 @@
       <c r="B3" s="66"/>
       <c r="C3" s="67"/>
       <c r="E3" s="32" t="s">
-        <v>285</v>
+        <v>282</v>
       </c>
       <c r="F3" s="33"/>
       <c r="H3" s="32" t="s">
-        <v>285</v>
+        <v>282</v>
       </c>
       <c r="I3" s="33"/>
       <c r="K3" s="32" t="s">
-        <v>285</v>
+        <v>282</v>
       </c>
       <c r="L3" s="33"/>
       <c r="N3" s="32" t="s">
-        <v>285</v>
+        <v>282</v>
       </c>
       <c r="O3" s="33"/>
       <c r="Q3" s="32" t="s">
-        <v>285</v>
+        <v>282</v>
       </c>
       <c r="R3" s="33"/>
       <c r="T3" s="6" t="s">
-        <v>286</v>
+        <v>283</v>
       </c>
     </row>
     <row r="4" spans="2:21" x14ac:dyDescent="0.2">
       <c r="B4" s="25" t="s">
-        <v>170</v>
+        <v>167</v>
       </c>
       <c r="C4" s="25" t="s">
-        <v>171</v>
+        <v>168</v>
       </c>
       <c r="E4" s="25" t="s">
-        <v>170</v>
+        <v>167</v>
       </c>
       <c r="F4" s="25" t="s">
-        <v>171</v>
+        <v>168</v>
       </c>
       <c r="H4" s="25" t="s">
-        <v>170</v>
+        <v>167</v>
       </c>
       <c r="I4" s="25" t="s">
-        <v>171</v>
+        <v>168</v>
       </c>
       <c r="K4" s="25" t="s">
-        <v>170</v>
+        <v>167</v>
       </c>
       <c r="L4" s="25" t="s">
-        <v>171</v>
+        <v>168</v>
       </c>
       <c r="N4" s="25" t="s">
-        <v>170</v>
+        <v>167</v>
       </c>
       <c r="O4" s="25" t="s">
-        <v>171</v>
+        <v>168</v>
       </c>
       <c r="Q4" s="25" t="s">
-        <v>170</v>
+        <v>167</v>
       </c>
       <c r="R4" s="25" t="s">
-        <v>171</v>
+        <v>168</v>
       </c>
       <c r="T4" s="1" t="s">
-        <v>285</v>
+        <v>282</v>
       </c>
       <c r="U4" t="s">
-        <v>287</v>
+        <v>284</v>
       </c>
     </row>
     <row r="5" spans="2:21" x14ac:dyDescent="0.2">
@@ -4542,10 +4613,10 @@
       <c r="Q5" s="3"/>
       <c r="R5" s="3"/>
       <c r="T5" s="1" t="s">
-        <v>288</v>
+        <v>285</v>
       </c>
       <c r="U5" t="s">
-        <v>289</v>
+        <v>286</v>
       </c>
     </row>
     <row r="6" spans="2:21" x14ac:dyDescent="0.2">
@@ -4562,7 +4633,7 @@
       <c r="Q6" s="3"/>
       <c r="R6" s="3"/>
       <c r="T6" s="1" t="s">
-        <v>290</v>
+        <v>287</v>
       </c>
       <c r="U6" s="9"/>
     </row>
@@ -4851,27 +4922,27 @@
   <sheetData>
     <row r="2" spans="2:21" x14ac:dyDescent="0.2">
       <c r="B2" s="68" t="s">
-        <v>291</v>
+        <v>288</v>
       </c>
       <c r="C2" s="65"/>
       <c r="E2" s="60" t="s">
-        <v>292</v>
+        <v>289</v>
       </c>
       <c r="F2" s="54"/>
       <c r="H2" s="60" t="s">
-        <v>293</v>
+        <v>290</v>
       </c>
       <c r="I2" s="54"/>
       <c r="K2" s="60" t="s">
-        <v>294</v>
+        <v>291</v>
       </c>
       <c r="L2" s="54"/>
       <c r="N2" s="60" t="s">
-        <v>295</v>
+        <v>292</v>
       </c>
       <c r="O2" s="54"/>
       <c r="Q2" s="60" t="s">
-        <v>296</v>
+        <v>293</v>
       </c>
       <c r="R2" s="54"/>
     </row>
@@ -4879,71 +4950,71 @@
       <c r="B3" s="66"/>
       <c r="C3" s="67"/>
       <c r="E3" s="34" t="s">
-        <v>285</v>
+        <v>282</v>
       </c>
       <c r="F3" s="35"/>
       <c r="H3" s="34" t="s">
-        <v>285</v>
+        <v>282</v>
       </c>
       <c r="I3" s="35"/>
       <c r="K3" s="34" t="s">
-        <v>285</v>
+        <v>282</v>
       </c>
       <c r="L3" s="35"/>
       <c r="N3" s="34" t="s">
-        <v>285</v>
+        <v>282</v>
       </c>
       <c r="O3" s="35"/>
       <c r="Q3" s="34" t="s">
-        <v>285</v>
+        <v>282</v>
       </c>
       <c r="R3" s="35"/>
       <c r="T3" s="6" t="s">
-        <v>286</v>
+        <v>283</v>
       </c>
     </row>
     <row r="4" spans="2:21" x14ac:dyDescent="0.2">
       <c r="B4" s="25" t="s">
-        <v>170</v>
+        <v>167</v>
       </c>
       <c r="C4" s="25" t="s">
-        <v>171</v>
+        <v>168</v>
       </c>
       <c r="E4" s="25" t="s">
-        <v>170</v>
+        <v>167</v>
       </c>
       <c r="F4" s="25" t="s">
-        <v>171</v>
+        <v>168</v>
       </c>
       <c r="H4" s="25" t="s">
-        <v>170</v>
+        <v>167</v>
       </c>
       <c r="I4" s="25" t="s">
-        <v>171</v>
+        <v>168</v>
       </c>
       <c r="K4" s="25" t="s">
-        <v>170</v>
+        <v>167</v>
       </c>
       <c r="L4" s="25" t="s">
-        <v>171</v>
+        <v>168</v>
       </c>
       <c r="N4" s="25" t="s">
-        <v>170</v>
+        <v>167</v>
       </c>
       <c r="O4" s="25" t="s">
-        <v>171</v>
+        <v>168</v>
       </c>
       <c r="Q4" s="25" t="s">
-        <v>170</v>
+        <v>167</v>
       </c>
       <c r="R4" s="25" t="s">
-        <v>171</v>
+        <v>168</v>
       </c>
       <c r="T4" s="1" t="s">
-        <v>285</v>
+        <v>282</v>
       </c>
       <c r="U4" t="s">
-        <v>287</v>
+        <v>284</v>
       </c>
     </row>
     <row r="5" spans="2:21" x14ac:dyDescent="0.2">
@@ -4960,10 +5031,10 @@
       <c r="Q5" s="3"/>
       <c r="R5" s="3"/>
       <c r="T5" s="1" t="s">
-        <v>288</v>
+        <v>285</v>
       </c>
       <c r="U5" t="s">
-        <v>289</v>
+        <v>286</v>
       </c>
     </row>
     <row r="6" spans="2:21" x14ac:dyDescent="0.2">
@@ -5262,22 +5333,22 @@
   <sheetData>
     <row r="2" spans="2:10" x14ac:dyDescent="0.2">
       <c r="B2" s="50" t="s">
+        <v>294</v>
+      </c>
+      <c r="C2" s="50" t="s">
+        <v>295</v>
+      </c>
+      <c r="D2" s="50" t="s">
+        <v>296</v>
+      </c>
+      <c r="E2" s="50" t="s">
         <v>297</v>
       </c>
-      <c r="C2" s="50" t="s">
+      <c r="F2" s="50" t="s">
         <v>298</v>
       </c>
-      <c r="D2" s="50" t="s">
+      <c r="G2" s="50" t="s">
         <v>299</v>
-      </c>
-      <c r="E2" s="50" t="s">
-        <v>300</v>
-      </c>
-      <c r="F2" s="50" t="s">
-        <v>301</v>
-      </c>
-      <c r="G2" s="50" t="s">
-        <v>302</v>
       </c>
     </row>
     <row r="3" spans="2:10" x14ac:dyDescent="0.2">
@@ -5288,7 +5359,7 @@
       <c r="F3" s="3"/>
       <c r="G3" s="3"/>
       <c r="I3" s="14" t="s">
-        <v>303</v>
+        <v>300</v>
       </c>
       <c r="J3" s="3"/>
     </row>
@@ -5310,7 +5381,7 @@
       <c r="F5" s="3"/>
       <c r="G5" s="3"/>
       <c r="I5" s="14" t="s">
-        <v>304</v>
+        <v>301</v>
       </c>
       <c r="J5" s="3"/>
     </row>
@@ -5332,7 +5403,7 @@
       <c r="F7" s="3"/>
       <c r="G7" s="3"/>
       <c r="I7" s="14" t="s">
-        <v>305</v>
+        <v>302</v>
       </c>
       <c r="J7" s="3"/>
     </row>
@@ -5344,7 +5415,7 @@
       <c r="F8" s="3"/>
       <c r="G8" s="3"/>
       <c r="I8" s="14" t="s">
-        <v>306</v>
+        <v>303</v>
       </c>
       <c r="J8" s="3"/>
     </row>
@@ -5356,7 +5427,7 @@
       <c r="F9" s="3"/>
       <c r="G9" s="3"/>
       <c r="I9" s="14" t="s">
-        <v>307</v>
+        <v>304</v>
       </c>
       <c r="J9" s="3"/>
     </row>
@@ -5376,7 +5447,7 @@
       <c r="F11" s="3"/>
       <c r="G11" s="3"/>
       <c r="J11" t="s">
-        <v>308</v>
+        <v>305</v>
       </c>
     </row>
     <row r="12" spans="2:10" x14ac:dyDescent="0.2">
@@ -6440,52 +6511,52 @@
         <v>135</v>
       </c>
       <c r="AA10" s="46" t="s">
-        <v>310</v>
+        <v>308</v>
       </c>
       <c r="AB10" s="46" t="s">
-        <v>311</v>
+        <v>307</v>
       </c>
       <c r="AC10" s="47" t="s">
         <v>136</v>
       </c>
       <c r="AD10" s="46" t="s">
+        <v>309</v>
+      </c>
+      <c r="AE10" s="46" t="s">
+        <v>310</v>
+      </c>
+      <c r="AF10" s="47" t="s">
+        <v>311</v>
+      </c>
+      <c r="AG10" s="23" t="s">
         <v>137</v>
       </c>
-      <c r="AE10" s="46" t="s">
+      <c r="AH10" s="23" t="s">
         <v>138</v>
       </c>
-      <c r="AF10" s="47" t="s">
+      <c r="AI10" s="23" t="s">
         <v>139</v>
       </c>
-      <c r="AG10" s="23" t="s">
+      <c r="AJ10" s="23" t="s">
         <v>140</v>
       </c>
-      <c r="AH10" s="23" t="s">
+      <c r="AK10" s="23" t="s">
         <v>141</v>
       </c>
-      <c r="AI10" s="23" t="s">
+      <c r="AL10" s="23" t="s">
         <v>142</v>
       </c>
-      <c r="AJ10" s="23" t="s">
+      <c r="AM10" s="23" t="s">
         <v>143</v>
       </c>
-      <c r="AK10" s="23" t="s">
+      <c r="AN10" s="23" t="s">
         <v>144</v>
       </c>
-      <c r="AL10" s="23" t="s">
+      <c r="AO10" s="23" t="s">
         <v>145</v>
       </c>
-      <c r="AM10" s="23" t="s">
+      <c r="AP10" s="23" t="s">
         <v>146</v>
-      </c>
-      <c r="AN10" s="23" t="s">
-        <v>147</v>
-      </c>
-      <c r="AO10" s="23" t="s">
-        <v>148</v>
-      </c>
-      <c r="AP10" s="23" t="s">
-        <v>149</v>
       </c>
     </row>
     <row r="11" spans="1:42" x14ac:dyDescent="0.2">
@@ -7966,183 +8037,183 @@
   <sheetData>
     <row r="2" spans="1:44" x14ac:dyDescent="0.2">
       <c r="A2" s="5" t="s">
-        <v>150</v>
+        <v>147</v>
       </c>
       <c r="B2" s="3">
         <v>0</v>
       </c>
       <c r="D2" s="24" t="s">
-        <v>151</v>
+        <v>148</v>
       </c>
       <c r="N2" s="24" t="s">
-        <v>152</v>
+        <v>149</v>
       </c>
     </row>
     <row r="4" spans="1:44" x14ac:dyDescent="0.2">
       <c r="A4" s="55" t="s">
-        <v>153</v>
+        <v>150</v>
       </c>
       <c r="B4" s="52"/>
       <c r="D4" s="55" t="s">
-        <v>154</v>
+        <v>151</v>
       </c>
       <c r="E4" s="52"/>
       <c r="G4" s="55" t="s">
-        <v>155</v>
+        <v>152</v>
       </c>
       <c r="H4" s="52"/>
       <c r="J4" s="55" t="s">
-        <v>156</v>
+        <v>153</v>
       </c>
       <c r="K4" s="52"/>
       <c r="M4" s="55" t="s">
-        <v>157</v>
+        <v>154</v>
       </c>
       <c r="N4" s="52"/>
       <c r="P4" s="55" t="s">
-        <v>158</v>
+        <v>155</v>
       </c>
       <c r="Q4" s="54"/>
       <c r="R4" s="1"/>
       <c r="S4" s="55" t="s">
-        <v>159</v>
+        <v>156</v>
       </c>
       <c r="T4" s="54"/>
       <c r="U4" s="1"/>
       <c r="V4" s="55" t="s">
-        <v>160</v>
+        <v>157</v>
       </c>
       <c r="W4" s="54"/>
       <c r="X4" s="1"/>
       <c r="Y4" s="55" t="s">
-        <v>161</v>
+        <v>158</v>
       </c>
       <c r="Z4" s="54"/>
       <c r="AA4" s="1"/>
       <c r="AB4" s="55" t="s">
-        <v>162</v>
+        <v>159</v>
       </c>
       <c r="AC4" s="54"/>
       <c r="AE4" s="55" t="s">
-        <v>163</v>
+        <v>160</v>
       </c>
       <c r="AF4" s="54"/>
       <c r="AG4" s="1"/>
       <c r="AH4" s="55" t="s">
-        <v>164</v>
+        <v>161</v>
       </c>
       <c r="AI4" s="54"/>
       <c r="AJ4" s="1"/>
       <c r="AK4" s="55" t="s">
-        <v>165</v>
+        <v>162</v>
       </c>
       <c r="AL4" s="54"/>
       <c r="AM4" s="1"/>
       <c r="AN4" s="55" t="s">
-        <v>166</v>
+        <v>163</v>
       </c>
       <c r="AO4" s="54"/>
       <c r="AP4" s="1"/>
       <c r="AQ4" s="55" t="s">
-        <v>167</v>
+        <v>164</v>
       </c>
       <c r="AR4" s="54"/>
     </row>
     <row r="5" spans="1:44" x14ac:dyDescent="0.2">
       <c r="A5" s="36" t="s">
-        <v>168</v>
+        <v>165</v>
       </c>
       <c r="B5" s="37">
         <v>1</v>
       </c>
       <c r="D5" s="36" t="s">
-        <v>168</v>
+        <v>165</v>
       </c>
       <c r="E5" s="37">
         <v>2</v>
       </c>
       <c r="G5" s="36" t="s">
-        <v>168</v>
+        <v>165</v>
       </c>
       <c r="H5" s="37">
         <v>3</v>
       </c>
       <c r="J5" s="36" t="s">
-        <v>168</v>
+        <v>165</v>
       </c>
       <c r="K5" s="37">
         <v>4</v>
       </c>
       <c r="M5" s="36" t="s">
-        <v>168</v>
+        <v>165</v>
       </c>
       <c r="N5" s="37">
         <v>5</v>
       </c>
       <c r="P5" s="36" t="s">
-        <v>168</v>
+        <v>165</v>
       </c>
       <c r="Q5" s="37">
         <v>6</v>
       </c>
       <c r="R5" s="1"/>
       <c r="S5" s="36" t="s">
-        <v>168</v>
+        <v>165</v>
       </c>
       <c r="T5" s="37">
         <v>7</v>
       </c>
       <c r="U5" s="1"/>
       <c r="V5" s="36" t="s">
-        <v>168</v>
+        <v>165</v>
       </c>
       <c r="W5" s="37">
         <v>8</v>
       </c>
       <c r="X5" s="1"/>
       <c r="Y5" s="36" t="s">
-        <v>168</v>
+        <v>165</v>
       </c>
       <c r="Z5" s="37">
         <v>9</v>
       </c>
       <c r="AA5" s="1"/>
       <c r="AB5" s="36" t="s">
-        <v>168</v>
+        <v>165</v>
       </c>
       <c r="AC5" s="37">
         <v>10</v>
       </c>
       <c r="AE5" s="36" t="s">
-        <v>168</v>
+        <v>165</v>
       </c>
       <c r="AF5" s="37">
         <v>11</v>
       </c>
       <c r="AG5" s="1"/>
       <c r="AH5" s="36" t="s">
-        <v>168</v>
+        <v>165</v>
       </c>
       <c r="AI5" s="37">
         <v>12</v>
       </c>
       <c r="AJ5" s="1"/>
       <c r="AK5" s="36" t="s">
-        <v>168</v>
+        <v>165</v>
       </c>
       <c r="AL5" s="37">
         <v>13</v>
       </c>
       <c r="AM5" s="1"/>
       <c r="AN5" s="36" t="s">
-        <v>168</v>
+        <v>165</v>
       </c>
       <c r="AO5" s="37">
         <v>14</v>
       </c>
       <c r="AP5" s="1"/>
       <c r="AQ5" s="36" t="s">
-        <v>168</v>
+        <v>165</v>
       </c>
       <c r="AR5" s="37">
         <v>15</v>
@@ -8235,172 +8306,172 @@
     </row>
     <row r="7" spans="1:44" x14ac:dyDescent="0.2">
       <c r="A7" s="36" t="s">
-        <v>169</v>
+        <v>166</v>
       </c>
       <c r="B7" s="37"/>
       <c r="D7" s="36" t="s">
-        <v>169</v>
+        <v>166</v>
       </c>
       <c r="E7" s="37"/>
       <c r="G7" s="36" t="s">
-        <v>169</v>
+        <v>166</v>
       </c>
       <c r="H7" s="37"/>
       <c r="J7" s="36" t="s">
-        <v>169</v>
+        <v>166</v>
       </c>
       <c r="K7" s="37"/>
       <c r="M7" s="36" t="s">
-        <v>169</v>
+        <v>166</v>
       </c>
       <c r="N7" s="37"/>
       <c r="P7" s="36" t="s">
-        <v>169</v>
+        <v>166</v>
       </c>
       <c r="Q7" s="37"/>
       <c r="R7" s="1"/>
       <c r="S7" s="36" t="s">
-        <v>169</v>
+        <v>166</v>
       </c>
       <c r="T7" s="37"/>
       <c r="U7" s="1"/>
       <c r="V7" s="36" t="s">
-        <v>169</v>
+        <v>166</v>
       </c>
       <c r="W7" s="37"/>
       <c r="X7" s="1"/>
       <c r="Y7" s="36" t="s">
-        <v>169</v>
+        <v>166</v>
       </c>
       <c r="Z7" s="37"/>
       <c r="AA7" s="1"/>
       <c r="AB7" s="36" t="s">
-        <v>169</v>
+        <v>166</v>
       </c>
       <c r="AC7" s="37"/>
       <c r="AE7" s="36" t="s">
-        <v>169</v>
+        <v>166</v>
       </c>
       <c r="AF7" s="37"/>
       <c r="AG7" s="1"/>
       <c r="AH7" s="36" t="s">
-        <v>169</v>
+        <v>166</v>
       </c>
       <c r="AI7" s="37"/>
       <c r="AJ7" s="1"/>
       <c r="AK7" s="36" t="s">
-        <v>169</v>
+        <v>166</v>
       </c>
       <c r="AL7" s="37"/>
       <c r="AM7" s="1"/>
       <c r="AN7" s="36" t="s">
-        <v>169</v>
+        <v>166</v>
       </c>
       <c r="AO7" s="37"/>
       <c r="AP7" s="1"/>
       <c r="AQ7" s="36" t="s">
-        <v>169</v>
+        <v>166</v>
       </c>
       <c r="AR7" s="37"/>
     </row>
     <row r="8" spans="1:44" x14ac:dyDescent="0.2">
       <c r="A8" s="2" t="s">
-        <v>170</v>
+        <v>167</v>
       </c>
       <c r="B8" s="2" t="s">
-        <v>171</v>
+        <v>168</v>
       </c>
       <c r="D8" s="2" t="s">
-        <v>170</v>
+        <v>167</v>
       </c>
       <c r="E8" s="2" t="s">
-        <v>171</v>
+        <v>168</v>
       </c>
       <c r="G8" s="2" t="s">
-        <v>170</v>
+        <v>167</v>
       </c>
       <c r="H8" s="2" t="s">
-        <v>171</v>
+        <v>168</v>
       </c>
       <c r="J8" s="2" t="s">
-        <v>170</v>
+        <v>167</v>
       </c>
       <c r="K8" s="2" t="s">
-        <v>171</v>
+        <v>168</v>
       </c>
       <c r="M8" s="2" t="s">
-        <v>170</v>
+        <v>167</v>
       </c>
       <c r="N8" s="2" t="s">
-        <v>171</v>
+        <v>168</v>
       </c>
       <c r="P8" s="2" t="s">
-        <v>170</v>
+        <v>167</v>
       </c>
       <c r="Q8" s="2" t="s">
-        <v>171</v>
+        <v>168</v>
       </c>
       <c r="R8" s="1"/>
       <c r="S8" s="2" t="s">
-        <v>170</v>
+        <v>167</v>
       </c>
       <c r="T8" s="2" t="s">
-        <v>171</v>
+        <v>168</v>
       </c>
       <c r="U8" s="1"/>
       <c r="V8" s="2" t="s">
-        <v>170</v>
+        <v>167</v>
       </c>
       <c r="W8" s="2" t="s">
-        <v>171</v>
+        <v>168</v>
       </c>
       <c r="X8" s="1"/>
       <c r="Y8" s="2" t="s">
-        <v>170</v>
+        <v>167</v>
       </c>
       <c r="Z8" s="2" t="s">
-        <v>171</v>
+        <v>168</v>
       </c>
       <c r="AA8" s="1"/>
       <c r="AB8" s="2" t="s">
-        <v>170</v>
+        <v>167</v>
       </c>
       <c r="AC8" s="2" t="s">
-        <v>171</v>
+        <v>168</v>
       </c>
       <c r="AE8" s="2" t="s">
-        <v>170</v>
+        <v>167</v>
       </c>
       <c r="AF8" s="2" t="s">
-        <v>171</v>
+        <v>168</v>
       </c>
       <c r="AG8" s="1"/>
       <c r="AH8" s="2" t="s">
-        <v>170</v>
+        <v>167</v>
       </c>
       <c r="AI8" s="2" t="s">
-        <v>171</v>
+        <v>168</v>
       </c>
       <c r="AJ8" s="1"/>
       <c r="AK8" s="2" t="s">
-        <v>170</v>
+        <v>167</v>
       </c>
       <c r="AL8" s="2" t="s">
-        <v>171</v>
+        <v>168</v>
       </c>
       <c r="AM8" s="1"/>
       <c r="AN8" s="2" t="s">
-        <v>170</v>
+        <v>167</v>
       </c>
       <c r="AO8" s="2" t="s">
-        <v>171</v>
+        <v>168</v>
       </c>
       <c r="AP8" s="1"/>
       <c r="AQ8" s="2" t="s">
-        <v>170</v>
+        <v>167</v>
       </c>
       <c r="AR8" s="2" t="s">
-        <v>171</v>
+        <v>168</v>
       </c>
     </row>
     <row r="9" spans="1:44" x14ac:dyDescent="0.2">
@@ -9221,6 +9292,13 @@
     <mergeCell ref="AH4:AI4"/>
     <mergeCell ref="J6:K6"/>
     <mergeCell ref="P6:Q6"/>
+    <mergeCell ref="D4:E4"/>
+    <mergeCell ref="P4:Q4"/>
+    <mergeCell ref="Y4:Z4"/>
+    <mergeCell ref="AB6:AC6"/>
+    <mergeCell ref="AN6:AO6"/>
+    <mergeCell ref="AB4:AC4"/>
+    <mergeCell ref="AN4:AO4"/>
     <mergeCell ref="G6:H6"/>
     <mergeCell ref="J4:K4"/>
     <mergeCell ref="V6:W6"/>
@@ -9228,13 +9306,6 @@
     <mergeCell ref="AH6:AI6"/>
     <mergeCell ref="S6:T6"/>
     <mergeCell ref="Y6:Z6"/>
-    <mergeCell ref="D4:E4"/>
-    <mergeCell ref="P4:Q4"/>
-    <mergeCell ref="Y4:Z4"/>
-    <mergeCell ref="AB6:AC6"/>
-    <mergeCell ref="AN6:AO6"/>
-    <mergeCell ref="AB4:AC4"/>
-    <mergeCell ref="AN4:AO4"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
@@ -9268,277 +9339,277 @@
   <sheetData>
     <row r="2" spans="1:44" x14ac:dyDescent="0.2">
       <c r="A2" s="24" t="s">
-        <v>172</v>
+        <v>169</v>
       </c>
       <c r="G2" s="9" t="s">
-        <v>173</v>
+        <v>170</v>
       </c>
     </row>
     <row r="4" spans="1:44" x14ac:dyDescent="0.2">
       <c r="A4" s="55" t="s">
-        <v>174</v>
+        <v>171</v>
       </c>
       <c r="B4" s="52"/>
       <c r="D4" s="55" t="s">
-        <v>175</v>
+        <v>172</v>
       </c>
       <c r="E4" s="52"/>
       <c r="G4" s="55" t="s">
-        <v>176</v>
+        <v>173</v>
       </c>
       <c r="H4" s="52"/>
       <c r="J4" s="55" t="s">
-        <v>177</v>
+        <v>174</v>
       </c>
       <c r="K4" s="52"/>
       <c r="M4" s="55" t="s">
-        <v>178</v>
+        <v>175</v>
       </c>
       <c r="N4" s="52"/>
       <c r="P4" s="55" t="s">
-        <v>179</v>
+        <v>176</v>
       </c>
       <c r="Q4" s="54"/>
       <c r="R4" s="1"/>
       <c r="S4" s="55" t="s">
-        <v>180</v>
+        <v>177</v>
       </c>
       <c r="T4" s="54"/>
       <c r="U4" s="1"/>
       <c r="V4" s="55" t="s">
-        <v>181</v>
+        <v>178</v>
       </c>
       <c r="W4" s="54"/>
       <c r="X4" s="1"/>
       <c r="Y4" s="55" t="s">
-        <v>182</v>
+        <v>179</v>
       </c>
       <c r="Z4" s="54"/>
       <c r="AA4" s="1"/>
       <c r="AB4" s="55" t="s">
-        <v>183</v>
+        <v>180</v>
       </c>
       <c r="AC4" s="54"/>
       <c r="AE4" s="55" t="s">
-        <v>184</v>
+        <v>181</v>
       </c>
       <c r="AF4" s="54"/>
       <c r="AG4" s="1"/>
       <c r="AH4" s="55" t="s">
-        <v>185</v>
+        <v>182</v>
       </c>
       <c r="AI4" s="54"/>
       <c r="AJ4" s="1"/>
       <c r="AK4" s="55" t="s">
-        <v>186</v>
+        <v>183</v>
       </c>
       <c r="AL4" s="54"/>
       <c r="AM4" s="1"/>
       <c r="AN4" s="55" t="s">
-        <v>187</v>
+        <v>184</v>
       </c>
       <c r="AO4" s="54"/>
       <c r="AP4" s="1"/>
       <c r="AQ4" s="55" t="s">
-        <v>188</v>
+        <v>185</v>
       </c>
       <c r="AR4" s="54"/>
     </row>
     <row r="5" spans="1:44" x14ac:dyDescent="0.2">
       <c r="A5" s="38" t="s">
-        <v>189</v>
+        <v>186</v>
       </c>
       <c r="B5" s="39" t="s">
-        <v>190</v>
+        <v>187</v>
       </c>
       <c r="D5" s="38" t="s">
-        <v>189</v>
+        <v>186</v>
       </c>
       <c r="E5" s="39" t="s">
-        <v>190</v>
+        <v>187</v>
       </c>
       <c r="G5" s="38" t="s">
-        <v>189</v>
+        <v>186</v>
       </c>
       <c r="H5" s="39" t="s">
-        <v>190</v>
+        <v>187</v>
       </c>
       <c r="J5" s="38" t="s">
-        <v>189</v>
+        <v>186</v>
       </c>
       <c r="K5" s="39" t="s">
-        <v>190</v>
+        <v>187</v>
       </c>
       <c r="M5" s="38" t="s">
-        <v>189</v>
+        <v>186</v>
       </c>
       <c r="N5" s="39" t="s">
-        <v>190</v>
+        <v>187</v>
       </c>
       <c r="P5" s="38" t="s">
-        <v>189</v>
+        <v>186</v>
       </c>
       <c r="Q5" s="39" t="s">
-        <v>190</v>
+        <v>187</v>
       </c>
       <c r="R5" s="1"/>
       <c r="S5" s="38" t="s">
-        <v>189</v>
+        <v>186</v>
       </c>
       <c r="T5" s="39" t="s">
-        <v>190</v>
+        <v>187</v>
       </c>
       <c r="U5" s="1"/>
       <c r="V5" s="38" t="s">
-        <v>189</v>
+        <v>186</v>
       </c>
       <c r="W5" s="39" t="s">
-        <v>190</v>
+        <v>187</v>
       </c>
       <c r="X5" s="1"/>
       <c r="Y5" s="38" t="s">
-        <v>189</v>
+        <v>186</v>
       </c>
       <c r="Z5" s="39" t="s">
-        <v>190</v>
+        <v>187</v>
       </c>
       <c r="AA5" s="1"/>
       <c r="AB5" s="38" t="s">
-        <v>189</v>
+        <v>186</v>
       </c>
       <c r="AC5" s="39" t="s">
-        <v>190</v>
+        <v>187</v>
       </c>
       <c r="AE5" s="38" t="s">
-        <v>189</v>
+        <v>186</v>
       </c>
       <c r="AF5" s="39" t="s">
-        <v>190</v>
+        <v>187</v>
       </c>
       <c r="AG5" s="1"/>
       <c r="AH5" s="38" t="s">
-        <v>189</v>
+        <v>186</v>
       </c>
       <c r="AI5" s="39" t="s">
-        <v>190</v>
+        <v>187</v>
       </c>
       <c r="AJ5" s="1"/>
       <c r="AK5" s="38" t="s">
-        <v>189</v>
+        <v>186</v>
       </c>
       <c r="AL5" s="39" t="s">
-        <v>190</v>
+        <v>187</v>
       </c>
       <c r="AM5" s="1"/>
       <c r="AN5" s="38" t="s">
-        <v>189</v>
+        <v>186</v>
       </c>
       <c r="AO5" s="39" t="s">
-        <v>190</v>
+        <v>187</v>
       </c>
       <c r="AP5" s="1"/>
       <c r="AQ5" s="38" t="s">
-        <v>189</v>
+        <v>186</v>
       </c>
       <c r="AR5" s="39" t="s">
-        <v>190</v>
+        <v>187</v>
       </c>
     </row>
     <row r="6" spans="1:44" x14ac:dyDescent="0.2">
       <c r="A6" s="38" t="s">
-        <v>168</v>
+        <v>165</v>
       </c>
       <c r="B6" s="39">
         <v>1</v>
       </c>
       <c r="D6" s="38" t="s">
-        <v>168</v>
+        <v>165</v>
       </c>
       <c r="E6" s="39">
         <v>2</v>
       </c>
       <c r="G6" s="38" t="s">
-        <v>168</v>
+        <v>165</v>
       </c>
       <c r="H6" s="39">
         <v>3</v>
       </c>
       <c r="J6" s="38" t="s">
-        <v>168</v>
+        <v>165</v>
       </c>
       <c r="K6" s="39">
         <v>4</v>
       </c>
       <c r="M6" s="38" t="s">
-        <v>168</v>
+        <v>165</v>
       </c>
       <c r="N6" s="39">
         <v>5</v>
       </c>
       <c r="P6" s="38" t="s">
-        <v>168</v>
+        <v>165</v>
       </c>
       <c r="Q6" s="39">
         <v>6</v>
       </c>
       <c r="R6" s="1"/>
       <c r="S6" s="38" t="s">
-        <v>168</v>
+        <v>165</v>
       </c>
       <c r="T6" s="39">
         <v>7</v>
       </c>
       <c r="U6" s="1"/>
       <c r="V6" s="38" t="s">
-        <v>168</v>
+        <v>165</v>
       </c>
       <c r="W6" s="39">
         <v>8</v>
       </c>
       <c r="X6" s="1"/>
       <c r="Y6" s="38" t="s">
-        <v>168</v>
+        <v>165</v>
       </c>
       <c r="Z6" s="39">
         <v>9</v>
       </c>
       <c r="AA6" s="1"/>
       <c r="AB6" s="38" t="s">
-        <v>168</v>
+        <v>165</v>
       </c>
       <c r="AC6" s="39">
         <v>10</v>
       </c>
       <c r="AE6" s="38" t="s">
-        <v>168</v>
+        <v>165</v>
       </c>
       <c r="AF6" s="39">
         <v>11</v>
       </c>
       <c r="AG6" s="1"/>
       <c r="AH6" s="38" t="s">
-        <v>168</v>
+        <v>165</v>
       </c>
       <c r="AI6" s="39">
         <v>12</v>
       </c>
       <c r="AJ6" s="1"/>
       <c r="AK6" s="38" t="s">
-        <v>168</v>
+        <v>165</v>
       </c>
       <c r="AL6" s="39">
         <v>13</v>
       </c>
       <c r="AM6" s="1"/>
       <c r="AN6" s="38" t="s">
-        <v>168</v>
+        <v>165</v>
       </c>
       <c r="AO6" s="39">
         <v>14</v>
       </c>
       <c r="AP6" s="1"/>
       <c r="AQ6" s="38" t="s">
-        <v>168</v>
+        <v>165</v>
       </c>
       <c r="AR6" s="39">
         <v>15</v>
@@ -9631,172 +9702,172 @@
     </row>
     <row r="8" spans="1:44" x14ac:dyDescent="0.2">
       <c r="A8" s="38" t="s">
-        <v>169</v>
+        <v>166</v>
       </c>
       <c r="B8" s="39"/>
       <c r="D8" s="38" t="s">
-        <v>169</v>
+        <v>166</v>
       </c>
       <c r="E8" s="39"/>
       <c r="G8" s="38" t="s">
-        <v>169</v>
+        <v>166</v>
       </c>
       <c r="H8" s="39"/>
       <c r="J8" s="38" t="s">
-        <v>169</v>
+        <v>166</v>
       </c>
       <c r="K8" s="39"/>
       <c r="M8" s="38" t="s">
-        <v>169</v>
+        <v>166</v>
       </c>
       <c r="N8" s="39"/>
       <c r="P8" s="38" t="s">
-        <v>169</v>
+        <v>166</v>
       </c>
       <c r="Q8" s="39"/>
       <c r="R8" s="1"/>
       <c r="S8" s="38" t="s">
-        <v>169</v>
+        <v>166</v>
       </c>
       <c r="T8" s="39"/>
       <c r="U8" s="1"/>
       <c r="V8" s="38" t="s">
-        <v>169</v>
+        <v>166</v>
       </c>
       <c r="W8" s="39"/>
       <c r="X8" s="1"/>
       <c r="Y8" s="38" t="s">
-        <v>169</v>
+        <v>166</v>
       </c>
       <c r="Z8" s="39"/>
       <c r="AA8" s="1"/>
       <c r="AB8" s="38" t="s">
-        <v>169</v>
+        <v>166</v>
       </c>
       <c r="AC8" s="39"/>
       <c r="AE8" s="38" t="s">
-        <v>169</v>
+        <v>166</v>
       </c>
       <c r="AF8" s="39"/>
       <c r="AG8" s="1"/>
       <c r="AH8" s="38" t="s">
-        <v>169</v>
+        <v>166</v>
       </c>
       <c r="AI8" s="39"/>
       <c r="AJ8" s="1"/>
       <c r="AK8" s="38" t="s">
-        <v>169</v>
+        <v>166</v>
       </c>
       <c r="AL8" s="39"/>
       <c r="AM8" s="1"/>
       <c r="AN8" s="38" t="s">
-        <v>169</v>
+        <v>166</v>
       </c>
       <c r="AO8" s="39"/>
       <c r="AP8" s="1"/>
       <c r="AQ8" s="38" t="s">
-        <v>169</v>
+        <v>166</v>
       </c>
       <c r="AR8" s="39"/>
     </row>
     <row r="9" spans="1:44" x14ac:dyDescent="0.2">
       <c r="A9" s="2" t="s">
-        <v>170</v>
+        <v>167</v>
       </c>
       <c r="B9" s="2" t="s">
-        <v>171</v>
+        <v>168</v>
       </c>
       <c r="D9" s="2" t="s">
-        <v>170</v>
+        <v>167</v>
       </c>
       <c r="E9" s="2" t="s">
-        <v>171</v>
+        <v>168</v>
       </c>
       <c r="G9" s="2" t="s">
-        <v>170</v>
+        <v>167</v>
       </c>
       <c r="H9" s="2" t="s">
-        <v>171</v>
+        <v>168</v>
       </c>
       <c r="J9" s="2" t="s">
-        <v>170</v>
+        <v>167</v>
       </c>
       <c r="K9" s="2" t="s">
-        <v>171</v>
+        <v>168</v>
       </c>
       <c r="M9" s="2" t="s">
-        <v>170</v>
+        <v>167</v>
       </c>
       <c r="N9" s="2" t="s">
-        <v>171</v>
+        <v>168</v>
       </c>
       <c r="P9" s="2" t="s">
-        <v>170</v>
+        <v>167</v>
       </c>
       <c r="Q9" s="2" t="s">
-        <v>171</v>
+        <v>168</v>
       </c>
       <c r="R9" s="1"/>
       <c r="S9" s="2" t="s">
-        <v>170</v>
+        <v>167</v>
       </c>
       <c r="T9" s="2" t="s">
-        <v>171</v>
+        <v>168</v>
       </c>
       <c r="U9" s="1"/>
       <c r="V9" s="2" t="s">
-        <v>170</v>
+        <v>167</v>
       </c>
       <c r="W9" s="2" t="s">
-        <v>171</v>
+        <v>168</v>
       </c>
       <c r="X9" s="1"/>
       <c r="Y9" s="2" t="s">
-        <v>170</v>
+        <v>167</v>
       </c>
       <c r="Z9" s="2" t="s">
-        <v>171</v>
+        <v>168</v>
       </c>
       <c r="AA9" s="1"/>
       <c r="AB9" s="2" t="s">
-        <v>170</v>
+        <v>167</v>
       </c>
       <c r="AC9" s="2" t="s">
-        <v>171</v>
+        <v>168</v>
       </c>
       <c r="AE9" s="2" t="s">
-        <v>170</v>
+        <v>167</v>
       </c>
       <c r="AF9" s="2" t="s">
-        <v>171</v>
+        <v>168</v>
       </c>
       <c r="AG9" s="1"/>
       <c r="AH9" s="2" t="s">
-        <v>170</v>
+        <v>167</v>
       </c>
       <c r="AI9" s="2" t="s">
-        <v>171</v>
+        <v>168</v>
       </c>
       <c r="AJ9" s="1"/>
       <c r="AK9" s="2" t="s">
-        <v>170</v>
+        <v>167</v>
       </c>
       <c r="AL9" s="2" t="s">
-        <v>171</v>
+        <v>168</v>
       </c>
       <c r="AM9" s="1"/>
       <c r="AN9" s="2" t="s">
-        <v>170</v>
+        <v>167</v>
       </c>
       <c r="AO9" s="2" t="s">
-        <v>171</v>
+        <v>168</v>
       </c>
       <c r="AP9" s="1"/>
       <c r="AQ9" s="2" t="s">
-        <v>170</v>
+        <v>167</v>
       </c>
       <c r="AR9" s="2" t="s">
-        <v>171</v>
+        <v>168</v>
       </c>
     </row>
     <row r="10" spans="1:44" x14ac:dyDescent="0.2">
@@ -10601,36 +10672,36 @@
     </row>
   </sheetData>
   <mergeCells count="30">
-    <mergeCell ref="AN7:AO7"/>
-    <mergeCell ref="M4:N4"/>
-    <mergeCell ref="S4:T4"/>
-    <mergeCell ref="AE4:AF4"/>
     <mergeCell ref="AQ7:AR7"/>
     <mergeCell ref="AN4:AO4"/>
     <mergeCell ref="AH4:AI4"/>
-    <mergeCell ref="A7:B7"/>
-    <mergeCell ref="G7:H7"/>
-    <mergeCell ref="S7:T7"/>
-    <mergeCell ref="M7:N7"/>
-    <mergeCell ref="J4:K4"/>
     <mergeCell ref="Y7:Z7"/>
-    <mergeCell ref="D7:E7"/>
-    <mergeCell ref="P7:Q7"/>
-    <mergeCell ref="J7:K7"/>
-    <mergeCell ref="D4:E4"/>
     <mergeCell ref="AQ4:AR4"/>
-    <mergeCell ref="A4:B4"/>
-    <mergeCell ref="G4:H4"/>
-    <mergeCell ref="P4:Q4"/>
     <mergeCell ref="Y4:Z4"/>
     <mergeCell ref="AE7:AF7"/>
     <mergeCell ref="AK7:AL7"/>
     <mergeCell ref="AB4:AC4"/>
     <mergeCell ref="AK4:AL4"/>
+    <mergeCell ref="A4:B4"/>
+    <mergeCell ref="G4:H4"/>
+    <mergeCell ref="P4:Q4"/>
+    <mergeCell ref="AN7:AO7"/>
+    <mergeCell ref="M4:N4"/>
+    <mergeCell ref="S4:T4"/>
+    <mergeCell ref="AE4:AF4"/>
     <mergeCell ref="V4:W4"/>
     <mergeCell ref="V7:W7"/>
+    <mergeCell ref="J4:K4"/>
+    <mergeCell ref="D7:E7"/>
+    <mergeCell ref="P7:Q7"/>
+    <mergeCell ref="J7:K7"/>
+    <mergeCell ref="D4:E4"/>
     <mergeCell ref="AB7:AC7"/>
     <mergeCell ref="AH7:AI7"/>
+    <mergeCell ref="A7:B7"/>
+    <mergeCell ref="G7:H7"/>
+    <mergeCell ref="S7:T7"/>
+    <mergeCell ref="M7:N7"/>
   </mergeCells>
   <conditionalFormatting sqref="B6 A7:B7">
     <cfRule type="expression" dxfId="17" priority="1">
@@ -10727,43 +10798,43 @@
   <sheetData>
     <row r="2" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A2" s="59" t="s">
-        <v>191</v>
+        <v>188</v>
       </c>
       <c r="B2" s="54"/>
       <c r="D2" s="60" t="s">
-        <v>192</v>
+        <v>189</v>
       </c>
       <c r="E2" s="54"/>
       <c r="G2" s="22" t="s">
-        <v>193</v>
+        <v>190</v>
       </c>
     </row>
     <row r="3" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A3" s="32" t="s">
-        <v>189</v>
+        <v>186</v>
       </c>
       <c r="B3" s="33"/>
       <c r="D3" s="34" t="s">
-        <v>189</v>
+        <v>186</v>
       </c>
       <c r="E3" s="35"/>
       <c r="G3" s="22"/>
     </row>
     <row r="4" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A4" s="2" t="s">
-        <v>170</v>
+        <v>167</v>
       </c>
       <c r="B4" s="2" t="s">
-        <v>171</v>
+        <v>168</v>
       </c>
       <c r="D4" s="2" t="s">
-        <v>170</v>
+        <v>167</v>
       </c>
       <c r="E4" s="2" t="s">
-        <v>171</v>
+        <v>168</v>
       </c>
       <c r="G4" s="6" t="s">
-        <v>194</v>
+        <v>191</v>
       </c>
       <c r="H4" s="1"/>
     </row>
@@ -10776,7 +10847,7 @@
         <v>18</v>
       </c>
       <c r="H5" t="s">
-        <v>195</v>
+        <v>192</v>
       </c>
     </row>
     <row r="6" spans="1:8" x14ac:dyDescent="0.2">
@@ -10785,10 +10856,10 @@
       <c r="D6" s="3"/>
       <c r="E6" s="3"/>
       <c r="G6" s="1" t="s">
-        <v>196</v>
+        <v>193</v>
       </c>
       <c r="H6" t="s">
-        <v>197</v>
+        <v>194</v>
       </c>
     </row>
     <row r="7" spans="1:8" x14ac:dyDescent="0.2">
@@ -10925,31 +10996,31 @@
   <sheetData>
     <row r="2" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A2" s="13" t="s">
+        <v>195</v>
+      </c>
+      <c r="B2" s="13" t="s">
+        <v>196</v>
+      </c>
+      <c r="C2" s="13" t="s">
+        <v>197</v>
+      </c>
+      <c r="D2" s="13" t="s">
         <v>198</v>
       </c>
-      <c r="B2" s="13" t="s">
+      <c r="E2" s="13" t="s">
         <v>199</v>
       </c>
-      <c r="C2" s="13" t="s">
+      <c r="F2" s="13" t="s">
         <v>200</v>
       </c>
-      <c r="D2" s="13" t="s">
+      <c r="G2" s="13" t="s">
         <v>201</v>
       </c>
-      <c r="E2" s="13" t="s">
+      <c r="H2" s="13" t="s">
         <v>202</v>
       </c>
-      <c r="F2" s="13" t="s">
+      <c r="J2" s="5" t="s">
         <v>203</v>
-      </c>
-      <c r="G2" s="13" t="s">
-        <v>204</v>
-      </c>
-      <c r="H2" s="13" t="s">
-        <v>205</v>
-      </c>
-      <c r="J2" s="5" t="s">
-        <v>206</v>
       </c>
       <c r="K2" s="10" t="s">
         <v>5</v>
@@ -10967,10 +11038,10 @@
       <c r="G3" s="3"/>
       <c r="H3" s="3"/>
       <c r="J3" s="1" t="s">
-        <v>202</v>
+        <v>199</v>
       </c>
       <c r="K3" s="9" t="s">
-        <v>207</v>
+        <v>204</v>
       </c>
     </row>
     <row r="4" spans="1:14" x14ac:dyDescent="0.2">
@@ -10985,10 +11056,10 @@
       <c r="G4" s="3"/>
       <c r="H4" s="3"/>
       <c r="J4" s="1" t="s">
-        <v>208</v>
+        <v>205</v>
       </c>
       <c r="K4" s="9" t="s">
-        <v>209</v>
+        <v>206</v>
       </c>
     </row>
     <row r="5" spans="1:14" x14ac:dyDescent="0.2">
@@ -11003,10 +11074,10 @@
       <c r="G5" s="3"/>
       <c r="H5" s="3"/>
       <c r="J5" s="1" t="s">
-        <v>210</v>
+        <v>207</v>
       </c>
       <c r="K5" t="s">
-        <v>211</v>
+        <v>208</v>
       </c>
     </row>
     <row r="6" spans="1:14" x14ac:dyDescent="0.2">
@@ -11033,7 +11104,7 @@
       <c r="G7" s="3"/>
       <c r="H7" s="3"/>
       <c r="J7" s="5" t="s">
-        <v>212</v>
+        <v>209</v>
       </c>
     </row>
     <row r="8" spans="1:14" x14ac:dyDescent="0.2">
@@ -11048,7 +11119,7 @@
       <c r="G8" s="3"/>
       <c r="H8" s="3"/>
       <c r="J8" s="14" t="s">
-        <v>213</v>
+        <v>210</v>
       </c>
     </row>
     <row r="9" spans="1:14" x14ac:dyDescent="0.2">
@@ -11063,7 +11134,7 @@
       <c r="G9" s="3"/>
       <c r="H9" s="3"/>
       <c r="J9" s="14" t="s">
-        <v>214</v>
+        <v>211</v>
       </c>
     </row>
     <row r="10" spans="1:14" x14ac:dyDescent="0.2">
@@ -11078,7 +11149,7 @@
       <c r="G10" s="3"/>
       <c r="H10" s="3"/>
       <c r="J10" s="14" t="s">
-        <v>215</v>
+        <v>212</v>
       </c>
     </row>
     <row r="11" spans="1:14" x14ac:dyDescent="0.2">
@@ -11093,7 +11164,7 @@
       <c r="G11" s="3"/>
       <c r="H11" s="3"/>
       <c r="J11" s="14" t="s">
-        <v>216</v>
+        <v>213</v>
       </c>
     </row>
     <row r="12" spans="1:14" x14ac:dyDescent="0.2">
@@ -11108,27 +11179,27 @@
       <c r="G12" s="3"/>
       <c r="H12" s="3"/>
       <c r="J12" s="14" t="s">
-        <v>217</v>
+        <v>214</v>
       </c>
     </row>
     <row r="13" spans="1:14" x14ac:dyDescent="0.2">
       <c r="J13" s="14" t="s">
-        <v>218</v>
+        <v>215</v>
       </c>
     </row>
     <row r="14" spans="1:14" x14ac:dyDescent="0.2">
       <c r="J14" s="14" t="s">
-        <v>219</v>
+        <v>216</v>
       </c>
     </row>
     <row r="15" spans="1:14" x14ac:dyDescent="0.2">
       <c r="J15" s="14" t="s">
-        <v>220</v>
+        <v>217</v>
       </c>
     </row>
     <row r="16" spans="1:14" x14ac:dyDescent="0.2">
       <c r="J16" s="14" t="s">
-        <v>221</v>
+        <v>218</v>
       </c>
       <c r="K16" s="1"/>
       <c r="L16" s="1"/>
@@ -11137,7 +11208,7 @@
     </row>
     <row r="17" spans="10:10" x14ac:dyDescent="0.2">
       <c r="J17" s="14" t="s">
-        <v>222</v>
+        <v>219</v>
       </c>
     </row>
   </sheetData>
@@ -11177,16 +11248,16 @@
   <sheetData>
     <row r="2" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A2" s="11" t="s">
-        <v>223</v>
+        <v>220</v>
       </c>
       <c r="B2" s="11" t="s">
-        <v>224</v>
+        <v>221</v>
       </c>
       <c r="C2" s="12" t="s">
-        <v>225</v>
+        <v>222</v>
       </c>
       <c r="E2" s="6" t="s">
-        <v>206</v>
+        <v>203</v>
       </c>
       <c r="F2" s="6" t="s">
         <v>5</v>
@@ -11197,10 +11268,10 @@
       <c r="B3" s="3"/>
       <c r="C3" s="3"/>
       <c r="E3" t="s">
-        <v>226</v>
+        <v>223</v>
       </c>
       <c r="F3" t="s">
-        <v>227</v>
+        <v>224</v>
       </c>
     </row>
     <row r="4" spans="1:6" x14ac:dyDescent="0.2">
@@ -11208,10 +11279,10 @@
       <c r="B4" s="3"/>
       <c r="C4" s="3"/>
       <c r="E4" t="s">
-        <v>228</v>
+        <v>225</v>
       </c>
       <c r="F4" t="s">
-        <v>229</v>
+        <v>226</v>
       </c>
     </row>
     <row r="5" spans="1:6" x14ac:dyDescent="0.2">
@@ -11219,10 +11290,10 @@
       <c r="B5" s="3"/>
       <c r="C5" s="3"/>
       <c r="E5" t="s">
-        <v>230</v>
+        <v>227</v>
       </c>
       <c r="F5" t="s">
-        <v>231</v>
+        <v>228</v>
       </c>
     </row>
     <row r="6" spans="1:6" x14ac:dyDescent="0.2">
@@ -11352,122 +11423,122 @@
     </row>
     <row r="4" spans="2:24" x14ac:dyDescent="0.2">
       <c r="B4" s="61" t="s">
-        <v>232</v>
+        <v>229</v>
       </c>
       <c r="C4" s="62"/>
       <c r="D4" s="62"/>
       <c r="F4" s="61" t="s">
-        <v>233</v>
+        <v>230</v>
       </c>
       <c r="G4" s="62"/>
       <c r="H4" s="62"/>
       <c r="J4" s="61" t="s">
-        <v>234</v>
+        <v>231</v>
       </c>
       <c r="K4" s="62"/>
       <c r="L4" s="62"/>
       <c r="N4" s="61" t="s">
-        <v>235</v>
+        <v>232</v>
       </c>
       <c r="O4" s="62"/>
       <c r="P4" s="62"/>
       <c r="R4" s="61" t="s">
-        <v>236</v>
+        <v>233</v>
       </c>
       <c r="S4" s="62"/>
       <c r="T4" s="62"/>
       <c r="V4" s="61" t="s">
-        <v>237</v>
+        <v>234</v>
       </c>
       <c r="W4" s="62"/>
       <c r="X4" s="62"/>
     </row>
     <row r="5" spans="2:24" x14ac:dyDescent="0.2">
       <c r="B5" s="58" t="s">
-        <v>238</v>
+        <v>235</v>
       </c>
       <c r="C5" s="57"/>
       <c r="D5" s="39"/>
       <c r="F5" s="58" t="s">
-        <v>238</v>
+        <v>235</v>
       </c>
       <c r="G5" s="57"/>
       <c r="H5" s="39"/>
       <c r="J5" s="58" t="s">
-        <v>238</v>
+        <v>235</v>
       </c>
       <c r="K5" s="57"/>
       <c r="L5" s="39"/>
       <c r="N5" s="58" t="s">
-        <v>238</v>
+        <v>235</v>
       </c>
       <c r="O5" s="57"/>
       <c r="P5" s="39"/>
       <c r="R5" s="58" t="s">
-        <v>238</v>
+        <v>235</v>
       </c>
       <c r="S5" s="57"/>
       <c r="T5" s="39"/>
       <c r="V5" s="58" t="s">
-        <v>238</v>
+        <v>235</v>
       </c>
       <c r="W5" s="57"/>
       <c r="X5" s="39"/>
     </row>
     <row r="6" spans="2:24" x14ac:dyDescent="0.2">
       <c r="B6" s="2" t="s">
-        <v>223</v>
+        <v>220</v>
       </c>
       <c r="C6" s="2" t="s">
-        <v>224</v>
+        <v>221</v>
       </c>
       <c r="D6" s="2" t="s">
-        <v>239</v>
+        <v>236</v>
       </c>
       <c r="F6" s="2" t="s">
-        <v>223</v>
+        <v>220</v>
       </c>
       <c r="G6" s="2" t="s">
-        <v>224</v>
+        <v>221</v>
       </c>
       <c r="H6" s="2" t="s">
-        <v>239</v>
+        <v>236</v>
       </c>
       <c r="J6" s="2" t="s">
-        <v>223</v>
+        <v>220</v>
       </c>
       <c r="K6" s="2" t="s">
-        <v>224</v>
+        <v>221</v>
       </c>
       <c r="L6" s="2" t="s">
-        <v>239</v>
+        <v>236</v>
       </c>
       <c r="N6" s="2" t="s">
-        <v>223</v>
+        <v>220</v>
       </c>
       <c r="O6" s="2" t="s">
-        <v>224</v>
+        <v>221</v>
       </c>
       <c r="P6" s="2" t="s">
-        <v>239</v>
+        <v>236</v>
       </c>
       <c r="R6" s="2" t="s">
-        <v>223</v>
+        <v>220</v>
       </c>
       <c r="S6" s="2" t="s">
-        <v>224</v>
+        <v>221</v>
       </c>
       <c r="T6" s="2" t="s">
-        <v>239</v>
+        <v>236</v>
       </c>
       <c r="V6" s="2" t="s">
-        <v>223</v>
+        <v>220</v>
       </c>
       <c r="W6" s="2" t="s">
-        <v>224</v>
+        <v>221</v>
       </c>
       <c r="X6" s="2" t="s">
-        <v>239</v>
+        <v>236</v>
       </c>
     </row>
     <row r="7" spans="2:24" x14ac:dyDescent="0.2">
@@ -11852,6 +11923,10 @@
     </row>
   </sheetData>
   <mergeCells count="12">
+    <mergeCell ref="B5:C5"/>
+    <mergeCell ref="F5:G5"/>
+    <mergeCell ref="R4:T4"/>
+    <mergeCell ref="B4:D4"/>
     <mergeCell ref="V5:W5"/>
     <mergeCell ref="F4:H4"/>
     <mergeCell ref="V4:X4"/>
@@ -11860,10 +11935,6 @@
     <mergeCell ref="N5:O5"/>
     <mergeCell ref="R5:S5"/>
     <mergeCell ref="J5:K5"/>
-    <mergeCell ref="B5:C5"/>
-    <mergeCell ref="F5:G5"/>
-    <mergeCell ref="R4:T4"/>
-    <mergeCell ref="B4:D4"/>
   </mergeCells>
   <dataValidations count="1">
     <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="D5 H5 L5 P5 T5 X5" xr:uid="{00000000-0002-0000-0700-000000000000}">
@@ -11901,122 +11972,122 @@
     </row>
     <row r="4" spans="2:24" x14ac:dyDescent="0.2">
       <c r="B4" s="63" t="s">
-        <v>240</v>
+        <v>237</v>
       </c>
       <c r="C4" s="62"/>
       <c r="D4" s="62"/>
       <c r="F4" s="63" t="s">
-        <v>241</v>
+        <v>238</v>
       </c>
       <c r="G4" s="62"/>
       <c r="H4" s="62"/>
       <c r="J4" s="63" t="s">
-        <v>242</v>
+        <v>239</v>
       </c>
       <c r="K4" s="62"/>
       <c r="L4" s="62"/>
       <c r="N4" s="63" t="s">
-        <v>243</v>
+        <v>240</v>
       </c>
       <c r="O4" s="62"/>
       <c r="P4" s="62"/>
       <c r="R4" s="63" t="s">
-        <v>244</v>
+        <v>241</v>
       </c>
       <c r="S4" s="62"/>
       <c r="T4" s="62"/>
       <c r="V4" s="63" t="s">
-        <v>245</v>
+        <v>242</v>
       </c>
       <c r="W4" s="62"/>
       <c r="X4" s="62"/>
     </row>
     <row r="5" spans="2:24" x14ac:dyDescent="0.2">
       <c r="B5" s="58" t="s">
-        <v>238</v>
+        <v>235</v>
       </c>
       <c r="C5" s="57"/>
       <c r="D5" s="39"/>
       <c r="F5" s="58" t="s">
-        <v>238</v>
+        <v>235</v>
       </c>
       <c r="G5" s="57"/>
       <c r="H5" s="39"/>
       <c r="J5" s="58" t="s">
-        <v>238</v>
+        <v>235</v>
       </c>
       <c r="K5" s="57"/>
       <c r="L5" s="39"/>
       <c r="N5" s="58" t="s">
-        <v>238</v>
+        <v>235</v>
       </c>
       <c r="O5" s="57"/>
       <c r="P5" s="39"/>
       <c r="R5" s="58" t="s">
-        <v>238</v>
+        <v>235</v>
       </c>
       <c r="S5" s="57"/>
       <c r="T5" s="39"/>
       <c r="V5" s="58" t="s">
-        <v>238</v>
+        <v>235</v>
       </c>
       <c r="W5" s="57"/>
       <c r="X5" s="39"/>
     </row>
     <row r="6" spans="2:24" x14ac:dyDescent="0.2">
       <c r="B6" s="2" t="s">
-        <v>223</v>
+        <v>220</v>
       </c>
       <c r="C6" s="2" t="s">
-        <v>224</v>
+        <v>221</v>
       </c>
       <c r="D6" s="2" t="s">
-        <v>239</v>
+        <v>236</v>
       </c>
       <c r="F6" s="2" t="s">
-        <v>223</v>
+        <v>220</v>
       </c>
       <c r="G6" s="2" t="s">
-        <v>224</v>
+        <v>221</v>
       </c>
       <c r="H6" s="2" t="s">
-        <v>239</v>
+        <v>236</v>
       </c>
       <c r="J6" s="2" t="s">
-        <v>223</v>
+        <v>220</v>
       </c>
       <c r="K6" s="2" t="s">
-        <v>224</v>
+        <v>221</v>
       </c>
       <c r="L6" s="2" t="s">
-        <v>239</v>
+        <v>236</v>
       </c>
       <c r="N6" s="2" t="s">
-        <v>223</v>
+        <v>220</v>
       </c>
       <c r="O6" s="2" t="s">
-        <v>224</v>
+        <v>221</v>
       </c>
       <c r="P6" s="2" t="s">
-        <v>239</v>
+        <v>236</v>
       </c>
       <c r="R6" s="2" t="s">
-        <v>223</v>
+        <v>220</v>
       </c>
       <c r="S6" s="2" t="s">
-        <v>224</v>
+        <v>221</v>
       </c>
       <c r="T6" s="2" t="s">
-        <v>239</v>
+        <v>236</v>
       </c>
       <c r="V6" s="2" t="s">
-        <v>223</v>
+        <v>220</v>
       </c>
       <c r="W6" s="2" t="s">
-        <v>224</v>
+        <v>221</v>
       </c>
       <c r="X6" s="2" t="s">
-        <v>239</v>
+        <v>236</v>
       </c>
     </row>
     <row r="7" spans="2:24" x14ac:dyDescent="0.2">
@@ -12401,6 +12472,10 @@
     </row>
   </sheetData>
   <mergeCells count="12">
+    <mergeCell ref="B5:C5"/>
+    <mergeCell ref="F5:G5"/>
+    <mergeCell ref="R4:T4"/>
+    <mergeCell ref="B4:D4"/>
     <mergeCell ref="V5:W5"/>
     <mergeCell ref="F4:H4"/>
     <mergeCell ref="V4:X4"/>
@@ -12409,10 +12484,6 @@
     <mergeCell ref="N5:O5"/>
     <mergeCell ref="R5:S5"/>
     <mergeCell ref="J5:K5"/>
-    <mergeCell ref="B5:C5"/>
-    <mergeCell ref="F5:G5"/>
-    <mergeCell ref="R4:T4"/>
-    <mergeCell ref="B4:D4"/>
   </mergeCells>
   <dataValidations count="1">
     <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="D5 H5 L5 P5 T5 X5" xr:uid="{00000000-0002-0000-0800-000000000000}">

</xml_diff>

<commit_message>
docs(inputs): template v25 master; v23 and v24 archived beside it
Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01XjjT2aBxw8gY7EFdpoUcpj
</commit_message>
<xml_diff>
--- a/docs/inputs/input_template.xlsx
+++ b/docs/inputs/input_template.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/njones/python_projects/xslope/docs/inputs/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{41C0E255-0472-174F-97B1-AC3DD61E05E3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BD1F2F76-FB33-0143-929F-736B2B93C722}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="18260" yWindow="3440" windowWidth="44060" windowHeight="18400" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="4560" yWindow="4320" windowWidth="46940" windowHeight="18400" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="main" sheetId="1" r:id="rId1"/>
@@ -59,7 +59,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="595" uniqueCount="312">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="599" uniqueCount="316">
   <si>
     <t>XSLOPE Input Template</t>
   </si>
@@ -875,9 +875,6 @@
   </si>
   <si>
     <t>I</t>
-  </si>
-  <si>
-    <t>Fixity</t>
   </si>
   <si>
     <t>P</t>
@@ -1116,6 +1113,21 @@
   </si>
   <si>
     <t>yr</t>
+  </si>
+  <si>
+    <t>Adhesion</t>
+  </si>
+  <si>
+    <t>Delta</t>
+  </si>
+  <si>
+    <t>1D element size:</t>
+  </si>
+  <si>
+    <t>Head</t>
+  </si>
+  <si>
+    <t>Tip</t>
   </si>
 </sst>
 </file>
@@ -1886,16 +1898,16 @@
 <xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
   <xdr:twoCellAnchor>
     <xdr:from>
-      <xdr:col>18</xdr:col>
+      <xdr:col>20</xdr:col>
       <xdr:colOff>217714</xdr:colOff>
       <xdr:row>1</xdr:row>
       <xdr:rowOff>54430</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>23</xdr:col>
-      <xdr:colOff>199571</xdr:colOff>
-      <xdr:row>20</xdr:row>
-      <xdr:rowOff>9071</xdr:rowOff>
+      <xdr:col>25</xdr:col>
+      <xdr:colOff>444500</xdr:colOff>
+      <xdr:row>21</xdr:row>
+      <xdr:rowOff>90714</xdr:rowOff>
     </xdr:to>
     <xdr:sp macro="" textlink="">
       <xdr:nvSpPr>
@@ -1910,8 +1922,8 @@
       </xdr:nvSpPr>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="14804571" y="254001"/>
-          <a:ext cx="3610429" cy="3746499"/>
+          <a:off x="16455571" y="254001"/>
+          <a:ext cx="3855358" cy="4027713"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -2035,6 +2047,31 @@
         <a:p>
           <a:r>
             <a:rPr lang="en-US" sz="1100" b="1"/>
+            <a:t>Adhesion</a:t>
+          </a:r>
+          <a:r>
+            <a:rPr lang="en-US" sz="1100" b="0"/>
+            <a:t> = soii-reinforcement interface adhesion (blank</a:t>
+          </a:r>
+          <a:r>
+            <a:rPr lang="en-US" sz="1100" b="0" baseline="0"/>
+            <a:t> = use Lp)</a:t>
+          </a:r>
+        </a:p>
+        <a:p>
+          <a:r>
+            <a:rPr lang="en-US" sz="1100" b="1" baseline="0"/>
+            <a:t>Delta</a:t>
+          </a:r>
+          <a:r>
+            <a:rPr lang="en-US" sz="1100" b="0" baseline="0"/>
+            <a:t> = soil-reinforcement interface friction angle (blank = use Lp)</a:t>
+          </a:r>
+          <a:endParaRPr lang="en-US" sz="1100" b="0"/>
+        </a:p>
+        <a:p>
+          <a:r>
+            <a:rPr lang="en-US" sz="1100" b="1"/>
             <a:t>Tend1, Tend2 </a:t>
           </a:r>
           <a:r>
@@ -2081,6 +2118,10 @@
             <a:rPr lang="en-US" sz="1100" b="0"/>
             <a:t> = cross-sectional area of reinforcement (FEM only)</a:t>
           </a:r>
+          <a:br>
+            <a:rPr lang="en-US" sz="1100" b="0"/>
+          </a:br>
+          <a:endParaRPr lang="en-US" sz="1100" b="0"/>
         </a:p>
       </xdr:txBody>
     </xdr:sp>
@@ -2093,16 +2134,16 @@
 <xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
   <xdr:twoCellAnchor>
     <xdr:from>
-      <xdr:col>16</xdr:col>
-      <xdr:colOff>308429</xdr:colOff>
+      <xdr:col>17</xdr:col>
+      <xdr:colOff>290286</xdr:colOff>
       <xdr:row>0</xdr:row>
-      <xdr:rowOff>190499</xdr:rowOff>
+      <xdr:rowOff>126999</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>20</xdr:col>
-      <xdr:colOff>571501</xdr:colOff>
-      <xdr:row>12</xdr:row>
-      <xdr:rowOff>145143</xdr:rowOff>
+      <xdr:col>21</xdr:col>
+      <xdr:colOff>553358</xdr:colOff>
+      <xdr:row>13</xdr:row>
+      <xdr:rowOff>54428</xdr:rowOff>
     </xdr:to>
     <xdr:sp macro="" textlink="">
       <xdr:nvSpPr>
@@ -2117,8 +2158,8 @@
       </xdr:nvSpPr>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="13398500" y="190499"/>
-          <a:ext cx="3156858" cy="2349501"/>
+          <a:off x="14205857" y="126999"/>
+          <a:ext cx="3156858" cy="2521858"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -2423,7 +2464,7 @@
               <a:ea typeface="+mn-ea"/>
               <a:cs typeface="+mn-cs"/>
             </a:rPr>
-            <a:t>Fixity</a:t>
+            <a:t>Head</a:t>
           </a:r>
           <a:r>
             <a:rPr lang="en-US" sz="1100" b="0" i="0" baseline="0">
@@ -2435,8 +2476,54 @@
               <a:ea typeface="+mn-ea"/>
               <a:cs typeface="+mn-cs"/>
             </a:rPr>
-            <a:t> = Pile head status (fixed or free)</a:t>
+            <a:t> = Pile head fixity status (fixed or free)</a:t>
           </a:r>
+        </a:p>
+        <a:p>
+          <a:pPr marL="0" marR="0" lvl="0" indent="0" defTabSz="914400" eaLnBrk="1" fontAlgn="auto" latinLnBrk="0" hangingPunct="1">
+            <a:lnSpc>
+              <a:spcPct val="100000"/>
+            </a:lnSpc>
+            <a:spcBef>
+              <a:spcPts val="0"/>
+            </a:spcBef>
+            <a:spcAft>
+              <a:spcPts val="0"/>
+            </a:spcAft>
+            <a:buClrTx/>
+            <a:buSzTx/>
+            <a:buFontTx/>
+            <a:buNone/>
+            <a:tabLst/>
+            <a:defRPr/>
+          </a:pPr>
+          <a:r>
+            <a:rPr lang="en-US" sz="1100" b="1" i="0" baseline="0">
+              <a:solidFill>
+                <a:schemeClr val="dk1"/>
+              </a:solidFill>
+              <a:effectLst/>
+              <a:latin typeface="+mn-lt"/>
+              <a:ea typeface="+mn-ea"/>
+              <a:cs typeface="+mn-cs"/>
+            </a:rPr>
+            <a:t>Tip</a:t>
+          </a:r>
+          <a:r>
+            <a:rPr lang="en-US" sz="1100" b="0" i="0" baseline="0">
+              <a:solidFill>
+                <a:schemeClr val="dk1"/>
+              </a:solidFill>
+              <a:effectLst/>
+              <a:latin typeface="+mn-lt"/>
+              <a:ea typeface="+mn-ea"/>
+              <a:cs typeface="+mn-cs"/>
+            </a:rPr>
+            <a:t> = Pile tip fixity status (fixed or free)</a:t>
+          </a:r>
+          <a:endParaRPr lang="en-US" sz="1100"/>
+        </a:p>
+        <a:p>
           <a:endParaRPr lang="en-US" sz="1100"/>
         </a:p>
       </xdr:txBody>
@@ -2788,7 +2875,7 @@
         <v>2</v>
       </c>
       <c r="D5" s="30">
-        <v>23</v>
+        <v>25</v>
       </c>
     </row>
     <row r="7" spans="1:7" x14ac:dyDescent="0.2">
@@ -2961,7 +3048,7 @@
     </row>
     <row r="20" spans="2:7" x14ac:dyDescent="0.2">
       <c r="C20" s="14" t="s">
-        <v>45</v>
+        <v>313</v>
       </c>
       <c r="F20" s="1" t="s">
         <v>46</v>
@@ -2972,7 +3059,7 @@
     </row>
     <row r="21" spans="2:7" x14ac:dyDescent="0.2">
       <c r="C21" s="14" t="s">
-        <v>48</v>
+        <v>45</v>
       </c>
       <c r="F21" s="1" t="s">
         <v>49</v>
@@ -2983,25 +3070,30 @@
     </row>
     <row r="22" spans="2:7" x14ac:dyDescent="0.2">
       <c r="C22" s="14" t="s">
-        <v>51</v>
-      </c>
-      <c r="D22" s="1" t="s">
-        <v>52</v>
+        <v>48</v>
       </c>
       <c r="F22" s="1"/>
     </row>
     <row r="23" spans="2:7" x14ac:dyDescent="0.2">
       <c r="B23" s="1"/>
       <c r="C23" s="14" t="s">
-        <v>53</v>
+        <v>51</v>
       </c>
       <c r="D23" s="1" t="s">
-        <v>54</v>
+        <v>52</v>
       </c>
     </row>
     <row r="24" spans="2:7" x14ac:dyDescent="0.2">
       <c r="B24" s="1"/>
       <c r="C24" s="14" t="s">
+        <v>53</v>
+      </c>
+      <c r="D24" s="1" t="s">
+        <v>54</v>
+      </c>
+    </row>
+    <row r="25" spans="2:7" x14ac:dyDescent="0.2">
+      <c r="C25" s="14" t="s">
         <v>55</v>
       </c>
     </row>
@@ -3047,7 +3139,7 @@
     </row>
     <row r="58" spans="4:4" x14ac:dyDescent="0.2">
       <c r="D58" s="1" t="s">
-        <v>311</v>
+        <v>310</v>
       </c>
     </row>
     <row r="60" spans="4:4" x14ac:dyDescent="0.2">
@@ -3145,7 +3237,7 @@
     <mergeCell ref="B7:D7"/>
   </mergeCells>
   <dataValidations count="8">
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="D22" xr:uid="{00000000-0002-0000-0000-000000000000}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="D23" xr:uid="{00000000-0002-0000-0000-000000000000}">
       <formula1>"rollers,fixed"</formula1>
     </dataValidation>
     <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="D8" xr:uid="{00000000-0002-0000-0000-000001000000}">
@@ -3163,10 +3255,10 @@
     <dataValidation type="list" allowBlank="1" sqref="D18" xr:uid="{00000000-0002-0000-0000-000005000000}">
       <formula1>$D$75:$D$79</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="D23" xr:uid="{00000000-0002-0000-0000-000006000000}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="D24" xr:uid="{00000000-0002-0000-0000-000006000000}">
       <formula1>"auto,manual"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" sqref="D24" xr:uid="{00000000-0002-0000-0000-000007000000}">
+    <dataValidation type="list" allowBlank="1" sqref="D25" xr:uid="{00000000-0002-0000-0000-000007000000}">
       <formula1>"circular,non-circular"</formula1>
     </dataValidation>
   </dataValidations>
@@ -3176,18 +3268,18 @@
 
 <file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0900-000000000000}">
-  <dimension ref="A2:AB25"/>
+  <dimension ref="A2:AD25"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="4.83203125" style="1" customWidth="1"/>
     <col min="2" max="6" width="10.83203125" style="1" customWidth="1"/>
     <col min="7" max="7" width="13.1640625" customWidth="1"/>
-    <col min="10" max="12" width="10.83203125" style="1" customWidth="1"/>
-    <col min="16" max="18" width="10.83203125" style="1" customWidth="1"/>
-    <col min="19" max="19" width="4.33203125" customWidth="1"/>
+    <col min="10" max="14" width="10.83203125" style="1" customWidth="1"/>
+    <col min="18" max="20" width="10.83203125" style="1" customWidth="1"/>
+    <col min="21" max="21" width="4.33203125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="2" spans="1:28" x14ac:dyDescent="0.2">
+    <row r="2" spans="1:30" x14ac:dyDescent="0.2">
       <c r="A2" s="12" t="s">
         <v>194</v>
       </c>
@@ -3225,34 +3317,40 @@
         <v>252</v>
       </c>
       <c r="M2" s="27" t="s">
+        <v>311</v>
+      </c>
+      <c r="N2" s="27" t="s">
+        <v>312</v>
+      </c>
+      <c r="O2" s="27" t="s">
         <v>253</v>
       </c>
-      <c r="N2" s="27" t="s">
+      <c r="P2" s="27" t="s">
         <v>254</v>
       </c>
-      <c r="O2" s="27" t="s">
+      <c r="Q2" s="27" t="s">
         <v>255</v>
       </c>
-      <c r="P2" s="28" t="s">
+      <c r="R2" s="28" t="s">
         <v>256</v>
       </c>
-      <c r="Q2" s="28" t="s">
+      <c r="S2" s="28" t="s">
         <v>122</v>
       </c>
-      <c r="R2" s="28" t="s">
+      <c r="T2" s="28" t="s">
         <v>257</v>
       </c>
-      <c r="Z2" t="s">
+      <c r="AB2" t="s">
         <v>258</v>
       </c>
-      <c r="AA2" t="s">
+      <c r="AC2" t="s">
         <v>259</v>
       </c>
-      <c r="AB2" t="s">
+      <c r="AD2" t="s">
         <v>260</v>
       </c>
     </row>
-    <row r="3" spans="1:28" x14ac:dyDescent="0.2">
+    <row r="3" spans="1:30" x14ac:dyDescent="0.2">
       <c r="A3" s="3">
         <v>1</v>
       </c>
@@ -3263,11 +3361,11 @@
       <c r="F3" s="3"/>
       <c r="G3" s="3"/>
       <c r="H3" s="3" t="str">
-        <f t="shared" ref="H3:H22" si="0">IF($G3="","",IFERROR(VLOOKUP($G3,$Z$8:$AB$11,2,0),""))</f>
+        <f t="shared" ref="H3:H22" si="0">IF($G3="","",IFERROR(VLOOKUP($G3,$AB$8:$AD$11,2,0),""))</f>
         <v/>
       </c>
       <c r="I3" s="3" t="str">
-        <f t="shared" ref="I3:I22" si="1">IF($G3="","",IFERROR(VLOOKUP($G3,$Z$8:$AB$11,3,0),""))</f>
+        <f t="shared" ref="I3:I22" si="1">IF($G3="","",IFERROR(VLOOKUP($G3,$AB$8:$AD$11,3,0),""))</f>
         <v/>
       </c>
       <c r="J3" s="3"/>
@@ -3279,17 +3377,19 @@
       <c r="P3" s="3"/>
       <c r="Q3" s="3"/>
       <c r="R3" s="3"/>
-      <c r="Z3" t="s">
+      <c r="S3" s="3"/>
+      <c r="T3" s="3"/>
+      <c r="AB3" t="s">
         <v>261</v>
       </c>
-      <c r="AA3" t="s">
+      <c r="AC3" t="s">
         <v>262</v>
       </c>
-      <c r="AB3" t="s">
+      <c r="AD3" t="s">
         <v>263</v>
       </c>
     </row>
-    <row r="4" spans="1:28" x14ac:dyDescent="0.2">
+    <row r="4" spans="1:30" x14ac:dyDescent="0.2">
       <c r="A4" s="3">
         <v>2</v>
       </c>
@@ -3316,11 +3416,13 @@
       <c r="P4" s="3"/>
       <c r="Q4" s="3"/>
       <c r="R4" s="3"/>
-      <c r="Z4" t="s">
+      <c r="S4" s="3"/>
+      <c r="T4" s="3"/>
+      <c r="AB4" t="s">
         <v>264</v>
       </c>
     </row>
-    <row r="5" spans="1:28" x14ac:dyDescent="0.2">
+    <row r="5" spans="1:30" x14ac:dyDescent="0.2">
       <c r="A5" s="3">
         <v>3</v>
       </c>
@@ -3347,11 +3449,13 @@
       <c r="P5" s="3"/>
       <c r="Q5" s="3"/>
       <c r="R5" s="3"/>
-      <c r="Z5" t="s">
+      <c r="S5" s="3"/>
+      <c r="T5" s="3"/>
+      <c r="AB5" t="s">
         <v>265</v>
       </c>
     </row>
-    <row r="6" spans="1:28" x14ac:dyDescent="0.2">
+    <row r="6" spans="1:30" x14ac:dyDescent="0.2">
       <c r="A6" s="3">
         <v>4</v>
       </c>
@@ -3378,8 +3482,10 @@
       <c r="P6" s="3"/>
       <c r="Q6" s="3"/>
       <c r="R6" s="3"/>
-    </row>
-    <row r="7" spans="1:28" x14ac:dyDescent="0.2">
+      <c r="S6" s="3"/>
+      <c r="T6" s="3"/>
+    </row>
+    <row r="7" spans="1:30" x14ac:dyDescent="0.2">
       <c r="A7" s="3">
         <v>5</v>
       </c>
@@ -3406,8 +3512,10 @@
       <c r="P7" s="3"/>
       <c r="Q7" s="3"/>
       <c r="R7" s="3"/>
-    </row>
-    <row r="8" spans="1:28" x14ac:dyDescent="0.2">
+      <c r="S7" s="3"/>
+      <c r="T7" s="3"/>
+    </row>
+    <row r="8" spans="1:30" x14ac:dyDescent="0.2">
       <c r="A8" s="3">
         <v>6</v>
       </c>
@@ -3434,17 +3542,19 @@
       <c r="P8" s="3"/>
       <c r="Q8" s="3"/>
       <c r="R8" s="3"/>
-      <c r="Z8" t="s">
+      <c r="S8" s="3"/>
+      <c r="T8" s="3"/>
+      <c r="AB8" t="s">
         <v>258</v>
       </c>
-      <c r="AA8" t="s">
+      <c r="AC8" t="s">
         <v>259</v>
       </c>
-      <c r="AB8" t="s">
+      <c r="AD8" t="s">
         <v>260</v>
       </c>
     </row>
-    <row r="9" spans="1:28" x14ac:dyDescent="0.2">
+    <row r="9" spans="1:30" x14ac:dyDescent="0.2">
       <c r="A9" s="3">
         <v>7</v>
       </c>
@@ -3471,17 +3581,19 @@
       <c r="P9" s="3"/>
       <c r="Q9" s="3"/>
       <c r="R9" s="3"/>
-      <c r="Z9" t="s">
+      <c r="S9" s="3"/>
+      <c r="T9" s="3"/>
+      <c r="AB9" t="s">
         <v>261</v>
       </c>
-      <c r="AA9" t="s">
+      <c r="AC9" t="s">
         <v>262</v>
       </c>
-      <c r="AB9" t="s">
+      <c r="AD9" t="s">
         <v>263</v>
       </c>
     </row>
-    <row r="10" spans="1:28" x14ac:dyDescent="0.2">
+    <row r="10" spans="1:30" x14ac:dyDescent="0.2">
       <c r="A10" s="3">
         <v>8</v>
       </c>
@@ -3508,17 +3620,19 @@
       <c r="P10" s="3"/>
       <c r="Q10" s="3"/>
       <c r="R10" s="3"/>
-      <c r="Z10" t="s">
+      <c r="S10" s="3"/>
+      <c r="T10" s="3"/>
+      <c r="AB10" t="s">
         <v>264</v>
       </c>
-      <c r="AA10" t="s">
+      <c r="AC10" t="s">
         <v>262</v>
       </c>
-      <c r="AB10" t="s">
+      <c r="AD10" t="s">
         <v>260</v>
       </c>
     </row>
-    <row r="11" spans="1:28" x14ac:dyDescent="0.2">
+    <row r="11" spans="1:30" x14ac:dyDescent="0.2">
       <c r="A11" s="3">
         <v>9</v>
       </c>
@@ -3545,17 +3659,19 @@
       <c r="P11" s="3"/>
       <c r="Q11" s="3"/>
       <c r="R11" s="3"/>
-      <c r="Z11" t="s">
+      <c r="S11" s="3"/>
+      <c r="T11" s="3"/>
+      <c r="AB11" t="s">
         <v>265</v>
       </c>
-      <c r="AA11" t="s">
+      <c r="AC11" t="s">
         <v>262</v>
       </c>
-      <c r="AB11" t="s">
+      <c r="AD11" t="s">
         <v>260</v>
       </c>
     </row>
-    <row r="12" spans="1:28" x14ac:dyDescent="0.2">
+    <row r="12" spans="1:30" x14ac:dyDescent="0.2">
       <c r="A12" s="3">
         <v>10</v>
       </c>
@@ -3582,8 +3698,10 @@
       <c r="P12" s="3"/>
       <c r="Q12" s="3"/>
       <c r="R12" s="3"/>
-    </row>
-    <row r="13" spans="1:28" x14ac:dyDescent="0.2">
+      <c r="S12" s="3"/>
+      <c r="T12" s="3"/>
+    </row>
+    <row r="13" spans="1:30" x14ac:dyDescent="0.2">
       <c r="A13" s="3">
         <v>11</v>
       </c>
@@ -3610,8 +3728,10 @@
       <c r="P13" s="3"/>
       <c r="Q13" s="3"/>
       <c r="R13" s="3"/>
-    </row>
-    <row r="14" spans="1:28" x14ac:dyDescent="0.2">
+      <c r="S13" s="3"/>
+      <c r="T13" s="3"/>
+    </row>
+    <row r="14" spans="1:30" x14ac:dyDescent="0.2">
       <c r="A14" s="3">
         <v>12</v>
       </c>
@@ -3638,8 +3758,10 @@
       <c r="P14" s="3"/>
       <c r="Q14" s="3"/>
       <c r="R14" s="3"/>
-    </row>
-    <row r="15" spans="1:28" x14ac:dyDescent="0.2">
+      <c r="S14" s="3"/>
+      <c r="T14" s="3"/>
+    </row>
+    <row r="15" spans="1:30" x14ac:dyDescent="0.2">
       <c r="A15" s="3">
         <v>13</v>
       </c>
@@ -3666,8 +3788,10 @@
       <c r="P15" s="3"/>
       <c r="Q15" s="3"/>
       <c r="R15" s="3"/>
-    </row>
-    <row r="16" spans="1:28" x14ac:dyDescent="0.2">
+      <c r="S15" s="3"/>
+      <c r="T15" s="3"/>
+    </row>
+    <row r="16" spans="1:30" x14ac:dyDescent="0.2">
       <c r="A16" s="3">
         <v>14</v>
       </c>
@@ -3694,8 +3818,10 @@
       <c r="P16" s="3"/>
       <c r="Q16" s="3"/>
       <c r="R16" s="3"/>
-    </row>
-    <row r="17" spans="1:21" x14ac:dyDescent="0.2">
+      <c r="S16" s="3"/>
+      <c r="T16" s="3"/>
+    </row>
+    <row r="17" spans="1:23" x14ac:dyDescent="0.2">
       <c r="A17" s="3">
         <v>15</v>
       </c>
@@ -3722,8 +3848,10 @@
       <c r="P17" s="3"/>
       <c r="Q17" s="3"/>
       <c r="R17" s="3"/>
-    </row>
-    <row r="18" spans="1:21" x14ac:dyDescent="0.2">
+      <c r="S17" s="3"/>
+      <c r="T17" s="3"/>
+    </row>
+    <row r="18" spans="1:23" x14ac:dyDescent="0.2">
       <c r="A18" s="3">
         <v>16</v>
       </c>
@@ -3750,8 +3878,10 @@
       <c r="P18" s="3"/>
       <c r="Q18" s="3"/>
       <c r="R18" s="3"/>
-    </row>
-    <row r="19" spans="1:21" x14ac:dyDescent="0.2">
+      <c r="S18" s="3"/>
+      <c r="T18" s="3"/>
+    </row>
+    <row r="19" spans="1:23" x14ac:dyDescent="0.2">
       <c r="A19" s="3">
         <v>17</v>
       </c>
@@ -3778,8 +3908,10 @@
       <c r="P19" s="3"/>
       <c r="Q19" s="3"/>
       <c r="R19" s="3"/>
-    </row>
-    <row r="20" spans="1:21" x14ac:dyDescent="0.2">
+      <c r="S19" s="3"/>
+      <c r="T19" s="3"/>
+    </row>
+    <row r="20" spans="1:23" x14ac:dyDescent="0.2">
       <c r="A20" s="3">
         <v>18</v>
       </c>
@@ -3806,8 +3938,10 @@
       <c r="P20" s="3"/>
       <c r="Q20" s="3"/>
       <c r="R20" s="3"/>
-    </row>
-    <row r="21" spans="1:21" x14ac:dyDescent="0.2">
+      <c r="S20" s="3"/>
+      <c r="T20" s="3"/>
+    </row>
+    <row r="21" spans="1:23" x14ac:dyDescent="0.2">
       <c r="A21" s="3">
         <v>19</v>
       </c>
@@ -3834,8 +3968,10 @@
       <c r="P21" s="3"/>
       <c r="Q21" s="3"/>
       <c r="R21" s="3"/>
-    </row>
-    <row r="22" spans="1:21" x14ac:dyDescent="0.2">
+      <c r="S21" s="3"/>
+      <c r="T21" s="3"/>
+    </row>
+    <row r="22" spans="1:23" x14ac:dyDescent="0.2">
       <c r="A22" s="3">
         <v>20</v>
       </c>
@@ -3862,39 +3998,41 @@
       <c r="P22" s="3"/>
       <c r="Q22" s="3"/>
       <c r="R22" s="3"/>
-    </row>
-    <row r="23" spans="1:21" x14ac:dyDescent="0.2">
-      <c r="T23" s="42"/>
-      <c r="U23" t="s">
+      <c r="S22" s="3"/>
+      <c r="T22" s="3"/>
+    </row>
+    <row r="23" spans="1:23" x14ac:dyDescent="0.2">
+      <c r="V23" s="42"/>
+      <c r="W23" t="s">
         <v>91</v>
       </c>
     </row>
-    <row r="24" spans="1:21" x14ac:dyDescent="0.2">
+    <row r="24" spans="1:23" x14ac:dyDescent="0.2">
       <c r="K24" s="9"/>
       <c r="L24" s="9"/>
-      <c r="T24" s="26"/>
-      <c r="U24" s="9" t="s">
+      <c r="V24" s="26"/>
+      <c r="W24" s="9" t="s">
         <v>97</v>
       </c>
     </row>
-    <row r="25" spans="1:21" x14ac:dyDescent="0.2">
+    <row r="25" spans="1:23" x14ac:dyDescent="0.2">
       <c r="K25" s="9"/>
       <c r="L25" s="9"/>
-      <c r="T25" s="29"/>
-      <c r="U25" s="9" t="s">
+      <c r="V25" s="29"/>
+      <c r="W25" s="9" t="s">
         <v>104</v>
       </c>
     </row>
   </sheetData>
   <dataValidations count="3">
     <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="G3:G22" xr:uid="{00000000-0002-0000-0900-000000000000}">
-      <formula1>$Z$2:$Z$5</formula1>
+      <formula1>$AB$2:$AB$5</formula1>
     </dataValidation>
     <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="H3:H22" xr:uid="{00000000-0002-0000-0900-000001000000}">
-      <formula1>$AA$2:$AA$3</formula1>
+      <formula1>$AC$2:$AC$3</formula1>
     </dataValidation>
     <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="I3:I22" xr:uid="{00000000-0002-0000-0900-000002000000}">
-      <formula1>$AB$2:$AB$3</formula1>
+      <formula1>$AD$2:$AD$3</formula1>
     </dataValidation>
   </dataValidations>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -3904,18 +4042,18 @@
 
 <file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0A00-000000000000}">
-  <dimension ref="A2:Z17"/>
+  <dimension ref="A2:AA17"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="4.83203125" style="1" customWidth="1"/>
     <col min="2" max="2" width="11.5" style="1" customWidth="1"/>
     <col min="3" max="7" width="10.83203125" style="1" customWidth="1"/>
     <col min="8" max="8" width="14.5" customWidth="1"/>
-    <col min="9" max="16" width="10.83203125" style="1" customWidth="1"/>
-    <col min="17" max="17" width="5.5" customWidth="1"/>
+    <col min="9" max="17" width="10.83203125" style="1" customWidth="1"/>
+    <col min="18" max="18" width="5.5" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="2" spans="1:26" x14ac:dyDescent="0.2">
+    <row r="2" spans="1:27" x14ac:dyDescent="0.2">
       <c r="A2" s="12" t="s">
         <v>194</v>
       </c>
@@ -3962,16 +4100,19 @@
         <v>257</v>
       </c>
       <c r="P2" s="28" t="s">
-        <v>272</v>
-      </c>
-      <c r="Y2" t="s">
+        <v>314</v>
+      </c>
+      <c r="Q2" s="28" t="s">
+        <v>315</v>
+      </c>
+      <c r="Z2" t="s">
         <v>222</v>
       </c>
-      <c r="Z2" t="s">
+      <c r="AA2" t="s">
         <v>260</v>
       </c>
     </row>
-    <row r="3" spans="1:26" x14ac:dyDescent="0.2">
+    <row r="3" spans="1:27" x14ac:dyDescent="0.2">
       <c r="A3" s="3">
         <v>1</v>
       </c>
@@ -3990,14 +4131,15 @@
       <c r="N3" s="3"/>
       <c r="O3" s="3"/>
       <c r="P3" s="3"/>
-      <c r="Y3" t="s">
+      <c r="Q3" s="3"/>
+      <c r="Z3" t="s">
         <v>226</v>
       </c>
-      <c r="Z3" t="s">
+      <c r="AA3" t="s">
         <v>263</v>
       </c>
     </row>
-    <row r="4" spans="1:26" x14ac:dyDescent="0.2">
+    <row r="4" spans="1:27" x14ac:dyDescent="0.2">
       <c r="A4" s="3">
         <v>2</v>
       </c>
@@ -4016,8 +4158,9 @@
       <c r="N4" s="3"/>
       <c r="O4" s="3"/>
       <c r="P4" s="3"/>
-    </row>
-    <row r="5" spans="1:26" x14ac:dyDescent="0.2">
+      <c r="Q4" s="3"/>
+    </row>
+    <row r="5" spans="1:27" x14ac:dyDescent="0.2">
       <c r="A5" s="3">
         <v>3</v>
       </c>
@@ -4036,8 +4179,9 @@
       <c r="N5" s="3"/>
       <c r="O5" s="3"/>
       <c r="P5" s="3"/>
-    </row>
-    <row r="6" spans="1:26" x14ac:dyDescent="0.2">
+      <c r="Q5" s="3"/>
+    </row>
+    <row r="6" spans="1:27" x14ac:dyDescent="0.2">
       <c r="A6" s="3">
         <v>4</v>
       </c>
@@ -4056,8 +4200,9 @@
       <c r="N6" s="3"/>
       <c r="O6" s="3"/>
       <c r="P6" s="3"/>
-    </row>
-    <row r="7" spans="1:26" x14ac:dyDescent="0.2">
+      <c r="Q6" s="3"/>
+    </row>
+    <row r="7" spans="1:27" x14ac:dyDescent="0.2">
       <c r="A7" s="3">
         <v>5</v>
       </c>
@@ -4076,8 +4221,9 @@
       <c r="N7" s="3"/>
       <c r="O7" s="3"/>
       <c r="P7" s="3"/>
-    </row>
-    <row r="8" spans="1:26" x14ac:dyDescent="0.2">
+      <c r="Q7" s="3"/>
+    </row>
+    <row r="8" spans="1:27" x14ac:dyDescent="0.2">
       <c r="A8" s="3">
         <v>6</v>
       </c>
@@ -4096,8 +4242,9 @@
       <c r="N8" s="3"/>
       <c r="O8" s="3"/>
       <c r="P8" s="3"/>
-    </row>
-    <row r="9" spans="1:26" x14ac:dyDescent="0.2">
+      <c r="Q8" s="3"/>
+    </row>
+    <row r="9" spans="1:27" x14ac:dyDescent="0.2">
       <c r="A9" s="3">
         <v>7</v>
       </c>
@@ -4116,8 +4263,9 @@
       <c r="N9" s="3"/>
       <c r="O9" s="3"/>
       <c r="P9" s="3"/>
-    </row>
-    <row r="10" spans="1:26" x14ac:dyDescent="0.2">
+      <c r="Q9" s="3"/>
+    </row>
+    <row r="10" spans="1:27" x14ac:dyDescent="0.2">
       <c r="A10" s="3">
         <v>8</v>
       </c>
@@ -4136,8 +4284,9 @@
       <c r="N10" s="3"/>
       <c r="O10" s="3"/>
       <c r="P10" s="3"/>
-    </row>
-    <row r="11" spans="1:26" x14ac:dyDescent="0.2">
+      <c r="Q10" s="3"/>
+    </row>
+    <row r="11" spans="1:27" x14ac:dyDescent="0.2">
       <c r="A11" s="3">
         <v>9</v>
       </c>
@@ -4156,8 +4305,9 @@
       <c r="N11" s="3"/>
       <c r="O11" s="3"/>
       <c r="P11" s="3"/>
-    </row>
-    <row r="12" spans="1:26" x14ac:dyDescent="0.2">
+      <c r="Q11" s="3"/>
+    </row>
+    <row r="12" spans="1:27" x14ac:dyDescent="0.2">
       <c r="A12" s="3">
         <v>10</v>
       </c>
@@ -4176,36 +4326,37 @@
       <c r="N12" s="3"/>
       <c r="O12" s="3"/>
       <c r="P12" s="3"/>
-    </row>
-    <row r="14" spans="1:26" x14ac:dyDescent="0.2">
+      <c r="Q12" s="3"/>
+    </row>
+    <row r="14" spans="1:27" x14ac:dyDescent="0.2">
       <c r="I14" s="9"/>
       <c r="J14" s="9"/>
     </row>
-    <row r="15" spans="1:26" x14ac:dyDescent="0.2">
-      <c r="R15" s="42"/>
-      <c r="S15" t="s">
+    <row r="15" spans="1:27" x14ac:dyDescent="0.2">
+      <c r="S15" s="42"/>
+      <c r="T15" t="s">
         <v>91</v>
       </c>
     </row>
-    <row r="16" spans="1:26" x14ac:dyDescent="0.2">
-      <c r="R16" s="26"/>
-      <c r="S16" s="9" t="s">
+    <row r="16" spans="1:27" x14ac:dyDescent="0.2">
+      <c r="S16" s="26"/>
+      <c r="T16" s="9" t="s">
         <v>97</v>
       </c>
     </row>
-    <row r="17" spans="18:19" x14ac:dyDescent="0.2">
-      <c r="R17" s="29"/>
-      <c r="S17" s="9" t="s">
+    <row r="17" spans="19:20" x14ac:dyDescent="0.2">
+      <c r="S17" s="29"/>
+      <c r="T17" s="9" t="s">
         <v>104</v>
       </c>
     </row>
   </sheetData>
   <dataValidations count="2">
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="P3:P12" xr:uid="{00000000-0002-0000-0A00-000000000000}">
-      <formula1>$Y$2:$Y$3</formula1>
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="P3:Q12" xr:uid="{00000000-0002-0000-0A00-000000000000}">
+      <formula1>$Z$2:$Z$3</formula1>
     </dataValidation>
     <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="H3:H12" xr:uid="{00000000-0002-0000-0A00-000001000000}">
-      <formula1>$Z$2:$Z$3</formula1>
+      <formula1>$AA$2:$AA$3</formula1>
     </dataValidation>
   </dataValidations>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -4237,10 +4388,10 @@
         <v>167</v>
       </c>
       <c r="E2" s="12" t="s">
+        <v>272</v>
+      </c>
+      <c r="F2" s="12" t="s">
         <v>273</v>
-      </c>
-      <c r="F2" s="12" t="s">
-        <v>274</v>
       </c>
     </row>
     <row r="3" spans="1:6" x14ac:dyDescent="0.2">
@@ -4463,27 +4614,27 @@
   <sheetData>
     <row r="2" spans="2:21" x14ac:dyDescent="0.2">
       <c r="B2" s="64" t="s">
-        <v>275</v>
+        <v>274</v>
       </c>
       <c r="C2" s="65"/>
       <c r="E2" s="59" t="s">
-        <v>276</v>
+        <v>275</v>
       </c>
       <c r="F2" s="54"/>
       <c r="H2" s="59" t="s">
-        <v>277</v>
+        <v>276</v>
       </c>
       <c r="I2" s="54"/>
       <c r="K2" s="59" t="s">
-        <v>278</v>
+        <v>277</v>
       </c>
       <c r="L2" s="54"/>
       <c r="N2" s="59" t="s">
-        <v>279</v>
+        <v>278</v>
       </c>
       <c r="O2" s="54"/>
       <c r="Q2" s="59" t="s">
-        <v>280</v>
+        <v>279</v>
       </c>
       <c r="R2" s="54"/>
     </row>
@@ -4491,27 +4642,27 @@
       <c r="B3" s="66"/>
       <c r="C3" s="67"/>
       <c r="E3" s="32" t="s">
-        <v>281</v>
+        <v>280</v>
       </c>
       <c r="F3" s="33"/>
       <c r="H3" s="32" t="s">
-        <v>281</v>
+        <v>280</v>
       </c>
       <c r="I3" s="33"/>
       <c r="K3" s="32" t="s">
-        <v>281</v>
+        <v>280</v>
       </c>
       <c r="L3" s="33"/>
       <c r="N3" s="32" t="s">
-        <v>281</v>
+        <v>280</v>
       </c>
       <c r="O3" s="33"/>
       <c r="Q3" s="32" t="s">
-        <v>281</v>
+        <v>280</v>
       </c>
       <c r="R3" s="33"/>
       <c r="T3" s="6" t="s">
-        <v>282</v>
+        <v>281</v>
       </c>
     </row>
     <row r="4" spans="2:21" x14ac:dyDescent="0.2">
@@ -4552,10 +4703,10 @@
         <v>167</v>
       </c>
       <c r="T4" s="1" t="s">
-        <v>281</v>
+        <v>280</v>
       </c>
       <c r="U4" t="s">
-        <v>283</v>
+        <v>282</v>
       </c>
     </row>
     <row r="5" spans="2:21" x14ac:dyDescent="0.2">
@@ -4572,10 +4723,10 @@
       <c r="Q5" s="3"/>
       <c r="R5" s="3"/>
       <c r="T5" s="1" t="s">
+        <v>283</v>
+      </c>
+      <c r="U5" t="s">
         <v>284</v>
-      </c>
-      <c r="U5" t="s">
-        <v>285</v>
       </c>
     </row>
     <row r="6" spans="2:21" x14ac:dyDescent="0.2">
@@ -4592,7 +4743,7 @@
       <c r="Q6" s="3"/>
       <c r="R6" s="3"/>
       <c r="T6" s="1" t="s">
-        <v>286</v>
+        <v>285</v>
       </c>
       <c r="U6" s="9"/>
     </row>
@@ -4881,27 +5032,27 @@
   <sheetData>
     <row r="2" spans="2:21" x14ac:dyDescent="0.2">
       <c r="B2" s="68" t="s">
-        <v>287</v>
+        <v>286</v>
       </c>
       <c r="C2" s="65"/>
       <c r="E2" s="60" t="s">
-        <v>288</v>
+        <v>287</v>
       </c>
       <c r="F2" s="54"/>
       <c r="H2" s="60" t="s">
-        <v>289</v>
+        <v>288</v>
       </c>
       <c r="I2" s="54"/>
       <c r="K2" s="60" t="s">
-        <v>290</v>
+        <v>289</v>
       </c>
       <c r="L2" s="54"/>
       <c r="N2" s="60" t="s">
-        <v>291</v>
+        <v>290</v>
       </c>
       <c r="O2" s="54"/>
       <c r="Q2" s="60" t="s">
-        <v>292</v>
+        <v>291</v>
       </c>
       <c r="R2" s="54"/>
     </row>
@@ -4909,27 +5060,27 @@
       <c r="B3" s="66"/>
       <c r="C3" s="67"/>
       <c r="E3" s="34" t="s">
-        <v>281</v>
+        <v>280</v>
       </c>
       <c r="F3" s="35"/>
       <c r="H3" s="34" t="s">
-        <v>281</v>
+        <v>280</v>
       </c>
       <c r="I3" s="35"/>
       <c r="K3" s="34" t="s">
-        <v>281</v>
+        <v>280</v>
       </c>
       <c r="L3" s="35"/>
       <c r="N3" s="34" t="s">
-        <v>281</v>
+        <v>280</v>
       </c>
       <c r="O3" s="35"/>
       <c r="Q3" s="34" t="s">
-        <v>281</v>
+        <v>280</v>
       </c>
       <c r="R3" s="35"/>
       <c r="T3" s="6" t="s">
-        <v>282</v>
+        <v>281</v>
       </c>
     </row>
     <row r="4" spans="2:21" x14ac:dyDescent="0.2">
@@ -4970,10 +5121,10 @@
         <v>167</v>
       </c>
       <c r="T4" s="1" t="s">
-        <v>281</v>
+        <v>280</v>
       </c>
       <c r="U4" t="s">
-        <v>283</v>
+        <v>282</v>
       </c>
     </row>
     <row r="5" spans="2:21" x14ac:dyDescent="0.2">
@@ -4990,10 +5141,10 @@
       <c r="Q5" s="3"/>
       <c r="R5" s="3"/>
       <c r="T5" s="1" t="s">
+        <v>283</v>
+      </c>
+      <c r="U5" t="s">
         <v>284</v>
-      </c>
-      <c r="U5" t="s">
-        <v>285</v>
       </c>
     </row>
     <row r="6" spans="2:21" x14ac:dyDescent="0.2">
@@ -5292,22 +5443,22 @@
   <sheetData>
     <row r="2" spans="2:10" x14ac:dyDescent="0.2">
       <c r="B2" s="50" t="s">
+        <v>292</v>
+      </c>
+      <c r="C2" s="50" t="s">
         <v>293</v>
       </c>
-      <c r="C2" s="50" t="s">
+      <c r="D2" s="50" t="s">
         <v>294</v>
       </c>
-      <c r="D2" s="50" t="s">
+      <c r="E2" s="50" t="s">
         <v>295</v>
       </c>
-      <c r="E2" s="50" t="s">
+      <c r="F2" s="50" t="s">
         <v>296</v>
       </c>
-      <c r="F2" s="50" t="s">
+      <c r="G2" s="50" t="s">
         <v>297</v>
-      </c>
-      <c r="G2" s="50" t="s">
-        <v>298</v>
       </c>
     </row>
     <row r="3" spans="2:10" x14ac:dyDescent="0.2">
@@ -5318,7 +5469,7 @@
       <c r="F3" s="3"/>
       <c r="G3" s="3"/>
       <c r="I3" s="14" t="s">
-        <v>299</v>
+        <v>298</v>
       </c>
       <c r="J3" s="3"/>
     </row>
@@ -5340,7 +5491,7 @@
       <c r="F5" s="3"/>
       <c r="G5" s="3"/>
       <c r="I5" s="14" t="s">
-        <v>300</v>
+        <v>299</v>
       </c>
       <c r="J5" s="3"/>
     </row>
@@ -5362,7 +5513,7 @@
       <c r="F7" s="3"/>
       <c r="G7" s="3"/>
       <c r="I7" s="14" t="s">
-        <v>301</v>
+        <v>300</v>
       </c>
       <c r="J7" s="3"/>
     </row>
@@ -5374,7 +5525,7 @@
       <c r="F8" s="3"/>
       <c r="G8" s="3"/>
       <c r="I8" s="14" t="s">
-        <v>302</v>
+        <v>301</v>
       </c>
       <c r="J8" s="3"/>
     </row>
@@ -5386,7 +5537,7 @@
       <c r="F9" s="3"/>
       <c r="G9" s="3"/>
       <c r="I9" s="14" t="s">
-        <v>303</v>
+        <v>302</v>
       </c>
       <c r="J9" s="3"/>
     </row>
@@ -5406,7 +5557,7 @@
       <c r="F11" s="3"/>
       <c r="G11" s="3"/>
       <c r="J11" t="s">
-        <v>304</v>
+        <v>303</v>
       </c>
     </row>
     <row r="12" spans="2:10" x14ac:dyDescent="0.2">
@@ -6401,7 +6552,7 @@
         <v>113</v>
       </c>
       <c r="D10" s="48" t="s">
-        <v>310</v>
+        <v>309</v>
       </c>
       <c r="E10" s="44" t="s">
         <v>114</v>
@@ -6470,22 +6621,22 @@
         <v>134</v>
       </c>
       <c r="AA10" s="46" t="s">
-        <v>306</v>
+        <v>305</v>
       </c>
       <c r="AB10" s="46" t="s">
-        <v>305</v>
+        <v>304</v>
       </c>
       <c r="AC10" s="47" t="s">
         <v>135</v>
       </c>
       <c r="AD10" s="46" t="s">
+        <v>306</v>
+      </c>
+      <c r="AE10" s="46" t="s">
         <v>307</v>
       </c>
-      <c r="AE10" s="46" t="s">
+      <c r="AF10" s="47" t="s">
         <v>308</v>
-      </c>
-      <c r="AF10" s="47" t="s">
-        <v>309</v>
       </c>
       <c r="AG10" s="23" t="s">
         <v>136</v>
@@ -10644,10 +10795,6 @@
     <mergeCell ref="AN7:AO7"/>
     <mergeCell ref="AH7:AI7"/>
     <mergeCell ref="AE4:AF4"/>
-    <mergeCell ref="V4:W4"/>
-    <mergeCell ref="V7:W7"/>
-    <mergeCell ref="P7:Q7"/>
-    <mergeCell ref="AB7:AC7"/>
     <mergeCell ref="A7:B7"/>
     <mergeCell ref="G7:H7"/>
     <mergeCell ref="S7:T7"/>
@@ -10661,6 +10808,10 @@
     <mergeCell ref="D4:E4"/>
     <mergeCell ref="M4:N4"/>
     <mergeCell ref="S4:T4"/>
+    <mergeCell ref="V4:W4"/>
+    <mergeCell ref="V7:W7"/>
+    <mergeCell ref="P7:Q7"/>
+    <mergeCell ref="AB7:AC7"/>
   </mergeCells>
   <conditionalFormatting sqref="B6 A7:B7">
     <cfRule type="expression" dxfId="17" priority="1">
@@ -11376,7 +11527,7 @@
   <sheetData>
     <row r="2" spans="2:24" x14ac:dyDescent="0.2">
       <c r="B2" t="str">
-        <f>IF(main!$D$23="auto","Enter non-water loads only — water loads derive automatically from the piezometric line / seepage boundary conditions.","")</f>
+        <f>IF(main!$D$24="auto","Enter non-water loads only — water loads derive automatically from the piezometric line / seepage boundary conditions.","")</f>
         <v>Enter non-water loads only — water loads derive automatically from the piezometric line / seepage boundary conditions.</v>
       </c>
     </row>
@@ -11925,7 +12076,7 @@
   <sheetData>
     <row r="2" spans="2:24" x14ac:dyDescent="0.2">
       <c r="B2" t="str">
-        <f>IF(main!$D$23="auto","Enter non-water loads only — water loads derive automatically from the piezometric line / seepage boundary conditions.","")</f>
+        <f>IF(main!$D$24="auto","Enter non-water loads only — water loads derive automatically from the piezometric line / seepage boundary conditions.","")</f>
         <v>Enter non-water loads only — water loads derive automatically from the piezometric line / seepage boundary conditions.</v>
       </c>
     </row>

</xml_diff>

<commit_message>
fem(piles): Tip takes free / pinned / fixed
free: the tip is restrained only by what surrounds it (soil, or the model
boundary it lands on); pinned: translations held, rotation free — a shaft
bearing on a hard stratum inside the mesh; fixed: translations and rotation
held — socketed into rock. Head keeps free / fixed. Template validation list
per Norm (v25, no version bump); packaged copy synced; loader, Studio editor,
skill and docs updated. Free and pinned are identical when the tip sits on the
base boundary, which is the tutorials' case.

Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01XjjT2aBxw8gY7EFdpoUcpj
</commit_message>
<xml_diff>
--- a/docs/inputs/input_template.xlsx
+++ b/docs/inputs/input_template.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/njones/python_projects/xslope/docs/inputs/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BD1F2F76-FB33-0143-929F-736B2B93C722}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5EE192E0-97C6-CB43-9291-6C4E11A86E6D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="4560" yWindow="4320" windowWidth="46940" windowHeight="18400" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -59,7 +59,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="599" uniqueCount="316">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="600" uniqueCount="317">
   <si>
     <t>XSLOPE Input Template</t>
   </si>
@@ -1128,6 +1128,9 @@
   </si>
   <si>
     <t>Tip</t>
+  </si>
+  <si>
+    <t>Pinned</t>
   </si>
 </sst>
 </file>
@@ -4133,7 +4136,7 @@
       <c r="P3" s="3"/>
       <c r="Q3" s="3"/>
       <c r="Z3" t="s">
-        <v>226</v>
+        <v>316</v>
       </c>
       <c r="AA3" t="s">
         <v>263</v>
@@ -4159,6 +4162,9 @@
       <c r="O4" s="3"/>
       <c r="P4" s="3"/>
       <c r="Q4" s="3"/>
+      <c r="Z4" t="s">
+        <v>226</v>
+      </c>
     </row>
     <row r="5" spans="1:27" x14ac:dyDescent="0.2">
       <c r="A5" s="3">
@@ -4352,11 +4358,11 @@
     </row>
   </sheetData>
   <dataValidations count="2">
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="P3:Q12" xr:uid="{00000000-0002-0000-0A00-000000000000}">
-      <formula1>$Z$2:$Z$3</formula1>
-    </dataValidation>
     <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="H3:H12" xr:uid="{00000000-0002-0000-0A00-000001000000}">
       <formula1>$AA$2:$AA$3</formula1>
+    </dataValidation>
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="P3:Q12" xr:uid="{00000000-0002-0000-0A00-000000000000}">
+      <formula1>$Z$2:$Z$4</formula1>
     </dataValidation>
   </dataValidations>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -9386,6 +9392,20 @@
     </row>
   </sheetData>
   <mergeCells count="30">
+    <mergeCell ref="D4:E4"/>
+    <mergeCell ref="P4:Q4"/>
+    <mergeCell ref="Y4:Z4"/>
+    <mergeCell ref="AB6:AC6"/>
+    <mergeCell ref="AN6:AO6"/>
+    <mergeCell ref="AB4:AC4"/>
+    <mergeCell ref="AN4:AO4"/>
+    <mergeCell ref="G6:H6"/>
+    <mergeCell ref="J4:K4"/>
+    <mergeCell ref="V6:W6"/>
+    <mergeCell ref="M6:N6"/>
+    <mergeCell ref="AH6:AI6"/>
+    <mergeCell ref="S6:T6"/>
+    <mergeCell ref="Y6:Z6"/>
     <mergeCell ref="AQ4:AR4"/>
     <mergeCell ref="A4:B4"/>
     <mergeCell ref="G4:H4"/>
@@ -9402,20 +9422,6 @@
     <mergeCell ref="AH4:AI4"/>
     <mergeCell ref="J6:K6"/>
     <mergeCell ref="P6:Q6"/>
-    <mergeCell ref="D4:E4"/>
-    <mergeCell ref="P4:Q4"/>
-    <mergeCell ref="Y4:Z4"/>
-    <mergeCell ref="AB6:AC6"/>
-    <mergeCell ref="AN6:AO6"/>
-    <mergeCell ref="AB4:AC4"/>
-    <mergeCell ref="AN4:AO4"/>
-    <mergeCell ref="G6:H6"/>
-    <mergeCell ref="J4:K4"/>
-    <mergeCell ref="V6:W6"/>
-    <mergeCell ref="M6:N6"/>
-    <mergeCell ref="AH6:AI6"/>
-    <mergeCell ref="S6:T6"/>
-    <mergeCell ref="Y6:Z6"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
@@ -10782,6 +10788,23 @@
     </row>
   </sheetData>
   <mergeCells count="30">
+    <mergeCell ref="V4:W4"/>
+    <mergeCell ref="V7:W7"/>
+    <mergeCell ref="P7:Q7"/>
+    <mergeCell ref="AB7:AC7"/>
+    <mergeCell ref="A7:B7"/>
+    <mergeCell ref="G7:H7"/>
+    <mergeCell ref="S7:T7"/>
+    <mergeCell ref="M7:N7"/>
+    <mergeCell ref="A4:B4"/>
+    <mergeCell ref="G4:H4"/>
+    <mergeCell ref="P4:Q4"/>
+    <mergeCell ref="J4:K4"/>
+    <mergeCell ref="D7:E7"/>
+    <mergeCell ref="J7:K7"/>
+    <mergeCell ref="D4:E4"/>
+    <mergeCell ref="M4:N4"/>
+    <mergeCell ref="S4:T4"/>
     <mergeCell ref="AQ7:AR7"/>
     <mergeCell ref="AN4:AO4"/>
     <mergeCell ref="AH4:AI4"/>
@@ -10795,23 +10818,6 @@
     <mergeCell ref="AN7:AO7"/>
     <mergeCell ref="AH7:AI7"/>
     <mergeCell ref="AE4:AF4"/>
-    <mergeCell ref="A7:B7"/>
-    <mergeCell ref="G7:H7"/>
-    <mergeCell ref="S7:T7"/>
-    <mergeCell ref="M7:N7"/>
-    <mergeCell ref="A4:B4"/>
-    <mergeCell ref="G4:H4"/>
-    <mergeCell ref="P4:Q4"/>
-    <mergeCell ref="J4:K4"/>
-    <mergeCell ref="D7:E7"/>
-    <mergeCell ref="J7:K7"/>
-    <mergeCell ref="D4:E4"/>
-    <mergeCell ref="M4:N4"/>
-    <mergeCell ref="S4:T4"/>
-    <mergeCell ref="V4:W4"/>
-    <mergeCell ref="V7:W7"/>
-    <mergeCell ref="P7:Q7"/>
-    <mergeCell ref="AB7:AC7"/>
   </mergeCells>
   <conditionalFormatting sqref="B6 A7:B7">
     <cfRule type="expression" dxfId="17" priority="1">

</xml_diff>

<commit_message>
fem(piles): Head and Tip each take free / pinned / unrotated / fixed — Cai & Ugai's four end conditions, the same at either end
pinned holds the translations, unrotated holds the rotation, fixed holds
both; free leaves the node to the soil or the boundary it sits on. Head
'fixed' had meant rotation only while Tip 'fixed' meant both — vp106c_fem_fix
now says Head = unrotated (the paper's condition for its 1.45), same run.
Template validation list per Norm (v25); packaged copy synced; loader,
Studio editor, skill, docs; verification page wording recertified.

Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01XjjT2aBxw8gY7EFdpoUcpj
</commit_message>
<xml_diff>
--- a/docs/inputs/input_template.xlsx
+++ b/docs/inputs/input_template.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/njones/python_projects/xslope/docs/inputs/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5EE192E0-97C6-CB43-9291-6C4E11A86E6D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{523500CF-89B8-4644-B955-31C74218CF4E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="4560" yWindow="4320" windowWidth="46940" windowHeight="18400" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -59,7 +59,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="600" uniqueCount="317">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="601" uniqueCount="318">
   <si>
     <t>XSLOPE Input Template</t>
   </si>
@@ -1131,6 +1131,9 @@
   </si>
   <si>
     <t>Pinned</t>
+  </si>
+  <si>
+    <t>Unrotated</t>
   </si>
 </sst>
 </file>
@@ -2479,7 +2482,7 @@
               <a:ea typeface="+mn-ea"/>
               <a:cs typeface="+mn-cs"/>
             </a:rPr>
-            <a:t> = Pile head fixity status (fixed or free)</a:t>
+            <a:t> = Pile head fixity status</a:t>
           </a:r>
         </a:p>
         <a:p>
@@ -2522,7 +2525,7 @@
               <a:ea typeface="+mn-ea"/>
               <a:cs typeface="+mn-cs"/>
             </a:rPr>
-            <a:t> = Pile tip fixity status (fixed or free)</a:t>
+            <a:t> = Pile tip fixity status</a:t>
           </a:r>
           <a:endParaRPr lang="en-US" sz="1100"/>
         </a:p>
@@ -4163,7 +4166,7 @@
       <c r="P4" s="3"/>
       <c r="Q4" s="3"/>
       <c r="Z4" t="s">
-        <v>226</v>
+        <v>317</v>
       </c>
     </row>
     <row r="5" spans="1:27" x14ac:dyDescent="0.2">
@@ -4186,6 +4189,9 @@
       <c r="O5" s="3"/>
       <c r="P5" s="3"/>
       <c r="Q5" s="3"/>
+      <c r="Z5" t="s">
+        <v>226</v>
+      </c>
     </row>
     <row r="6" spans="1:27" x14ac:dyDescent="0.2">
       <c r="A6" s="3">
@@ -4362,7 +4368,7 @@
       <formula1>$AA$2:$AA$3</formula1>
     </dataValidation>
     <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="P3:Q12" xr:uid="{00000000-0002-0000-0A00-000000000000}">
-      <formula1>$Z$2:$Z$4</formula1>
+      <formula1>$Z$2:$Z$5</formula1>
     </dataValidation>
   </dataValidations>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -9392,20 +9398,6 @@
     </row>
   </sheetData>
   <mergeCells count="30">
-    <mergeCell ref="D4:E4"/>
-    <mergeCell ref="P4:Q4"/>
-    <mergeCell ref="Y4:Z4"/>
-    <mergeCell ref="AB6:AC6"/>
-    <mergeCell ref="AN6:AO6"/>
-    <mergeCell ref="AB4:AC4"/>
-    <mergeCell ref="AN4:AO4"/>
-    <mergeCell ref="G6:H6"/>
-    <mergeCell ref="J4:K4"/>
-    <mergeCell ref="V6:W6"/>
-    <mergeCell ref="M6:N6"/>
-    <mergeCell ref="AH6:AI6"/>
-    <mergeCell ref="S6:T6"/>
-    <mergeCell ref="Y6:Z6"/>
     <mergeCell ref="AQ4:AR4"/>
     <mergeCell ref="A4:B4"/>
     <mergeCell ref="G4:H4"/>
@@ -9422,6 +9414,20 @@
     <mergeCell ref="AH4:AI4"/>
     <mergeCell ref="J6:K6"/>
     <mergeCell ref="P6:Q6"/>
+    <mergeCell ref="D4:E4"/>
+    <mergeCell ref="P4:Q4"/>
+    <mergeCell ref="Y4:Z4"/>
+    <mergeCell ref="AB6:AC6"/>
+    <mergeCell ref="AN6:AO6"/>
+    <mergeCell ref="AB4:AC4"/>
+    <mergeCell ref="AN4:AO4"/>
+    <mergeCell ref="G6:H6"/>
+    <mergeCell ref="J4:K4"/>
+    <mergeCell ref="V6:W6"/>
+    <mergeCell ref="M6:N6"/>
+    <mergeCell ref="AH6:AI6"/>
+    <mergeCell ref="S6:T6"/>
+    <mergeCell ref="Y6:Z6"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
@@ -10788,6 +10794,20 @@
     </row>
   </sheetData>
   <mergeCells count="30">
+    <mergeCell ref="S4:T4"/>
+    <mergeCell ref="AQ7:AR7"/>
+    <mergeCell ref="AN4:AO4"/>
+    <mergeCell ref="AH4:AI4"/>
+    <mergeCell ref="Y7:Z7"/>
+    <mergeCell ref="AQ4:AR4"/>
+    <mergeCell ref="Y4:Z4"/>
+    <mergeCell ref="AE7:AF7"/>
+    <mergeCell ref="AK7:AL7"/>
+    <mergeCell ref="AB4:AC4"/>
+    <mergeCell ref="AK4:AL4"/>
+    <mergeCell ref="AN7:AO7"/>
+    <mergeCell ref="AH7:AI7"/>
+    <mergeCell ref="AE4:AF4"/>
     <mergeCell ref="V4:W4"/>
     <mergeCell ref="V7:W7"/>
     <mergeCell ref="P7:Q7"/>
@@ -10804,20 +10824,6 @@
     <mergeCell ref="J7:K7"/>
     <mergeCell ref="D4:E4"/>
     <mergeCell ref="M4:N4"/>
-    <mergeCell ref="S4:T4"/>
-    <mergeCell ref="AQ7:AR7"/>
-    <mergeCell ref="AN4:AO4"/>
-    <mergeCell ref="AH4:AI4"/>
-    <mergeCell ref="Y7:Z7"/>
-    <mergeCell ref="AQ4:AR4"/>
-    <mergeCell ref="Y4:Z4"/>
-    <mergeCell ref="AE7:AF7"/>
-    <mergeCell ref="AK7:AL7"/>
-    <mergeCell ref="AB4:AC4"/>
-    <mergeCell ref="AK4:AL4"/>
-    <mergeCell ref="AN7:AO7"/>
-    <mergeCell ref="AH7:AI7"/>
-    <mergeCell ref="AE4:AF4"/>
   </mergeCells>
   <conditionalFormatting sqref="B6 A7:B7">
     <cfRule type="expression" dxfId="17" priority="1">

</xml_diff>

<commit_message>
docs(inputs): template v26 master (van Genuchten exponent l on the mat sheet); v25 archived beside it
Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01XjjT2aBxw8gY7EFdpoUcpj
</commit_message>
<xml_diff>
--- a/docs/inputs/input_template.xlsx
+++ b/docs/inputs/input_template.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10802"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10821"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/njones/python_projects/xslope/docs/inputs/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{523500CF-89B8-4644-B955-31C74218CF4E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E12967D2-A998-D342-B5ED-43CABE326A3A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="4560" yWindow="4320" windowWidth="46940" windowHeight="18400" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="15680" yWindow="4780" windowWidth="46940" windowHeight="18400" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="main" sheetId="1" r:id="rId1"/>
@@ -59,7 +59,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="601" uniqueCount="318">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="602" uniqueCount="319">
   <si>
     <t>XSLOPE Input Template</t>
   </si>
@@ -341,9 +341,6 @@
   </si>
   <si>
     <t>vg</t>
-  </si>
-  <si>
-    <t>van Genuchten model (a, n)</t>
   </si>
   <si>
     <t>pow</t>
@@ -1134,6 +1131,12 @@
   </si>
   <si>
     <t>Unrotated</t>
+  </si>
+  <si>
+    <t>van Genuchten model (a, n, l)</t>
+  </si>
+  <si>
+    <t>l</t>
   </si>
 </sst>
 </file>
@@ -2881,7 +2884,7 @@
         <v>2</v>
       </c>
       <c r="D5" s="30">
-        <v>25</v>
+        <v>26</v>
       </c>
     </row>
     <row r="7" spans="1:7" x14ac:dyDescent="0.2">
@@ -3054,7 +3057,7 @@
     </row>
     <row r="20" spans="2:7" x14ac:dyDescent="0.2">
       <c r="C20" s="14" t="s">
-        <v>313</v>
+        <v>312</v>
       </c>
       <c r="F20" s="1" t="s">
         <v>46</v>
@@ -3145,7 +3148,7 @@
     </row>
     <row r="58" spans="4:4" x14ac:dyDescent="0.2">
       <c r="D58" s="1" t="s">
-        <v>310</v>
+        <v>309</v>
       </c>
     </row>
     <row r="60" spans="4:4" x14ac:dyDescent="0.2">
@@ -3287,73 +3290,73 @@
   <sheetData>
     <row r="2" spans="1:30" x14ac:dyDescent="0.2">
       <c r="A2" s="12" t="s">
-        <v>194</v>
+        <v>193</v>
       </c>
       <c r="B2" s="12" t="s">
+        <v>241</v>
+      </c>
+      <c r="C2" s="12" t="s">
         <v>242</v>
       </c>
-      <c r="C2" s="12" t="s">
+      <c r="D2" s="12" t="s">
         <v>243</v>
       </c>
-      <c r="D2" s="12" t="s">
+      <c r="E2" s="12" t="s">
         <v>244</v>
       </c>
-      <c r="E2" s="12" t="s">
+      <c r="F2" s="12" t="s">
         <v>245</v>
       </c>
-      <c r="F2" s="12" t="s">
+      <c r="G2" s="40" t="s">
         <v>246</v>
       </c>
-      <c r="G2" s="40" t="s">
+      <c r="H2" s="40" t="s">
         <v>247</v>
       </c>
-      <c r="H2" s="40" t="s">
+      <c r="I2" s="40" t="s">
         <v>248</v>
       </c>
-      <c r="I2" s="40" t="s">
+      <c r="J2" s="27" t="s">
         <v>249</v>
       </c>
-      <c r="J2" s="27" t="s">
+      <c r="K2" s="27" t="s">
         <v>250</v>
       </c>
-      <c r="K2" s="27" t="s">
+      <c r="L2" s="27" t="s">
         <v>251</v>
       </c>
-      <c r="L2" s="27" t="s">
+      <c r="M2" s="27" t="s">
+        <v>310</v>
+      </c>
+      <c r="N2" s="27" t="s">
+        <v>311</v>
+      </c>
+      <c r="O2" s="27" t="s">
         <v>252</v>
       </c>
-      <c r="M2" s="27" t="s">
-        <v>311</v>
-      </c>
-      <c r="N2" s="27" t="s">
-        <v>312</v>
-      </c>
-      <c r="O2" s="27" t="s">
+      <c r="P2" s="27" t="s">
         <v>253</v>
       </c>
-      <c r="P2" s="27" t="s">
+      <c r="Q2" s="27" t="s">
         <v>254</v>
       </c>
-      <c r="Q2" s="27" t="s">
+      <c r="R2" s="28" t="s">
         <v>255</v>
       </c>
-      <c r="R2" s="28" t="s">
+      <c r="S2" s="28" t="s">
+        <v>121</v>
+      </c>
+      <c r="T2" s="28" t="s">
         <v>256</v>
       </c>
-      <c r="S2" s="28" t="s">
-        <v>122</v>
-      </c>
-      <c r="T2" s="28" t="s">
+      <c r="AB2" t="s">
         <v>257</v>
       </c>
-      <c r="AB2" t="s">
+      <c r="AC2" t="s">
         <v>258</v>
       </c>
-      <c r="AC2" t="s">
+      <c r="AD2" t="s">
         <v>259</v>
-      </c>
-      <c r="AD2" t="s">
-        <v>260</v>
       </c>
     </row>
     <row r="3" spans="1:30" x14ac:dyDescent="0.2">
@@ -3386,13 +3389,13 @@
       <c r="S3" s="3"/>
       <c r="T3" s="3"/>
       <c r="AB3" t="s">
+        <v>260</v>
+      </c>
+      <c r="AC3" t="s">
         <v>261</v>
       </c>
-      <c r="AC3" t="s">
+      <c r="AD3" t="s">
         <v>262</v>
-      </c>
-      <c r="AD3" t="s">
-        <v>263</v>
       </c>
     </row>
     <row r="4" spans="1:30" x14ac:dyDescent="0.2">
@@ -3425,7 +3428,7 @@
       <c r="S4" s="3"/>
       <c r="T4" s="3"/>
       <c r="AB4" t="s">
-        <v>264</v>
+        <v>263</v>
       </c>
     </row>
     <row r="5" spans="1:30" x14ac:dyDescent="0.2">
@@ -3458,7 +3461,7 @@
       <c r="S5" s="3"/>
       <c r="T5" s="3"/>
       <c r="AB5" t="s">
-        <v>265</v>
+        <v>264</v>
       </c>
     </row>
     <row r="6" spans="1:30" x14ac:dyDescent="0.2">
@@ -3551,13 +3554,13 @@
       <c r="S8" s="3"/>
       <c r="T8" s="3"/>
       <c r="AB8" t="s">
+        <v>257</v>
+      </c>
+      <c r="AC8" t="s">
         <v>258</v>
       </c>
-      <c r="AC8" t="s">
+      <c r="AD8" t="s">
         <v>259</v>
-      </c>
-      <c r="AD8" t="s">
-        <v>260</v>
       </c>
     </row>
     <row r="9" spans="1:30" x14ac:dyDescent="0.2">
@@ -3590,13 +3593,13 @@
       <c r="S9" s="3"/>
       <c r="T9" s="3"/>
       <c r="AB9" t="s">
+        <v>260</v>
+      </c>
+      <c r="AC9" t="s">
         <v>261</v>
       </c>
-      <c r="AC9" t="s">
+      <c r="AD9" t="s">
         <v>262</v>
-      </c>
-      <c r="AD9" t="s">
-        <v>263</v>
       </c>
     </row>
     <row r="10" spans="1:30" x14ac:dyDescent="0.2">
@@ -3629,13 +3632,13 @@
       <c r="S10" s="3"/>
       <c r="T10" s="3"/>
       <c r="AB10" t="s">
-        <v>264</v>
+        <v>263</v>
       </c>
       <c r="AC10" t="s">
-        <v>262</v>
+        <v>261</v>
       </c>
       <c r="AD10" t="s">
-        <v>260</v>
+        <v>259</v>
       </c>
     </row>
     <row r="11" spans="1:30" x14ac:dyDescent="0.2">
@@ -3668,13 +3671,13 @@
       <c r="S11" s="3"/>
       <c r="T11" s="3"/>
       <c r="AB11" t="s">
-        <v>265</v>
+        <v>264</v>
       </c>
       <c r="AC11" t="s">
-        <v>262</v>
+        <v>261</v>
       </c>
       <c r="AD11" t="s">
-        <v>260</v>
+        <v>259</v>
       </c>
     </row>
     <row r="12" spans="1:30" x14ac:dyDescent="0.2">
@@ -4018,7 +4021,7 @@
       <c r="L24" s="9"/>
       <c r="V24" s="26"/>
       <c r="W24" s="9" t="s">
-        <v>97</v>
+        <v>96</v>
       </c>
     </row>
     <row r="25" spans="1:23" x14ac:dyDescent="0.2">
@@ -4026,7 +4029,7 @@
       <c r="L25" s="9"/>
       <c r="V25" s="29"/>
       <c r="W25" s="9" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
     </row>
   </sheetData>
@@ -4061,61 +4064,61 @@
   <sheetData>
     <row r="2" spans="1:27" x14ac:dyDescent="0.2">
       <c r="A2" s="12" t="s">
-        <v>194</v>
+        <v>193</v>
       </c>
       <c r="B2" s="12" t="s">
+        <v>241</v>
+      </c>
+      <c r="C2" s="12" t="s">
         <v>242</v>
       </c>
-      <c r="C2" s="12" t="s">
+      <c r="D2" s="12" t="s">
         <v>243</v>
       </c>
-      <c r="D2" s="12" t="s">
+      <c r="E2" s="12" t="s">
         <v>244</v>
       </c>
-      <c r="E2" s="12" t="s">
+      <c r="F2" s="12" t="s">
         <v>245</v>
       </c>
-      <c r="F2" s="12" t="s">
-        <v>246</v>
-      </c>
       <c r="G2" s="40" t="s">
+        <v>265</v>
+      </c>
+      <c r="H2" s="40" t="s">
+        <v>248</v>
+      </c>
+      <c r="I2" s="27" t="s">
         <v>266</v>
       </c>
-      <c r="H2" s="40" t="s">
-        <v>249</v>
-      </c>
-      <c r="I2" s="27" t="s">
+      <c r="J2" s="27" t="s">
         <v>267</v>
       </c>
-      <c r="J2" s="27" t="s">
+      <c r="K2" s="41" t="s">
         <v>268</v>
       </c>
-      <c r="K2" s="41" t="s">
+      <c r="L2" s="41" t="s">
         <v>269</v>
       </c>
-      <c r="L2" s="41" t="s">
+      <c r="M2" s="28" t="s">
+        <v>121</v>
+      </c>
+      <c r="N2" s="28" t="s">
         <v>270</v>
       </c>
-      <c r="M2" s="28" t="s">
-        <v>122</v>
-      </c>
-      <c r="N2" s="28" t="s">
-        <v>271</v>
-      </c>
       <c r="O2" s="28" t="s">
-        <v>257</v>
+        <v>256</v>
       </c>
       <c r="P2" s="28" t="s">
+        <v>313</v>
+      </c>
+      <c r="Q2" s="28" t="s">
         <v>314</v>
       </c>
-      <c r="Q2" s="28" t="s">
-        <v>315</v>
-      </c>
       <c r="Z2" t="s">
-        <v>222</v>
+        <v>221</v>
       </c>
       <c r="AA2" t="s">
-        <v>260</v>
+        <v>259</v>
       </c>
     </row>
     <row r="3" spans="1:27" x14ac:dyDescent="0.2">
@@ -4139,10 +4142,10 @@
       <c r="P3" s="3"/>
       <c r="Q3" s="3"/>
       <c r="Z3" t="s">
-        <v>316</v>
+        <v>315</v>
       </c>
       <c r="AA3" t="s">
-        <v>263</v>
+        <v>262</v>
       </c>
     </row>
     <row r="4" spans="1:27" x14ac:dyDescent="0.2">
@@ -4166,7 +4169,7 @@
       <c r="P4" s="3"/>
       <c r="Q4" s="3"/>
       <c r="Z4" t="s">
-        <v>317</v>
+        <v>316</v>
       </c>
     </row>
     <row r="5" spans="1:27" x14ac:dyDescent="0.2">
@@ -4190,7 +4193,7 @@
       <c r="P5" s="3"/>
       <c r="Q5" s="3"/>
       <c r="Z5" t="s">
-        <v>226</v>
+        <v>225</v>
       </c>
     </row>
     <row r="6" spans="1:27" x14ac:dyDescent="0.2">
@@ -4353,13 +4356,13 @@
     <row r="16" spans="1:27" x14ac:dyDescent="0.2">
       <c r="S16" s="26"/>
       <c r="T16" s="9" t="s">
-        <v>97</v>
+        <v>96</v>
       </c>
     </row>
     <row r="17" spans="19:20" x14ac:dyDescent="0.2">
       <c r="S17" s="29"/>
       <c r="T17" s="9" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
     </row>
   </sheetData>
@@ -4388,22 +4391,22 @@
   <sheetData>
     <row r="2" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A2" s="12" t="s">
-        <v>194</v>
+        <v>193</v>
       </c>
       <c r="B2" s="12" t="s">
-        <v>242</v>
+        <v>241</v>
       </c>
       <c r="C2" s="12" t="s">
+        <v>165</v>
+      </c>
+      <c r="D2" s="12" t="s">
         <v>166</v>
       </c>
-      <c r="D2" s="12" t="s">
-        <v>167</v>
-      </c>
       <c r="E2" s="12" t="s">
+        <v>271</v>
+      </c>
+      <c r="F2" s="12" t="s">
         <v>272</v>
-      </c>
-      <c r="F2" s="12" t="s">
-        <v>273</v>
       </c>
     </row>
     <row r="3" spans="1:6" x14ac:dyDescent="0.2">
@@ -4626,27 +4629,27 @@
   <sheetData>
     <row r="2" spans="2:21" x14ac:dyDescent="0.2">
       <c r="B2" s="64" t="s">
-        <v>274</v>
+        <v>273</v>
       </c>
       <c r="C2" s="65"/>
       <c r="E2" s="59" t="s">
-        <v>275</v>
+        <v>274</v>
       </c>
       <c r="F2" s="54"/>
       <c r="H2" s="59" t="s">
-        <v>276</v>
+        <v>275</v>
       </c>
       <c r="I2" s="54"/>
       <c r="K2" s="59" t="s">
-        <v>277</v>
+        <v>276</v>
       </c>
       <c r="L2" s="54"/>
       <c r="N2" s="59" t="s">
-        <v>278</v>
+        <v>277</v>
       </c>
       <c r="O2" s="54"/>
       <c r="Q2" s="59" t="s">
-        <v>279</v>
+        <v>278</v>
       </c>
       <c r="R2" s="54"/>
     </row>
@@ -4654,71 +4657,71 @@
       <c r="B3" s="66"/>
       <c r="C3" s="67"/>
       <c r="E3" s="32" t="s">
-        <v>280</v>
+        <v>279</v>
       </c>
       <c r="F3" s="33"/>
       <c r="H3" s="32" t="s">
-        <v>280</v>
+        <v>279</v>
       </c>
       <c r="I3" s="33"/>
       <c r="K3" s="32" t="s">
-        <v>280</v>
+        <v>279</v>
       </c>
       <c r="L3" s="33"/>
       <c r="N3" s="32" t="s">
-        <v>280</v>
+        <v>279</v>
       </c>
       <c r="O3" s="33"/>
       <c r="Q3" s="32" t="s">
-        <v>280</v>
+        <v>279</v>
       </c>
       <c r="R3" s="33"/>
       <c r="T3" s="6" t="s">
-        <v>281</v>
+        <v>280</v>
       </c>
     </row>
     <row r="4" spans="2:21" x14ac:dyDescent="0.2">
       <c r="B4" s="25" t="s">
+        <v>165</v>
+      </c>
+      <c r="C4" s="25" t="s">
         <v>166</v>
       </c>
-      <c r="C4" s="25" t="s">
-        <v>167</v>
-      </c>
       <c r="E4" s="25" t="s">
+        <v>165</v>
+      </c>
+      <c r="F4" s="25" t="s">
         <v>166</v>
       </c>
-      <c r="F4" s="25" t="s">
-        <v>167</v>
-      </c>
       <c r="H4" s="25" t="s">
+        <v>165</v>
+      </c>
+      <c r="I4" s="25" t="s">
         <v>166</v>
       </c>
-      <c r="I4" s="25" t="s">
-        <v>167</v>
-      </c>
       <c r="K4" s="25" t="s">
+        <v>165</v>
+      </c>
+      <c r="L4" s="25" t="s">
         <v>166</v>
       </c>
-      <c r="L4" s="25" t="s">
-        <v>167</v>
-      </c>
       <c r="N4" s="25" t="s">
+        <v>165</v>
+      </c>
+      <c r="O4" s="25" t="s">
         <v>166</v>
       </c>
-      <c r="O4" s="25" t="s">
-        <v>167</v>
-      </c>
       <c r="Q4" s="25" t="s">
+        <v>165</v>
+      </c>
+      <c r="R4" s="25" t="s">
         <v>166</v>
       </c>
-      <c r="R4" s="25" t="s">
-        <v>167</v>
-      </c>
       <c r="T4" s="1" t="s">
-        <v>280</v>
+        <v>279</v>
       </c>
       <c r="U4" t="s">
-        <v>282</v>
+        <v>281</v>
       </c>
     </row>
     <row r="5" spans="2:21" x14ac:dyDescent="0.2">
@@ -4735,10 +4738,10 @@
       <c r="Q5" s="3"/>
       <c r="R5" s="3"/>
       <c r="T5" s="1" t="s">
+        <v>282</v>
+      </c>
+      <c r="U5" t="s">
         <v>283</v>
-      </c>
-      <c r="U5" t="s">
-        <v>284</v>
       </c>
     </row>
     <row r="6" spans="2:21" x14ac:dyDescent="0.2">
@@ -4755,7 +4758,7 @@
       <c r="Q6" s="3"/>
       <c r="R6" s="3"/>
       <c r="T6" s="1" t="s">
-        <v>285</v>
+        <v>284</v>
       </c>
       <c r="U6" s="9"/>
     </row>
@@ -5044,27 +5047,27 @@
   <sheetData>
     <row r="2" spans="2:21" x14ac:dyDescent="0.2">
       <c r="B2" s="68" t="s">
-        <v>286</v>
+        <v>285</v>
       </c>
       <c r="C2" s="65"/>
       <c r="E2" s="60" t="s">
-        <v>287</v>
+        <v>286</v>
       </c>
       <c r="F2" s="54"/>
       <c r="H2" s="60" t="s">
-        <v>288</v>
+        <v>287</v>
       </c>
       <c r="I2" s="54"/>
       <c r="K2" s="60" t="s">
-        <v>289</v>
+        <v>288</v>
       </c>
       <c r="L2" s="54"/>
       <c r="N2" s="60" t="s">
-        <v>290</v>
+        <v>289</v>
       </c>
       <c r="O2" s="54"/>
       <c r="Q2" s="60" t="s">
-        <v>291</v>
+        <v>290</v>
       </c>
       <c r="R2" s="54"/>
     </row>
@@ -5072,71 +5075,71 @@
       <c r="B3" s="66"/>
       <c r="C3" s="67"/>
       <c r="E3" s="34" t="s">
-        <v>280</v>
+        <v>279</v>
       </c>
       <c r="F3" s="35"/>
       <c r="H3" s="34" t="s">
-        <v>280</v>
+        <v>279</v>
       </c>
       <c r="I3" s="35"/>
       <c r="K3" s="34" t="s">
-        <v>280</v>
+        <v>279</v>
       </c>
       <c r="L3" s="35"/>
       <c r="N3" s="34" t="s">
-        <v>280</v>
+        <v>279</v>
       </c>
       <c r="O3" s="35"/>
       <c r="Q3" s="34" t="s">
-        <v>280</v>
+        <v>279</v>
       </c>
       <c r="R3" s="35"/>
       <c r="T3" s="6" t="s">
-        <v>281</v>
+        <v>280</v>
       </c>
     </row>
     <row r="4" spans="2:21" x14ac:dyDescent="0.2">
       <c r="B4" s="25" t="s">
+        <v>165</v>
+      </c>
+      <c r="C4" s="25" t="s">
         <v>166</v>
       </c>
-      <c r="C4" s="25" t="s">
-        <v>167</v>
-      </c>
       <c r="E4" s="25" t="s">
+        <v>165</v>
+      </c>
+      <c r="F4" s="25" t="s">
         <v>166</v>
       </c>
-      <c r="F4" s="25" t="s">
-        <v>167</v>
-      </c>
       <c r="H4" s="25" t="s">
+        <v>165</v>
+      </c>
+      <c r="I4" s="25" t="s">
         <v>166</v>
       </c>
-      <c r="I4" s="25" t="s">
-        <v>167</v>
-      </c>
       <c r="K4" s="25" t="s">
+        <v>165</v>
+      </c>
+      <c r="L4" s="25" t="s">
         <v>166</v>
       </c>
-      <c r="L4" s="25" t="s">
-        <v>167</v>
-      </c>
       <c r="N4" s="25" t="s">
+        <v>165</v>
+      </c>
+      <c r="O4" s="25" t="s">
         <v>166</v>
       </c>
-      <c r="O4" s="25" t="s">
-        <v>167</v>
-      </c>
       <c r="Q4" s="25" t="s">
+        <v>165</v>
+      </c>
+      <c r="R4" s="25" t="s">
         <v>166</v>
       </c>
-      <c r="R4" s="25" t="s">
-        <v>167</v>
-      </c>
       <c r="T4" s="1" t="s">
-        <v>280</v>
+        <v>279</v>
       </c>
       <c r="U4" t="s">
-        <v>282</v>
+        <v>281</v>
       </c>
     </row>
     <row r="5" spans="2:21" x14ac:dyDescent="0.2">
@@ -5153,10 +5156,10 @@
       <c r="Q5" s="3"/>
       <c r="R5" s="3"/>
       <c r="T5" s="1" t="s">
+        <v>282</v>
+      </c>
+      <c r="U5" t="s">
         <v>283</v>
-      </c>
-      <c r="U5" t="s">
-        <v>284</v>
       </c>
     </row>
     <row r="6" spans="2:21" x14ac:dyDescent="0.2">
@@ -5455,22 +5458,22 @@
   <sheetData>
     <row r="2" spans="2:10" x14ac:dyDescent="0.2">
       <c r="B2" s="50" t="s">
+        <v>291</v>
+      </c>
+      <c r="C2" s="50" t="s">
         <v>292</v>
       </c>
-      <c r="C2" s="50" t="s">
+      <c r="D2" s="50" t="s">
         <v>293</v>
       </c>
-      <c r="D2" s="50" t="s">
+      <c r="E2" s="50" t="s">
         <v>294</v>
       </c>
-      <c r="E2" s="50" t="s">
+      <c r="F2" s="50" t="s">
         <v>295</v>
       </c>
-      <c r="F2" s="50" t="s">
+      <c r="G2" s="50" t="s">
         <v>296</v>
-      </c>
-      <c r="G2" s="50" t="s">
-        <v>297</v>
       </c>
     </row>
     <row r="3" spans="2:10" x14ac:dyDescent="0.2">
@@ -5481,7 +5484,7 @@
       <c r="F3" s="3"/>
       <c r="G3" s="3"/>
       <c r="I3" s="14" t="s">
-        <v>298</v>
+        <v>297</v>
       </c>
       <c r="J3" s="3"/>
     </row>
@@ -5503,7 +5506,7 @@
       <c r="F5" s="3"/>
       <c r="G5" s="3"/>
       <c r="I5" s="14" t="s">
-        <v>299</v>
+        <v>298</v>
       </c>
       <c r="J5" s="3"/>
     </row>
@@ -5525,7 +5528,7 @@
       <c r="F7" s="3"/>
       <c r="G7" s="3"/>
       <c r="I7" s="14" t="s">
-        <v>300</v>
+        <v>299</v>
       </c>
       <c r="J7" s="3"/>
     </row>
@@ -5537,7 +5540,7 @@
       <c r="F8" s="3"/>
       <c r="G8" s="3"/>
       <c r="I8" s="14" t="s">
-        <v>301</v>
+        <v>300</v>
       </c>
       <c r="J8" s="3"/>
     </row>
@@ -5549,7 +5552,7 @@
       <c r="F9" s="3"/>
       <c r="G9" s="3"/>
       <c r="I9" s="14" t="s">
-        <v>302</v>
+        <v>301</v>
       </c>
       <c r="J9" s="3"/>
     </row>
@@ -5569,7 +5572,7 @@
       <c r="F11" s="3"/>
       <c r="G11" s="3"/>
       <c r="J11" t="s">
-        <v>303</v>
+        <v>302</v>
       </c>
     </row>
     <row r="12" spans="2:10" x14ac:dyDescent="0.2">
@@ -6380,16 +6383,16 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
-  <dimension ref="A2:AP52"/>
+  <dimension ref="A2:AQ52"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="7" style="1" customWidth="1"/>
     <col min="2" max="2" width="17.33203125" style="1" customWidth="1"/>
     <col min="3" max="10" width="8.5" style="1" customWidth="1"/>
-    <col min="11" max="41" width="8.5" customWidth="1"/>
+    <col min="11" max="42" width="8.5" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="2" spans="1:42" x14ac:dyDescent="0.2">
+    <row r="2" spans="1:43" x14ac:dyDescent="0.2">
       <c r="C2" s="6" t="s">
         <v>79</v>
       </c>
@@ -6404,7 +6407,7 @@
         <v>82</v>
       </c>
     </row>
-    <row r="3" spans="1:42" x14ac:dyDescent="0.2">
+    <row r="3" spans="1:43" x14ac:dyDescent="0.2">
       <c r="C3" s="1" t="s">
         <v>83</v>
       </c>
@@ -6425,7 +6428,7 @@
         <v>88</v>
       </c>
     </row>
-    <row r="4" spans="1:42" x14ac:dyDescent="0.2">
+    <row r="4" spans="1:43" x14ac:dyDescent="0.2">
       <c r="C4" s="1" t="s">
         <v>89</v>
       </c>
@@ -6447,67 +6450,67 @@
         <v>93</v>
       </c>
       <c r="AK4" t="s">
+        <v>317</v>
+      </c>
+    </row>
+    <row r="5" spans="1:43" x14ac:dyDescent="0.2">
+      <c r="C5" s="1" t="s">
         <v>94</v>
       </c>
-    </row>
-    <row r="5" spans="1:42" x14ac:dyDescent="0.2">
-      <c r="C5" s="1" t="s">
+      <c r="D5" t="s">
         <v>95</v>
-      </c>
-      <c r="D5" t="s">
-        <v>96</v>
       </c>
       <c r="L5" s="26"/>
       <c r="M5" s="9" t="s">
+        <v>96</v>
+      </c>
+      <c r="O5" s="1" t="s">
         <v>97</v>
       </c>
-      <c r="O5" s="1" t="s">
+      <c r="P5" s="9" t="s">
         <v>98</v>
-      </c>
-      <c r="P5" s="9" t="s">
-        <v>99</v>
       </c>
       <c r="AD5" s="14"/>
       <c r="AJ5" s="1" t="s">
+        <v>99</v>
+      </c>
+      <c r="AK5" s="9" t="s">
         <v>100</v>
       </c>
-      <c r="AK5" s="9" t="s">
+    </row>
+    <row r="6" spans="1:43" x14ac:dyDescent="0.2">
+      <c r="C6" s="1" t="s">
         <v>101</v>
       </c>
-    </row>
-    <row r="6" spans="1:42" x14ac:dyDescent="0.2">
-      <c r="C6" s="1" t="s">
+      <c r="D6" s="9" t="s">
         <v>102</v>
-      </c>
-      <c r="D6" s="9" t="s">
-        <v>103</v>
       </c>
       <c r="L6" s="29"/>
       <c r="M6" s="9" t="s">
+        <v>103</v>
+      </c>
+      <c r="O6" s="1" t="s">
         <v>104</v>
       </c>
-      <c r="O6" s="1" t="s">
+      <c r="P6" t="s">
         <v>105</v>
-      </c>
-      <c r="P6" t="s">
-        <v>106</v>
       </c>
       <c r="AE6" s="1"/>
       <c r="AF6" s="1"/>
     </row>
-    <row r="7" spans="1:42" x14ac:dyDescent="0.2">
+    <row r="7" spans="1:43" x14ac:dyDescent="0.2">
       <c r="C7" s="1" t="s">
+        <v>106</v>
+      </c>
+      <c r="D7" s="9" t="s">
         <v>107</v>
-      </c>
-      <c r="D7" s="9" t="s">
-        <v>108</v>
       </c>
       <c r="AE7" s="1"/>
       <c r="AF7" s="1"/>
     </row>
-    <row r="9" spans="1:42" x14ac:dyDescent="0.2">
+    <row r="9" spans="1:43" x14ac:dyDescent="0.2">
       <c r="C9" s="53" t="s">
-        <v>109</v>
+        <v>108</v>
       </c>
       <c r="D9" s="52"/>
       <c r="E9" s="52"/>
@@ -6533,7 +6536,7 @@
       <c r="Y9" s="54"/>
       <c r="Z9" s="54"/>
       <c r="AA9" s="53" t="s">
-        <v>110</v>
+        <v>109</v>
       </c>
       <c r="AB9" s="54"/>
       <c r="AC9" s="54"/>
@@ -6541,7 +6544,7 @@
       <c r="AE9" s="54"/>
       <c r="AF9" s="54"/>
       <c r="AG9" s="53" t="s">
-        <v>111</v>
+        <v>110</v>
       </c>
       <c r="AH9" s="54"/>
       <c r="AI9" s="54"/>
@@ -6552,136 +6555,140 @@
       <c r="AN9" s="54"/>
       <c r="AO9" s="54"/>
       <c r="AP9" s="54"/>
-    </row>
-    <row r="10" spans="1:42" ht="18" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="AQ9" s="54"/>
+    </row>
+    <row r="10" spans="1:43" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A10" s="20" t="s">
         <v>8</v>
       </c>
       <c r="B10" s="20" t="s">
+        <v>111</v>
+      </c>
+      <c r="C10" s="45" t="s">
         <v>112</v>
       </c>
-      <c r="C10" s="45" t="s">
+      <c r="D10" s="48" t="s">
+        <v>308</v>
+      </c>
+      <c r="E10" s="44" t="s">
         <v>113</v>
       </c>
-      <c r="D10" s="48" t="s">
-        <v>309</v>
-      </c>
-      <c r="E10" s="44" t="s">
+      <c r="F10" s="44" t="s">
         <v>114</v>
       </c>
-      <c r="F10" s="44" t="s">
+      <c r="G10" s="45" t="s">
         <v>115</v>
       </c>
-      <c r="G10" s="45" t="s">
+      <c r="H10" s="44" t="s">
         <v>116</v>
       </c>
-      <c r="H10" s="44" t="s">
+      <c r="I10" s="44" t="s">
         <v>117</v>
       </c>
-      <c r="I10" s="44" t="s">
+      <c r="J10" s="49" t="s">
         <v>118</v>
       </c>
-      <c r="J10" s="49" t="s">
+      <c r="K10" s="49" t="s">
         <v>119</v>
       </c>
-      <c r="K10" s="49" t="s">
+      <c r="L10" s="21" t="s">
         <v>120</v>
       </c>
-      <c r="L10" s="21" t="s">
+      <c r="M10" s="21" t="s">
         <v>121</v>
       </c>
-      <c r="M10" s="21" t="s">
+      <c r="N10" s="43" t="s">
         <v>122</v>
       </c>
-      <c r="N10" s="43" t="s">
+      <c r="O10" s="44" t="s">
         <v>123</v>
       </c>
-      <c r="O10" s="44" t="s">
+      <c r="P10" s="44" t="s">
+        <v>104</v>
+      </c>
+      <c r="Q10" s="44" t="s">
         <v>124</v>
       </c>
-      <c r="P10" s="44" t="s">
-        <v>105</v>
-      </c>
-      <c r="Q10" s="44" t="s">
+      <c r="R10" s="44" t="s">
         <v>125</v>
       </c>
-      <c r="R10" s="44" t="s">
+      <c r="S10" s="44" t="s">
         <v>126</v>
       </c>
-      <c r="S10" s="44" t="s">
+      <c r="T10" s="44" t="s">
         <v>127</v>
       </c>
-      <c r="T10" s="44" t="s">
+      <c r="U10" s="44" t="s">
         <v>128</v>
       </c>
-      <c r="U10" s="44" t="s">
+      <c r="V10" s="44" t="s">
         <v>129</v>
       </c>
-      <c r="V10" s="44" t="s">
+      <c r="W10" s="44" t="s">
         <v>130</v>
       </c>
-      <c r="W10" s="44" t="s">
+      <c r="X10" s="44" t="s">
         <v>131</v>
       </c>
-      <c r="X10" s="44" t="s">
+      <c r="Y10" s="44" t="s">
         <v>132</v>
       </c>
-      <c r="Y10" s="44" t="s">
+      <c r="Z10" s="44" t="s">
         <v>133</v>
       </c>
-      <c r="Z10" s="44" t="s">
+      <c r="AA10" s="46" t="s">
+        <v>304</v>
+      </c>
+      <c r="AB10" s="46" t="s">
+        <v>303</v>
+      </c>
+      <c r="AC10" s="47" t="s">
         <v>134</v>
       </c>
-      <c r="AA10" s="46" t="s">
+      <c r="AD10" s="46" t="s">
         <v>305</v>
       </c>
-      <c r="AB10" s="46" t="s">
-        <v>304</v>
-      </c>
-      <c r="AC10" s="47" t="s">
+      <c r="AE10" s="46" t="s">
+        <v>306</v>
+      </c>
+      <c r="AF10" s="47" t="s">
+        <v>307</v>
+      </c>
+      <c r="AG10" s="23" t="s">
         <v>135</v>
       </c>
-      <c r="AD10" s="46" t="s">
-        <v>306</v>
-      </c>
-      <c r="AE10" s="46" t="s">
-        <v>307</v>
-      </c>
-      <c r="AF10" s="47" t="s">
-        <v>308</v>
-      </c>
-      <c r="AG10" s="23" t="s">
+      <c r="AH10" s="23" t="s">
         <v>136</v>
       </c>
-      <c r="AH10" s="23" t="s">
+      <c r="AI10" s="23" t="s">
         <v>137</v>
       </c>
-      <c r="AI10" s="23" t="s">
+      <c r="AJ10" s="23" t="s">
         <v>138</v>
       </c>
-      <c r="AJ10" s="23" t="s">
+      <c r="AK10" s="23" t="s">
         <v>139</v>
       </c>
-      <c r="AK10" s="23" t="s">
+      <c r="AL10" s="23" t="s">
         <v>140</v>
       </c>
-      <c r="AL10" s="23" t="s">
+      <c r="AM10" s="23" t="s">
         <v>141</v>
       </c>
-      <c r="AM10" s="23" t="s">
+      <c r="AN10" s="23" t="s">
         <v>142</v>
       </c>
-      <c r="AN10" s="23" t="s">
+      <c r="AO10" s="23" t="s">
+        <v>318</v>
+      </c>
+      <c r="AP10" s="23" t="s">
         <v>143</v>
       </c>
-      <c r="AO10" s="23" t="s">
+      <c r="AQ10" s="23" t="s">
         <v>144</v>
       </c>
-      <c r="AP10" s="23" t="s">
-        <v>145</v>
-      </c>
-    </row>
-    <row r="11" spans="1:42" x14ac:dyDescent="0.2">
+    </row>
+    <row r="11" spans="1:43" x14ac:dyDescent="0.2">
       <c r="A11" s="3">
         <v>1</v>
       </c>
@@ -6726,8 +6733,9 @@
       <c r="AN11" s="3"/>
       <c r="AO11" s="3"/>
       <c r="AP11" s="3"/>
-    </row>
-    <row r="12" spans="1:42" x14ac:dyDescent="0.2">
+      <c r="AQ11" s="3"/>
+    </row>
+    <row r="12" spans="1:43" x14ac:dyDescent="0.2">
       <c r="A12" s="3">
         <v>2</v>
       </c>
@@ -6772,8 +6780,9 @@
       <c r="AN12" s="19"/>
       <c r="AO12" s="19"/>
       <c r="AP12" s="19"/>
-    </row>
-    <row r="13" spans="1:42" x14ac:dyDescent="0.2">
+      <c r="AQ12" s="19"/>
+    </row>
+    <row r="13" spans="1:43" x14ac:dyDescent="0.2">
       <c r="A13" s="3">
         <v>3</v>
       </c>
@@ -6818,8 +6827,9 @@
       <c r="AN13" s="19"/>
       <c r="AO13" s="19"/>
       <c r="AP13" s="19"/>
-    </row>
-    <row r="14" spans="1:42" x14ac:dyDescent="0.2">
+      <c r="AQ13" s="19"/>
+    </row>
+    <row r="14" spans="1:43" x14ac:dyDescent="0.2">
       <c r="A14" s="3">
         <v>4</v>
       </c>
@@ -6864,8 +6874,9 @@
       <c r="AN14" s="3"/>
       <c r="AO14" s="3"/>
       <c r="AP14" s="3"/>
-    </row>
-    <row r="15" spans="1:42" x14ac:dyDescent="0.2">
+      <c r="AQ14" s="3"/>
+    </row>
+    <row r="15" spans="1:43" x14ac:dyDescent="0.2">
       <c r="A15" s="3">
         <v>5</v>
       </c>
@@ -6910,8 +6921,9 @@
       <c r="AN15" s="3"/>
       <c r="AO15" s="3"/>
       <c r="AP15" s="3"/>
-    </row>
-    <row r="16" spans="1:42" x14ac:dyDescent="0.2">
+      <c r="AQ15" s="3"/>
+    </row>
+    <row r="16" spans="1:43" x14ac:dyDescent="0.2">
       <c r="A16" s="3">
         <v>6</v>
       </c>
@@ -6956,8 +6968,9 @@
       <c r="AN16" s="3"/>
       <c r="AO16" s="3"/>
       <c r="AP16" s="3"/>
-    </row>
-    <row r="17" spans="1:42" x14ac:dyDescent="0.2">
+      <c r="AQ16" s="3"/>
+    </row>
+    <row r="17" spans="1:43" x14ac:dyDescent="0.2">
       <c r="A17" s="3">
         <v>7</v>
       </c>
@@ -7002,8 +7015,9 @@
       <c r="AN17" s="3"/>
       <c r="AO17" s="3"/>
       <c r="AP17" s="3"/>
-    </row>
-    <row r="18" spans="1:42" x14ac:dyDescent="0.2">
+      <c r="AQ17" s="3"/>
+    </row>
+    <row r="18" spans="1:43" x14ac:dyDescent="0.2">
       <c r="A18" s="3">
         <v>8</v>
       </c>
@@ -7048,8 +7062,9 @@
       <c r="AN18" s="3"/>
       <c r="AO18" s="3"/>
       <c r="AP18" s="3"/>
-    </row>
-    <row r="19" spans="1:42" x14ac:dyDescent="0.2">
+      <c r="AQ18" s="3"/>
+    </row>
+    <row r="19" spans="1:43" x14ac:dyDescent="0.2">
       <c r="A19" s="3">
         <v>9</v>
       </c>
@@ -7094,8 +7109,9 @@
       <c r="AN19" s="3"/>
       <c r="AO19" s="3"/>
       <c r="AP19" s="3"/>
-    </row>
-    <row r="20" spans="1:42" x14ac:dyDescent="0.2">
+      <c r="AQ19" s="3"/>
+    </row>
+    <row r="20" spans="1:43" x14ac:dyDescent="0.2">
       <c r="A20" s="3">
         <v>10</v>
       </c>
@@ -7140,8 +7156,9 @@
       <c r="AN20" s="3"/>
       <c r="AO20" s="3"/>
       <c r="AP20" s="3"/>
-    </row>
-    <row r="21" spans="1:42" x14ac:dyDescent="0.2">
+      <c r="AQ20" s="3"/>
+    </row>
+    <row r="21" spans="1:43" x14ac:dyDescent="0.2">
       <c r="A21" s="3">
         <v>11</v>
       </c>
@@ -7186,8 +7203,9 @@
       <c r="AN21" s="3"/>
       <c r="AO21" s="3"/>
       <c r="AP21" s="3"/>
-    </row>
-    <row r="22" spans="1:42" x14ac:dyDescent="0.2">
+      <c r="AQ21" s="3"/>
+    </row>
+    <row r="22" spans="1:43" x14ac:dyDescent="0.2">
       <c r="A22" s="3">
         <v>12</v>
       </c>
@@ -7232,8 +7250,9 @@
       <c r="AN22" s="3"/>
       <c r="AO22" s="3"/>
       <c r="AP22" s="3"/>
-    </row>
-    <row r="23" spans="1:42" x14ac:dyDescent="0.2">
+      <c r="AQ22" s="3"/>
+    </row>
+    <row r="23" spans="1:43" x14ac:dyDescent="0.2">
       <c r="A23" s="3">
         <v>13</v>
       </c>
@@ -7278,8 +7297,9 @@
       <c r="AN23" s="3"/>
       <c r="AO23" s="3"/>
       <c r="AP23" s="3"/>
-    </row>
-    <row r="24" spans="1:42" x14ac:dyDescent="0.2">
+      <c r="AQ23" s="3"/>
+    </row>
+    <row r="24" spans="1:43" x14ac:dyDescent="0.2">
       <c r="A24" s="3">
         <v>14</v>
       </c>
@@ -7324,8 +7344,9 @@
       <c r="AN24" s="3"/>
       <c r="AO24" s="3"/>
       <c r="AP24" s="3"/>
-    </row>
-    <row r="25" spans="1:42" x14ac:dyDescent="0.2">
+      <c r="AQ24" s="3"/>
+    </row>
+    <row r="25" spans="1:43" x14ac:dyDescent="0.2">
       <c r="A25" s="3">
         <v>15</v>
       </c>
@@ -7370,8 +7391,9 @@
       <c r="AN25" s="3"/>
       <c r="AO25" s="3"/>
       <c r="AP25" s="3"/>
-    </row>
-    <row r="26" spans="1:42" x14ac:dyDescent="0.2">
+      <c r="AQ25" s="3"/>
+    </row>
+    <row r="26" spans="1:43" x14ac:dyDescent="0.2">
       <c r="K26" s="1"/>
       <c r="L26" s="1"/>
       <c r="M26" s="1"/>
@@ -7404,8 +7426,9 @@
       <c r="AN26" s="1"/>
       <c r="AO26" s="1"/>
       <c r="AP26" s="1"/>
-    </row>
-    <row r="27" spans="1:42" x14ac:dyDescent="0.2">
+      <c r="AQ26" s="1"/>
+    </row>
+    <row r="27" spans="1:43" x14ac:dyDescent="0.2">
       <c r="K27" s="1"/>
       <c r="L27" s="1"/>
       <c r="M27" s="1"/>
@@ -7429,7 +7452,7 @@
       <c r="AE27" s="1"/>
       <c r="AF27" s="1"/>
     </row>
-    <row r="28" spans="1:42" x14ac:dyDescent="0.2">
+    <row r="28" spans="1:43" x14ac:dyDescent="0.2">
       <c r="K28" s="1"/>
       <c r="L28" s="1"/>
       <c r="M28" s="1"/>
@@ -7453,7 +7476,7 @@
       <c r="AE28" s="1"/>
       <c r="AF28" s="1"/>
     </row>
-    <row r="29" spans="1:42" x14ac:dyDescent="0.2">
+    <row r="29" spans="1:43" x14ac:dyDescent="0.2">
       <c r="K29" s="1"/>
       <c r="L29" s="1"/>
       <c r="M29" s="1"/>
@@ -7477,7 +7500,7 @@
       <c r="AE29" s="1"/>
       <c r="AF29" s="1"/>
     </row>
-    <row r="30" spans="1:42" x14ac:dyDescent="0.2">
+    <row r="30" spans="1:43" x14ac:dyDescent="0.2">
       <c r="K30" s="1"/>
       <c r="L30" s="1"/>
       <c r="M30" s="1"/>
@@ -7501,7 +7524,7 @@
       <c r="AE30" s="1"/>
       <c r="AF30" s="1"/>
     </row>
-    <row r="31" spans="1:42" x14ac:dyDescent="0.2">
+    <row r="31" spans="1:43" x14ac:dyDescent="0.2">
       <c r="K31" s="1"/>
       <c r="L31" s="1"/>
       <c r="M31" s="1"/>
@@ -7525,7 +7548,7 @@
       <c r="AE31" s="1"/>
       <c r="AF31" s="1"/>
     </row>
-    <row r="32" spans="1:42" x14ac:dyDescent="0.2">
+    <row r="32" spans="1:43" x14ac:dyDescent="0.2">
       <c r="K32" s="1"/>
       <c r="L32" s="1"/>
       <c r="M32" s="1"/>
@@ -8031,7 +8054,7 @@
     </row>
   </sheetData>
   <mergeCells count="3">
-    <mergeCell ref="AG9:AP9"/>
+    <mergeCell ref="AG9:AQ9"/>
     <mergeCell ref="AA9:AF9"/>
     <mergeCell ref="C9:Z9"/>
   </mergeCells>
@@ -8111,7 +8134,7 @@
       <formula>OR($AJ11="vg",$AJ11="gard")</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="AM11:AN52">
+  <conditionalFormatting sqref="AM11:AO52">
     <cfRule type="expression" dxfId="18" priority="1">
       <formula>$AJ11="lf"</formula>
     </cfRule>
@@ -8159,183 +8182,183 @@
   <sheetData>
     <row r="2" spans="1:44" x14ac:dyDescent="0.2">
       <c r="A2" s="5" t="s">
-        <v>146</v>
+        <v>145</v>
       </c>
       <c r="B2" s="3">
         <v>0</v>
       </c>
       <c r="D2" s="24" t="s">
+        <v>146</v>
+      </c>
+      <c r="N2" s="24" t="s">
         <v>147</v>
-      </c>
-      <c r="N2" s="24" t="s">
-        <v>148</v>
       </c>
     </row>
     <row r="4" spans="1:44" x14ac:dyDescent="0.2">
       <c r="A4" s="55" t="s">
-        <v>149</v>
+        <v>148</v>
       </c>
       <c r="B4" s="52"/>
       <c r="D4" s="55" t="s">
-        <v>150</v>
+        <v>149</v>
       </c>
       <c r="E4" s="52"/>
       <c r="G4" s="55" t="s">
-        <v>151</v>
+        <v>150</v>
       </c>
       <c r="H4" s="52"/>
       <c r="J4" s="55" t="s">
-        <v>152</v>
+        <v>151</v>
       </c>
       <c r="K4" s="52"/>
       <c r="M4" s="55" t="s">
-        <v>153</v>
+        <v>152</v>
       </c>
       <c r="N4" s="52"/>
       <c r="P4" s="55" t="s">
-        <v>154</v>
+        <v>153</v>
       </c>
       <c r="Q4" s="54"/>
       <c r="R4" s="1"/>
       <c r="S4" s="55" t="s">
-        <v>155</v>
+        <v>154</v>
       </c>
       <c r="T4" s="54"/>
       <c r="U4" s="1"/>
       <c r="V4" s="55" t="s">
-        <v>156</v>
+        <v>155</v>
       </c>
       <c r="W4" s="54"/>
       <c r="X4" s="1"/>
       <c r="Y4" s="55" t="s">
-        <v>157</v>
+        <v>156</v>
       </c>
       <c r="Z4" s="54"/>
       <c r="AA4" s="1"/>
       <c r="AB4" s="55" t="s">
-        <v>158</v>
+        <v>157</v>
       </c>
       <c r="AC4" s="54"/>
       <c r="AE4" s="55" t="s">
-        <v>159</v>
+        <v>158</v>
       </c>
       <c r="AF4" s="54"/>
       <c r="AG4" s="1"/>
       <c r="AH4" s="55" t="s">
-        <v>160</v>
+        <v>159</v>
       </c>
       <c r="AI4" s="54"/>
       <c r="AJ4" s="1"/>
       <c r="AK4" s="55" t="s">
-        <v>161</v>
+        <v>160</v>
       </c>
       <c r="AL4" s="54"/>
       <c r="AM4" s="1"/>
       <c r="AN4" s="55" t="s">
-        <v>162</v>
+        <v>161</v>
       </c>
       <c r="AO4" s="54"/>
       <c r="AP4" s="1"/>
       <c r="AQ4" s="55" t="s">
-        <v>163</v>
+        <v>162</v>
       </c>
       <c r="AR4" s="54"/>
     </row>
     <row r="5" spans="1:44" x14ac:dyDescent="0.2">
       <c r="A5" s="36" t="s">
-        <v>164</v>
+        <v>163</v>
       </c>
       <c r="B5" s="37">
         <v>1</v>
       </c>
       <c r="D5" s="36" t="s">
-        <v>164</v>
+        <v>163</v>
       </c>
       <c r="E5" s="37">
         <v>2</v>
       </c>
       <c r="G5" s="36" t="s">
-        <v>164</v>
+        <v>163</v>
       </c>
       <c r="H5" s="37">
         <v>3</v>
       </c>
       <c r="J5" s="36" t="s">
-        <v>164</v>
+        <v>163</v>
       </c>
       <c r="K5" s="37">
         <v>4</v>
       </c>
       <c r="M5" s="36" t="s">
-        <v>164</v>
+        <v>163</v>
       </c>
       <c r="N5" s="37">
         <v>5</v>
       </c>
       <c r="P5" s="36" t="s">
-        <v>164</v>
+        <v>163</v>
       </c>
       <c r="Q5" s="37">
         <v>6</v>
       </c>
       <c r="R5" s="1"/>
       <c r="S5" s="36" t="s">
-        <v>164</v>
+        <v>163</v>
       </c>
       <c r="T5" s="37">
         <v>7</v>
       </c>
       <c r="U5" s="1"/>
       <c r="V5" s="36" t="s">
-        <v>164</v>
+        <v>163</v>
       </c>
       <c r="W5" s="37">
         <v>8</v>
       </c>
       <c r="X5" s="1"/>
       <c r="Y5" s="36" t="s">
-        <v>164</v>
+        <v>163</v>
       </c>
       <c r="Z5" s="37">
         <v>9</v>
       </c>
       <c r="AA5" s="1"/>
       <c r="AB5" s="36" t="s">
-        <v>164</v>
+        <v>163</v>
       </c>
       <c r="AC5" s="37">
         <v>10</v>
       </c>
       <c r="AE5" s="36" t="s">
-        <v>164</v>
+        <v>163</v>
       </c>
       <c r="AF5" s="37">
         <v>11</v>
       </c>
       <c r="AG5" s="1"/>
       <c r="AH5" s="36" t="s">
-        <v>164</v>
+        <v>163</v>
       </c>
       <c r="AI5" s="37">
         <v>12</v>
       </c>
       <c r="AJ5" s="1"/>
       <c r="AK5" s="36" t="s">
-        <v>164</v>
+        <v>163</v>
       </c>
       <c r="AL5" s="37">
         <v>13</v>
       </c>
       <c r="AM5" s="1"/>
       <c r="AN5" s="36" t="s">
-        <v>164</v>
+        <v>163</v>
       </c>
       <c r="AO5" s="37">
         <v>14</v>
       </c>
       <c r="AP5" s="1"/>
       <c r="AQ5" s="36" t="s">
-        <v>164</v>
+        <v>163</v>
       </c>
       <c r="AR5" s="37">
         <v>15</v>
@@ -8428,172 +8451,172 @@
     </row>
     <row r="7" spans="1:44" x14ac:dyDescent="0.2">
       <c r="A7" s="36" t="s">
-        <v>165</v>
+        <v>164</v>
       </c>
       <c r="B7" s="37"/>
       <c r="D7" s="36" t="s">
-        <v>165</v>
+        <v>164</v>
       </c>
       <c r="E7" s="37"/>
       <c r="G7" s="36" t="s">
-        <v>165</v>
+        <v>164</v>
       </c>
       <c r="H7" s="37"/>
       <c r="J7" s="36" t="s">
-        <v>165</v>
+        <v>164</v>
       </c>
       <c r="K7" s="37"/>
       <c r="M7" s="36" t="s">
-        <v>165</v>
+        <v>164</v>
       </c>
       <c r="N7" s="37"/>
       <c r="P7" s="36" t="s">
-        <v>165</v>
+        <v>164</v>
       </c>
       <c r="Q7" s="37"/>
       <c r="R7" s="1"/>
       <c r="S7" s="36" t="s">
-        <v>165</v>
+        <v>164</v>
       </c>
       <c r="T7" s="37"/>
       <c r="U7" s="1"/>
       <c r="V7" s="36" t="s">
-        <v>165</v>
+        <v>164</v>
       </c>
       <c r="W7" s="37"/>
       <c r="X7" s="1"/>
       <c r="Y7" s="36" t="s">
-        <v>165</v>
+        <v>164</v>
       </c>
       <c r="Z7" s="37"/>
       <c r="AA7" s="1"/>
       <c r="AB7" s="36" t="s">
-        <v>165</v>
+        <v>164</v>
       </c>
       <c r="AC7" s="37"/>
       <c r="AE7" s="36" t="s">
-        <v>165</v>
+        <v>164</v>
       </c>
       <c r="AF7" s="37"/>
       <c r="AG7" s="1"/>
       <c r="AH7" s="36" t="s">
-        <v>165</v>
+        <v>164</v>
       </c>
       <c r="AI7" s="37"/>
       <c r="AJ7" s="1"/>
       <c r="AK7" s="36" t="s">
-        <v>165</v>
+        <v>164</v>
       </c>
       <c r="AL7" s="37"/>
       <c r="AM7" s="1"/>
       <c r="AN7" s="36" t="s">
-        <v>165</v>
+        <v>164</v>
       </c>
       <c r="AO7" s="37"/>
       <c r="AP7" s="1"/>
       <c r="AQ7" s="36" t="s">
-        <v>165</v>
+        <v>164</v>
       </c>
       <c r="AR7" s="37"/>
     </row>
     <row r="8" spans="1:44" x14ac:dyDescent="0.2">
       <c r="A8" s="2" t="s">
+        <v>165</v>
+      </c>
+      <c r="B8" s="2" t="s">
         <v>166</v>
       </c>
-      <c r="B8" s="2" t="s">
-        <v>167</v>
-      </c>
       <c r="D8" s="2" t="s">
+        <v>165</v>
+      </c>
+      <c r="E8" s="2" t="s">
         <v>166</v>
       </c>
-      <c r="E8" s="2" t="s">
-        <v>167</v>
-      </c>
       <c r="G8" s="2" t="s">
+        <v>165</v>
+      </c>
+      <c r="H8" s="2" t="s">
         <v>166</v>
       </c>
-      <c r="H8" s="2" t="s">
-        <v>167</v>
-      </c>
       <c r="J8" s="2" t="s">
+        <v>165</v>
+      </c>
+      <c r="K8" s="2" t="s">
         <v>166</v>
       </c>
-      <c r="K8" s="2" t="s">
-        <v>167</v>
-      </c>
       <c r="M8" s="2" t="s">
+        <v>165</v>
+      </c>
+      <c r="N8" s="2" t="s">
         <v>166</v>
       </c>
-      <c r="N8" s="2" t="s">
-        <v>167</v>
-      </c>
       <c r="P8" s="2" t="s">
+        <v>165</v>
+      </c>
+      <c r="Q8" s="2" t="s">
         <v>166</v>
-      </c>
-      <c r="Q8" s="2" t="s">
-        <v>167</v>
       </c>
       <c r="R8" s="1"/>
       <c r="S8" s="2" t="s">
+        <v>165</v>
+      </c>
+      <c r="T8" s="2" t="s">
         <v>166</v>
-      </c>
-      <c r="T8" s="2" t="s">
-        <v>167</v>
       </c>
       <c r="U8" s="1"/>
       <c r="V8" s="2" t="s">
+        <v>165</v>
+      </c>
+      <c r="W8" s="2" t="s">
         <v>166</v>
-      </c>
-      <c r="W8" s="2" t="s">
-        <v>167</v>
       </c>
       <c r="X8" s="1"/>
       <c r="Y8" s="2" t="s">
+        <v>165</v>
+      </c>
+      <c r="Z8" s="2" t="s">
         <v>166</v>
-      </c>
-      <c r="Z8" s="2" t="s">
-        <v>167</v>
       </c>
       <c r="AA8" s="1"/>
       <c r="AB8" s="2" t="s">
+        <v>165</v>
+      </c>
+      <c r="AC8" s="2" t="s">
         <v>166</v>
       </c>
-      <c r="AC8" s="2" t="s">
-        <v>167</v>
-      </c>
       <c r="AE8" s="2" t="s">
+        <v>165</v>
+      </c>
+      <c r="AF8" s="2" t="s">
         <v>166</v>
-      </c>
-      <c r="AF8" s="2" t="s">
-        <v>167</v>
       </c>
       <c r="AG8" s="1"/>
       <c r="AH8" s="2" t="s">
+        <v>165</v>
+      </c>
+      <c r="AI8" s="2" t="s">
         <v>166</v>
-      </c>
-      <c r="AI8" s="2" t="s">
-        <v>167</v>
       </c>
       <c r="AJ8" s="1"/>
       <c r="AK8" s="2" t="s">
+        <v>165</v>
+      </c>
+      <c r="AL8" s="2" t="s">
         <v>166</v>
-      </c>
-      <c r="AL8" s="2" t="s">
-        <v>167</v>
       </c>
       <c r="AM8" s="1"/>
       <c r="AN8" s="2" t="s">
+        <v>165</v>
+      </c>
+      <c r="AO8" s="2" t="s">
         <v>166</v>
-      </c>
-      <c r="AO8" s="2" t="s">
-        <v>167</v>
       </c>
       <c r="AP8" s="1"/>
       <c r="AQ8" s="2" t="s">
+        <v>165</v>
+      </c>
+      <c r="AR8" s="2" t="s">
         <v>166</v>
-      </c>
-      <c r="AR8" s="2" t="s">
-        <v>167</v>
       </c>
     </row>
     <row r="9" spans="1:44" x14ac:dyDescent="0.2">
@@ -9398,6 +9421,20 @@
     </row>
   </sheetData>
   <mergeCells count="30">
+    <mergeCell ref="D4:E4"/>
+    <mergeCell ref="P4:Q4"/>
+    <mergeCell ref="Y4:Z4"/>
+    <mergeCell ref="AB6:AC6"/>
+    <mergeCell ref="AN6:AO6"/>
+    <mergeCell ref="AB4:AC4"/>
+    <mergeCell ref="AN4:AO4"/>
+    <mergeCell ref="G6:H6"/>
+    <mergeCell ref="J4:K4"/>
+    <mergeCell ref="V6:W6"/>
+    <mergeCell ref="M6:N6"/>
+    <mergeCell ref="AH6:AI6"/>
+    <mergeCell ref="S6:T6"/>
+    <mergeCell ref="Y6:Z6"/>
     <mergeCell ref="AQ4:AR4"/>
     <mergeCell ref="A4:B4"/>
     <mergeCell ref="G4:H4"/>
@@ -9414,20 +9451,6 @@
     <mergeCell ref="AH4:AI4"/>
     <mergeCell ref="J6:K6"/>
     <mergeCell ref="P6:Q6"/>
-    <mergeCell ref="D4:E4"/>
-    <mergeCell ref="P4:Q4"/>
-    <mergeCell ref="Y4:Z4"/>
-    <mergeCell ref="AB6:AC6"/>
-    <mergeCell ref="AN6:AO6"/>
-    <mergeCell ref="AB4:AC4"/>
-    <mergeCell ref="AN4:AO4"/>
-    <mergeCell ref="G6:H6"/>
-    <mergeCell ref="J4:K4"/>
-    <mergeCell ref="V6:W6"/>
-    <mergeCell ref="M6:N6"/>
-    <mergeCell ref="AH6:AI6"/>
-    <mergeCell ref="S6:T6"/>
-    <mergeCell ref="Y6:Z6"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
@@ -9461,277 +9484,277 @@
   <sheetData>
     <row r="2" spans="1:44" x14ac:dyDescent="0.2">
       <c r="A2" s="24" t="s">
+        <v>167</v>
+      </c>
+      <c r="G2" s="9" t="s">
         <v>168</v>
-      </c>
-      <c r="G2" s="9" t="s">
-        <v>169</v>
       </c>
     </row>
     <row r="4" spans="1:44" x14ac:dyDescent="0.2">
       <c r="A4" s="55" t="s">
-        <v>170</v>
+        <v>169</v>
       </c>
       <c r="B4" s="52"/>
       <c r="D4" s="55" t="s">
-        <v>171</v>
+        <v>170</v>
       </c>
       <c r="E4" s="52"/>
       <c r="G4" s="55" t="s">
-        <v>172</v>
+        <v>171</v>
       </c>
       <c r="H4" s="52"/>
       <c r="J4" s="55" t="s">
-        <v>173</v>
+        <v>172</v>
       </c>
       <c r="K4" s="52"/>
       <c r="M4" s="55" t="s">
-        <v>174</v>
+        <v>173</v>
       </c>
       <c r="N4" s="52"/>
       <c r="P4" s="55" t="s">
-        <v>175</v>
+        <v>174</v>
       </c>
       <c r="Q4" s="54"/>
       <c r="R4" s="1"/>
       <c r="S4" s="55" t="s">
-        <v>176</v>
+        <v>175</v>
       </c>
       <c r="T4" s="54"/>
       <c r="U4" s="1"/>
       <c r="V4" s="55" t="s">
-        <v>177</v>
+        <v>176</v>
       </c>
       <c r="W4" s="54"/>
       <c r="X4" s="1"/>
       <c r="Y4" s="55" t="s">
-        <v>178</v>
+        <v>177</v>
       </c>
       <c r="Z4" s="54"/>
       <c r="AA4" s="1"/>
       <c r="AB4" s="55" t="s">
-        <v>179</v>
+        <v>178</v>
       </c>
       <c r="AC4" s="54"/>
       <c r="AE4" s="55" t="s">
-        <v>180</v>
+        <v>179</v>
       </c>
       <c r="AF4" s="54"/>
       <c r="AG4" s="1"/>
       <c r="AH4" s="55" t="s">
-        <v>181</v>
+        <v>180</v>
       </c>
       <c r="AI4" s="54"/>
       <c r="AJ4" s="1"/>
       <c r="AK4" s="55" t="s">
-        <v>182</v>
+        <v>181</v>
       </c>
       <c r="AL4" s="54"/>
       <c r="AM4" s="1"/>
       <c r="AN4" s="55" t="s">
-        <v>183</v>
+        <v>182</v>
       </c>
       <c r="AO4" s="54"/>
       <c r="AP4" s="1"/>
       <c r="AQ4" s="55" t="s">
-        <v>184</v>
+        <v>183</v>
       </c>
       <c r="AR4" s="54"/>
     </row>
     <row r="5" spans="1:44" x14ac:dyDescent="0.2">
       <c r="A5" s="38" t="s">
+        <v>184</v>
+      </c>
+      <c r="B5" s="39" t="s">
         <v>185</v>
       </c>
-      <c r="B5" s="39" t="s">
-        <v>186</v>
-      </c>
       <c r="D5" s="38" t="s">
+        <v>184</v>
+      </c>
+      <c r="E5" s="39" t="s">
         <v>185</v>
       </c>
-      <c r="E5" s="39" t="s">
-        <v>186</v>
-      </c>
       <c r="G5" s="38" t="s">
+        <v>184</v>
+      </c>
+      <c r="H5" s="39" t="s">
         <v>185</v>
       </c>
-      <c r="H5" s="39" t="s">
-        <v>186</v>
-      </c>
       <c r="J5" s="38" t="s">
+        <v>184</v>
+      </c>
+      <c r="K5" s="39" t="s">
         <v>185</v>
       </c>
-      <c r="K5" s="39" t="s">
-        <v>186</v>
-      </c>
       <c r="M5" s="38" t="s">
+        <v>184</v>
+      </c>
+      <c r="N5" s="39" t="s">
         <v>185</v>
       </c>
-      <c r="N5" s="39" t="s">
-        <v>186</v>
-      </c>
       <c r="P5" s="38" t="s">
+        <v>184</v>
+      </c>
+      <c r="Q5" s="39" t="s">
         <v>185</v>
-      </c>
-      <c r="Q5" s="39" t="s">
-        <v>186</v>
       </c>
       <c r="R5" s="1"/>
       <c r="S5" s="38" t="s">
+        <v>184</v>
+      </c>
+      <c r="T5" s="39" t="s">
         <v>185</v>
-      </c>
-      <c r="T5" s="39" t="s">
-        <v>186</v>
       </c>
       <c r="U5" s="1"/>
       <c r="V5" s="38" t="s">
+        <v>184</v>
+      </c>
+      <c r="W5" s="39" t="s">
         <v>185</v>
-      </c>
-      <c r="W5" s="39" t="s">
-        <v>186</v>
       </c>
       <c r="X5" s="1"/>
       <c r="Y5" s="38" t="s">
+        <v>184</v>
+      </c>
+      <c r="Z5" s="39" t="s">
         <v>185</v>
-      </c>
-      <c r="Z5" s="39" t="s">
-        <v>186</v>
       </c>
       <c r="AA5" s="1"/>
       <c r="AB5" s="38" t="s">
+        <v>184</v>
+      </c>
+      <c r="AC5" s="39" t="s">
         <v>185</v>
       </c>
-      <c r="AC5" s="39" t="s">
-        <v>186</v>
-      </c>
       <c r="AE5" s="38" t="s">
+        <v>184</v>
+      </c>
+      <c r="AF5" s="39" t="s">
         <v>185</v>
-      </c>
-      <c r="AF5" s="39" t="s">
-        <v>186</v>
       </c>
       <c r="AG5" s="1"/>
       <c r="AH5" s="38" t="s">
+        <v>184</v>
+      </c>
+      <c r="AI5" s="39" t="s">
         <v>185</v>
-      </c>
-      <c r="AI5" s="39" t="s">
-        <v>186</v>
       </c>
       <c r="AJ5" s="1"/>
       <c r="AK5" s="38" t="s">
+        <v>184</v>
+      </c>
+      <c r="AL5" s="39" t="s">
         <v>185</v>
-      </c>
-      <c r="AL5" s="39" t="s">
-        <v>186</v>
       </c>
       <c r="AM5" s="1"/>
       <c r="AN5" s="38" t="s">
+        <v>184</v>
+      </c>
+      <c r="AO5" s="39" t="s">
         <v>185</v>
-      </c>
-      <c r="AO5" s="39" t="s">
-        <v>186</v>
       </c>
       <c r="AP5" s="1"/>
       <c r="AQ5" s="38" t="s">
+        <v>184</v>
+      </c>
+      <c r="AR5" s="39" t="s">
         <v>185</v>
-      </c>
-      <c r="AR5" s="39" t="s">
-        <v>186</v>
       </c>
     </row>
     <row r="6" spans="1:44" x14ac:dyDescent="0.2">
       <c r="A6" s="38" t="s">
-        <v>164</v>
+        <v>163</v>
       </c>
       <c r="B6" s="39">
         <v>1</v>
       </c>
       <c r="D6" s="38" t="s">
-        <v>164</v>
+        <v>163</v>
       </c>
       <c r="E6" s="39">
         <v>2</v>
       </c>
       <c r="G6" s="38" t="s">
-        <v>164</v>
+        <v>163</v>
       </c>
       <c r="H6" s="39">
         <v>3</v>
       </c>
       <c r="J6" s="38" t="s">
-        <v>164</v>
+        <v>163</v>
       </c>
       <c r="K6" s="39">
         <v>4</v>
       </c>
       <c r="M6" s="38" t="s">
-        <v>164</v>
+        <v>163</v>
       </c>
       <c r="N6" s="39">
         <v>5</v>
       </c>
       <c r="P6" s="38" t="s">
-        <v>164</v>
+        <v>163</v>
       </c>
       <c r="Q6" s="39">
         <v>6</v>
       </c>
       <c r="R6" s="1"/>
       <c r="S6" s="38" t="s">
-        <v>164</v>
+        <v>163</v>
       </c>
       <c r="T6" s="39">
         <v>7</v>
       </c>
       <c r="U6" s="1"/>
       <c r="V6" s="38" t="s">
-        <v>164</v>
+        <v>163</v>
       </c>
       <c r="W6" s="39">
         <v>8</v>
       </c>
       <c r="X6" s="1"/>
       <c r="Y6" s="38" t="s">
-        <v>164</v>
+        <v>163</v>
       </c>
       <c r="Z6" s="39">
         <v>9</v>
       </c>
       <c r="AA6" s="1"/>
       <c r="AB6" s="38" t="s">
-        <v>164</v>
+        <v>163</v>
       </c>
       <c r="AC6" s="39">
         <v>10</v>
       </c>
       <c r="AE6" s="38" t="s">
-        <v>164</v>
+        <v>163</v>
       </c>
       <c r="AF6" s="39">
         <v>11</v>
       </c>
       <c r="AG6" s="1"/>
       <c r="AH6" s="38" t="s">
-        <v>164</v>
+        <v>163</v>
       </c>
       <c r="AI6" s="39">
         <v>12</v>
       </c>
       <c r="AJ6" s="1"/>
       <c r="AK6" s="38" t="s">
-        <v>164</v>
+        <v>163</v>
       </c>
       <c r="AL6" s="39">
         <v>13</v>
       </c>
       <c r="AM6" s="1"/>
       <c r="AN6" s="38" t="s">
-        <v>164</v>
+        <v>163</v>
       </c>
       <c r="AO6" s="39">
         <v>14</v>
       </c>
       <c r="AP6" s="1"/>
       <c r="AQ6" s="38" t="s">
-        <v>164</v>
+        <v>163</v>
       </c>
       <c r="AR6" s="39">
         <v>15</v>
@@ -9824,172 +9847,172 @@
     </row>
     <row r="8" spans="1:44" x14ac:dyDescent="0.2">
       <c r="A8" s="38" t="s">
-        <v>165</v>
+        <v>164</v>
       </c>
       <c r="B8" s="39"/>
       <c r="D8" s="38" t="s">
-        <v>165</v>
+        <v>164</v>
       </c>
       <c r="E8" s="39"/>
       <c r="G8" s="38" t="s">
-        <v>165</v>
+        <v>164</v>
       </c>
       <c r="H8" s="39"/>
       <c r="J8" s="38" t="s">
-        <v>165</v>
+        <v>164</v>
       </c>
       <c r="K8" s="39"/>
       <c r="M8" s="38" t="s">
-        <v>165</v>
+        <v>164</v>
       </c>
       <c r="N8" s="39"/>
       <c r="P8" s="38" t="s">
-        <v>165</v>
+        <v>164</v>
       </c>
       <c r="Q8" s="39"/>
       <c r="R8" s="1"/>
       <c r="S8" s="38" t="s">
-        <v>165</v>
+        <v>164</v>
       </c>
       <c r="T8" s="39"/>
       <c r="U8" s="1"/>
       <c r="V8" s="38" t="s">
-        <v>165</v>
+        <v>164</v>
       </c>
       <c r="W8" s="39"/>
       <c r="X8" s="1"/>
       <c r="Y8" s="38" t="s">
-        <v>165</v>
+        <v>164</v>
       </c>
       <c r="Z8" s="39"/>
       <c r="AA8" s="1"/>
       <c r="AB8" s="38" t="s">
-        <v>165</v>
+        <v>164</v>
       </c>
       <c r="AC8" s="39"/>
       <c r="AE8" s="38" t="s">
-        <v>165</v>
+        <v>164</v>
       </c>
       <c r="AF8" s="39"/>
       <c r="AG8" s="1"/>
       <c r="AH8" s="38" t="s">
-        <v>165</v>
+        <v>164</v>
       </c>
       <c r="AI8" s="39"/>
       <c r="AJ8" s="1"/>
       <c r="AK8" s="38" t="s">
-        <v>165</v>
+        <v>164</v>
       </c>
       <c r="AL8" s="39"/>
       <c r="AM8" s="1"/>
       <c r="AN8" s="38" t="s">
-        <v>165</v>
+        <v>164</v>
       </c>
       <c r="AO8" s="39"/>
       <c r="AP8" s="1"/>
       <c r="AQ8" s="38" t="s">
-        <v>165</v>
+        <v>164</v>
       </c>
       <c r="AR8" s="39"/>
     </row>
     <row r="9" spans="1:44" x14ac:dyDescent="0.2">
       <c r="A9" s="2" t="s">
+        <v>165</v>
+      </c>
+      <c r="B9" s="2" t="s">
         <v>166</v>
       </c>
-      <c r="B9" s="2" t="s">
-        <v>167</v>
-      </c>
       <c r="D9" s="2" t="s">
+        <v>165</v>
+      </c>
+      <c r="E9" s="2" t="s">
         <v>166</v>
       </c>
-      <c r="E9" s="2" t="s">
-        <v>167</v>
-      </c>
       <c r="G9" s="2" t="s">
+        <v>165</v>
+      </c>
+      <c r="H9" s="2" t="s">
         <v>166</v>
       </c>
-      <c r="H9" s="2" t="s">
-        <v>167</v>
-      </c>
       <c r="J9" s="2" t="s">
+        <v>165</v>
+      </c>
+      <c r="K9" s="2" t="s">
         <v>166</v>
       </c>
-      <c r="K9" s="2" t="s">
-        <v>167</v>
-      </c>
       <c r="M9" s="2" t="s">
+        <v>165</v>
+      </c>
+      <c r="N9" s="2" t="s">
         <v>166</v>
       </c>
-      <c r="N9" s="2" t="s">
-        <v>167</v>
-      </c>
       <c r="P9" s="2" t="s">
+        <v>165</v>
+      </c>
+      <c r="Q9" s="2" t="s">
         <v>166</v>
-      </c>
-      <c r="Q9" s="2" t="s">
-        <v>167</v>
       </c>
       <c r="R9" s="1"/>
       <c r="S9" s="2" t="s">
+        <v>165</v>
+      </c>
+      <c r="T9" s="2" t="s">
         <v>166</v>
-      </c>
-      <c r="T9" s="2" t="s">
-        <v>167</v>
       </c>
       <c r="U9" s="1"/>
       <c r="V9" s="2" t="s">
+        <v>165</v>
+      </c>
+      <c r="W9" s="2" t="s">
         <v>166</v>
-      </c>
-      <c r="W9" s="2" t="s">
-        <v>167</v>
       </c>
       <c r="X9" s="1"/>
       <c r="Y9" s="2" t="s">
+        <v>165</v>
+      </c>
+      <c r="Z9" s="2" t="s">
         <v>166</v>
-      </c>
-      <c r="Z9" s="2" t="s">
-        <v>167</v>
       </c>
       <c r="AA9" s="1"/>
       <c r="AB9" s="2" t="s">
+        <v>165</v>
+      </c>
+      <c r="AC9" s="2" t="s">
         <v>166</v>
       </c>
-      <c r="AC9" s="2" t="s">
-        <v>167</v>
-      </c>
       <c r="AE9" s="2" t="s">
+        <v>165</v>
+      </c>
+      <c r="AF9" s="2" t="s">
         <v>166</v>
-      </c>
-      <c r="AF9" s="2" t="s">
-        <v>167</v>
       </c>
       <c r="AG9" s="1"/>
       <c r="AH9" s="2" t="s">
+        <v>165</v>
+      </c>
+      <c r="AI9" s="2" t="s">
         <v>166</v>
-      </c>
-      <c r="AI9" s="2" t="s">
-        <v>167</v>
       </c>
       <c r="AJ9" s="1"/>
       <c r="AK9" s="2" t="s">
+        <v>165</v>
+      </c>
+      <c r="AL9" s="2" t="s">
         <v>166</v>
-      </c>
-      <c r="AL9" s="2" t="s">
-        <v>167</v>
       </c>
       <c r="AM9" s="1"/>
       <c r="AN9" s="2" t="s">
+        <v>165</v>
+      </c>
+      <c r="AO9" s="2" t="s">
         <v>166</v>
-      </c>
-      <c r="AO9" s="2" t="s">
-        <v>167</v>
       </c>
       <c r="AP9" s="1"/>
       <c r="AQ9" s="2" t="s">
+        <v>165</v>
+      </c>
+      <c r="AR9" s="2" t="s">
         <v>166</v>
-      </c>
-      <c r="AR9" s="2" t="s">
-        <v>167</v>
       </c>
     </row>
     <row r="10" spans="1:44" x14ac:dyDescent="0.2">
@@ -10794,6 +10817,20 @@
     </row>
   </sheetData>
   <mergeCells count="30">
+    <mergeCell ref="A4:B4"/>
+    <mergeCell ref="G4:H4"/>
+    <mergeCell ref="P4:Q4"/>
+    <mergeCell ref="J4:K4"/>
+    <mergeCell ref="D7:E7"/>
+    <mergeCell ref="J7:K7"/>
+    <mergeCell ref="D4:E4"/>
+    <mergeCell ref="M4:N4"/>
+    <mergeCell ref="P7:Q7"/>
+    <mergeCell ref="AB7:AC7"/>
+    <mergeCell ref="A7:B7"/>
+    <mergeCell ref="G7:H7"/>
+    <mergeCell ref="S7:T7"/>
+    <mergeCell ref="M7:N7"/>
     <mergeCell ref="S4:T4"/>
     <mergeCell ref="AQ7:AR7"/>
     <mergeCell ref="AN4:AO4"/>
@@ -10810,20 +10847,6 @@
     <mergeCell ref="AE4:AF4"/>
     <mergeCell ref="V4:W4"/>
     <mergeCell ref="V7:W7"/>
-    <mergeCell ref="P7:Q7"/>
-    <mergeCell ref="AB7:AC7"/>
-    <mergeCell ref="A7:B7"/>
-    <mergeCell ref="G7:H7"/>
-    <mergeCell ref="S7:T7"/>
-    <mergeCell ref="M7:N7"/>
-    <mergeCell ref="A4:B4"/>
-    <mergeCell ref="G4:H4"/>
-    <mergeCell ref="P4:Q4"/>
-    <mergeCell ref="J4:K4"/>
-    <mergeCell ref="D7:E7"/>
-    <mergeCell ref="J7:K7"/>
-    <mergeCell ref="D4:E4"/>
-    <mergeCell ref="M4:N4"/>
   </mergeCells>
   <conditionalFormatting sqref="B6 A7:B7">
     <cfRule type="expression" dxfId="17" priority="1">
@@ -10920,43 +10943,43 @@
   <sheetData>
     <row r="2" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A2" s="59" t="s">
-        <v>187</v>
+        <v>186</v>
       </c>
       <c r="B2" s="54"/>
       <c r="D2" s="60" t="s">
-        <v>188</v>
+        <v>187</v>
       </c>
       <c r="E2" s="54"/>
       <c r="G2" s="22" t="s">
-        <v>189</v>
+        <v>188</v>
       </c>
     </row>
     <row r="3" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A3" s="32" t="s">
-        <v>185</v>
+        <v>184</v>
       </c>
       <c r="B3" s="33"/>
       <c r="D3" s="34" t="s">
-        <v>185</v>
+        <v>184</v>
       </c>
       <c r="E3" s="35"/>
       <c r="G3" s="22"/>
     </row>
     <row r="4" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A4" s="2" t="s">
+        <v>165</v>
+      </c>
+      <c r="B4" s="2" t="s">
         <v>166</v>
       </c>
-      <c r="B4" s="2" t="s">
-        <v>167</v>
-      </c>
       <c r="D4" s="2" t="s">
+        <v>165</v>
+      </c>
+      <c r="E4" s="2" t="s">
         <v>166</v>
       </c>
-      <c r="E4" s="2" t="s">
-        <v>167</v>
-      </c>
       <c r="G4" s="6" t="s">
-        <v>190</v>
+        <v>189</v>
       </c>
       <c r="H4" s="1"/>
     </row>
@@ -10969,7 +10992,7 @@
         <v>18</v>
       </c>
       <c r="H5" t="s">
-        <v>191</v>
+        <v>190</v>
       </c>
     </row>
     <row r="6" spans="1:8" x14ac:dyDescent="0.2">
@@ -10978,10 +11001,10 @@
       <c r="D6" s="3"/>
       <c r="E6" s="3"/>
       <c r="G6" s="1" t="s">
+        <v>191</v>
+      </c>
+      <c r="H6" t="s">
         <v>192</v>
-      </c>
-      <c r="H6" t="s">
-        <v>193</v>
       </c>
     </row>
     <row r="7" spans="1:8" x14ac:dyDescent="0.2">
@@ -11118,31 +11141,31 @@
   <sheetData>
     <row r="2" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A2" s="13" t="s">
+        <v>193</v>
+      </c>
+      <c r="B2" s="13" t="s">
         <v>194</v>
       </c>
-      <c r="B2" s="13" t="s">
+      <c r="C2" s="13" t="s">
         <v>195</v>
       </c>
-      <c r="C2" s="13" t="s">
+      <c r="D2" s="13" t="s">
         <v>196</v>
       </c>
-      <c r="D2" s="13" t="s">
+      <c r="E2" s="13" t="s">
         <v>197</v>
       </c>
-      <c r="E2" s="13" t="s">
+      <c r="F2" s="13" t="s">
         <v>198</v>
       </c>
-      <c r="F2" s="13" t="s">
+      <c r="G2" s="13" t="s">
         <v>199</v>
       </c>
-      <c r="G2" s="13" t="s">
+      <c r="H2" s="13" t="s">
         <v>200</v>
       </c>
-      <c r="H2" s="13" t="s">
+      <c r="J2" s="5" t="s">
         <v>201</v>
-      </c>
-      <c r="J2" s="5" t="s">
-        <v>202</v>
       </c>
       <c r="K2" s="10" t="s">
         <v>5</v>
@@ -11160,10 +11183,10 @@
       <c r="G3" s="3"/>
       <c r="H3" s="3"/>
       <c r="J3" s="1" t="s">
-        <v>198</v>
+        <v>197</v>
       </c>
       <c r="K3" s="9" t="s">
-        <v>203</v>
+        <v>202</v>
       </c>
     </row>
     <row r="4" spans="1:14" x14ac:dyDescent="0.2">
@@ -11178,10 +11201,10 @@
       <c r="G4" s="3"/>
       <c r="H4" s="3"/>
       <c r="J4" s="1" t="s">
+        <v>203</v>
+      </c>
+      <c r="K4" s="9" t="s">
         <v>204</v>
-      </c>
-      <c r="K4" s="9" t="s">
-        <v>205</v>
       </c>
     </row>
     <row r="5" spans="1:14" x14ac:dyDescent="0.2">
@@ -11196,10 +11219,10 @@
       <c r="G5" s="3"/>
       <c r="H5" s="3"/>
       <c r="J5" s="1" t="s">
+        <v>205</v>
+      </c>
+      <c r="K5" t="s">
         <v>206</v>
-      </c>
-      <c r="K5" t="s">
-        <v>207</v>
       </c>
     </row>
     <row r="6" spans="1:14" x14ac:dyDescent="0.2">
@@ -11226,7 +11249,7 @@
       <c r="G7" s="3"/>
       <c r="H7" s="3"/>
       <c r="J7" s="5" t="s">
-        <v>208</v>
+        <v>207</v>
       </c>
     </row>
     <row r="8" spans="1:14" x14ac:dyDescent="0.2">
@@ -11241,7 +11264,7 @@
       <c r="G8" s="3"/>
       <c r="H8" s="3"/>
       <c r="J8" s="14" t="s">
-        <v>209</v>
+        <v>208</v>
       </c>
     </row>
     <row r="9" spans="1:14" x14ac:dyDescent="0.2">
@@ -11256,7 +11279,7 @@
       <c r="G9" s="3"/>
       <c r="H9" s="3"/>
       <c r="J9" s="14" t="s">
-        <v>210</v>
+        <v>209</v>
       </c>
     </row>
     <row r="10" spans="1:14" x14ac:dyDescent="0.2">
@@ -11271,7 +11294,7 @@
       <c r="G10" s="3"/>
       <c r="H10" s="3"/>
       <c r="J10" s="14" t="s">
-        <v>211</v>
+        <v>210</v>
       </c>
     </row>
     <row r="11" spans="1:14" x14ac:dyDescent="0.2">
@@ -11286,7 +11309,7 @@
       <c r="G11" s="3"/>
       <c r="H11" s="3"/>
       <c r="J11" s="14" t="s">
-        <v>212</v>
+        <v>211</v>
       </c>
     </row>
     <row r="12" spans="1:14" x14ac:dyDescent="0.2">
@@ -11301,27 +11324,27 @@
       <c r="G12" s="3"/>
       <c r="H12" s="3"/>
       <c r="J12" s="14" t="s">
-        <v>213</v>
+        <v>212</v>
       </c>
     </row>
     <row r="13" spans="1:14" x14ac:dyDescent="0.2">
       <c r="J13" s="14" t="s">
-        <v>214</v>
+        <v>213</v>
       </c>
     </row>
     <row r="14" spans="1:14" x14ac:dyDescent="0.2">
       <c r="J14" s="14" t="s">
-        <v>215</v>
+        <v>214</v>
       </c>
     </row>
     <row r="15" spans="1:14" x14ac:dyDescent="0.2">
       <c r="J15" s="14" t="s">
-        <v>216</v>
+        <v>215</v>
       </c>
     </row>
     <row r="16" spans="1:14" x14ac:dyDescent="0.2">
       <c r="J16" s="14" t="s">
-        <v>217</v>
+        <v>216</v>
       </c>
       <c r="K16" s="1"/>
       <c r="L16" s="1"/>
@@ -11330,7 +11353,7 @@
     </row>
     <row r="17" spans="10:10" x14ac:dyDescent="0.2">
       <c r="J17" s="14" t="s">
-        <v>218</v>
+        <v>217</v>
       </c>
     </row>
   </sheetData>
@@ -11370,16 +11393,16 @@
   <sheetData>
     <row r="2" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A2" s="11" t="s">
+        <v>218</v>
+      </c>
+      <c r="B2" s="11" t="s">
         <v>219</v>
       </c>
-      <c r="B2" s="11" t="s">
+      <c r="C2" s="12" t="s">
         <v>220</v>
       </c>
-      <c r="C2" s="12" t="s">
-        <v>221</v>
-      </c>
       <c r="E2" s="6" t="s">
-        <v>202</v>
+        <v>201</v>
       </c>
       <c r="F2" s="6" t="s">
         <v>5</v>
@@ -11390,10 +11413,10 @@
       <c r="B3" s="3"/>
       <c r="C3" s="3"/>
       <c r="E3" t="s">
+        <v>221</v>
+      </c>
+      <c r="F3" t="s">
         <v>222</v>
-      </c>
-      <c r="F3" t="s">
-        <v>223</v>
       </c>
     </row>
     <row r="4" spans="1:6" x14ac:dyDescent="0.2">
@@ -11401,10 +11424,10 @@
       <c r="B4" s="3"/>
       <c r="C4" s="3"/>
       <c r="E4" t="s">
+        <v>223</v>
+      </c>
+      <c r="F4" t="s">
         <v>224</v>
-      </c>
-      <c r="F4" t="s">
-        <v>225</v>
       </c>
     </row>
     <row r="5" spans="1:6" x14ac:dyDescent="0.2">
@@ -11412,10 +11435,10 @@
       <c r="B5" s="3"/>
       <c r="C5" s="3"/>
       <c r="E5" t="s">
+        <v>225</v>
+      </c>
+      <c r="F5" t="s">
         <v>226</v>
-      </c>
-      <c r="F5" t="s">
-        <v>227</v>
       </c>
     </row>
     <row r="6" spans="1:6" x14ac:dyDescent="0.2">
@@ -11545,122 +11568,122 @@
     </row>
     <row r="4" spans="2:24" x14ac:dyDescent="0.2">
       <c r="B4" s="61" t="s">
-        <v>228</v>
+        <v>227</v>
       </c>
       <c r="C4" s="62"/>
       <c r="D4" s="62"/>
       <c r="F4" s="61" t="s">
-        <v>229</v>
+        <v>228</v>
       </c>
       <c r="G4" s="62"/>
       <c r="H4" s="62"/>
       <c r="J4" s="61" t="s">
-        <v>230</v>
+        <v>229</v>
       </c>
       <c r="K4" s="62"/>
       <c r="L4" s="62"/>
       <c r="N4" s="61" t="s">
-        <v>231</v>
+        <v>230</v>
       </c>
       <c r="O4" s="62"/>
       <c r="P4" s="62"/>
       <c r="R4" s="61" t="s">
-        <v>232</v>
+        <v>231</v>
       </c>
       <c r="S4" s="62"/>
       <c r="T4" s="62"/>
       <c r="V4" s="61" t="s">
-        <v>233</v>
+        <v>232</v>
       </c>
       <c r="W4" s="62"/>
       <c r="X4" s="62"/>
     </row>
     <row r="5" spans="2:24" x14ac:dyDescent="0.2">
       <c r="B5" s="58" t="s">
-        <v>234</v>
+        <v>233</v>
       </c>
       <c r="C5" s="57"/>
       <c r="D5" s="39"/>
       <c r="F5" s="58" t="s">
-        <v>234</v>
+        <v>233</v>
       </c>
       <c r="G5" s="57"/>
       <c r="H5" s="39"/>
       <c r="J5" s="58" t="s">
-        <v>234</v>
+        <v>233</v>
       </c>
       <c r="K5" s="57"/>
       <c r="L5" s="39"/>
       <c r="N5" s="58" t="s">
-        <v>234</v>
+        <v>233</v>
       </c>
       <c r="O5" s="57"/>
       <c r="P5" s="39"/>
       <c r="R5" s="58" t="s">
-        <v>234</v>
+        <v>233</v>
       </c>
       <c r="S5" s="57"/>
       <c r="T5" s="39"/>
       <c r="V5" s="58" t="s">
-        <v>234</v>
+        <v>233</v>
       </c>
       <c r="W5" s="57"/>
       <c r="X5" s="39"/>
     </row>
     <row r="6" spans="2:24" x14ac:dyDescent="0.2">
       <c r="B6" s="2" t="s">
+        <v>218</v>
+      </c>
+      <c r="C6" s="2" t="s">
         <v>219</v>
       </c>
-      <c r="C6" s="2" t="s">
-        <v>220</v>
-      </c>
       <c r="D6" s="2" t="s">
-        <v>235</v>
+        <v>234</v>
       </c>
       <c r="F6" s="2" t="s">
+        <v>218</v>
+      </c>
+      <c r="G6" s="2" t="s">
         <v>219</v>
       </c>
-      <c r="G6" s="2" t="s">
-        <v>220</v>
-      </c>
       <c r="H6" s="2" t="s">
-        <v>235</v>
+        <v>234</v>
       </c>
       <c r="J6" s="2" t="s">
+        <v>218</v>
+      </c>
+      <c r="K6" s="2" t="s">
         <v>219</v>
       </c>
-      <c r="K6" s="2" t="s">
-        <v>220</v>
-      </c>
       <c r="L6" s="2" t="s">
-        <v>235</v>
+        <v>234</v>
       </c>
       <c r="N6" s="2" t="s">
+        <v>218</v>
+      </c>
+      <c r="O6" s="2" t="s">
         <v>219</v>
       </c>
-      <c r="O6" s="2" t="s">
-        <v>220</v>
-      </c>
       <c r="P6" s="2" t="s">
-        <v>235</v>
+        <v>234</v>
       </c>
       <c r="R6" s="2" t="s">
+        <v>218</v>
+      </c>
+      <c r="S6" s="2" t="s">
         <v>219</v>
       </c>
-      <c r="S6" s="2" t="s">
-        <v>220</v>
-      </c>
       <c r="T6" s="2" t="s">
-        <v>235</v>
+        <v>234</v>
       </c>
       <c r="V6" s="2" t="s">
+        <v>218</v>
+      </c>
+      <c r="W6" s="2" t="s">
         <v>219</v>
       </c>
-      <c r="W6" s="2" t="s">
-        <v>220</v>
-      </c>
       <c r="X6" s="2" t="s">
-        <v>235</v>
+        <v>234</v>
       </c>
     </row>
     <row r="7" spans="2:24" x14ac:dyDescent="0.2">
@@ -12094,122 +12117,122 @@
     </row>
     <row r="4" spans="2:24" x14ac:dyDescent="0.2">
       <c r="B4" s="63" t="s">
-        <v>236</v>
+        <v>235</v>
       </c>
       <c r="C4" s="62"/>
       <c r="D4" s="62"/>
       <c r="F4" s="63" t="s">
-        <v>237</v>
+        <v>236</v>
       </c>
       <c r="G4" s="62"/>
       <c r="H4" s="62"/>
       <c r="J4" s="63" t="s">
-        <v>238</v>
+        <v>237</v>
       </c>
       <c r="K4" s="62"/>
       <c r="L4" s="62"/>
       <c r="N4" s="63" t="s">
-        <v>239</v>
+        <v>238</v>
       </c>
       <c r="O4" s="62"/>
       <c r="P4" s="62"/>
       <c r="R4" s="63" t="s">
-        <v>240</v>
+        <v>239</v>
       </c>
       <c r="S4" s="62"/>
       <c r="T4" s="62"/>
       <c r="V4" s="63" t="s">
-        <v>241</v>
+        <v>240</v>
       </c>
       <c r="W4" s="62"/>
       <c r="X4" s="62"/>
     </row>
     <row r="5" spans="2:24" x14ac:dyDescent="0.2">
       <c r="B5" s="58" t="s">
-        <v>234</v>
+        <v>233</v>
       </c>
       <c r="C5" s="57"/>
       <c r="D5" s="39"/>
       <c r="F5" s="58" t="s">
-        <v>234</v>
+        <v>233</v>
       </c>
       <c r="G5" s="57"/>
       <c r="H5" s="39"/>
       <c r="J5" s="58" t="s">
-        <v>234</v>
+        <v>233</v>
       </c>
       <c r="K5" s="57"/>
       <c r="L5" s="39"/>
       <c r="N5" s="58" t="s">
-        <v>234</v>
+        <v>233</v>
       </c>
       <c r="O5" s="57"/>
       <c r="P5" s="39"/>
       <c r="R5" s="58" t="s">
-        <v>234</v>
+        <v>233</v>
       </c>
       <c r="S5" s="57"/>
       <c r="T5" s="39"/>
       <c r="V5" s="58" t="s">
-        <v>234</v>
+        <v>233</v>
       </c>
       <c r="W5" s="57"/>
       <c r="X5" s="39"/>
     </row>
     <row r="6" spans="2:24" x14ac:dyDescent="0.2">
       <c r="B6" s="2" t="s">
+        <v>218</v>
+      </c>
+      <c r="C6" s="2" t="s">
         <v>219</v>
       </c>
-      <c r="C6" s="2" t="s">
-        <v>220</v>
-      </c>
       <c r="D6" s="2" t="s">
-        <v>235</v>
+        <v>234</v>
       </c>
       <c r="F6" s="2" t="s">
+        <v>218</v>
+      </c>
+      <c r="G6" s="2" t="s">
         <v>219</v>
       </c>
-      <c r="G6" s="2" t="s">
-        <v>220</v>
-      </c>
       <c r="H6" s="2" t="s">
-        <v>235</v>
+        <v>234</v>
       </c>
       <c r="J6" s="2" t="s">
+        <v>218</v>
+      </c>
+      <c r="K6" s="2" t="s">
         <v>219</v>
       </c>
-      <c r="K6" s="2" t="s">
-        <v>220</v>
-      </c>
       <c r="L6" s="2" t="s">
-        <v>235</v>
+        <v>234</v>
       </c>
       <c r="N6" s="2" t="s">
+        <v>218</v>
+      </c>
+      <c r="O6" s="2" t="s">
         <v>219</v>
       </c>
-      <c r="O6" s="2" t="s">
-        <v>220</v>
-      </c>
       <c r="P6" s="2" t="s">
-        <v>235</v>
+        <v>234</v>
       </c>
       <c r="R6" s="2" t="s">
+        <v>218</v>
+      </c>
+      <c r="S6" s="2" t="s">
         <v>219</v>
       </c>
-      <c r="S6" s="2" t="s">
-        <v>220</v>
-      </c>
       <c r="T6" s="2" t="s">
-        <v>235</v>
+        <v>234</v>
       </c>
       <c r="V6" s="2" t="s">
+        <v>218</v>
+      </c>
+      <c r="W6" s="2" t="s">
         <v>219</v>
       </c>
-      <c r="W6" s="2" t="s">
-        <v>220</v>
-      </c>
       <c r="X6" s="2" t="s">
-        <v>235</v>
+        <v>234</v>
       </c>
     </row>
     <row r="7" spans="2:24" x14ac:dyDescent="0.2">

</xml_diff>

<commit_message>
template v27: Joint, kn, ks, Jred on the reinforce sheet; loader, writer and Studio editor carry them
The owner's v27 master (v26 archived beside it), the packaged copy synced.
The loader accepts 27 and reads the four columns as entered; a blank Joint
leaves the line the bonded bar it is today. Studio's reinforcement editor
shows them with tooltips, in a Joint group of the list view. The tutorial
check finds the support-type presets table by its header now that a column
insert moved it. Preflight 46/46, roundtrip 75/75.

Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01XjjT2aBxw8gY7EFdpoUcpj
</commit_message>
<xml_diff>
--- a/docs/inputs/input_template.xlsx
+++ b/docs/inputs/input_template.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/njones/python_projects/xslope/docs/inputs/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E12967D2-A998-D342-B5ED-43CABE326A3A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{904BD95E-2C21-0841-A7DF-ECBA420EAAD7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="15680" yWindow="4780" windowWidth="46940" windowHeight="18400" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="27680" yWindow="3200" windowWidth="31600" windowHeight="18400" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="main" sheetId="1" r:id="rId1"/>
@@ -59,7 +59,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="602" uniqueCount="319">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="606" uniqueCount="323">
   <si>
     <t>XSLOPE Input Template</t>
   </si>
@@ -1137,6 +1137,18 @@
   </si>
   <si>
     <t>l</t>
+  </si>
+  <si>
+    <t>Joint</t>
+  </si>
+  <si>
+    <t>kn</t>
+  </si>
+  <si>
+    <t>ks</t>
+  </si>
+  <si>
+    <t>Jred</t>
   </si>
 </sst>
 </file>
@@ -1644,7 +1656,21 @@
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="35">
+  <dxfs count="37">
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="0" tint="-0.499984740745262"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="0" tint="-0.499984740745262"/>
+        </patternFill>
+      </fill>
+    </dxf>
     <dxf>
       <fill>
         <patternFill>
@@ -1907,16 +1933,16 @@
 <xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
   <xdr:twoCellAnchor>
     <xdr:from>
-      <xdr:col>20</xdr:col>
+      <xdr:col>24</xdr:col>
       <xdr:colOff>217714</xdr:colOff>
       <xdr:row>1</xdr:row>
       <xdr:rowOff>54430</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>25</xdr:col>
+      <xdr:col>29</xdr:col>
       <xdr:colOff>444500</xdr:colOff>
-      <xdr:row>21</xdr:row>
-      <xdr:rowOff>90714</xdr:rowOff>
+      <xdr:row>25</xdr:row>
+      <xdr:rowOff>18143</xdr:rowOff>
     </xdr:to>
     <xdr:sp macro="" textlink="">
       <xdr:nvSpPr>
@@ -1931,8 +1957,8 @@
       </xdr:nvSpPr>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="16455571" y="254001"/>
-          <a:ext cx="3855358" cy="4027713"/>
+          <a:off x="19757571" y="254001"/>
+          <a:ext cx="3855358" cy="4753428"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -2105,7 +2131,7 @@
           </a:r>
           <a:r>
             <a:rPr lang="en-US" sz="1100" b="0"/>
-            <a:t> = residual capacity after rupture (FEM only)</a:t>
+            <a:t> = residual capacity after rupture</a:t>
           </a:r>
         </a:p>
         <a:p>
@@ -2115,7 +2141,7 @@
           </a:r>
           <a:r>
             <a:rPr lang="en-US" sz="1100" b="0"/>
-            <a:t> = modulus of elasticity of reinforcement (FEM only)</a:t>
+            <a:t> = modulus of elasticity of reinforcement</a:t>
           </a:r>
         </a:p>
         <a:p>
@@ -2125,7 +2151,48 @@
           </a:r>
           <a:r>
             <a:rPr lang="en-US" sz="1100" b="0"/>
-            <a:t> = cross-sectional area of reinforcement (FEM only)</a:t>
+            <a:t> = cross-sectional area of reinforcement</a:t>
+          </a:r>
+        </a:p>
+        <a:p>
+          <a:r>
+            <a:rPr lang="en-US" sz="1100" b="1"/>
+            <a:t>Joint</a:t>
+          </a:r>
+          <a:r>
+            <a:rPr lang="en-US" sz="1100" b="0"/>
+            <a:t> = model as slip element; mesh splits along line</a:t>
+          </a:r>
+          <a:endParaRPr lang="en-US" sz="1100" b="0" baseline="0"/>
+        </a:p>
+        <a:p>
+          <a:r>
+            <a:rPr lang="en-US" sz="1100" b="1" baseline="0"/>
+            <a:t>kn</a:t>
+          </a:r>
+          <a:r>
+            <a:rPr lang="en-US" sz="1100" b="0" baseline="0"/>
+            <a:t> = joint normal stiffness (blank = from soil E and size)</a:t>
+          </a:r>
+        </a:p>
+        <a:p>
+          <a:r>
+            <a:rPr lang="en-US" sz="1100" b="1" baseline="0"/>
+            <a:t>ks</a:t>
+          </a:r>
+          <a:r>
+            <a:rPr lang="en-US" sz="1100" b="0" baseline="0"/>
+            <a:t> = joint shear stiffness (blank = from soil G and size)</a:t>
+          </a:r>
+        </a:p>
+        <a:p>
+          <a:r>
+            <a:rPr lang="en-US" sz="1100" b="1" baseline="0"/>
+            <a:t>Jred</a:t>
+          </a:r>
+          <a:r>
+            <a:rPr lang="en-US" sz="1100" b="0" baseline="0"/>
+            <a:t> = reduce joint strength in SSRM (blank = Yes)</a:t>
           </a:r>
           <a:br>
             <a:rPr lang="en-US" sz="1100" b="0"/>
@@ -2884,7 +2951,7 @@
         <v>2</v>
       </c>
       <c r="D5" s="30">
-        <v>26</v>
+        <v>27</v>
       </c>
     </row>
     <row r="7" spans="1:7" x14ac:dyDescent="0.2">
@@ -3277,18 +3344,18 @@
 
 <file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0900-000000000000}">
-  <dimension ref="A2:AD25"/>
+  <dimension ref="A2:AH29"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="4.83203125" style="1" customWidth="1"/>
     <col min="2" max="6" width="10.83203125" style="1" customWidth="1"/>
     <col min="7" max="7" width="13.1640625" customWidth="1"/>
     <col min="10" max="14" width="10.83203125" style="1" customWidth="1"/>
-    <col min="18" max="20" width="10.83203125" style="1" customWidth="1"/>
-    <col min="21" max="21" width="4.33203125" customWidth="1"/>
+    <col min="18" max="24" width="10.83203125" style="1" customWidth="1"/>
+    <col min="25" max="25" width="4.33203125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="2" spans="1:30" x14ac:dyDescent="0.2">
+    <row r="2" spans="1:34" x14ac:dyDescent="0.2">
       <c r="A2" s="12" t="s">
         <v>193</v>
       </c>
@@ -3349,17 +3416,29 @@
       <c r="T2" s="28" t="s">
         <v>256</v>
       </c>
-      <c r="AB2" t="s">
+      <c r="U2" s="28" t="s">
+        <v>319</v>
+      </c>
+      <c r="V2" s="28" t="s">
+        <v>320</v>
+      </c>
+      <c r="W2" s="28" t="s">
+        <v>321</v>
+      </c>
+      <c r="X2" s="28" t="s">
+        <v>322</v>
+      </c>
+      <c r="AF2" t="s">
         <v>257</v>
       </c>
-      <c r="AC2" t="s">
+      <c r="AG2" t="s">
         <v>258</v>
       </c>
-      <c r="AD2" t="s">
+      <c r="AH2" t="s">
         <v>259</v>
       </c>
     </row>
-    <row r="3" spans="1:30" x14ac:dyDescent="0.2">
+    <row r="3" spans="1:34" x14ac:dyDescent="0.2">
       <c r="A3" s="3">
         <v>1</v>
       </c>
@@ -3370,11 +3449,11 @@
       <c r="F3" s="3"/>
       <c r="G3" s="3"/>
       <c r="H3" s="3" t="str">
-        <f t="shared" ref="H3:H22" si="0">IF($G3="","",IFERROR(VLOOKUP($G3,$AB$8:$AD$11,2,0),""))</f>
+        <f t="shared" ref="H3:H22" si="0">IF($G3="","",IFERROR(VLOOKUP($G3,$AF$8:$AH$11,2,0),""))</f>
         <v/>
       </c>
       <c r="I3" s="3" t="str">
-        <f t="shared" ref="I3:I22" si="1">IF($G3="","",IFERROR(VLOOKUP($G3,$AB$8:$AD$11,3,0),""))</f>
+        <f t="shared" ref="I3:I22" si="1">IF($G3="","",IFERROR(VLOOKUP($G3,$AF$8:$AH$11,3,0),""))</f>
         <v/>
       </c>
       <c r="J3" s="3"/>
@@ -3388,17 +3467,21 @@
       <c r="R3" s="3"/>
       <c r="S3" s="3"/>
       <c r="T3" s="3"/>
-      <c r="AB3" t="s">
+      <c r="U3" s="3"/>
+      <c r="V3" s="3"/>
+      <c r="W3" s="3"/>
+      <c r="X3" s="3"/>
+      <c r="AF3" t="s">
         <v>260</v>
       </c>
-      <c r="AC3" t="s">
+      <c r="AG3" t="s">
         <v>261</v>
       </c>
-      <c r="AD3" t="s">
+      <c r="AH3" t="s">
         <v>262</v>
       </c>
     </row>
-    <row r="4" spans="1:30" x14ac:dyDescent="0.2">
+    <row r="4" spans="1:34" x14ac:dyDescent="0.2">
       <c r="A4" s="3">
         <v>2</v>
       </c>
@@ -3427,11 +3510,15 @@
       <c r="R4" s="3"/>
       <c r="S4" s="3"/>
       <c r="T4" s="3"/>
-      <c r="AB4" t="s">
+      <c r="U4" s="3"/>
+      <c r="V4" s="3"/>
+      <c r="W4" s="3"/>
+      <c r="X4" s="3"/>
+      <c r="AF4" t="s">
         <v>263</v>
       </c>
     </row>
-    <row r="5" spans="1:30" x14ac:dyDescent="0.2">
+    <row r="5" spans="1:34" x14ac:dyDescent="0.2">
       <c r="A5" s="3">
         <v>3</v>
       </c>
@@ -3460,11 +3547,15 @@
       <c r="R5" s="3"/>
       <c r="S5" s="3"/>
       <c r="T5" s="3"/>
-      <c r="AB5" t="s">
+      <c r="U5" s="3"/>
+      <c r="V5" s="3"/>
+      <c r="W5" s="3"/>
+      <c r="X5" s="3"/>
+      <c r="AF5" t="s">
         <v>264</v>
       </c>
     </row>
-    <row r="6" spans="1:30" x14ac:dyDescent="0.2">
+    <row r="6" spans="1:34" x14ac:dyDescent="0.2">
       <c r="A6" s="3">
         <v>4</v>
       </c>
@@ -3493,8 +3584,12 @@
       <c r="R6" s="3"/>
       <c r="S6" s="3"/>
       <c r="T6" s="3"/>
-    </row>
-    <row r="7" spans="1:30" x14ac:dyDescent="0.2">
+      <c r="U6" s="3"/>
+      <c r="V6" s="3"/>
+      <c r="W6" s="3"/>
+      <c r="X6" s="3"/>
+    </row>
+    <row r="7" spans="1:34" x14ac:dyDescent="0.2">
       <c r="A7" s="3">
         <v>5</v>
       </c>
@@ -3523,8 +3618,12 @@
       <c r="R7" s="3"/>
       <c r="S7" s="3"/>
       <c r="T7" s="3"/>
-    </row>
-    <row r="8" spans="1:30" x14ac:dyDescent="0.2">
+      <c r="U7" s="3"/>
+      <c r="V7" s="3"/>
+      <c r="W7" s="3"/>
+      <c r="X7" s="3"/>
+    </row>
+    <row r="8" spans="1:34" x14ac:dyDescent="0.2">
       <c r="A8" s="3">
         <v>6</v>
       </c>
@@ -3553,17 +3652,21 @@
       <c r="R8" s="3"/>
       <c r="S8" s="3"/>
       <c r="T8" s="3"/>
-      <c r="AB8" t="s">
+      <c r="U8" s="3"/>
+      <c r="V8" s="3"/>
+      <c r="W8" s="3"/>
+      <c r="X8" s="3"/>
+      <c r="AF8" t="s">
         <v>257</v>
       </c>
-      <c r="AC8" t="s">
+      <c r="AG8" t="s">
         <v>258</v>
       </c>
-      <c r="AD8" t="s">
+      <c r="AH8" t="s">
         <v>259</v>
       </c>
     </row>
-    <row r="9" spans="1:30" x14ac:dyDescent="0.2">
+    <row r="9" spans="1:34" x14ac:dyDescent="0.2">
       <c r="A9" s="3">
         <v>7</v>
       </c>
@@ -3592,17 +3695,21 @@
       <c r="R9" s="3"/>
       <c r="S9" s="3"/>
       <c r="T9" s="3"/>
-      <c r="AB9" t="s">
+      <c r="U9" s="3"/>
+      <c r="V9" s="3"/>
+      <c r="W9" s="3"/>
+      <c r="X9" s="3"/>
+      <c r="AF9" t="s">
         <v>260</v>
       </c>
-      <c r="AC9" t="s">
+      <c r="AG9" t="s">
         <v>261</v>
       </c>
-      <c r="AD9" t="s">
+      <c r="AH9" t="s">
         <v>262</v>
       </c>
     </row>
-    <row r="10" spans="1:30" x14ac:dyDescent="0.2">
+    <row r="10" spans="1:34" x14ac:dyDescent="0.2">
       <c r="A10" s="3">
         <v>8</v>
       </c>
@@ -3631,17 +3738,21 @@
       <c r="R10" s="3"/>
       <c r="S10" s="3"/>
       <c r="T10" s="3"/>
-      <c r="AB10" t="s">
+      <c r="U10" s="3"/>
+      <c r="V10" s="3"/>
+      <c r="W10" s="3"/>
+      <c r="X10" s="3"/>
+      <c r="AF10" t="s">
         <v>263</v>
       </c>
-      <c r="AC10" t="s">
+      <c r="AG10" t="s">
         <v>261</v>
       </c>
-      <c r="AD10" t="s">
+      <c r="AH10" t="s">
         <v>259</v>
       </c>
     </row>
-    <row r="11" spans="1:30" x14ac:dyDescent="0.2">
+    <row r="11" spans="1:34" x14ac:dyDescent="0.2">
       <c r="A11" s="3">
         <v>9</v>
       </c>
@@ -3670,17 +3781,21 @@
       <c r="R11" s="3"/>
       <c r="S11" s="3"/>
       <c r="T11" s="3"/>
-      <c r="AB11" t="s">
+      <c r="U11" s="3"/>
+      <c r="V11" s="3"/>
+      <c r="W11" s="3"/>
+      <c r="X11" s="3"/>
+      <c r="AF11" t="s">
         <v>264</v>
       </c>
-      <c r="AC11" t="s">
+      <c r="AG11" t="s">
         <v>261</v>
       </c>
-      <c r="AD11" t="s">
+      <c r="AH11" t="s">
         <v>259</v>
       </c>
     </row>
-    <row r="12" spans="1:30" x14ac:dyDescent="0.2">
+    <row r="12" spans="1:34" x14ac:dyDescent="0.2">
       <c r="A12" s="3">
         <v>10</v>
       </c>
@@ -3709,8 +3824,12 @@
       <c r="R12" s="3"/>
       <c r="S12" s="3"/>
       <c r="T12" s="3"/>
-    </row>
-    <row r="13" spans="1:30" x14ac:dyDescent="0.2">
+      <c r="U12" s="3"/>
+      <c r="V12" s="3"/>
+      <c r="W12" s="3"/>
+      <c r="X12" s="3"/>
+    </row>
+    <row r="13" spans="1:34" x14ac:dyDescent="0.2">
       <c r="A13" s="3">
         <v>11</v>
       </c>
@@ -3739,8 +3858,12 @@
       <c r="R13" s="3"/>
       <c r="S13" s="3"/>
       <c r="T13" s="3"/>
-    </row>
-    <row r="14" spans="1:30" x14ac:dyDescent="0.2">
+      <c r="U13" s="3"/>
+      <c r="V13" s="3"/>
+      <c r="W13" s="3"/>
+      <c r="X13" s="3"/>
+    </row>
+    <row r="14" spans="1:34" x14ac:dyDescent="0.2">
       <c r="A14" s="3">
         <v>12</v>
       </c>
@@ -3769,8 +3892,12 @@
       <c r="R14" s="3"/>
       <c r="S14" s="3"/>
       <c r="T14" s="3"/>
-    </row>
-    <row r="15" spans="1:30" x14ac:dyDescent="0.2">
+      <c r="U14" s="3"/>
+      <c r="V14" s="3"/>
+      <c r="W14" s="3"/>
+      <c r="X14" s="3"/>
+    </row>
+    <row r="15" spans="1:34" x14ac:dyDescent="0.2">
       <c r="A15" s="3">
         <v>13</v>
       </c>
@@ -3799,8 +3926,12 @@
       <c r="R15" s="3"/>
       <c r="S15" s="3"/>
       <c r="T15" s="3"/>
-    </row>
-    <row r="16" spans="1:30" x14ac:dyDescent="0.2">
+      <c r="U15" s="3"/>
+      <c r="V15" s="3"/>
+      <c r="W15" s="3"/>
+      <c r="X15" s="3"/>
+    </row>
+    <row r="16" spans="1:34" x14ac:dyDescent="0.2">
       <c r="A16" s="3">
         <v>14</v>
       </c>
@@ -3829,8 +3960,12 @@
       <c r="R16" s="3"/>
       <c r="S16" s="3"/>
       <c r="T16" s="3"/>
-    </row>
-    <row r="17" spans="1:23" x14ac:dyDescent="0.2">
+      <c r="U16" s="3"/>
+      <c r="V16" s="3"/>
+      <c r="W16" s="3"/>
+      <c r="X16" s="3"/>
+    </row>
+    <row r="17" spans="1:27" x14ac:dyDescent="0.2">
       <c r="A17" s="3">
         <v>15</v>
       </c>
@@ -3859,8 +3994,12 @@
       <c r="R17" s="3"/>
       <c r="S17" s="3"/>
       <c r="T17" s="3"/>
-    </row>
-    <row r="18" spans="1:23" x14ac:dyDescent="0.2">
+      <c r="U17" s="3"/>
+      <c r="V17" s="3"/>
+      <c r="W17" s="3"/>
+      <c r="X17" s="3"/>
+    </row>
+    <row r="18" spans="1:27" x14ac:dyDescent="0.2">
       <c r="A18" s="3">
         <v>16</v>
       </c>
@@ -3889,8 +4028,12 @@
       <c r="R18" s="3"/>
       <c r="S18" s="3"/>
       <c r="T18" s="3"/>
-    </row>
-    <row r="19" spans="1:23" x14ac:dyDescent="0.2">
+      <c r="U18" s="3"/>
+      <c r="V18" s="3"/>
+      <c r="W18" s="3"/>
+      <c r="X18" s="3"/>
+    </row>
+    <row r="19" spans="1:27" x14ac:dyDescent="0.2">
       <c r="A19" s="3">
         <v>17</v>
       </c>
@@ -3919,8 +4062,12 @@
       <c r="R19" s="3"/>
       <c r="S19" s="3"/>
       <c r="T19" s="3"/>
-    </row>
-    <row r="20" spans="1:23" x14ac:dyDescent="0.2">
+      <c r="U19" s="3"/>
+      <c r="V19" s="3"/>
+      <c r="W19" s="3"/>
+      <c r="X19" s="3"/>
+    </row>
+    <row r="20" spans="1:27" x14ac:dyDescent="0.2">
       <c r="A20" s="3">
         <v>18</v>
       </c>
@@ -3949,8 +4096,12 @@
       <c r="R20" s="3"/>
       <c r="S20" s="3"/>
       <c r="T20" s="3"/>
-    </row>
-    <row r="21" spans="1:23" x14ac:dyDescent="0.2">
+      <c r="U20" s="3"/>
+      <c r="V20" s="3"/>
+      <c r="W20" s="3"/>
+      <c r="X20" s="3"/>
+    </row>
+    <row r="21" spans="1:27" x14ac:dyDescent="0.2">
       <c r="A21" s="3">
         <v>19</v>
       </c>
@@ -3979,8 +4130,12 @@
       <c r="R21" s="3"/>
       <c r="S21" s="3"/>
       <c r="T21" s="3"/>
-    </row>
-    <row r="22" spans="1:23" x14ac:dyDescent="0.2">
+      <c r="U21" s="3"/>
+      <c r="V21" s="3"/>
+      <c r="W21" s="3"/>
+      <c r="X21" s="3"/>
+    </row>
+    <row r="22" spans="1:27" x14ac:dyDescent="0.2">
       <c r="A22" s="3">
         <v>20</v>
       </c>
@@ -4009,39 +4164,60 @@
       <c r="R22" s="3"/>
       <c r="S22" s="3"/>
       <c r="T22" s="3"/>
-    </row>
-    <row r="23" spans="1:23" x14ac:dyDescent="0.2">
-      <c r="V23" s="42"/>
-      <c r="W23" t="s">
-        <v>91</v>
-      </c>
-    </row>
-    <row r="24" spans="1:23" x14ac:dyDescent="0.2">
+      <c r="U22" s="3"/>
+      <c r="V22" s="3"/>
+      <c r="W22" s="3"/>
+      <c r="X22" s="3"/>
+    </row>
+    <row r="24" spans="1:27" x14ac:dyDescent="0.2">
       <c r="K24" s="9"/>
       <c r="L24" s="9"/>
-      <c r="V24" s="26"/>
-      <c r="W24" s="9" t="s">
-        <v>96</v>
-      </c>
-    </row>
-    <row r="25" spans="1:23" x14ac:dyDescent="0.2">
+    </row>
+    <row r="25" spans="1:27" x14ac:dyDescent="0.2">
       <c r="K25" s="9"/>
       <c r="L25" s="9"/>
-      <c r="V25" s="29"/>
-      <c r="W25" s="9" t="s">
+    </row>
+    <row r="27" spans="1:27" x14ac:dyDescent="0.2">
+      <c r="Z27" s="42"/>
+      <c r="AA27" t="s">
+        <v>91</v>
+      </c>
+    </row>
+    <row r="28" spans="1:27" x14ac:dyDescent="0.2">
+      <c r="Z28" s="26"/>
+      <c r="AA28" s="9" t="s">
+        <v>96</v>
+      </c>
+    </row>
+    <row r="29" spans="1:27" x14ac:dyDescent="0.2">
+      <c r="Z29" s="29"/>
+      <c r="AA29" s="9" t="s">
         <v>103</v>
       </c>
     </row>
   </sheetData>
-  <dataValidations count="3">
+  <conditionalFormatting sqref="K3:L22">
+    <cfRule type="expression" dxfId="1" priority="1">
+      <formula>$U3="Yes"</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="V3:X22">
+    <cfRule type="expression" dxfId="0" priority="4">
+      <formula>$U3&lt;&gt;"Yes"</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <dataValidations count="4">
     <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="G3:G22" xr:uid="{00000000-0002-0000-0900-000000000000}">
-      <formula1>$AB$2:$AB$5</formula1>
+      <formula1>$AF$2:$AF$5</formula1>
     </dataValidation>
     <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="H3:H22" xr:uid="{00000000-0002-0000-0900-000001000000}">
-      <formula1>$AC$2:$AC$3</formula1>
+      <formula1>$AG$2:$AG$3</formula1>
     </dataValidation>
     <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="I3:I22" xr:uid="{00000000-0002-0000-0900-000002000000}">
-      <formula1>$AD$2:$AD$3</formula1>
+      <formula1>$AH$2:$AH$3</formula1>
+    </dataValidation>
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="U3:U22 X3:X22" xr:uid="{8FB27197-C456-2D4D-8100-E78D5059F972}">
+      <formula1>"Yes,No"</formula1>
     </dataValidation>
   </dataValidations>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -8059,83 +8235,83 @@
     <mergeCell ref="C9:Z9"/>
   </mergeCells>
   <conditionalFormatting sqref="F11:K52 AB11:AF52">
-    <cfRule type="expression" dxfId="34" priority="6">
+    <cfRule type="expression" dxfId="36" priority="6">
       <formula>$E11="hb"</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="33" priority="7">
+    <cfRule type="expression" dxfId="35" priority="7">
       <formula>$E11="pow"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="F11:L52 O11:R52">
-    <cfRule type="expression" dxfId="32" priority="19">
+    <cfRule type="expression" dxfId="34" priority="19">
       <formula>$E11="elastic"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="G11:G52">
-    <cfRule type="expression" dxfId="31" priority="8">
+    <cfRule type="expression" dxfId="33" priority="8">
       <formula>$E11="cp"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="H11:I52">
-    <cfRule type="expression" dxfId="30" priority="9">
+    <cfRule type="expression" dxfId="32" priority="9">
       <formula>$E11="mc"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="J11:K52">
-    <cfRule type="expression" dxfId="29" priority="10">
+    <cfRule type="expression" dxfId="31" priority="10">
       <formula>$E11="cp"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="P11:P52">
-    <cfRule type="expression" dxfId="28" priority="13">
+    <cfRule type="expression" dxfId="30" priority="13">
       <formula>AND($O11&lt;&gt;"",$O11&lt;&gt;"ru")</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="Q11:R52">
-    <cfRule type="expression" dxfId="27" priority="23">
+    <cfRule type="expression" dxfId="29" priority="23">
       <formula>$E11="cp"</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="26" priority="24">
+    <cfRule type="expression" dxfId="28" priority="24">
       <formula>AND($O11&lt;&gt;"",$O11&lt;&gt;"piezo",$O11&lt;&gt;"seep")</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="S11:V52">
-    <cfRule type="expression" dxfId="25" priority="11">
+    <cfRule type="expression" dxfId="27" priority="11">
       <formula>AND($E11&lt;&gt;"",$E11&lt;&gt;"pow")</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="W11:Z52">
-    <cfRule type="expression" dxfId="24" priority="12">
+    <cfRule type="expression" dxfId="26" priority="12">
       <formula>AND($E11&lt;&gt;"",$E11&lt;&gt;"hb")</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="AB11:AF52">
-    <cfRule type="expression" dxfId="23" priority="21">
+    <cfRule type="expression" dxfId="25" priority="21">
       <formula>$E11="elastic"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="AC11:AC52">
-    <cfRule type="expression" dxfId="22" priority="14">
+    <cfRule type="expression" dxfId="24" priority="14">
       <formula>$E11="cp"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="AD11:AD52">
-    <cfRule type="expression" dxfId="21" priority="15">
+    <cfRule type="expression" dxfId="23" priority="15">
       <formula>$E11="mc"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="AE11:AF52">
-    <cfRule type="expression" dxfId="20" priority="16">
+    <cfRule type="expression" dxfId="22" priority="16">
       <formula>$E11="cp"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="AK11:AL52">
-    <cfRule type="expression" dxfId="19" priority="17">
+    <cfRule type="expression" dxfId="21" priority="17">
       <formula>OR($AJ11="vg",$AJ11="gard")</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="AM11:AO52">
-    <cfRule type="expression" dxfId="18" priority="1">
+    <cfRule type="expression" dxfId="20" priority="1">
       <formula>$AJ11="lf"</formula>
     </cfRule>
   </conditionalFormatting>
@@ -10849,77 +11025,77 @@
     <mergeCell ref="V7:W7"/>
   </mergeCells>
   <conditionalFormatting sqref="B6 A7:B7">
-    <cfRule type="expression" dxfId="17" priority="1">
+    <cfRule type="expression" dxfId="19" priority="1">
       <formula>AND($B$5&lt;&gt;"",$B$5&lt;&gt;"material")</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="E6 D7:E7">
-    <cfRule type="expression" dxfId="16" priority="2">
+    <cfRule type="expression" dxfId="18" priority="2">
       <formula>AND($E$5&lt;&gt;"",$E$5&lt;&gt;"material")</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="H6 G7:H7">
-    <cfRule type="expression" dxfId="15" priority="3">
+    <cfRule type="expression" dxfId="17" priority="3">
       <formula>AND($H$5&lt;&gt;"",$H$5&lt;&gt;"material")</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="K6 J7:K7">
-    <cfRule type="expression" dxfId="14" priority="4">
+    <cfRule type="expression" dxfId="16" priority="4">
       <formula>AND($K$5&lt;&gt;"",$K$5&lt;&gt;"material")</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="N6 M7:N7">
-    <cfRule type="expression" dxfId="13" priority="5">
+    <cfRule type="expression" dxfId="15" priority="5">
       <formula>AND($N$5&lt;&gt;"",$N$5&lt;&gt;"material")</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="Q6 P7:Q7">
-    <cfRule type="expression" dxfId="12" priority="6">
+    <cfRule type="expression" dxfId="14" priority="6">
       <formula>AND($Q$5&lt;&gt;"",$Q$5&lt;&gt;"material")</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="T6 S7:T7">
-    <cfRule type="expression" dxfId="11" priority="7">
+    <cfRule type="expression" dxfId="13" priority="7">
       <formula>AND($T$5&lt;&gt;"",$T$5&lt;&gt;"material")</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="W6 V7:W7">
-    <cfRule type="expression" dxfId="10" priority="8">
+    <cfRule type="expression" dxfId="12" priority="8">
       <formula>AND($W$5&lt;&gt;"",$W$5&lt;&gt;"material")</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="Z6 Y7:Z7">
-    <cfRule type="expression" dxfId="9" priority="9">
+    <cfRule type="expression" dxfId="11" priority="9">
       <formula>AND($Z$5&lt;&gt;"",$Z$5&lt;&gt;"material")</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="AC6 AB7:AC7">
-    <cfRule type="expression" dxfId="8" priority="10">
+    <cfRule type="expression" dxfId="10" priority="10">
       <formula>AND($AC$5&lt;&gt;"",$AC$5&lt;&gt;"material")</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="AF6 AE7:AF7">
-    <cfRule type="expression" dxfId="7" priority="11">
+    <cfRule type="expression" dxfId="9" priority="11">
       <formula>AND($AF$5&lt;&gt;"",$AF$5&lt;&gt;"material")</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="AI6 AH7:AI7">
-    <cfRule type="expression" dxfId="6" priority="12">
+    <cfRule type="expression" dxfId="8" priority="12">
       <formula>AND($AI$5&lt;&gt;"",$AI$5&lt;&gt;"material")</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="AL6 AK7:AL7">
-    <cfRule type="expression" dxfId="5" priority="13">
+    <cfRule type="expression" dxfId="7" priority="13">
       <formula>AND($AL$5&lt;&gt;"",$AL$5&lt;&gt;"material")</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="AO6 AN7:AO7">
-    <cfRule type="expression" dxfId="4" priority="14">
+    <cfRule type="expression" dxfId="6" priority="14">
       <formula>AND($AO$5&lt;&gt;"",$AO$5&lt;&gt;"material")</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="AR6 AQ7:AR7">
-    <cfRule type="expression" dxfId="3" priority="15">
+    <cfRule type="expression" dxfId="5" priority="15">
       <formula>AND($AR$5&lt;&gt;"",$AR$5&lt;&gt;"material")</formula>
     </cfRule>
   </conditionalFormatting>
@@ -11358,17 +11534,17 @@
     </row>
   </sheetData>
   <conditionalFormatting sqref="E3:E42">
-    <cfRule type="expression" dxfId="2" priority="3">
+    <cfRule type="expression" dxfId="4" priority="3">
       <formula>OR($D3="Intercept", $D3="Radius")</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="F3:G42">
-    <cfRule type="expression" dxfId="1" priority="2">
+    <cfRule type="expression" dxfId="3" priority="2">
       <formula>OR($D3="Depth",$D3="Radius")</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="H3:H42">
-    <cfRule type="expression" dxfId="0" priority="1">
+    <cfRule type="expression" dxfId="2" priority="1">
       <formula>OR($D3="Depth",$D3="Intercept")</formula>
     </cfRule>
   </conditionalFormatting>

</xml_diff>

<commit_message>
template v27: the joints sheet (slip joints with no reinforcement) and ten more reinforce rows
Owner's edit. A joints sheet after reinforce — Label, endpoints, c, phi, t_cut,
kn, ks, Jred (Yes/No list), rows 3-32, help box — and the reinforce table
extended from 20 rows to 30 with its lists and gray-out rules following. The
version stays 27: it never shipped, so nothing in the wild carries it. Packaged
copy synced byte-identical.

Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01XjjT2aBxw8gY7EFdpoUcpj
</commit_message>
<xml_diff>
--- a/docs/inputs/input_template.xlsx
+++ b/docs/inputs/input_template.xlsx
@@ -5,12 +5,12 @@
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/njones/python_projects/xslope/docs/inputs/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/njones/python_projects/xslope/.claude/worktrees/joints-r1/docs/inputs/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{904BD95E-2C21-0841-A7DF-ECBA420EAAD7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{42723C2E-F56A-D348-AC02-78080B1F6523}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="27680" yWindow="3200" windowWidth="31600" windowHeight="18400" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="9960" yWindow="2320" windowWidth="30380" windowHeight="22500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="main" sheetId="1" r:id="rId1"/>
@@ -23,11 +23,12 @@
     <sheet name="dloads" sheetId="8" r:id="rId8"/>
     <sheet name="dloads (2)" sheetId="9" r:id="rId9"/>
     <sheet name="reinforce" sheetId="10" r:id="rId10"/>
-    <sheet name="piles" sheetId="11" r:id="rId11"/>
-    <sheet name="lloads" sheetId="12" r:id="rId12"/>
-    <sheet name="seep bc" sheetId="13" r:id="rId13"/>
-    <sheet name="seep bc (2)" sheetId="14" r:id="rId14"/>
-    <sheet name="tseep" sheetId="15" r:id="rId15"/>
+    <sheet name="joints" sheetId="16" r:id="rId11"/>
+    <sheet name="piles" sheetId="11" r:id="rId12"/>
+    <sheet name="lloads" sheetId="12" r:id="rId13"/>
+    <sheet name="seep bc" sheetId="13" r:id="rId14"/>
+    <sheet name="seep bc (2)" sheetId="14" r:id="rId15"/>
+    <sheet name="tseep" sheetId="15" r:id="rId16"/>
   </sheets>
   <definedNames>
     <definedName name="crack_depth">main!$D$11</definedName>
@@ -59,7 +60,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="606" uniqueCount="323">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="621" uniqueCount="326">
   <si>
     <t>XSLOPE Input Template</t>
   </si>
@@ -1149,6 +1150,15 @@
   </si>
   <si>
     <t>Jred</t>
+  </si>
+  <si>
+    <t>phi</t>
+  </si>
+  <si>
+    <t>joints</t>
+  </si>
+  <si>
+    <t>Slip joints (interfaces with no reinforcement)</t>
   </si>
 </sst>
 </file>
@@ -1656,7 +1666,7 @@
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="37">
+  <dxfs count="38">
     <dxf>
       <fill>
         <patternFill>
@@ -1916,6 +1926,13 @@
         </patternFill>
       </fill>
     </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="0" tint="-0.499984740745262"/>
+        </patternFill>
+      </fill>
+    </dxf>
   </dxfs>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
   <extLst>
@@ -1934,15 +1951,15 @@
   <xdr:twoCellAnchor>
     <xdr:from>
       <xdr:col>24</xdr:col>
-      <xdr:colOff>217714</xdr:colOff>
-      <xdr:row>1</xdr:row>
-      <xdr:rowOff>54430</xdr:rowOff>
+      <xdr:colOff>326571</xdr:colOff>
+      <xdr:row>5</xdr:row>
+      <xdr:rowOff>9073</xdr:rowOff>
     </xdr:from>
     <xdr:to>
       <xdr:col>29</xdr:col>
-      <xdr:colOff>444500</xdr:colOff>
-      <xdr:row>25</xdr:row>
-      <xdr:rowOff>18143</xdr:rowOff>
+      <xdr:colOff>553357</xdr:colOff>
+      <xdr:row>28</xdr:row>
+      <xdr:rowOff>172358</xdr:rowOff>
     </xdr:to>
     <xdr:sp macro="" textlink="">
       <xdr:nvSpPr>
@@ -1957,7 +1974,7 @@
       </xdr:nvSpPr>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="19757571" y="254001"/>
+          <a:off x="19866428" y="1006930"/>
           <a:ext cx="3855358" cy="4753428"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
@@ -2086,7 +2103,7 @@
           </a:r>
           <a:r>
             <a:rPr lang="en-US" sz="1100" b="0"/>
-            <a:t> = soii-reinforcement interface adhesion (blank</a:t>
+            <a:t> = soil-reinforcement interface adhesion (blank</a:t>
           </a:r>
           <a:r>
             <a:rPr lang="en-US" sz="1100" b="0" baseline="0"/>
@@ -2207,6 +2224,177 @@
 </file>
 
 <file path=xl/drawings/drawing2.xml><?xml version="1.0" encoding="utf-8"?>
+<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>12</xdr:col>
+      <xdr:colOff>308428</xdr:colOff>
+      <xdr:row>2</xdr:row>
+      <xdr:rowOff>172358</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>17</xdr:col>
+      <xdr:colOff>381000</xdr:colOff>
+      <xdr:row>10</xdr:row>
+      <xdr:rowOff>81643</xdr:rowOff>
+    </xdr:to>
+    <xdr:sp macro="" textlink="">
+      <xdr:nvSpPr>
+        <xdr:cNvPr id="2" name="TextBox 1">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{1DA6D3C4-0920-BE4C-AFB2-D27825A644F5}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvSpPr txBox="1"/>
+      </xdr:nvSpPr>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="9760857" y="571501"/>
+          <a:ext cx="3701143" cy="1505856"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+        <a:solidFill>
+          <a:schemeClr val="lt1"/>
+        </a:solidFill>
+        <a:ln w="9525" cmpd="sng">
+          <a:solidFill>
+            <a:schemeClr val="lt1">
+              <a:shade val="50000"/>
+            </a:schemeClr>
+          </a:solidFill>
+        </a:ln>
+      </xdr:spPr>
+      <xdr:style>
+        <a:lnRef idx="0">
+          <a:scrgbClr r="0" g="0" b="0"/>
+        </a:lnRef>
+        <a:fillRef idx="0">
+          <a:scrgbClr r="0" g="0" b="0"/>
+        </a:fillRef>
+        <a:effectRef idx="0">
+          <a:scrgbClr r="0" g="0" b="0"/>
+        </a:effectRef>
+        <a:fontRef idx="minor">
+          <a:schemeClr val="dk1"/>
+        </a:fontRef>
+      </xdr:style>
+      <xdr:txBody>
+        <a:bodyPr vertOverflow="clip" horzOverflow="clip" wrap="square" rtlCol="0" anchor="t"/>
+        <a:lstStyle/>
+        <a:p>
+          <a:r>
+            <a:rPr lang="en-US" sz="1100" b="1"/>
+            <a:t>Label</a:t>
+          </a:r>
+          <a:r>
+            <a:rPr lang="en-US" sz="1100" b="0"/>
+            <a:t> = name used in error messages, summaries, and plots</a:t>
+          </a:r>
+        </a:p>
+        <a:p>
+          <a:pPr marL="0" marR="0" lvl="0" indent="0" defTabSz="914400" eaLnBrk="1" fontAlgn="auto" latinLnBrk="0" hangingPunct="1">
+            <a:lnSpc>
+              <a:spcPct val="100000"/>
+            </a:lnSpc>
+            <a:spcBef>
+              <a:spcPts val="0"/>
+            </a:spcBef>
+            <a:spcAft>
+              <a:spcPts val="0"/>
+            </a:spcAft>
+            <a:buClrTx/>
+            <a:buSzTx/>
+            <a:buFontTx/>
+            <a:buNone/>
+            <a:tabLst/>
+            <a:defRPr/>
+          </a:pPr>
+          <a:r>
+            <a:rPr lang="en-US" sz="1100" b="1"/>
+            <a:t>(x1, y1), (x2, y2) </a:t>
+          </a:r>
+          <a:r>
+            <a:rPr lang="en-US" sz="1100" b="0"/>
+            <a:t>= start and end of joint line</a:t>
+          </a:r>
+          <a:endParaRPr lang="en-US" sz="1100" b="1"/>
+        </a:p>
+        <a:p>
+          <a:r>
+            <a:rPr lang="en-US" sz="1100" b="1"/>
+            <a:t>c</a:t>
+          </a:r>
+          <a:r>
+            <a:rPr lang="en-US" sz="1100" b="0" baseline="0"/>
+            <a:t> = joint cohesion</a:t>
+          </a:r>
+        </a:p>
+        <a:p>
+          <a:r>
+            <a:rPr lang="en-US" sz="1100" b="1" baseline="0"/>
+            <a:t>phi</a:t>
+          </a:r>
+          <a:r>
+            <a:rPr lang="en-US" sz="1100" b="0" baseline="0"/>
+            <a:t> = joint friction angle, degrees</a:t>
+          </a:r>
+        </a:p>
+        <a:p>
+          <a:r>
+            <a:rPr lang="en-US" sz="1100" b="1" baseline="0"/>
+            <a:t>t_cut</a:t>
+          </a:r>
+          <a:r>
+            <a:rPr lang="en-US" sz="1100" b="0" baseline="0"/>
+            <a:t> = tension cutoff</a:t>
+          </a:r>
+        </a:p>
+        <a:p>
+          <a:r>
+            <a:rPr lang="en-US" sz="1100" b="1" baseline="0"/>
+            <a:t>kn</a:t>
+          </a:r>
+          <a:r>
+            <a:rPr lang="en-US" sz="1100" b="0" baseline="0"/>
+            <a:t> = joint normal stiffness (blank = from soil E and size)</a:t>
+          </a:r>
+        </a:p>
+        <a:p>
+          <a:r>
+            <a:rPr lang="en-US" sz="1100" b="1" baseline="0"/>
+            <a:t>ks</a:t>
+          </a:r>
+          <a:r>
+            <a:rPr lang="en-US" sz="1100" b="0" baseline="0"/>
+            <a:t> = joint shear stiffness (blank = from soil G and size)</a:t>
+          </a:r>
+        </a:p>
+        <a:p>
+          <a:r>
+            <a:rPr lang="en-US" sz="1100" b="1" baseline="0"/>
+            <a:t>Jred</a:t>
+          </a:r>
+          <a:r>
+            <a:rPr lang="en-US" sz="1100" b="0" baseline="0"/>
+            <a:t> = reduce joint strength in SSRM (blank = Yes)</a:t>
+          </a:r>
+          <a:br>
+            <a:rPr lang="en-US" sz="1100" b="0"/>
+          </a:br>
+          <a:endParaRPr lang="en-US" sz="1100" b="0"/>
+        </a:p>
+      </xdr:txBody>
+    </xdr:sp>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+</xdr:wsDr>
+</file>
+
+<file path=xl/drawings/drawing3.xml><?xml version="1.0" encoding="utf-8"?>
 <xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
   <xdr:twoCellAnchor>
     <xdr:from>
@@ -3094,10 +3282,10 @@
         <v>36</v>
       </c>
       <c r="F17" s="1" t="s">
-        <v>37</v>
-      </c>
-      <c r="G17" t="s">
-        <v>38</v>
+        <v>324</v>
+      </c>
+      <c r="G17" s="9" t="s">
+        <v>325</v>
       </c>
     </row>
     <row r="18" spans="2:7" x14ac:dyDescent="0.2">
@@ -3105,10 +3293,10 @@
         <v>39</v>
       </c>
       <c r="F18" s="1" t="s">
-        <v>40</v>
+        <v>37</v>
       </c>
       <c r="G18" t="s">
-        <v>41</v>
+        <v>38</v>
       </c>
     </row>
     <row r="19" spans="2:7" x14ac:dyDescent="0.2">
@@ -3116,10 +3304,10 @@
         <v>42</v>
       </c>
       <c r="F19" s="1" t="s">
-        <v>43</v>
-      </c>
-      <c r="G19" s="9" t="s">
-        <v>44</v>
+        <v>40</v>
+      </c>
+      <c r="G19" t="s">
+        <v>41</v>
       </c>
     </row>
     <row r="20" spans="2:7" x14ac:dyDescent="0.2">
@@ -3127,10 +3315,10 @@
         <v>312</v>
       </c>
       <c r="F20" s="1" t="s">
-        <v>46</v>
+        <v>43</v>
       </c>
       <c r="G20" s="9" t="s">
-        <v>47</v>
+        <v>44</v>
       </c>
     </row>
     <row r="21" spans="2:7" x14ac:dyDescent="0.2">
@@ -3138,17 +3326,22 @@
         <v>45</v>
       </c>
       <c r="F21" s="1" t="s">
-        <v>49</v>
-      </c>
-      <c r="G21" t="s">
-        <v>50</v>
+        <v>46</v>
+      </c>
+      <c r="G21" s="9" t="s">
+        <v>47</v>
       </c>
     </row>
     <row r="22" spans="2:7" x14ac:dyDescent="0.2">
       <c r="C22" s="14" t="s">
         <v>48</v>
       </c>
-      <c r="F22" s="1"/>
+      <c r="F22" s="1" t="s">
+        <v>49</v>
+      </c>
+      <c r="G22" t="s">
+        <v>50</v>
+      </c>
     </row>
     <row r="23" spans="2:7" x14ac:dyDescent="0.2">
       <c r="B23" s="1"/>
@@ -3344,7 +3537,7 @@
 
 <file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0900-000000000000}">
-  <dimension ref="A2:AH29"/>
+  <dimension ref="A2:AJ32"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="4.83203125" style="1" customWidth="1"/>
@@ -3355,7 +3548,7 @@
     <col min="25" max="25" width="4.33203125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="2" spans="1:34" x14ac:dyDescent="0.2">
+    <row r="2" spans="1:36" x14ac:dyDescent="0.2">
       <c r="A2" s="12" t="s">
         <v>193</v>
       </c>
@@ -3428,17 +3621,21 @@
       <c r="X2" s="28" t="s">
         <v>322</v>
       </c>
-      <c r="AF2" t="s">
+      <c r="Z2" s="42"/>
+      <c r="AA2" t="s">
+        <v>91</v>
+      </c>
+      <c r="AH2" t="s">
         <v>257</v>
       </c>
-      <c r="AG2" t="s">
+      <c r="AI2" t="s">
         <v>258</v>
       </c>
-      <c r="AH2" t="s">
+      <c r="AJ2" t="s">
         <v>259</v>
       </c>
     </row>
-    <row r="3" spans="1:34" x14ac:dyDescent="0.2">
+    <row r="3" spans="1:36" x14ac:dyDescent="0.2">
       <c r="A3" s="3">
         <v>1</v>
       </c>
@@ -3449,11 +3646,11 @@
       <c r="F3" s="3"/>
       <c r="G3" s="3"/>
       <c r="H3" s="3" t="str">
-        <f t="shared" ref="H3:H22" si="0">IF($G3="","",IFERROR(VLOOKUP($G3,$AF$8:$AH$11,2,0),""))</f>
+        <f t="shared" ref="H3:H32" si="0">IF($G3="","",IFERROR(VLOOKUP($G3,$AH$8:$AJ$11,2,0),""))</f>
         <v/>
       </c>
       <c r="I3" s="3" t="str">
-        <f t="shared" ref="I3:I22" si="1">IF($G3="","",IFERROR(VLOOKUP($G3,$AF$8:$AH$11,3,0),""))</f>
+        <f t="shared" ref="I3:I32" si="1">IF($G3="","",IFERROR(VLOOKUP($G3,$AH$8:$AJ$11,3,0),""))</f>
         <v/>
       </c>
       <c r="J3" s="3"/>
@@ -3471,17 +3668,21 @@
       <c r="V3" s="3"/>
       <c r="W3" s="3"/>
       <c r="X3" s="3"/>
-      <c r="AF3" t="s">
+      <c r="Z3" s="26"/>
+      <c r="AA3" s="9" t="s">
+        <v>96</v>
+      </c>
+      <c r="AH3" t="s">
         <v>260</v>
       </c>
-      <c r="AG3" t="s">
+      <c r="AI3" t="s">
         <v>261</v>
       </c>
-      <c r="AH3" t="s">
+      <c r="AJ3" t="s">
         <v>262</v>
       </c>
     </row>
-    <row r="4" spans="1:34" x14ac:dyDescent="0.2">
+    <row r="4" spans="1:36" x14ac:dyDescent="0.2">
       <c r="A4" s="3">
         <v>2</v>
       </c>
@@ -3514,11 +3715,15 @@
       <c r="V4" s="3"/>
       <c r="W4" s="3"/>
       <c r="X4" s="3"/>
-      <c r="AF4" t="s">
+      <c r="Z4" s="29"/>
+      <c r="AA4" s="9" t="s">
+        <v>103</v>
+      </c>
+      <c r="AH4" t="s">
         <v>263</v>
       </c>
     </row>
-    <row r="5" spans="1:34" x14ac:dyDescent="0.2">
+    <row r="5" spans="1:36" x14ac:dyDescent="0.2">
       <c r="A5" s="3">
         <v>3</v>
       </c>
@@ -3551,11 +3756,11 @@
       <c r="V5" s="3"/>
       <c r="W5" s="3"/>
       <c r="X5" s="3"/>
-      <c r="AF5" t="s">
+      <c r="AH5" t="s">
         <v>264</v>
       </c>
     </row>
-    <row r="6" spans="1:34" x14ac:dyDescent="0.2">
+    <row r="6" spans="1:36" x14ac:dyDescent="0.2">
       <c r="A6" s="3">
         <v>4</v>
       </c>
@@ -3589,7 +3794,7 @@
       <c r="W6" s="3"/>
       <c r="X6" s="3"/>
     </row>
-    <row r="7" spans="1:34" x14ac:dyDescent="0.2">
+    <row r="7" spans="1:36" x14ac:dyDescent="0.2">
       <c r="A7" s="3">
         <v>5</v>
       </c>
@@ -3623,7 +3828,7 @@
       <c r="W7" s="3"/>
       <c r="X7" s="3"/>
     </row>
-    <row r="8" spans="1:34" x14ac:dyDescent="0.2">
+    <row r="8" spans="1:36" x14ac:dyDescent="0.2">
       <c r="A8" s="3">
         <v>6</v>
       </c>
@@ -3656,17 +3861,17 @@
       <c r="V8" s="3"/>
       <c r="W8" s="3"/>
       <c r="X8" s="3"/>
-      <c r="AF8" t="s">
+      <c r="AH8" t="s">
         <v>257</v>
       </c>
-      <c r="AG8" t="s">
+      <c r="AI8" t="s">
         <v>258</v>
       </c>
-      <c r="AH8" t="s">
+      <c r="AJ8" t="s">
         <v>259</v>
       </c>
     </row>
-    <row r="9" spans="1:34" x14ac:dyDescent="0.2">
+    <row r="9" spans="1:36" x14ac:dyDescent="0.2">
       <c r="A9" s="3">
         <v>7</v>
       </c>
@@ -3699,17 +3904,17 @@
       <c r="V9" s="3"/>
       <c r="W9" s="3"/>
       <c r="X9" s="3"/>
-      <c r="AF9" t="s">
+      <c r="AH9" t="s">
         <v>260</v>
       </c>
-      <c r="AG9" t="s">
+      <c r="AI9" t="s">
         <v>261</v>
       </c>
-      <c r="AH9" t="s">
+      <c r="AJ9" t="s">
         <v>262</v>
       </c>
     </row>
-    <row r="10" spans="1:34" x14ac:dyDescent="0.2">
+    <row r="10" spans="1:36" x14ac:dyDescent="0.2">
       <c r="A10" s="3">
         <v>8</v>
       </c>
@@ -3742,17 +3947,17 @@
       <c r="V10" s="3"/>
       <c r="W10" s="3"/>
       <c r="X10" s="3"/>
-      <c r="AF10" t="s">
+      <c r="AH10" t="s">
         <v>263</v>
       </c>
-      <c r="AG10" t="s">
+      <c r="AI10" t="s">
         <v>261</v>
       </c>
-      <c r="AH10" t="s">
+      <c r="AJ10" t="s">
         <v>259</v>
       </c>
     </row>
-    <row r="11" spans="1:34" x14ac:dyDescent="0.2">
+    <row r="11" spans="1:36" x14ac:dyDescent="0.2">
       <c r="A11" s="3">
         <v>9</v>
       </c>
@@ -3785,17 +3990,17 @@
       <c r="V11" s="3"/>
       <c r="W11" s="3"/>
       <c r="X11" s="3"/>
-      <c r="AF11" t="s">
+      <c r="AH11" t="s">
         <v>264</v>
       </c>
-      <c r="AG11" t="s">
+      <c r="AI11" t="s">
         <v>261</v>
       </c>
-      <c r="AH11" t="s">
+      <c r="AJ11" t="s">
         <v>259</v>
       </c>
     </row>
-    <row r="12" spans="1:34" x14ac:dyDescent="0.2">
+    <row r="12" spans="1:36" x14ac:dyDescent="0.2">
       <c r="A12" s="3">
         <v>10</v>
       </c>
@@ -3829,7 +4034,7 @@
       <c r="W12" s="3"/>
       <c r="X12" s="3"/>
     </row>
-    <row r="13" spans="1:34" x14ac:dyDescent="0.2">
+    <row r="13" spans="1:36" x14ac:dyDescent="0.2">
       <c r="A13" s="3">
         <v>11</v>
       </c>
@@ -3863,7 +4068,7 @@
       <c r="W13" s="3"/>
       <c r="X13" s="3"/>
     </row>
-    <row r="14" spans="1:34" x14ac:dyDescent="0.2">
+    <row r="14" spans="1:36" x14ac:dyDescent="0.2">
       <c r="A14" s="3">
         <v>12</v>
       </c>
@@ -3897,7 +4102,7 @@
       <c r="W14" s="3"/>
       <c r="X14" s="3"/>
     </row>
-    <row r="15" spans="1:34" x14ac:dyDescent="0.2">
+    <row r="15" spans="1:36" x14ac:dyDescent="0.2">
       <c r="A15" s="3">
         <v>13</v>
       </c>
@@ -3931,7 +4136,7 @@
       <c r="W15" s="3"/>
       <c r="X15" s="3"/>
     </row>
-    <row r="16" spans="1:34" x14ac:dyDescent="0.2">
+    <row r="16" spans="1:36" x14ac:dyDescent="0.2">
       <c r="A16" s="3">
         <v>14</v>
       </c>
@@ -3965,7 +4170,7 @@
       <c r="W16" s="3"/>
       <c r="X16" s="3"/>
     </row>
-    <row r="17" spans="1:27" x14ac:dyDescent="0.2">
+    <row r="17" spans="1:24" x14ac:dyDescent="0.2">
       <c r="A17" s="3">
         <v>15</v>
       </c>
@@ -3999,7 +4204,7 @@
       <c r="W17" s="3"/>
       <c r="X17" s="3"/>
     </row>
-    <row r="18" spans="1:27" x14ac:dyDescent="0.2">
+    <row r="18" spans="1:24" x14ac:dyDescent="0.2">
       <c r="A18" s="3">
         <v>16</v>
       </c>
@@ -4033,7 +4238,7 @@
       <c r="W18" s="3"/>
       <c r="X18" s="3"/>
     </row>
-    <row r="19" spans="1:27" x14ac:dyDescent="0.2">
+    <row r="19" spans="1:24" x14ac:dyDescent="0.2">
       <c r="A19" s="3">
         <v>17</v>
       </c>
@@ -4067,7 +4272,7 @@
       <c r="W19" s="3"/>
       <c r="X19" s="3"/>
     </row>
-    <row r="20" spans="1:27" x14ac:dyDescent="0.2">
+    <row r="20" spans="1:24" x14ac:dyDescent="0.2">
       <c r="A20" s="3">
         <v>18</v>
       </c>
@@ -4101,7 +4306,7 @@
       <c r="W20" s="3"/>
       <c r="X20" s="3"/>
     </row>
-    <row r="21" spans="1:27" x14ac:dyDescent="0.2">
+    <row r="21" spans="1:24" x14ac:dyDescent="0.2">
       <c r="A21" s="3">
         <v>19</v>
       </c>
@@ -4135,7 +4340,7 @@
       <c r="W21" s="3"/>
       <c r="X21" s="3"/>
     </row>
-    <row r="22" spans="1:27" x14ac:dyDescent="0.2">
+    <row r="22" spans="1:24" x14ac:dyDescent="0.2">
       <c r="A22" s="3">
         <v>20</v>
       </c>
@@ -4169,54 +4374,368 @@
       <c r="W22" s="3"/>
       <c r="X22" s="3"/>
     </row>
-    <row r="24" spans="1:27" x14ac:dyDescent="0.2">
-      <c r="K24" s="9"/>
-      <c r="L24" s="9"/>
-    </row>
-    <row r="25" spans="1:27" x14ac:dyDescent="0.2">
-      <c r="K25" s="9"/>
-      <c r="L25" s="9"/>
-    </row>
-    <row r="27" spans="1:27" x14ac:dyDescent="0.2">
-      <c r="Z27" s="42"/>
-      <c r="AA27" t="s">
-        <v>91</v>
-      </c>
-    </row>
-    <row r="28" spans="1:27" x14ac:dyDescent="0.2">
-      <c r="Z28" s="26"/>
-      <c r="AA28" s="9" t="s">
-        <v>96</v>
-      </c>
-    </row>
-    <row r="29" spans="1:27" x14ac:dyDescent="0.2">
-      <c r="Z29" s="29"/>
-      <c r="AA29" s="9" t="s">
-        <v>103</v>
-      </c>
+    <row r="23" spans="1:24" x14ac:dyDescent="0.2">
+      <c r="A23" s="3">
+        <v>21</v>
+      </c>
+      <c r="B23" s="3"/>
+      <c r="C23" s="3"/>
+      <c r="D23" s="3"/>
+      <c r="E23" s="3"/>
+      <c r="F23" s="3"/>
+      <c r="G23" s="3"/>
+      <c r="H23" s="3" t="str">
+        <f t="shared" si="0"/>
+        <v/>
+      </c>
+      <c r="I23" s="3" t="str">
+        <f t="shared" si="1"/>
+        <v/>
+      </c>
+      <c r="J23" s="3"/>
+      <c r="K23" s="3"/>
+      <c r="L23" s="3"/>
+      <c r="M23" s="3"/>
+      <c r="N23" s="3"/>
+      <c r="O23" s="3"/>
+      <c r="P23" s="3"/>
+      <c r="Q23" s="3"/>
+      <c r="R23" s="3"/>
+      <c r="S23" s="3"/>
+      <c r="T23" s="3"/>
+      <c r="U23" s="3"/>
+      <c r="V23" s="3"/>
+      <c r="W23" s="3"/>
+      <c r="X23" s="3"/>
+    </row>
+    <row r="24" spans="1:24" x14ac:dyDescent="0.2">
+      <c r="A24" s="3">
+        <v>22</v>
+      </c>
+      <c r="B24" s="3"/>
+      <c r="C24" s="3"/>
+      <c r="D24" s="3"/>
+      <c r="E24" s="3"/>
+      <c r="F24" s="3"/>
+      <c r="G24" s="3"/>
+      <c r="H24" s="3" t="str">
+        <f t="shared" si="0"/>
+        <v/>
+      </c>
+      <c r="I24" s="3" t="str">
+        <f t="shared" si="1"/>
+        <v/>
+      </c>
+      <c r="J24" s="3"/>
+      <c r="K24" s="3"/>
+      <c r="L24" s="3"/>
+      <c r="M24" s="3"/>
+      <c r="N24" s="3"/>
+      <c r="O24" s="3"/>
+      <c r="P24" s="3"/>
+      <c r="Q24" s="3"/>
+      <c r="R24" s="3"/>
+      <c r="S24" s="3"/>
+      <c r="T24" s="3"/>
+      <c r="U24" s="3"/>
+      <c r="V24" s="3"/>
+      <c r="W24" s="3"/>
+      <c r="X24" s="3"/>
+    </row>
+    <row r="25" spans="1:24" x14ac:dyDescent="0.2">
+      <c r="A25" s="3">
+        <v>23</v>
+      </c>
+      <c r="B25" s="3"/>
+      <c r="C25" s="3"/>
+      <c r="D25" s="3"/>
+      <c r="E25" s="3"/>
+      <c r="F25" s="3"/>
+      <c r="G25" s="3"/>
+      <c r="H25" s="3" t="str">
+        <f t="shared" si="0"/>
+        <v/>
+      </c>
+      <c r="I25" s="3" t="str">
+        <f t="shared" si="1"/>
+        <v/>
+      </c>
+      <c r="J25" s="3"/>
+      <c r="K25" s="3"/>
+      <c r="L25" s="3"/>
+      <c r="M25" s="3"/>
+      <c r="N25" s="3"/>
+      <c r="O25" s="3"/>
+      <c r="P25" s="3"/>
+      <c r="Q25" s="3"/>
+      <c r="R25" s="3"/>
+      <c r="S25" s="3"/>
+      <c r="T25" s="3"/>
+      <c r="U25" s="3"/>
+      <c r="V25" s="3"/>
+      <c r="W25" s="3"/>
+      <c r="X25" s="3"/>
+    </row>
+    <row r="26" spans="1:24" x14ac:dyDescent="0.2">
+      <c r="A26" s="3">
+        <v>24</v>
+      </c>
+      <c r="B26" s="3"/>
+      <c r="C26" s="3"/>
+      <c r="D26" s="3"/>
+      <c r="E26" s="3"/>
+      <c r="F26" s="3"/>
+      <c r="G26" s="3"/>
+      <c r="H26" s="3" t="str">
+        <f t="shared" si="0"/>
+        <v/>
+      </c>
+      <c r="I26" s="3" t="str">
+        <f t="shared" si="1"/>
+        <v/>
+      </c>
+      <c r="J26" s="3"/>
+      <c r="K26" s="3"/>
+      <c r="L26" s="3"/>
+      <c r="M26" s="3"/>
+      <c r="N26" s="3"/>
+      <c r="O26" s="3"/>
+      <c r="P26" s="3"/>
+      <c r="Q26" s="3"/>
+      <c r="R26" s="3"/>
+      <c r="S26" s="3"/>
+      <c r="T26" s="3"/>
+      <c r="U26" s="3"/>
+      <c r="V26" s="3"/>
+      <c r="W26" s="3"/>
+      <c r="X26" s="3"/>
+    </row>
+    <row r="27" spans="1:24" x14ac:dyDescent="0.2">
+      <c r="A27" s="3">
+        <v>25</v>
+      </c>
+      <c r="B27" s="3"/>
+      <c r="C27" s="3"/>
+      <c r="D27" s="3"/>
+      <c r="E27" s="3"/>
+      <c r="F27" s="3"/>
+      <c r="G27" s="3"/>
+      <c r="H27" s="3" t="str">
+        <f t="shared" si="0"/>
+        <v/>
+      </c>
+      <c r="I27" s="3" t="str">
+        <f t="shared" si="1"/>
+        <v/>
+      </c>
+      <c r="J27" s="3"/>
+      <c r="K27" s="3"/>
+      <c r="L27" s="3"/>
+      <c r="M27" s="3"/>
+      <c r="N27" s="3"/>
+      <c r="O27" s="3"/>
+      <c r="P27" s="3"/>
+      <c r="Q27" s="3"/>
+      <c r="R27" s="3"/>
+      <c r="S27" s="3"/>
+      <c r="T27" s="3"/>
+      <c r="U27" s="3"/>
+      <c r="V27" s="3"/>
+      <c r="W27" s="3"/>
+      <c r="X27" s="3"/>
+    </row>
+    <row r="28" spans="1:24" x14ac:dyDescent="0.2">
+      <c r="A28" s="3">
+        <v>26</v>
+      </c>
+      <c r="B28" s="3"/>
+      <c r="C28" s="3"/>
+      <c r="D28" s="3"/>
+      <c r="E28" s="3"/>
+      <c r="F28" s="3"/>
+      <c r="G28" s="3"/>
+      <c r="H28" s="3" t="str">
+        <f t="shared" si="0"/>
+        <v/>
+      </c>
+      <c r="I28" s="3" t="str">
+        <f t="shared" si="1"/>
+        <v/>
+      </c>
+      <c r="J28" s="3"/>
+      <c r="K28" s="3"/>
+      <c r="L28" s="3"/>
+      <c r="M28" s="3"/>
+      <c r="N28" s="3"/>
+      <c r="O28" s="3"/>
+      <c r="P28" s="3"/>
+      <c r="Q28" s="3"/>
+      <c r="R28" s="3"/>
+      <c r="S28" s="3"/>
+      <c r="T28" s="3"/>
+      <c r="U28" s="3"/>
+      <c r="V28" s="3"/>
+      <c r="W28" s="3"/>
+      <c r="X28" s="3"/>
+    </row>
+    <row r="29" spans="1:24" x14ac:dyDescent="0.2">
+      <c r="A29" s="3">
+        <v>27</v>
+      </c>
+      <c r="B29" s="3"/>
+      <c r="C29" s="3"/>
+      <c r="D29" s="3"/>
+      <c r="E29" s="3"/>
+      <c r="F29" s="3"/>
+      <c r="G29" s="3"/>
+      <c r="H29" s="3" t="str">
+        <f t="shared" si="0"/>
+        <v/>
+      </c>
+      <c r="I29" s="3" t="str">
+        <f t="shared" si="1"/>
+        <v/>
+      </c>
+      <c r="J29" s="3"/>
+      <c r="K29" s="3"/>
+      <c r="L29" s="3"/>
+      <c r="M29" s="3"/>
+      <c r="N29" s="3"/>
+      <c r="O29" s="3"/>
+      <c r="P29" s="3"/>
+      <c r="Q29" s="3"/>
+      <c r="R29" s="3"/>
+      <c r="S29" s="3"/>
+      <c r="T29" s="3"/>
+      <c r="U29" s="3"/>
+      <c r="V29" s="3"/>
+      <c r="W29" s="3"/>
+      <c r="X29" s="3"/>
+    </row>
+    <row r="30" spans="1:24" x14ac:dyDescent="0.2">
+      <c r="A30" s="3">
+        <v>28</v>
+      </c>
+      <c r="B30" s="3"/>
+      <c r="C30" s="3"/>
+      <c r="D30" s="3"/>
+      <c r="E30" s="3"/>
+      <c r="F30" s="3"/>
+      <c r="G30" s="3"/>
+      <c r="H30" s="3" t="str">
+        <f t="shared" si="0"/>
+        <v/>
+      </c>
+      <c r="I30" s="3" t="str">
+        <f t="shared" si="1"/>
+        <v/>
+      </c>
+      <c r="J30" s="3"/>
+      <c r="K30" s="3"/>
+      <c r="L30" s="3"/>
+      <c r="M30" s="3"/>
+      <c r="N30" s="3"/>
+      <c r="O30" s="3"/>
+      <c r="P30" s="3"/>
+      <c r="Q30" s="3"/>
+      <c r="R30" s="3"/>
+      <c r="S30" s="3"/>
+      <c r="T30" s="3"/>
+      <c r="U30" s="3"/>
+      <c r="V30" s="3"/>
+      <c r="W30" s="3"/>
+      <c r="X30" s="3"/>
+    </row>
+    <row r="31" spans="1:24" x14ac:dyDescent="0.2">
+      <c r="A31" s="3">
+        <v>29</v>
+      </c>
+      <c r="B31" s="3"/>
+      <c r="C31" s="3"/>
+      <c r="D31" s="3"/>
+      <c r="E31" s="3"/>
+      <c r="F31" s="3"/>
+      <c r="G31" s="3"/>
+      <c r="H31" s="3" t="str">
+        <f t="shared" si="0"/>
+        <v/>
+      </c>
+      <c r="I31" s="3" t="str">
+        <f t="shared" si="1"/>
+        <v/>
+      </c>
+      <c r="J31" s="3"/>
+      <c r="K31" s="3"/>
+      <c r="L31" s="3"/>
+      <c r="M31" s="3"/>
+      <c r="N31" s="3"/>
+      <c r="O31" s="3"/>
+      <c r="P31" s="3"/>
+      <c r="Q31" s="3"/>
+      <c r="R31" s="3"/>
+      <c r="S31" s="3"/>
+      <c r="T31" s="3"/>
+      <c r="U31" s="3"/>
+      <c r="V31" s="3"/>
+      <c r="W31" s="3"/>
+      <c r="X31" s="3"/>
+    </row>
+    <row r="32" spans="1:24" x14ac:dyDescent="0.2">
+      <c r="A32" s="3">
+        <v>30</v>
+      </c>
+      <c r="B32" s="3"/>
+      <c r="C32" s="3"/>
+      <c r="D32" s="3"/>
+      <c r="E32" s="3"/>
+      <c r="F32" s="3"/>
+      <c r="G32" s="3"/>
+      <c r="H32" s="3" t="str">
+        <f t="shared" si="0"/>
+        <v/>
+      </c>
+      <c r="I32" s="3" t="str">
+        <f t="shared" si="1"/>
+        <v/>
+      </c>
+      <c r="J32" s="3"/>
+      <c r="K32" s="3"/>
+      <c r="L32" s="3"/>
+      <c r="M32" s="3"/>
+      <c r="N32" s="3"/>
+      <c r="O32" s="3"/>
+      <c r="P32" s="3"/>
+      <c r="Q32" s="3"/>
+      <c r="R32" s="3"/>
+      <c r="S32" s="3"/>
+      <c r="T32" s="3"/>
+      <c r="U32" s="3"/>
+      <c r="V32" s="3"/>
+      <c r="W32" s="3"/>
+      <c r="X32" s="3"/>
     </row>
   </sheetData>
-  <conditionalFormatting sqref="K3:L22">
+  <conditionalFormatting sqref="K3:L32">
     <cfRule type="expression" dxfId="1" priority="1">
       <formula>$U3="Yes"</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="V3:X22">
+  <conditionalFormatting sqref="V3:X32">
     <cfRule type="expression" dxfId="0" priority="4">
       <formula>$U3&lt;&gt;"Yes"</formula>
     </cfRule>
   </conditionalFormatting>
   <dataValidations count="4">
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="G3:G22" xr:uid="{00000000-0002-0000-0900-000000000000}">
-      <formula1>$AF$2:$AF$5</formula1>
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="G3:G32" xr:uid="{00000000-0002-0000-0900-000000000000}">
+      <formula1>$AH$2:$AH$5</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="H3:H22" xr:uid="{00000000-0002-0000-0900-000001000000}">
-      <formula1>$AG$2:$AG$3</formula1>
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="H3:H32" xr:uid="{00000000-0002-0000-0900-000001000000}">
+      <formula1>$AI$2:$AI$3</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="I3:I22" xr:uid="{00000000-0002-0000-0900-000002000000}">
-      <formula1>$AH$2:$AH$3</formula1>
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="I3:I32" xr:uid="{00000000-0002-0000-0900-000002000000}">
+      <formula1>$AJ$2:$AJ$3</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="U3:U22 X3:X22" xr:uid="{8FB27197-C456-2D4D-8100-E78D5059F972}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="U3:U32 X3:X32" xr:uid="{8FB27197-C456-2D4D-8100-E78D5059F972}">
       <formula1>"Yes,No"</formula1>
     </dataValidation>
   </dataValidations>
@@ -4226,6 +4745,549 @@
 </file>
 
 <file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{1C676759-96FB-7F49-B49A-BD8077ECE53B}">
+  <dimension ref="A2:O32"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
+  <cols>
+    <col min="1" max="1" width="4.83203125" style="1" customWidth="1"/>
+    <col min="2" max="12" width="10.83203125" style="1" customWidth="1"/>
+    <col min="13" max="13" width="4.33203125" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="2" spans="1:15" x14ac:dyDescent="0.2">
+      <c r="A2" s="12" t="s">
+        <v>193</v>
+      </c>
+      <c r="B2" s="12" t="s">
+        <v>241</v>
+      </c>
+      <c r="C2" s="12" t="s">
+        <v>242</v>
+      </c>
+      <c r="D2" s="12" t="s">
+        <v>243</v>
+      </c>
+      <c r="E2" s="12" t="s">
+        <v>244</v>
+      </c>
+      <c r="F2" s="12" t="s">
+        <v>245</v>
+      </c>
+      <c r="G2" s="28" t="s">
+        <v>114</v>
+      </c>
+      <c r="H2" s="28" t="s">
+        <v>323</v>
+      </c>
+      <c r="I2" s="28" t="s">
+        <v>120</v>
+      </c>
+      <c r="J2" s="28" t="s">
+        <v>320</v>
+      </c>
+      <c r="K2" s="28" t="s">
+        <v>321</v>
+      </c>
+      <c r="L2" s="28" t="s">
+        <v>322</v>
+      </c>
+      <c r="N2" s="29"/>
+      <c r="O2" s="9" t="s">
+        <v>103</v>
+      </c>
+    </row>
+    <row r="3" spans="1:15" x14ac:dyDescent="0.2">
+      <c r="A3" s="3">
+        <v>1</v>
+      </c>
+      <c r="B3" s="3"/>
+      <c r="C3" s="3"/>
+      <c r="D3" s="3"/>
+      <c r="E3" s="3"/>
+      <c r="F3" s="3"/>
+      <c r="G3" s="3"/>
+      <c r="H3" s="3"/>
+      <c r="I3" s="3"/>
+      <c r="J3" s="3"/>
+      <c r="K3" s="3"/>
+      <c r="L3" s="3"/>
+    </row>
+    <row r="4" spans="1:15" x14ac:dyDescent="0.2">
+      <c r="A4" s="3">
+        <v>2</v>
+      </c>
+      <c r="B4" s="3"/>
+      <c r="C4" s="3"/>
+      <c r="D4" s="3"/>
+      <c r="E4" s="3"/>
+      <c r="F4" s="3"/>
+      <c r="G4" s="3"/>
+      <c r="H4" s="3"/>
+      <c r="I4" s="3"/>
+      <c r="J4" s="3"/>
+      <c r="K4" s="3"/>
+      <c r="L4" s="3"/>
+    </row>
+    <row r="5" spans="1:15" x14ac:dyDescent="0.2">
+      <c r="A5" s="3">
+        <v>3</v>
+      </c>
+      <c r="B5" s="3"/>
+      <c r="C5" s="3"/>
+      <c r="D5" s="3"/>
+      <c r="E5" s="3"/>
+      <c r="F5" s="3"/>
+      <c r="G5" s="3"/>
+      <c r="H5" s="3"/>
+      <c r="I5" s="3"/>
+      <c r="J5" s="3"/>
+      <c r="K5" s="3"/>
+      <c r="L5" s="3"/>
+    </row>
+    <row r="6" spans="1:15" x14ac:dyDescent="0.2">
+      <c r="A6" s="3">
+        <v>4</v>
+      </c>
+      <c r="B6" s="3"/>
+      <c r="C6" s="3"/>
+      <c r="D6" s="3"/>
+      <c r="E6" s="3"/>
+      <c r="F6" s="3"/>
+      <c r="G6" s="3"/>
+      <c r="H6" s="3"/>
+      <c r="I6" s="3"/>
+      <c r="J6" s="3"/>
+      <c r="K6" s="3"/>
+      <c r="L6" s="3"/>
+    </row>
+    <row r="7" spans="1:15" x14ac:dyDescent="0.2">
+      <c r="A7" s="3">
+        <v>5</v>
+      </c>
+      <c r="B7" s="3"/>
+      <c r="C7" s="3"/>
+      <c r="D7" s="3"/>
+      <c r="E7" s="3"/>
+      <c r="F7" s="3"/>
+      <c r="G7" s="3"/>
+      <c r="H7" s="3"/>
+      <c r="I7" s="3"/>
+      <c r="J7" s="3"/>
+      <c r="K7" s="3"/>
+      <c r="L7" s="3"/>
+    </row>
+    <row r="8" spans="1:15" x14ac:dyDescent="0.2">
+      <c r="A8" s="3">
+        <v>6</v>
+      </c>
+      <c r="B8" s="3"/>
+      <c r="C8" s="3"/>
+      <c r="D8" s="3"/>
+      <c r="E8" s="3"/>
+      <c r="F8" s="3"/>
+      <c r="G8" s="3"/>
+      <c r="H8" s="3"/>
+      <c r="I8" s="3"/>
+      <c r="J8" s="3"/>
+      <c r="K8" s="3"/>
+      <c r="L8" s="3"/>
+    </row>
+    <row r="9" spans="1:15" x14ac:dyDescent="0.2">
+      <c r="A9" s="3">
+        <v>7</v>
+      </c>
+      <c r="B9" s="3"/>
+      <c r="C9" s="3"/>
+      <c r="D9" s="3"/>
+      <c r="E9" s="3"/>
+      <c r="F9" s="3"/>
+      <c r="G9" s="3"/>
+      <c r="H9" s="3"/>
+      <c r="I9" s="3"/>
+      <c r="J9" s="3"/>
+      <c r="K9" s="3"/>
+      <c r="L9" s="3"/>
+    </row>
+    <row r="10" spans="1:15" x14ac:dyDescent="0.2">
+      <c r="A10" s="3">
+        <v>8</v>
+      </c>
+      <c r="B10" s="3"/>
+      <c r="C10" s="3"/>
+      <c r="D10" s="3"/>
+      <c r="E10" s="3"/>
+      <c r="F10" s="3"/>
+      <c r="G10" s="3"/>
+      <c r="H10" s="3"/>
+      <c r="I10" s="3"/>
+      <c r="J10" s="3"/>
+      <c r="K10" s="3"/>
+      <c r="L10" s="3"/>
+    </row>
+    <row r="11" spans="1:15" x14ac:dyDescent="0.2">
+      <c r="A11" s="3">
+        <v>9</v>
+      </c>
+      <c r="B11" s="3"/>
+      <c r="C11" s="3"/>
+      <c r="D11" s="3"/>
+      <c r="E11" s="3"/>
+      <c r="F11" s="3"/>
+      <c r="G11" s="3"/>
+      <c r="H11" s="3"/>
+      <c r="I11" s="3"/>
+      <c r="J11" s="3"/>
+      <c r="K11" s="3"/>
+      <c r="L11" s="3"/>
+    </row>
+    <row r="12" spans="1:15" x14ac:dyDescent="0.2">
+      <c r="A12" s="3">
+        <v>10</v>
+      </c>
+      <c r="B12" s="3"/>
+      <c r="C12" s="3"/>
+      <c r="D12" s="3"/>
+      <c r="E12" s="3"/>
+      <c r="F12" s="3"/>
+      <c r="G12" s="3"/>
+      <c r="H12" s="3"/>
+      <c r="I12" s="3"/>
+      <c r="J12" s="3"/>
+      <c r="K12" s="3"/>
+      <c r="L12" s="3"/>
+    </row>
+    <row r="13" spans="1:15" x14ac:dyDescent="0.2">
+      <c r="A13" s="3">
+        <v>11</v>
+      </c>
+      <c r="B13" s="3"/>
+      <c r="C13" s="3"/>
+      <c r="D13" s="3"/>
+      <c r="E13" s="3"/>
+      <c r="F13" s="3"/>
+      <c r="G13" s="3"/>
+      <c r="H13" s="3"/>
+      <c r="I13" s="3"/>
+      <c r="J13" s="3"/>
+      <c r="K13" s="3"/>
+      <c r="L13" s="3"/>
+    </row>
+    <row r="14" spans="1:15" x14ac:dyDescent="0.2">
+      <c r="A14" s="3">
+        <v>12</v>
+      </c>
+      <c r="B14" s="3"/>
+      <c r="C14" s="3"/>
+      <c r="D14" s="3"/>
+      <c r="E14" s="3"/>
+      <c r="F14" s="3"/>
+      <c r="G14" s="3"/>
+      <c r="H14" s="3"/>
+      <c r="I14" s="3"/>
+      <c r="J14" s="3"/>
+      <c r="K14" s="3"/>
+      <c r="L14" s="3"/>
+    </row>
+    <row r="15" spans="1:15" x14ac:dyDescent="0.2">
+      <c r="A15" s="3">
+        <v>13</v>
+      </c>
+      <c r="B15" s="3"/>
+      <c r="C15" s="3"/>
+      <c r="D15" s="3"/>
+      <c r="E15" s="3"/>
+      <c r="F15" s="3"/>
+      <c r="G15" s="3"/>
+      <c r="H15" s="3"/>
+      <c r="I15" s="3"/>
+      <c r="J15" s="3"/>
+      <c r="K15" s="3"/>
+      <c r="L15" s="3"/>
+    </row>
+    <row r="16" spans="1:15" x14ac:dyDescent="0.2">
+      <c r="A16" s="3">
+        <v>14</v>
+      </c>
+      <c r="B16" s="3"/>
+      <c r="C16" s="3"/>
+      <c r="D16" s="3"/>
+      <c r="E16" s="3"/>
+      <c r="F16" s="3"/>
+      <c r="G16" s="3"/>
+      <c r="H16" s="3"/>
+      <c r="I16" s="3"/>
+      <c r="J16" s="3"/>
+      <c r="K16" s="3"/>
+      <c r="L16" s="3"/>
+    </row>
+    <row r="17" spans="1:12" x14ac:dyDescent="0.2">
+      <c r="A17" s="3">
+        <v>15</v>
+      </c>
+      <c r="B17" s="3"/>
+      <c r="C17" s="3"/>
+      <c r="D17" s="3"/>
+      <c r="E17" s="3"/>
+      <c r="F17" s="3"/>
+      <c r="G17" s="3"/>
+      <c r="H17" s="3"/>
+      <c r="I17" s="3"/>
+      <c r="J17" s="3"/>
+      <c r="K17" s="3"/>
+      <c r="L17" s="3"/>
+    </row>
+    <row r="18" spans="1:12" x14ac:dyDescent="0.2">
+      <c r="A18" s="3">
+        <v>16</v>
+      </c>
+      <c r="B18" s="3"/>
+      <c r="C18" s="3"/>
+      <c r="D18" s="3"/>
+      <c r="E18" s="3"/>
+      <c r="F18" s="3"/>
+      <c r="G18" s="3"/>
+      <c r="H18" s="3"/>
+      <c r="I18" s="3"/>
+      <c r="J18" s="3"/>
+      <c r="K18" s="3"/>
+      <c r="L18" s="3"/>
+    </row>
+    <row r="19" spans="1:12" x14ac:dyDescent="0.2">
+      <c r="A19" s="3">
+        <v>17</v>
+      </c>
+      <c r="B19" s="3"/>
+      <c r="C19" s="3"/>
+      <c r="D19" s="3"/>
+      <c r="E19" s="3"/>
+      <c r="F19" s="3"/>
+      <c r="G19" s="3"/>
+      <c r="H19" s="3"/>
+      <c r="I19" s="3"/>
+      <c r="J19" s="3"/>
+      <c r="K19" s="3"/>
+      <c r="L19" s="3"/>
+    </row>
+    <row r="20" spans="1:12" x14ac:dyDescent="0.2">
+      <c r="A20" s="3">
+        <v>18</v>
+      </c>
+      <c r="B20" s="3"/>
+      <c r="C20" s="3"/>
+      <c r="D20" s="3"/>
+      <c r="E20" s="3"/>
+      <c r="F20" s="3"/>
+      <c r="G20" s="3"/>
+      <c r="H20" s="3"/>
+      <c r="I20" s="3"/>
+      <c r="J20" s="3"/>
+      <c r="K20" s="3"/>
+      <c r="L20" s="3"/>
+    </row>
+    <row r="21" spans="1:12" x14ac:dyDescent="0.2">
+      <c r="A21" s="3">
+        <v>19</v>
+      </c>
+      <c r="B21" s="3"/>
+      <c r="C21" s="3"/>
+      <c r="D21" s="3"/>
+      <c r="E21" s="3"/>
+      <c r="F21" s="3"/>
+      <c r="G21" s="3"/>
+      <c r="H21" s="3"/>
+      <c r="I21" s="3"/>
+      <c r="J21" s="3"/>
+      <c r="K21" s="3"/>
+      <c r="L21" s="3"/>
+    </row>
+    <row r="22" spans="1:12" x14ac:dyDescent="0.2">
+      <c r="A22" s="3">
+        <v>20</v>
+      </c>
+      <c r="B22" s="3"/>
+      <c r="C22" s="3"/>
+      <c r="D22" s="3"/>
+      <c r="E22" s="3"/>
+      <c r="F22" s="3"/>
+      <c r="G22" s="3"/>
+      <c r="H22" s="3"/>
+      <c r="I22" s="3"/>
+      <c r="J22" s="3"/>
+      <c r="K22" s="3"/>
+      <c r="L22" s="3"/>
+    </row>
+    <row r="23" spans="1:12" x14ac:dyDescent="0.2">
+      <c r="A23" s="3">
+        <v>21</v>
+      </c>
+      <c r="B23" s="3"/>
+      <c r="C23" s="3"/>
+      <c r="D23" s="3"/>
+      <c r="E23" s="3"/>
+      <c r="F23" s="3"/>
+      <c r="G23" s="3"/>
+      <c r="H23" s="3"/>
+      <c r="I23" s="3"/>
+      <c r="J23" s="3"/>
+      <c r="K23" s="3"/>
+      <c r="L23" s="3"/>
+    </row>
+    <row r="24" spans="1:12" x14ac:dyDescent="0.2">
+      <c r="A24" s="3">
+        <v>22</v>
+      </c>
+      <c r="B24" s="3"/>
+      <c r="C24" s="3"/>
+      <c r="D24" s="3"/>
+      <c r="E24" s="3"/>
+      <c r="F24" s="3"/>
+      <c r="G24" s="3"/>
+      <c r="H24" s="3"/>
+      <c r="I24" s="3"/>
+      <c r="J24" s="3"/>
+      <c r="K24" s="3"/>
+      <c r="L24" s="3"/>
+    </row>
+    <row r="25" spans="1:12" x14ac:dyDescent="0.2">
+      <c r="A25" s="3">
+        <v>23</v>
+      </c>
+      <c r="B25" s="3"/>
+      <c r="C25" s="3"/>
+      <c r="D25" s="3"/>
+      <c r="E25" s="3"/>
+      <c r="F25" s="3"/>
+      <c r="G25" s="3"/>
+      <c r="H25" s="3"/>
+      <c r="I25" s="3"/>
+      <c r="J25" s="3"/>
+      <c r="K25" s="3"/>
+      <c r="L25" s="3"/>
+    </row>
+    <row r="26" spans="1:12" x14ac:dyDescent="0.2">
+      <c r="A26" s="3">
+        <v>24</v>
+      </c>
+      <c r="B26" s="3"/>
+      <c r="C26" s="3"/>
+      <c r="D26" s="3"/>
+      <c r="E26" s="3"/>
+      <c r="F26" s="3"/>
+      <c r="G26" s="3"/>
+      <c r="H26" s="3"/>
+      <c r="I26" s="3"/>
+      <c r="J26" s="3"/>
+      <c r="K26" s="3"/>
+      <c r="L26" s="3"/>
+    </row>
+    <row r="27" spans="1:12" x14ac:dyDescent="0.2">
+      <c r="A27" s="3">
+        <v>25</v>
+      </c>
+      <c r="B27" s="3"/>
+      <c r="C27" s="3"/>
+      <c r="D27" s="3"/>
+      <c r="E27" s="3"/>
+      <c r="F27" s="3"/>
+      <c r="G27" s="3"/>
+      <c r="H27" s="3"/>
+      <c r="I27" s="3"/>
+      <c r="J27" s="3"/>
+      <c r="K27" s="3"/>
+      <c r="L27" s="3"/>
+    </row>
+    <row r="28" spans="1:12" x14ac:dyDescent="0.2">
+      <c r="A28" s="3">
+        <v>26</v>
+      </c>
+      <c r="B28" s="3"/>
+      <c r="C28" s="3"/>
+      <c r="D28" s="3"/>
+      <c r="E28" s="3"/>
+      <c r="F28" s="3"/>
+      <c r="G28" s="3"/>
+      <c r="H28" s="3"/>
+      <c r="I28" s="3"/>
+      <c r="J28" s="3"/>
+      <c r="K28" s="3"/>
+      <c r="L28" s="3"/>
+    </row>
+    <row r="29" spans="1:12" x14ac:dyDescent="0.2">
+      <c r="A29" s="3">
+        <v>27</v>
+      </c>
+      <c r="B29" s="3"/>
+      <c r="C29" s="3"/>
+      <c r="D29" s="3"/>
+      <c r="E29" s="3"/>
+      <c r="F29" s="3"/>
+      <c r="G29" s="3"/>
+      <c r="H29" s="3"/>
+      <c r="I29" s="3"/>
+      <c r="J29" s="3"/>
+      <c r="K29" s="3"/>
+      <c r="L29" s="3"/>
+    </row>
+    <row r="30" spans="1:12" x14ac:dyDescent="0.2">
+      <c r="A30" s="3">
+        <v>28</v>
+      </c>
+      <c r="B30" s="3"/>
+      <c r="C30" s="3"/>
+      <c r="D30" s="3"/>
+      <c r="E30" s="3"/>
+      <c r="F30" s="3"/>
+      <c r="G30" s="3"/>
+      <c r="H30" s="3"/>
+      <c r="I30" s="3"/>
+      <c r="J30" s="3"/>
+      <c r="K30" s="3"/>
+      <c r="L30" s="3"/>
+    </row>
+    <row r="31" spans="1:12" x14ac:dyDescent="0.2">
+      <c r="A31" s="3">
+        <v>29</v>
+      </c>
+      <c r="B31" s="3"/>
+      <c r="C31" s="3"/>
+      <c r="D31" s="3"/>
+      <c r="E31" s="3"/>
+      <c r="F31" s="3"/>
+      <c r="G31" s="3"/>
+      <c r="H31" s="3"/>
+      <c r="I31" s="3"/>
+      <c r="J31" s="3"/>
+      <c r="K31" s="3"/>
+      <c r="L31" s="3"/>
+    </row>
+    <row r="32" spans="1:12" x14ac:dyDescent="0.2">
+      <c r="A32" s="3">
+        <v>30</v>
+      </c>
+      <c r="B32" s="3"/>
+      <c r="C32" s="3"/>
+      <c r="D32" s="3"/>
+      <c r="E32" s="3"/>
+      <c r="F32" s="3"/>
+      <c r="G32" s="3"/>
+      <c r="H32" s="3"/>
+      <c r="I32" s="3"/>
+      <c r="J32" s="3"/>
+      <c r="K32" s="3"/>
+      <c r="L32" s="3"/>
+    </row>
+  </sheetData>
+  <dataValidations count="1">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="L3:L32" xr:uid="{D1121F3C-F660-0E46-8AEB-8C1F95C55489}">
+      <formula1>"Yes,No"</formula1>
+    </dataValidation>
+  </dataValidations>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <drawing r:id="rId1"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0A00-000000000000}">
   <dimension ref="A2:AA17"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
@@ -4555,7 +5617,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet13.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0B00-000000000000}">
   <dimension ref="A2:F22"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
@@ -4790,7 +5852,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet13.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet14.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0C00-000000000000}">
   <dimension ref="B2:U24"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
@@ -5208,7 +6270,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet14.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet15.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0D00-000000000000}">
   <dimension ref="B2:U24"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
@@ -5622,7 +6684,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet15.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet16.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0E00-000000000000}">
   <dimension ref="B2:J100"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>

</xml_diff>

<commit_message>
template v27: the joints sheet gains c_res, phi_res and dil, peak beside residual; fifty rows
Owner's edit. Column order c, c_res, phi, phi_res, dil, t_cut, kn, ks, Jred;
the Yes/No list follows Jred to column O; rows 3-52; help box states the two
blank rules that differ from the mat sheet (t_cut blank = 0; residuals blank =
peak). Loader, editor and solver pick the three columns up in the phase 2
verification round. Packaged copy synced byte-identical.

Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01XjjT2aBxw8gY7EFdpoUcpj
</commit_message>
<xml_diff>
--- a/docs/inputs/input_template.xlsx
+++ b/docs/inputs/input_template.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/njones/python_projects/xslope/.claude/worktrees/joints-r1/docs/inputs/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{42723C2E-F56A-D348-AC02-78080B1F6523}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{518FA263-91FA-F44E-9CA5-998A9947A78D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="9960" yWindow="2320" windowWidth="30380" windowHeight="22500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="4280" yWindow="2000" windowWidth="40460" windowHeight="22500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="main" sheetId="1" r:id="rId1"/>
@@ -60,7 +60,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="621" uniqueCount="326">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="624" uniqueCount="329">
   <si>
     <t>XSLOPE Input Template</t>
   </si>
@@ -1159,6 +1159,15 @@
   </si>
   <si>
     <t>Slip joints (interfaces with no reinforcement)</t>
+  </si>
+  <si>
+    <t>c_res</t>
+  </si>
+  <si>
+    <t>phi_res</t>
+  </si>
+  <si>
+    <t>dil</t>
   </si>
 </sst>
 </file>
@@ -1666,7 +1675,7 @@
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="38">
+  <dxfs count="37">
     <dxf>
       <fill>
         <patternFill>
@@ -1699,13 +1708,6 @@
       <fill>
         <patternFill>
           <bgColor theme="1" tint="0.499984740745262"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor theme="0" tint="-0.499984740745262"/>
         </patternFill>
       </fill>
     </dxf>
@@ -2227,16 +2229,16 @@
 <xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
   <xdr:twoCellAnchor>
     <xdr:from>
-      <xdr:col>12</xdr:col>
+      <xdr:col>15</xdr:col>
       <xdr:colOff>308428</xdr:colOff>
       <xdr:row>2</xdr:row>
-      <xdr:rowOff>172358</xdr:rowOff>
+      <xdr:rowOff>172357</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>17</xdr:col>
+      <xdr:col>20</xdr:col>
       <xdr:colOff>381000</xdr:colOff>
-      <xdr:row>10</xdr:row>
-      <xdr:rowOff>81643</xdr:rowOff>
+      <xdr:row>12</xdr:row>
+      <xdr:rowOff>172356</xdr:rowOff>
     </xdr:to>
     <xdr:sp macro="" textlink="">
       <xdr:nvSpPr>
@@ -2251,8 +2253,8 @@
       </xdr:nvSpPr>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="9760857" y="571501"/>
-          <a:ext cx="3701143" cy="1505856"/>
+          <a:off x="12237357" y="571500"/>
+          <a:ext cx="3701143" cy="1995713"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -2334,6 +2336,33 @@
           </a:r>
         </a:p>
         <a:p>
+          <a:pPr marL="0" marR="0" lvl="0" indent="0" defTabSz="914400" eaLnBrk="1" fontAlgn="auto" latinLnBrk="0" hangingPunct="1">
+            <a:lnSpc>
+              <a:spcPct val="100000"/>
+            </a:lnSpc>
+            <a:spcBef>
+              <a:spcPts val="0"/>
+            </a:spcBef>
+            <a:spcAft>
+              <a:spcPts val="0"/>
+            </a:spcAft>
+            <a:buClrTx/>
+            <a:buSzTx/>
+            <a:buFontTx/>
+            <a:buNone/>
+            <a:tabLst/>
+            <a:defRPr/>
+          </a:pPr>
+          <a:r>
+            <a:rPr lang="en-US" sz="1100" b="1"/>
+            <a:t>c_res</a:t>
+          </a:r>
+          <a:r>
+            <a:rPr lang="en-US" sz="1100" b="0" baseline="0"/>
+            <a:t> = residual joint cohesion (blank = same as c)</a:t>
+          </a:r>
+        </a:p>
+        <a:p>
           <a:r>
             <a:rPr lang="en-US" sz="1100" b="1" baseline="0"/>
             <a:t>phi</a:t>
@@ -2344,13 +2373,67 @@
           </a:r>
         </a:p>
         <a:p>
+          <a:pPr marL="0" marR="0" lvl="0" indent="0" defTabSz="914400" eaLnBrk="1" fontAlgn="auto" latinLnBrk="0" hangingPunct="1">
+            <a:lnSpc>
+              <a:spcPct val="100000"/>
+            </a:lnSpc>
+            <a:spcBef>
+              <a:spcPts val="0"/>
+            </a:spcBef>
+            <a:spcAft>
+              <a:spcPts val="0"/>
+            </a:spcAft>
+            <a:buClrTx/>
+            <a:buSzTx/>
+            <a:buFontTx/>
+            <a:buNone/>
+            <a:tabLst/>
+            <a:defRPr/>
+          </a:pPr>
+          <a:r>
+            <a:rPr lang="en-US" sz="1100" b="1" baseline="0"/>
+            <a:t>phi_res</a:t>
+          </a:r>
+          <a:r>
+            <a:rPr lang="en-US" sz="1100" b="0" baseline="0"/>
+            <a:t> = residual joint friction angle (blank = same as phi)</a:t>
+          </a:r>
+        </a:p>
+        <a:p>
+          <a:pPr marL="0" marR="0" lvl="0" indent="0" defTabSz="914400" eaLnBrk="1" fontAlgn="auto" latinLnBrk="0" hangingPunct="1">
+            <a:lnSpc>
+              <a:spcPct val="100000"/>
+            </a:lnSpc>
+            <a:spcBef>
+              <a:spcPts val="0"/>
+            </a:spcBef>
+            <a:spcAft>
+              <a:spcPts val="0"/>
+            </a:spcAft>
+            <a:buClrTx/>
+            <a:buSzTx/>
+            <a:buFontTx/>
+            <a:buNone/>
+            <a:tabLst/>
+            <a:defRPr/>
+          </a:pPr>
+          <a:r>
+            <a:rPr lang="en-US" sz="1100" b="1" baseline="0"/>
+            <a:t>dil</a:t>
+          </a:r>
+          <a:r>
+            <a:rPr lang="en-US" sz="1100" b="0" baseline="0"/>
+            <a:t> = joint dilation angle, degrees (blank = 0)</a:t>
+          </a:r>
+        </a:p>
+        <a:p>
           <a:r>
             <a:rPr lang="en-US" sz="1100" b="1" baseline="0"/>
             <a:t>t_cut</a:t>
           </a:r>
           <a:r>
             <a:rPr lang="en-US" sz="1100" b="0" baseline="0"/>
-            <a:t> = tension cutoff</a:t>
+            <a:t> = tension cutoff (blank = 0)</a:t>
           </a:r>
         </a:p>
         <a:p>
@@ -4746,15 +4829,15 @@
 
 <file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{1C676759-96FB-7F49-B49A-BD8077ECE53B}">
-  <dimension ref="A2:O32"/>
+  <dimension ref="A2:R52"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="4.83203125" style="1" customWidth="1"/>
-    <col min="2" max="12" width="10.83203125" style="1" customWidth="1"/>
-    <col min="13" max="13" width="4.33203125" customWidth="1"/>
+    <col min="2" max="15" width="10.83203125" style="1" customWidth="1"/>
+    <col min="16" max="16" width="4.33203125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="2" spans="1:15" x14ac:dyDescent="0.2">
+    <row r="2" spans="1:18" x14ac:dyDescent="0.2">
       <c r="A2" s="12" t="s">
         <v>193</v>
       </c>
@@ -4777,26 +4860,35 @@
         <v>114</v>
       </c>
       <c r="H2" s="28" t="s">
+        <v>326</v>
+      </c>
+      <c r="I2" s="28" t="s">
         <v>323</v>
       </c>
-      <c r="I2" s="28" t="s">
+      <c r="J2" s="28" t="s">
+        <v>327</v>
+      </c>
+      <c r="K2" s="28" t="s">
+        <v>328</v>
+      </c>
+      <c r="L2" s="28" t="s">
         <v>120</v>
       </c>
-      <c r="J2" s="28" t="s">
+      <c r="M2" s="28" t="s">
         <v>320</v>
       </c>
-      <c r="K2" s="28" t="s">
+      <c r="N2" s="28" t="s">
         <v>321</v>
       </c>
-      <c r="L2" s="28" t="s">
+      <c r="O2" s="28" t="s">
         <v>322</v>
       </c>
-      <c r="N2" s="29"/>
-      <c r="O2" s="9" t="s">
+      <c r="Q2" s="29"/>
+      <c r="R2" s="9" t="s">
         <v>103</v>
       </c>
     </row>
-    <row r="3" spans="1:15" x14ac:dyDescent="0.2">
+    <row r="3" spans="1:18" x14ac:dyDescent="0.2">
       <c r="A3" s="3">
         <v>1</v>
       </c>
@@ -4811,8 +4903,11 @@
       <c r="J3" s="3"/>
       <c r="K3" s="3"/>
       <c r="L3" s="3"/>
-    </row>
-    <row r="4" spans="1:15" x14ac:dyDescent="0.2">
+      <c r="M3" s="3"/>
+      <c r="N3" s="3"/>
+      <c r="O3" s="3"/>
+    </row>
+    <row r="4" spans="1:18" x14ac:dyDescent="0.2">
       <c r="A4" s="3">
         <v>2</v>
       </c>
@@ -4827,8 +4922,11 @@
       <c r="J4" s="3"/>
       <c r="K4" s="3"/>
       <c r="L4" s="3"/>
-    </row>
-    <row r="5" spans="1:15" x14ac:dyDescent="0.2">
+      <c r="M4" s="3"/>
+      <c r="N4" s="3"/>
+      <c r="O4" s="3"/>
+    </row>
+    <row r="5" spans="1:18" x14ac:dyDescent="0.2">
       <c r="A5" s="3">
         <v>3</v>
       </c>
@@ -4843,8 +4941,11 @@
       <c r="J5" s="3"/>
       <c r="K5" s="3"/>
       <c r="L5" s="3"/>
-    </row>
-    <row r="6" spans="1:15" x14ac:dyDescent="0.2">
+      <c r="M5" s="3"/>
+      <c r="N5" s="3"/>
+      <c r="O5" s="3"/>
+    </row>
+    <row r="6" spans="1:18" x14ac:dyDescent="0.2">
       <c r="A6" s="3">
         <v>4</v>
       </c>
@@ -4859,8 +4960,11 @@
       <c r="J6" s="3"/>
       <c r="K6" s="3"/>
       <c r="L6" s="3"/>
-    </row>
-    <row r="7" spans="1:15" x14ac:dyDescent="0.2">
+      <c r="M6" s="3"/>
+      <c r="N6" s="3"/>
+      <c r="O6" s="3"/>
+    </row>
+    <row r="7" spans="1:18" x14ac:dyDescent="0.2">
       <c r="A7" s="3">
         <v>5</v>
       </c>
@@ -4875,8 +4979,11 @@
       <c r="J7" s="3"/>
       <c r="K7" s="3"/>
       <c r="L7" s="3"/>
-    </row>
-    <row r="8" spans="1:15" x14ac:dyDescent="0.2">
+      <c r="M7" s="3"/>
+      <c r="N7" s="3"/>
+      <c r="O7" s="3"/>
+    </row>
+    <row r="8" spans="1:18" x14ac:dyDescent="0.2">
       <c r="A8" s="3">
         <v>6</v>
       </c>
@@ -4891,8 +4998,11 @@
       <c r="J8" s="3"/>
       <c r="K8" s="3"/>
       <c r="L8" s="3"/>
-    </row>
-    <row r="9" spans="1:15" x14ac:dyDescent="0.2">
+      <c r="M8" s="3"/>
+      <c r="N8" s="3"/>
+      <c r="O8" s="3"/>
+    </row>
+    <row r="9" spans="1:18" x14ac:dyDescent="0.2">
       <c r="A9" s="3">
         <v>7</v>
       </c>
@@ -4907,8 +5017,11 @@
       <c r="J9" s="3"/>
       <c r="K9" s="3"/>
       <c r="L9" s="3"/>
-    </row>
-    <row r="10" spans="1:15" x14ac:dyDescent="0.2">
+      <c r="M9" s="3"/>
+      <c r="N9" s="3"/>
+      <c r="O9" s="3"/>
+    </row>
+    <row r="10" spans="1:18" x14ac:dyDescent="0.2">
       <c r="A10" s="3">
         <v>8</v>
       </c>
@@ -4923,8 +5036,11 @@
       <c r="J10" s="3"/>
       <c r="K10" s="3"/>
       <c r="L10" s="3"/>
-    </row>
-    <row r="11" spans="1:15" x14ac:dyDescent="0.2">
+      <c r="M10" s="3"/>
+      <c r="N10" s="3"/>
+      <c r="O10" s="3"/>
+    </row>
+    <row r="11" spans="1:18" x14ac:dyDescent="0.2">
       <c r="A11" s="3">
         <v>9</v>
       </c>
@@ -4939,8 +5055,11 @@
       <c r="J11" s="3"/>
       <c r="K11" s="3"/>
       <c r="L11" s="3"/>
-    </row>
-    <row r="12" spans="1:15" x14ac:dyDescent="0.2">
+      <c r="M11" s="3"/>
+      <c r="N11" s="3"/>
+      <c r="O11" s="3"/>
+    </row>
+    <row r="12" spans="1:18" x14ac:dyDescent="0.2">
       <c r="A12" s="3">
         <v>10</v>
       </c>
@@ -4955,8 +5074,11 @@
       <c r="J12" s="3"/>
       <c r="K12" s="3"/>
       <c r="L12" s="3"/>
-    </row>
-    <row r="13" spans="1:15" x14ac:dyDescent="0.2">
+      <c r="M12" s="3"/>
+      <c r="N12" s="3"/>
+      <c r="O12" s="3"/>
+    </row>
+    <row r="13" spans="1:18" x14ac:dyDescent="0.2">
       <c r="A13" s="3">
         <v>11</v>
       </c>
@@ -4971,8 +5093,11 @@
       <c r="J13" s="3"/>
       <c r="K13" s="3"/>
       <c r="L13" s="3"/>
-    </row>
-    <row r="14" spans="1:15" x14ac:dyDescent="0.2">
+      <c r="M13" s="3"/>
+      <c r="N13" s="3"/>
+      <c r="O13" s="3"/>
+    </row>
+    <row r="14" spans="1:18" x14ac:dyDescent="0.2">
       <c r="A14" s="3">
         <v>12</v>
       </c>
@@ -4987,8 +5112,11 @@
       <c r="J14" s="3"/>
       <c r="K14" s="3"/>
       <c r="L14" s="3"/>
-    </row>
-    <row r="15" spans="1:15" x14ac:dyDescent="0.2">
+      <c r="M14" s="3"/>
+      <c r="N14" s="3"/>
+      <c r="O14" s="3"/>
+    </row>
+    <row r="15" spans="1:18" x14ac:dyDescent="0.2">
       <c r="A15" s="3">
         <v>13</v>
       </c>
@@ -5003,8 +5131,11 @@
       <c r="J15" s="3"/>
       <c r="K15" s="3"/>
       <c r="L15" s="3"/>
-    </row>
-    <row r="16" spans="1:15" x14ac:dyDescent="0.2">
+      <c r="M15" s="3"/>
+      <c r="N15" s="3"/>
+      <c r="O15" s="3"/>
+    </row>
+    <row r="16" spans="1:18" x14ac:dyDescent="0.2">
       <c r="A16" s="3">
         <v>14</v>
       </c>
@@ -5019,8 +5150,11 @@
       <c r="J16" s="3"/>
       <c r="K16" s="3"/>
       <c r="L16" s="3"/>
-    </row>
-    <row r="17" spans="1:12" x14ac:dyDescent="0.2">
+      <c r="M16" s="3"/>
+      <c r="N16" s="3"/>
+      <c r="O16" s="3"/>
+    </row>
+    <row r="17" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A17" s="3">
         <v>15</v>
       </c>
@@ -5035,8 +5169,11 @@
       <c r="J17" s="3"/>
       <c r="K17" s="3"/>
       <c r="L17" s="3"/>
-    </row>
-    <row r="18" spans="1:12" x14ac:dyDescent="0.2">
+      <c r="M17" s="3"/>
+      <c r="N17" s="3"/>
+      <c r="O17" s="3"/>
+    </row>
+    <row r="18" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A18" s="3">
         <v>16</v>
       </c>
@@ -5051,8 +5188,11 @@
       <c r="J18" s="3"/>
       <c r="K18" s="3"/>
       <c r="L18" s="3"/>
-    </row>
-    <row r="19" spans="1:12" x14ac:dyDescent="0.2">
+      <c r="M18" s="3"/>
+      <c r="N18" s="3"/>
+      <c r="O18" s="3"/>
+    </row>
+    <row r="19" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A19" s="3">
         <v>17</v>
       </c>
@@ -5067,8 +5207,11 @@
       <c r="J19" s="3"/>
       <c r="K19" s="3"/>
       <c r="L19" s="3"/>
-    </row>
-    <row r="20" spans="1:12" x14ac:dyDescent="0.2">
+      <c r="M19" s="3"/>
+      <c r="N19" s="3"/>
+      <c r="O19" s="3"/>
+    </row>
+    <row r="20" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A20" s="3">
         <v>18</v>
       </c>
@@ -5083,8 +5226,11 @@
       <c r="J20" s="3"/>
       <c r="K20" s="3"/>
       <c r="L20" s="3"/>
-    </row>
-    <row r="21" spans="1:12" x14ac:dyDescent="0.2">
+      <c r="M20" s="3"/>
+      <c r="N20" s="3"/>
+      <c r="O20" s="3"/>
+    </row>
+    <row r="21" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A21" s="3">
         <v>19</v>
       </c>
@@ -5099,8 +5245,11 @@
       <c r="J21" s="3"/>
       <c r="K21" s="3"/>
       <c r="L21" s="3"/>
-    </row>
-    <row r="22" spans="1:12" x14ac:dyDescent="0.2">
+      <c r="M21" s="3"/>
+      <c r="N21" s="3"/>
+      <c r="O21" s="3"/>
+    </row>
+    <row r="22" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A22" s="3">
         <v>20</v>
       </c>
@@ -5115,8 +5264,11 @@
       <c r="J22" s="3"/>
       <c r="K22" s="3"/>
       <c r="L22" s="3"/>
-    </row>
-    <row r="23" spans="1:12" x14ac:dyDescent="0.2">
+      <c r="M22" s="3"/>
+      <c r="N22" s="3"/>
+      <c r="O22" s="3"/>
+    </row>
+    <row r="23" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A23" s="3">
         <v>21</v>
       </c>
@@ -5131,8 +5283,11 @@
       <c r="J23" s="3"/>
       <c r="K23" s="3"/>
       <c r="L23" s="3"/>
-    </row>
-    <row r="24" spans="1:12" x14ac:dyDescent="0.2">
+      <c r="M23" s="3"/>
+      <c r="N23" s="3"/>
+      <c r="O23" s="3"/>
+    </row>
+    <row r="24" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A24" s="3">
         <v>22</v>
       </c>
@@ -5147,8 +5302,11 @@
       <c r="J24" s="3"/>
       <c r="K24" s="3"/>
       <c r="L24" s="3"/>
-    </row>
-    <row r="25" spans="1:12" x14ac:dyDescent="0.2">
+      <c r="M24" s="3"/>
+      <c r="N24" s="3"/>
+      <c r="O24" s="3"/>
+    </row>
+    <row r="25" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A25" s="3">
         <v>23</v>
       </c>
@@ -5163,8 +5321,11 @@
       <c r="J25" s="3"/>
       <c r="K25" s="3"/>
       <c r="L25" s="3"/>
-    </row>
-    <row r="26" spans="1:12" x14ac:dyDescent="0.2">
+      <c r="M25" s="3"/>
+      <c r="N25" s="3"/>
+      <c r="O25" s="3"/>
+    </row>
+    <row r="26" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A26" s="3">
         <v>24</v>
       </c>
@@ -5179,8 +5340,11 @@
       <c r="J26" s="3"/>
       <c r="K26" s="3"/>
       <c r="L26" s="3"/>
-    </row>
-    <row r="27" spans="1:12" x14ac:dyDescent="0.2">
+      <c r="M26" s="3"/>
+      <c r="N26" s="3"/>
+      <c r="O26" s="3"/>
+    </row>
+    <row r="27" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A27" s="3">
         <v>25</v>
       </c>
@@ -5195,8 +5359,11 @@
       <c r="J27" s="3"/>
       <c r="K27" s="3"/>
       <c r="L27" s="3"/>
-    </row>
-    <row r="28" spans="1:12" x14ac:dyDescent="0.2">
+      <c r="M27" s="3"/>
+      <c r="N27" s="3"/>
+      <c r="O27" s="3"/>
+    </row>
+    <row r="28" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A28" s="3">
         <v>26</v>
       </c>
@@ -5211,8 +5378,11 @@
       <c r="J28" s="3"/>
       <c r="K28" s="3"/>
       <c r="L28" s="3"/>
-    </row>
-    <row r="29" spans="1:12" x14ac:dyDescent="0.2">
+      <c r="M28" s="3"/>
+      <c r="N28" s="3"/>
+      <c r="O28" s="3"/>
+    </row>
+    <row r="29" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A29" s="3">
         <v>27</v>
       </c>
@@ -5227,8 +5397,11 @@
       <c r="J29" s="3"/>
       <c r="K29" s="3"/>
       <c r="L29" s="3"/>
-    </row>
-    <row r="30" spans="1:12" x14ac:dyDescent="0.2">
+      <c r="M29" s="3"/>
+      <c r="N29" s="3"/>
+      <c r="O29" s="3"/>
+    </row>
+    <row r="30" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A30" s="3">
         <v>28</v>
       </c>
@@ -5243,8 +5416,11 @@
       <c r="J30" s="3"/>
       <c r="K30" s="3"/>
       <c r="L30" s="3"/>
-    </row>
-    <row r="31" spans="1:12" x14ac:dyDescent="0.2">
+      <c r="M30" s="3"/>
+      <c r="N30" s="3"/>
+      <c r="O30" s="3"/>
+    </row>
+    <row r="31" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A31" s="3">
         <v>29</v>
       </c>
@@ -5259,8 +5435,11 @@
       <c r="J31" s="3"/>
       <c r="K31" s="3"/>
       <c r="L31" s="3"/>
-    </row>
-    <row r="32" spans="1:12" x14ac:dyDescent="0.2">
+      <c r="M31" s="3"/>
+      <c r="N31" s="3"/>
+      <c r="O31" s="3"/>
+    </row>
+    <row r="32" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A32" s="3">
         <v>30</v>
       </c>
@@ -5275,10 +5454,393 @@
       <c r="J32" s="3"/>
       <c r="K32" s="3"/>
       <c r="L32" s="3"/>
+      <c r="M32" s="3"/>
+      <c r="N32" s="3"/>
+      <c r="O32" s="3"/>
+    </row>
+    <row r="33" spans="1:15" x14ac:dyDescent="0.2">
+      <c r="A33" s="3">
+        <v>31</v>
+      </c>
+      <c r="B33" s="3"/>
+      <c r="C33" s="3"/>
+      <c r="D33" s="3"/>
+      <c r="E33" s="3"/>
+      <c r="F33" s="3"/>
+      <c r="G33" s="3"/>
+      <c r="H33" s="3"/>
+      <c r="I33" s="3"/>
+      <c r="J33" s="3"/>
+      <c r="K33" s="3"/>
+      <c r="L33" s="3"/>
+      <c r="M33" s="3"/>
+      <c r="N33" s="3"/>
+      <c r="O33" s="3"/>
+    </row>
+    <row r="34" spans="1:15" x14ac:dyDescent="0.2">
+      <c r="A34" s="3">
+        <v>32</v>
+      </c>
+      <c r="B34" s="3"/>
+      <c r="C34" s="3"/>
+      <c r="D34" s="3"/>
+      <c r="E34" s="3"/>
+      <c r="F34" s="3"/>
+      <c r="G34" s="3"/>
+      <c r="H34" s="3"/>
+      <c r="I34" s="3"/>
+      <c r="J34" s="3"/>
+      <c r="K34" s="3"/>
+      <c r="L34" s="3"/>
+      <c r="M34" s="3"/>
+      <c r="N34" s="3"/>
+      <c r="O34" s="3"/>
+    </row>
+    <row r="35" spans="1:15" x14ac:dyDescent="0.2">
+      <c r="A35" s="3">
+        <v>33</v>
+      </c>
+      <c r="B35" s="3"/>
+      <c r="C35" s="3"/>
+      <c r="D35" s="3"/>
+      <c r="E35" s="3"/>
+      <c r="F35" s="3"/>
+      <c r="G35" s="3"/>
+      <c r="H35" s="3"/>
+      <c r="I35" s="3"/>
+      <c r="J35" s="3"/>
+      <c r="K35" s="3"/>
+      <c r="L35" s="3"/>
+      <c r="M35" s="3"/>
+      <c r="N35" s="3"/>
+      <c r="O35" s="3"/>
+    </row>
+    <row r="36" spans="1:15" x14ac:dyDescent="0.2">
+      <c r="A36" s="3">
+        <v>34</v>
+      </c>
+      <c r="B36" s="3"/>
+      <c r="C36" s="3"/>
+      <c r="D36" s="3"/>
+      <c r="E36" s="3"/>
+      <c r="F36" s="3"/>
+      <c r="G36" s="3"/>
+      <c r="H36" s="3"/>
+      <c r="I36" s="3"/>
+      <c r="J36" s="3"/>
+      <c r="K36" s="3"/>
+      <c r="L36" s="3"/>
+      <c r="M36" s="3"/>
+      <c r="N36" s="3"/>
+      <c r="O36" s="3"/>
+    </row>
+    <row r="37" spans="1:15" x14ac:dyDescent="0.2">
+      <c r="A37" s="3">
+        <v>35</v>
+      </c>
+      <c r="B37" s="3"/>
+      <c r="C37" s="3"/>
+      <c r="D37" s="3"/>
+      <c r="E37" s="3"/>
+      <c r="F37" s="3"/>
+      <c r="G37" s="3"/>
+      <c r="H37" s="3"/>
+      <c r="I37" s="3"/>
+      <c r="J37" s="3"/>
+      <c r="K37" s="3"/>
+      <c r="L37" s="3"/>
+      <c r="M37" s="3"/>
+      <c r="N37" s="3"/>
+      <c r="O37" s="3"/>
+    </row>
+    <row r="38" spans="1:15" x14ac:dyDescent="0.2">
+      <c r="A38" s="3">
+        <v>36</v>
+      </c>
+      <c r="B38" s="3"/>
+      <c r="C38" s="3"/>
+      <c r="D38" s="3"/>
+      <c r="E38" s="3"/>
+      <c r="F38" s="3"/>
+      <c r="G38" s="3"/>
+      <c r="H38" s="3"/>
+      <c r="I38" s="3"/>
+      <c r="J38" s="3"/>
+      <c r="K38" s="3"/>
+      <c r="L38" s="3"/>
+      <c r="M38" s="3"/>
+      <c r="N38" s="3"/>
+      <c r="O38" s="3"/>
+    </row>
+    <row r="39" spans="1:15" x14ac:dyDescent="0.2">
+      <c r="A39" s="3">
+        <v>37</v>
+      </c>
+      <c r="B39" s="3"/>
+      <c r="C39" s="3"/>
+      <c r="D39" s="3"/>
+      <c r="E39" s="3"/>
+      <c r="F39" s="3"/>
+      <c r="G39" s="3"/>
+      <c r="H39" s="3"/>
+      <c r="I39" s="3"/>
+      <c r="J39" s="3"/>
+      <c r="K39" s="3"/>
+      <c r="L39" s="3"/>
+      <c r="M39" s="3"/>
+      <c r="N39" s="3"/>
+      <c r="O39" s="3"/>
+    </row>
+    <row r="40" spans="1:15" x14ac:dyDescent="0.2">
+      <c r="A40" s="3">
+        <v>38</v>
+      </c>
+      <c r="B40" s="3"/>
+      <c r="C40" s="3"/>
+      <c r="D40" s="3"/>
+      <c r="E40" s="3"/>
+      <c r="F40" s="3"/>
+      <c r="G40" s="3"/>
+      <c r="H40" s="3"/>
+      <c r="I40" s="3"/>
+      <c r="J40" s="3"/>
+      <c r="K40" s="3"/>
+      <c r="L40" s="3"/>
+      <c r="M40" s="3"/>
+      <c r="N40" s="3"/>
+      <c r="O40" s="3"/>
+    </row>
+    <row r="41" spans="1:15" x14ac:dyDescent="0.2">
+      <c r="A41" s="3">
+        <v>39</v>
+      </c>
+      <c r="B41" s="3"/>
+      <c r="C41" s="3"/>
+      <c r="D41" s="3"/>
+      <c r="E41" s="3"/>
+      <c r="F41" s="3"/>
+      <c r="G41" s="3"/>
+      <c r="H41" s="3"/>
+      <c r="I41" s="3"/>
+      <c r="J41" s="3"/>
+      <c r="K41" s="3"/>
+      <c r="L41" s="3"/>
+      <c r="M41" s="3"/>
+      <c r="N41" s="3"/>
+      <c r="O41" s="3"/>
+    </row>
+    <row r="42" spans="1:15" x14ac:dyDescent="0.2">
+      <c r="A42" s="3">
+        <v>40</v>
+      </c>
+      <c r="B42" s="3"/>
+      <c r="C42" s="3"/>
+      <c r="D42" s="3"/>
+      <c r="E42" s="3"/>
+      <c r="F42" s="3"/>
+      <c r="G42" s="3"/>
+      <c r="H42" s="3"/>
+      <c r="I42" s="3"/>
+      <c r="J42" s="3"/>
+      <c r="K42" s="3"/>
+      <c r="L42" s="3"/>
+      <c r="M42" s="3"/>
+      <c r="N42" s="3"/>
+      <c r="O42" s="3"/>
+    </row>
+    <row r="43" spans="1:15" x14ac:dyDescent="0.2">
+      <c r="A43" s="3">
+        <v>41</v>
+      </c>
+      <c r="B43" s="3"/>
+      <c r="C43" s="3"/>
+      <c r="D43" s="3"/>
+      <c r="E43" s="3"/>
+      <c r="F43" s="3"/>
+      <c r="G43" s="3"/>
+      <c r="H43" s="3"/>
+      <c r="I43" s="3"/>
+      <c r="J43" s="3"/>
+      <c r="K43" s="3"/>
+      <c r="L43" s="3"/>
+      <c r="M43" s="3"/>
+      <c r="N43" s="3"/>
+      <c r="O43" s="3"/>
+    </row>
+    <row r="44" spans="1:15" x14ac:dyDescent="0.2">
+      <c r="A44" s="3">
+        <v>42</v>
+      </c>
+      <c r="B44" s="3"/>
+      <c r="C44" s="3"/>
+      <c r="D44" s="3"/>
+      <c r="E44" s="3"/>
+      <c r="F44" s="3"/>
+      <c r="G44" s="3"/>
+      <c r="H44" s="3"/>
+      <c r="I44" s="3"/>
+      <c r="J44" s="3"/>
+      <c r="K44" s="3"/>
+      <c r="L44" s="3"/>
+      <c r="M44" s="3"/>
+      <c r="N44" s="3"/>
+      <c r="O44" s="3"/>
+    </row>
+    <row r="45" spans="1:15" x14ac:dyDescent="0.2">
+      <c r="A45" s="3">
+        <v>43</v>
+      </c>
+      <c r="B45" s="3"/>
+      <c r="C45" s="3"/>
+      <c r="D45" s="3"/>
+      <c r="E45" s="3"/>
+      <c r="F45" s="3"/>
+      <c r="G45" s="3"/>
+      <c r="H45" s="3"/>
+      <c r="I45" s="3"/>
+      <c r="J45" s="3"/>
+      <c r="K45" s="3"/>
+      <c r="L45" s="3"/>
+      <c r="M45" s="3"/>
+      <c r="N45" s="3"/>
+      <c r="O45" s="3"/>
+    </row>
+    <row r="46" spans="1:15" x14ac:dyDescent="0.2">
+      <c r="A46" s="3">
+        <v>44</v>
+      </c>
+      <c r="B46" s="3"/>
+      <c r="C46" s="3"/>
+      <c r="D46" s="3"/>
+      <c r="E46" s="3"/>
+      <c r="F46" s="3"/>
+      <c r="G46" s="3"/>
+      <c r="H46" s="3"/>
+      <c r="I46" s="3"/>
+      <c r="J46" s="3"/>
+      <c r="K46" s="3"/>
+      <c r="L46" s="3"/>
+      <c r="M46" s="3"/>
+      <c r="N46" s="3"/>
+      <c r="O46" s="3"/>
+    </row>
+    <row r="47" spans="1:15" x14ac:dyDescent="0.2">
+      <c r="A47" s="3">
+        <v>45</v>
+      </c>
+      <c r="B47" s="3"/>
+      <c r="C47" s="3"/>
+      <c r="D47" s="3"/>
+      <c r="E47" s="3"/>
+      <c r="F47" s="3"/>
+      <c r="G47" s="3"/>
+      <c r="H47" s="3"/>
+      <c r="I47" s="3"/>
+      <c r="J47" s="3"/>
+      <c r="K47" s="3"/>
+      <c r="L47" s="3"/>
+      <c r="M47" s="3"/>
+      <c r="N47" s="3"/>
+      <c r="O47" s="3"/>
+    </row>
+    <row r="48" spans="1:15" x14ac:dyDescent="0.2">
+      <c r="A48" s="3">
+        <v>46</v>
+      </c>
+      <c r="B48" s="3"/>
+      <c r="C48" s="3"/>
+      <c r="D48" s="3"/>
+      <c r="E48" s="3"/>
+      <c r="F48" s="3"/>
+      <c r="G48" s="3"/>
+      <c r="H48" s="3"/>
+      <c r="I48" s="3"/>
+      <c r="J48" s="3"/>
+      <c r="K48" s="3"/>
+      <c r="L48" s="3"/>
+      <c r="M48" s="3"/>
+      <c r="N48" s="3"/>
+      <c r="O48" s="3"/>
+    </row>
+    <row r="49" spans="1:15" x14ac:dyDescent="0.2">
+      <c r="A49" s="3">
+        <v>47</v>
+      </c>
+      <c r="B49" s="3"/>
+      <c r="C49" s="3"/>
+      <c r="D49" s="3"/>
+      <c r="E49" s="3"/>
+      <c r="F49" s="3"/>
+      <c r="G49" s="3"/>
+      <c r="H49" s="3"/>
+      <c r="I49" s="3"/>
+      <c r="J49" s="3"/>
+      <c r="K49" s="3"/>
+      <c r="L49" s="3"/>
+      <c r="M49" s="3"/>
+      <c r="N49" s="3"/>
+      <c r="O49" s="3"/>
+    </row>
+    <row r="50" spans="1:15" x14ac:dyDescent="0.2">
+      <c r="A50" s="3">
+        <v>48</v>
+      </c>
+      <c r="B50" s="3"/>
+      <c r="C50" s="3"/>
+      <c r="D50" s="3"/>
+      <c r="E50" s="3"/>
+      <c r="F50" s="3"/>
+      <c r="G50" s="3"/>
+      <c r="H50" s="3"/>
+      <c r="I50" s="3"/>
+      <c r="J50" s="3"/>
+      <c r="K50" s="3"/>
+      <c r="L50" s="3"/>
+      <c r="M50" s="3"/>
+      <c r="N50" s="3"/>
+      <c r="O50" s="3"/>
+    </row>
+    <row r="51" spans="1:15" x14ac:dyDescent="0.2">
+      <c r="A51" s="3">
+        <v>49</v>
+      </c>
+      <c r="B51" s="3"/>
+      <c r="C51" s="3"/>
+      <c r="D51" s="3"/>
+      <c r="E51" s="3"/>
+      <c r="F51" s="3"/>
+      <c r="G51" s="3"/>
+      <c r="H51" s="3"/>
+      <c r="I51" s="3"/>
+      <c r="J51" s="3"/>
+      <c r="K51" s="3"/>
+      <c r="L51" s="3"/>
+      <c r="M51" s="3"/>
+      <c r="N51" s="3"/>
+      <c r="O51" s="3"/>
+    </row>
+    <row r="52" spans="1:15" x14ac:dyDescent="0.2">
+      <c r="A52" s="3">
+        <v>50</v>
+      </c>
+      <c r="B52" s="3"/>
+      <c r="C52" s="3"/>
+      <c r="D52" s="3"/>
+      <c r="E52" s="3"/>
+      <c r="F52" s="3"/>
+      <c r="G52" s="3"/>
+      <c r="H52" s="3"/>
+      <c r="I52" s="3"/>
+      <c r="J52" s="3"/>
+      <c r="K52" s="3"/>
+      <c r="L52" s="3"/>
+      <c r="M52" s="3"/>
+      <c r="N52" s="3"/>
+      <c r="O52" s="3"/>
     </row>
   </sheetData>
   <dataValidations count="1">
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="L3:L32" xr:uid="{D1121F3C-F660-0E46-8AEB-8C1F95C55489}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="O3:O52" xr:uid="{D1121F3C-F660-0E46-8AEB-8C1F95C55489}">
       <formula1>"Yes,No"</formula1>
     </dataValidation>
   </dataValidations>
@@ -10659,20 +11221,6 @@
     </row>
   </sheetData>
   <mergeCells count="30">
-    <mergeCell ref="D4:E4"/>
-    <mergeCell ref="P4:Q4"/>
-    <mergeCell ref="Y4:Z4"/>
-    <mergeCell ref="AB6:AC6"/>
-    <mergeCell ref="AN6:AO6"/>
-    <mergeCell ref="AB4:AC4"/>
-    <mergeCell ref="AN4:AO4"/>
-    <mergeCell ref="G6:H6"/>
-    <mergeCell ref="J4:K4"/>
-    <mergeCell ref="V6:W6"/>
-    <mergeCell ref="M6:N6"/>
-    <mergeCell ref="AH6:AI6"/>
-    <mergeCell ref="S6:T6"/>
-    <mergeCell ref="Y6:Z6"/>
     <mergeCell ref="AQ4:AR4"/>
     <mergeCell ref="A4:B4"/>
     <mergeCell ref="G4:H4"/>
@@ -10689,6 +11237,20 @@
     <mergeCell ref="AH4:AI4"/>
     <mergeCell ref="J6:K6"/>
     <mergeCell ref="P6:Q6"/>
+    <mergeCell ref="D4:E4"/>
+    <mergeCell ref="P4:Q4"/>
+    <mergeCell ref="Y4:Z4"/>
+    <mergeCell ref="AB6:AC6"/>
+    <mergeCell ref="AN6:AO6"/>
+    <mergeCell ref="AB4:AC4"/>
+    <mergeCell ref="AN4:AO4"/>
+    <mergeCell ref="G6:H6"/>
+    <mergeCell ref="J4:K4"/>
+    <mergeCell ref="V6:W6"/>
+    <mergeCell ref="M6:N6"/>
+    <mergeCell ref="AH6:AI6"/>
+    <mergeCell ref="S6:T6"/>
+    <mergeCell ref="Y6:Z6"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
@@ -12055,20 +12617,6 @@
     </row>
   </sheetData>
   <mergeCells count="30">
-    <mergeCell ref="A4:B4"/>
-    <mergeCell ref="G4:H4"/>
-    <mergeCell ref="P4:Q4"/>
-    <mergeCell ref="J4:K4"/>
-    <mergeCell ref="D7:E7"/>
-    <mergeCell ref="J7:K7"/>
-    <mergeCell ref="D4:E4"/>
-    <mergeCell ref="M4:N4"/>
-    <mergeCell ref="P7:Q7"/>
-    <mergeCell ref="AB7:AC7"/>
-    <mergeCell ref="A7:B7"/>
-    <mergeCell ref="G7:H7"/>
-    <mergeCell ref="S7:T7"/>
-    <mergeCell ref="M7:N7"/>
     <mergeCell ref="S4:T4"/>
     <mergeCell ref="AQ7:AR7"/>
     <mergeCell ref="AN4:AO4"/>
@@ -12085,6 +12633,20 @@
     <mergeCell ref="AE4:AF4"/>
     <mergeCell ref="V4:W4"/>
     <mergeCell ref="V7:W7"/>
+    <mergeCell ref="AB7:AC7"/>
+    <mergeCell ref="A7:B7"/>
+    <mergeCell ref="G7:H7"/>
+    <mergeCell ref="S7:T7"/>
+    <mergeCell ref="M7:N7"/>
+    <mergeCell ref="A4:B4"/>
+    <mergeCell ref="G4:H4"/>
+    <mergeCell ref="P4:Q4"/>
+    <mergeCell ref="J4:K4"/>
+    <mergeCell ref="D7:E7"/>
+    <mergeCell ref="J7:K7"/>
+    <mergeCell ref="D4:E4"/>
+    <mergeCell ref="M4:N4"/>
+    <mergeCell ref="P7:Q7"/>
   </mergeCells>
   <conditionalFormatting sqref="B6 A7:B7">
     <cfRule type="expression" dxfId="19" priority="1">

</xml_diff>

<commit_message>
template v27: joints sheet keeps c and phi together, residuals after them
Owner's edit: c, phi, c_res, phi_res, dil, t_cut, kn, ks, Jred, so a plain
Coulomb joint fills two adjacent cells and leaves the rest blank. Help box in
the same order. Packaged copy synced byte-identical.

Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01XjjT2aBxw8gY7EFdpoUcpj
</commit_message>
<xml_diff>
--- a/docs/inputs/input_template.xlsx
+++ b/docs/inputs/input_template.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/njones/python_projects/xslope/.claude/worktrees/joints-r1/docs/inputs/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{518FA263-91FA-F44E-9CA5-998A9947A78D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9855A05C-E080-7E4F-9B02-CD939BBA37C6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="4280" yWindow="2000" windowWidth="40460" windowHeight="22500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="4280" yWindow="2000" windowWidth="40460" windowHeight="22500" activeTab="10" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="main" sheetId="1" r:id="rId1"/>
@@ -2354,22 +2354,39 @@
             <a:defRPr/>
           </a:pPr>
           <a:r>
+            <a:rPr lang="en-US" sz="1100" b="1" baseline="0"/>
+            <a:t>phi</a:t>
+          </a:r>
+          <a:r>
+            <a:rPr lang="en-US" sz="1100" b="0" baseline="0"/>
+            <a:t> = joint friction angle, degrees</a:t>
+          </a:r>
+        </a:p>
+        <a:p>
+          <a:pPr marL="0" marR="0" lvl="0" indent="0" defTabSz="914400" eaLnBrk="1" fontAlgn="auto" latinLnBrk="0" hangingPunct="1">
+            <a:lnSpc>
+              <a:spcPct val="100000"/>
+            </a:lnSpc>
+            <a:spcBef>
+              <a:spcPts val="0"/>
+            </a:spcBef>
+            <a:spcAft>
+              <a:spcPts val="0"/>
+            </a:spcAft>
+            <a:buClrTx/>
+            <a:buSzTx/>
+            <a:buFontTx/>
+            <a:buNone/>
+            <a:tabLst/>
+            <a:defRPr/>
+          </a:pPr>
+          <a:r>
             <a:rPr lang="en-US" sz="1100" b="1"/>
             <a:t>c_res</a:t>
           </a:r>
           <a:r>
             <a:rPr lang="en-US" sz="1100" b="0" baseline="0"/>
             <a:t> = residual joint cohesion (blank = same as c)</a:t>
-          </a:r>
-        </a:p>
-        <a:p>
-          <a:r>
-            <a:rPr lang="en-US" sz="1100" b="1" baseline="0"/>
-            <a:t>phi</a:t>
-          </a:r>
-          <a:r>
-            <a:rPr lang="en-US" sz="1100" b="0" baseline="0"/>
-            <a:t> = joint friction angle, degrees</a:t>
           </a:r>
         </a:p>
         <a:p>
@@ -4860,10 +4877,10 @@
         <v>114</v>
       </c>
       <c r="H2" s="28" t="s">
+        <v>323</v>
+      </c>
+      <c r="I2" s="28" t="s">
         <v>326</v>
-      </c>
-      <c r="I2" s="28" t="s">
-        <v>323</v>
       </c>
       <c r="J2" s="28" t="s">
         <v>327</v>

</xml_diff>

<commit_message>
template v27: 'joints' is a polygon Type — a region a joint network is generated in
Owner's edit: the polygon sheet's Type list gains 'joints' on all fifteen
tables. A joints polygon carries no material and is never meshed as a zone; the
network generator clips its traces to it. Loader and generator pick it up with
the Studio network dialog. Packaged copy synced byte-identical.

Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01XjjT2aBxw8gY7EFdpoUcpj
</commit_message>
<xml_diff>
--- a/docs/inputs/input_template.xlsx
+++ b/docs/inputs/input_template.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/njones/python_projects/xslope/.claude/worktrees/joints-r1/docs/inputs/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9855A05C-E080-7E4F-9B02-CD939BBA37C6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{119A1861-00BF-3949-902B-66F34C8769AA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="4280" yWindow="2000" windowWidth="40460" windowHeight="22500" activeTab="10" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="4280" yWindow="2000" windowWidth="40460" windowHeight="22500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="main" sheetId="1" r:id="rId1"/>
@@ -11238,6 +11238,20 @@
     </row>
   </sheetData>
   <mergeCells count="30">
+    <mergeCell ref="D4:E4"/>
+    <mergeCell ref="P4:Q4"/>
+    <mergeCell ref="Y4:Z4"/>
+    <mergeCell ref="AB6:AC6"/>
+    <mergeCell ref="AN6:AO6"/>
+    <mergeCell ref="AB4:AC4"/>
+    <mergeCell ref="AN4:AO4"/>
+    <mergeCell ref="G6:H6"/>
+    <mergeCell ref="J4:K4"/>
+    <mergeCell ref="V6:W6"/>
+    <mergeCell ref="M6:N6"/>
+    <mergeCell ref="AH6:AI6"/>
+    <mergeCell ref="S6:T6"/>
+    <mergeCell ref="Y6:Z6"/>
     <mergeCell ref="AQ4:AR4"/>
     <mergeCell ref="A4:B4"/>
     <mergeCell ref="G4:H4"/>
@@ -11254,20 +11268,6 @@
     <mergeCell ref="AH4:AI4"/>
     <mergeCell ref="J6:K6"/>
     <mergeCell ref="P6:Q6"/>
-    <mergeCell ref="D4:E4"/>
-    <mergeCell ref="P4:Q4"/>
-    <mergeCell ref="Y4:Z4"/>
-    <mergeCell ref="AB6:AC6"/>
-    <mergeCell ref="AN6:AO6"/>
-    <mergeCell ref="AB4:AC4"/>
-    <mergeCell ref="AN4:AO4"/>
-    <mergeCell ref="G6:H6"/>
-    <mergeCell ref="J4:K4"/>
-    <mergeCell ref="V6:W6"/>
-    <mergeCell ref="M6:N6"/>
-    <mergeCell ref="AH6:AI6"/>
-    <mergeCell ref="S6:T6"/>
-    <mergeCell ref="Y6:Z6"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
@@ -12634,6 +12634,20 @@
     </row>
   </sheetData>
   <mergeCells count="30">
+    <mergeCell ref="A4:B4"/>
+    <mergeCell ref="G4:H4"/>
+    <mergeCell ref="P4:Q4"/>
+    <mergeCell ref="J4:K4"/>
+    <mergeCell ref="D7:E7"/>
+    <mergeCell ref="J7:K7"/>
+    <mergeCell ref="D4:E4"/>
+    <mergeCell ref="M4:N4"/>
+    <mergeCell ref="P7:Q7"/>
+    <mergeCell ref="AB7:AC7"/>
+    <mergeCell ref="A7:B7"/>
+    <mergeCell ref="G7:H7"/>
+    <mergeCell ref="S7:T7"/>
+    <mergeCell ref="M7:N7"/>
     <mergeCell ref="S4:T4"/>
     <mergeCell ref="AQ7:AR7"/>
     <mergeCell ref="AN4:AO4"/>
@@ -12650,20 +12664,6 @@
     <mergeCell ref="AE4:AF4"/>
     <mergeCell ref="V4:W4"/>
     <mergeCell ref="V7:W7"/>
-    <mergeCell ref="AB7:AC7"/>
-    <mergeCell ref="A7:B7"/>
-    <mergeCell ref="G7:H7"/>
-    <mergeCell ref="S7:T7"/>
-    <mergeCell ref="M7:N7"/>
-    <mergeCell ref="A4:B4"/>
-    <mergeCell ref="G4:H4"/>
-    <mergeCell ref="P4:Q4"/>
-    <mergeCell ref="J4:K4"/>
-    <mergeCell ref="D7:E7"/>
-    <mergeCell ref="J7:K7"/>
-    <mergeCell ref="D4:E4"/>
-    <mergeCell ref="M4:N4"/>
-    <mergeCell ref="P7:Q7"/>
   </mergeCells>
   <conditionalFormatting sqref="B6 A7:B7">
     <cfRule type="expression" dxfId="19" priority="1">
@@ -12741,8 +12741,8 @@
     </cfRule>
   </conditionalFormatting>
   <dataValidations count="1">
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="B5 E5 H5 K5 N5 Q5 T5 W5 Z5 AC5 AF5 AI5 AL5 AO5 AR5" xr:uid="{00000000-0002-0000-0300-000000000000}">
-      <formula1>"material,ssr reduce,ssr hold,ssr elastic,refine"</formula1>
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="B5 E5 H5 K5 N5 Q5 T5 W5 Z5 AC5 AF5 AI5 AL5 AO5 AR5" xr:uid="{2C58C22E-BB25-6145-9297-FDBC71F3461D}">
+      <formula1>"material,ssr reduce,ssr hold,ssr elastic,refine,joints"</formula1>
     </dataValidation>
   </dataValidations>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>